<commit_message>
TASK: Parking lot - add 3 backlog items (VeritaTrack calendar expand, VeritaScan evidence link, hide unused master-list sections)
PLAN:
  1. Add OPEN entries 45 (VeritaTrack calendar cells not clickable/expandable, hidden +N tasks unreachable), 46 (VeritaScan cannot attach/link policy or evidence to a line item), 47 (prospect asked to hide unused sections from a master list to reduce clutter).
  2. Regenerate PARKING_LOT.xlsx from the markdown source.

Self-check:
  - Each entry carries Effort + Importance + a paragraph per the parking-lot format.
  - xlsx regenerated and committed with the md (OPEN 19 / CLOSED 35 / RETIRED 6); no drift.
  - Docs-only change; no code or customer-facing surface touched.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PARKING_LOT.xlsx
+++ b/PARKING_LOT.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RETIRED" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$36</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RETIRED'!$A$1:$H$7</definedName>
   </definedNames>
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1172,8 +1172,206 @@
       </c>
       <c r="H15" s="3" t="inlineStr"/>
     </row>
+    <row r="16" ht="90" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>License stamp clobbers the §6 lab-identity header/footer and can name the wrong lab</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Parked by operator decision 2026-07-16 ("log it, finish PR 4 first"). Not started. No code touched.
+---</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>S-M (one shared helper plus a verify script; 8 callsites to re-check)</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Medium-High. Every customer-facing workbook currently prints a header and foo...</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>licenseCtxFromReq (server/routes.ts:57-61) resolves the licensee lab from resolveActiveLabForRequest, which reads the X-Active-Lab-Id header and silently falls back to the user's default lab inside a bare catch {}. The export body meanwhile resolves the lab from req.scope.labId (the URL path param, set by labScopeMiddleware). Two sources of truth for one document. Separately and unconditionally, applyLicenseToExcelJSWorkbook (shared/licenseExceljs.ts:93-96) *assigns* rather than merges oddHeader/oddFooter on every sheet, so the six lines in the VeritaMap export that carefully set ${labName} CLIA: ${cliaNumber} (routes.ts:13932-13933, 14215-14216, 14224-14225) are dead code, overwritten at routes.ts:14237. §6 rule 3 exists so identity survives cell-level copy-paste; layers (b) and (c) do not currently exist in any shipped workbook.</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-16 session, PR 4 (#1046) Gate 3 render. Related: feedback_pdf_lab_identity_resolution memory (same resolveActiveLabForRequest swallowed-throw shape).</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17" ht="90" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Long Excel column headers are clipped, truncating CFR citations mid-string</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Parked by operator decision 2026-07-16. Not started. No code touched.
+---</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>S (compute the header row height from the longest wrapped header, or raise th...</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Medium. The VeritaMap workbook currently prints "Reference Range Attestation...</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>CLAUDE.md §6 specifies both "row height 20" for the header row and "wrap text" for cells. Those two rules conflict for any header longer than its column width. Row height 20 renders roughly one line of Calibri 11, so a header that wraps to two or three lines has its tail clipped in print and in PDF export. Confirmed on the live VeritaMap Compliance Map export: header row height is 20.0 with wrapText: true, and the three longest headers are "AMR Attestation (42 CFR 493.1253, per instrument)" (49 chars), "Reference Range Attestation (42 CFR 493.1253)" (45), and "Last Correlation / Method Comparison Date" (41). "Last SOP Review Date" and "AMR High (per instrument)" clip too.</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-16 session, PR 4 (#1046) Gate 3 render. Sibling of [[#43]]; both were found by looking at the rendered workbook, and neither was catchable by the verify scripts.</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr"/>
+    </row>
+    <row r="18" ht="90" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>VeritaTrack calendar month cells are not expandable, so hidden tasks are unreachable</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Open. Not started.
+---</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>S (1-3 days) — make each month cell open a detail view or expand in place, an...</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>High — a compliance calendar that hides tasks with no way to see them undercu...</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Effort: S (1-3 days) — make each month cell open a detail view or expand in place, and wire the "+N more" affordance to reveal the full task list. The data is already loaded, this is a UI interaction gap, not a data one.
+Importance: High — a compliance calendar that hides tasks with no way to see them undercuts the module's core promise of showing what a lab owes and when.</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23 session, Michael screenshot of the VeritaTrack calendar (lab 3, September cell).</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19" ht="90" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>VeritaScan line items cannot attach or link evidence (policy or uploaded document)</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Open. Not started.
+---</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>M (1-2 weeks) — add a per-item evidence link that reuses the VeritaScan URL-p...</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>High — showing evidence per line item is the whole point of a self-inspection...</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Effort: M (1-2 weeks) — add a per-item evidence link that reuses the VeritaScan URL-pointer model rather than storing files: let a line item reference an existing VeritaDC controlled document or an external URL, then surface it as completion evidence.
+Importance: High — showing evidence per line item is the whole point of a self-inspection; without it the scan records a status but cannot show the policy or document that satisfies it.</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-23 session, Michael. Recurring request.</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr"/>
+    </row>
+    <row r="20" ht="90" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Hide sections a lab does not use from a master list, to reduce clutter (prospect-requested)</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Open. Not started. Needs a one-line scope confirmation (which master list).
+---</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>S-M (a few days to ~2 weeks depending on scope) — a lab-level visibility togg...</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Medium-High — came straight from a live prospect today as an onboarding-frict...</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Effort: S-M (a few days to ~2 weeks depending on scope) — a lab-level visibility toggle that hides not-applicable or unused sections from a master-list view. Smaller if it is a "hide N/A" filter on the existing VeritaDC master list, larger if it also spans VeritaScan domains.
+Importance: Medium-High — came straight from a live prospect today as an onboarding-friction point; a lab that does not run a service line should not have to wade past its requirements.</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23 session, Michael relaying a prospect ask from a demo today.</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H15"/>
+  <autoFilter ref="A1:H20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
TASK: Parking lot - add 3 backlog items (VeritaTrack calendar, VeritaScan evidence, hide unused sections)
PLAN:
  1. Add OPEN entries 45/46/47 with Effort + Importance + paragraph.
  2. Regenerate PARKING_LOT.xlsx.

Self-check:
  - xlsx in sync (OPEN 19); docs-only.
</commit_message>
<xml_diff>
--- a/PARKING_LOT.xlsx
+++ b/PARKING_LOT.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RETIRED" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$36</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RETIRED'!$A$1:$H$7</definedName>
   </definedNames>
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1172,8 +1172,206 @@
       </c>
       <c r="H15" s="3" t="inlineStr"/>
     </row>
+    <row r="16" ht="90" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>License stamp clobbers the §6 lab-identity header/footer and can name the wrong lab</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Parked by operator decision 2026-07-16 ("log it, finish PR 4 first"). Not started. No code touched.
+---</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>S-M (one shared helper plus a verify script; 8 callsites to re-check)</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Medium-High. Every customer-facing workbook currently prints a header and foo...</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>licenseCtxFromReq (server/routes.ts:57-61) resolves the licensee lab from resolveActiveLabForRequest, which reads the X-Active-Lab-Id header and silently falls back to the user's default lab inside a bare catch {}. The export body meanwhile resolves the lab from req.scope.labId (the URL path param, set by labScopeMiddleware). Two sources of truth for one document. Separately and unconditionally, applyLicenseToExcelJSWorkbook (shared/licenseExceljs.ts:93-96) *assigns* rather than merges oddHeader/oddFooter on every sheet, so the six lines in the VeritaMap export that carefully set ${labName} CLIA: ${cliaNumber} (routes.ts:13932-13933, 14215-14216, 14224-14225) are dead code, overwritten at routes.ts:14237. §6 rule 3 exists so identity survives cell-level copy-paste; layers (b) and (c) do not currently exist in any shipped workbook.</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-16 session, PR 4 (#1046) Gate 3 render. Related: feedback_pdf_lab_identity_resolution memory (same resolveActiveLabForRequest swallowed-throw shape).</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17" ht="90" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Long Excel column headers are clipped, truncating CFR citations mid-string</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Parked by operator decision 2026-07-16. Not started. No code touched.
+---</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>S (compute the header row height from the longest wrapped header, or raise th...</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Medium. The VeritaMap workbook currently prints "Reference Range Attestation...</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>CLAUDE.md §6 specifies both "row height 20" for the header row and "wrap text" for cells. Those two rules conflict for any header longer than its column width. Row height 20 renders roughly one line of Calibri 11, so a header that wraps to two or three lines has its tail clipped in print and in PDF export. Confirmed on the live VeritaMap Compliance Map export: header row height is 20.0 with wrapText: true, and the three longest headers are "AMR Attestation (42 CFR 493.1253, per instrument)" (49 chars), "Reference Range Attestation (42 CFR 493.1253)" (45), and "Last Correlation / Method Comparison Date" (41). "Last SOP Review Date" and "AMR High (per instrument)" clip too.</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-16 session, PR 4 (#1046) Gate 3 render. Sibling of [[#43]]; both were found by looking at the rendered workbook, and neither was catchable by the verify scripts.</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr"/>
+    </row>
+    <row r="18" ht="90" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>VeritaTrack calendar month cells are not expandable, so hidden tasks are unreachable</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Open. Not started.
+---</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>S (1-3 days) — make each month cell open a detail view or expand in place, an...</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>High — a compliance calendar that hides tasks with no way to see them undercu...</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Effort: S (1-3 days) — make each month cell open a detail view or expand in place, and wire the "+N more" affordance to reveal the full task list. The data is already loaded, this is a UI interaction gap, not a data one.
+Importance: High — a compliance calendar that hides tasks with no way to see them undercuts the module's core promise of showing what a lab owes and when.</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23 session, Michael screenshot of the VeritaTrack calendar (lab 3, September cell).</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19" ht="90" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>VeritaScan line items cannot attach or link evidence (policy or uploaded document)</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Open. Not started.
+---</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>M (1-2 weeks) — add a per-item evidence link that reuses the VeritaScan URL-p...</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>High — showing evidence per line item is the whole point of a self-inspection...</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Effort: M (1-2 weeks) — add a per-item evidence link that reuses the VeritaScan URL-pointer model rather than storing files: let a line item reference an existing VeritaDC controlled document or an external URL, then surface it as completion evidence.
+Importance: High — showing evidence per line item is the whole point of a self-inspection; without it the scan records a status but cannot show the policy or document that satisfies it.</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-23 session, Michael. Recurring request.</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr"/>
+    </row>
+    <row r="20" ht="90" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Hide sections a lab does not use from a master list, to reduce clutter (prospect-requested)</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Open. Not started. Needs a one-line scope confirmation (which master list).
+---</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>S-M (a few days to ~2 weeks depending on scope) — a lab-level visibility togg...</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Medium-High — came straight from a live prospect today as an onboarding-frict...</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Effort: S-M (a few days to ~2 weeks depending on scope) — a lab-level visibility toggle that hides not-applicable or unused sections from a master-list view. Smaller if it is a "hide N/A" filter on the existing VeritaDC master list, larger if it also spans VeritaScan domains.
+Importance: Medium-High — came straight from a live prospect today as an onboarding-friction point; a lab that does not run a service line should not have to wade past its requirements.</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23 session, Michael relaying a prospect ask from a demo today.</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H15"/>
+  <autoFilter ref="A1:H20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
TASK: Parking lot - close #45 (VeritaTrack calendar, shipped) and add #48 (VeritaComp competency derivation)
PLAN:
  1. Move #45 (calendar expand) to CLOSED as C36 with closure evidence (PR #1309).
  2. Add OPEN #48: VeritaComp derive owed competencies from VeritaStaff assignments (mock-first, two design forks documented).
  3. Regenerate PARKING_LOT.xlsx.

Self-check:
  - C36 has closure evidence; #48 has Effort + Importance + paragraph.
  - xlsx regenerated from md; docs-only.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PARKING_LOT.xlsx
+++ b/PARKING_LOT.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$20</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$37</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RETIRED'!$A$1:$H$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1253,12 +1253,12 @@
     <row r="18" ht="90" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>46</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>VeritaTrack calendar month cells are not expandable, so hidden tasks are unreachable</t>
+          <t>VeritaScan line items cannot attach or link evidence (policy or uploaded document)</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -1269,23 +1269,23 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>S (1-3 days) — make each month cell open a detail view or expand in place, an...</t>
+          <t>M (1-2 weeks) — add a per-item evidence link that reuses the VeritaScan URL-p...</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>High — a compliance calendar that hides tasks with no way to see them undercu...</t>
+          <t>High — showing evidence per line item is the whole point of a self-inspection...</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Effort: S (1-3 days) — make each month cell open a detail view or expand in place, and wire the "+N more" affordance to reveal the full task list. The data is already loaded, this is a UI interaction gap, not a data one.
-Importance: High — a compliance calendar that hides tasks with no way to see them undercuts the module's core promise of showing what a lab owes and when.</t>
+          <t>Effort: M (1-2 weeks) — add a per-item evidence link that reuses the VeritaScan URL-pointer model rather than storing files: let a line item reference an existing VeritaDC controlled document or an external URL, then surface it as completion evidence.
+Importance: High — showing evidence per line item is the whole point of a self-inspection; without it the scan records a status but cannot show the policy or document that satisfies it.</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23 session, Michael screenshot of the VeritaTrack calendar (lab 3, September cell).</t>
+          <t>2026-09-23 session, Michael. Recurring request.</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr"/>
@@ -1293,39 +1293,39 @@
     <row r="19" ht="90" customHeight="1">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>46</t>
+          <t>47</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>VeritaScan line items cannot attach or link evidence (policy or uploaded document)</t>
+          <t>Hide sections a lab does not use from a master list, to reduce clutter (prospect-requested)</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Open. Not started.
+          <t>Open. Not started. Needs a one-line scope confirmation (which master list).
 ---</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>M (1-2 weeks) — add a per-item evidence link that reuses the VeritaScan URL-p...</t>
+          <t>S-M (a few days to ~2 weeks depending on scope) — a lab-level visibility togg...</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>High — showing evidence per line item is the whole point of a self-inspection...</t>
+          <t>Medium-High — came straight from a live prospect today as an onboarding-frict...</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>Effort: M (1-2 weeks) — add a per-item evidence link that reuses the VeritaScan URL-pointer model rather than storing files: let a line item reference an existing VeritaDC controlled document or an external URL, then surface it as completion evidence.
-Importance: High — showing evidence per line item is the whole point of a self-inspection; without it the scan records a status but cannot show the policy or document that satisfies it.</t>
+          <t>Effort: S-M (a few days to ~2 weeks depending on scope) — a lab-level visibility toggle that hides not-applicable or unused sections from a master-list view. Smaller if it is a "hide N/A" filter on the existing VeritaDC master list, larger if it also spans VeritaScan domains.
+Importance: Medium-High — came straight from a live prospect today as an onboarding-friction point; a lab that does not run a service line should not have to wade past its requirements.</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>2026-09-23 session, Michael. Recurring request.</t>
+          <t>2026-09-23 session, Michael relaying a prospect ask from a demo today.</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr"/>
@@ -1333,39 +1333,39 @@
     <row r="20" ht="90" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>48</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Hide sections a lab does not use from a master list, to reduce clutter (prospect-requested)</t>
+          <t>VeritaComp: derive owed competencies from VeritaStaff instrument/test assignments</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Open. Not started. Needs a one-line scope confirmation (which master list).
+          <t>Open. Investigated 2026-09-24; ready to build mock-first, pending Michael's steer on the two forks.
 ---</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>S-M (a few days to ~2 weeks depending on scope) — a lab-level visibility togg...</t>
+          <t>M-L (mock-first design plus the derivation and UI). The data model exists but...</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Medium-High — came straight from a live prospect today as an onboarding-frict...</t>
+          <t>High — Michael pitches to prospects that VeritaComp bases owed competencies o...</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Effort: S-M (a few days to ~2 weeks depending on scope) — a lab-level visibility toggle that hides not-applicable or unused sections from a master-list view. Smaller if it is a "hide N/A" filter on the existing VeritaDC master list, larger if it also spans VeritaScan domains.
-Importance: Medium-High — came straight from a live prospect today as an onboarding-friction point; a lab that does not run a service line should not have to wade past its requirements.</t>
+          <t>Effort: M-L (mock-first design plus the derivation and UI). The data model exists but the join is not trivial.
+Importance: High — Michael pitches to prospects that VeritaComp bases owed competencies on each staffer's VeritaStaff instrument/test selections. Currently untrue; making the pitch honest is the point.</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23 session, Michael relaying a prospect ask from a demo today.</t>
+          <t>2026-09-24 session, Michael (pitch-integrity gap).</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr"/>
@@ -1382,7 +1382,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H36"/>
+  <dimension ref="A1:H37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1440,18 +1440,40 @@
     <row r="2" ht="90" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>C34</t>
+          <t>C36</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Wire the two static-audit guards into CI (was #43)</t>
+          <t>VeritaTrack calendar month cells expand to reveal hidden tasks (was #45)</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr"/>
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Closure evidence: PR #1309 (squash on main e398d341), client/src/pages/VeritaTrackAppPage.tsx CalendarView. Month cells with more than 3 tasks are clickable and expand in place (chevron, "+N more" toggles to "Show less", due dates shown when open). Shipped and deployed 2026-09-24. Env-gated spec tests/playwright/veritatrack-calendar-expand.spec.ts.</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3" ht="90" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>C34</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Wire the two static-audit guards into CI (was #43)</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr"/>
+      <c r="D3" s="3" t="inlineStr"/>
+      <c r="E3" s="3" t="inlineStr"/>
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: both guards wired into the Multi-Lab Mutations Audit CI
 workflow (.github/workflows/multilab-mutations-audit.yml) as steps:
@@ -1463,24 +1485,24 @@
 (same caveat as the existing guards already in that workflow).</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr"/>
-    </row>
-    <row r="3" ht="90" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr"/>
+      <c r="H3" s="3" t="inlineStr"/>
+    </row>
+    <row r="4" ht="90" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>C35</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Legacy /api/studies over-returns studies across labs (was #44)</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr"/>
-      <c r="D3" s="3" t="inlineStr"/>
-      <c r="E3" s="3" t="inlineStr"/>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr"/>
+      <c r="D4" s="2" t="inlineStr"/>
+      <c r="E4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: GET /api/studies now scopes its list to the active lab
 when one is resolved from the Referer (server/routes.ts), so every returned row
@@ -1490,24 +1512,24 @@
 mirroring the /api/labs/:labId/studies handler. Closed 2026-06-14.</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr"/>
-      <c r="H3" s="3" t="inlineStr"/>
-    </row>
-    <row r="4" ht="90" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5" ht="90" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>C30</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>Verify-script convention backfill (was #41)</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr"/>
-      <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="2" t="inlineStr"/>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr"/>
+      <c r="D5" s="3" t="inlineStr"/>
+      <c r="E5" s="3" t="inlineStr"/>
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: all 8 high-stakes math/logic commits now ship a paired
 scripts/verify-*.js (EP17 sensitivity, Deming lot-to-lot, CUMSUM+QC+multi-analyte,
@@ -1515,30 +1537,30 @@
 TEa boundary), per the strike-throughs in #41. Closed 2026-06-13.</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>scripts/audit_verify_script_coverage.py lookback, 2026-06-02; backfills
 landed 2026-06-03..06.
 ---</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr"/>
-    </row>
-    <row r="5" ht="90" customHeight="1">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr"/>
+    </row>
+    <row r="6" ht="90" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>C31</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>VeritaPT AAA create/update/delete silently no-op in the multi-lab UI</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr"/>
-      <c r="D5" s="3" t="inlineStr"/>
-      <c r="E5" s="3" t="inlineStr"/>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr"/>
+      <c r="D6" s="2" t="inlineStr"/>
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #754 (commit 92ad499) added lab-scoped POST/PUT/DELETE
 /api/labs/:labId/pt/aa-records. The UI posted to the lab-scoped path but only GET
@@ -1549,30 +1571,30 @@
 route mis-filed records to the user's default lab on multi-lab accounts).</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>2026-06-13, found during #18 Phase 3 QA;
 scripts/audit-labscoped-write-routes.mjs now guards the class.
 ---</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr"/>
-    </row>
-    <row r="6" ht="90" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7" ht="90" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>C32</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>VeritaComp "Unlock assessment" false-success no-op</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr"/>
-      <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr"/>
+      <c r="D7" s="3" t="inlineStr"/>
+      <c r="E7" s="3" t="inlineStr"/>
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #755 (commit 4234007) moved the unlock route to
 /api/labs/:labId/competency/assessments/:id/unlock (the path the client calls).
@@ -1583,29 +1605,29 @@
 HTML).</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G7" s="3" t="inlineStr">
         <is>
           <t>2026-06-13, found by scripts/audit-labscoped-write-routes.mjs.
 ---</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr"/>
-    </row>
-    <row r="7" ht="90" customHeight="1">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="H7" s="3" t="inlineStr"/>
+    </row>
+    <row r="8" ht="90" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>C33</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>FK-cascade delete 500s + NavBar laptop-width overflow</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr"/>
-      <c r="D7" s="3" t="inlineStr"/>
-      <c r="E7" s="3" t="inlineStr"/>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr"/>
+      <c r="D8" s="2" t="inlineStr"/>
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PRs #749/#750 fixed NavBar horizontal overflow at laptop
 widths (collapse to the hamburger below 1560px); prod-verified at 1280-1920 with the
@@ -1616,37 +1638,9 @@
 500 -&gt; 200. scripts/audit-delete-cascades.mjs guards the class.</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>2026-06-13 browser QA of the A7-D4 wave + retro-QC of the 72h PR window.
----</t>
-        </is>
-      </c>
-      <c r="H7" s="3" t="inlineStr"/>
-    </row>
-    <row r="8" ht="90" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>C1</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>FAQ "over 25 years" -&gt; "over 23 years"</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr"/>
-      <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>Closure evidence: client/src/pages/FAQPage.tsx line 20 reads "over
-23 years" as of 2026-05-01.</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>session 299e9a73 turn 14, ~2026-04-28.
 ---</t>
         </is>
       </c>
@@ -1655,18 +1649,46 @@
     <row r="9" ht="90" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>C5</t>
+          <t>C1</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>David's VeritaQA grey-button bug (seat permissions mode)</t>
+          <t>FAQ "over 25 years" -&gt; "over 23 years"</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr"/>
       <c r="D9" s="3" t="inlineStr"/>
       <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Closure evidence: client/src/pages/FAQPage.tsx line 20 reads "over
+23 years" as of 2026-05-01.</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>session 299e9a73 turn 14, ~2026-04-28.
+---</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr"/>
+    </row>
+    <row r="10" ht="90" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>David's VeritaQA grey-button bug (seat permissions mode)</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr"/>
+      <c r="D10" s="2" t="inlineStr"/>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #10 squash-merged as commit a43fbba on
 2026-05-01 23:19 MST. Railway deploy succeeded; deployed bundle
@@ -1679,7 +1701,7 @@
 against his exact stored shape (14 of 14 expected outcomes matched).</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>2026-05-01 David's report; veritabench + veritastock
 weren't in MODULE_LIST so seat permissions silently defaulted to
@@ -1687,46 +1709,17 @@
 ---</t>
         </is>
       </c>
-      <c r="H9" s="3" t="inlineStr"/>
-    </row>
-    <row r="10" ht="90" customHeight="1">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>C2</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>TeamPage present-tense "TJC surveyor" check</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr"/>
-      <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>Closure evidence: site-wide search confirmed all surveyor language
-is past-tense, consistent with user's 2021-2025 service. User closed
-the item in session 299e9a73 turn 4.</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>session 299e9a73, ~2026-04-28.
----</t>
-        </is>
-      </c>
       <c r="H10" s="2" t="inlineStr"/>
     </row>
     <row r="11" ht="90" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>C3</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>My Studies CSV/XLSX export (John as design partner)</t>
+          <t>TeamPage present-tense "TJC surveyor" check</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr"/>
@@ -1734,14 +1727,14 @@
       <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: client/src/pages/DashboardPage.tsx line 46 calls
-/api/my-studies/export. server/routes.ts line 1491 implements the
-endpoint. Pulled forward into pre-COLA per user instruction.</t>
+          <t>Closure evidence: site-wide search confirmed all surveyor language
+is past-tense, consistent with user's 2021-2025 service. User closed
+the item in session 299e9a73 turn 4.</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>session 299e9a73 turn 5, ~2026-04-28.
+          <t>session 299e9a73, ~2026-04-28.
 ---</t>
         </is>
       </c>
@@ -1750,12 +1743,12 @@
     <row r="12" ht="90" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>C4</t>
+          <t>C3</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Rotate GitHub PAT (because old PAT was committed in SESSION_HANDOFF files)</t>
+          <t>My Studies CSV/XLSX export (John as design partner)</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr"/>
@@ -1763,13 +1756,14 @@
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: no ghp_* or github_pat_* patterns in current
-SESSION_HANDOFF.md or SESSION_HANDOFF-2.md as of 2026-05-01.</t>
+          <t>Closure evidence: client/src/pages/DashboardPage.tsx line 46 calls
+/api/my-studies/export. server/routes.ts line 1491 implements the
+endpoint. Pulled forward into pre-COLA per user instruction.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>session 299e9a73, ~2026-04-28.
+          <t>session 299e9a73 turn 5, ~2026-04-28.
 ---</t>
         </is>
       </c>
@@ -1778,18 +1772,46 @@
     <row r="13" ht="90" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>C6</t>
+          <t>C4</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>VeritaPolicy service-line filtering removed (formerly #4)</t>
+          <t>Rotate GitHub PAT (because old PAT was committed in SESSION_HANDOFF files)</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr"/>
       <c r="D13" s="3" t="inlineStr"/>
       <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Closure evidence: no ghp_* or github_pat_* patterns in current
+SESSION_HANDOFF.md or SESSION_HANDOFF-2.md as of 2026-05-01.</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>session 299e9a73, ~2026-04-28.
+---</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14" ht="90" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>C6</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>VeritaPolicy service-line filtering removed (formerly #4)</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr"/>
+      <c r="D14" s="2" t="inlineStr"/>
+      <c r="E14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>Closure rationale (operator decision 2026-05-10): Keep all
 VeritaPolicy rows. CFR-only references with no accreditor reference
@@ -1798,29 +1820,29 @@
 report misread the design intent.</t>
         </is>
       </c>
-      <c r="G13" s="3" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H13" s="3" t="inlineStr"/>
-    </row>
-    <row r="14" ht="90" customHeight="1">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="H14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15" ht="90" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>C7</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>CLIA number format validation (formerly #13)</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr"/>
-      <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="2" t="inlineStr"/>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr"/>
+      <c r="D15" s="3" t="inlineStr"/>
+      <c r="E15" s="3" t="inlineStr"/>
+      <c r="F15" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: shared/validateClia.ts defines CLIA_REGEX =
 /^\d{2}D\d{7}$/ (line 24), validateClia() helper with whitespace
@@ -1831,30 +1853,30 @@
 shape exists and behaves as specified.</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="G15" s="3" t="inlineStr">
         <is>
           <t>Agent verification 2026-05-10 via grep + file read.
 Operator confirmed shipped 2026-05-10.
 ---</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr"/>
-    </row>
-    <row r="15" ht="90" customHeight="1">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="H15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16" ht="90" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>C8</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>VeritaMap lab-wide menu toggle (formerly #19)</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr"/>
-      <c r="D15" s="3" t="inlineStr"/>
-      <c r="E15" s="3" t="inlineStr"/>
-      <c r="F15" s="3" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr"/>
+      <c r="D16" s="2" t="inlineStr"/>
+      <c r="E16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: client/src/pages/VeritaMapLabwidePage.tsx
 exists and implements the labwide read-only union view. Route is
@@ -1864,59 +1886,59 @@
 parking lot plan (read-only union view, per-session toggle) shipped.</t>
         </is>
       </c>
-      <c r="G15" s="3" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>Agent verification 2026-05-10 via grep + file read.
 Operator confirmed shipped 2026-05-10.
 ---</t>
         </is>
       </c>
-      <c r="H15" s="3" t="inlineStr"/>
-    </row>
-    <row r="16" ht="90" customHeight="1">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>C9</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>Tier-1 smoke test checklist (formerly #6)</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr"/>
-      <c r="D16" s="2" t="inlineStr"/>
-      <c r="E16" s="2" t="inlineStr"/>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>Closure evidence: docs/smoke-test-tier1.md documents the Tier-1
-smoke-test process and post-deploy verification steps. Shipped via
-PR #81 as part of the 2026-05-10 wave.</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>Operator instruction 2026-05-10 in this session.
----</t>
-        </is>
-      </c>
       <c r="H16" s="2" t="inlineStr"/>
     </row>
     <row r="17" ht="90" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>C10</t>
+          <t>C9</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Per-module gating (formerly #7)</t>
+          <t>Tier-1 smoke test checklist (formerly #6)</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr"/>
       <c r="D17" s="3" t="inlineStr"/>
       <c r="E17" s="3" t="inlineStr"/>
       <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Closure evidence: docs/smoke-test-tier1.md documents the Tier-1
+smoke-test process and post-deploy verification steps. Shipped via
+PR #81 as part of the 2026-05-10 wave.</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>Operator instruction 2026-05-10 in this session.
+---</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr"/>
+    </row>
+    <row r="18" ht="90" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>C10</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Per-module gating (formerly #7)</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr"/>
+      <c r="D18" s="2" t="inlineStr"/>
+      <c r="E18" s="2" t="inlineStr"/>
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: Client-side useIsReadOnly module keys wired
 on client/src/pages/VeritaPolicyAppPage.tsx and
@@ -1931,29 +1953,29 @@
 PR #76.</t>
         </is>
       </c>
-      <c r="G17" s="3" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H17" s="3" t="inlineStr"/>
-    </row>
-    <row r="18" ht="90" customHeight="1">
-      <c r="A18" s="2" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19" ht="90" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>C11</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>VeritaStock shipped copy (formerly #8)</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr"/>
-      <c r="D18" s="2" t="inlineStr"/>
-      <c r="E18" s="2" t="inlineStr"/>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="C19" s="3" t="inlineStr"/>
+      <c r="D19" s="3" t="inlineStr"/>
+      <c r="E19" s="3" t="inlineStr"/>
+      <c r="F19" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: client/src/pages/ArticleInventoryManagementPage.tsx
 line 305 footer reads "platform that includes VeritaStock™" instead
@@ -1961,29 +1983,29 @@
 on /resources/laboratory-inventory-management. Shipped via PR #75.</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="G19" s="3" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H18" s="2" t="inlineStr"/>
-    </row>
-    <row r="19" ht="90" customHeight="1">
-      <c r="A19" s="3" t="inlineStr">
+      <c r="H19" s="3" t="inlineStr"/>
+    </row>
+    <row r="20" ht="90" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>C12</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>Admin report one-row-per-lab (formerly #14)</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr"/>
-      <c r="D19" s="3" t="inlineStr"/>
-      <c r="E19" s="3" t="inlineStr"/>
-      <c r="F19" s="3" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr"/>
+      <c r="D20" s="2" t="inlineStr"/>
+      <c r="E20" s="2" t="inlineStr"/>
+      <c r="F20" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: /api/admin/report rewritten in
 server/routes.ts (~line 595) to LEFT JOIN labs on
@@ -1998,33 +2020,6 @@
 prerequisite, not a code bug). Shipped via PR #85.</t>
         </is>
       </c>
-      <c r="G19" s="3" t="inlineStr">
-        <is>
-          <t>Operator instruction 2026-05-10 in this session.
----</t>
-        </is>
-      </c>
-      <c r="H19" s="3" t="inlineStr"/>
-    </row>
-    <row r="20" ht="90" customHeight="1">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>C14</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>UI relabel "CLIA TEa" -&gt; "Lab-Set Internal Goal" (formerly #1)</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr"/>
-      <c r="D20" s="2" t="inlineStr"/>
-      <c r="E20" s="2" t="inlineStr"/>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>Closure evidence: Shipped across four PRs over 2026-05-10.</t>
-        </is>
-      </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
@@ -2036,18 +2031,45 @@
     <row r="21" ht="90" customHeight="1">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>C13</t>
+          <t>C14</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>WSLH PT vendor (formerly #15)</t>
+          <t>UI relabel "CLIA TEa" -&gt; "Lab-Set Internal Goal" (formerly #1)</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr"/>
       <c r="D21" s="3" t="inlineStr"/>
       <c r="E21" s="3" t="inlineStr"/>
       <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>Closure evidence: Shipped across four PRs over 2026-05-10.</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>Operator instruction 2026-05-10 in this session.
+---</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22" ht="90" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>C13</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>WSLH PT vendor (formerly #15)</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr"/>
+      <c r="D22" s="2" t="inlineStr"/>
+      <c r="E22" s="2" t="inlineStr"/>
+      <c r="F22" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: Shipped 2026-05-10 via PR #79 (merge commit
 eeebc6e; merged after rebase to resolve a server/db.ts collision
@@ -2065,38 +2087,9 @@
 'WSLH' is the post-deploy success signal. Shipped via PR #79.</t>
         </is>
       </c>
-      <c r="G21" s="3" t="inlineStr">
+      <c r="G22" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
----</t>
-        </is>
-      </c>
-      <c r="H21" s="3" t="inlineStr"/>
-    </row>
-    <row r="22" ht="90" customHeight="1">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>C15</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>VeritaStock lot tracking + expiration + reorder alerts (formerly #21)</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr"/>
-      <c r="D22" s="2" t="inlineStr"/>
-      <c r="E22" s="2" t="inlineStr"/>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>Closure evidence: VeritaStock™ shipped the bench-level inventory
-features the Perplexity competitor analysis identified as a gap:</t>
-        </is>
-      </c>
-      <c r="G22" s="2" t="inlineStr">
-        <is>
-          <t>Originally Perplexity competitor analysis 2026-05-10.
-Audit 2026-05-21 confirmed the feature set ships today.
 ---</t>
         </is>
       </c>
@@ -2105,12 +2098,12 @@
     <row r="23" ht="90" customHeight="1">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>C16</t>
+          <t>C15</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>PAL studies guided workflow (formerly #23)</t>
+          <t>VeritaStock lot tracking + expiration + reorder alerts (formerly #21)</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr"/>
@@ -2118,15 +2111,14 @@
       <c r="E23" s="3" t="inlineStr"/>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: VeritaCheck™ already ships the Precision /
-Accuracy / Linearity (PAL) study set under EP-protocol naming:</t>
+          <t>Closure evidence: VeritaStock™ shipped the bench-level inventory
+features the Perplexity competitor analysis identified as a gap:</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
           <t>Originally Perplexity competitor analysis 2026-05-10.
-Audit 2026-05-21 confirmed the EP studies cover the PAL framing in
-full.
+Audit 2026-05-21 confirmed the feature set ships today.
 ---</t>
         </is>
       </c>
@@ -2135,12 +2127,12 @@
     <row r="24" ht="90" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>C17</t>
+          <t>C16</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Source-grounded 21/29/45 CFR + 42 CFR 482-485 (formerly #26)</t>
+          <t>PAL studies guided workflow (formerly #23)</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr"/>
@@ -2148,35 +2140,65 @@
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="2" t="inlineStr">
         <is>
+          <t>Closure evidence: VeritaCheck™ already ships the Precision /
+Accuracy / Linearity (PAL) study set under EP-protocol naming:</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>Originally Perplexity competitor analysis 2026-05-10.
+Audit 2026-05-21 confirmed the EP studies cover the PAL framing in
+full.
+---</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25" ht="90" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>C17</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Source-grounded 21/29/45 CFR + 42 CFR 482-485 (formerly #26)</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr"/>
+      <c r="D25" s="3" t="inlineStr"/>
+      <c r="E25" s="3" t="inlineStr"/>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
           <t>Closure evidence: PR #301 (commit 8c27806, merged 2026-05-21)
 source-grounded the 74 remaining non-493 entries in
 server/cfrRequirements.ts against verbatim eCFR XML. Breakdown
 shipped:</t>
         </is>
       </c>
-      <c r="G24" s="2" t="inlineStr">
+      <c r="G25" s="3" t="inlineStr">
         <is>
           <t>PR #301; tasks #18 in the in-session task tracker.
 ---</t>
         </is>
       </c>
-      <c r="H24" s="2" t="inlineStr"/>
-    </row>
-    <row r="25" ht="90" customHeight="1">
-      <c r="A25" s="3" t="inlineStr">
+      <c r="H25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26" ht="90" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>C18</t>
         </is>
       </c>
-      <c r="B25" s="3" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t>VeritaPolicy "Non CLIA" chapter rename (formerly #3)</t>
         </is>
       </c>
-      <c r="C25" s="3" t="inlineStr"/>
-      <c r="D25" s="3" t="inlineStr"/>
-      <c r="E25" s="3" t="inlineStr"/>
-      <c r="F25" s="3" t="inlineStr">
+      <c r="C26" s="2" t="inlineStr"/>
+      <c r="D26" s="2" t="inlineStr"/>
+      <c r="E26" s="2" t="inlineStr"/>
+      <c r="F26" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #300 (commit 34d7707, merged 2026-05-21)
 renamed all 44 user-facing chapter labels in
@@ -2187,7 +2209,7 @@
 page.</t>
         </is>
       </c>
-      <c r="G25" s="3" t="inlineStr">
+      <c r="G26" s="2" t="inlineStr">
         <is>
           <t>CAP customer screenshot of the /veritapolicy chapter
 headers, 2026-05-01 evening. PR #300; tasks #17 in the in-session
@@ -2195,23 +2217,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H25" s="3" t="inlineStr"/>
-    </row>
-    <row r="26" ht="90" customHeight="1">
-      <c r="A26" s="2" t="inlineStr">
+      <c r="H26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27" ht="90" customHeight="1">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>C19</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="B27" s="3" t="inlineStr">
         <is>
           <t>VeritaStock department-scope toggle (formerly #31)</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr"/>
-      <c r="D26" s="2" t="inlineStr"/>
-      <c r="E26" s="2" t="inlineStr"/>
-      <c r="F26" s="2" t="inlineStr">
+      <c r="C27" s="3" t="inlineStr"/>
+      <c r="D27" s="3" t="inlineStr"/>
+      <c r="E27" s="3" t="inlineStr"/>
+      <c r="F27" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #319 (commit d01f5fe, merged 2026-05-22)
 shipped the persistent dept-scope toggle on VeritaStockPage. A new
@@ -2222,7 +2244,7 @@
 workspace without re-filtering.</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr">
+      <c r="G27" s="3" t="inlineStr">
         <is>
           <t>John, San Carlos lab, 2026-05-21. Same conversation that
 drove the vendor dropdown (PR #304), FILTERED VIEW banner (PR #305),
@@ -2230,23 +2252,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H26" s="2" t="inlineStr"/>
-    </row>
-    <row r="27" ht="90" customHeight="1">
-      <c r="A27" s="3" t="inlineStr">
+      <c r="H27" s="3" t="inlineStr"/>
+    </row>
+    <row r="28" ht="90" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>C20</t>
         </is>
       </c>
-      <c r="B27" s="3" t="inlineStr">
+      <c r="B28" s="2" t="inlineStr">
         <is>
           <t>Primary-lab seat counting (formerly #12)</t>
         </is>
       </c>
-      <c r="C27" s="3" t="inlineStr"/>
-      <c r="D27" s="3" t="inlineStr"/>
-      <c r="E27" s="3" t="inlineStr"/>
-      <c r="F27" s="3" t="inlineStr">
+      <c r="C28" s="2" t="inlineStr"/>
+      <c r="D28" s="2" t="inlineStr"/>
+      <c r="E28" s="2" t="inlineStr"/>
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: is_primary_lab INTEGER NOT NULL DEFAULT 0
 column was added to the lab_members table at db.ts:1276, with the
@@ -2257,7 +2279,7 @@
 is_primary_lab=1 ordering).</t>
         </is>
       </c>
-      <c r="G27" s="3" t="inlineStr">
+      <c r="G28" s="2" t="inlineStr">
         <is>
           <t>2026-05-07 multi-lab discussion. Build shipped as part
 of the Multi-Lab Tier 2 architecture work (Phase 3.x series, prior
@@ -2266,23 +2288,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H27" s="3" t="inlineStr"/>
-    </row>
-    <row r="28" ht="90" customHeight="1">
-      <c r="A28" s="2" t="inlineStr">
+      <c r="H28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29" ht="90" customHeight="1">
+      <c r="A29" s="3" t="inlineStr">
         <is>
           <t>C21</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="B29" s="3" t="inlineStr">
         <is>
           <t>Multi-lab pricing model — Option A (formerly #11)</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr"/>
-      <c r="D28" s="2" t="inlineStr"/>
-      <c r="E28" s="2" t="inlineStr"/>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="C29" s="3" t="inlineStr"/>
+      <c r="D29" s="3" t="inlineStr"/>
+      <c r="E29" s="3" t="inlineStr"/>
+      <c r="F29" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #322 (commit 0ccd925, merged 2026-05-22)
 added the customer-facing line to the pricing page that reflects
@@ -2295,7 +2317,7 @@
 Enterprise+ block, reads:</t>
         </is>
       </c>
-      <c r="G28" s="2" t="inlineStr">
+      <c r="G29" s="3" t="inlineStr">
         <is>
           <t>2026-05-07 multi-lab discussion (Lisa Veri's
 canonical-case session). PR #322 (initial build); softening PR
@@ -2304,30 +2326,30 @@
 ---</t>
         </is>
       </c>
-      <c r="H28" s="2" t="inlineStr"/>
-    </row>
-    <row r="29" ht="90" customHeight="1">
-      <c r="A29" s="3" t="inlineStr">
+      <c r="H29" s="3" t="inlineStr"/>
+    </row>
+    <row r="30" ht="90" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>C22</t>
         </is>
       </c>
-      <c r="B29" s="3" t="inlineStr">
+      <c r="B30" s="2" t="inlineStr">
         <is>
           <t>VeritaOps cost-per-test module (formerly #10)</t>
         </is>
       </c>
-      <c r="C29" s="3" t="inlineStr"/>
-      <c r="D29" s="3" t="inlineStr"/>
-      <c r="E29" s="3" t="inlineStr"/>
-      <c r="F29" s="3" t="inlineStr">
+      <c r="C30" s="2" t="inlineStr"/>
+      <c r="D30" s="2" t="inlineStr"/>
+      <c r="E30" s="2" t="inlineStr"/>
+      <c r="F30" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: v1 of the VeritaOps Cost-Per-Reportable-Test
 (CPRT) module shipped across PR #325 through PR #330 on 2026-05-22.
 The module is feature-complete for the typical lab director workflow.</t>
         </is>
       </c>
-      <c r="G29" s="3" t="inlineStr">
+      <c r="G30" s="2" t="inlineStr">
         <is>
           <t>This thread, 2026-05-07 12:05 PM CDT, user message:
 "Parking lot: build an operations module for cost per test
@@ -2336,262 +2358,262 @@
 ---</t>
         </is>
       </c>
-      <c r="H29" s="3" t="inlineStr"/>
-    </row>
-    <row r="30" ht="90" customHeight="1">
-      <c r="A30" s="2" t="inlineStr">
+      <c r="H30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31" ht="90" customHeight="1">
+      <c r="A31" s="3" t="inlineStr">
         <is>
           <t>C23</t>
         </is>
       </c>
-      <c r="B30" s="2" t="inlineStr">
+      <c r="B31" s="3" t="inlineStr">
         <is>
           <t>CCL lab name visual disambiguation in lab switcher (formerly #34)</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr"/>
-      <c r="D30" s="2" t="inlineStr">
+      <c r="C31" s="3" t="inlineStr"/>
+      <c r="D31" s="3" t="inlineStr">
         <is>
           <t>XS (under 1 day, actual)</t>
         </is>
       </c>
-      <c r="E30" s="2" t="inlineStr">
+      <c r="E31" s="3" t="inlineStr">
         <is>
           <t>Low — cosmetic; only mattered when Lisa or Michael picked the wrong lab from...</t>
         </is>
       </c>
-      <c r="F30" s="2" t="inlineStr">
+      <c r="F31" s="3" t="inlineStr">
         <is>
           <t>Effort: XS (under 1 day, actual)
 Importance: Low — cosmetic; only mattered when Lisa or Michael picked the wrong lab from the dropdown.</t>
         </is>
       </c>
-      <c r="G30" s="2" t="inlineStr">
+      <c r="G31" s="3" t="inlineStr">
         <is>
           <t>flagged 2026-05-23 immediately after provisioning Lisa's CCL lab; closed 2026-05-24.
 ---</t>
         </is>
       </c>
-      <c r="H30" s="2" t="inlineStr"/>
-    </row>
-    <row r="31" ht="90" customHeight="1">
-      <c r="A31" s="3" t="inlineStr">
+      <c r="H31" s="3" t="inlineStr"/>
+    </row>
+    <row r="32" ht="90" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t>C24</t>
         </is>
       </c>
-      <c r="B31" s="3" t="inlineStr">
+      <c r="B32" s="2" t="inlineStr">
         <is>
           <t>VC Unlimited Y1/Y2 price disclosure UX (formerly #35)</t>
         </is>
       </c>
-      <c r="C31" s="3" t="inlineStr"/>
-      <c r="D31" s="3" t="inlineStr">
+      <c r="C32" s="2" t="inlineStr"/>
+      <c r="D32" s="2" t="inlineStr">
         <is>
           <t>XS (under 1 day, actual)</t>
         </is>
       </c>
-      <c r="E31" s="3" t="inlineStr">
+      <c r="E32" s="2" t="inlineStr">
         <is>
           <t>Low when shipped (proactive, no customer complaint yet) — but high if a procu...</t>
         </is>
       </c>
-      <c r="F31" s="3" t="inlineStr">
+      <c r="F32" s="2" t="inlineStr">
         <is>
           <t>Effort: XS (under 1 day, actual)
 Importance: Low when shipped (proactive, no customer complaint yet) — but high if a procurement reviewer later disputes the $499 renewal as undisclosed.</t>
         </is>
       </c>
-      <c r="G31" s="3" t="inlineStr">
+      <c r="G32" s="2" t="inlineStr">
         <is>
           <t>Pricing rebuild 2026-05-23; closed 2026-05-24 proactively before any customer dispute.
 ---</t>
         </is>
       </c>
-      <c r="H31" s="3" t="inlineStr"/>
-    </row>
-    <row r="32" ht="90" customHeight="1">
-      <c r="A32" s="2" t="inlineStr">
+      <c r="H32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33" ht="90" customHeight="1">
+      <c r="A33" s="3" t="inlineStr">
         <is>
           <t>C25</t>
         </is>
       </c>
-      <c r="B32" s="2" t="inlineStr">
+      <c r="B33" s="3" t="inlineStr">
         <is>
           <t>VeritaQC Phase 1 (Levey-Jennings + Westgard live engine) (formerly #20)</t>
         </is>
       </c>
-      <c r="C32" s="2" t="inlineStr"/>
-      <c r="D32" s="2" t="inlineStr">
+      <c r="C33" s="3" t="inlineStr"/>
+      <c r="D33" s="3" t="inlineStr">
         <is>
           <t>L (about 5 days end-to-end, actual: Phase 0 schema → Phase 1A evaluator → 1B...</t>
         </is>
       </c>
-      <c r="E32" s="2" t="inlineStr">
+      <c r="E33" s="3" t="inlineStr">
         <is>
           <t>High — largest single gap vs myLabCompliance.io per Perplexity competitor ana...</t>
         </is>
       </c>
-      <c r="F32" s="2" t="inlineStr">
+      <c r="F33" s="3" t="inlineStr">
         <is>
           <t>Effort: L (about 5 days end-to-end, actual: Phase 0 schema → Phase 1A evaluator → 1B entry UI → 1C daily review → 1D monthly PDF + attestation)
 Importance: High — largest single gap vs myLabCompliance.io per Perplexity competitor analysis; promotes VeritaAssure from documentation tool to lab operations platform.</t>
         </is>
       </c>
-      <c r="G32" s="2" t="inlineStr">
+      <c r="G33" s="3" t="inlineStr">
         <is>
           <t>Perplexity competitor analysis 2026-05-10. Scoping confirmed via the build_phase1_mockup.py iterations 2026-05-24. Shipped 2026-05-25.
 ---</t>
         </is>
       </c>
-      <c r="H32" s="2" t="inlineStr"/>
-    </row>
-    <row r="33" ht="90" customHeight="1">
-      <c r="A33" s="3" t="inlineStr">
+      <c r="H33" s="3" t="inlineStr"/>
+    </row>
+    <row r="34" ht="90" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
         <is>
           <t>C26</t>
         </is>
       </c>
-      <c r="B33" s="3" t="inlineStr">
+      <c r="B34" s="2" t="inlineStr">
         <is>
           <t>VeritaLab CMS-116 application support + state licensing registry (formerly #22)</t>
         </is>
       </c>
-      <c r="C33" s="3" t="inlineStr"/>
-      <c r="D33" s="3" t="inlineStr">
+      <c r="C34" s="2" t="inlineStr"/>
+      <c r="D34" s="2" t="inlineStr">
         <is>
           <t>M (1-2 weeks for v1, actual)</t>
         </is>
       </c>
-      <c r="E33" s="3" t="inlineStr">
+      <c r="E34" s="2" t="inlineStr">
         <is>
           <t>Medium — competitor parity (myLabCompliance.io) plus useful at lab startup an...</t>
         </is>
       </c>
-      <c r="F33" s="3" t="inlineStr">
+      <c r="F34" s="2" t="inlineStr">
         <is>
           <t>Effort: M (1-2 weeks for v1, actual)
 Importance: Medium — competitor parity (myLabCompliance.io) plus useful at lab startup and at certificate-type changes.</t>
         </is>
       </c>
-      <c r="G33" s="3" t="inlineStr">
+      <c r="G34" s="2" t="inlineStr">
         <is>
           <t>Perplexity competitor analysis (myLabCompliance.io), 2026-05-10. Reclassified as a VeritaLab extension 2026-05-25. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H33" s="3" t="inlineStr"/>
-    </row>
-    <row r="34" ht="90" customHeight="1">
-      <c r="A34" s="2" t="inlineStr">
+      <c r="H34" s="2" t="inlineStr"/>
+    </row>
+    <row r="35" ht="90" customHeight="1">
+      <c r="A35" s="3" t="inlineStr">
         <is>
           <t>C27</t>
         </is>
       </c>
-      <c r="B34" s="2" t="inlineStr">
+      <c r="B35" s="3" t="inlineStr">
         <is>
           <t>Active vs view-only seat split (formerly #33)</t>
         </is>
       </c>
-      <c r="C34" s="2" t="inlineStr"/>
-      <c r="D34" s="2" t="inlineStr">
+      <c r="C35" s="3" t="inlineStr"/>
+      <c r="D35" s="3" t="inlineStr">
         <is>
           <t>M (~1 week of engineering, actual: shipped in a single multi-PR session)</t>
         </is>
       </c>
-      <c r="E34" s="2" t="inlineStr">
+      <c r="E35" s="3" t="inlineStr">
         <is>
           <t>Medium — closed the gap between /pricing copy and product behavior; gives sal...</t>
         </is>
       </c>
-      <c r="F34" s="2" t="inlineStr">
+      <c r="F35" s="3" t="inlineStr">
         <is>
           <t>Effort: M (~1 week of engineering, actual: shipped in a single multi-PR session)
 Importance: Medium — closed the gap between /pricing copy and product behavior; gives sales a clean answer for "do you charge for our medical director?"</t>
         </is>
       </c>
-      <c r="G34" s="2" t="inlineStr">
+      <c r="G35" s="3" t="inlineStr">
         <is>
           <t>Pricing analysis doc Decision 3 (2026-05-21); MEDIUM scenario revised 2026-05-29 to retire the "unlimited view-only" claim. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H34" s="2" t="inlineStr"/>
-    </row>
-    <row r="35" ht="90" customHeight="1">
-      <c r="A35" s="3" t="inlineStr">
+      <c r="H35" s="3" t="inlineStr"/>
+    </row>
+    <row r="36" ht="90" customHeight="1">
+      <c r="A36" s="2" t="inlineStr">
         <is>
           <t>C28</t>
         </is>
       </c>
-      <c r="B35" s="3" t="inlineStr">
+      <c r="B36" s="2" t="inlineStr">
         <is>
           <t>"Why VeritaCheck" comparative one-pager (formerly #37)</t>
         </is>
       </c>
-      <c r="C35" s="3" t="inlineStr"/>
-      <c r="D35" s="3" t="inlineStr">
+      <c r="C36" s="2" t="inlineStr"/>
+      <c r="D36" s="2" t="inlineStr">
         <is>
           <t>S (one design pass + four claim paragraphs + PDF + matching marketing-site pa...</t>
         </is>
       </c>
-      <c r="E35" s="3" t="inlineStr">
+      <c r="E36" s="2" t="inlineStr">
         <is>
           <t>Medium — closed a positioning gap surfaced by six COLA conference attendees a...</t>
         </is>
       </c>
-      <c r="F35" s="3" t="inlineStr">
+      <c r="F36" s="2" t="inlineStr">
         <is>
           <t>Effort: S (one design pass + four claim paragraphs + PDF + matching marketing-site page, actual)
 Importance: Medium — closed a positioning gap surfaced by six COLA conference attendees attached to a legacy verification tool; converts product-quality advantage into a leave-behind Lisa can hand out.</t>
         </is>
       </c>
-      <c r="G35" s="3" t="inlineStr">
+      <c r="G36" s="2" t="inlineStr">
         <is>
           <t>2026-05-11 / 2026-05-12 conference notes review with Michael. Conference attendees (Whitehead, Odegard, Othman, Molinelli, Kyle, Allred) expressed interest in equivalent / superior product. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H35" s="3" t="inlineStr"/>
-    </row>
-    <row r="36" ht="90" customHeight="1">
-      <c r="A36" s="2" t="inlineStr">
+      <c r="H36" s="2" t="inlineStr"/>
+    </row>
+    <row r="37" ht="90" customHeight="1">
+      <c r="A37" s="3" t="inlineStr">
         <is>
           <t>C29</t>
         </is>
       </c>
-      <c r="B36" s="2" t="inlineStr">
+      <c r="B37" s="3" t="inlineStr">
         <is>
           <t>VeritaPolicy approval workflow — MediaLab functional mirror</t>
         </is>
       </c>
-      <c r="C36" s="2" t="inlineStr"/>
-      <c r="D36" s="2" t="inlineStr">
+      <c r="C37" s="3" t="inlineStr"/>
+      <c r="D37" s="3" t="inlineStr">
         <is>
           <t>XL (one focused session, 12 PRs landed)</t>
         </is>
       </c>
-      <c r="E36" s="2" t="inlineStr">
+      <c r="E37" s="3" t="inlineStr">
         <is>
           <t>High — replaces MediaLab Document Control ($752/$2,250 starting price, scalin...</t>
         </is>
       </c>
-      <c r="F36" s="2" t="inlineStr">
+      <c r="F37" s="3" t="inlineStr">
         <is>
           <t>Effort: XL (one focused session, 12 PRs landed)
 Importance: High — replaces MediaLab Document Control ($752/$2,250 starting price, scaling to $10K-$20K/yr at enterprise per Capterra public data) with an included VeritaPolicy feature; closes a real positioning gap and gives sales a direct comparator line.</t>
         </is>
       </c>
-      <c r="G36" s="2" t="inlineStr">
+      <c r="G37" s="3" t="inlineStr">
         <is>
           <t>Pricing strategy conversation 2026-05-29 (Michael: "I don't like bolt-ons; we should replicate this") → scoped 8 phases → shipped all 12 PRs in single session. Shipped 2026-05-29.
 ---</t>
         </is>
       </c>
-      <c r="H36" s="2" t="inlineStr"/>
+      <c r="H37" s="3" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H36"/>
+  <autoFilter ref="A1:H37"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
TASK: Parking-lot sync (2026-09-24) - close #43,#44,#45,#46 (done/verified) and add #48 (shipped) as CLOSED.
PLAN:
  1. Move #43 (already fixed), #44 (already fixed), #45 (shipped), #46 (PR #1312) from OPEN to CLOSED as C36-C39.
  2. Add #48 (PR #1314, VeritaComp competencies owed + gap detection) as C40 with live-verify evidence.
  3. Regenerate PARKING_LOT.xlsx via build_parking_lot_xlsx.py; keep #47 open (needs scope confirmation).

Self-check:
  - OPEN 19 -> 15 (four moved); CLOSED +5 (four moved + #48 net-new) = 40; RETIRED unchanged.
  - Closure evidence cites commit/PR + live verification for each; #43/#44 note they were verified already-fixed, not re-coded.
  - #47 intentionally left OPEN.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PARKING_LOT.xlsx
+++ b/PARKING_LOT.xlsx
@@ -12,8 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RETIRED" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$20</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$41</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RETIRED'!$A$1:$H$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1175,203 +1175,45 @@
     <row r="16" ht="90" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>47</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>License stamp clobbers the §6 lab-identity header/footer and can name the wrong lab</t>
+          <t>Hide sections a lab does not use from a master list, to reduce clutter (prospect-requested)</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Parked by operator decision 2026-07-16 ("log it, finish PR 4 first"). Not started. No code touched.
+          <t>Open. Not started. Needs a one-line scope confirmation (which master list).
 ---</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>S-M (one shared helper plus a verify script; 8 callsites to re-check)</t>
+          <t>S-M (a few days to ~2 weeks depending on scope) — a lab-level visibility togg...</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Medium-High. Every customer-facing workbook currently prints a header and foo...</t>
+          <t>Medium-High — came straight from a live prospect today as an onboarding-frict...</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>licenseCtxFromReq (server/routes.ts:57-61) resolves the licensee lab from resolveActiveLabForRequest, which reads the X-Active-Lab-Id header and silently falls back to the user's default lab inside a bare catch {}. The export body meanwhile resolves the lab from req.scope.labId (the URL path param, set by labScopeMiddleware). Two sources of truth for one document. Separately and unconditionally, applyLicenseToExcelJSWorkbook (shared/licenseExceljs.ts:93-96) *assigns* rather than merges oddHeader/oddFooter on every sheet, so the six lines in the VeritaMap export that carefully set ${labName} CLIA: ${cliaNumber} (routes.ts:13932-13933, 14215-14216, 14224-14225) are dead code, overwritten at routes.ts:14237. §6 rule 3 exists so identity survives cell-level copy-paste; layers (b) and (c) do not currently exist in any shipped workbook.</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-16 session, PR 4 (#1046) Gate 3 render. Related: feedback_pdf_lab_identity_resolution memory (same resolveActiveLabForRequest swallowed-throw shape).</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr"/>
-    </row>
-    <row r="17" ht="90" customHeight="1">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>44</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>Long Excel column headers are clipped, truncating CFR citations mid-string</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>Parked by operator decision 2026-07-16. Not started. No code touched.
----</t>
-        </is>
-      </c>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>S (compute the header row height from the longest wrapped header, or raise th...</t>
-        </is>
-      </c>
-      <c r="E17" s="3" t="inlineStr">
-        <is>
-          <t>Medium. The VeritaMap workbook currently prints "Reference Range Attestation...</t>
-        </is>
-      </c>
-      <c r="F17" s="3" t="inlineStr">
-        <is>
-          <t>CLAUDE.md §6 specifies both "row height 20" for the header row and "wrap text" for cells. Those two rules conflict for any header longer than its column width. Row height 20 renders roughly one line of Calibri 11, so a header that wraps to two or three lines has its tail clipped in print and in PDF export. Confirmed on the live VeritaMap Compliance Map export: header row height is 20.0 with wrapText: true, and the three longest headers are "AMR Attestation (42 CFR 493.1253, per instrument)" (49 chars), "Reference Range Attestation (42 CFR 493.1253)" (45), and "Last Correlation / Method Comparison Date" (41). "Last SOP Review Date" and "AMR High (per instrument)" clip too.</t>
-        </is>
-      </c>
-      <c r="G17" s="3" t="inlineStr">
-        <is>
-          <t>2026-07-16 session, PR 4 (#1046) Gate 3 render. Sibling of [[#43]]; both were found by looking at the rendered workbook, and neither was catchable by the verify scripts.</t>
-        </is>
-      </c>
-      <c r="H17" s="3" t="inlineStr"/>
-    </row>
-    <row r="18" ht="90" customHeight="1">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>45</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>VeritaTrack calendar month cells are not expandable, so hidden tasks are unreachable</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>Open. Not started.
----</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>S (1-3 days) — make each month cell open a detail view or expand in place, an...</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>High — a compliance calendar that hides tasks with no way to see them undercu...</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>Effort: S (1-3 days) — make each month cell open a detail view or expand in place, and wire the "+N more" affordance to reveal the full task list. The data is already loaded, this is a UI interaction gap, not a data one.
-Importance: High — a compliance calendar that hides tasks with no way to see them undercuts the module's core promise of showing what a lab owes and when.</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-23 session, Michael screenshot of the VeritaTrack calendar (lab 3, September cell).</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="inlineStr"/>
-    </row>
-    <row r="19" ht="90" customHeight="1">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>46</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>VeritaScan line items cannot attach or link evidence (policy or uploaded document)</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>Open. Not started.
----</t>
-        </is>
-      </c>
-      <c r="D19" s="3" t="inlineStr">
-        <is>
-          <t>M (1-2 weeks) — add a per-item evidence link that reuses the VeritaScan URL-p...</t>
-        </is>
-      </c>
-      <c r="E19" s="3" t="inlineStr">
-        <is>
-          <t>High — showing evidence per line item is the whole point of a self-inspection...</t>
-        </is>
-      </c>
-      <c r="F19" s="3" t="inlineStr">
-        <is>
-          <t>Effort: M (1-2 weeks) — add a per-item evidence link that reuses the VeritaScan URL-pointer model rather than storing files: let a line item reference an existing VeritaDC controlled document or an external URL, then surface it as completion evidence.
-Importance: High — showing evidence per line item is the whole point of a self-inspection; without it the scan records a status but cannot show the policy or document that satisfies it.</t>
-        </is>
-      </c>
-      <c r="G19" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-23 session, Michael. Recurring request.</t>
-        </is>
-      </c>
-      <c r="H19" s="3" t="inlineStr"/>
-    </row>
-    <row r="20" ht="90" customHeight="1">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>47</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>Hide sections a lab does not use from a master list, to reduce clutter (prospect-requested)</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>Open. Not started. Needs a one-line scope confirmation (which master list).
----</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>S-M (a few days to ~2 weeks depending on scope) — a lab-level visibility togg...</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>Medium-High — came straight from a live prospect today as an onboarding-frict...</t>
-        </is>
-      </c>
-      <c r="F20" s="2" t="inlineStr">
         <is>
           <t>Effort: S-M (a few days to ~2 weeks depending on scope) — a lab-level visibility toggle that hides not-applicable or unused sections from a master-list view. Smaller if it is a "hide N/A" filter on the existing VeritaDC master list, larger if it also spans VeritaScan domains.
 Importance: Medium-High — came straight from a live prospect today as an onboarding-friction point; a lab that does not run a service line should not have to wade past its requirements.</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>2026-09-23 session, Michael relaying a prospect ask from a demo today.</t>
         </is>
       </c>
-      <c r="H20" s="2" t="inlineStr"/>
+      <c r="H16" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H20"/>
+  <autoFilter ref="A1:H16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1382,7 +1224,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H36"/>
+  <dimension ref="A1:H41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1440,18 +1282,153 @@
     <row r="2" ht="90" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>C34</t>
+          <t>C40</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Wire the two static-audit guards into CI (was #43)</t>
+          <t>VeritaComp Competencies Owed derived from VeritaStaff, with gap detection (was #48)</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr"/>
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Closure evidence: PR #1314 (squash 2bcb0db9). GET /api/labs/:labId/competency/owed derives each VeritaStaff testing employee's owed competencies from their assigned instruments (staff_employee_instruments -&gt; veritamap_instruments + tests), on the CLIA timeline, and flags instruments not covered by any competency program as gaps. CompetenciesOwedSection renders it on the VeritaComp landing page. Reuses the shipped bridge + suggested-method-groups match rules; no new tables. Verified live on prod with real assignment data: 2 instruments assigned to a demo staffer produced owed=2, gaps=2 (HIGH, Technical Supervisor), then reverted cleanly. Closed 2026-09-24.</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23/24 session, Michael ("veritacomp bases what competencies they owe (currently untrue, but needs to be true)"). Option 1 (unify roster on VeritaStaff, match instruments by id).
+---</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3" ht="90" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>C39</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>VeritaScan line items can attach or link evidence (was #46)</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr"/>
+      <c r="D3" s="3" t="inlineStr"/>
+      <c r="E3" s="3" t="inlineStr"/>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Closure evidence: PR #1312 (squash a1dda93d). VeritaScan scan checklist items now show linked evidence as chips (open link, remove) plus a writer "Link evidence" affordance whose picker links an existing VeritaDC/Library document; a shortcut deep-links to the Library for new (governed) documents. Reuses the already-shipped lab_documents + document_checklist_links + coverage endpoints (URL-pointer only, no file storage, no new tables). Browser-verified live on prod (scan 23): the affordance renders and the picker opens. Closed 2026-09-24.</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-23 session, Michael. Recurring request. Companion: cross-module evidence display on the VeritaDC policy shipped in PR #1313 (by-target cross-links surfaced in the policy View modal, browser-verified live).
+---</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr"/>
+    </row>
+    <row r="4" ht="90" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>C38</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>VeritaTrack calendar month cells expand to reveal hidden tasks (was #45)</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr"/>
+      <c r="D4" s="2" t="inlineStr"/>
+      <c r="E4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Closure evidence: VeritaTrack CalendarView month cells with more than three tasks now expand in place (chevron, "+N more" toggling to "Show less", due dates), so no task is hidden with no path to it (client/src/pages/VeritaTrackAppPage.tsx CalendarView). Shipped 2026-09-23. Closed 2026-09-24.</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23 session, Michael screenshot of the VeritaTrack calendar (lab 3, September cell).
+---</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5" ht="90" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>C37</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Long Excel column headers no longer clip CFR citations (was #44)</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr"/>
+      <c r="D5" s="3" t="inlineStr"/>
+      <c r="E5" s="3" t="inlineStr"/>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. The VeritaMap export derives the header row height from the longest wrapped header via headerRowHeight(headers, colWidths) (server/routes.ts:15935) instead of a fixed 20, so "Reference Range Attestation (42 CFR 493.1253)" and the other long headers print in full. No new code this session. Closed 2026-09-24.</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+---</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr"/>
+    </row>
+    <row r="6" ht="90" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>C36</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>License stamp no longer clobbers the §6 header/footer or names the wrong lab (was #43)</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr"/>
+      <c r="D6" s="2" t="inlineStr"/>
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. setHeaderFooter (shared/licenseExceljs.ts:155-209) now preserves an existing §6 header and appends (not overwrites) the footer left section, and customer-facing exports name the scoped lab: the VeritaScan library export reads req.scope.lab.name / clia_number (server/routes.ts:16572-16573), not the licensee. No new code this session (avoided regressing the existing fix). Closed 2026-09-24.</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+---</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7" ht="90" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>C34</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Wire the two static-audit guards into CI (was #43)</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr"/>
+      <c r="D7" s="3" t="inlineStr"/>
+      <c r="E7" s="3" t="inlineStr"/>
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: both guards wired into the Multi-Lab Mutations Audit CI
 workflow (.github/workflows/multilab-mutations-audit.yml) as steps:
@@ -1463,24 +1440,24 @@
 (same caveat as the existing guards already in that workflow).</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr"/>
-    </row>
-    <row r="3" ht="90" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="G7" s="3" t="inlineStr"/>
+      <c r="H7" s="3" t="inlineStr"/>
+    </row>
+    <row r="8" ht="90" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>C35</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>Legacy /api/studies over-returns studies across labs (was #44)</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr"/>
-      <c r="D3" s="3" t="inlineStr"/>
-      <c r="E3" s="3" t="inlineStr"/>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr"/>
+      <c r="D8" s="2" t="inlineStr"/>
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: GET /api/studies now scopes its list to the active lab
 when one is resolved from the Referer (server/routes.ts), so every returned row
@@ -1490,24 +1467,24 @@
 mirroring the /api/labs/:labId/studies handler. Closed 2026-06-14.</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr"/>
-      <c r="H3" s="3" t="inlineStr"/>
-    </row>
-    <row r="4" ht="90" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9" ht="90" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>C30</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>Verify-script convention backfill (was #41)</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr"/>
-      <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="2" t="inlineStr"/>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr"/>
+      <c r="D9" s="3" t="inlineStr"/>
+      <c r="E9" s="3" t="inlineStr"/>
+      <c r="F9" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: all 8 high-stakes math/logic commits now ship a paired
 scripts/verify-*.js (EP17 sensitivity, Deming lot-to-lot, CUMSUM+QC+multi-analyte,
@@ -1515,30 +1492,30 @@
 TEa boundary), per the strike-throughs in #41. Closed 2026-06-13.</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G9" s="3" t="inlineStr">
         <is>
           <t>scripts/audit_verify_script_coverage.py lookback, 2026-06-02; backfills
 landed 2026-06-03..06.
 ---</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr"/>
-    </row>
-    <row r="5" ht="90" customHeight="1">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="H9" s="3" t="inlineStr"/>
+    </row>
+    <row r="10" ht="90" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>C31</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>VeritaPT AAA create/update/delete silently no-op in the multi-lab UI</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr"/>
-      <c r="D5" s="3" t="inlineStr"/>
-      <c r="E5" s="3" t="inlineStr"/>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr"/>
+      <c r="D10" s="2" t="inlineStr"/>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #754 (commit 92ad499) added lab-scoped POST/PUT/DELETE
 /api/labs/:labId/pt/aa-records. The UI posted to the lab-scoped path but only GET
@@ -1549,30 +1526,30 @@
 route mis-filed records to the user's default lab on multi-lab accounts).</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>2026-06-13, found during #18 Phase 3 QA;
 scripts/audit-labscoped-write-routes.mjs now guards the class.
 ---</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr"/>
-    </row>
-    <row r="6" ht="90" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11" ht="90" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>C32</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>VeritaComp "Unlock assessment" false-success no-op</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr"/>
-      <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr"/>
+      <c r="D11" s="3" t="inlineStr"/>
+      <c r="E11" s="3" t="inlineStr"/>
+      <c r="F11" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #755 (commit 4234007) moved the unlock route to
 /api/labs/:labId/competency/assessments/:id/unlock (the path the client calls).
@@ -1583,29 +1560,29 @@
 HTML).</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G11" s="3" t="inlineStr">
         <is>
           <t>2026-06-13, found by scripts/audit-labscoped-write-routes.mjs.
 ---</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr"/>
-    </row>
-    <row r="7" ht="90" customHeight="1">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="H11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12" ht="90" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>C33</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>FK-cascade delete 500s + NavBar laptop-width overflow</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr"/>
-      <c r="D7" s="3" t="inlineStr"/>
-      <c r="E7" s="3" t="inlineStr"/>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr"/>
+      <c r="D12" s="2" t="inlineStr"/>
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PRs #749/#750 fixed NavBar horizontal overflow at laptop
 widths (collapse to the hamburger below 1560px); prod-verified at 1280-1920 with the
@@ -1616,57 +1593,57 @@
 500 -&gt; 200. scripts/audit-delete-cascades.mjs guards the class.</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>2026-06-13 browser QA of the A7-D4 wave + retro-QC of the 72h PR window.
 ---</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr"/>
-    </row>
-    <row r="8" ht="90" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13" ht="90" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>C1</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>FAQ "over 25 years" -&gt; "over 23 years"</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr"/>
-      <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr"/>
+      <c r="D13" s="3" t="inlineStr"/>
+      <c r="E13" s="3" t="inlineStr"/>
+      <c r="F13" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: client/src/pages/FAQPage.tsx line 20 reads "over
 23 years" as of 2026-05-01.</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G13" s="3" t="inlineStr">
         <is>
           <t>session 299e9a73 turn 14, ~2026-04-28.
 ---</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr"/>
-    </row>
-    <row r="9" ht="90" customHeight="1">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="H13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14" ht="90" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>C5</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>David's VeritaQA grey-button bug (seat permissions mode)</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr"/>
-      <c r="D9" s="3" t="inlineStr"/>
-      <c r="E9" s="3" t="inlineStr"/>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr"/>
+      <c r="D14" s="2" t="inlineStr"/>
+      <c r="E14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #10 squash-merged as commit a43fbba on
 2026-05-01 23:19 MST. Railway deploy succeeded; deployed bundle
@@ -1679,7 +1656,7 @@
 against his exact stored shape (14 of 14 expected outcomes matched).</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>2026-05-01 David's report; veritabench + veritastock
 weren't in MODULE_LIST so seat permissions silently defaulted to
@@ -1687,109 +1664,109 @@
 ---</t>
         </is>
       </c>
-      <c r="H9" s="3" t="inlineStr"/>
-    </row>
-    <row r="10" ht="90" customHeight="1">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="H14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15" ht="90" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>C2</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>TeamPage present-tense "TJC surveyor" check</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr"/>
-      <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr"/>
+      <c r="D15" s="3" t="inlineStr"/>
+      <c r="E15" s="3" t="inlineStr"/>
+      <c r="F15" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: site-wide search confirmed all surveyor language
 is past-tense, consistent with user's 2021-2025 service. User closed
 the item in session 299e9a73 turn 4.</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G15" s="3" t="inlineStr">
         <is>
           <t>session 299e9a73, ~2026-04-28.
 ---</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr"/>
-    </row>
-    <row r="11" ht="90" customHeight="1">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="H15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16" ht="90" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>C3</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>My Studies CSV/XLSX export (John as design partner)</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr"/>
-      <c r="D11" s="3" t="inlineStr"/>
-      <c r="E11" s="3" t="inlineStr"/>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr"/>
+      <c r="D16" s="2" t="inlineStr"/>
+      <c r="E16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: client/src/pages/DashboardPage.tsx line 46 calls
 /api/my-studies/export. server/routes.ts line 1491 implements the
 endpoint. Pulled forward into pre-COLA per user instruction.</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>session 299e9a73 turn 5, ~2026-04-28.
 ---</t>
         </is>
       </c>
-      <c r="H11" s="3" t="inlineStr"/>
-    </row>
-    <row r="12" ht="90" customHeight="1">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="H16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17" ht="90" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>C4</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>Rotate GitHub PAT (because old PAT was committed in SESSION_HANDOFF files)</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr"/>
-      <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="2" t="inlineStr"/>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr"/>
+      <c r="D17" s="3" t="inlineStr"/>
+      <c r="E17" s="3" t="inlineStr"/>
+      <c r="F17" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: no ghp_* or github_pat_* patterns in current
 SESSION_HANDOFF.md or SESSION_HANDOFF-2.md as of 2026-05-01.</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G17" s="3" t="inlineStr">
         <is>
           <t>session 299e9a73, ~2026-04-28.
 ---</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr"/>
-    </row>
-    <row r="13" ht="90" customHeight="1">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="H17" s="3" t="inlineStr"/>
+    </row>
+    <row r="18" ht="90" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>C6</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>VeritaPolicy service-line filtering removed (formerly #4)</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr"/>
-      <c r="D13" s="3" t="inlineStr"/>
-      <c r="E13" s="3" t="inlineStr"/>
-      <c r="F13" s="3" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr"/>
+      <c r="D18" s="2" t="inlineStr"/>
+      <c r="E18" s="2" t="inlineStr"/>
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>Closure rationale (operator decision 2026-05-10): Keep all
 VeritaPolicy rows. CFR-only references with no accreditor reference
@@ -1798,29 +1775,29 @@
 report misread the design intent.</t>
         </is>
       </c>
-      <c r="G13" s="3" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H13" s="3" t="inlineStr"/>
-    </row>
-    <row r="14" ht="90" customHeight="1">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19" ht="90" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>C7</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>CLIA number format validation (formerly #13)</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr"/>
-      <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="2" t="inlineStr"/>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="C19" s="3" t="inlineStr"/>
+      <c r="D19" s="3" t="inlineStr"/>
+      <c r="E19" s="3" t="inlineStr"/>
+      <c r="F19" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: shared/validateClia.ts defines CLIA_REGEX =
 /^\d{2}D\d{7}$/ (line 24), validateClia() helper with whitespace
@@ -1831,30 +1808,30 @@
 shape exists and behaves as specified.</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="G19" s="3" t="inlineStr">
         <is>
           <t>Agent verification 2026-05-10 via grep + file read.
 Operator confirmed shipped 2026-05-10.
 ---</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr"/>
-    </row>
-    <row r="15" ht="90" customHeight="1">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="H19" s="3" t="inlineStr"/>
+    </row>
+    <row r="20" ht="90" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>C8</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>VeritaMap lab-wide menu toggle (formerly #19)</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr"/>
-      <c r="D15" s="3" t="inlineStr"/>
-      <c r="E15" s="3" t="inlineStr"/>
-      <c r="F15" s="3" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr"/>
+      <c r="D20" s="2" t="inlineStr"/>
+      <c r="E20" s="2" t="inlineStr"/>
+      <c r="F20" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: client/src/pages/VeritaMapLabwidePage.tsx
 exists and implements the labwide read-only union view. Route is
@@ -1864,59 +1841,59 @@
 parking lot plan (read-only union view, per-session toggle) shipped.</t>
         </is>
       </c>
-      <c r="G15" s="3" t="inlineStr">
+      <c r="G20" s="2" t="inlineStr">
         <is>
           <t>Agent verification 2026-05-10 via grep + file read.
 Operator confirmed shipped 2026-05-10.
 ---</t>
         </is>
       </c>
-      <c r="H15" s="3" t="inlineStr"/>
-    </row>
-    <row r="16" ht="90" customHeight="1">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="H20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21" ht="90" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>C9</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>Tier-1 smoke test checklist (formerly #6)</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr"/>
-      <c r="D16" s="2" t="inlineStr"/>
-      <c r="E16" s="2" t="inlineStr"/>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="C21" s="3" t="inlineStr"/>
+      <c r="D21" s="3" t="inlineStr"/>
+      <c r="E21" s="3" t="inlineStr"/>
+      <c r="F21" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: docs/smoke-test-tier1.md documents the Tier-1
 smoke-test process and post-deploy verification steps. Shipped via
 PR #81 as part of the 2026-05-10 wave.</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="G21" s="3" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr"/>
-    </row>
-    <row r="17" ht="90" customHeight="1">
-      <c r="A17" s="3" t="inlineStr">
+      <c r="H21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22" ht="90" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>C10</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B22" s="2" t="inlineStr">
         <is>
           <t>Per-module gating (formerly #7)</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr"/>
-      <c r="D17" s="3" t="inlineStr"/>
-      <c r="E17" s="3" t="inlineStr"/>
-      <c r="F17" s="3" t="inlineStr">
+      <c r="C22" s="2" t="inlineStr"/>
+      <c r="D22" s="2" t="inlineStr"/>
+      <c r="E22" s="2" t="inlineStr"/>
+      <c r="F22" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: Client-side useIsReadOnly module keys wired
 on client/src/pages/VeritaPolicyAppPage.tsx and
@@ -1931,29 +1908,29 @@
 PR #76.</t>
         </is>
       </c>
-      <c r="G17" s="3" t="inlineStr">
+      <c r="G22" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H17" s="3" t="inlineStr"/>
-    </row>
-    <row r="18" ht="90" customHeight="1">
-      <c r="A18" s="2" t="inlineStr">
+      <c r="H22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23" ht="90" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>C11</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>VeritaStock shipped copy (formerly #8)</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr"/>
-      <c r="D18" s="2" t="inlineStr"/>
-      <c r="E18" s="2" t="inlineStr"/>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="C23" s="3" t="inlineStr"/>
+      <c r="D23" s="3" t="inlineStr"/>
+      <c r="E23" s="3" t="inlineStr"/>
+      <c r="F23" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: client/src/pages/ArticleInventoryManagementPage.tsx
 line 305 footer reads "platform that includes VeritaStock™" instead
@@ -1961,29 +1938,29 @@
 on /resources/laboratory-inventory-management. Shipped via PR #75.</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="G23" s="3" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H18" s="2" t="inlineStr"/>
-    </row>
-    <row r="19" ht="90" customHeight="1">
-      <c r="A19" s="3" t="inlineStr">
+      <c r="H23" s="3" t="inlineStr"/>
+    </row>
+    <row r="24" ht="90" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>C12</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>Admin report one-row-per-lab (formerly #14)</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr"/>
-      <c r="D19" s="3" t="inlineStr"/>
-      <c r="E19" s="3" t="inlineStr"/>
-      <c r="F19" s="3" t="inlineStr">
+      <c r="C24" s="2" t="inlineStr"/>
+      <c r="D24" s="2" t="inlineStr"/>
+      <c r="E24" s="2" t="inlineStr"/>
+      <c r="F24" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: /api/admin/report rewritten in
 server/routes.ts (~line 595) to LEFT JOIN labs on
@@ -1998,56 +1975,56 @@
 prerequisite, not a code bug). Shipped via PR #85.</t>
         </is>
       </c>
-      <c r="G19" s="3" t="inlineStr">
+      <c r="G24" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H19" s="3" t="inlineStr"/>
-    </row>
-    <row r="20" ht="90" customHeight="1">
-      <c r="A20" s="2" t="inlineStr">
+      <c r="H24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25" ht="90" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
         <is>
           <t>C14</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>UI relabel "CLIA TEa" -&gt; "Lab-Set Internal Goal" (formerly #1)</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr"/>
-      <c r="D20" s="2" t="inlineStr"/>
-      <c r="E20" s="2" t="inlineStr"/>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="C25" s="3" t="inlineStr"/>
+      <c r="D25" s="3" t="inlineStr"/>
+      <c r="E25" s="3" t="inlineStr"/>
+      <c r="F25" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: Shipped across four PRs over 2026-05-10.</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr">
+      <c r="G25" s="3" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H20" s="2" t="inlineStr"/>
-    </row>
-    <row r="21" ht="90" customHeight="1">
-      <c r="A21" s="3" t="inlineStr">
+      <c r="H25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26" ht="90" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>C13</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t>WSLH PT vendor (formerly #15)</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr"/>
-      <c r="D21" s="3" t="inlineStr"/>
-      <c r="E21" s="3" t="inlineStr"/>
-      <c r="F21" s="3" t="inlineStr">
+      <c r="C26" s="2" t="inlineStr"/>
+      <c r="D26" s="2" t="inlineStr"/>
+      <c r="E26" s="2" t="inlineStr"/>
+      <c r="F26" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: Shipped 2026-05-10 via PR #79 (merge commit
 eeebc6e; merged after rebase to resolve a server/db.ts collision
@@ -2065,64 +2042,64 @@
 'WSLH' is the post-deploy success signal. Shipped via PR #79.</t>
         </is>
       </c>
-      <c r="G21" s="3" t="inlineStr">
+      <c r="G26" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H21" s="3" t="inlineStr"/>
-    </row>
-    <row r="22" ht="90" customHeight="1">
-      <c r="A22" s="2" t="inlineStr">
+      <c r="H26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27" ht="90" customHeight="1">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>C15</t>
         </is>
       </c>
-      <c r="B22" s="2" t="inlineStr">
+      <c r="B27" s="3" t="inlineStr">
         <is>
           <t>VeritaStock lot tracking + expiration + reorder alerts (formerly #21)</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr"/>
-      <c r="D22" s="2" t="inlineStr"/>
-      <c r="E22" s="2" t="inlineStr"/>
-      <c r="F22" s="2" t="inlineStr">
+      <c r="C27" s="3" t="inlineStr"/>
+      <c r="D27" s="3" t="inlineStr"/>
+      <c r="E27" s="3" t="inlineStr"/>
+      <c r="F27" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: VeritaStock™ shipped the bench-level inventory
 features the Perplexity competitor analysis identified as a gap:</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr">
+      <c r="G27" s="3" t="inlineStr">
         <is>
           <t>Originally Perplexity competitor analysis 2026-05-10.
 Audit 2026-05-21 confirmed the feature set ships today.
 ---</t>
         </is>
       </c>
-      <c r="H22" s="2" t="inlineStr"/>
-    </row>
-    <row r="23" ht="90" customHeight="1">
-      <c r="A23" s="3" t="inlineStr">
+      <c r="H27" s="3" t="inlineStr"/>
+    </row>
+    <row r="28" ht="90" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>C16</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="B28" s="2" t="inlineStr">
         <is>
           <t>PAL studies guided workflow (formerly #23)</t>
         </is>
       </c>
-      <c r="C23" s="3" t="inlineStr"/>
-      <c r="D23" s="3" t="inlineStr"/>
-      <c r="E23" s="3" t="inlineStr"/>
-      <c r="F23" s="3" t="inlineStr">
+      <c r="C28" s="2" t="inlineStr"/>
+      <c r="D28" s="2" t="inlineStr"/>
+      <c r="E28" s="2" t="inlineStr"/>
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: VeritaCheck™ already ships the Precision /
 Accuracy / Linearity (PAL) study set under EP-protocol naming:</t>
         </is>
       </c>
-      <c r="G23" s="3" t="inlineStr">
+      <c r="G28" s="2" t="inlineStr">
         <is>
           <t>Originally Perplexity competitor analysis 2026-05-10.
 Audit 2026-05-21 confirmed the EP studies cover the PAL framing in
@@ -2130,23 +2107,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H23" s="3" t="inlineStr"/>
-    </row>
-    <row r="24" ht="90" customHeight="1">
-      <c r="A24" s="2" t="inlineStr">
+      <c r="H28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29" ht="90" customHeight="1">
+      <c r="A29" s="3" t="inlineStr">
         <is>
           <t>C17</t>
         </is>
       </c>
-      <c r="B24" s="2" t="inlineStr">
+      <c r="B29" s="3" t="inlineStr">
         <is>
           <t>Source-grounded 21/29/45 CFR + 42 CFR 482-485 (formerly #26)</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr"/>
-      <c r="D24" s="2" t="inlineStr"/>
-      <c r="E24" s="2" t="inlineStr"/>
-      <c r="F24" s="2" t="inlineStr">
+      <c r="C29" s="3" t="inlineStr"/>
+      <c r="D29" s="3" t="inlineStr"/>
+      <c r="E29" s="3" t="inlineStr"/>
+      <c r="F29" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #301 (commit 8c27806, merged 2026-05-21)
 source-grounded the 74 remaining non-493 entries in
@@ -2154,29 +2131,29 @@
 shipped:</t>
         </is>
       </c>
-      <c r="G24" s="2" t="inlineStr">
+      <c r="G29" s="3" t="inlineStr">
         <is>
           <t>PR #301; tasks #18 in the in-session task tracker.
 ---</t>
         </is>
       </c>
-      <c r="H24" s="2" t="inlineStr"/>
-    </row>
-    <row r="25" ht="90" customHeight="1">
-      <c r="A25" s="3" t="inlineStr">
+      <c r="H29" s="3" t="inlineStr"/>
+    </row>
+    <row r="30" ht="90" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>C18</t>
         </is>
       </c>
-      <c r="B25" s="3" t="inlineStr">
+      <c r="B30" s="2" t="inlineStr">
         <is>
           <t>VeritaPolicy "Non CLIA" chapter rename (formerly #3)</t>
         </is>
       </c>
-      <c r="C25" s="3" t="inlineStr"/>
-      <c r="D25" s="3" t="inlineStr"/>
-      <c r="E25" s="3" t="inlineStr"/>
-      <c r="F25" s="3" t="inlineStr">
+      <c r="C30" s="2" t="inlineStr"/>
+      <c r="D30" s="2" t="inlineStr"/>
+      <c r="E30" s="2" t="inlineStr"/>
+      <c r="F30" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #300 (commit 34d7707, merged 2026-05-21)
 renamed all 44 user-facing chapter labels in
@@ -2187,7 +2164,7 @@
 page.</t>
         </is>
       </c>
-      <c r="G25" s="3" t="inlineStr">
+      <c r="G30" s="2" t="inlineStr">
         <is>
           <t>CAP customer screenshot of the /veritapolicy chapter
 headers, 2026-05-01 evening. PR #300; tasks #17 in the in-session
@@ -2195,23 +2172,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H25" s="3" t="inlineStr"/>
-    </row>
-    <row r="26" ht="90" customHeight="1">
-      <c r="A26" s="2" t="inlineStr">
+      <c r="H30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31" ht="90" customHeight="1">
+      <c r="A31" s="3" t="inlineStr">
         <is>
           <t>C19</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="B31" s="3" t="inlineStr">
         <is>
           <t>VeritaStock department-scope toggle (formerly #31)</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr"/>
-      <c r="D26" s="2" t="inlineStr"/>
-      <c r="E26" s="2" t="inlineStr"/>
-      <c r="F26" s="2" t="inlineStr">
+      <c r="C31" s="3" t="inlineStr"/>
+      <c r="D31" s="3" t="inlineStr"/>
+      <c r="E31" s="3" t="inlineStr"/>
+      <c r="F31" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #319 (commit d01f5fe, merged 2026-05-22)
 shipped the persistent dept-scope toggle on VeritaStockPage. A new
@@ -2222,7 +2199,7 @@
 workspace without re-filtering.</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr">
+      <c r="G31" s="3" t="inlineStr">
         <is>
           <t>John, San Carlos lab, 2026-05-21. Same conversation that
 drove the vendor dropdown (PR #304), FILTERED VIEW banner (PR #305),
@@ -2230,23 +2207,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H26" s="2" t="inlineStr"/>
-    </row>
-    <row r="27" ht="90" customHeight="1">
-      <c r="A27" s="3" t="inlineStr">
+      <c r="H31" s="3" t="inlineStr"/>
+    </row>
+    <row r="32" ht="90" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t>C20</t>
         </is>
       </c>
-      <c r="B27" s="3" t="inlineStr">
+      <c r="B32" s="2" t="inlineStr">
         <is>
           <t>Primary-lab seat counting (formerly #12)</t>
         </is>
       </c>
-      <c r="C27" s="3" t="inlineStr"/>
-      <c r="D27" s="3" t="inlineStr"/>
-      <c r="E27" s="3" t="inlineStr"/>
-      <c r="F27" s="3" t="inlineStr">
+      <c r="C32" s="2" t="inlineStr"/>
+      <c r="D32" s="2" t="inlineStr"/>
+      <c r="E32" s="2" t="inlineStr"/>
+      <c r="F32" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: is_primary_lab INTEGER NOT NULL DEFAULT 0
 column was added to the lab_members table at db.ts:1276, with the
@@ -2257,7 +2234,7 @@
 is_primary_lab=1 ordering).</t>
         </is>
       </c>
-      <c r="G27" s="3" t="inlineStr">
+      <c r="G32" s="2" t="inlineStr">
         <is>
           <t>2026-05-07 multi-lab discussion. Build shipped as part
 of the Multi-Lab Tier 2 architecture work (Phase 3.x series, prior
@@ -2266,23 +2243,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H27" s="3" t="inlineStr"/>
-    </row>
-    <row r="28" ht="90" customHeight="1">
-      <c r="A28" s="2" t="inlineStr">
+      <c r="H32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33" ht="90" customHeight="1">
+      <c r="A33" s="3" t="inlineStr">
         <is>
           <t>C21</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="B33" s="3" t="inlineStr">
         <is>
           <t>Multi-lab pricing model — Option A (formerly #11)</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr"/>
-      <c r="D28" s="2" t="inlineStr"/>
-      <c r="E28" s="2" t="inlineStr"/>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="C33" s="3" t="inlineStr"/>
+      <c r="D33" s="3" t="inlineStr"/>
+      <c r="E33" s="3" t="inlineStr"/>
+      <c r="F33" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #322 (commit 0ccd925, merged 2026-05-22)
 added the customer-facing line to the pricing page that reflects
@@ -2295,7 +2272,7 @@
 Enterprise+ block, reads:</t>
         </is>
       </c>
-      <c r="G28" s="2" t="inlineStr">
+      <c r="G33" s="3" t="inlineStr">
         <is>
           <t>2026-05-07 multi-lab discussion (Lisa Veri's
 canonical-case session). PR #322 (initial build); softening PR
@@ -2304,30 +2281,30 @@
 ---</t>
         </is>
       </c>
-      <c r="H28" s="2" t="inlineStr"/>
-    </row>
-    <row r="29" ht="90" customHeight="1">
-      <c r="A29" s="3" t="inlineStr">
+      <c r="H33" s="3" t="inlineStr"/>
+    </row>
+    <row r="34" ht="90" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
         <is>
           <t>C22</t>
         </is>
       </c>
-      <c r="B29" s="3" t="inlineStr">
+      <c r="B34" s="2" t="inlineStr">
         <is>
           <t>VeritaOps cost-per-test module (formerly #10)</t>
         </is>
       </c>
-      <c r="C29" s="3" t="inlineStr"/>
-      <c r="D29" s="3" t="inlineStr"/>
-      <c r="E29" s="3" t="inlineStr"/>
-      <c r="F29" s="3" t="inlineStr">
+      <c r="C34" s="2" t="inlineStr"/>
+      <c r="D34" s="2" t="inlineStr"/>
+      <c r="E34" s="2" t="inlineStr"/>
+      <c r="F34" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: v1 of the VeritaOps Cost-Per-Reportable-Test
 (CPRT) module shipped across PR #325 through PR #330 on 2026-05-22.
 The module is feature-complete for the typical lab director workflow.</t>
         </is>
       </c>
-      <c r="G29" s="3" t="inlineStr">
+      <c r="G34" s="2" t="inlineStr">
         <is>
           <t>This thread, 2026-05-07 12:05 PM CDT, user message:
 "Parking lot: build an operations module for cost per test
@@ -2336,262 +2313,262 @@
 ---</t>
         </is>
       </c>
-      <c r="H29" s="3" t="inlineStr"/>
-    </row>
-    <row r="30" ht="90" customHeight="1">
-      <c r="A30" s="2" t="inlineStr">
+      <c r="H34" s="2" t="inlineStr"/>
+    </row>
+    <row r="35" ht="90" customHeight="1">
+      <c r="A35" s="3" t="inlineStr">
         <is>
           <t>C23</t>
         </is>
       </c>
-      <c r="B30" s="2" t="inlineStr">
+      <c r="B35" s="3" t="inlineStr">
         <is>
           <t>CCL lab name visual disambiguation in lab switcher (formerly #34)</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr"/>
-      <c r="D30" s="2" t="inlineStr">
+      <c r="C35" s="3" t="inlineStr"/>
+      <c r="D35" s="3" t="inlineStr">
         <is>
           <t>XS (under 1 day, actual)</t>
         </is>
       </c>
-      <c r="E30" s="2" t="inlineStr">
+      <c r="E35" s="3" t="inlineStr">
         <is>
           <t>Low — cosmetic; only mattered when Lisa or Michael picked the wrong lab from...</t>
         </is>
       </c>
-      <c r="F30" s="2" t="inlineStr">
+      <c r="F35" s="3" t="inlineStr">
         <is>
           <t>Effort: XS (under 1 day, actual)
 Importance: Low — cosmetic; only mattered when Lisa or Michael picked the wrong lab from the dropdown.</t>
         </is>
       </c>
-      <c r="G30" s="2" t="inlineStr">
+      <c r="G35" s="3" t="inlineStr">
         <is>
           <t>flagged 2026-05-23 immediately after provisioning Lisa's CCL lab; closed 2026-05-24.
 ---</t>
         </is>
       </c>
-      <c r="H30" s="2" t="inlineStr"/>
-    </row>
-    <row r="31" ht="90" customHeight="1">
-      <c r="A31" s="3" t="inlineStr">
+      <c r="H35" s="3" t="inlineStr"/>
+    </row>
+    <row r="36" ht="90" customHeight="1">
+      <c r="A36" s="2" t="inlineStr">
         <is>
           <t>C24</t>
         </is>
       </c>
-      <c r="B31" s="3" t="inlineStr">
+      <c r="B36" s="2" t="inlineStr">
         <is>
           <t>VC Unlimited Y1/Y2 price disclosure UX (formerly #35)</t>
         </is>
       </c>
-      <c r="C31" s="3" t="inlineStr"/>
-      <c r="D31" s="3" t="inlineStr">
+      <c r="C36" s="2" t="inlineStr"/>
+      <c r="D36" s="2" t="inlineStr">
         <is>
           <t>XS (under 1 day, actual)</t>
         </is>
       </c>
-      <c r="E31" s="3" t="inlineStr">
+      <c r="E36" s="2" t="inlineStr">
         <is>
           <t>Low when shipped (proactive, no customer complaint yet) — but high if a procu...</t>
         </is>
       </c>
-      <c r="F31" s="3" t="inlineStr">
+      <c r="F36" s="2" t="inlineStr">
         <is>
           <t>Effort: XS (under 1 day, actual)
 Importance: Low when shipped (proactive, no customer complaint yet) — but high if a procurement reviewer later disputes the $499 renewal as undisclosed.</t>
         </is>
       </c>
-      <c r="G31" s="3" t="inlineStr">
+      <c r="G36" s="2" t="inlineStr">
         <is>
           <t>Pricing rebuild 2026-05-23; closed 2026-05-24 proactively before any customer dispute.
 ---</t>
         </is>
       </c>
-      <c r="H31" s="3" t="inlineStr"/>
-    </row>
-    <row r="32" ht="90" customHeight="1">
-      <c r="A32" s="2" t="inlineStr">
+      <c r="H36" s="2" t="inlineStr"/>
+    </row>
+    <row r="37" ht="90" customHeight="1">
+      <c r="A37" s="3" t="inlineStr">
         <is>
           <t>C25</t>
         </is>
       </c>
-      <c r="B32" s="2" t="inlineStr">
+      <c r="B37" s="3" t="inlineStr">
         <is>
           <t>VeritaQC Phase 1 (Levey-Jennings + Westgard live engine) (formerly #20)</t>
         </is>
       </c>
-      <c r="C32" s="2" t="inlineStr"/>
-      <c r="D32" s="2" t="inlineStr">
+      <c r="C37" s="3" t="inlineStr"/>
+      <c r="D37" s="3" t="inlineStr">
         <is>
           <t>L (about 5 days end-to-end, actual: Phase 0 schema → Phase 1A evaluator → 1B...</t>
         </is>
       </c>
-      <c r="E32" s="2" t="inlineStr">
+      <c r="E37" s="3" t="inlineStr">
         <is>
           <t>High — largest single gap vs myLabCompliance.io per Perplexity competitor ana...</t>
         </is>
       </c>
-      <c r="F32" s="2" t="inlineStr">
+      <c r="F37" s="3" t="inlineStr">
         <is>
           <t>Effort: L (about 5 days end-to-end, actual: Phase 0 schema → Phase 1A evaluator → 1B entry UI → 1C daily review → 1D monthly PDF + attestation)
 Importance: High — largest single gap vs myLabCompliance.io per Perplexity competitor analysis; promotes VeritaAssure from documentation tool to lab operations platform.</t>
         </is>
       </c>
-      <c r="G32" s="2" t="inlineStr">
+      <c r="G37" s="3" t="inlineStr">
         <is>
           <t>Perplexity competitor analysis 2026-05-10. Scoping confirmed via the build_phase1_mockup.py iterations 2026-05-24. Shipped 2026-05-25.
 ---</t>
         </is>
       </c>
-      <c r="H32" s="2" t="inlineStr"/>
-    </row>
-    <row r="33" ht="90" customHeight="1">
-      <c r="A33" s="3" t="inlineStr">
+      <c r="H37" s="3" t="inlineStr"/>
+    </row>
+    <row r="38" ht="90" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
         <is>
           <t>C26</t>
         </is>
       </c>
-      <c r="B33" s="3" t="inlineStr">
+      <c r="B38" s="2" t="inlineStr">
         <is>
           <t>VeritaLab CMS-116 application support + state licensing registry (formerly #22)</t>
         </is>
       </c>
-      <c r="C33" s="3" t="inlineStr"/>
-      <c r="D33" s="3" t="inlineStr">
+      <c r="C38" s="2" t="inlineStr"/>
+      <c r="D38" s="2" t="inlineStr">
         <is>
           <t>M (1-2 weeks for v1, actual)</t>
         </is>
       </c>
-      <c r="E33" s="3" t="inlineStr">
+      <c r="E38" s="2" t="inlineStr">
         <is>
           <t>Medium — competitor parity (myLabCompliance.io) plus useful at lab startup an...</t>
         </is>
       </c>
-      <c r="F33" s="3" t="inlineStr">
+      <c r="F38" s="2" t="inlineStr">
         <is>
           <t>Effort: M (1-2 weeks for v1, actual)
 Importance: Medium — competitor parity (myLabCompliance.io) plus useful at lab startup and at certificate-type changes.</t>
         </is>
       </c>
-      <c r="G33" s="3" t="inlineStr">
+      <c r="G38" s="2" t="inlineStr">
         <is>
           <t>Perplexity competitor analysis (myLabCompliance.io), 2026-05-10. Reclassified as a VeritaLab extension 2026-05-25. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H33" s="3" t="inlineStr"/>
-    </row>
-    <row r="34" ht="90" customHeight="1">
-      <c r="A34" s="2" t="inlineStr">
+      <c r="H38" s="2" t="inlineStr"/>
+    </row>
+    <row r="39" ht="90" customHeight="1">
+      <c r="A39" s="3" t="inlineStr">
         <is>
           <t>C27</t>
         </is>
       </c>
-      <c r="B34" s="2" t="inlineStr">
+      <c r="B39" s="3" t="inlineStr">
         <is>
           <t>Active vs view-only seat split (formerly #33)</t>
         </is>
       </c>
-      <c r="C34" s="2" t="inlineStr"/>
-      <c r="D34" s="2" t="inlineStr">
+      <c r="C39" s="3" t="inlineStr"/>
+      <c r="D39" s="3" t="inlineStr">
         <is>
           <t>M (~1 week of engineering, actual: shipped in a single multi-PR session)</t>
         </is>
       </c>
-      <c r="E34" s="2" t="inlineStr">
+      <c r="E39" s="3" t="inlineStr">
         <is>
           <t>Medium — closed the gap between /pricing copy and product behavior; gives sal...</t>
         </is>
       </c>
-      <c r="F34" s="2" t="inlineStr">
+      <c r="F39" s="3" t="inlineStr">
         <is>
           <t>Effort: M (~1 week of engineering, actual: shipped in a single multi-PR session)
 Importance: Medium — closed the gap between /pricing copy and product behavior; gives sales a clean answer for "do you charge for our medical director?"</t>
         </is>
       </c>
-      <c r="G34" s="2" t="inlineStr">
+      <c r="G39" s="3" t="inlineStr">
         <is>
           <t>Pricing analysis doc Decision 3 (2026-05-21); MEDIUM scenario revised 2026-05-29 to retire the "unlimited view-only" claim. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H34" s="2" t="inlineStr"/>
-    </row>
-    <row r="35" ht="90" customHeight="1">
-      <c r="A35" s="3" t="inlineStr">
+      <c r="H39" s="3" t="inlineStr"/>
+    </row>
+    <row r="40" ht="90" customHeight="1">
+      <c r="A40" s="2" t="inlineStr">
         <is>
           <t>C28</t>
         </is>
       </c>
-      <c r="B35" s="3" t="inlineStr">
+      <c r="B40" s="2" t="inlineStr">
         <is>
           <t>"Why VeritaCheck" comparative one-pager (formerly #37)</t>
         </is>
       </c>
-      <c r="C35" s="3" t="inlineStr"/>
-      <c r="D35" s="3" t="inlineStr">
+      <c r="C40" s="2" t="inlineStr"/>
+      <c r="D40" s="2" t="inlineStr">
         <is>
           <t>S (one design pass + four claim paragraphs + PDF + matching marketing-site pa...</t>
         </is>
       </c>
-      <c r="E35" s="3" t="inlineStr">
+      <c r="E40" s="2" t="inlineStr">
         <is>
           <t>Medium — closed a positioning gap surfaced by six COLA conference attendees a...</t>
         </is>
       </c>
-      <c r="F35" s="3" t="inlineStr">
+      <c r="F40" s="2" t="inlineStr">
         <is>
           <t>Effort: S (one design pass + four claim paragraphs + PDF + matching marketing-site page, actual)
 Importance: Medium — closed a positioning gap surfaced by six COLA conference attendees attached to a legacy verification tool; converts product-quality advantage into a leave-behind Lisa can hand out.</t>
         </is>
       </c>
-      <c r="G35" s="3" t="inlineStr">
+      <c r="G40" s="2" t="inlineStr">
         <is>
           <t>2026-05-11 / 2026-05-12 conference notes review with Michael. Conference attendees (Whitehead, Odegard, Othman, Molinelli, Kyle, Allred) expressed interest in equivalent / superior product. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H35" s="3" t="inlineStr"/>
-    </row>
-    <row r="36" ht="90" customHeight="1">
-      <c r="A36" s="2" t="inlineStr">
+      <c r="H40" s="2" t="inlineStr"/>
+    </row>
+    <row r="41" ht="90" customHeight="1">
+      <c r="A41" s="3" t="inlineStr">
         <is>
           <t>C29</t>
         </is>
       </c>
-      <c r="B36" s="2" t="inlineStr">
+      <c r="B41" s="3" t="inlineStr">
         <is>
           <t>VeritaPolicy approval workflow — MediaLab functional mirror</t>
         </is>
       </c>
-      <c r="C36" s="2" t="inlineStr"/>
-      <c r="D36" s="2" t="inlineStr">
+      <c r="C41" s="3" t="inlineStr"/>
+      <c r="D41" s="3" t="inlineStr">
         <is>
           <t>XL (one focused session, 12 PRs landed)</t>
         </is>
       </c>
-      <c r="E36" s="2" t="inlineStr">
+      <c r="E41" s="3" t="inlineStr">
         <is>
           <t>High — replaces MediaLab Document Control ($752/$2,250 starting price, scalin...</t>
         </is>
       </c>
-      <c r="F36" s="2" t="inlineStr">
+      <c r="F41" s="3" t="inlineStr">
         <is>
           <t>Effort: XL (one focused session, 12 PRs landed)
 Importance: High — replaces MediaLab Document Control ($752/$2,250 starting price, scaling to $10K-$20K/yr at enterprise per Capterra public data) with an included VeritaPolicy feature; closes a real positioning gap and gives sales a direct comparator line.</t>
         </is>
       </c>
-      <c r="G36" s="2" t="inlineStr">
+      <c r="G41" s="3" t="inlineStr">
         <is>
           <t>Pricing strategy conversation 2026-05-29 (Michael: "I don't like bolt-ons; we should replicate this") → scoped 8 phases → shipped all 12 PRs in single session. Shipped 2026-05-29.
 ---</t>
         </is>
       </c>
-      <c r="H36" s="2" t="inlineStr"/>
+      <c r="H41" s="3" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H36"/>
+  <autoFilter ref="A1:H41"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
TASK: Parking-lot sync 2026-09-24 (close #43/#44/#45/#46, add #48 as C40)
PLAN:
  1. Move #43,#44 (verified already-fixed), #45 (shipped), #46 (PR #1312) OPEN->CLOSED as C36-C39.
  2. Add #48 (PR #1314) as C40 with live-verify evidence.
  3. Regenerate PARKING_LOT.xlsx; keep #47 OPEN; supersede #1311.

Self-check:
  - OPEN 19->15; CLOSED->40; RETIRED 6.
  - #43/#44 noted verified-fixed, not re-coded.
  - #1311 closed as superseded.
</commit_message>
<xml_diff>
--- a/PARKING_LOT.xlsx
+++ b/PARKING_LOT.xlsx
@@ -12,8 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RETIRED" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$20</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$41</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RETIRED'!$A$1:$H$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1175,203 +1175,45 @@
     <row r="16" ht="90" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>47</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>License stamp clobbers the §6 lab-identity header/footer and can name the wrong lab</t>
+          <t>Hide sections a lab does not use from a master list, to reduce clutter (prospect-requested)</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Parked by operator decision 2026-07-16 ("log it, finish PR 4 first"). Not started. No code touched.
+          <t>Open. Not started. Needs a one-line scope confirmation (which master list).
 ---</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>S-M (one shared helper plus a verify script; 8 callsites to re-check)</t>
+          <t>S-M (a few days to ~2 weeks depending on scope) — a lab-level visibility togg...</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Medium-High. Every customer-facing workbook currently prints a header and foo...</t>
+          <t>Medium-High — came straight from a live prospect today as an onboarding-frict...</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>licenseCtxFromReq (server/routes.ts:57-61) resolves the licensee lab from resolveActiveLabForRequest, which reads the X-Active-Lab-Id header and silently falls back to the user's default lab inside a bare catch {}. The export body meanwhile resolves the lab from req.scope.labId (the URL path param, set by labScopeMiddleware). Two sources of truth for one document. Separately and unconditionally, applyLicenseToExcelJSWorkbook (shared/licenseExceljs.ts:93-96) *assigns* rather than merges oddHeader/oddFooter on every sheet, so the six lines in the VeritaMap export that carefully set ${labName} CLIA: ${cliaNumber} (routes.ts:13932-13933, 14215-14216, 14224-14225) are dead code, overwritten at routes.ts:14237. §6 rule 3 exists so identity survives cell-level copy-paste; layers (b) and (c) do not currently exist in any shipped workbook.</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-16 session, PR 4 (#1046) Gate 3 render. Related: feedback_pdf_lab_identity_resolution memory (same resolveActiveLabForRequest swallowed-throw shape).</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr"/>
-    </row>
-    <row r="17" ht="90" customHeight="1">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>44</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>Long Excel column headers are clipped, truncating CFR citations mid-string</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>Parked by operator decision 2026-07-16. Not started. No code touched.
----</t>
-        </is>
-      </c>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>S (compute the header row height from the longest wrapped header, or raise th...</t>
-        </is>
-      </c>
-      <c r="E17" s="3" t="inlineStr">
-        <is>
-          <t>Medium. The VeritaMap workbook currently prints "Reference Range Attestation...</t>
-        </is>
-      </c>
-      <c r="F17" s="3" t="inlineStr">
-        <is>
-          <t>CLAUDE.md §6 specifies both "row height 20" for the header row and "wrap text" for cells. Those two rules conflict for any header longer than its column width. Row height 20 renders roughly one line of Calibri 11, so a header that wraps to two or three lines has its tail clipped in print and in PDF export. Confirmed on the live VeritaMap Compliance Map export: header row height is 20.0 with wrapText: true, and the three longest headers are "AMR Attestation (42 CFR 493.1253, per instrument)" (49 chars), "Reference Range Attestation (42 CFR 493.1253)" (45), and "Last Correlation / Method Comparison Date" (41). "Last SOP Review Date" and "AMR High (per instrument)" clip too.</t>
-        </is>
-      </c>
-      <c r="G17" s="3" t="inlineStr">
-        <is>
-          <t>2026-07-16 session, PR 4 (#1046) Gate 3 render. Sibling of [[#43]]; both were found by looking at the rendered workbook, and neither was catchable by the verify scripts.</t>
-        </is>
-      </c>
-      <c r="H17" s="3" t="inlineStr"/>
-    </row>
-    <row r="18" ht="90" customHeight="1">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>45</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>VeritaTrack calendar month cells are not expandable, so hidden tasks are unreachable</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>Open. Not started.
----</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>S (1-3 days) — make each month cell open a detail view or expand in place, an...</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>High — a compliance calendar that hides tasks with no way to see them undercu...</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>Effort: S (1-3 days) — make each month cell open a detail view or expand in place, and wire the "+N more" affordance to reveal the full task list. The data is already loaded, this is a UI interaction gap, not a data one.
-Importance: High — a compliance calendar that hides tasks with no way to see them undercuts the module's core promise of showing what a lab owes and when.</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-23 session, Michael screenshot of the VeritaTrack calendar (lab 3, September cell).</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="inlineStr"/>
-    </row>
-    <row r="19" ht="90" customHeight="1">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>46</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>VeritaScan line items cannot attach or link evidence (policy or uploaded document)</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>Open. Not started.
----</t>
-        </is>
-      </c>
-      <c r="D19" s="3" t="inlineStr">
-        <is>
-          <t>M (1-2 weeks) — add a per-item evidence link that reuses the VeritaScan URL-p...</t>
-        </is>
-      </c>
-      <c r="E19" s="3" t="inlineStr">
-        <is>
-          <t>High — showing evidence per line item is the whole point of a self-inspection...</t>
-        </is>
-      </c>
-      <c r="F19" s="3" t="inlineStr">
-        <is>
-          <t>Effort: M (1-2 weeks) — add a per-item evidence link that reuses the VeritaScan URL-pointer model rather than storing files: let a line item reference an existing VeritaDC controlled document or an external URL, then surface it as completion evidence.
-Importance: High — showing evidence per line item is the whole point of a self-inspection; without it the scan records a status but cannot show the policy or document that satisfies it.</t>
-        </is>
-      </c>
-      <c r="G19" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-23 session, Michael. Recurring request.</t>
-        </is>
-      </c>
-      <c r="H19" s="3" t="inlineStr"/>
-    </row>
-    <row r="20" ht="90" customHeight="1">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>47</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>Hide sections a lab does not use from a master list, to reduce clutter (prospect-requested)</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>Open. Not started. Needs a one-line scope confirmation (which master list).
----</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>S-M (a few days to ~2 weeks depending on scope) — a lab-level visibility togg...</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>Medium-High — came straight from a live prospect today as an onboarding-frict...</t>
-        </is>
-      </c>
-      <c r="F20" s="2" t="inlineStr">
         <is>
           <t>Effort: S-M (a few days to ~2 weeks depending on scope) — a lab-level visibility toggle that hides not-applicable or unused sections from a master-list view. Smaller if it is a "hide N/A" filter on the existing VeritaDC master list, larger if it also spans VeritaScan domains.
 Importance: Medium-High — came straight from a live prospect today as an onboarding-friction point; a lab that does not run a service line should not have to wade past its requirements.</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>2026-09-23 session, Michael relaying a prospect ask from a demo today.</t>
         </is>
       </c>
-      <c r="H20" s="2" t="inlineStr"/>
+      <c r="H16" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H20"/>
+  <autoFilter ref="A1:H16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1382,7 +1224,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H36"/>
+  <dimension ref="A1:H41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1440,18 +1282,153 @@
     <row r="2" ht="90" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>C34</t>
+          <t>C40</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Wire the two static-audit guards into CI (was #43)</t>
+          <t>VeritaComp Competencies Owed derived from VeritaStaff, with gap detection (was #48)</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr"/>
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Closure evidence: PR #1314 (squash 2bcb0db9). GET /api/labs/:labId/competency/owed derives each VeritaStaff testing employee's owed competencies from their assigned instruments (staff_employee_instruments -&gt; veritamap_instruments + tests), on the CLIA timeline, and flags instruments not covered by any competency program as gaps. CompetenciesOwedSection renders it on the VeritaComp landing page. Reuses the shipped bridge + suggested-method-groups match rules; no new tables. Verified live on prod with real assignment data: 2 instruments assigned to a demo staffer produced owed=2, gaps=2 (HIGH, Technical Supervisor), then reverted cleanly. Closed 2026-09-24.</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23/24 session, Michael ("veritacomp bases what competencies they owe (currently untrue, but needs to be true)"). Option 1 (unify roster on VeritaStaff, match instruments by id).
+---</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3" ht="90" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>C39</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>VeritaScan line items can attach or link evidence (was #46)</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr"/>
+      <c r="D3" s="3" t="inlineStr"/>
+      <c r="E3" s="3" t="inlineStr"/>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Closure evidence: PR #1312 (squash a1dda93d). VeritaScan scan checklist items now show linked evidence as chips (open link, remove) plus a writer "Link evidence" affordance whose picker links an existing VeritaDC/Library document; a shortcut deep-links to the Library for new (governed) documents. Reuses the already-shipped lab_documents + document_checklist_links + coverage endpoints (URL-pointer only, no file storage, no new tables). Browser-verified live on prod (scan 23): the affordance renders and the picker opens. Closed 2026-09-24.</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-23 session, Michael. Recurring request. Companion: cross-module evidence display on the VeritaDC policy shipped in PR #1313 (by-target cross-links surfaced in the policy View modal, browser-verified live).
+---</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr"/>
+    </row>
+    <row r="4" ht="90" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>C38</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>VeritaTrack calendar month cells expand to reveal hidden tasks (was #45)</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr"/>
+      <c r="D4" s="2" t="inlineStr"/>
+      <c r="E4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Closure evidence: VeritaTrack CalendarView month cells with more than three tasks now expand in place (chevron, "+N more" toggling to "Show less", due dates), so no task is hidden with no path to it (client/src/pages/VeritaTrackAppPage.tsx CalendarView). Shipped 2026-09-23. Closed 2026-09-24.</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23 session, Michael screenshot of the VeritaTrack calendar (lab 3, September cell).
+---</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5" ht="90" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>C37</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Long Excel column headers no longer clip CFR citations (was #44)</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr"/>
+      <c r="D5" s="3" t="inlineStr"/>
+      <c r="E5" s="3" t="inlineStr"/>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. The VeritaMap export derives the header row height from the longest wrapped header via headerRowHeight(headers, colWidths) (server/routes.ts:15935) instead of a fixed 20, so "Reference Range Attestation (42 CFR 493.1253)" and the other long headers print in full. No new code this session. Closed 2026-09-24.</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+---</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr"/>
+    </row>
+    <row r="6" ht="90" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>C36</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>License stamp no longer clobbers the §6 header/footer or names the wrong lab (was #43)</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr"/>
+      <c r="D6" s="2" t="inlineStr"/>
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. setHeaderFooter (shared/licenseExceljs.ts:155-209) now preserves an existing §6 header and appends (not overwrites) the footer left section, and customer-facing exports name the scoped lab: the VeritaScan library export reads req.scope.lab.name / clia_number (server/routes.ts:16572-16573), not the licensee. No new code this session (avoided regressing the existing fix). Closed 2026-09-24.</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+---</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7" ht="90" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>C34</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Wire the two static-audit guards into CI (was #43)</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr"/>
+      <c r="D7" s="3" t="inlineStr"/>
+      <c r="E7" s="3" t="inlineStr"/>
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: both guards wired into the Multi-Lab Mutations Audit CI
 workflow (.github/workflows/multilab-mutations-audit.yml) as steps:
@@ -1463,24 +1440,24 @@
 (same caveat as the existing guards already in that workflow).</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr"/>
-    </row>
-    <row r="3" ht="90" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="G7" s="3" t="inlineStr"/>
+      <c r="H7" s="3" t="inlineStr"/>
+    </row>
+    <row r="8" ht="90" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>C35</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>Legacy /api/studies over-returns studies across labs (was #44)</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr"/>
-      <c r="D3" s="3" t="inlineStr"/>
-      <c r="E3" s="3" t="inlineStr"/>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr"/>
+      <c r="D8" s="2" t="inlineStr"/>
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: GET /api/studies now scopes its list to the active lab
 when one is resolved from the Referer (server/routes.ts), so every returned row
@@ -1490,24 +1467,24 @@
 mirroring the /api/labs/:labId/studies handler. Closed 2026-06-14.</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr"/>
-      <c r="H3" s="3" t="inlineStr"/>
-    </row>
-    <row r="4" ht="90" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9" ht="90" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>C30</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>Verify-script convention backfill (was #41)</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr"/>
-      <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="2" t="inlineStr"/>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr"/>
+      <c r="D9" s="3" t="inlineStr"/>
+      <c r="E9" s="3" t="inlineStr"/>
+      <c r="F9" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: all 8 high-stakes math/logic commits now ship a paired
 scripts/verify-*.js (EP17 sensitivity, Deming lot-to-lot, CUMSUM+QC+multi-analyte,
@@ -1515,30 +1492,30 @@
 TEa boundary), per the strike-throughs in #41. Closed 2026-06-13.</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G9" s="3" t="inlineStr">
         <is>
           <t>scripts/audit_verify_script_coverage.py lookback, 2026-06-02; backfills
 landed 2026-06-03..06.
 ---</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr"/>
-    </row>
-    <row r="5" ht="90" customHeight="1">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="H9" s="3" t="inlineStr"/>
+    </row>
+    <row r="10" ht="90" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>C31</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>VeritaPT AAA create/update/delete silently no-op in the multi-lab UI</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr"/>
-      <c r="D5" s="3" t="inlineStr"/>
-      <c r="E5" s="3" t="inlineStr"/>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr"/>
+      <c r="D10" s="2" t="inlineStr"/>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #754 (commit 92ad499) added lab-scoped POST/PUT/DELETE
 /api/labs/:labId/pt/aa-records. The UI posted to the lab-scoped path but only GET
@@ -1549,30 +1526,30 @@
 route mis-filed records to the user's default lab on multi-lab accounts).</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>2026-06-13, found during #18 Phase 3 QA;
 scripts/audit-labscoped-write-routes.mjs now guards the class.
 ---</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr"/>
-    </row>
-    <row r="6" ht="90" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11" ht="90" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>C32</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>VeritaComp "Unlock assessment" false-success no-op</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr"/>
-      <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr"/>
+      <c r="D11" s="3" t="inlineStr"/>
+      <c r="E11" s="3" t="inlineStr"/>
+      <c r="F11" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #755 (commit 4234007) moved the unlock route to
 /api/labs/:labId/competency/assessments/:id/unlock (the path the client calls).
@@ -1583,29 +1560,29 @@
 HTML).</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G11" s="3" t="inlineStr">
         <is>
           <t>2026-06-13, found by scripts/audit-labscoped-write-routes.mjs.
 ---</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr"/>
-    </row>
-    <row r="7" ht="90" customHeight="1">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="H11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12" ht="90" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>C33</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>FK-cascade delete 500s + NavBar laptop-width overflow</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr"/>
-      <c r="D7" s="3" t="inlineStr"/>
-      <c r="E7" s="3" t="inlineStr"/>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr"/>
+      <c r="D12" s="2" t="inlineStr"/>
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PRs #749/#750 fixed NavBar horizontal overflow at laptop
 widths (collapse to the hamburger below 1560px); prod-verified at 1280-1920 with the
@@ -1616,57 +1593,57 @@
 500 -&gt; 200. scripts/audit-delete-cascades.mjs guards the class.</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>2026-06-13 browser QA of the A7-D4 wave + retro-QC of the 72h PR window.
 ---</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr"/>
-    </row>
-    <row r="8" ht="90" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13" ht="90" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>C1</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>FAQ "over 25 years" -&gt; "over 23 years"</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr"/>
-      <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr"/>
+      <c r="D13" s="3" t="inlineStr"/>
+      <c r="E13" s="3" t="inlineStr"/>
+      <c r="F13" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: client/src/pages/FAQPage.tsx line 20 reads "over
 23 years" as of 2026-05-01.</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G13" s="3" t="inlineStr">
         <is>
           <t>session 299e9a73 turn 14, ~2026-04-28.
 ---</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr"/>
-    </row>
-    <row r="9" ht="90" customHeight="1">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="H13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14" ht="90" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>C5</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>David's VeritaQA grey-button bug (seat permissions mode)</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr"/>
-      <c r="D9" s="3" t="inlineStr"/>
-      <c r="E9" s="3" t="inlineStr"/>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr"/>
+      <c r="D14" s="2" t="inlineStr"/>
+      <c r="E14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #10 squash-merged as commit a43fbba on
 2026-05-01 23:19 MST. Railway deploy succeeded; deployed bundle
@@ -1679,7 +1656,7 @@
 against his exact stored shape (14 of 14 expected outcomes matched).</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>2026-05-01 David's report; veritabench + veritastock
 weren't in MODULE_LIST so seat permissions silently defaulted to
@@ -1687,109 +1664,109 @@
 ---</t>
         </is>
       </c>
-      <c r="H9" s="3" t="inlineStr"/>
-    </row>
-    <row r="10" ht="90" customHeight="1">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="H14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15" ht="90" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>C2</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>TeamPage present-tense "TJC surveyor" check</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr"/>
-      <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr"/>
+      <c r="D15" s="3" t="inlineStr"/>
+      <c r="E15" s="3" t="inlineStr"/>
+      <c r="F15" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: site-wide search confirmed all surveyor language
 is past-tense, consistent with user's 2021-2025 service. User closed
 the item in session 299e9a73 turn 4.</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G15" s="3" t="inlineStr">
         <is>
           <t>session 299e9a73, ~2026-04-28.
 ---</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr"/>
-    </row>
-    <row r="11" ht="90" customHeight="1">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="H15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16" ht="90" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>C3</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>My Studies CSV/XLSX export (John as design partner)</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr"/>
-      <c r="D11" s="3" t="inlineStr"/>
-      <c r="E11" s="3" t="inlineStr"/>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr"/>
+      <c r="D16" s="2" t="inlineStr"/>
+      <c r="E16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: client/src/pages/DashboardPage.tsx line 46 calls
 /api/my-studies/export. server/routes.ts line 1491 implements the
 endpoint. Pulled forward into pre-COLA per user instruction.</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>session 299e9a73 turn 5, ~2026-04-28.
 ---</t>
         </is>
       </c>
-      <c r="H11" s="3" t="inlineStr"/>
-    </row>
-    <row r="12" ht="90" customHeight="1">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="H16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17" ht="90" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>C4</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>Rotate GitHub PAT (because old PAT was committed in SESSION_HANDOFF files)</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr"/>
-      <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="2" t="inlineStr"/>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr"/>
+      <c r="D17" s="3" t="inlineStr"/>
+      <c r="E17" s="3" t="inlineStr"/>
+      <c r="F17" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: no ghp_* or github_pat_* patterns in current
 SESSION_HANDOFF.md or SESSION_HANDOFF-2.md as of 2026-05-01.</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G17" s="3" t="inlineStr">
         <is>
           <t>session 299e9a73, ~2026-04-28.
 ---</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr"/>
-    </row>
-    <row r="13" ht="90" customHeight="1">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="H17" s="3" t="inlineStr"/>
+    </row>
+    <row r="18" ht="90" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>C6</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>VeritaPolicy service-line filtering removed (formerly #4)</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr"/>
-      <c r="D13" s="3" t="inlineStr"/>
-      <c r="E13" s="3" t="inlineStr"/>
-      <c r="F13" s="3" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr"/>
+      <c r="D18" s="2" t="inlineStr"/>
+      <c r="E18" s="2" t="inlineStr"/>
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>Closure rationale (operator decision 2026-05-10): Keep all
 VeritaPolicy rows. CFR-only references with no accreditor reference
@@ -1798,29 +1775,29 @@
 report misread the design intent.</t>
         </is>
       </c>
-      <c r="G13" s="3" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H13" s="3" t="inlineStr"/>
-    </row>
-    <row r="14" ht="90" customHeight="1">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19" ht="90" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>C7</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>CLIA number format validation (formerly #13)</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr"/>
-      <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="2" t="inlineStr"/>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="C19" s="3" t="inlineStr"/>
+      <c r="D19" s="3" t="inlineStr"/>
+      <c r="E19" s="3" t="inlineStr"/>
+      <c r="F19" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: shared/validateClia.ts defines CLIA_REGEX =
 /^\d{2}D\d{7}$/ (line 24), validateClia() helper with whitespace
@@ -1831,30 +1808,30 @@
 shape exists and behaves as specified.</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="G19" s="3" t="inlineStr">
         <is>
           <t>Agent verification 2026-05-10 via grep + file read.
 Operator confirmed shipped 2026-05-10.
 ---</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr"/>
-    </row>
-    <row r="15" ht="90" customHeight="1">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="H19" s="3" t="inlineStr"/>
+    </row>
+    <row r="20" ht="90" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>C8</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>VeritaMap lab-wide menu toggle (formerly #19)</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr"/>
-      <c r="D15" s="3" t="inlineStr"/>
-      <c r="E15" s="3" t="inlineStr"/>
-      <c r="F15" s="3" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr"/>
+      <c r="D20" s="2" t="inlineStr"/>
+      <c r="E20" s="2" t="inlineStr"/>
+      <c r="F20" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: client/src/pages/VeritaMapLabwidePage.tsx
 exists and implements the labwide read-only union view. Route is
@@ -1864,59 +1841,59 @@
 parking lot plan (read-only union view, per-session toggle) shipped.</t>
         </is>
       </c>
-      <c r="G15" s="3" t="inlineStr">
+      <c r="G20" s="2" t="inlineStr">
         <is>
           <t>Agent verification 2026-05-10 via grep + file read.
 Operator confirmed shipped 2026-05-10.
 ---</t>
         </is>
       </c>
-      <c r="H15" s="3" t="inlineStr"/>
-    </row>
-    <row r="16" ht="90" customHeight="1">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="H20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21" ht="90" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>C9</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>Tier-1 smoke test checklist (formerly #6)</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr"/>
-      <c r="D16" s="2" t="inlineStr"/>
-      <c r="E16" s="2" t="inlineStr"/>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="C21" s="3" t="inlineStr"/>
+      <c r="D21" s="3" t="inlineStr"/>
+      <c r="E21" s="3" t="inlineStr"/>
+      <c r="F21" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: docs/smoke-test-tier1.md documents the Tier-1
 smoke-test process and post-deploy verification steps. Shipped via
 PR #81 as part of the 2026-05-10 wave.</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="G21" s="3" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr"/>
-    </row>
-    <row r="17" ht="90" customHeight="1">
-      <c r="A17" s="3" t="inlineStr">
+      <c r="H21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22" ht="90" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>C10</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B22" s="2" t="inlineStr">
         <is>
           <t>Per-module gating (formerly #7)</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr"/>
-      <c r="D17" s="3" t="inlineStr"/>
-      <c r="E17" s="3" t="inlineStr"/>
-      <c r="F17" s="3" t="inlineStr">
+      <c r="C22" s="2" t="inlineStr"/>
+      <c r="D22" s="2" t="inlineStr"/>
+      <c r="E22" s="2" t="inlineStr"/>
+      <c r="F22" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: Client-side useIsReadOnly module keys wired
 on client/src/pages/VeritaPolicyAppPage.tsx and
@@ -1931,29 +1908,29 @@
 PR #76.</t>
         </is>
       </c>
-      <c r="G17" s="3" t="inlineStr">
+      <c r="G22" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H17" s="3" t="inlineStr"/>
-    </row>
-    <row r="18" ht="90" customHeight="1">
-      <c r="A18" s="2" t="inlineStr">
+      <c r="H22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23" ht="90" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>C11</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>VeritaStock shipped copy (formerly #8)</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr"/>
-      <c r="D18" s="2" t="inlineStr"/>
-      <c r="E18" s="2" t="inlineStr"/>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="C23" s="3" t="inlineStr"/>
+      <c r="D23" s="3" t="inlineStr"/>
+      <c r="E23" s="3" t="inlineStr"/>
+      <c r="F23" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: client/src/pages/ArticleInventoryManagementPage.tsx
 line 305 footer reads "platform that includes VeritaStock™" instead
@@ -1961,29 +1938,29 @@
 on /resources/laboratory-inventory-management. Shipped via PR #75.</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="G23" s="3" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H18" s="2" t="inlineStr"/>
-    </row>
-    <row r="19" ht="90" customHeight="1">
-      <c r="A19" s="3" t="inlineStr">
+      <c r="H23" s="3" t="inlineStr"/>
+    </row>
+    <row r="24" ht="90" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>C12</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>Admin report one-row-per-lab (formerly #14)</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr"/>
-      <c r="D19" s="3" t="inlineStr"/>
-      <c r="E19" s="3" t="inlineStr"/>
-      <c r="F19" s="3" t="inlineStr">
+      <c r="C24" s="2" t="inlineStr"/>
+      <c r="D24" s="2" t="inlineStr"/>
+      <c r="E24" s="2" t="inlineStr"/>
+      <c r="F24" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: /api/admin/report rewritten in
 server/routes.ts (~line 595) to LEFT JOIN labs on
@@ -1998,56 +1975,56 @@
 prerequisite, not a code bug). Shipped via PR #85.</t>
         </is>
       </c>
-      <c r="G19" s="3" t="inlineStr">
+      <c r="G24" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H19" s="3" t="inlineStr"/>
-    </row>
-    <row r="20" ht="90" customHeight="1">
-      <c r="A20" s="2" t="inlineStr">
+      <c r="H24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25" ht="90" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
         <is>
           <t>C14</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>UI relabel "CLIA TEa" -&gt; "Lab-Set Internal Goal" (formerly #1)</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr"/>
-      <c r="D20" s="2" t="inlineStr"/>
-      <c r="E20" s="2" t="inlineStr"/>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="C25" s="3" t="inlineStr"/>
+      <c r="D25" s="3" t="inlineStr"/>
+      <c r="E25" s="3" t="inlineStr"/>
+      <c r="F25" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: Shipped across four PRs over 2026-05-10.</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr">
+      <c r="G25" s="3" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H20" s="2" t="inlineStr"/>
-    </row>
-    <row r="21" ht="90" customHeight="1">
-      <c r="A21" s="3" t="inlineStr">
+      <c r="H25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26" ht="90" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>C13</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t>WSLH PT vendor (formerly #15)</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr"/>
-      <c r="D21" s="3" t="inlineStr"/>
-      <c r="E21" s="3" t="inlineStr"/>
-      <c r="F21" s="3" t="inlineStr">
+      <c r="C26" s="2" t="inlineStr"/>
+      <c r="D26" s="2" t="inlineStr"/>
+      <c r="E26" s="2" t="inlineStr"/>
+      <c r="F26" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: Shipped 2026-05-10 via PR #79 (merge commit
 eeebc6e; merged after rebase to resolve a server/db.ts collision
@@ -2065,64 +2042,64 @@
 'WSLH' is the post-deploy success signal. Shipped via PR #79.</t>
         </is>
       </c>
-      <c r="G21" s="3" t="inlineStr">
+      <c r="G26" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H21" s="3" t="inlineStr"/>
-    </row>
-    <row r="22" ht="90" customHeight="1">
-      <c r="A22" s="2" t="inlineStr">
+      <c r="H26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27" ht="90" customHeight="1">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>C15</t>
         </is>
       </c>
-      <c r="B22" s="2" t="inlineStr">
+      <c r="B27" s="3" t="inlineStr">
         <is>
           <t>VeritaStock lot tracking + expiration + reorder alerts (formerly #21)</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr"/>
-      <c r="D22" s="2" t="inlineStr"/>
-      <c r="E22" s="2" t="inlineStr"/>
-      <c r="F22" s="2" t="inlineStr">
+      <c r="C27" s="3" t="inlineStr"/>
+      <c r="D27" s="3" t="inlineStr"/>
+      <c r="E27" s="3" t="inlineStr"/>
+      <c r="F27" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: VeritaStock™ shipped the bench-level inventory
 features the Perplexity competitor analysis identified as a gap:</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr">
+      <c r="G27" s="3" t="inlineStr">
         <is>
           <t>Originally Perplexity competitor analysis 2026-05-10.
 Audit 2026-05-21 confirmed the feature set ships today.
 ---</t>
         </is>
       </c>
-      <c r="H22" s="2" t="inlineStr"/>
-    </row>
-    <row r="23" ht="90" customHeight="1">
-      <c r="A23" s="3" t="inlineStr">
+      <c r="H27" s="3" t="inlineStr"/>
+    </row>
+    <row r="28" ht="90" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>C16</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="B28" s="2" t="inlineStr">
         <is>
           <t>PAL studies guided workflow (formerly #23)</t>
         </is>
       </c>
-      <c r="C23" s="3" t="inlineStr"/>
-      <c r="D23" s="3" t="inlineStr"/>
-      <c r="E23" s="3" t="inlineStr"/>
-      <c r="F23" s="3" t="inlineStr">
+      <c r="C28" s="2" t="inlineStr"/>
+      <c r="D28" s="2" t="inlineStr"/>
+      <c r="E28" s="2" t="inlineStr"/>
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: VeritaCheck™ already ships the Precision /
 Accuracy / Linearity (PAL) study set under EP-protocol naming:</t>
         </is>
       </c>
-      <c r="G23" s="3" t="inlineStr">
+      <c r="G28" s="2" t="inlineStr">
         <is>
           <t>Originally Perplexity competitor analysis 2026-05-10.
 Audit 2026-05-21 confirmed the EP studies cover the PAL framing in
@@ -2130,23 +2107,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H23" s="3" t="inlineStr"/>
-    </row>
-    <row r="24" ht="90" customHeight="1">
-      <c r="A24" s="2" t="inlineStr">
+      <c r="H28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29" ht="90" customHeight="1">
+      <c r="A29" s="3" t="inlineStr">
         <is>
           <t>C17</t>
         </is>
       </c>
-      <c r="B24" s="2" t="inlineStr">
+      <c r="B29" s="3" t="inlineStr">
         <is>
           <t>Source-grounded 21/29/45 CFR + 42 CFR 482-485 (formerly #26)</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr"/>
-      <c r="D24" s="2" t="inlineStr"/>
-      <c r="E24" s="2" t="inlineStr"/>
-      <c r="F24" s="2" t="inlineStr">
+      <c r="C29" s="3" t="inlineStr"/>
+      <c r="D29" s="3" t="inlineStr"/>
+      <c r="E29" s="3" t="inlineStr"/>
+      <c r="F29" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #301 (commit 8c27806, merged 2026-05-21)
 source-grounded the 74 remaining non-493 entries in
@@ -2154,29 +2131,29 @@
 shipped:</t>
         </is>
       </c>
-      <c r="G24" s="2" t="inlineStr">
+      <c r="G29" s="3" t="inlineStr">
         <is>
           <t>PR #301; tasks #18 in the in-session task tracker.
 ---</t>
         </is>
       </c>
-      <c r="H24" s="2" t="inlineStr"/>
-    </row>
-    <row r="25" ht="90" customHeight="1">
-      <c r="A25" s="3" t="inlineStr">
+      <c r="H29" s="3" t="inlineStr"/>
+    </row>
+    <row r="30" ht="90" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>C18</t>
         </is>
       </c>
-      <c r="B25" s="3" t="inlineStr">
+      <c r="B30" s="2" t="inlineStr">
         <is>
           <t>VeritaPolicy "Non CLIA" chapter rename (formerly #3)</t>
         </is>
       </c>
-      <c r="C25" s="3" t="inlineStr"/>
-      <c r="D25" s="3" t="inlineStr"/>
-      <c r="E25" s="3" t="inlineStr"/>
-      <c r="F25" s="3" t="inlineStr">
+      <c r="C30" s="2" t="inlineStr"/>
+      <c r="D30" s="2" t="inlineStr"/>
+      <c r="E30" s="2" t="inlineStr"/>
+      <c r="F30" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #300 (commit 34d7707, merged 2026-05-21)
 renamed all 44 user-facing chapter labels in
@@ -2187,7 +2164,7 @@
 page.</t>
         </is>
       </c>
-      <c r="G25" s="3" t="inlineStr">
+      <c r="G30" s="2" t="inlineStr">
         <is>
           <t>CAP customer screenshot of the /veritapolicy chapter
 headers, 2026-05-01 evening. PR #300; tasks #17 in the in-session
@@ -2195,23 +2172,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H25" s="3" t="inlineStr"/>
-    </row>
-    <row r="26" ht="90" customHeight="1">
-      <c r="A26" s="2" t="inlineStr">
+      <c r="H30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31" ht="90" customHeight="1">
+      <c r="A31" s="3" t="inlineStr">
         <is>
           <t>C19</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="B31" s="3" t="inlineStr">
         <is>
           <t>VeritaStock department-scope toggle (formerly #31)</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr"/>
-      <c r="D26" s="2" t="inlineStr"/>
-      <c r="E26" s="2" t="inlineStr"/>
-      <c r="F26" s="2" t="inlineStr">
+      <c r="C31" s="3" t="inlineStr"/>
+      <c r="D31" s="3" t="inlineStr"/>
+      <c r="E31" s="3" t="inlineStr"/>
+      <c r="F31" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #319 (commit d01f5fe, merged 2026-05-22)
 shipped the persistent dept-scope toggle on VeritaStockPage. A new
@@ -2222,7 +2199,7 @@
 workspace without re-filtering.</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr">
+      <c r="G31" s="3" t="inlineStr">
         <is>
           <t>John, San Carlos lab, 2026-05-21. Same conversation that
 drove the vendor dropdown (PR #304), FILTERED VIEW banner (PR #305),
@@ -2230,23 +2207,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H26" s="2" t="inlineStr"/>
-    </row>
-    <row r="27" ht="90" customHeight="1">
-      <c r="A27" s="3" t="inlineStr">
+      <c r="H31" s="3" t="inlineStr"/>
+    </row>
+    <row r="32" ht="90" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t>C20</t>
         </is>
       </c>
-      <c r="B27" s="3" t="inlineStr">
+      <c r="B32" s="2" t="inlineStr">
         <is>
           <t>Primary-lab seat counting (formerly #12)</t>
         </is>
       </c>
-      <c r="C27" s="3" t="inlineStr"/>
-      <c r="D27" s="3" t="inlineStr"/>
-      <c r="E27" s="3" t="inlineStr"/>
-      <c r="F27" s="3" t="inlineStr">
+      <c r="C32" s="2" t="inlineStr"/>
+      <c r="D32" s="2" t="inlineStr"/>
+      <c r="E32" s="2" t="inlineStr"/>
+      <c r="F32" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: is_primary_lab INTEGER NOT NULL DEFAULT 0
 column was added to the lab_members table at db.ts:1276, with the
@@ -2257,7 +2234,7 @@
 is_primary_lab=1 ordering).</t>
         </is>
       </c>
-      <c r="G27" s="3" t="inlineStr">
+      <c r="G32" s="2" t="inlineStr">
         <is>
           <t>2026-05-07 multi-lab discussion. Build shipped as part
 of the Multi-Lab Tier 2 architecture work (Phase 3.x series, prior
@@ -2266,23 +2243,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H27" s="3" t="inlineStr"/>
-    </row>
-    <row r="28" ht="90" customHeight="1">
-      <c r="A28" s="2" t="inlineStr">
+      <c r="H32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33" ht="90" customHeight="1">
+      <c r="A33" s="3" t="inlineStr">
         <is>
           <t>C21</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="B33" s="3" t="inlineStr">
         <is>
           <t>Multi-lab pricing model — Option A (formerly #11)</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr"/>
-      <c r="D28" s="2" t="inlineStr"/>
-      <c r="E28" s="2" t="inlineStr"/>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="C33" s="3" t="inlineStr"/>
+      <c r="D33" s="3" t="inlineStr"/>
+      <c r="E33" s="3" t="inlineStr"/>
+      <c r="F33" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #322 (commit 0ccd925, merged 2026-05-22)
 added the customer-facing line to the pricing page that reflects
@@ -2295,7 +2272,7 @@
 Enterprise+ block, reads:</t>
         </is>
       </c>
-      <c r="G28" s="2" t="inlineStr">
+      <c r="G33" s="3" t="inlineStr">
         <is>
           <t>2026-05-07 multi-lab discussion (Lisa Veri's
 canonical-case session). PR #322 (initial build); softening PR
@@ -2304,30 +2281,30 @@
 ---</t>
         </is>
       </c>
-      <c r="H28" s="2" t="inlineStr"/>
-    </row>
-    <row r="29" ht="90" customHeight="1">
-      <c r="A29" s="3" t="inlineStr">
+      <c r="H33" s="3" t="inlineStr"/>
+    </row>
+    <row r="34" ht="90" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
         <is>
           <t>C22</t>
         </is>
       </c>
-      <c r="B29" s="3" t="inlineStr">
+      <c r="B34" s="2" t="inlineStr">
         <is>
           <t>VeritaOps cost-per-test module (formerly #10)</t>
         </is>
       </c>
-      <c r="C29" s="3" t="inlineStr"/>
-      <c r="D29" s="3" t="inlineStr"/>
-      <c r="E29" s="3" t="inlineStr"/>
-      <c r="F29" s="3" t="inlineStr">
+      <c r="C34" s="2" t="inlineStr"/>
+      <c r="D34" s="2" t="inlineStr"/>
+      <c r="E34" s="2" t="inlineStr"/>
+      <c r="F34" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: v1 of the VeritaOps Cost-Per-Reportable-Test
 (CPRT) module shipped across PR #325 through PR #330 on 2026-05-22.
 The module is feature-complete for the typical lab director workflow.</t>
         </is>
       </c>
-      <c r="G29" s="3" t="inlineStr">
+      <c r="G34" s="2" t="inlineStr">
         <is>
           <t>This thread, 2026-05-07 12:05 PM CDT, user message:
 "Parking lot: build an operations module for cost per test
@@ -2336,262 +2313,262 @@
 ---</t>
         </is>
       </c>
-      <c r="H29" s="3" t="inlineStr"/>
-    </row>
-    <row r="30" ht="90" customHeight="1">
-      <c r="A30" s="2" t="inlineStr">
+      <c r="H34" s="2" t="inlineStr"/>
+    </row>
+    <row r="35" ht="90" customHeight="1">
+      <c r="A35" s="3" t="inlineStr">
         <is>
           <t>C23</t>
         </is>
       </c>
-      <c r="B30" s="2" t="inlineStr">
+      <c r="B35" s="3" t="inlineStr">
         <is>
           <t>CCL lab name visual disambiguation in lab switcher (formerly #34)</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr"/>
-      <c r="D30" s="2" t="inlineStr">
+      <c r="C35" s="3" t="inlineStr"/>
+      <c r="D35" s="3" t="inlineStr">
         <is>
           <t>XS (under 1 day, actual)</t>
         </is>
       </c>
-      <c r="E30" s="2" t="inlineStr">
+      <c r="E35" s="3" t="inlineStr">
         <is>
           <t>Low — cosmetic; only mattered when Lisa or Michael picked the wrong lab from...</t>
         </is>
       </c>
-      <c r="F30" s="2" t="inlineStr">
+      <c r="F35" s="3" t="inlineStr">
         <is>
           <t>Effort: XS (under 1 day, actual)
 Importance: Low — cosmetic; only mattered when Lisa or Michael picked the wrong lab from the dropdown.</t>
         </is>
       </c>
-      <c r="G30" s="2" t="inlineStr">
+      <c r="G35" s="3" t="inlineStr">
         <is>
           <t>flagged 2026-05-23 immediately after provisioning Lisa's CCL lab; closed 2026-05-24.
 ---</t>
         </is>
       </c>
-      <c r="H30" s="2" t="inlineStr"/>
-    </row>
-    <row r="31" ht="90" customHeight="1">
-      <c r="A31" s="3" t="inlineStr">
+      <c r="H35" s="3" t="inlineStr"/>
+    </row>
+    <row r="36" ht="90" customHeight="1">
+      <c r="A36" s="2" t="inlineStr">
         <is>
           <t>C24</t>
         </is>
       </c>
-      <c r="B31" s="3" t="inlineStr">
+      <c r="B36" s="2" t="inlineStr">
         <is>
           <t>VC Unlimited Y1/Y2 price disclosure UX (formerly #35)</t>
         </is>
       </c>
-      <c r="C31" s="3" t="inlineStr"/>
-      <c r="D31" s="3" t="inlineStr">
+      <c r="C36" s="2" t="inlineStr"/>
+      <c r="D36" s="2" t="inlineStr">
         <is>
           <t>XS (under 1 day, actual)</t>
         </is>
       </c>
-      <c r="E31" s="3" t="inlineStr">
+      <c r="E36" s="2" t="inlineStr">
         <is>
           <t>Low when shipped (proactive, no customer complaint yet) — but high if a procu...</t>
         </is>
       </c>
-      <c r="F31" s="3" t="inlineStr">
+      <c r="F36" s="2" t="inlineStr">
         <is>
           <t>Effort: XS (under 1 day, actual)
 Importance: Low when shipped (proactive, no customer complaint yet) — but high if a procurement reviewer later disputes the $499 renewal as undisclosed.</t>
         </is>
       </c>
-      <c r="G31" s="3" t="inlineStr">
+      <c r="G36" s="2" t="inlineStr">
         <is>
           <t>Pricing rebuild 2026-05-23; closed 2026-05-24 proactively before any customer dispute.
 ---</t>
         </is>
       </c>
-      <c r="H31" s="3" t="inlineStr"/>
-    </row>
-    <row r="32" ht="90" customHeight="1">
-      <c r="A32" s="2" t="inlineStr">
+      <c r="H36" s="2" t="inlineStr"/>
+    </row>
+    <row r="37" ht="90" customHeight="1">
+      <c r="A37" s="3" t="inlineStr">
         <is>
           <t>C25</t>
         </is>
       </c>
-      <c r="B32" s="2" t="inlineStr">
+      <c r="B37" s="3" t="inlineStr">
         <is>
           <t>VeritaQC Phase 1 (Levey-Jennings + Westgard live engine) (formerly #20)</t>
         </is>
       </c>
-      <c r="C32" s="2" t="inlineStr"/>
-      <c r="D32" s="2" t="inlineStr">
+      <c r="C37" s="3" t="inlineStr"/>
+      <c r="D37" s="3" t="inlineStr">
         <is>
           <t>L (about 5 days end-to-end, actual: Phase 0 schema → Phase 1A evaluator → 1B...</t>
         </is>
       </c>
-      <c r="E32" s="2" t="inlineStr">
+      <c r="E37" s="3" t="inlineStr">
         <is>
           <t>High — largest single gap vs myLabCompliance.io per Perplexity competitor ana...</t>
         </is>
       </c>
-      <c r="F32" s="2" t="inlineStr">
+      <c r="F37" s="3" t="inlineStr">
         <is>
           <t>Effort: L (about 5 days end-to-end, actual: Phase 0 schema → Phase 1A evaluator → 1B entry UI → 1C daily review → 1D monthly PDF + attestation)
 Importance: High — largest single gap vs myLabCompliance.io per Perplexity competitor analysis; promotes VeritaAssure from documentation tool to lab operations platform.</t>
         </is>
       </c>
-      <c r="G32" s="2" t="inlineStr">
+      <c r="G37" s="3" t="inlineStr">
         <is>
           <t>Perplexity competitor analysis 2026-05-10. Scoping confirmed via the build_phase1_mockup.py iterations 2026-05-24. Shipped 2026-05-25.
 ---</t>
         </is>
       </c>
-      <c r="H32" s="2" t="inlineStr"/>
-    </row>
-    <row r="33" ht="90" customHeight="1">
-      <c r="A33" s="3" t="inlineStr">
+      <c r="H37" s="3" t="inlineStr"/>
+    </row>
+    <row r="38" ht="90" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
         <is>
           <t>C26</t>
         </is>
       </c>
-      <c r="B33" s="3" t="inlineStr">
+      <c r="B38" s="2" t="inlineStr">
         <is>
           <t>VeritaLab CMS-116 application support + state licensing registry (formerly #22)</t>
         </is>
       </c>
-      <c r="C33" s="3" t="inlineStr"/>
-      <c r="D33" s="3" t="inlineStr">
+      <c r="C38" s="2" t="inlineStr"/>
+      <c r="D38" s="2" t="inlineStr">
         <is>
           <t>M (1-2 weeks for v1, actual)</t>
         </is>
       </c>
-      <c r="E33" s="3" t="inlineStr">
+      <c r="E38" s="2" t="inlineStr">
         <is>
           <t>Medium — competitor parity (myLabCompliance.io) plus useful at lab startup an...</t>
         </is>
       </c>
-      <c r="F33" s="3" t="inlineStr">
+      <c r="F38" s="2" t="inlineStr">
         <is>
           <t>Effort: M (1-2 weeks for v1, actual)
 Importance: Medium — competitor parity (myLabCompliance.io) plus useful at lab startup and at certificate-type changes.</t>
         </is>
       </c>
-      <c r="G33" s="3" t="inlineStr">
+      <c r="G38" s="2" t="inlineStr">
         <is>
           <t>Perplexity competitor analysis (myLabCompliance.io), 2026-05-10. Reclassified as a VeritaLab extension 2026-05-25. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H33" s="3" t="inlineStr"/>
-    </row>
-    <row r="34" ht="90" customHeight="1">
-      <c r="A34" s="2" t="inlineStr">
+      <c r="H38" s="2" t="inlineStr"/>
+    </row>
+    <row r="39" ht="90" customHeight="1">
+      <c r="A39" s="3" t="inlineStr">
         <is>
           <t>C27</t>
         </is>
       </c>
-      <c r="B34" s="2" t="inlineStr">
+      <c r="B39" s="3" t="inlineStr">
         <is>
           <t>Active vs view-only seat split (formerly #33)</t>
         </is>
       </c>
-      <c r="C34" s="2" t="inlineStr"/>
-      <c r="D34" s="2" t="inlineStr">
+      <c r="C39" s="3" t="inlineStr"/>
+      <c r="D39" s="3" t="inlineStr">
         <is>
           <t>M (~1 week of engineering, actual: shipped in a single multi-PR session)</t>
         </is>
       </c>
-      <c r="E34" s="2" t="inlineStr">
+      <c r="E39" s="3" t="inlineStr">
         <is>
           <t>Medium — closed the gap between /pricing copy and product behavior; gives sal...</t>
         </is>
       </c>
-      <c r="F34" s="2" t="inlineStr">
+      <c r="F39" s="3" t="inlineStr">
         <is>
           <t>Effort: M (~1 week of engineering, actual: shipped in a single multi-PR session)
 Importance: Medium — closed the gap between /pricing copy and product behavior; gives sales a clean answer for "do you charge for our medical director?"</t>
         </is>
       </c>
-      <c r="G34" s="2" t="inlineStr">
+      <c r="G39" s="3" t="inlineStr">
         <is>
           <t>Pricing analysis doc Decision 3 (2026-05-21); MEDIUM scenario revised 2026-05-29 to retire the "unlimited view-only" claim. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H34" s="2" t="inlineStr"/>
-    </row>
-    <row r="35" ht="90" customHeight="1">
-      <c r="A35" s="3" t="inlineStr">
+      <c r="H39" s="3" t="inlineStr"/>
+    </row>
+    <row r="40" ht="90" customHeight="1">
+      <c r="A40" s="2" t="inlineStr">
         <is>
           <t>C28</t>
         </is>
       </c>
-      <c r="B35" s="3" t="inlineStr">
+      <c r="B40" s="2" t="inlineStr">
         <is>
           <t>"Why VeritaCheck" comparative one-pager (formerly #37)</t>
         </is>
       </c>
-      <c r="C35" s="3" t="inlineStr"/>
-      <c r="D35" s="3" t="inlineStr">
+      <c r="C40" s="2" t="inlineStr"/>
+      <c r="D40" s="2" t="inlineStr">
         <is>
           <t>S (one design pass + four claim paragraphs + PDF + matching marketing-site pa...</t>
         </is>
       </c>
-      <c r="E35" s="3" t="inlineStr">
+      <c r="E40" s="2" t="inlineStr">
         <is>
           <t>Medium — closed a positioning gap surfaced by six COLA conference attendees a...</t>
         </is>
       </c>
-      <c r="F35" s="3" t="inlineStr">
+      <c r="F40" s="2" t="inlineStr">
         <is>
           <t>Effort: S (one design pass + four claim paragraphs + PDF + matching marketing-site page, actual)
 Importance: Medium — closed a positioning gap surfaced by six COLA conference attendees attached to a legacy verification tool; converts product-quality advantage into a leave-behind Lisa can hand out.</t>
         </is>
       </c>
-      <c r="G35" s="3" t="inlineStr">
+      <c r="G40" s="2" t="inlineStr">
         <is>
           <t>2026-05-11 / 2026-05-12 conference notes review with Michael. Conference attendees (Whitehead, Odegard, Othman, Molinelli, Kyle, Allred) expressed interest in equivalent / superior product. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H35" s="3" t="inlineStr"/>
-    </row>
-    <row r="36" ht="90" customHeight="1">
-      <c r="A36" s="2" t="inlineStr">
+      <c r="H40" s="2" t="inlineStr"/>
+    </row>
+    <row r="41" ht="90" customHeight="1">
+      <c r="A41" s="3" t="inlineStr">
         <is>
           <t>C29</t>
         </is>
       </c>
-      <c r="B36" s="2" t="inlineStr">
+      <c r="B41" s="3" t="inlineStr">
         <is>
           <t>VeritaPolicy approval workflow — MediaLab functional mirror</t>
         </is>
       </c>
-      <c r="C36" s="2" t="inlineStr"/>
-      <c r="D36" s="2" t="inlineStr">
+      <c r="C41" s="3" t="inlineStr"/>
+      <c r="D41" s="3" t="inlineStr">
         <is>
           <t>XL (one focused session, 12 PRs landed)</t>
         </is>
       </c>
-      <c r="E36" s="2" t="inlineStr">
+      <c r="E41" s="3" t="inlineStr">
         <is>
           <t>High — replaces MediaLab Document Control ($752/$2,250 starting price, scalin...</t>
         </is>
       </c>
-      <c r="F36" s="2" t="inlineStr">
+      <c r="F41" s="3" t="inlineStr">
         <is>
           <t>Effort: XL (one focused session, 12 PRs landed)
 Importance: High — replaces MediaLab Document Control ($752/$2,250 starting price, scaling to $10K-$20K/yr at enterprise per Capterra public data) with an included VeritaPolicy feature; closes a real positioning gap and gives sales a direct comparator line.</t>
         </is>
       </c>
-      <c r="G36" s="2" t="inlineStr">
+      <c r="G41" s="3" t="inlineStr">
         <is>
           <t>Pricing strategy conversation 2026-05-29 (Michael: "I don't like bolt-ons; we should replicate this") → scoped 8 phases → shipped all 12 PRs in single session. Shipped 2026-05-29.
 ---</t>
         </is>
       </c>
-      <c r="H36" s="2" t="inlineStr"/>
+      <c r="H41" s="3" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H36"/>
+  <autoFilter ref="A1:H41"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
TASK: Parking-lot sync (2026-09-24 pass 2) - log the coverage-recurrence, VeritaComp coverage-map, and VeritaStaff dual-view work + two follow-ups.
PLAN:
  1. Add CLOSED C41 (VeritaCheck coverage recurrence, PRs #1317/#1318/#1321), C42 (VeritaComp coverage map, #1319/#1316), C43 (VeritaStaff dual assignment view, #1320).
  2. Add OPEN #49 (shared recurrence helper, hygiene) and #50 (competency assessed-this-cycle window refinement).
  3. Regenerate PARKING_LOT.xlsx.

Self-check:
  - OPEN 15 -> 17; CLOSED 40 -> 43; RETIRED unchanged; total 66.
  - Each closure cites PRs + live verification; follow-ups flagged low/medium with no live defect.
  - md + xlsx committed together per the sync convention.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PARKING_LOT.xlsx
+++ b/PARKING_LOT.xlsx
@@ -12,8 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RETIRED" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$44</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RETIRED'!$A$1:$H$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1212,8 +1212,80 @@
       </c>
       <c r="H16" s="2" t="inlineStr"/>
     </row>
+    <row r="17" ht="90" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Unify the coverage/competency recurrence into one shared helper (tech debt)</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr"/>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>S (a few hours) - extract "latest study/assessment -&gt; status / nextDueOn / ov...</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Low - the three paths duplicate the +6-month / signed-resets-to-missing logic...</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Effort: S (a few hours) - extract "latest study/assessment -&gt; status / nextDueOn / overdue" into one helper used by method comparison, cal-ver/linearity, and the competency owed derivation.
+Importance: Low - the three paths duplicate the +6-month / signed-resets-to-missing logic. They agree today (verified), but a shared helper prevents future drift and settles the dateless-signed edge in one place. No user-facing impact; studies.date is NOT NULL so the one known divergence is unreachable in practice.</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-24 session, surfaced during the coverage-recurrence build. No live defect; hygiene.
+---</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr"/>
+    </row>
+    <row r="18" ht="90" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Competency "assessed this cycle" uses a flat 365-day window</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr"/>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>S-M - anchor the coverage-map "assessed this cycle" to the person's actual CL...</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Medium - in an employee's first year the semiannual windows differ from a fla...</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Effort: S-M - anchor the coverage-map "assessed this cycle" to the person's actual CLIA cadence (semiannual in year 1 per 42 CFR 493.1451(b)(8), annual thereafter) from staff_competency_schedules, instead of the v1 flat 365-day lookback.
+Importance: Medium - in an employee's first year the semiannual windows differ from a flat annual window, so a first-year assessment could read as current slightly longer or shorter than the true cadence. Fine for the common annual case; refine for year-1 accuracy.</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24 session, VeritaComp coverage map (#48 Phase 3) v1 simplification, noted in PR #1319.
+---</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H16"/>
+  <autoFilter ref="A1:H18"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1224,7 +1296,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H41"/>
+  <dimension ref="A1:H44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1282,12 +1354,12 @@
     <row r="2" ht="90" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>C40</t>
+          <t>C43</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>VeritaComp Competencies Owed derived from VeritaStaff, with gap detection (was #48)</t>
+          <t>VeritaStaff instrument-centric (dual) assignment view</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr"/>
@@ -1295,12 +1367,12 @@
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1314 (squash 2bcb0db9). GET /api/labs/:labId/competency/owed derives each VeritaStaff testing employee's owed competencies from their assigned instruments (staff_employee_instruments -&gt; veritamap_instruments + tests), on the CLIA timeline, and flags instruments not covered by any competency program as gaps. CompetenciesOwedSection renders it on the VeritaComp landing page. Reuses the shipped bridge + suggested-method-groups match rules; no new tables. Verified live on prod with real assignment data: 2 instruments assigned to a demo staffer produced owed=2, gaps=2 (HIGH, Technical Supervisor), then reverted cleanly. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1320. GET/PUT /staff/instruments/:id/employees (transpose of the per-employee endpoints); an "Assign by Instrument" dialog lets a director pick a test system or manual test and check off who runs it. Same staff_employee_instruments join, with the 42 CFR 493.1235(a) duty-change event emitted on newly-added pairs so both orientations trigger the same reassessment. GET verified live on SCAHC lab 2. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23/24 session, Michael ("veritacomp bases what competencies they owe (currently untrue, but needs to be true)"). Option 1 (unify roster on VeritaStaff, match instruments by id).
+          <t>2026-09-24 session, Michael ("in staff we should also give the dual view when assigning coverage to test systems or manual tests").
 ---</t>
         </is>
       </c>
@@ -1309,12 +1381,12 @@
     <row r="3" ht="90" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>C39</t>
+          <t>C42</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>VeritaScan line items can attach or link evidence (was #46)</t>
+          <t>VeritaComp coverage map (required-vs-assessed matrix, dual view)</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr"/>
@@ -1322,12 +1394,12 @@
       <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1312 (squash a1dda93d). VeritaScan scan checklist items now show linked evidence as chips (open link, remove) plus a writer "Link evidence" affordance whose picker links an existing VeritaDC/Library document; a shortcut deep-links to the Library for new (governed) documents. Reuses the already-shipped lab_documents + document_checklist_links + coverage endpoints (URL-pointer only, no file storage, no new tables). Browser-verified live on prod (scan 23): the affordance renders and the picker opens. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1319 (+ status layer PR #1316). /competency/owed returns per-item assessed (locked passing assessment this cycle on a covering method group) + per-employee CLIA status; CompetencyCoverageMap renders a By-employee / By-instrument matrix (Assessed / Owed / Overdue / Gap). Verified live on SCAHC lab 2 (owed 116, assessed 2, gaps 0). Completes #48 as the VeritaCheck-parity coverage map. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>2026-09-23 session, Michael. Recurring request. Companion: cross-module evidence display on the VeritaDC policy shipped in PR #1313 (by-target cross-links surfaced in the policy View modal, browser-verified live).
+          <t>2026-09-24 session, Michael ("are we building the competencies to have a coverage map, same as veritacheck?" then "build it").
 ---</t>
         </is>
       </c>
@@ -1336,12 +1408,12 @@
     <row r="4" ht="90" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>C38</t>
+          <t>C41</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>VeritaTrack calendar month cells expand to reveal hidden tasks (was #45)</t>
+          <t>VeritaCheck coverage recurrence (method comparison + cal-ver/linearity + reports)</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr"/>
@@ -1349,12 +1421,12 @@
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: VeritaTrack CalendarView month cells with more than three tasks now expand in place (chevron, "+N more" toggling to "Show less", due dates), so no task is hidden with no path to it (client/src/pages/VeritaTrackAppPage.tsx CalendarView). Shipped 2026-09-23. Closed 2026-09-24.</t>
+          <t>Closure evidence: PRs #1317 (method comparison), #1318 (cal-ver/linearity), #1321 (report Next-due columns). Periodic verification (correlation/method comparison 42 CFR 493.1281; cal-ver/linearity 42 CFR 493.1255; both 6-month) now recurs: a signed study banks the cycle and rolls to next-due = signed + 6 months instead of reading "done" forever. Status Missing/Failed/Completed-unsigned + a "Next due on" column on-screen and in both coverage exports; also credits the previously-ignored "correlation" study type. Root cause: computeCoverageFrom marked requirements done on mere existence, no date logic. Verified live on SCAHC lab 2 (101 correlations + 11 cal-ver rows now carry a next-due). Engine-level, all facilities. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23 session, Michael screenshot of the VeritaTrack calendar (lab 3, September cell).
+          <t>2026-09-24 session, Michael ("Look at San Carlos... they finished their last set of correlations (all 103) but their menu never reset").
 ---</t>
         </is>
       </c>
@@ -1363,12 +1435,12 @@
     <row r="5" ht="90" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>C37</t>
+          <t>C40</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Long Excel column headers no longer clip CFR citations (was #44)</t>
+          <t>VeritaComp Competencies Owed derived from VeritaStaff, with gap detection (was #48)</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr"/>
@@ -1376,12 +1448,12 @@
       <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. The VeritaMap export derives the header row height from the longest wrapped header via headerRowHeight(headers, colWidths) (server/routes.ts:15935) instead of a fixed 20, so "Reference Range Attestation (42 CFR 493.1253)" and the other long headers print in full. No new code this session. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1314 (squash 2bcb0db9). GET /api/labs/:labId/competency/owed derives each VeritaStaff testing employee's owed competencies from their assigned instruments (staff_employee_instruments -&gt; veritamap_instruments + tests), on the CLIA timeline, and flags instruments not covered by any competency program as gaps. CompetenciesOwedSection renders it on the VeritaComp landing page. Reuses the shipped bridge + suggested-method-groups match rules; no new tables. Verified live on prod with real assignment data: 2 instruments assigned to a demo staffer produced owed=2, gaps=2 (HIGH, Technical Supervisor), then reverted cleanly. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+          <t>2026-09-23/24 session, Michael ("veritacomp bases what competencies they owe (currently untrue, but needs to be true)"). Option 1 (unify roster on VeritaStaff, match instruments by id).
 ---</t>
         </is>
       </c>
@@ -1390,12 +1462,12 @@
     <row r="6" ht="90" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>C36</t>
+          <t>C39</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>License stamp no longer clobbers the §6 header/footer or names the wrong lab (was #43)</t>
+          <t>VeritaScan line items can attach or link evidence (was #46)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr"/>
@@ -1403,12 +1475,12 @@
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. setHeaderFooter (shared/licenseExceljs.ts:155-209) now preserves an existing §6 header and appends (not overwrites) the footer left section, and customer-facing exports name the scoped lab: the VeritaScan library export reads req.scope.lab.name / clia_number (server/routes.ts:16572-16573), not the licensee. No new code this session (avoided regressing the existing fix). Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1312 (squash a1dda93d). VeritaScan scan checklist items now show linked evidence as chips (open link, remove) plus a writer "Link evidence" affordance whose picker links an existing VeritaDC/Library document; a shortcut deep-links to the Library for new (governed) documents. Reuses the already-shipped lab_documents + document_checklist_links + coverage endpoints (URL-pointer only, no file storage, no new tables). Browser-verified live on prod (scan 23): the affordance renders and the picker opens. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+          <t>2026-09-23 session, Michael. Recurring request. Companion: cross-module evidence display on the VeritaDC policy shipped in PR #1313 (by-target cross-links surfaced in the policy View modal, browser-verified live).
 ---</t>
         </is>
       </c>
@@ -1417,18 +1489,99 @@
     <row r="7" ht="90" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>C34</t>
+          <t>C38</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Wire the two static-audit guards into CI (was #43)</t>
+          <t>VeritaTrack calendar month cells expand to reveal hidden tasks (was #45)</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr"/>
       <c r="D7" s="3" t="inlineStr"/>
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Closure evidence: VeritaTrack CalendarView month cells with more than three tasks now expand in place (chevron, "+N more" toggling to "Show less", due dates), so no task is hidden with no path to it (client/src/pages/VeritaTrackAppPage.tsx CalendarView). Shipped 2026-09-23. Closed 2026-09-24.</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-23 session, Michael screenshot of the VeritaTrack calendar (lab 3, September cell).
+---</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr"/>
+    </row>
+    <row r="8" ht="90" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>C37</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Long Excel column headers no longer clip CFR citations (was #44)</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr"/>
+      <c r="D8" s="2" t="inlineStr"/>
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. The VeritaMap export derives the header row height from the longest wrapped header via headerRowHeight(headers, colWidths) (server/routes.ts:15935) instead of a fixed 20, so "Reference Range Attestation (42 CFR 493.1253)" and the other long headers print in full. No new code this session. Closed 2026-09-24.</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+---</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9" ht="90" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>C36</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>License stamp no longer clobbers the §6 header/footer or names the wrong lab (was #43)</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr"/>
+      <c r="D9" s="3" t="inlineStr"/>
+      <c r="E9" s="3" t="inlineStr"/>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. setHeaderFooter (shared/licenseExceljs.ts:155-209) now preserves an existing §6 header and appends (not overwrites) the footer left section, and customer-facing exports name the scoped lab: the VeritaScan library export reads req.scope.lab.name / clia_number (server/routes.ts:16572-16573), not the licensee. No new code this session (avoided regressing the existing fix). Closed 2026-09-24.</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+---</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr"/>
+    </row>
+    <row r="10" ht="90" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>C34</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Wire the two static-audit guards into CI (was #43)</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr"/>
+      <c r="D10" s="2" t="inlineStr"/>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: both guards wired into the Multi-Lab Mutations Audit CI
 workflow (.github/workflows/multilab-mutations-audit.yml) as steps:
@@ -1440,24 +1593,24 @@
 (same caveat as the existing guards already in that workflow).</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr"/>
-      <c r="H7" s="3" t="inlineStr"/>
-    </row>
-    <row r="8" ht="90" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11" ht="90" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>C35</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>Legacy /api/studies over-returns studies across labs (was #44)</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr"/>
-      <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr"/>
+      <c r="D11" s="3" t="inlineStr"/>
+      <c r="E11" s="3" t="inlineStr"/>
+      <c r="F11" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: GET /api/studies now scopes its list to the active lab
 when one is resolved from the Referer (server/routes.ts), so every returned row
@@ -1467,24 +1620,24 @@
 mirroring the /api/labs/:labId/studies handler. Closed 2026-06-14.</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr"/>
-      <c r="H8" s="2" t="inlineStr"/>
-    </row>
-    <row r="9" ht="90" customHeight="1">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="G11" s="3" t="inlineStr"/>
+      <c r="H11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12" ht="90" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>C30</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>Verify-script convention backfill (was #41)</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr"/>
-      <c r="D9" s="3" t="inlineStr"/>
-      <c r="E9" s="3" t="inlineStr"/>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr"/>
+      <c r="D12" s="2" t="inlineStr"/>
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: all 8 high-stakes math/logic commits now ship a paired
 scripts/verify-*.js (EP17 sensitivity, Deming lot-to-lot, CUMSUM+QC+multi-analyte,
@@ -1492,30 +1645,30 @@
 TEa boundary), per the strike-throughs in #41. Closed 2026-06-13.</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>scripts/audit_verify_script_coverage.py lookback, 2026-06-02; backfills
 landed 2026-06-03..06.
 ---</t>
         </is>
       </c>
-      <c r="H9" s="3" t="inlineStr"/>
-    </row>
-    <row r="10" ht="90" customHeight="1">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13" ht="90" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>C31</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>VeritaPT AAA create/update/delete silently no-op in the multi-lab UI</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr"/>
-      <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr"/>
+      <c r="D13" s="3" t="inlineStr"/>
+      <c r="E13" s="3" t="inlineStr"/>
+      <c r="F13" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #754 (commit 92ad499) added lab-scoped POST/PUT/DELETE
 /api/labs/:labId/pt/aa-records. The UI posted to the lab-scoped path but only GET
@@ -1526,30 +1679,30 @@
 route mis-filed records to the user's default lab on multi-lab accounts).</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G13" s="3" t="inlineStr">
         <is>
           <t>2026-06-13, found during #18 Phase 3 QA;
 scripts/audit-labscoped-write-routes.mjs now guards the class.
 ---</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr"/>
-    </row>
-    <row r="11" ht="90" customHeight="1">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="H13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14" ht="90" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>C32</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>VeritaComp "Unlock assessment" false-success no-op</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr"/>
-      <c r="D11" s="3" t="inlineStr"/>
-      <c r="E11" s="3" t="inlineStr"/>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr"/>
+      <c r="D14" s="2" t="inlineStr"/>
+      <c r="E14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #755 (commit 4234007) moved the unlock route to
 /api/labs/:labId/competency/assessments/:id/unlock (the path the client calls).
@@ -1560,29 +1713,29 @@
 HTML).</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>2026-06-13, found by scripts/audit-labscoped-write-routes.mjs.
 ---</t>
         </is>
       </c>
-      <c r="H11" s="3" t="inlineStr"/>
-    </row>
-    <row r="12" ht="90" customHeight="1">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="H14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15" ht="90" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>C33</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>FK-cascade delete 500s + NavBar laptop-width overflow</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr"/>
-      <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="2" t="inlineStr"/>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr"/>
+      <c r="D15" s="3" t="inlineStr"/>
+      <c r="E15" s="3" t="inlineStr"/>
+      <c r="F15" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PRs #749/#750 fixed NavBar horizontal overflow at laptop
 widths (collapse to the hamburger below 1560px); prod-verified at 1280-1920 with the
@@ -1593,57 +1746,57 @@
 500 -&gt; 200. scripts/audit-delete-cascades.mjs guards the class.</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G15" s="3" t="inlineStr">
         <is>
           <t>2026-06-13 browser QA of the A7-D4 wave + retro-QC of the 72h PR window.
 ---</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr"/>
-    </row>
-    <row r="13" ht="90" customHeight="1">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="H15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16" ht="90" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>C1</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>FAQ "over 25 years" -&gt; "over 23 years"</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr"/>
-      <c r="D13" s="3" t="inlineStr"/>
-      <c r="E13" s="3" t="inlineStr"/>
-      <c r="F13" s="3" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr"/>
+      <c r="D16" s="2" t="inlineStr"/>
+      <c r="E16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: client/src/pages/FAQPage.tsx line 20 reads "over
 23 years" as of 2026-05-01.</t>
         </is>
       </c>
-      <c r="G13" s="3" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>session 299e9a73 turn 14, ~2026-04-28.
 ---</t>
         </is>
       </c>
-      <c r="H13" s="3" t="inlineStr"/>
-    </row>
-    <row r="14" ht="90" customHeight="1">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="H16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17" ht="90" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>C5</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>David's VeritaQA grey-button bug (seat permissions mode)</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr"/>
-      <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="2" t="inlineStr"/>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr"/>
+      <c r="D17" s="3" t="inlineStr"/>
+      <c r="E17" s="3" t="inlineStr"/>
+      <c r="F17" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #10 squash-merged as commit a43fbba on
 2026-05-01 23:19 MST. Railway deploy succeeded; deployed bundle
@@ -1656,7 +1809,7 @@
 against his exact stored shape (14 of 14 expected outcomes matched).</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="G17" s="3" t="inlineStr">
         <is>
           <t>2026-05-01 David's report; veritabench + veritastock
 weren't in MODULE_LIST so seat permissions silently defaulted to
@@ -1664,109 +1817,109 @@
 ---</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr"/>
-    </row>
-    <row r="15" ht="90" customHeight="1">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>C2</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>TeamPage present-tense "TJC surveyor" check</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr"/>
-      <c r="D15" s="3" t="inlineStr"/>
-      <c r="E15" s="3" t="inlineStr"/>
-      <c r="F15" s="3" t="inlineStr">
-        <is>
-          <t>Closure evidence: site-wide search confirmed all surveyor language
-is past-tense, consistent with user's 2021-2025 service. User closed
-the item in session 299e9a73 turn 4.</t>
-        </is>
-      </c>
-      <c r="G15" s="3" t="inlineStr">
-        <is>
-          <t>session 299e9a73, ~2026-04-28.
----</t>
-        </is>
-      </c>
-      <c r="H15" s="3" t="inlineStr"/>
-    </row>
-    <row r="16" ht="90" customHeight="1">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>C3</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>My Studies CSV/XLSX export (John as design partner)</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr"/>
-      <c r="D16" s="2" t="inlineStr"/>
-      <c r="E16" s="2" t="inlineStr"/>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>Closure evidence: client/src/pages/DashboardPage.tsx line 46 calls
-/api/my-studies/export. server/routes.ts line 1491 implements the
-endpoint. Pulled forward into pre-COLA per user instruction.</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>session 299e9a73 turn 5, ~2026-04-28.
----</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr"/>
-    </row>
-    <row r="17" ht="90" customHeight="1">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>C4</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>Rotate GitHub PAT (because old PAT was committed in SESSION_HANDOFF files)</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="inlineStr"/>
-      <c r="D17" s="3" t="inlineStr"/>
-      <c r="E17" s="3" t="inlineStr"/>
-      <c r="F17" s="3" t="inlineStr">
-        <is>
-          <t>Closure evidence: no ghp_* or github_pat_* patterns in current
-SESSION_HANDOFF.md or SESSION_HANDOFF-2.md as of 2026-05-01.</t>
-        </is>
-      </c>
-      <c r="G17" s="3" t="inlineStr">
-        <is>
-          <t>session 299e9a73, ~2026-04-28.
----</t>
-        </is>
-      </c>
       <c r="H17" s="3" t="inlineStr"/>
     </row>
     <row r="18" ht="90" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>C6</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>VeritaPolicy service-line filtering removed (formerly #4)</t>
+          <t>TeamPage present-tense "TJC surveyor" check</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr"/>
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Closure evidence: site-wide search confirmed all surveyor language
+is past-tense, consistent with user's 2021-2025 service. User closed
+the item in session 299e9a73 turn 4.</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>session 299e9a73, ~2026-04-28.
+---</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19" ht="90" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>C3</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>My Studies CSV/XLSX export (John as design partner)</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr"/>
+      <c r="D19" s="3" t="inlineStr"/>
+      <c r="E19" s="3" t="inlineStr"/>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Closure evidence: client/src/pages/DashboardPage.tsx line 46 calls
+/api/my-studies/export. server/routes.ts line 1491 implements the
+endpoint. Pulled forward into pre-COLA per user instruction.</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>session 299e9a73 turn 5, ~2026-04-28.
+---</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr"/>
+    </row>
+    <row r="20" ht="90" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Rotate GitHub PAT (because old PAT was committed in SESSION_HANDOFF files)</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr"/>
+      <c r="D20" s="2" t="inlineStr"/>
+      <c r="E20" s="2" t="inlineStr"/>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Closure evidence: no ghp_* or github_pat_* patterns in current
+SESSION_HANDOFF.md or SESSION_HANDOFF-2.md as of 2026-05-01.</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>session 299e9a73, ~2026-04-28.
+---</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21" ht="90" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>C6</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>VeritaPolicy service-line filtering removed (formerly #4)</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr"/>
+      <c r="D21" s="3" t="inlineStr"/>
+      <c r="E21" s="3" t="inlineStr"/>
+      <c r="F21" s="3" t="inlineStr">
         <is>
           <t>Closure rationale (operator decision 2026-05-10): Keep all
 VeritaPolicy rows. CFR-only references with no accreditor reference
@@ -1775,29 +1928,29 @@
 report misread the design intent.</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="G21" s="3" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H18" s="2" t="inlineStr"/>
-    </row>
-    <row r="19" ht="90" customHeight="1">
-      <c r="A19" s="3" t="inlineStr">
+      <c r="H21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22" ht="90" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>C7</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B22" s="2" t="inlineStr">
         <is>
           <t>CLIA number format validation (formerly #13)</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr"/>
-      <c r="D19" s="3" t="inlineStr"/>
-      <c r="E19" s="3" t="inlineStr"/>
-      <c r="F19" s="3" t="inlineStr">
+      <c r="C22" s="2" t="inlineStr"/>
+      <c r="D22" s="2" t="inlineStr"/>
+      <c r="E22" s="2" t="inlineStr"/>
+      <c r="F22" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: shared/validateClia.ts defines CLIA_REGEX =
 /^\d{2}D\d{7}$/ (line 24), validateClia() helper with whitespace
@@ -1808,30 +1961,30 @@
 shape exists and behaves as specified.</t>
         </is>
       </c>
-      <c r="G19" s="3" t="inlineStr">
+      <c r="G22" s="2" t="inlineStr">
         <is>
           <t>Agent verification 2026-05-10 via grep + file read.
 Operator confirmed shipped 2026-05-10.
 ---</t>
         </is>
       </c>
-      <c r="H19" s="3" t="inlineStr"/>
-    </row>
-    <row r="20" ht="90" customHeight="1">
-      <c r="A20" s="2" t="inlineStr">
+      <c r="H22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23" ht="90" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>C8</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>VeritaMap lab-wide menu toggle (formerly #19)</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr"/>
-      <c r="D20" s="2" t="inlineStr"/>
-      <c r="E20" s="2" t="inlineStr"/>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="C23" s="3" t="inlineStr"/>
+      <c r="D23" s="3" t="inlineStr"/>
+      <c r="E23" s="3" t="inlineStr"/>
+      <c r="F23" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: client/src/pages/VeritaMapLabwidePage.tsx
 exists and implements the labwide read-only union view. Route is
@@ -1841,59 +1994,59 @@
 parking lot plan (read-only union view, per-session toggle) shipped.</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr">
+      <c r="G23" s="3" t="inlineStr">
         <is>
           <t>Agent verification 2026-05-10 via grep + file read.
 Operator confirmed shipped 2026-05-10.
 ---</t>
         </is>
       </c>
-      <c r="H20" s="2" t="inlineStr"/>
-    </row>
-    <row r="21" ht="90" customHeight="1">
-      <c r="A21" s="3" t="inlineStr">
+      <c r="H23" s="3" t="inlineStr"/>
+    </row>
+    <row r="24" ht="90" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>C9</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>Tier-1 smoke test checklist (formerly #6)</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr"/>
-      <c r="D21" s="3" t="inlineStr"/>
-      <c r="E21" s="3" t="inlineStr"/>
-      <c r="F21" s="3" t="inlineStr">
+      <c r="C24" s="2" t="inlineStr"/>
+      <c r="D24" s="2" t="inlineStr"/>
+      <c r="E24" s="2" t="inlineStr"/>
+      <c r="F24" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: docs/smoke-test-tier1.md documents the Tier-1
 smoke-test process and post-deploy verification steps. Shipped via
 PR #81 as part of the 2026-05-10 wave.</t>
         </is>
       </c>
-      <c r="G21" s="3" t="inlineStr">
+      <c r="G24" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H21" s="3" t="inlineStr"/>
-    </row>
-    <row r="22" ht="90" customHeight="1">
-      <c r="A22" s="2" t="inlineStr">
+      <c r="H24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25" ht="90" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
         <is>
           <t>C10</t>
         </is>
       </c>
-      <c r="B22" s="2" t="inlineStr">
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>Per-module gating (formerly #7)</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr"/>
-      <c r="D22" s="2" t="inlineStr"/>
-      <c r="E22" s="2" t="inlineStr"/>
-      <c r="F22" s="2" t="inlineStr">
+      <c r="C25" s="3" t="inlineStr"/>
+      <c r="D25" s="3" t="inlineStr"/>
+      <c r="E25" s="3" t="inlineStr"/>
+      <c r="F25" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: Client-side useIsReadOnly module keys wired
 on client/src/pages/VeritaPolicyAppPage.tsx and
@@ -1908,29 +2061,29 @@
 PR #76.</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr">
+      <c r="G25" s="3" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H22" s="2" t="inlineStr"/>
-    </row>
-    <row r="23" ht="90" customHeight="1">
-      <c r="A23" s="3" t="inlineStr">
+      <c r="H25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26" ht="90" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>C11</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t>VeritaStock shipped copy (formerly #8)</t>
         </is>
       </c>
-      <c r="C23" s="3" t="inlineStr"/>
-      <c r="D23" s="3" t="inlineStr"/>
-      <c r="E23" s="3" t="inlineStr"/>
-      <c r="F23" s="3" t="inlineStr">
+      <c r="C26" s="2" t="inlineStr"/>
+      <c r="D26" s="2" t="inlineStr"/>
+      <c r="E26" s="2" t="inlineStr"/>
+      <c r="F26" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: client/src/pages/ArticleInventoryManagementPage.tsx
 line 305 footer reads "platform that includes VeritaStock™" instead
@@ -1938,29 +2091,29 @@
 on /resources/laboratory-inventory-management. Shipped via PR #75.</t>
         </is>
       </c>
-      <c r="G23" s="3" t="inlineStr">
+      <c r="G26" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H23" s="3" t="inlineStr"/>
-    </row>
-    <row r="24" ht="90" customHeight="1">
-      <c r="A24" s="2" t="inlineStr">
+      <c r="H26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27" ht="90" customHeight="1">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>C12</t>
         </is>
       </c>
-      <c r="B24" s="2" t="inlineStr">
+      <c r="B27" s="3" t="inlineStr">
         <is>
           <t>Admin report one-row-per-lab (formerly #14)</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr"/>
-      <c r="D24" s="2" t="inlineStr"/>
-      <c r="E24" s="2" t="inlineStr"/>
-      <c r="F24" s="2" t="inlineStr">
+      <c r="C27" s="3" t="inlineStr"/>
+      <c r="D27" s="3" t="inlineStr"/>
+      <c r="E27" s="3" t="inlineStr"/>
+      <c r="F27" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: /api/admin/report rewritten in
 server/routes.ts (~line 595) to LEFT JOIN labs on
@@ -1975,56 +2128,56 @@
 prerequisite, not a code bug). Shipped via PR #85.</t>
         </is>
       </c>
-      <c r="G24" s="2" t="inlineStr">
+      <c r="G27" s="3" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H24" s="2" t="inlineStr"/>
-    </row>
-    <row r="25" ht="90" customHeight="1">
-      <c r="A25" s="3" t="inlineStr">
+      <c r="H27" s="3" t="inlineStr"/>
+    </row>
+    <row r="28" ht="90" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>C14</t>
         </is>
       </c>
-      <c r="B25" s="3" t="inlineStr">
+      <c r="B28" s="2" t="inlineStr">
         <is>
           <t>UI relabel "CLIA TEa" -&gt; "Lab-Set Internal Goal" (formerly #1)</t>
         </is>
       </c>
-      <c r="C25" s="3" t="inlineStr"/>
-      <c r="D25" s="3" t="inlineStr"/>
-      <c r="E25" s="3" t="inlineStr"/>
-      <c r="F25" s="3" t="inlineStr">
+      <c r="C28" s="2" t="inlineStr"/>
+      <c r="D28" s="2" t="inlineStr"/>
+      <c r="E28" s="2" t="inlineStr"/>
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: Shipped across four PRs over 2026-05-10.</t>
         </is>
       </c>
-      <c r="G25" s="3" t="inlineStr">
+      <c r="G28" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H25" s="3" t="inlineStr"/>
-    </row>
-    <row r="26" ht="90" customHeight="1">
-      <c r="A26" s="2" t="inlineStr">
+      <c r="H28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29" ht="90" customHeight="1">
+      <c r="A29" s="3" t="inlineStr">
         <is>
           <t>C13</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="B29" s="3" t="inlineStr">
         <is>
           <t>WSLH PT vendor (formerly #15)</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr"/>
-      <c r="D26" s="2" t="inlineStr"/>
-      <c r="E26" s="2" t="inlineStr"/>
-      <c r="F26" s="2" t="inlineStr">
+      <c r="C29" s="3" t="inlineStr"/>
+      <c r="D29" s="3" t="inlineStr"/>
+      <c r="E29" s="3" t="inlineStr"/>
+      <c r="F29" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: Shipped 2026-05-10 via PR #79 (merge commit
 eeebc6e; merged after rebase to resolve a server/db.ts collision
@@ -2042,64 +2195,64 @@
 'WSLH' is the post-deploy success signal. Shipped via PR #79.</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr">
+      <c r="G29" s="3" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H26" s="2" t="inlineStr"/>
-    </row>
-    <row r="27" ht="90" customHeight="1">
-      <c r="A27" s="3" t="inlineStr">
+      <c r="H29" s="3" t="inlineStr"/>
+    </row>
+    <row r="30" ht="90" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>C15</t>
         </is>
       </c>
-      <c r="B27" s="3" t="inlineStr">
+      <c r="B30" s="2" t="inlineStr">
         <is>
           <t>VeritaStock lot tracking + expiration + reorder alerts (formerly #21)</t>
         </is>
       </c>
-      <c r="C27" s="3" t="inlineStr"/>
-      <c r="D27" s="3" t="inlineStr"/>
-      <c r="E27" s="3" t="inlineStr"/>
-      <c r="F27" s="3" t="inlineStr">
+      <c r="C30" s="2" t="inlineStr"/>
+      <c r="D30" s="2" t="inlineStr"/>
+      <c r="E30" s="2" t="inlineStr"/>
+      <c r="F30" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: VeritaStock™ shipped the bench-level inventory
 features the Perplexity competitor analysis identified as a gap:</t>
         </is>
       </c>
-      <c r="G27" s="3" t="inlineStr">
+      <c r="G30" s="2" t="inlineStr">
         <is>
           <t>Originally Perplexity competitor analysis 2026-05-10.
 Audit 2026-05-21 confirmed the feature set ships today.
 ---</t>
         </is>
       </c>
-      <c r="H27" s="3" t="inlineStr"/>
-    </row>
-    <row r="28" ht="90" customHeight="1">
-      <c r="A28" s="2" t="inlineStr">
+      <c r="H30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31" ht="90" customHeight="1">
+      <c r="A31" s="3" t="inlineStr">
         <is>
           <t>C16</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="B31" s="3" t="inlineStr">
         <is>
           <t>PAL studies guided workflow (formerly #23)</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr"/>
-      <c r="D28" s="2" t="inlineStr"/>
-      <c r="E28" s="2" t="inlineStr"/>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="C31" s="3" t="inlineStr"/>
+      <c r="D31" s="3" t="inlineStr"/>
+      <c r="E31" s="3" t="inlineStr"/>
+      <c r="F31" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: VeritaCheck™ already ships the Precision /
 Accuracy / Linearity (PAL) study set under EP-protocol naming:</t>
         </is>
       </c>
-      <c r="G28" s="2" t="inlineStr">
+      <c r="G31" s="3" t="inlineStr">
         <is>
           <t>Originally Perplexity competitor analysis 2026-05-10.
 Audit 2026-05-21 confirmed the EP studies cover the PAL framing in
@@ -2107,23 +2260,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H28" s="2" t="inlineStr"/>
-    </row>
-    <row r="29" ht="90" customHeight="1">
-      <c r="A29" s="3" t="inlineStr">
+      <c r="H31" s="3" t="inlineStr"/>
+    </row>
+    <row r="32" ht="90" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t>C17</t>
         </is>
       </c>
-      <c r="B29" s="3" t="inlineStr">
+      <c r="B32" s="2" t="inlineStr">
         <is>
           <t>Source-grounded 21/29/45 CFR + 42 CFR 482-485 (formerly #26)</t>
         </is>
       </c>
-      <c r="C29" s="3" t="inlineStr"/>
-      <c r="D29" s="3" t="inlineStr"/>
-      <c r="E29" s="3" t="inlineStr"/>
-      <c r="F29" s="3" t="inlineStr">
+      <c r="C32" s="2" t="inlineStr"/>
+      <c r="D32" s="2" t="inlineStr"/>
+      <c r="E32" s="2" t="inlineStr"/>
+      <c r="F32" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #301 (commit 8c27806, merged 2026-05-21)
 source-grounded the 74 remaining non-493 entries in
@@ -2131,29 +2284,29 @@
 shipped:</t>
         </is>
       </c>
-      <c r="G29" s="3" t="inlineStr">
+      <c r="G32" s="2" t="inlineStr">
         <is>
           <t>PR #301; tasks #18 in the in-session task tracker.
 ---</t>
         </is>
       </c>
-      <c r="H29" s="3" t="inlineStr"/>
-    </row>
-    <row r="30" ht="90" customHeight="1">
-      <c r="A30" s="2" t="inlineStr">
+      <c r="H32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33" ht="90" customHeight="1">
+      <c r="A33" s="3" t="inlineStr">
         <is>
           <t>C18</t>
         </is>
       </c>
-      <c r="B30" s="2" t="inlineStr">
+      <c r="B33" s="3" t="inlineStr">
         <is>
           <t>VeritaPolicy "Non CLIA" chapter rename (formerly #3)</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr"/>
-      <c r="D30" s="2" t="inlineStr"/>
-      <c r="E30" s="2" t="inlineStr"/>
-      <c r="F30" s="2" t="inlineStr">
+      <c r="C33" s="3" t="inlineStr"/>
+      <c r="D33" s="3" t="inlineStr"/>
+      <c r="E33" s="3" t="inlineStr"/>
+      <c r="F33" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #300 (commit 34d7707, merged 2026-05-21)
 renamed all 44 user-facing chapter labels in
@@ -2164,7 +2317,7 @@
 page.</t>
         </is>
       </c>
-      <c r="G30" s="2" t="inlineStr">
+      <c r="G33" s="3" t="inlineStr">
         <is>
           <t>CAP customer screenshot of the /veritapolicy chapter
 headers, 2026-05-01 evening. PR #300; tasks #17 in the in-session
@@ -2172,23 +2325,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H30" s="2" t="inlineStr"/>
-    </row>
-    <row r="31" ht="90" customHeight="1">
-      <c r="A31" s="3" t="inlineStr">
+      <c r="H33" s="3" t="inlineStr"/>
+    </row>
+    <row r="34" ht="90" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
         <is>
           <t>C19</t>
         </is>
       </c>
-      <c r="B31" s="3" t="inlineStr">
+      <c r="B34" s="2" t="inlineStr">
         <is>
           <t>VeritaStock department-scope toggle (formerly #31)</t>
         </is>
       </c>
-      <c r="C31" s="3" t="inlineStr"/>
-      <c r="D31" s="3" t="inlineStr"/>
-      <c r="E31" s="3" t="inlineStr"/>
-      <c r="F31" s="3" t="inlineStr">
+      <c r="C34" s="2" t="inlineStr"/>
+      <c r="D34" s="2" t="inlineStr"/>
+      <c r="E34" s="2" t="inlineStr"/>
+      <c r="F34" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #319 (commit d01f5fe, merged 2026-05-22)
 shipped the persistent dept-scope toggle on VeritaStockPage. A new
@@ -2199,7 +2352,7 @@
 workspace without re-filtering.</t>
         </is>
       </c>
-      <c r="G31" s="3" t="inlineStr">
+      <c r="G34" s="2" t="inlineStr">
         <is>
           <t>John, San Carlos lab, 2026-05-21. Same conversation that
 drove the vendor dropdown (PR #304), FILTERED VIEW banner (PR #305),
@@ -2207,23 +2360,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H31" s="3" t="inlineStr"/>
-    </row>
-    <row r="32" ht="90" customHeight="1">
-      <c r="A32" s="2" t="inlineStr">
+      <c r="H34" s="2" t="inlineStr"/>
+    </row>
+    <row r="35" ht="90" customHeight="1">
+      <c r="A35" s="3" t="inlineStr">
         <is>
           <t>C20</t>
         </is>
       </c>
-      <c r="B32" s="2" t="inlineStr">
+      <c r="B35" s="3" t="inlineStr">
         <is>
           <t>Primary-lab seat counting (formerly #12)</t>
         </is>
       </c>
-      <c r="C32" s="2" t="inlineStr"/>
-      <c r="D32" s="2" t="inlineStr"/>
-      <c r="E32" s="2" t="inlineStr"/>
-      <c r="F32" s="2" t="inlineStr">
+      <c r="C35" s="3" t="inlineStr"/>
+      <c r="D35" s="3" t="inlineStr"/>
+      <c r="E35" s="3" t="inlineStr"/>
+      <c r="F35" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: is_primary_lab INTEGER NOT NULL DEFAULT 0
 column was added to the lab_members table at db.ts:1276, with the
@@ -2234,7 +2387,7 @@
 is_primary_lab=1 ordering).</t>
         </is>
       </c>
-      <c r="G32" s="2" t="inlineStr">
+      <c r="G35" s="3" t="inlineStr">
         <is>
           <t>2026-05-07 multi-lab discussion. Build shipped as part
 of the Multi-Lab Tier 2 architecture work (Phase 3.x series, prior
@@ -2243,23 +2396,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H32" s="2" t="inlineStr"/>
-    </row>
-    <row r="33" ht="90" customHeight="1">
-      <c r="A33" s="3" t="inlineStr">
+      <c r="H35" s="3" t="inlineStr"/>
+    </row>
+    <row r="36" ht="90" customHeight="1">
+      <c r="A36" s="2" t="inlineStr">
         <is>
           <t>C21</t>
         </is>
       </c>
-      <c r="B33" s="3" t="inlineStr">
+      <c r="B36" s="2" t="inlineStr">
         <is>
           <t>Multi-lab pricing model — Option A (formerly #11)</t>
         </is>
       </c>
-      <c r="C33" s="3" t="inlineStr"/>
-      <c r="D33" s="3" t="inlineStr"/>
-      <c r="E33" s="3" t="inlineStr"/>
-      <c r="F33" s="3" t="inlineStr">
+      <c r="C36" s="2" t="inlineStr"/>
+      <c r="D36" s="2" t="inlineStr"/>
+      <c r="E36" s="2" t="inlineStr"/>
+      <c r="F36" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #322 (commit 0ccd925, merged 2026-05-22)
 added the customer-facing line to the pricing page that reflects
@@ -2272,7 +2425,7 @@
 Enterprise+ block, reads:</t>
         </is>
       </c>
-      <c r="G33" s="3" t="inlineStr">
+      <c r="G36" s="2" t="inlineStr">
         <is>
           <t>2026-05-07 multi-lab discussion (Lisa Veri's
 canonical-case session). PR #322 (initial build); softening PR
@@ -2281,30 +2434,30 @@
 ---</t>
         </is>
       </c>
-      <c r="H33" s="3" t="inlineStr"/>
-    </row>
-    <row r="34" ht="90" customHeight="1">
-      <c r="A34" s="2" t="inlineStr">
+      <c r="H36" s="2" t="inlineStr"/>
+    </row>
+    <row r="37" ht="90" customHeight="1">
+      <c r="A37" s="3" t="inlineStr">
         <is>
           <t>C22</t>
         </is>
       </c>
-      <c r="B34" s="2" t="inlineStr">
+      <c r="B37" s="3" t="inlineStr">
         <is>
           <t>VeritaOps cost-per-test module (formerly #10)</t>
         </is>
       </c>
-      <c r="C34" s="2" t="inlineStr"/>
-      <c r="D34" s="2" t="inlineStr"/>
-      <c r="E34" s="2" t="inlineStr"/>
-      <c r="F34" s="2" t="inlineStr">
+      <c r="C37" s="3" t="inlineStr"/>
+      <c r="D37" s="3" t="inlineStr"/>
+      <c r="E37" s="3" t="inlineStr"/>
+      <c r="F37" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: v1 of the VeritaOps Cost-Per-Reportable-Test
 (CPRT) module shipped across PR #325 through PR #330 on 2026-05-22.
 The module is feature-complete for the typical lab director workflow.</t>
         </is>
       </c>
-      <c r="G34" s="2" t="inlineStr">
+      <c r="G37" s="3" t="inlineStr">
         <is>
           <t>This thread, 2026-05-07 12:05 PM CDT, user message:
 "Parking lot: build an operations module for cost per test
@@ -2313,262 +2466,262 @@
 ---</t>
         </is>
       </c>
-      <c r="H34" s="2" t="inlineStr"/>
-    </row>
-    <row r="35" ht="90" customHeight="1">
-      <c r="A35" s="3" t="inlineStr">
+      <c r="H37" s="3" t="inlineStr"/>
+    </row>
+    <row r="38" ht="90" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
         <is>
           <t>C23</t>
         </is>
       </c>
-      <c r="B35" s="3" t="inlineStr">
+      <c r="B38" s="2" t="inlineStr">
         <is>
           <t>CCL lab name visual disambiguation in lab switcher (formerly #34)</t>
         </is>
       </c>
-      <c r="C35" s="3" t="inlineStr"/>
-      <c r="D35" s="3" t="inlineStr">
+      <c r="C38" s="2" t="inlineStr"/>
+      <c r="D38" s="2" t="inlineStr">
         <is>
           <t>XS (under 1 day, actual)</t>
         </is>
       </c>
-      <c r="E35" s="3" t="inlineStr">
+      <c r="E38" s="2" t="inlineStr">
         <is>
           <t>Low — cosmetic; only mattered when Lisa or Michael picked the wrong lab from...</t>
         </is>
       </c>
-      <c r="F35" s="3" t="inlineStr">
+      <c r="F38" s="2" t="inlineStr">
         <is>
           <t>Effort: XS (under 1 day, actual)
 Importance: Low — cosmetic; only mattered when Lisa or Michael picked the wrong lab from the dropdown.</t>
         </is>
       </c>
-      <c r="G35" s="3" t="inlineStr">
+      <c r="G38" s="2" t="inlineStr">
         <is>
           <t>flagged 2026-05-23 immediately after provisioning Lisa's CCL lab; closed 2026-05-24.
 ---</t>
         </is>
       </c>
-      <c r="H35" s="3" t="inlineStr"/>
-    </row>
-    <row r="36" ht="90" customHeight="1">
-      <c r="A36" s="2" t="inlineStr">
+      <c r="H38" s="2" t="inlineStr"/>
+    </row>
+    <row r="39" ht="90" customHeight="1">
+      <c r="A39" s="3" t="inlineStr">
         <is>
           <t>C24</t>
         </is>
       </c>
-      <c r="B36" s="2" t="inlineStr">
+      <c r="B39" s="3" t="inlineStr">
         <is>
           <t>VC Unlimited Y1/Y2 price disclosure UX (formerly #35)</t>
         </is>
       </c>
-      <c r="C36" s="2" t="inlineStr"/>
-      <c r="D36" s="2" t="inlineStr">
+      <c r="C39" s="3" t="inlineStr"/>
+      <c r="D39" s="3" t="inlineStr">
         <is>
           <t>XS (under 1 day, actual)</t>
         </is>
       </c>
-      <c r="E36" s="2" t="inlineStr">
+      <c r="E39" s="3" t="inlineStr">
         <is>
           <t>Low when shipped (proactive, no customer complaint yet) — but high if a procu...</t>
         </is>
       </c>
-      <c r="F36" s="2" t="inlineStr">
+      <c r="F39" s="3" t="inlineStr">
         <is>
           <t>Effort: XS (under 1 day, actual)
 Importance: Low when shipped (proactive, no customer complaint yet) — but high if a procurement reviewer later disputes the $499 renewal as undisclosed.</t>
         </is>
       </c>
-      <c r="G36" s="2" t="inlineStr">
+      <c r="G39" s="3" t="inlineStr">
         <is>
           <t>Pricing rebuild 2026-05-23; closed 2026-05-24 proactively before any customer dispute.
 ---</t>
         </is>
       </c>
-      <c r="H36" s="2" t="inlineStr"/>
-    </row>
-    <row r="37" ht="90" customHeight="1">
-      <c r="A37" s="3" t="inlineStr">
+      <c r="H39" s="3" t="inlineStr"/>
+    </row>
+    <row r="40" ht="90" customHeight="1">
+      <c r="A40" s="2" t="inlineStr">
         <is>
           <t>C25</t>
         </is>
       </c>
-      <c r="B37" s="3" t="inlineStr">
+      <c r="B40" s="2" t="inlineStr">
         <is>
           <t>VeritaQC Phase 1 (Levey-Jennings + Westgard live engine) (formerly #20)</t>
         </is>
       </c>
-      <c r="C37" s="3" t="inlineStr"/>
-      <c r="D37" s="3" t="inlineStr">
+      <c r="C40" s="2" t="inlineStr"/>
+      <c r="D40" s="2" t="inlineStr">
         <is>
           <t>L (about 5 days end-to-end, actual: Phase 0 schema → Phase 1A evaluator → 1B...</t>
         </is>
       </c>
-      <c r="E37" s="3" t="inlineStr">
+      <c r="E40" s="2" t="inlineStr">
         <is>
           <t>High — largest single gap vs myLabCompliance.io per Perplexity competitor ana...</t>
         </is>
       </c>
-      <c r="F37" s="3" t="inlineStr">
+      <c r="F40" s="2" t="inlineStr">
         <is>
           <t>Effort: L (about 5 days end-to-end, actual: Phase 0 schema → Phase 1A evaluator → 1B entry UI → 1C daily review → 1D monthly PDF + attestation)
 Importance: High — largest single gap vs myLabCompliance.io per Perplexity competitor analysis; promotes VeritaAssure from documentation tool to lab operations platform.</t>
         </is>
       </c>
-      <c r="G37" s="3" t="inlineStr">
+      <c r="G40" s="2" t="inlineStr">
         <is>
           <t>Perplexity competitor analysis 2026-05-10. Scoping confirmed via the build_phase1_mockup.py iterations 2026-05-24. Shipped 2026-05-25.
 ---</t>
         </is>
       </c>
-      <c r="H37" s="3" t="inlineStr"/>
-    </row>
-    <row r="38" ht="90" customHeight="1">
-      <c r="A38" s="2" t="inlineStr">
+      <c r="H40" s="2" t="inlineStr"/>
+    </row>
+    <row r="41" ht="90" customHeight="1">
+      <c r="A41" s="3" t="inlineStr">
         <is>
           <t>C26</t>
         </is>
       </c>
-      <c r="B38" s="2" t="inlineStr">
+      <c r="B41" s="3" t="inlineStr">
         <is>
           <t>VeritaLab CMS-116 application support + state licensing registry (formerly #22)</t>
         </is>
       </c>
-      <c r="C38" s="2" t="inlineStr"/>
-      <c r="D38" s="2" t="inlineStr">
+      <c r="C41" s="3" t="inlineStr"/>
+      <c r="D41" s="3" t="inlineStr">
         <is>
           <t>M (1-2 weeks for v1, actual)</t>
         </is>
       </c>
-      <c r="E38" s="2" t="inlineStr">
+      <c r="E41" s="3" t="inlineStr">
         <is>
           <t>Medium — competitor parity (myLabCompliance.io) plus useful at lab startup an...</t>
         </is>
       </c>
-      <c r="F38" s="2" t="inlineStr">
+      <c r="F41" s="3" t="inlineStr">
         <is>
           <t>Effort: M (1-2 weeks for v1, actual)
 Importance: Medium — competitor parity (myLabCompliance.io) plus useful at lab startup and at certificate-type changes.</t>
         </is>
       </c>
-      <c r="G38" s="2" t="inlineStr">
+      <c r="G41" s="3" t="inlineStr">
         <is>
           <t>Perplexity competitor analysis (myLabCompliance.io), 2026-05-10. Reclassified as a VeritaLab extension 2026-05-25. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H38" s="2" t="inlineStr"/>
-    </row>
-    <row r="39" ht="90" customHeight="1">
-      <c r="A39" s="3" t="inlineStr">
+      <c r="H41" s="3" t="inlineStr"/>
+    </row>
+    <row r="42" ht="90" customHeight="1">
+      <c r="A42" s="2" t="inlineStr">
         <is>
           <t>C27</t>
         </is>
       </c>
-      <c r="B39" s="3" t="inlineStr">
+      <c r="B42" s="2" t="inlineStr">
         <is>
           <t>Active vs view-only seat split (formerly #33)</t>
         </is>
       </c>
-      <c r="C39" s="3" t="inlineStr"/>
-      <c r="D39" s="3" t="inlineStr">
+      <c r="C42" s="2" t="inlineStr"/>
+      <c r="D42" s="2" t="inlineStr">
         <is>
           <t>M (~1 week of engineering, actual: shipped in a single multi-PR session)</t>
         </is>
       </c>
-      <c r="E39" s="3" t="inlineStr">
+      <c r="E42" s="2" t="inlineStr">
         <is>
           <t>Medium — closed the gap between /pricing copy and product behavior; gives sal...</t>
         </is>
       </c>
-      <c r="F39" s="3" t="inlineStr">
+      <c r="F42" s="2" t="inlineStr">
         <is>
           <t>Effort: M (~1 week of engineering, actual: shipped in a single multi-PR session)
 Importance: Medium — closed the gap between /pricing copy and product behavior; gives sales a clean answer for "do you charge for our medical director?"</t>
         </is>
       </c>
-      <c r="G39" s="3" t="inlineStr">
+      <c r="G42" s="2" t="inlineStr">
         <is>
           <t>Pricing analysis doc Decision 3 (2026-05-21); MEDIUM scenario revised 2026-05-29 to retire the "unlimited view-only" claim. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H39" s="3" t="inlineStr"/>
-    </row>
-    <row r="40" ht="90" customHeight="1">
-      <c r="A40" s="2" t="inlineStr">
+      <c r="H42" s="2" t="inlineStr"/>
+    </row>
+    <row r="43" ht="90" customHeight="1">
+      <c r="A43" s="3" t="inlineStr">
         <is>
           <t>C28</t>
         </is>
       </c>
-      <c r="B40" s="2" t="inlineStr">
+      <c r="B43" s="3" t="inlineStr">
         <is>
           <t>"Why VeritaCheck" comparative one-pager (formerly #37)</t>
         </is>
       </c>
-      <c r="C40" s="2" t="inlineStr"/>
-      <c r="D40" s="2" t="inlineStr">
+      <c r="C43" s="3" t="inlineStr"/>
+      <c r="D43" s="3" t="inlineStr">
         <is>
           <t>S (one design pass + four claim paragraphs + PDF + matching marketing-site pa...</t>
         </is>
       </c>
-      <c r="E40" s="2" t="inlineStr">
+      <c r="E43" s="3" t="inlineStr">
         <is>
           <t>Medium — closed a positioning gap surfaced by six COLA conference attendees a...</t>
         </is>
       </c>
-      <c r="F40" s="2" t="inlineStr">
+      <c r="F43" s="3" t="inlineStr">
         <is>
           <t>Effort: S (one design pass + four claim paragraphs + PDF + matching marketing-site page, actual)
 Importance: Medium — closed a positioning gap surfaced by six COLA conference attendees attached to a legacy verification tool; converts product-quality advantage into a leave-behind Lisa can hand out.</t>
         </is>
       </c>
-      <c r="G40" s="2" t="inlineStr">
+      <c r="G43" s="3" t="inlineStr">
         <is>
           <t>2026-05-11 / 2026-05-12 conference notes review with Michael. Conference attendees (Whitehead, Odegard, Othman, Molinelli, Kyle, Allred) expressed interest in equivalent / superior product. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H40" s="2" t="inlineStr"/>
-    </row>
-    <row r="41" ht="90" customHeight="1">
-      <c r="A41" s="3" t="inlineStr">
+      <c r="H43" s="3" t="inlineStr"/>
+    </row>
+    <row r="44" ht="90" customHeight="1">
+      <c r="A44" s="2" t="inlineStr">
         <is>
           <t>C29</t>
         </is>
       </c>
-      <c r="B41" s="3" t="inlineStr">
+      <c r="B44" s="2" t="inlineStr">
         <is>
           <t>VeritaPolicy approval workflow — MediaLab functional mirror</t>
         </is>
       </c>
-      <c r="C41" s="3" t="inlineStr"/>
-      <c r="D41" s="3" t="inlineStr">
+      <c r="C44" s="2" t="inlineStr"/>
+      <c r="D44" s="2" t="inlineStr">
         <is>
           <t>XL (one focused session, 12 PRs landed)</t>
         </is>
       </c>
-      <c r="E41" s="3" t="inlineStr">
+      <c r="E44" s="2" t="inlineStr">
         <is>
           <t>High — replaces MediaLab Document Control ($752/$2,250 starting price, scalin...</t>
         </is>
       </c>
-      <c r="F41" s="3" t="inlineStr">
+      <c r="F44" s="2" t="inlineStr">
         <is>
           <t>Effort: XL (one focused session, 12 PRs landed)
 Importance: High — replaces MediaLab Document Control ($752/$2,250 starting price, scaling to $10K-$20K/yr at enterprise per Capterra public data) with an included VeritaPolicy feature; closes a real positioning gap and gives sales a direct comparator line.</t>
         </is>
       </c>
-      <c r="G41" s="3" t="inlineStr">
+      <c r="G44" s="2" t="inlineStr">
         <is>
           <t>Pricing strategy conversation 2026-05-29 (Michael: "I don't like bolt-ons; we should replicate this") → scoped 8 phases → shipped all 12 PRs in single session. Shipped 2026-05-29.
 ---</t>
         </is>
       </c>
-      <c r="H41" s="3" t="inlineStr"/>
+      <c r="H44" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H41"/>
+  <autoFilter ref="A1:H44"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
TASK: Parking-lot sync 2026-09-24 pass 2 (C41-C43 closed, #49-#50 open)
PLAN:
  1. CLOSED C41 (coverage recurrence #1317/#1318/#1321), C42 (VeritaComp coverage map #1319/#1316), C43 (VeritaStaff dual view #1320).
  2. OPEN #49 (shared recurrence helper), #50 (competency assessed-cycle window).
  3. Regenerate xlsx.

Self-check:
  - OPEN 15->17; CLOSED 40->43.
  - Closures cite PRs + live verification.
</commit_message>
<xml_diff>
--- a/PARKING_LOT.xlsx
+++ b/PARKING_LOT.xlsx
@@ -12,8 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RETIRED" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$44</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RETIRED'!$A$1:$H$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1212,8 +1212,80 @@
       </c>
       <c r="H16" s="2" t="inlineStr"/>
     </row>
+    <row r="17" ht="90" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Unify the coverage/competency recurrence into one shared helper (tech debt)</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr"/>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>S (a few hours) - extract "latest study/assessment -&gt; status / nextDueOn / ov...</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Low - the three paths duplicate the +6-month / signed-resets-to-missing logic...</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Effort: S (a few hours) - extract "latest study/assessment -&gt; status / nextDueOn / overdue" into one helper used by method comparison, cal-ver/linearity, and the competency owed derivation.
+Importance: Low - the three paths duplicate the +6-month / signed-resets-to-missing logic. They agree today (verified), but a shared helper prevents future drift and settles the dateless-signed edge in one place. No user-facing impact; studies.date is NOT NULL so the one known divergence is unreachable in practice.</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-24 session, surfaced during the coverage-recurrence build. No live defect; hygiene.
+---</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr"/>
+    </row>
+    <row r="18" ht="90" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Competency "assessed this cycle" uses a flat 365-day window</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr"/>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>S-M - anchor the coverage-map "assessed this cycle" to the person's actual CL...</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Medium - in an employee's first year the semiannual windows differ from a fla...</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Effort: S-M - anchor the coverage-map "assessed this cycle" to the person's actual CLIA cadence (semiannual in year 1 per 42 CFR 493.1451(b)(8), annual thereafter) from staff_competency_schedules, instead of the v1 flat 365-day lookback.
+Importance: Medium - in an employee's first year the semiannual windows differ from a flat annual window, so a first-year assessment could read as current slightly longer or shorter than the true cadence. Fine for the common annual case; refine for year-1 accuracy.</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24 session, VeritaComp coverage map (#48 Phase 3) v1 simplification, noted in PR #1319.
+---</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H16"/>
+  <autoFilter ref="A1:H18"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1224,7 +1296,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H41"/>
+  <dimension ref="A1:H44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1282,12 +1354,12 @@
     <row r="2" ht="90" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>C40</t>
+          <t>C43</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>VeritaComp Competencies Owed derived from VeritaStaff, with gap detection (was #48)</t>
+          <t>VeritaStaff instrument-centric (dual) assignment view</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr"/>
@@ -1295,12 +1367,12 @@
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1314 (squash 2bcb0db9). GET /api/labs/:labId/competency/owed derives each VeritaStaff testing employee's owed competencies from their assigned instruments (staff_employee_instruments -&gt; veritamap_instruments + tests), on the CLIA timeline, and flags instruments not covered by any competency program as gaps. CompetenciesOwedSection renders it on the VeritaComp landing page. Reuses the shipped bridge + suggested-method-groups match rules; no new tables. Verified live on prod with real assignment data: 2 instruments assigned to a demo staffer produced owed=2, gaps=2 (HIGH, Technical Supervisor), then reverted cleanly. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1320. GET/PUT /staff/instruments/:id/employees (transpose of the per-employee endpoints); an "Assign by Instrument" dialog lets a director pick a test system or manual test and check off who runs it. Same staff_employee_instruments join, with the 42 CFR 493.1235(a) duty-change event emitted on newly-added pairs so both orientations trigger the same reassessment. GET verified live on SCAHC lab 2. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23/24 session, Michael ("veritacomp bases what competencies they owe (currently untrue, but needs to be true)"). Option 1 (unify roster on VeritaStaff, match instruments by id).
+          <t>2026-09-24 session, Michael ("in staff we should also give the dual view when assigning coverage to test systems or manual tests").
 ---</t>
         </is>
       </c>
@@ -1309,12 +1381,12 @@
     <row r="3" ht="90" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>C39</t>
+          <t>C42</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>VeritaScan line items can attach or link evidence (was #46)</t>
+          <t>VeritaComp coverage map (required-vs-assessed matrix, dual view)</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr"/>
@@ -1322,12 +1394,12 @@
       <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1312 (squash a1dda93d). VeritaScan scan checklist items now show linked evidence as chips (open link, remove) plus a writer "Link evidence" affordance whose picker links an existing VeritaDC/Library document; a shortcut deep-links to the Library for new (governed) documents. Reuses the already-shipped lab_documents + document_checklist_links + coverage endpoints (URL-pointer only, no file storage, no new tables). Browser-verified live on prod (scan 23): the affordance renders and the picker opens. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1319 (+ status layer PR #1316). /competency/owed returns per-item assessed (locked passing assessment this cycle on a covering method group) + per-employee CLIA status; CompetencyCoverageMap renders a By-employee / By-instrument matrix (Assessed / Owed / Overdue / Gap). Verified live on SCAHC lab 2 (owed 116, assessed 2, gaps 0). Completes #48 as the VeritaCheck-parity coverage map. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>2026-09-23 session, Michael. Recurring request. Companion: cross-module evidence display on the VeritaDC policy shipped in PR #1313 (by-target cross-links surfaced in the policy View modal, browser-verified live).
+          <t>2026-09-24 session, Michael ("are we building the competencies to have a coverage map, same as veritacheck?" then "build it").
 ---</t>
         </is>
       </c>
@@ -1336,12 +1408,12 @@
     <row r="4" ht="90" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>C38</t>
+          <t>C41</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>VeritaTrack calendar month cells expand to reveal hidden tasks (was #45)</t>
+          <t>VeritaCheck coverage recurrence (method comparison + cal-ver/linearity + reports)</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr"/>
@@ -1349,12 +1421,12 @@
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: VeritaTrack CalendarView month cells with more than three tasks now expand in place (chevron, "+N more" toggling to "Show less", due dates), so no task is hidden with no path to it (client/src/pages/VeritaTrackAppPage.tsx CalendarView). Shipped 2026-09-23. Closed 2026-09-24.</t>
+          <t>Closure evidence: PRs #1317 (method comparison), #1318 (cal-ver/linearity), #1321 (report Next-due columns). Periodic verification (correlation/method comparison 42 CFR 493.1281; cal-ver/linearity 42 CFR 493.1255; both 6-month) now recurs: a signed study banks the cycle and rolls to next-due = signed + 6 months instead of reading "done" forever. Status Missing/Failed/Completed-unsigned + a "Next due on" column on-screen and in both coverage exports; also credits the previously-ignored "correlation" study type. Root cause: computeCoverageFrom marked requirements done on mere existence, no date logic. Verified live on SCAHC lab 2 (101 correlations + 11 cal-ver rows now carry a next-due). Engine-level, all facilities. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23 session, Michael screenshot of the VeritaTrack calendar (lab 3, September cell).
+          <t>2026-09-24 session, Michael ("Look at San Carlos... they finished their last set of correlations (all 103) but their menu never reset").
 ---</t>
         </is>
       </c>
@@ -1363,12 +1435,12 @@
     <row r="5" ht="90" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>C37</t>
+          <t>C40</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Long Excel column headers no longer clip CFR citations (was #44)</t>
+          <t>VeritaComp Competencies Owed derived from VeritaStaff, with gap detection (was #48)</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr"/>
@@ -1376,12 +1448,12 @@
       <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. The VeritaMap export derives the header row height from the longest wrapped header via headerRowHeight(headers, colWidths) (server/routes.ts:15935) instead of a fixed 20, so "Reference Range Attestation (42 CFR 493.1253)" and the other long headers print in full. No new code this session. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1314 (squash 2bcb0db9). GET /api/labs/:labId/competency/owed derives each VeritaStaff testing employee's owed competencies from their assigned instruments (staff_employee_instruments -&gt; veritamap_instruments + tests), on the CLIA timeline, and flags instruments not covered by any competency program as gaps. CompetenciesOwedSection renders it on the VeritaComp landing page. Reuses the shipped bridge + suggested-method-groups match rules; no new tables. Verified live on prod with real assignment data: 2 instruments assigned to a demo staffer produced owed=2, gaps=2 (HIGH, Technical Supervisor), then reverted cleanly. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+          <t>2026-09-23/24 session, Michael ("veritacomp bases what competencies they owe (currently untrue, but needs to be true)"). Option 1 (unify roster on VeritaStaff, match instruments by id).
 ---</t>
         </is>
       </c>
@@ -1390,12 +1462,12 @@
     <row r="6" ht="90" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>C36</t>
+          <t>C39</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>License stamp no longer clobbers the §6 header/footer or names the wrong lab (was #43)</t>
+          <t>VeritaScan line items can attach or link evidence (was #46)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr"/>
@@ -1403,12 +1475,12 @@
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. setHeaderFooter (shared/licenseExceljs.ts:155-209) now preserves an existing §6 header and appends (not overwrites) the footer left section, and customer-facing exports name the scoped lab: the VeritaScan library export reads req.scope.lab.name / clia_number (server/routes.ts:16572-16573), not the licensee. No new code this session (avoided regressing the existing fix). Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1312 (squash a1dda93d). VeritaScan scan checklist items now show linked evidence as chips (open link, remove) plus a writer "Link evidence" affordance whose picker links an existing VeritaDC/Library document; a shortcut deep-links to the Library for new (governed) documents. Reuses the already-shipped lab_documents + document_checklist_links + coverage endpoints (URL-pointer only, no file storage, no new tables). Browser-verified live on prod (scan 23): the affordance renders and the picker opens. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+          <t>2026-09-23 session, Michael. Recurring request. Companion: cross-module evidence display on the VeritaDC policy shipped in PR #1313 (by-target cross-links surfaced in the policy View modal, browser-verified live).
 ---</t>
         </is>
       </c>
@@ -1417,18 +1489,99 @@
     <row r="7" ht="90" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>C34</t>
+          <t>C38</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Wire the two static-audit guards into CI (was #43)</t>
+          <t>VeritaTrack calendar month cells expand to reveal hidden tasks (was #45)</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr"/>
       <c r="D7" s="3" t="inlineStr"/>
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Closure evidence: VeritaTrack CalendarView month cells with more than three tasks now expand in place (chevron, "+N more" toggling to "Show less", due dates), so no task is hidden with no path to it (client/src/pages/VeritaTrackAppPage.tsx CalendarView). Shipped 2026-09-23. Closed 2026-09-24.</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-23 session, Michael screenshot of the VeritaTrack calendar (lab 3, September cell).
+---</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr"/>
+    </row>
+    <row r="8" ht="90" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>C37</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Long Excel column headers no longer clip CFR citations (was #44)</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr"/>
+      <c r="D8" s="2" t="inlineStr"/>
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. The VeritaMap export derives the header row height from the longest wrapped header via headerRowHeight(headers, colWidths) (server/routes.ts:15935) instead of a fixed 20, so "Reference Range Attestation (42 CFR 493.1253)" and the other long headers print in full. No new code this session. Closed 2026-09-24.</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+---</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9" ht="90" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>C36</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>License stamp no longer clobbers the §6 header/footer or names the wrong lab (was #43)</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr"/>
+      <c r="D9" s="3" t="inlineStr"/>
+      <c r="E9" s="3" t="inlineStr"/>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. setHeaderFooter (shared/licenseExceljs.ts:155-209) now preserves an existing §6 header and appends (not overwrites) the footer left section, and customer-facing exports name the scoped lab: the VeritaScan library export reads req.scope.lab.name / clia_number (server/routes.ts:16572-16573), not the licensee. No new code this session (avoided regressing the existing fix). Closed 2026-09-24.</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+---</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr"/>
+    </row>
+    <row r="10" ht="90" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>C34</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Wire the two static-audit guards into CI (was #43)</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr"/>
+      <c r="D10" s="2" t="inlineStr"/>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: both guards wired into the Multi-Lab Mutations Audit CI
 workflow (.github/workflows/multilab-mutations-audit.yml) as steps:
@@ -1440,24 +1593,24 @@
 (same caveat as the existing guards already in that workflow).</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr"/>
-      <c r="H7" s="3" t="inlineStr"/>
-    </row>
-    <row r="8" ht="90" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11" ht="90" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>C35</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>Legacy /api/studies over-returns studies across labs (was #44)</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr"/>
-      <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr"/>
+      <c r="D11" s="3" t="inlineStr"/>
+      <c r="E11" s="3" t="inlineStr"/>
+      <c r="F11" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: GET /api/studies now scopes its list to the active lab
 when one is resolved from the Referer (server/routes.ts), so every returned row
@@ -1467,24 +1620,24 @@
 mirroring the /api/labs/:labId/studies handler. Closed 2026-06-14.</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr"/>
-      <c r="H8" s="2" t="inlineStr"/>
-    </row>
-    <row r="9" ht="90" customHeight="1">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="G11" s="3" t="inlineStr"/>
+      <c r="H11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12" ht="90" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>C30</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>Verify-script convention backfill (was #41)</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr"/>
-      <c r="D9" s="3" t="inlineStr"/>
-      <c r="E9" s="3" t="inlineStr"/>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr"/>
+      <c r="D12" s="2" t="inlineStr"/>
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: all 8 high-stakes math/logic commits now ship a paired
 scripts/verify-*.js (EP17 sensitivity, Deming lot-to-lot, CUMSUM+QC+multi-analyte,
@@ -1492,30 +1645,30 @@
 TEa boundary), per the strike-throughs in #41. Closed 2026-06-13.</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>scripts/audit_verify_script_coverage.py lookback, 2026-06-02; backfills
 landed 2026-06-03..06.
 ---</t>
         </is>
       </c>
-      <c r="H9" s="3" t="inlineStr"/>
-    </row>
-    <row r="10" ht="90" customHeight="1">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13" ht="90" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>C31</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>VeritaPT AAA create/update/delete silently no-op in the multi-lab UI</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr"/>
-      <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr"/>
+      <c r="D13" s="3" t="inlineStr"/>
+      <c r="E13" s="3" t="inlineStr"/>
+      <c r="F13" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #754 (commit 92ad499) added lab-scoped POST/PUT/DELETE
 /api/labs/:labId/pt/aa-records. The UI posted to the lab-scoped path but only GET
@@ -1526,30 +1679,30 @@
 route mis-filed records to the user's default lab on multi-lab accounts).</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G13" s="3" t="inlineStr">
         <is>
           <t>2026-06-13, found during #18 Phase 3 QA;
 scripts/audit-labscoped-write-routes.mjs now guards the class.
 ---</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr"/>
-    </row>
-    <row r="11" ht="90" customHeight="1">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="H13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14" ht="90" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>C32</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>VeritaComp "Unlock assessment" false-success no-op</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr"/>
-      <c r="D11" s="3" t="inlineStr"/>
-      <c r="E11" s="3" t="inlineStr"/>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr"/>
+      <c r="D14" s="2" t="inlineStr"/>
+      <c r="E14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #755 (commit 4234007) moved the unlock route to
 /api/labs/:labId/competency/assessments/:id/unlock (the path the client calls).
@@ -1560,29 +1713,29 @@
 HTML).</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>2026-06-13, found by scripts/audit-labscoped-write-routes.mjs.
 ---</t>
         </is>
       </c>
-      <c r="H11" s="3" t="inlineStr"/>
-    </row>
-    <row r="12" ht="90" customHeight="1">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="H14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15" ht="90" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>C33</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>FK-cascade delete 500s + NavBar laptop-width overflow</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr"/>
-      <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="2" t="inlineStr"/>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr"/>
+      <c r="D15" s="3" t="inlineStr"/>
+      <c r="E15" s="3" t="inlineStr"/>
+      <c r="F15" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PRs #749/#750 fixed NavBar horizontal overflow at laptop
 widths (collapse to the hamburger below 1560px); prod-verified at 1280-1920 with the
@@ -1593,57 +1746,57 @@
 500 -&gt; 200. scripts/audit-delete-cascades.mjs guards the class.</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G15" s="3" t="inlineStr">
         <is>
           <t>2026-06-13 browser QA of the A7-D4 wave + retro-QC of the 72h PR window.
 ---</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr"/>
-    </row>
-    <row r="13" ht="90" customHeight="1">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="H15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16" ht="90" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>C1</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>FAQ "over 25 years" -&gt; "over 23 years"</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr"/>
-      <c r="D13" s="3" t="inlineStr"/>
-      <c r="E13" s="3" t="inlineStr"/>
-      <c r="F13" s="3" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr"/>
+      <c r="D16" s="2" t="inlineStr"/>
+      <c r="E16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: client/src/pages/FAQPage.tsx line 20 reads "over
 23 years" as of 2026-05-01.</t>
         </is>
       </c>
-      <c r="G13" s="3" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>session 299e9a73 turn 14, ~2026-04-28.
 ---</t>
         </is>
       </c>
-      <c r="H13" s="3" t="inlineStr"/>
-    </row>
-    <row r="14" ht="90" customHeight="1">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="H16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17" ht="90" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>C5</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>David's VeritaQA grey-button bug (seat permissions mode)</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr"/>
-      <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="2" t="inlineStr"/>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr"/>
+      <c r="D17" s="3" t="inlineStr"/>
+      <c r="E17" s="3" t="inlineStr"/>
+      <c r="F17" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #10 squash-merged as commit a43fbba on
 2026-05-01 23:19 MST. Railway deploy succeeded; deployed bundle
@@ -1656,7 +1809,7 @@
 against his exact stored shape (14 of 14 expected outcomes matched).</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="G17" s="3" t="inlineStr">
         <is>
           <t>2026-05-01 David's report; veritabench + veritastock
 weren't in MODULE_LIST so seat permissions silently defaulted to
@@ -1664,109 +1817,109 @@
 ---</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr"/>
-    </row>
-    <row r="15" ht="90" customHeight="1">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>C2</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>TeamPage present-tense "TJC surveyor" check</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr"/>
-      <c r="D15" s="3" t="inlineStr"/>
-      <c r="E15" s="3" t="inlineStr"/>
-      <c r="F15" s="3" t="inlineStr">
-        <is>
-          <t>Closure evidence: site-wide search confirmed all surveyor language
-is past-tense, consistent with user's 2021-2025 service. User closed
-the item in session 299e9a73 turn 4.</t>
-        </is>
-      </c>
-      <c r="G15" s="3" t="inlineStr">
-        <is>
-          <t>session 299e9a73, ~2026-04-28.
----</t>
-        </is>
-      </c>
-      <c r="H15" s="3" t="inlineStr"/>
-    </row>
-    <row r="16" ht="90" customHeight="1">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>C3</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>My Studies CSV/XLSX export (John as design partner)</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr"/>
-      <c r="D16" s="2" t="inlineStr"/>
-      <c r="E16" s="2" t="inlineStr"/>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>Closure evidence: client/src/pages/DashboardPage.tsx line 46 calls
-/api/my-studies/export. server/routes.ts line 1491 implements the
-endpoint. Pulled forward into pre-COLA per user instruction.</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>session 299e9a73 turn 5, ~2026-04-28.
----</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr"/>
-    </row>
-    <row r="17" ht="90" customHeight="1">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>C4</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>Rotate GitHub PAT (because old PAT was committed in SESSION_HANDOFF files)</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="inlineStr"/>
-      <c r="D17" s="3" t="inlineStr"/>
-      <c r="E17" s="3" t="inlineStr"/>
-      <c r="F17" s="3" t="inlineStr">
-        <is>
-          <t>Closure evidence: no ghp_* or github_pat_* patterns in current
-SESSION_HANDOFF.md or SESSION_HANDOFF-2.md as of 2026-05-01.</t>
-        </is>
-      </c>
-      <c r="G17" s="3" t="inlineStr">
-        <is>
-          <t>session 299e9a73, ~2026-04-28.
----</t>
-        </is>
-      </c>
       <c r="H17" s="3" t="inlineStr"/>
     </row>
     <row r="18" ht="90" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>C6</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>VeritaPolicy service-line filtering removed (formerly #4)</t>
+          <t>TeamPage present-tense "TJC surveyor" check</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr"/>
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Closure evidence: site-wide search confirmed all surveyor language
+is past-tense, consistent with user's 2021-2025 service. User closed
+the item in session 299e9a73 turn 4.</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>session 299e9a73, ~2026-04-28.
+---</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19" ht="90" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>C3</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>My Studies CSV/XLSX export (John as design partner)</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr"/>
+      <c r="D19" s="3" t="inlineStr"/>
+      <c r="E19" s="3" t="inlineStr"/>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Closure evidence: client/src/pages/DashboardPage.tsx line 46 calls
+/api/my-studies/export. server/routes.ts line 1491 implements the
+endpoint. Pulled forward into pre-COLA per user instruction.</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>session 299e9a73 turn 5, ~2026-04-28.
+---</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr"/>
+    </row>
+    <row r="20" ht="90" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Rotate GitHub PAT (because old PAT was committed in SESSION_HANDOFF files)</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr"/>
+      <c r="D20" s="2" t="inlineStr"/>
+      <c r="E20" s="2" t="inlineStr"/>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Closure evidence: no ghp_* or github_pat_* patterns in current
+SESSION_HANDOFF.md or SESSION_HANDOFF-2.md as of 2026-05-01.</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>session 299e9a73, ~2026-04-28.
+---</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21" ht="90" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>C6</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>VeritaPolicy service-line filtering removed (formerly #4)</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr"/>
+      <c r="D21" s="3" t="inlineStr"/>
+      <c r="E21" s="3" t="inlineStr"/>
+      <c r="F21" s="3" t="inlineStr">
         <is>
           <t>Closure rationale (operator decision 2026-05-10): Keep all
 VeritaPolicy rows. CFR-only references with no accreditor reference
@@ -1775,29 +1928,29 @@
 report misread the design intent.</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="G21" s="3" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H18" s="2" t="inlineStr"/>
-    </row>
-    <row r="19" ht="90" customHeight="1">
-      <c r="A19" s="3" t="inlineStr">
+      <c r="H21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22" ht="90" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>C7</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B22" s="2" t="inlineStr">
         <is>
           <t>CLIA number format validation (formerly #13)</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr"/>
-      <c r="D19" s="3" t="inlineStr"/>
-      <c r="E19" s="3" t="inlineStr"/>
-      <c r="F19" s="3" t="inlineStr">
+      <c r="C22" s="2" t="inlineStr"/>
+      <c r="D22" s="2" t="inlineStr"/>
+      <c r="E22" s="2" t="inlineStr"/>
+      <c r="F22" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: shared/validateClia.ts defines CLIA_REGEX =
 /^\d{2}D\d{7}$/ (line 24), validateClia() helper with whitespace
@@ -1808,30 +1961,30 @@
 shape exists and behaves as specified.</t>
         </is>
       </c>
-      <c r="G19" s="3" t="inlineStr">
+      <c r="G22" s="2" t="inlineStr">
         <is>
           <t>Agent verification 2026-05-10 via grep + file read.
 Operator confirmed shipped 2026-05-10.
 ---</t>
         </is>
       </c>
-      <c r="H19" s="3" t="inlineStr"/>
-    </row>
-    <row r="20" ht="90" customHeight="1">
-      <c r="A20" s="2" t="inlineStr">
+      <c r="H22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23" ht="90" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>C8</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>VeritaMap lab-wide menu toggle (formerly #19)</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr"/>
-      <c r="D20" s="2" t="inlineStr"/>
-      <c r="E20" s="2" t="inlineStr"/>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="C23" s="3" t="inlineStr"/>
+      <c r="D23" s="3" t="inlineStr"/>
+      <c r="E23" s="3" t="inlineStr"/>
+      <c r="F23" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: client/src/pages/VeritaMapLabwidePage.tsx
 exists and implements the labwide read-only union view. Route is
@@ -1841,59 +1994,59 @@
 parking lot plan (read-only union view, per-session toggle) shipped.</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr">
+      <c r="G23" s="3" t="inlineStr">
         <is>
           <t>Agent verification 2026-05-10 via grep + file read.
 Operator confirmed shipped 2026-05-10.
 ---</t>
         </is>
       </c>
-      <c r="H20" s="2" t="inlineStr"/>
-    </row>
-    <row r="21" ht="90" customHeight="1">
-      <c r="A21" s="3" t="inlineStr">
+      <c r="H23" s="3" t="inlineStr"/>
+    </row>
+    <row r="24" ht="90" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>C9</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>Tier-1 smoke test checklist (formerly #6)</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr"/>
-      <c r="D21" s="3" t="inlineStr"/>
-      <c r="E21" s="3" t="inlineStr"/>
-      <c r="F21" s="3" t="inlineStr">
+      <c r="C24" s="2" t="inlineStr"/>
+      <c r="D24" s="2" t="inlineStr"/>
+      <c r="E24" s="2" t="inlineStr"/>
+      <c r="F24" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: docs/smoke-test-tier1.md documents the Tier-1
 smoke-test process and post-deploy verification steps. Shipped via
 PR #81 as part of the 2026-05-10 wave.</t>
         </is>
       </c>
-      <c r="G21" s="3" t="inlineStr">
+      <c r="G24" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H21" s="3" t="inlineStr"/>
-    </row>
-    <row r="22" ht="90" customHeight="1">
-      <c r="A22" s="2" t="inlineStr">
+      <c r="H24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25" ht="90" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
         <is>
           <t>C10</t>
         </is>
       </c>
-      <c r="B22" s="2" t="inlineStr">
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>Per-module gating (formerly #7)</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr"/>
-      <c r="D22" s="2" t="inlineStr"/>
-      <c r="E22" s="2" t="inlineStr"/>
-      <c r="F22" s="2" t="inlineStr">
+      <c r="C25" s="3" t="inlineStr"/>
+      <c r="D25" s="3" t="inlineStr"/>
+      <c r="E25" s="3" t="inlineStr"/>
+      <c r="F25" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: Client-side useIsReadOnly module keys wired
 on client/src/pages/VeritaPolicyAppPage.tsx and
@@ -1908,29 +2061,29 @@
 PR #76.</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr">
+      <c r="G25" s="3" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H22" s="2" t="inlineStr"/>
-    </row>
-    <row r="23" ht="90" customHeight="1">
-      <c r="A23" s="3" t="inlineStr">
+      <c r="H25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26" ht="90" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>C11</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t>VeritaStock shipped copy (formerly #8)</t>
         </is>
       </c>
-      <c r="C23" s="3" t="inlineStr"/>
-      <c r="D23" s="3" t="inlineStr"/>
-      <c r="E23" s="3" t="inlineStr"/>
-      <c r="F23" s="3" t="inlineStr">
+      <c r="C26" s="2" t="inlineStr"/>
+      <c r="D26" s="2" t="inlineStr"/>
+      <c r="E26" s="2" t="inlineStr"/>
+      <c r="F26" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: client/src/pages/ArticleInventoryManagementPage.tsx
 line 305 footer reads "platform that includes VeritaStock™" instead
@@ -1938,29 +2091,29 @@
 on /resources/laboratory-inventory-management. Shipped via PR #75.</t>
         </is>
       </c>
-      <c r="G23" s="3" t="inlineStr">
+      <c r="G26" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H23" s="3" t="inlineStr"/>
-    </row>
-    <row r="24" ht="90" customHeight="1">
-      <c r="A24" s="2" t="inlineStr">
+      <c r="H26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27" ht="90" customHeight="1">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>C12</t>
         </is>
       </c>
-      <c r="B24" s="2" t="inlineStr">
+      <c r="B27" s="3" t="inlineStr">
         <is>
           <t>Admin report one-row-per-lab (formerly #14)</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr"/>
-      <c r="D24" s="2" t="inlineStr"/>
-      <c r="E24" s="2" t="inlineStr"/>
-      <c r="F24" s="2" t="inlineStr">
+      <c r="C27" s="3" t="inlineStr"/>
+      <c r="D27" s="3" t="inlineStr"/>
+      <c r="E27" s="3" t="inlineStr"/>
+      <c r="F27" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: /api/admin/report rewritten in
 server/routes.ts (~line 595) to LEFT JOIN labs on
@@ -1975,56 +2128,56 @@
 prerequisite, not a code bug). Shipped via PR #85.</t>
         </is>
       </c>
-      <c r="G24" s="2" t="inlineStr">
+      <c r="G27" s="3" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H24" s="2" t="inlineStr"/>
-    </row>
-    <row r="25" ht="90" customHeight="1">
-      <c r="A25" s="3" t="inlineStr">
+      <c r="H27" s="3" t="inlineStr"/>
+    </row>
+    <row r="28" ht="90" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>C14</t>
         </is>
       </c>
-      <c r="B25" s="3" t="inlineStr">
+      <c r="B28" s="2" t="inlineStr">
         <is>
           <t>UI relabel "CLIA TEa" -&gt; "Lab-Set Internal Goal" (formerly #1)</t>
         </is>
       </c>
-      <c r="C25" s="3" t="inlineStr"/>
-      <c r="D25" s="3" t="inlineStr"/>
-      <c r="E25" s="3" t="inlineStr"/>
-      <c r="F25" s="3" t="inlineStr">
+      <c r="C28" s="2" t="inlineStr"/>
+      <c r="D28" s="2" t="inlineStr"/>
+      <c r="E28" s="2" t="inlineStr"/>
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: Shipped across four PRs over 2026-05-10.</t>
         </is>
       </c>
-      <c r="G25" s="3" t="inlineStr">
+      <c r="G28" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H25" s="3" t="inlineStr"/>
-    </row>
-    <row r="26" ht="90" customHeight="1">
-      <c r="A26" s="2" t="inlineStr">
+      <c r="H28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29" ht="90" customHeight="1">
+      <c r="A29" s="3" t="inlineStr">
         <is>
           <t>C13</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="B29" s="3" t="inlineStr">
         <is>
           <t>WSLH PT vendor (formerly #15)</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr"/>
-      <c r="D26" s="2" t="inlineStr"/>
-      <c r="E26" s="2" t="inlineStr"/>
-      <c r="F26" s="2" t="inlineStr">
+      <c r="C29" s="3" t="inlineStr"/>
+      <c r="D29" s="3" t="inlineStr"/>
+      <c r="E29" s="3" t="inlineStr"/>
+      <c r="F29" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: Shipped 2026-05-10 via PR #79 (merge commit
 eeebc6e; merged after rebase to resolve a server/db.ts collision
@@ -2042,64 +2195,64 @@
 'WSLH' is the post-deploy success signal. Shipped via PR #79.</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr">
+      <c r="G29" s="3" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H26" s="2" t="inlineStr"/>
-    </row>
-    <row r="27" ht="90" customHeight="1">
-      <c r="A27" s="3" t="inlineStr">
+      <c r="H29" s="3" t="inlineStr"/>
+    </row>
+    <row r="30" ht="90" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>C15</t>
         </is>
       </c>
-      <c r="B27" s="3" t="inlineStr">
+      <c r="B30" s="2" t="inlineStr">
         <is>
           <t>VeritaStock lot tracking + expiration + reorder alerts (formerly #21)</t>
         </is>
       </c>
-      <c r="C27" s="3" t="inlineStr"/>
-      <c r="D27" s="3" t="inlineStr"/>
-      <c r="E27" s="3" t="inlineStr"/>
-      <c r="F27" s="3" t="inlineStr">
+      <c r="C30" s="2" t="inlineStr"/>
+      <c r="D30" s="2" t="inlineStr"/>
+      <c r="E30" s="2" t="inlineStr"/>
+      <c r="F30" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: VeritaStock™ shipped the bench-level inventory
 features the Perplexity competitor analysis identified as a gap:</t>
         </is>
       </c>
-      <c r="G27" s="3" t="inlineStr">
+      <c r="G30" s="2" t="inlineStr">
         <is>
           <t>Originally Perplexity competitor analysis 2026-05-10.
 Audit 2026-05-21 confirmed the feature set ships today.
 ---</t>
         </is>
       </c>
-      <c r="H27" s="3" t="inlineStr"/>
-    </row>
-    <row r="28" ht="90" customHeight="1">
-      <c r="A28" s="2" t="inlineStr">
+      <c r="H30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31" ht="90" customHeight="1">
+      <c r="A31" s="3" t="inlineStr">
         <is>
           <t>C16</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="B31" s="3" t="inlineStr">
         <is>
           <t>PAL studies guided workflow (formerly #23)</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr"/>
-      <c r="D28" s="2" t="inlineStr"/>
-      <c r="E28" s="2" t="inlineStr"/>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="C31" s="3" t="inlineStr"/>
+      <c r="D31" s="3" t="inlineStr"/>
+      <c r="E31" s="3" t="inlineStr"/>
+      <c r="F31" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: VeritaCheck™ already ships the Precision /
 Accuracy / Linearity (PAL) study set under EP-protocol naming:</t>
         </is>
       </c>
-      <c r="G28" s="2" t="inlineStr">
+      <c r="G31" s="3" t="inlineStr">
         <is>
           <t>Originally Perplexity competitor analysis 2026-05-10.
 Audit 2026-05-21 confirmed the EP studies cover the PAL framing in
@@ -2107,23 +2260,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H28" s="2" t="inlineStr"/>
-    </row>
-    <row r="29" ht="90" customHeight="1">
-      <c r="A29" s="3" t="inlineStr">
+      <c r="H31" s="3" t="inlineStr"/>
+    </row>
+    <row r="32" ht="90" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t>C17</t>
         </is>
       </c>
-      <c r="B29" s="3" t="inlineStr">
+      <c r="B32" s="2" t="inlineStr">
         <is>
           <t>Source-grounded 21/29/45 CFR + 42 CFR 482-485 (formerly #26)</t>
         </is>
       </c>
-      <c r="C29" s="3" t="inlineStr"/>
-      <c r="D29" s="3" t="inlineStr"/>
-      <c r="E29" s="3" t="inlineStr"/>
-      <c r="F29" s="3" t="inlineStr">
+      <c r="C32" s="2" t="inlineStr"/>
+      <c r="D32" s="2" t="inlineStr"/>
+      <c r="E32" s="2" t="inlineStr"/>
+      <c r="F32" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #301 (commit 8c27806, merged 2026-05-21)
 source-grounded the 74 remaining non-493 entries in
@@ -2131,29 +2284,29 @@
 shipped:</t>
         </is>
       </c>
-      <c r="G29" s="3" t="inlineStr">
+      <c r="G32" s="2" t="inlineStr">
         <is>
           <t>PR #301; tasks #18 in the in-session task tracker.
 ---</t>
         </is>
       </c>
-      <c r="H29" s="3" t="inlineStr"/>
-    </row>
-    <row r="30" ht="90" customHeight="1">
-      <c r="A30" s="2" t="inlineStr">
+      <c r="H32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33" ht="90" customHeight="1">
+      <c r="A33" s="3" t="inlineStr">
         <is>
           <t>C18</t>
         </is>
       </c>
-      <c r="B30" s="2" t="inlineStr">
+      <c r="B33" s="3" t="inlineStr">
         <is>
           <t>VeritaPolicy "Non CLIA" chapter rename (formerly #3)</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr"/>
-      <c r="D30" s="2" t="inlineStr"/>
-      <c r="E30" s="2" t="inlineStr"/>
-      <c r="F30" s="2" t="inlineStr">
+      <c r="C33" s="3" t="inlineStr"/>
+      <c r="D33" s="3" t="inlineStr"/>
+      <c r="E33" s="3" t="inlineStr"/>
+      <c r="F33" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #300 (commit 34d7707, merged 2026-05-21)
 renamed all 44 user-facing chapter labels in
@@ -2164,7 +2317,7 @@
 page.</t>
         </is>
       </c>
-      <c r="G30" s="2" t="inlineStr">
+      <c r="G33" s="3" t="inlineStr">
         <is>
           <t>CAP customer screenshot of the /veritapolicy chapter
 headers, 2026-05-01 evening. PR #300; tasks #17 in the in-session
@@ -2172,23 +2325,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H30" s="2" t="inlineStr"/>
-    </row>
-    <row r="31" ht="90" customHeight="1">
-      <c r="A31" s="3" t="inlineStr">
+      <c r="H33" s="3" t="inlineStr"/>
+    </row>
+    <row r="34" ht="90" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
         <is>
           <t>C19</t>
         </is>
       </c>
-      <c r="B31" s="3" t="inlineStr">
+      <c r="B34" s="2" t="inlineStr">
         <is>
           <t>VeritaStock department-scope toggle (formerly #31)</t>
         </is>
       </c>
-      <c r="C31" s="3" t="inlineStr"/>
-      <c r="D31" s="3" t="inlineStr"/>
-      <c r="E31" s="3" t="inlineStr"/>
-      <c r="F31" s="3" t="inlineStr">
+      <c r="C34" s="2" t="inlineStr"/>
+      <c r="D34" s="2" t="inlineStr"/>
+      <c r="E34" s="2" t="inlineStr"/>
+      <c r="F34" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #319 (commit d01f5fe, merged 2026-05-22)
 shipped the persistent dept-scope toggle on VeritaStockPage. A new
@@ -2199,7 +2352,7 @@
 workspace without re-filtering.</t>
         </is>
       </c>
-      <c r="G31" s="3" t="inlineStr">
+      <c r="G34" s="2" t="inlineStr">
         <is>
           <t>John, San Carlos lab, 2026-05-21. Same conversation that
 drove the vendor dropdown (PR #304), FILTERED VIEW banner (PR #305),
@@ -2207,23 +2360,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H31" s="3" t="inlineStr"/>
-    </row>
-    <row r="32" ht="90" customHeight="1">
-      <c r="A32" s="2" t="inlineStr">
+      <c r="H34" s="2" t="inlineStr"/>
+    </row>
+    <row r="35" ht="90" customHeight="1">
+      <c r="A35" s="3" t="inlineStr">
         <is>
           <t>C20</t>
         </is>
       </c>
-      <c r="B32" s="2" t="inlineStr">
+      <c r="B35" s="3" t="inlineStr">
         <is>
           <t>Primary-lab seat counting (formerly #12)</t>
         </is>
       </c>
-      <c r="C32" s="2" t="inlineStr"/>
-      <c r="D32" s="2" t="inlineStr"/>
-      <c r="E32" s="2" t="inlineStr"/>
-      <c r="F32" s="2" t="inlineStr">
+      <c r="C35" s="3" t="inlineStr"/>
+      <c r="D35" s="3" t="inlineStr"/>
+      <c r="E35" s="3" t="inlineStr"/>
+      <c r="F35" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: is_primary_lab INTEGER NOT NULL DEFAULT 0
 column was added to the lab_members table at db.ts:1276, with the
@@ -2234,7 +2387,7 @@
 is_primary_lab=1 ordering).</t>
         </is>
       </c>
-      <c r="G32" s="2" t="inlineStr">
+      <c r="G35" s="3" t="inlineStr">
         <is>
           <t>2026-05-07 multi-lab discussion. Build shipped as part
 of the Multi-Lab Tier 2 architecture work (Phase 3.x series, prior
@@ -2243,23 +2396,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H32" s="2" t="inlineStr"/>
-    </row>
-    <row r="33" ht="90" customHeight="1">
-      <c r="A33" s="3" t="inlineStr">
+      <c r="H35" s="3" t="inlineStr"/>
+    </row>
+    <row r="36" ht="90" customHeight="1">
+      <c r="A36" s="2" t="inlineStr">
         <is>
           <t>C21</t>
         </is>
       </c>
-      <c r="B33" s="3" t="inlineStr">
+      <c r="B36" s="2" t="inlineStr">
         <is>
           <t>Multi-lab pricing model — Option A (formerly #11)</t>
         </is>
       </c>
-      <c r="C33" s="3" t="inlineStr"/>
-      <c r="D33" s="3" t="inlineStr"/>
-      <c r="E33" s="3" t="inlineStr"/>
-      <c r="F33" s="3" t="inlineStr">
+      <c r="C36" s="2" t="inlineStr"/>
+      <c r="D36" s="2" t="inlineStr"/>
+      <c r="E36" s="2" t="inlineStr"/>
+      <c r="F36" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #322 (commit 0ccd925, merged 2026-05-22)
 added the customer-facing line to the pricing page that reflects
@@ -2272,7 +2425,7 @@
 Enterprise+ block, reads:</t>
         </is>
       </c>
-      <c r="G33" s="3" t="inlineStr">
+      <c r="G36" s="2" t="inlineStr">
         <is>
           <t>2026-05-07 multi-lab discussion (Lisa Veri's
 canonical-case session). PR #322 (initial build); softening PR
@@ -2281,30 +2434,30 @@
 ---</t>
         </is>
       </c>
-      <c r="H33" s="3" t="inlineStr"/>
-    </row>
-    <row r="34" ht="90" customHeight="1">
-      <c r="A34" s="2" t="inlineStr">
+      <c r="H36" s="2" t="inlineStr"/>
+    </row>
+    <row r="37" ht="90" customHeight="1">
+      <c r="A37" s="3" t="inlineStr">
         <is>
           <t>C22</t>
         </is>
       </c>
-      <c r="B34" s="2" t="inlineStr">
+      <c r="B37" s="3" t="inlineStr">
         <is>
           <t>VeritaOps cost-per-test module (formerly #10)</t>
         </is>
       </c>
-      <c r="C34" s="2" t="inlineStr"/>
-      <c r="D34" s="2" t="inlineStr"/>
-      <c r="E34" s="2" t="inlineStr"/>
-      <c r="F34" s="2" t="inlineStr">
+      <c r="C37" s="3" t="inlineStr"/>
+      <c r="D37" s="3" t="inlineStr"/>
+      <c r="E37" s="3" t="inlineStr"/>
+      <c r="F37" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: v1 of the VeritaOps Cost-Per-Reportable-Test
 (CPRT) module shipped across PR #325 through PR #330 on 2026-05-22.
 The module is feature-complete for the typical lab director workflow.</t>
         </is>
       </c>
-      <c r="G34" s="2" t="inlineStr">
+      <c r="G37" s="3" t="inlineStr">
         <is>
           <t>This thread, 2026-05-07 12:05 PM CDT, user message:
 "Parking lot: build an operations module for cost per test
@@ -2313,262 +2466,262 @@
 ---</t>
         </is>
       </c>
-      <c r="H34" s="2" t="inlineStr"/>
-    </row>
-    <row r="35" ht="90" customHeight="1">
-      <c r="A35" s="3" t="inlineStr">
+      <c r="H37" s="3" t="inlineStr"/>
+    </row>
+    <row r="38" ht="90" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
         <is>
           <t>C23</t>
         </is>
       </c>
-      <c r="B35" s="3" t="inlineStr">
+      <c r="B38" s="2" t="inlineStr">
         <is>
           <t>CCL lab name visual disambiguation in lab switcher (formerly #34)</t>
         </is>
       </c>
-      <c r="C35" s="3" t="inlineStr"/>
-      <c r="D35" s="3" t="inlineStr">
+      <c r="C38" s="2" t="inlineStr"/>
+      <c r="D38" s="2" t="inlineStr">
         <is>
           <t>XS (under 1 day, actual)</t>
         </is>
       </c>
-      <c r="E35" s="3" t="inlineStr">
+      <c r="E38" s="2" t="inlineStr">
         <is>
           <t>Low — cosmetic; only mattered when Lisa or Michael picked the wrong lab from...</t>
         </is>
       </c>
-      <c r="F35" s="3" t="inlineStr">
+      <c r="F38" s="2" t="inlineStr">
         <is>
           <t>Effort: XS (under 1 day, actual)
 Importance: Low — cosmetic; only mattered when Lisa or Michael picked the wrong lab from the dropdown.</t>
         </is>
       </c>
-      <c r="G35" s="3" t="inlineStr">
+      <c r="G38" s="2" t="inlineStr">
         <is>
           <t>flagged 2026-05-23 immediately after provisioning Lisa's CCL lab; closed 2026-05-24.
 ---</t>
         </is>
       </c>
-      <c r="H35" s="3" t="inlineStr"/>
-    </row>
-    <row r="36" ht="90" customHeight="1">
-      <c r="A36" s="2" t="inlineStr">
+      <c r="H38" s="2" t="inlineStr"/>
+    </row>
+    <row r="39" ht="90" customHeight="1">
+      <c r="A39" s="3" t="inlineStr">
         <is>
           <t>C24</t>
         </is>
       </c>
-      <c r="B36" s="2" t="inlineStr">
+      <c r="B39" s="3" t="inlineStr">
         <is>
           <t>VC Unlimited Y1/Y2 price disclosure UX (formerly #35)</t>
         </is>
       </c>
-      <c r="C36" s="2" t="inlineStr"/>
-      <c r="D36" s="2" t="inlineStr">
+      <c r="C39" s="3" t="inlineStr"/>
+      <c r="D39" s="3" t="inlineStr">
         <is>
           <t>XS (under 1 day, actual)</t>
         </is>
       </c>
-      <c r="E36" s="2" t="inlineStr">
+      <c r="E39" s="3" t="inlineStr">
         <is>
           <t>Low when shipped (proactive, no customer complaint yet) — but high if a procu...</t>
         </is>
       </c>
-      <c r="F36" s="2" t="inlineStr">
+      <c r="F39" s="3" t="inlineStr">
         <is>
           <t>Effort: XS (under 1 day, actual)
 Importance: Low when shipped (proactive, no customer complaint yet) — but high if a procurement reviewer later disputes the $499 renewal as undisclosed.</t>
         </is>
       </c>
-      <c r="G36" s="2" t="inlineStr">
+      <c r="G39" s="3" t="inlineStr">
         <is>
           <t>Pricing rebuild 2026-05-23; closed 2026-05-24 proactively before any customer dispute.
 ---</t>
         </is>
       </c>
-      <c r="H36" s="2" t="inlineStr"/>
-    </row>
-    <row r="37" ht="90" customHeight="1">
-      <c r="A37" s="3" t="inlineStr">
+      <c r="H39" s="3" t="inlineStr"/>
+    </row>
+    <row r="40" ht="90" customHeight="1">
+      <c r="A40" s="2" t="inlineStr">
         <is>
           <t>C25</t>
         </is>
       </c>
-      <c r="B37" s="3" t="inlineStr">
+      <c r="B40" s="2" t="inlineStr">
         <is>
           <t>VeritaQC Phase 1 (Levey-Jennings + Westgard live engine) (formerly #20)</t>
         </is>
       </c>
-      <c r="C37" s="3" t="inlineStr"/>
-      <c r="D37" s="3" t="inlineStr">
+      <c r="C40" s="2" t="inlineStr"/>
+      <c r="D40" s="2" t="inlineStr">
         <is>
           <t>L (about 5 days end-to-end, actual: Phase 0 schema → Phase 1A evaluator → 1B...</t>
         </is>
       </c>
-      <c r="E37" s="3" t="inlineStr">
+      <c r="E40" s="2" t="inlineStr">
         <is>
           <t>High — largest single gap vs myLabCompliance.io per Perplexity competitor ana...</t>
         </is>
       </c>
-      <c r="F37" s="3" t="inlineStr">
+      <c r="F40" s="2" t="inlineStr">
         <is>
           <t>Effort: L (about 5 days end-to-end, actual: Phase 0 schema → Phase 1A evaluator → 1B entry UI → 1C daily review → 1D monthly PDF + attestation)
 Importance: High — largest single gap vs myLabCompliance.io per Perplexity competitor analysis; promotes VeritaAssure from documentation tool to lab operations platform.</t>
         </is>
       </c>
-      <c r="G37" s="3" t="inlineStr">
+      <c r="G40" s="2" t="inlineStr">
         <is>
           <t>Perplexity competitor analysis 2026-05-10. Scoping confirmed via the build_phase1_mockup.py iterations 2026-05-24. Shipped 2026-05-25.
 ---</t>
         </is>
       </c>
-      <c r="H37" s="3" t="inlineStr"/>
-    </row>
-    <row r="38" ht="90" customHeight="1">
-      <c r="A38" s="2" t="inlineStr">
+      <c r="H40" s="2" t="inlineStr"/>
+    </row>
+    <row r="41" ht="90" customHeight="1">
+      <c r="A41" s="3" t="inlineStr">
         <is>
           <t>C26</t>
         </is>
       </c>
-      <c r="B38" s="2" t="inlineStr">
+      <c r="B41" s="3" t="inlineStr">
         <is>
           <t>VeritaLab CMS-116 application support + state licensing registry (formerly #22)</t>
         </is>
       </c>
-      <c r="C38" s="2" t="inlineStr"/>
-      <c r="D38" s="2" t="inlineStr">
+      <c r="C41" s="3" t="inlineStr"/>
+      <c r="D41" s="3" t="inlineStr">
         <is>
           <t>M (1-2 weeks for v1, actual)</t>
         </is>
       </c>
-      <c r="E38" s="2" t="inlineStr">
+      <c r="E41" s="3" t="inlineStr">
         <is>
           <t>Medium — competitor parity (myLabCompliance.io) plus useful at lab startup an...</t>
         </is>
       </c>
-      <c r="F38" s="2" t="inlineStr">
+      <c r="F41" s="3" t="inlineStr">
         <is>
           <t>Effort: M (1-2 weeks for v1, actual)
 Importance: Medium — competitor parity (myLabCompliance.io) plus useful at lab startup and at certificate-type changes.</t>
         </is>
       </c>
-      <c r="G38" s="2" t="inlineStr">
+      <c r="G41" s="3" t="inlineStr">
         <is>
           <t>Perplexity competitor analysis (myLabCompliance.io), 2026-05-10. Reclassified as a VeritaLab extension 2026-05-25. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H38" s="2" t="inlineStr"/>
-    </row>
-    <row r="39" ht="90" customHeight="1">
-      <c r="A39" s="3" t="inlineStr">
+      <c r="H41" s="3" t="inlineStr"/>
+    </row>
+    <row r="42" ht="90" customHeight="1">
+      <c r="A42" s="2" t="inlineStr">
         <is>
           <t>C27</t>
         </is>
       </c>
-      <c r="B39" s="3" t="inlineStr">
+      <c r="B42" s="2" t="inlineStr">
         <is>
           <t>Active vs view-only seat split (formerly #33)</t>
         </is>
       </c>
-      <c r="C39" s="3" t="inlineStr"/>
-      <c r="D39" s="3" t="inlineStr">
+      <c r="C42" s="2" t="inlineStr"/>
+      <c r="D42" s="2" t="inlineStr">
         <is>
           <t>M (~1 week of engineering, actual: shipped in a single multi-PR session)</t>
         </is>
       </c>
-      <c r="E39" s="3" t="inlineStr">
+      <c r="E42" s="2" t="inlineStr">
         <is>
           <t>Medium — closed the gap between /pricing copy and product behavior; gives sal...</t>
         </is>
       </c>
-      <c r="F39" s="3" t="inlineStr">
+      <c r="F42" s="2" t="inlineStr">
         <is>
           <t>Effort: M (~1 week of engineering, actual: shipped in a single multi-PR session)
 Importance: Medium — closed the gap between /pricing copy and product behavior; gives sales a clean answer for "do you charge for our medical director?"</t>
         </is>
       </c>
-      <c r="G39" s="3" t="inlineStr">
+      <c r="G42" s="2" t="inlineStr">
         <is>
           <t>Pricing analysis doc Decision 3 (2026-05-21); MEDIUM scenario revised 2026-05-29 to retire the "unlimited view-only" claim. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H39" s="3" t="inlineStr"/>
-    </row>
-    <row r="40" ht="90" customHeight="1">
-      <c r="A40" s="2" t="inlineStr">
+      <c r="H42" s="2" t="inlineStr"/>
+    </row>
+    <row r="43" ht="90" customHeight="1">
+      <c r="A43" s="3" t="inlineStr">
         <is>
           <t>C28</t>
         </is>
       </c>
-      <c r="B40" s="2" t="inlineStr">
+      <c r="B43" s="3" t="inlineStr">
         <is>
           <t>"Why VeritaCheck" comparative one-pager (formerly #37)</t>
         </is>
       </c>
-      <c r="C40" s="2" t="inlineStr"/>
-      <c r="D40" s="2" t="inlineStr">
+      <c r="C43" s="3" t="inlineStr"/>
+      <c r="D43" s="3" t="inlineStr">
         <is>
           <t>S (one design pass + four claim paragraphs + PDF + matching marketing-site pa...</t>
         </is>
       </c>
-      <c r="E40" s="2" t="inlineStr">
+      <c r="E43" s="3" t="inlineStr">
         <is>
           <t>Medium — closed a positioning gap surfaced by six COLA conference attendees a...</t>
         </is>
       </c>
-      <c r="F40" s="2" t="inlineStr">
+      <c r="F43" s="3" t="inlineStr">
         <is>
           <t>Effort: S (one design pass + four claim paragraphs + PDF + matching marketing-site page, actual)
 Importance: Medium — closed a positioning gap surfaced by six COLA conference attendees attached to a legacy verification tool; converts product-quality advantage into a leave-behind Lisa can hand out.</t>
         </is>
       </c>
-      <c r="G40" s="2" t="inlineStr">
+      <c r="G43" s="3" t="inlineStr">
         <is>
           <t>2026-05-11 / 2026-05-12 conference notes review with Michael. Conference attendees (Whitehead, Odegard, Othman, Molinelli, Kyle, Allred) expressed interest in equivalent / superior product. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H40" s="2" t="inlineStr"/>
-    </row>
-    <row r="41" ht="90" customHeight="1">
-      <c r="A41" s="3" t="inlineStr">
+      <c r="H43" s="3" t="inlineStr"/>
+    </row>
+    <row r="44" ht="90" customHeight="1">
+      <c r="A44" s="2" t="inlineStr">
         <is>
           <t>C29</t>
         </is>
       </c>
-      <c r="B41" s="3" t="inlineStr">
+      <c r="B44" s="2" t="inlineStr">
         <is>
           <t>VeritaPolicy approval workflow — MediaLab functional mirror</t>
         </is>
       </c>
-      <c r="C41" s="3" t="inlineStr"/>
-      <c r="D41" s="3" t="inlineStr">
+      <c r="C44" s="2" t="inlineStr"/>
+      <c r="D44" s="2" t="inlineStr">
         <is>
           <t>XL (one focused session, 12 PRs landed)</t>
         </is>
       </c>
-      <c r="E41" s="3" t="inlineStr">
+      <c r="E44" s="2" t="inlineStr">
         <is>
           <t>High — replaces MediaLab Document Control ($752/$2,250 starting price, scalin...</t>
         </is>
       </c>
-      <c r="F41" s="3" t="inlineStr">
+      <c r="F44" s="2" t="inlineStr">
         <is>
           <t>Effort: XL (one focused session, 12 PRs landed)
 Importance: High — replaces MediaLab Document Control ($752/$2,250 starting price, scaling to $10K-$20K/yr at enterprise per Capterra public data) with an included VeritaPolicy feature; closes a real positioning gap and gives sales a direct comparator line.</t>
         </is>
       </c>
-      <c r="G41" s="3" t="inlineStr">
+      <c r="G44" s="2" t="inlineStr">
         <is>
           <t>Pricing strategy conversation 2026-05-29 (Michael: "I don't like bolt-ons; we should replicate this") → scoped 8 phases → shipped all 12 PRs in single session. Shipped 2026-05-29.
 ---</t>
         </is>
       </c>
-      <c r="H41" s="3" t="inlineStr"/>
+      <c r="H44" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H41"/>
+  <autoFilter ref="A1:H44"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
TASK: Fix verify-script coverage audit matcher + correct #41 parking-lot placement
PLAN:
  1. Widen audit_verify_script_coverage.py matcher to accept .mjs/.mts/.ts, not just .js/.cjs.
  2. Move parking-lot #41 (already CLOSED in-body, see C30) from OPEN into CLOSED as C44.
  3. Rebuild PARKING_LOT.xlsx.

Self-check:
  - Matcher widening is additive; audit re-run shows 5/5 covered, 0 debt.
  - #41 removed from OPEN once; C44 in CLOSED; xlsx counts OPEN 16 / CLOSED 44 / RETIRED 6.
  - Internal scripts + parking-lot docs only; Gate 3 N/A.
</commit_message>
<xml_diff>
--- a/PARKING_LOT.xlsx
+++ b/PARKING_LOT.xlsx
@@ -12,8 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RETIRED" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$18</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$44</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$45</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RETIRED'!$A$1:$H$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1095,40 +1095,38 @@
     <row r="14" ht="90" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>42</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Verify-script convention backfill (CLAUDE.md §2)</t>
+          <t>Outbound demo-invite messaging campaign to 1st-degree LinkedIn contacts</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>CLOSED 2026-06-13. All 8 high-stakes backfill scripts landed (the
-strike-throughs above); see C30. Pre- vs post-COLA: indifferent.
+          <t>Parked. Plan documented. Implementation deferred until trigger conditions met.
 ---</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>L (8 backfill scripts, each ~2-4 hours, total ~3-5 working days if done as on...</t>
+          <t>L (1 week prep + 4-6 weeks of staged sends)</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Medium-High. Procedural-debt cleanup against a NON-NEGOTIABLE convention. CLA...</t>
+          <t>High. Converts existing warm network (~2,500 1st-degree contacts and growing...</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Effort: L (8 backfill scripts, each ~2-4 hours, total ~3-5 working days if done as one focused sweep).
-Importance: Medium-High. Procedural-debt cleanup against a NON-NEGOTIABLE convention. CLAUDE.md §2 verify-*.js: every math/logic change ships with a paired script that exercises every meaningful branch. The audit run on 2026-06-02 found 31 of 35 math/logic commits in the last 90 days violated the convention. Some are exempt (renames, citation swaps, copy changes) but at least 8 introduced new math or fixed math defects and should have shipped with verification.</t>
+          <t>A staged outbound DM campaign walking Michael's 1st-degree LinkedIn contacts through tier-segmented demo invitations for VeritaAssure. Goal: convert warmest contacts into demo conversations first, then chain into trials and paid subscriptions. Separate pipeline from COLA cohort follow-up and from content-driven inbound; all three feed the same demo funnel but originate from different warmth sources.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>scripts/audit_verify_script_coverage.py output, run 2026-06-02. Captured as the formal lookback that surfaced the gap.</t>
+          <t>2026-06-04 session, after weekly LinkedIn invite batch completion (80 sent, cap hit at #84 Victoria Allen).</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr"/>
@@ -1136,38 +1134,39 @@
     <row r="15" ht="90" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>47</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Outbound demo-invite messaging campaign to 1st-degree LinkedIn contacts</t>
+          <t>Hide sections a lab does not use from a master list, to reduce clutter (prospect-requested)</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Parked. Plan documented. Implementation deferred until trigger conditions met.
+          <t>Open. Not started. Needs a one-line scope confirmation (which master list).
 ---</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>L (1 week prep + 4-6 weeks of staged sends)</t>
+          <t>S-M (a few days to ~2 weeks depending on scope) — a lab-level visibility togg...</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>High. Converts existing warm network (~2,500 1st-degree contacts and growing...</t>
+          <t>Medium-High — came straight from a live prospect today as an onboarding-frict...</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>A staged outbound DM campaign walking Michael's 1st-degree LinkedIn contacts through tier-segmented demo invitations for VeritaAssure. Goal: convert warmest contacts into demo conversations first, then chain into trials and paid subscriptions. Separate pipeline from COLA cohort follow-up and from content-driven inbound; all three feed the same demo funnel but originate from different warmth sources.</t>
+          <t>Effort: S-M (a few days to ~2 weeks depending on scope) — a lab-level visibility toggle that hides not-applicable or unused sections from a master-list view. Smaller if it is a "hide N/A" filter on the existing VeritaDC master list, larger if it also spans VeritaScan domains.
+Importance: Medium-High — came straight from a live prospect today as an onboarding-friction point; a lab that does not run a service line should not have to wade past its requirements.</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>2026-06-04 session, after weekly LinkedIn invite batch completion (80 sent, cap hit at #84 Victoria Allen).</t>
+          <t>2026-09-23 session, Michael relaying a prospect ask from a demo today.</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr"/>
@@ -1175,39 +1174,35 @@
     <row r="16" ht="90" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>49</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Hide sections a lab does not use from a master list, to reduce clutter (prospect-requested)</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Open. Not started. Needs a one-line scope confirmation (which master list).
----</t>
-        </is>
-      </c>
+          <t>Unify the coverage/competency recurrence into one shared helper (tech debt)</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr"/>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>S-M (a few days to ~2 weeks depending on scope) — a lab-level visibility togg...</t>
+          <t>S (a few hours) - extract "latest study/assessment -&gt; status / nextDueOn / ov...</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Medium-High — came straight from a live prospect today as an onboarding-frict...</t>
+          <t>Low - the three paths duplicate the +6-month / signed-resets-to-missing logic...</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Effort: S-M (a few days to ~2 weeks depending on scope) — a lab-level visibility toggle that hides not-applicable or unused sections from a master-list view. Smaller if it is a "hide N/A" filter on the existing VeritaDC master list, larger if it also spans VeritaScan domains.
-Importance: Medium-High — came straight from a live prospect today as an onboarding-friction point; a lab that does not run a service line should not have to wade past its requirements.</t>
+          <t>Effort: S (a few hours) - extract "latest study/assessment -&gt; status / nextDueOn / overdue" into one helper used by method comparison, cal-ver/linearity, and the competency owed derivation.
+Importance: Low - the three paths duplicate the +6-month / signed-resets-to-missing logic. They agree today (verified), but a shared helper prevents future drift and settles the dateless-signed edge in one place. No user-facing impact; studies.date is NOT NULL so the one known divergence is unreachable in practice.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23 session, Michael relaying a prospect ask from a demo today.</t>
+          <t>2026-09-24 session, surfaced during the coverage-recurrence build. No live defect; hygiene.
+---</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr"/>
@@ -1215,77 +1210,41 @@
     <row r="17" ht="90" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>50</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Unify the coverage/competency recurrence into one shared helper (tech debt)</t>
+          <t>Competency "assessed this cycle" uses a flat 365-day window</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr"/>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>S (a few hours) - extract "latest study/assessment -&gt; status / nextDueOn / ov...</t>
+          <t>S-M - anchor the coverage-map "assessed this cycle" to the person's actual CL...</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>Low - the three paths duplicate the +6-month / signed-resets-to-missing logic...</t>
+          <t>Medium - in an employee's first year the semiannual windows differ from a fla...</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
-        <is>
-          <t>Effort: S (a few hours) - extract "latest study/assessment -&gt; status / nextDueOn / overdue" into one helper used by method comparison, cal-ver/linearity, and the competency owed derivation.
-Importance: Low - the three paths duplicate the +6-month / signed-resets-to-missing logic. They agree today (verified), but a shared helper prevents future drift and settles the dateless-signed edge in one place. No user-facing impact; studies.date is NOT NULL so the one known divergence is unreachable in practice.</t>
-        </is>
-      </c>
-      <c r="G17" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-24 session, surfaced during the coverage-recurrence build. No live defect; hygiene.
----</t>
-        </is>
-      </c>
-      <c r="H17" s="3" t="inlineStr"/>
-    </row>
-    <row r="18" ht="90" customHeight="1">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Competency "assessed this cycle" uses a flat 365-day window</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr"/>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>S-M - anchor the coverage-map "assessed this cycle" to the person's actual CL...</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>Medium - in an employee's first year the semiannual windows differ from a fla...</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>Effort: S-M - anchor the coverage-map "assessed this cycle" to the person's actual CLIA cadence (semiannual in year 1 per 42 CFR 493.1451(b)(8), annual thereafter) from staff_competency_schedules, instead of the v1 flat 365-day lookback.
 Importance: Medium - in an employee's first year the semiannual windows differ from a flat annual window, so a first-year assessment could read as current slightly longer or shorter than the true cadence. Fine for the common annual case; refine for year-1 accuracy.</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="G17" s="3" t="inlineStr">
         <is>
           <t>2026-09-24 session, VeritaComp coverage map (#48 Phase 3) v1 simplification, noted in PR #1319.
 ---</t>
         </is>
       </c>
-      <c r="H18" s="2" t="inlineStr"/>
+      <c r="H17" s="3" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H18"/>
+  <autoFilter ref="A1:H17"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1296,7 +1255,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H44"/>
+  <dimension ref="A1:H45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1354,12 +1313,12 @@
     <row r="2" ht="90" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>C43</t>
+          <t>C44</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>VeritaStaff instrument-centric (dual) assignment view</t>
+          <t>Verify-script convention backfill (was #41) + audit matcher fix</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr"/>
@@ -1367,12 +1326,12 @@
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1320. GET/PUT /staff/instruments/:id/employees (transpose of the per-employee endpoints); an "Assign by Instrument" dialog lets a director pick a test system or manual test and check off who runs it. Same staff_employee_instruments join, with the 42 CFR 493.1235(a) duty-change event emitted on newly-added pairs so both orientations trigger the same reassessment. GET verified live on SCAHC lab 2. Closed 2026-09-24.</t>
+          <t>Closure evidence: #41 was fully backfilled on 2026-06-13 (all 8 high-stakes scripts landed; see C30); it had only been mis-filed in OPEN. A 2026-09-24 re-audit initially reported 4 of 5 recent math/logic commits as missing a verify script, which was a FALSE POSITIVE: scripts/audit_verify_script_coverage.py matched only scripts/verify-*.js / .cjs, so it ignored the .mjs / .mts / .ts verify scripts the repo now ships (e.g. verify-ptcoag-multi.mts, verify-tea-criterion-format.mjs). Fixed the matcher to accept .js/.cjs/.mjs/.ts/.mts; re-run shows 5 of 5 covered, 0 debt. The convention is being followed. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 session, Michael ("in staff we should also give the dual view when assigning coverage to test systems or manual tests").
+          <t>2026-09-24 session, "keep working" pass; audit tooling bug found + fixed.
 ---</t>
         </is>
       </c>
@@ -1381,12 +1340,12 @@
     <row r="3" ht="90" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>C42</t>
+          <t>C43</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>VeritaComp coverage map (required-vs-assessed matrix, dual view)</t>
+          <t>VeritaStaff instrument-centric (dual) assignment view</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr"/>
@@ -1394,12 +1353,12 @@
       <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1319 (+ status layer PR #1316). /competency/owed returns per-item assessed (locked passing assessment this cycle on a covering method group) + per-employee CLIA status; CompetencyCoverageMap renders a By-employee / By-instrument matrix (Assessed / Owed / Overdue / Gap). Verified live on SCAHC lab 2 (owed 116, assessed 2, gaps 0). Completes #48 as the VeritaCheck-parity coverage map. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1320. GET/PUT /staff/instruments/:id/employees (transpose of the per-employee endpoints); an "Assign by Instrument" dialog lets a director pick a test system or manual test and check off who runs it. Same staff_employee_instruments join, with the 42 CFR 493.1235(a) duty-change event emitted on newly-added pairs so both orientations trigger the same reassessment. GET verified live on SCAHC lab 2. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>2026-09-24 session, Michael ("are we building the competencies to have a coverage map, same as veritacheck?" then "build it").
+          <t>2026-09-24 session, Michael ("in staff we should also give the dual view when assigning coverage to test systems or manual tests").
 ---</t>
         </is>
       </c>
@@ -1408,12 +1367,12 @@
     <row r="4" ht="90" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>C41</t>
+          <t>C42</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>VeritaCheck coverage recurrence (method comparison + cal-ver/linearity + reports)</t>
+          <t>VeritaComp coverage map (required-vs-assessed matrix, dual view)</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr"/>
@@ -1421,12 +1380,12 @@
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: PRs #1317 (method comparison), #1318 (cal-ver/linearity), #1321 (report Next-due columns). Periodic verification (correlation/method comparison 42 CFR 493.1281; cal-ver/linearity 42 CFR 493.1255; both 6-month) now recurs: a signed study banks the cycle and rolls to next-due = signed + 6 months instead of reading "done" forever. Status Missing/Failed/Completed-unsigned + a "Next due on" column on-screen and in both coverage exports; also credits the previously-ignored "correlation" study type. Root cause: computeCoverageFrom marked requirements done on mere existence, no date logic. Verified live on SCAHC lab 2 (101 correlations + 11 cal-ver rows now carry a next-due). Engine-level, all facilities. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1319 (+ status layer PR #1316). /competency/owed returns per-item assessed (locked passing assessment this cycle on a covering method group) + per-employee CLIA status; CompetencyCoverageMap renders a By-employee / By-instrument matrix (Assessed / Owed / Overdue / Gap). Verified live on SCAHC lab 2 (owed 116, assessed 2, gaps 0). Completes #48 as the VeritaCheck-parity coverage map. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 session, Michael ("Look at San Carlos... they finished their last set of correlations (all 103) but their menu never reset").
+          <t>2026-09-24 session, Michael ("are we building the competencies to have a coverage map, same as veritacheck?" then "build it").
 ---</t>
         </is>
       </c>
@@ -1435,12 +1394,12 @@
     <row r="5" ht="90" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>C40</t>
+          <t>C41</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>VeritaComp Competencies Owed derived from VeritaStaff, with gap detection (was #48)</t>
+          <t>VeritaCheck coverage recurrence (method comparison + cal-ver/linearity + reports)</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr"/>
@@ -1448,12 +1407,12 @@
       <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1314 (squash 2bcb0db9). GET /api/labs/:labId/competency/owed derives each VeritaStaff testing employee's owed competencies from their assigned instruments (staff_employee_instruments -&gt; veritamap_instruments + tests), on the CLIA timeline, and flags instruments not covered by any competency program as gaps. CompetenciesOwedSection renders it on the VeritaComp landing page. Reuses the shipped bridge + suggested-method-groups match rules; no new tables. Verified live on prod with real assignment data: 2 instruments assigned to a demo staffer produced owed=2, gaps=2 (HIGH, Technical Supervisor), then reverted cleanly. Closed 2026-09-24.</t>
+          <t>Closure evidence: PRs #1317 (method comparison), #1318 (cal-ver/linearity), #1321 (report Next-due columns). Periodic verification (correlation/method comparison 42 CFR 493.1281; cal-ver/linearity 42 CFR 493.1255; both 6-month) now recurs: a signed study banks the cycle and rolls to next-due = signed + 6 months instead of reading "done" forever. Status Missing/Failed/Completed-unsigned + a "Next due on" column on-screen and in both coverage exports; also credits the previously-ignored "correlation" study type. Root cause: computeCoverageFrom marked requirements done on mere existence, no date logic. Verified live on SCAHC lab 2 (101 correlations + 11 cal-ver rows now carry a next-due). Engine-level, all facilities. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>2026-09-23/24 session, Michael ("veritacomp bases what competencies they owe (currently untrue, but needs to be true)"). Option 1 (unify roster on VeritaStaff, match instruments by id).
+          <t>2026-09-24 session, Michael ("Look at San Carlos... they finished their last set of correlations (all 103) but their menu never reset").
 ---</t>
         </is>
       </c>
@@ -1462,12 +1421,12 @@
     <row r="6" ht="90" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>C39</t>
+          <t>C40</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>VeritaScan line items can attach or link evidence (was #46)</t>
+          <t>VeritaComp Competencies Owed derived from VeritaStaff, with gap detection (was #48)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr"/>
@@ -1475,12 +1434,12 @@
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1312 (squash a1dda93d). VeritaScan scan checklist items now show linked evidence as chips (open link, remove) plus a writer "Link evidence" affordance whose picker links an existing VeritaDC/Library document; a shortcut deep-links to the Library for new (governed) documents. Reuses the already-shipped lab_documents + document_checklist_links + coverage endpoints (URL-pointer only, no file storage, no new tables). Browser-verified live on prod (scan 23): the affordance renders and the picker opens. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1314 (squash 2bcb0db9). GET /api/labs/:labId/competency/owed derives each VeritaStaff testing employee's owed competencies from their assigned instruments (staff_employee_instruments -&gt; veritamap_instruments + tests), on the CLIA timeline, and flags instruments not covered by any competency program as gaps. CompetenciesOwedSection renders it on the VeritaComp landing page. Reuses the shipped bridge + suggested-method-groups match rules; no new tables. Verified live on prod with real assignment data: 2 instruments assigned to a demo staffer produced owed=2, gaps=2 (HIGH, Technical Supervisor), then reverted cleanly. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23 session, Michael. Recurring request. Companion: cross-module evidence display on the VeritaDC policy shipped in PR #1313 (by-target cross-links surfaced in the policy View modal, browser-verified live).
+          <t>2026-09-23/24 session, Michael ("veritacomp bases what competencies they owe (currently untrue, but needs to be true)"). Option 1 (unify roster on VeritaStaff, match instruments by id).
 ---</t>
         </is>
       </c>
@@ -1489,12 +1448,12 @@
     <row r="7" ht="90" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>C38</t>
+          <t>C39</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>VeritaTrack calendar month cells expand to reveal hidden tasks (was #45)</t>
+          <t>VeritaScan line items can attach or link evidence (was #46)</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr"/>
@@ -1502,12 +1461,12 @@
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: VeritaTrack CalendarView month cells with more than three tasks now expand in place (chevron, "+N more" toggling to "Show less", due dates), so no task is hidden with no path to it (client/src/pages/VeritaTrackAppPage.tsx CalendarView). Shipped 2026-09-23. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1312 (squash a1dda93d). VeritaScan scan checklist items now show linked evidence as chips (open link, remove) plus a writer "Link evidence" affordance whose picker links an existing VeritaDC/Library document; a shortcut deep-links to the Library for new (governed) documents. Reuses the already-shipped lab_documents + document_checklist_links + coverage endpoints (URL-pointer only, no file storage, no new tables). Browser-verified live on prod (scan 23): the affordance renders and the picker opens. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>2026-09-23 session, Michael screenshot of the VeritaTrack calendar (lab 3, September cell).
+          <t>2026-09-23 session, Michael. Recurring request. Companion: cross-module evidence display on the VeritaDC policy shipped in PR #1313 (by-target cross-links surfaced in the policy View modal, browser-verified live).
 ---</t>
         </is>
       </c>
@@ -1516,12 +1475,12 @@
     <row r="8" ht="90" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>C37</t>
+          <t>C38</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Long Excel column headers no longer clip CFR citations (was #44)</t>
+          <t>VeritaTrack calendar month cells expand to reveal hidden tasks (was #45)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr"/>
@@ -1529,12 +1488,12 @@
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. The VeritaMap export derives the header row height from the longest wrapped header via headerRowHeight(headers, colWidths) (server/routes.ts:15935) instead of a fixed 20, so "Reference Range Attestation (42 CFR 493.1253)" and the other long headers print in full. No new code this session. Closed 2026-09-24.</t>
+          <t>Closure evidence: VeritaTrack CalendarView month cells with more than three tasks now expand in place (chevron, "+N more" toggling to "Show less", due dates), so no task is hidden with no path to it (client/src/pages/VeritaTrackAppPage.tsx CalendarView). Shipped 2026-09-23. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+          <t>2026-09-23 session, Michael screenshot of the VeritaTrack calendar (lab 3, September cell).
 ---</t>
         </is>
       </c>
@@ -1543,12 +1502,12 @@
     <row r="9" ht="90" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>C36</t>
+          <t>C37</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>License stamp no longer clobbers the §6 header/footer or names the wrong lab (was #43)</t>
+          <t>Long Excel column headers no longer clip CFR citations (was #44)</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr"/>
@@ -1556,7 +1515,7 @@
       <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. setHeaderFooter (shared/licenseExceljs.ts:155-209) now preserves an existing §6 header and appends (not overwrites) the footer left section, and customer-facing exports name the scoped lab: the VeritaScan library export reads req.scope.lab.name / clia_number (server/routes.ts:16572-16573), not the licensee. No new code this session (avoided regressing the existing fix). Closed 2026-09-24.</t>
+          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. The VeritaMap export derives the header row height from the longest wrapped header via headerRowHeight(headers, colWidths) (server/routes.ts:15935) instead of a fixed 20, so "Reference Range Attestation (42 CFR 493.1253)" and the other long headers print in full. No new code this session. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -1570,18 +1529,45 @@
     <row r="10" ht="90" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>C34</t>
+          <t>C36</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Wire the two static-audit guards into CI (was #43)</t>
+          <t>License stamp no longer clobbers the §6 header/footer or names the wrong lab (was #43)</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr"/>
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. setHeaderFooter (shared/licenseExceljs.ts:155-209) now preserves an existing §6 header and appends (not overwrites) the footer left section, and customer-facing exports name the scoped lab: the VeritaScan library export reads req.scope.lab.name / clia_number (server/routes.ts:16572-16573), not the licensee. No new code this session (avoided regressing the existing fix). Closed 2026-09-24.</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+---</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11" ht="90" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>C34</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Wire the two static-audit guards into CI (was #43)</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr"/>
+      <c r="D11" s="3" t="inlineStr"/>
+      <c r="E11" s="3" t="inlineStr"/>
+      <c r="F11" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: both guards wired into the Multi-Lab Mutations Audit CI
 workflow (.github/workflows/multilab-mutations-audit.yml) as steps:
@@ -1593,24 +1579,24 @@
 (same caveat as the existing guards already in that workflow).</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr"/>
-      <c r="H10" s="2" t="inlineStr"/>
-    </row>
-    <row r="11" ht="90" customHeight="1">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="G11" s="3" t="inlineStr"/>
+      <c r="H11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12" ht="90" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>C35</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>Legacy /api/studies over-returns studies across labs (was #44)</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr"/>
-      <c r="D11" s="3" t="inlineStr"/>
-      <c r="E11" s="3" t="inlineStr"/>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr"/>
+      <c r="D12" s="2" t="inlineStr"/>
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: GET /api/studies now scopes its list to the active lab
 when one is resolved from the Referer (server/routes.ts), so every returned row
@@ -1620,24 +1606,24 @@
 mirroring the /api/labs/:labId/studies handler. Closed 2026-06-14.</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr"/>
-      <c r="H11" s="3" t="inlineStr"/>
-    </row>
-    <row r="12" ht="90" customHeight="1">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr"/>
+      <c r="H12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13" ht="90" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>C30</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>Verify-script convention backfill (was #41)</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr"/>
-      <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="2" t="inlineStr"/>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr"/>
+      <c r="D13" s="3" t="inlineStr"/>
+      <c r="E13" s="3" t="inlineStr"/>
+      <c r="F13" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: all 8 high-stakes math/logic commits now ship a paired
 scripts/verify-*.js (EP17 sensitivity, Deming lot-to-lot, CUMSUM+QC+multi-analyte,
@@ -1645,30 +1631,30 @@
 TEa boundary), per the strike-throughs in #41. Closed 2026-06-13.</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G13" s="3" t="inlineStr">
         <is>
           <t>scripts/audit_verify_script_coverage.py lookback, 2026-06-02; backfills
 landed 2026-06-03..06.
 ---</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr"/>
-    </row>
-    <row r="13" ht="90" customHeight="1">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="H13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14" ht="90" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>C31</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>VeritaPT AAA create/update/delete silently no-op in the multi-lab UI</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr"/>
-      <c r="D13" s="3" t="inlineStr"/>
-      <c r="E13" s="3" t="inlineStr"/>
-      <c r="F13" s="3" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr"/>
+      <c r="D14" s="2" t="inlineStr"/>
+      <c r="E14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #754 (commit 92ad499) added lab-scoped POST/PUT/DELETE
 /api/labs/:labId/pt/aa-records. The UI posted to the lab-scoped path but only GET
@@ -1679,30 +1665,30 @@
 route mis-filed records to the user's default lab on multi-lab accounts).</t>
         </is>
       </c>
-      <c r="G13" s="3" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>2026-06-13, found during #18 Phase 3 QA;
 scripts/audit-labscoped-write-routes.mjs now guards the class.
 ---</t>
         </is>
       </c>
-      <c r="H13" s="3" t="inlineStr"/>
-    </row>
-    <row r="14" ht="90" customHeight="1">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="H14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15" ht="90" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>C32</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>VeritaComp "Unlock assessment" false-success no-op</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr"/>
-      <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="2" t="inlineStr"/>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr"/>
+      <c r="D15" s="3" t="inlineStr"/>
+      <c r="E15" s="3" t="inlineStr"/>
+      <c r="F15" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #755 (commit 4234007) moved the unlock route to
 /api/labs/:labId/competency/assessments/:id/unlock (the path the client calls).
@@ -1713,29 +1699,29 @@
 HTML).</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="G15" s="3" t="inlineStr">
         <is>
           <t>2026-06-13, found by scripts/audit-labscoped-write-routes.mjs.
 ---</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr"/>
-    </row>
-    <row r="15" ht="90" customHeight="1">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="H15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16" ht="90" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>C33</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>FK-cascade delete 500s + NavBar laptop-width overflow</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr"/>
-      <c r="D15" s="3" t="inlineStr"/>
-      <c r="E15" s="3" t="inlineStr"/>
-      <c r="F15" s="3" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr"/>
+      <c r="D16" s="2" t="inlineStr"/>
+      <c r="E16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PRs #749/#750 fixed NavBar horizontal overflow at laptop
 widths (collapse to the hamburger below 1560px); prod-verified at 1280-1920 with the
@@ -1746,37 +1732,9 @@
 500 -&gt; 200. scripts/audit-delete-cascades.mjs guards the class.</t>
         </is>
       </c>
-      <c r="G15" s="3" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>2026-06-13 browser QA of the A7-D4 wave + retro-QC of the 72h PR window.
----</t>
-        </is>
-      </c>
-      <c r="H15" s="3" t="inlineStr"/>
-    </row>
-    <row r="16" ht="90" customHeight="1">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>C1</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>FAQ "over 25 years" -&gt; "over 23 years"</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr"/>
-      <c r="D16" s="2" t="inlineStr"/>
-      <c r="E16" s="2" t="inlineStr"/>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>Closure evidence: client/src/pages/FAQPage.tsx line 20 reads "over
-23 years" as of 2026-05-01.</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>session 299e9a73 turn 14, ~2026-04-28.
 ---</t>
         </is>
       </c>
@@ -1785,18 +1743,46 @@
     <row r="17" ht="90" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>C5</t>
+          <t>C1</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>David's VeritaQA grey-button bug (seat permissions mode)</t>
+          <t>FAQ "over 25 years" -&gt; "over 23 years"</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr"/>
       <c r="D17" s="3" t="inlineStr"/>
       <c r="E17" s="3" t="inlineStr"/>
       <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Closure evidence: client/src/pages/FAQPage.tsx line 20 reads "over
+23 years" as of 2026-05-01.</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>session 299e9a73 turn 14, ~2026-04-28.
+---</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr"/>
+    </row>
+    <row r="18" ht="90" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>David's VeritaQA grey-button bug (seat permissions mode)</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr"/>
+      <c r="D18" s="2" t="inlineStr"/>
+      <c r="E18" s="2" t="inlineStr"/>
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #10 squash-merged as commit a43fbba on
 2026-05-01 23:19 MST. Railway deploy succeeded; deployed bundle
@@ -1809,7 +1795,7 @@
 against his exact stored shape (14 of 14 expected outcomes matched).</t>
         </is>
       </c>
-      <c r="G17" s="3" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>2026-05-01 David's report; veritabench + veritastock
 weren't in MODULE_LIST so seat permissions silently defaulted to
@@ -1817,46 +1803,17 @@
 ---</t>
         </is>
       </c>
-      <c r="H17" s="3" t="inlineStr"/>
-    </row>
-    <row r="18" ht="90" customHeight="1">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>C2</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>TeamPage present-tense "TJC surveyor" check</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr"/>
-      <c r="D18" s="2" t="inlineStr"/>
-      <c r="E18" s="2" t="inlineStr"/>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>Closure evidence: site-wide search confirmed all surveyor language
-is past-tense, consistent with user's 2021-2025 service. User closed
-the item in session 299e9a73 turn 4.</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="inlineStr">
-        <is>
-          <t>session 299e9a73, ~2026-04-28.
----</t>
-        </is>
-      </c>
       <c r="H18" s="2" t="inlineStr"/>
     </row>
     <row r="19" ht="90" customHeight="1">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>C3</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>My Studies CSV/XLSX export (John as design partner)</t>
+          <t>TeamPage present-tense "TJC surveyor" check</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr"/>
@@ -1864,14 +1821,14 @@
       <c r="E19" s="3" t="inlineStr"/>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: client/src/pages/DashboardPage.tsx line 46 calls
-/api/my-studies/export. server/routes.ts line 1491 implements the
-endpoint. Pulled forward into pre-COLA per user instruction.</t>
+          <t>Closure evidence: site-wide search confirmed all surveyor language
+is past-tense, consistent with user's 2021-2025 service. User closed
+the item in session 299e9a73 turn 4.</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>session 299e9a73 turn 5, ~2026-04-28.
+          <t>session 299e9a73, ~2026-04-28.
 ---</t>
         </is>
       </c>
@@ -1880,12 +1837,12 @@
     <row r="20" ht="90" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>C4</t>
+          <t>C3</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Rotate GitHub PAT (because old PAT was committed in SESSION_HANDOFF files)</t>
+          <t>My Studies CSV/XLSX export (John as design partner)</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr"/>
@@ -1893,13 +1850,14 @@
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: no ghp_* or github_pat_* patterns in current
-SESSION_HANDOFF.md or SESSION_HANDOFF-2.md as of 2026-05-01.</t>
+          <t>Closure evidence: client/src/pages/DashboardPage.tsx line 46 calls
+/api/my-studies/export. server/routes.ts line 1491 implements the
+endpoint. Pulled forward into pre-COLA per user instruction.</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>session 299e9a73, ~2026-04-28.
+          <t>session 299e9a73 turn 5, ~2026-04-28.
 ---</t>
         </is>
       </c>
@@ -1908,18 +1866,46 @@
     <row r="21" ht="90" customHeight="1">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>C6</t>
+          <t>C4</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>VeritaPolicy service-line filtering removed (formerly #4)</t>
+          <t>Rotate GitHub PAT (because old PAT was committed in SESSION_HANDOFF files)</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr"/>
       <c r="D21" s="3" t="inlineStr"/>
       <c r="E21" s="3" t="inlineStr"/>
       <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>Closure evidence: no ghp_* or github_pat_* patterns in current
+SESSION_HANDOFF.md or SESSION_HANDOFF-2.md as of 2026-05-01.</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>session 299e9a73, ~2026-04-28.
+---</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22" ht="90" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>C6</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>VeritaPolicy service-line filtering removed (formerly #4)</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr"/>
+      <c r="D22" s="2" t="inlineStr"/>
+      <c r="E22" s="2" t="inlineStr"/>
+      <c r="F22" s="2" t="inlineStr">
         <is>
           <t>Closure rationale (operator decision 2026-05-10): Keep all
 VeritaPolicy rows. CFR-only references with no accreditor reference
@@ -1928,29 +1914,29 @@
 report misread the design intent.</t>
         </is>
       </c>
-      <c r="G21" s="3" t="inlineStr">
+      <c r="G22" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H21" s="3" t="inlineStr"/>
-    </row>
-    <row r="22" ht="90" customHeight="1">
-      <c r="A22" s="2" t="inlineStr">
+      <c r="H22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23" ht="90" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>C7</t>
         </is>
       </c>
-      <c r="B22" s="2" t="inlineStr">
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>CLIA number format validation (formerly #13)</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr"/>
-      <c r="D22" s="2" t="inlineStr"/>
-      <c r="E22" s="2" t="inlineStr"/>
-      <c r="F22" s="2" t="inlineStr">
+      <c r="C23" s="3" t="inlineStr"/>
+      <c r="D23" s="3" t="inlineStr"/>
+      <c r="E23" s="3" t="inlineStr"/>
+      <c r="F23" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: shared/validateClia.ts defines CLIA_REGEX =
 /^\d{2}D\d{7}$/ (line 24), validateClia() helper with whitespace
@@ -1961,30 +1947,30 @@
 shape exists and behaves as specified.</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr">
+      <c r="G23" s="3" t="inlineStr">
         <is>
           <t>Agent verification 2026-05-10 via grep + file read.
 Operator confirmed shipped 2026-05-10.
 ---</t>
         </is>
       </c>
-      <c r="H22" s="2" t="inlineStr"/>
-    </row>
-    <row r="23" ht="90" customHeight="1">
-      <c r="A23" s="3" t="inlineStr">
+      <c r="H23" s="3" t="inlineStr"/>
+    </row>
+    <row r="24" ht="90" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>C8</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>VeritaMap lab-wide menu toggle (formerly #19)</t>
         </is>
       </c>
-      <c r="C23" s="3" t="inlineStr"/>
-      <c r="D23" s="3" t="inlineStr"/>
-      <c r="E23" s="3" t="inlineStr"/>
-      <c r="F23" s="3" t="inlineStr">
+      <c r="C24" s="2" t="inlineStr"/>
+      <c r="D24" s="2" t="inlineStr"/>
+      <c r="E24" s="2" t="inlineStr"/>
+      <c r="F24" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: client/src/pages/VeritaMapLabwidePage.tsx
 exists and implements the labwide read-only union view. Route is
@@ -1994,59 +1980,59 @@
 parking lot plan (read-only union view, per-session toggle) shipped.</t>
         </is>
       </c>
-      <c r="G23" s="3" t="inlineStr">
+      <c r="G24" s="2" t="inlineStr">
         <is>
           <t>Agent verification 2026-05-10 via grep + file read.
 Operator confirmed shipped 2026-05-10.
 ---</t>
         </is>
       </c>
-      <c r="H23" s="3" t="inlineStr"/>
-    </row>
-    <row r="24" ht="90" customHeight="1">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>C9</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>Tier-1 smoke test checklist (formerly #6)</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr"/>
-      <c r="D24" s="2" t="inlineStr"/>
-      <c r="E24" s="2" t="inlineStr"/>
-      <c r="F24" s="2" t="inlineStr">
-        <is>
-          <t>Closure evidence: docs/smoke-test-tier1.md documents the Tier-1
-smoke-test process and post-deploy verification steps. Shipped via
-PR #81 as part of the 2026-05-10 wave.</t>
-        </is>
-      </c>
-      <c r="G24" s="2" t="inlineStr">
-        <is>
-          <t>Operator instruction 2026-05-10 in this session.
----</t>
-        </is>
-      </c>
       <c r="H24" s="2" t="inlineStr"/>
     </row>
     <row r="25" ht="90" customHeight="1">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>C10</t>
+          <t>C9</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>Per-module gating (formerly #7)</t>
+          <t>Tier-1 smoke test checklist (formerly #6)</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr"/>
       <c r="D25" s="3" t="inlineStr"/>
       <c r="E25" s="3" t="inlineStr"/>
       <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>Closure evidence: docs/smoke-test-tier1.md documents the Tier-1
+smoke-test process and post-deploy verification steps. Shipped via
+PR #81 as part of the 2026-05-10 wave.</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>Operator instruction 2026-05-10 in this session.
+---</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26" ht="90" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>C10</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Per-module gating (formerly #7)</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr"/>
+      <c r="D26" s="2" t="inlineStr"/>
+      <c r="E26" s="2" t="inlineStr"/>
+      <c r="F26" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: Client-side useIsReadOnly module keys wired
 on client/src/pages/VeritaPolicyAppPage.tsx and
@@ -2061,29 +2047,29 @@
 PR #76.</t>
         </is>
       </c>
-      <c r="G25" s="3" t="inlineStr">
+      <c r="G26" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H25" s="3" t="inlineStr"/>
-    </row>
-    <row r="26" ht="90" customHeight="1">
-      <c r="A26" s="2" t="inlineStr">
+      <c r="H26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27" ht="90" customHeight="1">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>C11</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="B27" s="3" t="inlineStr">
         <is>
           <t>VeritaStock shipped copy (formerly #8)</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr"/>
-      <c r="D26" s="2" t="inlineStr"/>
-      <c r="E26" s="2" t="inlineStr"/>
-      <c r="F26" s="2" t="inlineStr">
+      <c r="C27" s="3" t="inlineStr"/>
+      <c r="D27" s="3" t="inlineStr"/>
+      <c r="E27" s="3" t="inlineStr"/>
+      <c r="F27" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: client/src/pages/ArticleInventoryManagementPage.tsx
 line 305 footer reads "platform that includes VeritaStock™" instead
@@ -2091,29 +2077,29 @@
 on /resources/laboratory-inventory-management. Shipped via PR #75.</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr">
+      <c r="G27" s="3" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H26" s="2" t="inlineStr"/>
-    </row>
-    <row r="27" ht="90" customHeight="1">
-      <c r="A27" s="3" t="inlineStr">
+      <c r="H27" s="3" t="inlineStr"/>
+    </row>
+    <row r="28" ht="90" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>C12</t>
         </is>
       </c>
-      <c r="B27" s="3" t="inlineStr">
+      <c r="B28" s="2" t="inlineStr">
         <is>
           <t>Admin report one-row-per-lab (formerly #14)</t>
         </is>
       </c>
-      <c r="C27" s="3" t="inlineStr"/>
-      <c r="D27" s="3" t="inlineStr"/>
-      <c r="E27" s="3" t="inlineStr"/>
-      <c r="F27" s="3" t="inlineStr">
+      <c r="C28" s="2" t="inlineStr"/>
+      <c r="D28" s="2" t="inlineStr"/>
+      <c r="E28" s="2" t="inlineStr"/>
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: /api/admin/report rewritten in
 server/routes.ts (~line 595) to LEFT JOIN labs on
@@ -2128,33 +2114,6 @@
 prerequisite, not a code bug). Shipped via PR #85.</t>
         </is>
       </c>
-      <c r="G27" s="3" t="inlineStr">
-        <is>
-          <t>Operator instruction 2026-05-10 in this session.
----</t>
-        </is>
-      </c>
-      <c r="H27" s="3" t="inlineStr"/>
-    </row>
-    <row r="28" ht="90" customHeight="1">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>C14</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>UI relabel "CLIA TEa" -&gt; "Lab-Set Internal Goal" (formerly #1)</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="inlineStr"/>
-      <c r="D28" s="2" t="inlineStr"/>
-      <c r="E28" s="2" t="inlineStr"/>
-      <c r="F28" s="2" t="inlineStr">
-        <is>
-          <t>Closure evidence: Shipped across four PRs over 2026-05-10.</t>
-        </is>
-      </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
@@ -2166,18 +2125,45 @@
     <row r="29" ht="90" customHeight="1">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>C13</t>
+          <t>C14</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>WSLH PT vendor (formerly #15)</t>
+          <t>UI relabel "CLIA TEa" -&gt; "Lab-Set Internal Goal" (formerly #1)</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr"/>
       <c r="D29" s="3" t="inlineStr"/>
       <c r="E29" s="3" t="inlineStr"/>
       <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>Closure evidence: Shipped across four PRs over 2026-05-10.</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>Operator instruction 2026-05-10 in this session.
+---</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr"/>
+    </row>
+    <row r="30" ht="90" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>C13</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>WSLH PT vendor (formerly #15)</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr"/>
+      <c r="D30" s="2" t="inlineStr"/>
+      <c r="E30" s="2" t="inlineStr"/>
+      <c r="F30" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: Shipped 2026-05-10 via PR #79 (merge commit
 eeebc6e; merged after rebase to resolve a server/db.ts collision
@@ -2195,38 +2181,9 @@
 'WSLH' is the post-deploy success signal. Shipped via PR #79.</t>
         </is>
       </c>
-      <c r="G29" s="3" t="inlineStr">
+      <c r="G30" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
----</t>
-        </is>
-      </c>
-      <c r="H29" s="3" t="inlineStr"/>
-    </row>
-    <row r="30" ht="90" customHeight="1">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>C15</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>VeritaStock lot tracking + expiration + reorder alerts (formerly #21)</t>
-        </is>
-      </c>
-      <c r="C30" s="2" t="inlineStr"/>
-      <c r="D30" s="2" t="inlineStr"/>
-      <c r="E30" s="2" t="inlineStr"/>
-      <c r="F30" s="2" t="inlineStr">
-        <is>
-          <t>Closure evidence: VeritaStock™ shipped the bench-level inventory
-features the Perplexity competitor analysis identified as a gap:</t>
-        </is>
-      </c>
-      <c r="G30" s="2" t="inlineStr">
-        <is>
-          <t>Originally Perplexity competitor analysis 2026-05-10.
-Audit 2026-05-21 confirmed the feature set ships today.
 ---</t>
         </is>
       </c>
@@ -2235,12 +2192,12 @@
     <row r="31" ht="90" customHeight="1">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>C16</t>
+          <t>C15</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>PAL studies guided workflow (formerly #23)</t>
+          <t>VeritaStock lot tracking + expiration + reorder alerts (formerly #21)</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr"/>
@@ -2248,15 +2205,14 @@
       <c r="E31" s="3" t="inlineStr"/>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: VeritaCheck™ already ships the Precision /
-Accuracy / Linearity (PAL) study set under EP-protocol naming:</t>
+          <t>Closure evidence: VeritaStock™ shipped the bench-level inventory
+features the Perplexity competitor analysis identified as a gap:</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
           <t>Originally Perplexity competitor analysis 2026-05-10.
-Audit 2026-05-21 confirmed the EP studies cover the PAL framing in
-full.
+Audit 2026-05-21 confirmed the feature set ships today.
 ---</t>
         </is>
       </c>
@@ -2265,12 +2221,12 @@
     <row r="32" ht="90" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>C17</t>
+          <t>C16</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Source-grounded 21/29/45 CFR + 42 CFR 482-485 (formerly #26)</t>
+          <t>PAL studies guided workflow (formerly #23)</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr"/>
@@ -2278,35 +2234,65 @@
       <c r="E32" s="2" t="inlineStr"/>
       <c r="F32" s="2" t="inlineStr">
         <is>
+          <t>Closure evidence: VeritaCheck™ already ships the Precision /
+Accuracy / Linearity (PAL) study set under EP-protocol naming:</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>Originally Perplexity competitor analysis 2026-05-10.
+Audit 2026-05-21 confirmed the EP studies cover the PAL framing in
+full.
+---</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33" ht="90" customHeight="1">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>C17</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Source-grounded 21/29/45 CFR + 42 CFR 482-485 (formerly #26)</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr"/>
+      <c r="D33" s="3" t="inlineStr"/>
+      <c r="E33" s="3" t="inlineStr"/>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
           <t>Closure evidence: PR #301 (commit 8c27806, merged 2026-05-21)
 source-grounded the 74 remaining non-493 entries in
 server/cfrRequirements.ts against verbatim eCFR XML. Breakdown
 shipped:</t>
         </is>
       </c>
-      <c r="G32" s="2" t="inlineStr">
+      <c r="G33" s="3" t="inlineStr">
         <is>
           <t>PR #301; tasks #18 in the in-session task tracker.
 ---</t>
         </is>
       </c>
-      <c r="H32" s="2" t="inlineStr"/>
-    </row>
-    <row r="33" ht="90" customHeight="1">
-      <c r="A33" s="3" t="inlineStr">
+      <c r="H33" s="3" t="inlineStr"/>
+    </row>
+    <row r="34" ht="90" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
         <is>
           <t>C18</t>
         </is>
       </c>
-      <c r="B33" s="3" t="inlineStr">
+      <c r="B34" s="2" t="inlineStr">
         <is>
           <t>VeritaPolicy "Non CLIA" chapter rename (formerly #3)</t>
         </is>
       </c>
-      <c r="C33" s="3" t="inlineStr"/>
-      <c r="D33" s="3" t="inlineStr"/>
-      <c r="E33" s="3" t="inlineStr"/>
-      <c r="F33" s="3" t="inlineStr">
+      <c r="C34" s="2" t="inlineStr"/>
+      <c r="D34" s="2" t="inlineStr"/>
+      <c r="E34" s="2" t="inlineStr"/>
+      <c r="F34" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #300 (commit 34d7707, merged 2026-05-21)
 renamed all 44 user-facing chapter labels in
@@ -2317,7 +2303,7 @@
 page.</t>
         </is>
       </c>
-      <c r="G33" s="3" t="inlineStr">
+      <c r="G34" s="2" t="inlineStr">
         <is>
           <t>CAP customer screenshot of the /veritapolicy chapter
 headers, 2026-05-01 evening. PR #300; tasks #17 in the in-session
@@ -2325,23 +2311,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H33" s="3" t="inlineStr"/>
-    </row>
-    <row r="34" ht="90" customHeight="1">
-      <c r="A34" s="2" t="inlineStr">
+      <c r="H34" s="2" t="inlineStr"/>
+    </row>
+    <row r="35" ht="90" customHeight="1">
+      <c r="A35" s="3" t="inlineStr">
         <is>
           <t>C19</t>
         </is>
       </c>
-      <c r="B34" s="2" t="inlineStr">
+      <c r="B35" s="3" t="inlineStr">
         <is>
           <t>VeritaStock department-scope toggle (formerly #31)</t>
         </is>
       </c>
-      <c r="C34" s="2" t="inlineStr"/>
-      <c r="D34" s="2" t="inlineStr"/>
-      <c r="E34" s="2" t="inlineStr"/>
-      <c r="F34" s="2" t="inlineStr">
+      <c r="C35" s="3" t="inlineStr"/>
+      <c r="D35" s="3" t="inlineStr"/>
+      <c r="E35" s="3" t="inlineStr"/>
+      <c r="F35" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #319 (commit d01f5fe, merged 2026-05-22)
 shipped the persistent dept-scope toggle on VeritaStockPage. A new
@@ -2352,7 +2338,7 @@
 workspace without re-filtering.</t>
         </is>
       </c>
-      <c r="G34" s="2" t="inlineStr">
+      <c r="G35" s="3" t="inlineStr">
         <is>
           <t>John, San Carlos lab, 2026-05-21. Same conversation that
 drove the vendor dropdown (PR #304), FILTERED VIEW banner (PR #305),
@@ -2360,23 +2346,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H34" s="2" t="inlineStr"/>
-    </row>
-    <row r="35" ht="90" customHeight="1">
-      <c r="A35" s="3" t="inlineStr">
+      <c r="H35" s="3" t="inlineStr"/>
+    </row>
+    <row r="36" ht="90" customHeight="1">
+      <c r="A36" s="2" t="inlineStr">
         <is>
           <t>C20</t>
         </is>
       </c>
-      <c r="B35" s="3" t="inlineStr">
+      <c r="B36" s="2" t="inlineStr">
         <is>
           <t>Primary-lab seat counting (formerly #12)</t>
         </is>
       </c>
-      <c r="C35" s="3" t="inlineStr"/>
-      <c r="D35" s="3" t="inlineStr"/>
-      <c r="E35" s="3" t="inlineStr"/>
-      <c r="F35" s="3" t="inlineStr">
+      <c r="C36" s="2" t="inlineStr"/>
+      <c r="D36" s="2" t="inlineStr"/>
+      <c r="E36" s="2" t="inlineStr"/>
+      <c r="F36" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: is_primary_lab INTEGER NOT NULL DEFAULT 0
 column was added to the lab_members table at db.ts:1276, with the
@@ -2387,7 +2373,7 @@
 is_primary_lab=1 ordering).</t>
         </is>
       </c>
-      <c r="G35" s="3" t="inlineStr">
+      <c r="G36" s="2" t="inlineStr">
         <is>
           <t>2026-05-07 multi-lab discussion. Build shipped as part
 of the Multi-Lab Tier 2 architecture work (Phase 3.x series, prior
@@ -2396,23 +2382,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H35" s="3" t="inlineStr"/>
-    </row>
-    <row r="36" ht="90" customHeight="1">
-      <c r="A36" s="2" t="inlineStr">
+      <c r="H36" s="2" t="inlineStr"/>
+    </row>
+    <row r="37" ht="90" customHeight="1">
+      <c r="A37" s="3" t="inlineStr">
         <is>
           <t>C21</t>
         </is>
       </c>
-      <c r="B36" s="2" t="inlineStr">
+      <c r="B37" s="3" t="inlineStr">
         <is>
           <t>Multi-lab pricing model — Option A (formerly #11)</t>
         </is>
       </c>
-      <c r="C36" s="2" t="inlineStr"/>
-      <c r="D36" s="2" t="inlineStr"/>
-      <c r="E36" s="2" t="inlineStr"/>
-      <c r="F36" s="2" t="inlineStr">
+      <c r="C37" s="3" t="inlineStr"/>
+      <c r="D37" s="3" t="inlineStr"/>
+      <c r="E37" s="3" t="inlineStr"/>
+      <c r="F37" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #322 (commit 0ccd925, merged 2026-05-22)
 added the customer-facing line to the pricing page that reflects
@@ -2425,7 +2411,7 @@
 Enterprise+ block, reads:</t>
         </is>
       </c>
-      <c r="G36" s="2" t="inlineStr">
+      <c r="G37" s="3" t="inlineStr">
         <is>
           <t>2026-05-07 multi-lab discussion (Lisa Veri's
 canonical-case session). PR #322 (initial build); softening PR
@@ -2434,30 +2420,30 @@
 ---</t>
         </is>
       </c>
-      <c r="H36" s="2" t="inlineStr"/>
-    </row>
-    <row r="37" ht="90" customHeight="1">
-      <c r="A37" s="3" t="inlineStr">
+      <c r="H37" s="3" t="inlineStr"/>
+    </row>
+    <row r="38" ht="90" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
         <is>
           <t>C22</t>
         </is>
       </c>
-      <c r="B37" s="3" t="inlineStr">
+      <c r="B38" s="2" t="inlineStr">
         <is>
           <t>VeritaOps cost-per-test module (formerly #10)</t>
         </is>
       </c>
-      <c r="C37" s="3" t="inlineStr"/>
-      <c r="D37" s="3" t="inlineStr"/>
-      <c r="E37" s="3" t="inlineStr"/>
-      <c r="F37" s="3" t="inlineStr">
+      <c r="C38" s="2" t="inlineStr"/>
+      <c r="D38" s="2" t="inlineStr"/>
+      <c r="E38" s="2" t="inlineStr"/>
+      <c r="F38" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: v1 of the VeritaOps Cost-Per-Reportable-Test
 (CPRT) module shipped across PR #325 through PR #330 on 2026-05-22.
 The module is feature-complete for the typical lab director workflow.</t>
         </is>
       </c>
-      <c r="G37" s="3" t="inlineStr">
+      <c r="G38" s="2" t="inlineStr">
         <is>
           <t>This thread, 2026-05-07 12:05 PM CDT, user message:
 "Parking lot: build an operations module for cost per test
@@ -2466,262 +2452,262 @@
 ---</t>
         </is>
       </c>
-      <c r="H37" s="3" t="inlineStr"/>
-    </row>
-    <row r="38" ht="90" customHeight="1">
-      <c r="A38" s="2" t="inlineStr">
+      <c r="H38" s="2" t="inlineStr"/>
+    </row>
+    <row r="39" ht="90" customHeight="1">
+      <c r="A39" s="3" t="inlineStr">
         <is>
           <t>C23</t>
         </is>
       </c>
-      <c r="B38" s="2" t="inlineStr">
+      <c r="B39" s="3" t="inlineStr">
         <is>
           <t>CCL lab name visual disambiguation in lab switcher (formerly #34)</t>
         </is>
       </c>
-      <c r="C38" s="2" t="inlineStr"/>
-      <c r="D38" s="2" t="inlineStr">
+      <c r="C39" s="3" t="inlineStr"/>
+      <c r="D39" s="3" t="inlineStr">
         <is>
           <t>XS (under 1 day, actual)</t>
         </is>
       </c>
-      <c r="E38" s="2" t="inlineStr">
+      <c r="E39" s="3" t="inlineStr">
         <is>
           <t>Low — cosmetic; only mattered when Lisa or Michael picked the wrong lab from...</t>
         </is>
       </c>
-      <c r="F38" s="2" t="inlineStr">
+      <c r="F39" s="3" t="inlineStr">
         <is>
           <t>Effort: XS (under 1 day, actual)
 Importance: Low — cosmetic; only mattered when Lisa or Michael picked the wrong lab from the dropdown.</t>
         </is>
       </c>
-      <c r="G38" s="2" t="inlineStr">
+      <c r="G39" s="3" t="inlineStr">
         <is>
           <t>flagged 2026-05-23 immediately after provisioning Lisa's CCL lab; closed 2026-05-24.
 ---</t>
         </is>
       </c>
-      <c r="H38" s="2" t="inlineStr"/>
-    </row>
-    <row r="39" ht="90" customHeight="1">
-      <c r="A39" s="3" t="inlineStr">
+      <c r="H39" s="3" t="inlineStr"/>
+    </row>
+    <row r="40" ht="90" customHeight="1">
+      <c r="A40" s="2" t="inlineStr">
         <is>
           <t>C24</t>
         </is>
       </c>
-      <c r="B39" s="3" t="inlineStr">
+      <c r="B40" s="2" t="inlineStr">
         <is>
           <t>VC Unlimited Y1/Y2 price disclosure UX (formerly #35)</t>
         </is>
       </c>
-      <c r="C39" s="3" t="inlineStr"/>
-      <c r="D39" s="3" t="inlineStr">
+      <c r="C40" s="2" t="inlineStr"/>
+      <c r="D40" s="2" t="inlineStr">
         <is>
           <t>XS (under 1 day, actual)</t>
         </is>
       </c>
-      <c r="E39" s="3" t="inlineStr">
+      <c r="E40" s="2" t="inlineStr">
         <is>
           <t>Low when shipped (proactive, no customer complaint yet) — but high if a procu...</t>
         </is>
       </c>
-      <c r="F39" s="3" t="inlineStr">
+      <c r="F40" s="2" t="inlineStr">
         <is>
           <t>Effort: XS (under 1 day, actual)
 Importance: Low when shipped (proactive, no customer complaint yet) — but high if a procurement reviewer later disputes the $499 renewal as undisclosed.</t>
         </is>
       </c>
-      <c r="G39" s="3" t="inlineStr">
+      <c r="G40" s="2" t="inlineStr">
         <is>
           <t>Pricing rebuild 2026-05-23; closed 2026-05-24 proactively before any customer dispute.
 ---</t>
         </is>
       </c>
-      <c r="H39" s="3" t="inlineStr"/>
-    </row>
-    <row r="40" ht="90" customHeight="1">
-      <c r="A40" s="2" t="inlineStr">
+      <c r="H40" s="2" t="inlineStr"/>
+    </row>
+    <row r="41" ht="90" customHeight="1">
+      <c r="A41" s="3" t="inlineStr">
         <is>
           <t>C25</t>
         </is>
       </c>
-      <c r="B40" s="2" t="inlineStr">
+      <c r="B41" s="3" t="inlineStr">
         <is>
           <t>VeritaQC Phase 1 (Levey-Jennings + Westgard live engine) (formerly #20)</t>
         </is>
       </c>
-      <c r="C40" s="2" t="inlineStr"/>
-      <c r="D40" s="2" t="inlineStr">
+      <c r="C41" s="3" t="inlineStr"/>
+      <c r="D41" s="3" t="inlineStr">
         <is>
           <t>L (about 5 days end-to-end, actual: Phase 0 schema → Phase 1A evaluator → 1B...</t>
         </is>
       </c>
-      <c r="E40" s="2" t="inlineStr">
+      <c r="E41" s="3" t="inlineStr">
         <is>
           <t>High — largest single gap vs myLabCompliance.io per Perplexity competitor ana...</t>
         </is>
       </c>
-      <c r="F40" s="2" t="inlineStr">
+      <c r="F41" s="3" t="inlineStr">
         <is>
           <t>Effort: L (about 5 days end-to-end, actual: Phase 0 schema → Phase 1A evaluator → 1B entry UI → 1C daily review → 1D monthly PDF + attestation)
 Importance: High — largest single gap vs myLabCompliance.io per Perplexity competitor analysis; promotes VeritaAssure from documentation tool to lab operations platform.</t>
         </is>
       </c>
-      <c r="G40" s="2" t="inlineStr">
+      <c r="G41" s="3" t="inlineStr">
         <is>
           <t>Perplexity competitor analysis 2026-05-10. Scoping confirmed via the build_phase1_mockup.py iterations 2026-05-24. Shipped 2026-05-25.
 ---</t>
         </is>
       </c>
-      <c r="H40" s="2" t="inlineStr"/>
-    </row>
-    <row r="41" ht="90" customHeight="1">
-      <c r="A41" s="3" t="inlineStr">
+      <c r="H41" s="3" t="inlineStr"/>
+    </row>
+    <row r="42" ht="90" customHeight="1">
+      <c r="A42" s="2" t="inlineStr">
         <is>
           <t>C26</t>
         </is>
       </c>
-      <c r="B41" s="3" t="inlineStr">
+      <c r="B42" s="2" t="inlineStr">
         <is>
           <t>VeritaLab CMS-116 application support + state licensing registry (formerly #22)</t>
         </is>
       </c>
-      <c r="C41" s="3" t="inlineStr"/>
-      <c r="D41" s="3" t="inlineStr">
+      <c r="C42" s="2" t="inlineStr"/>
+      <c r="D42" s="2" t="inlineStr">
         <is>
           <t>M (1-2 weeks for v1, actual)</t>
         </is>
       </c>
-      <c r="E41" s="3" t="inlineStr">
+      <c r="E42" s="2" t="inlineStr">
         <is>
           <t>Medium — competitor parity (myLabCompliance.io) plus useful at lab startup an...</t>
         </is>
       </c>
-      <c r="F41" s="3" t="inlineStr">
+      <c r="F42" s="2" t="inlineStr">
         <is>
           <t>Effort: M (1-2 weeks for v1, actual)
 Importance: Medium — competitor parity (myLabCompliance.io) plus useful at lab startup and at certificate-type changes.</t>
         </is>
       </c>
-      <c r="G41" s="3" t="inlineStr">
+      <c r="G42" s="2" t="inlineStr">
         <is>
           <t>Perplexity competitor analysis (myLabCompliance.io), 2026-05-10. Reclassified as a VeritaLab extension 2026-05-25. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H41" s="3" t="inlineStr"/>
-    </row>
-    <row r="42" ht="90" customHeight="1">
-      <c r="A42" s="2" t="inlineStr">
+      <c r="H42" s="2" t="inlineStr"/>
+    </row>
+    <row r="43" ht="90" customHeight="1">
+      <c r="A43" s="3" t="inlineStr">
         <is>
           <t>C27</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
+      <c r="B43" s="3" t="inlineStr">
         <is>
           <t>Active vs view-only seat split (formerly #33)</t>
         </is>
       </c>
-      <c r="C42" s="2" t="inlineStr"/>
-      <c r="D42" s="2" t="inlineStr">
+      <c r="C43" s="3" t="inlineStr"/>
+      <c r="D43" s="3" t="inlineStr">
         <is>
           <t>M (~1 week of engineering, actual: shipped in a single multi-PR session)</t>
         </is>
       </c>
-      <c r="E42" s="2" t="inlineStr">
+      <c r="E43" s="3" t="inlineStr">
         <is>
           <t>Medium — closed the gap between /pricing copy and product behavior; gives sal...</t>
         </is>
       </c>
-      <c r="F42" s="2" t="inlineStr">
+      <c r="F43" s="3" t="inlineStr">
         <is>
           <t>Effort: M (~1 week of engineering, actual: shipped in a single multi-PR session)
 Importance: Medium — closed the gap between /pricing copy and product behavior; gives sales a clean answer for "do you charge for our medical director?"</t>
         </is>
       </c>
-      <c r="G42" s="2" t="inlineStr">
+      <c r="G43" s="3" t="inlineStr">
         <is>
           <t>Pricing analysis doc Decision 3 (2026-05-21); MEDIUM scenario revised 2026-05-29 to retire the "unlimited view-only" claim. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H42" s="2" t="inlineStr"/>
-    </row>
-    <row r="43" ht="90" customHeight="1">
-      <c r="A43" s="3" t="inlineStr">
+      <c r="H43" s="3" t="inlineStr"/>
+    </row>
+    <row r="44" ht="90" customHeight="1">
+      <c r="A44" s="2" t="inlineStr">
         <is>
           <t>C28</t>
         </is>
       </c>
-      <c r="B43" s="3" t="inlineStr">
+      <c r="B44" s="2" t="inlineStr">
         <is>
           <t>"Why VeritaCheck" comparative one-pager (formerly #37)</t>
         </is>
       </c>
-      <c r="C43" s="3" t="inlineStr"/>
-      <c r="D43" s="3" t="inlineStr">
+      <c r="C44" s="2" t="inlineStr"/>
+      <c r="D44" s="2" t="inlineStr">
         <is>
           <t>S (one design pass + four claim paragraphs + PDF + matching marketing-site pa...</t>
         </is>
       </c>
-      <c r="E43" s="3" t="inlineStr">
+      <c r="E44" s="2" t="inlineStr">
         <is>
           <t>Medium — closed a positioning gap surfaced by six COLA conference attendees a...</t>
         </is>
       </c>
-      <c r="F43" s="3" t="inlineStr">
+      <c r="F44" s="2" t="inlineStr">
         <is>
           <t>Effort: S (one design pass + four claim paragraphs + PDF + matching marketing-site page, actual)
 Importance: Medium — closed a positioning gap surfaced by six COLA conference attendees attached to a legacy verification tool; converts product-quality advantage into a leave-behind Lisa can hand out.</t>
         </is>
       </c>
-      <c r="G43" s="3" t="inlineStr">
+      <c r="G44" s="2" t="inlineStr">
         <is>
           <t>2026-05-11 / 2026-05-12 conference notes review with Michael. Conference attendees (Whitehead, Odegard, Othman, Molinelli, Kyle, Allred) expressed interest in equivalent / superior product. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H43" s="3" t="inlineStr"/>
-    </row>
-    <row r="44" ht="90" customHeight="1">
-      <c r="A44" s="2" t="inlineStr">
+      <c r="H44" s="2" t="inlineStr"/>
+    </row>
+    <row r="45" ht="90" customHeight="1">
+      <c r="A45" s="3" t="inlineStr">
         <is>
           <t>C29</t>
         </is>
       </c>
-      <c r="B44" s="2" t="inlineStr">
+      <c r="B45" s="3" t="inlineStr">
         <is>
           <t>VeritaPolicy approval workflow — MediaLab functional mirror</t>
         </is>
       </c>
-      <c r="C44" s="2" t="inlineStr"/>
-      <c r="D44" s="2" t="inlineStr">
+      <c r="C45" s="3" t="inlineStr"/>
+      <c r="D45" s="3" t="inlineStr">
         <is>
           <t>XL (one focused session, 12 PRs landed)</t>
         </is>
       </c>
-      <c r="E44" s="2" t="inlineStr">
+      <c r="E45" s="3" t="inlineStr">
         <is>
           <t>High — replaces MediaLab Document Control ($752/$2,250 starting price, scalin...</t>
         </is>
       </c>
-      <c r="F44" s="2" t="inlineStr">
+      <c r="F45" s="3" t="inlineStr">
         <is>
           <t>Effort: XL (one focused session, 12 PRs landed)
 Importance: High — replaces MediaLab Document Control ($752/$2,250 starting price, scaling to $10K-$20K/yr at enterprise per Capterra public data) with an included VeritaPolicy feature; closes a real positioning gap and gives sales a direct comparator line.</t>
         </is>
       </c>
-      <c r="G44" s="2" t="inlineStr">
+      <c r="G45" s="3" t="inlineStr">
         <is>
           <t>Pricing strategy conversation 2026-05-29 (Michael: "I don't like bolt-ons; we should replicate this") → scoped 8 phases → shipped all 12 PRs in single session. Shipped 2026-05-29.
 ---</t>
         </is>
       </c>
-      <c r="H44" s="2" t="inlineStr"/>
+      <c r="H45" s="3" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H44"/>
+  <autoFilter ref="A1:H45"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
TASK: Parking-lot sync - close #49 as a non-issue and log the shipped verified-users email path.
PLAN:
  1. Close #49 (unify recurrence helper): investigation showed coverage recurrence is already single-source and competency cadence is a different CFR interval that should not be merged. Move to CLOSED as C45.
  2. Log the verified-users product-update send path (PR #1324) as CLOSED C46 with the incident context.
  3. Rebuild PARKING_LOT.xlsx.

Self-check:
  - #49 removed from OPEN exactly once (regex subn asserted ==1); C45 + C46 present; #50 left open.
  - Counts: OPEN 15 / CLOSED 46 / RETIRED 6.
  - Internal docs + sync script only; Gate 3 N/A.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PARKING_LOT.xlsx
+++ b/PARKING_LOT.xlsx
@@ -12,8 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RETIRED" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$45</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$47</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RETIRED'!$A$1:$H$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1174,77 +1174,41 @@
     <row r="16" ht="90" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>50</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Unify the coverage/competency recurrence into one shared helper (tech debt)</t>
+          <t>Competency "assessed this cycle" uses a flat 365-day window</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr"/>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>S (a few hours) - extract "latest study/assessment -&gt; status / nextDueOn / ov...</t>
+          <t>S-M - anchor the coverage-map "assessed this cycle" to the person's actual CL...</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Low - the three paths duplicate the +6-month / signed-resets-to-missing logic...</t>
+          <t>Medium - in an employee's first year the semiannual windows differ from a fla...</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>Effort: S (a few hours) - extract "latest study/assessment -&gt; status / nextDueOn / overdue" into one helper used by method comparison, cal-ver/linearity, and the competency owed derivation.
-Importance: Low - the three paths duplicate the +6-month / signed-resets-to-missing logic. They agree today (verified), but a shared helper prevents future drift and settles the dateless-signed edge in one place. No user-facing impact; studies.date is NOT NULL so the one known divergence is unreachable in practice.</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-24 session, surfaced during the coverage-recurrence build. No live defect; hygiene.
----</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr"/>
-    </row>
-    <row r="17" ht="90" customHeight="1">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>Competency "assessed this cycle" uses a flat 365-day window</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="inlineStr"/>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>S-M - anchor the coverage-map "assessed this cycle" to the person's actual CL...</t>
-        </is>
-      </c>
-      <c r="E17" s="3" t="inlineStr">
-        <is>
-          <t>Medium - in an employee's first year the semiannual windows differ from a fla...</t>
-        </is>
-      </c>
-      <c r="F17" s="3" t="inlineStr">
         <is>
           <t>Effort: S-M - anchor the coverage-map "assessed this cycle" to the person's actual CLIA cadence (semiannual in year 1 per 42 CFR 493.1451(b)(8), annual thereafter) from staff_competency_schedules, instead of the v1 flat 365-day lookback.
 Importance: Medium - in an employee's first year the semiannual windows differ from a flat annual window, so a first-year assessment could read as current slightly longer or shorter than the true cadence. Fine for the common annual case; refine for year-1 accuracy.</t>
         </is>
       </c>
-      <c r="G17" s="3" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>2026-09-24 session, VeritaComp coverage map (#48 Phase 3) v1 simplification, noted in PR #1319.
 ---</t>
         </is>
       </c>
-      <c r="H17" s="3" t="inlineStr"/>
+      <c r="H16" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H17"/>
+  <autoFilter ref="A1:H16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1255,7 +1219,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H45"/>
+  <dimension ref="A1:H47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1313,12 +1277,12 @@
     <row r="2" ht="90" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>C44</t>
+          <t>C45</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Verify-script convention backfill (was #41) + audit matcher fix</t>
+          <t>Unify coverage/competency recurrence helper (was #49) - closed as non-issue</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr"/>
@@ -1326,12 +1290,12 @@
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: #41 was fully backfilled on 2026-06-13 (all 8 high-stakes scripts landed; see C30); it had only been mis-filed in OPEN. A 2026-09-24 re-audit initially reported 4 of 5 recent math/logic commits as missing a verify script, which was a FALSE POSITIVE: scripts/audit_verify_script_coverage.py matched only scripts/verify-*.js / .cjs, so it ignored the .mjs / .mts / .ts verify scripts the repo now ships (e.g. verify-ptcoag-multi.mts, verify-tea-criterion-format.mjs). Fixed the matcher to accept .js/.cjs/.mjs/.ts/.mts; re-run shows 5 of 5 covered, 0 debt. The convention is being followed. Closed 2026-09-24.</t>
+          <t>Closure evidence: Investigated 2026-09-24 before building. The coverage recurrence math (+6-month interval, signed-resets-to-missing, nextDueOn/overdue, isFailVerdict) is ALREADY single-source in server/veritacheckCoverage.ts (computeCoverageFrom). server/coverageReport.ts and the routes.ts coverage export do not recompute it; they consume the computed nextDueOn/overdue/status fields and apply small surface-specific presentation labels (deliberately different vocabularies per surface, so they should not be merged). The only truly identical duplicate is a one-line date formatter. The competency "owed" derivation is NOT the same cadence: competency follows the CLIA milestone schedule (initial / semiannual year 1 / annual, 42 CFR 493.1451(b)(8) and 493.1235), which is a different regulatory interval from the coverage 6-month rule (493.1281 / 493.1255) and must stay separate. No worthwhile extraction; merging the two cadences would be wrong. Closed 2026-09-24. (The year-1 competency-window refinement remains tracked separately as #50.)</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 session, "keep working" pass; audit tooling bug found + fixed.
+          <t>2026-09-24 session, "keep working" pass; scoped read-only, found no real duplication.
 ---</t>
         </is>
       </c>
@@ -1340,12 +1304,12 @@
     <row r="3" ht="90" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>C43</t>
+          <t>C46</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>VeritaStaff instrument-centric (dual) assignment view</t>
+          <t>Verified-users product-update send path (wrong-list incident fix)</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr"/>
@@ -1353,12 +1317,12 @@
       <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1320. GET/PUT /staff/instruments/:id/employees (transpose of the per-employee endpoints); an "Assign by Instrument" dialog lets a director pick a test system or manual test and check off who runs it. Same staff_employee_instruments join, with the 42 CFR 493.1235(a) duty-change event emitted on newly-added pairs so both orientations trigger the same reassessment. GET verified live on SCAHC lab 2. Closed 2026-09-24.</t>
+          <t>Closure evidence: Shipped PR #1324 (merged 4e05506a, deploy ACTIVE). New POST /api/admin/users/send targets registered VeritaAssure account holders (the users table), never the Lab Director's Briefing subscriber list. Separate explicitly-named endpoint (not a flag with a dangerous default), account-holder email framing, excludes suppressed emails and RFC-reserved test domains, CC owner, dryRun + testTo previews. Public unsubscribe now upserts a suppression row so opt-outs are honored across both audiences. Live dryRun: 49 verified-user recipients vs 673 on the Briefing list. Receipts: scripts/verify-product-update-send.mts 24/24, tsc clean, rendered sample inspected. Fixes the fallout from the 2026-09-23/24 wrong-list send (a product update went to the 675-person Briefing list). Nothing sends without Michael's explicit "send it."</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>2026-09-24 session, Michael ("in staff we should also give the dual view when assigning coverage to test systems or manual tests").
+          <t>2026-09-24 session; Michael selected this as the next build after the #41 close.
 ---</t>
         </is>
       </c>
@@ -1367,12 +1331,12 @@
     <row r="4" ht="90" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>C42</t>
+          <t>C44</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>VeritaComp coverage map (required-vs-assessed matrix, dual view)</t>
+          <t>Verify-script convention backfill (was #41) + audit matcher fix</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr"/>
@@ -1380,12 +1344,12 @@
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1319 (+ status layer PR #1316). /competency/owed returns per-item assessed (locked passing assessment this cycle on a covering method group) + per-employee CLIA status; CompetencyCoverageMap renders a By-employee / By-instrument matrix (Assessed / Owed / Overdue / Gap). Verified live on SCAHC lab 2 (owed 116, assessed 2, gaps 0). Completes #48 as the VeritaCheck-parity coverage map. Closed 2026-09-24.</t>
+          <t>Closure evidence: #41 was fully backfilled on 2026-06-13 (all 8 high-stakes scripts landed; see C30); it had only been mis-filed in OPEN. A 2026-09-24 re-audit initially reported 4 of 5 recent math/logic commits as missing a verify script, which was a FALSE POSITIVE: scripts/audit_verify_script_coverage.py matched only scripts/verify-*.js / .cjs, so it ignored the .mjs / .mts / .ts verify scripts the repo now ships (e.g. verify-ptcoag-multi.mts, verify-tea-criterion-format.mjs). Fixed the matcher to accept .js/.cjs/.mjs/.ts/.mts; re-run shows 5 of 5 covered, 0 debt. The convention is being followed. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 session, Michael ("are we building the competencies to have a coverage map, same as veritacheck?" then "build it").
+          <t>2026-09-24 session, "keep working" pass; audit tooling bug found + fixed.
 ---</t>
         </is>
       </c>
@@ -1394,12 +1358,12 @@
     <row r="5" ht="90" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>C41</t>
+          <t>C43</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>VeritaCheck coverage recurrence (method comparison + cal-ver/linearity + reports)</t>
+          <t>VeritaStaff instrument-centric (dual) assignment view</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr"/>
@@ -1407,12 +1371,12 @@
       <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: PRs #1317 (method comparison), #1318 (cal-ver/linearity), #1321 (report Next-due columns). Periodic verification (correlation/method comparison 42 CFR 493.1281; cal-ver/linearity 42 CFR 493.1255; both 6-month) now recurs: a signed study banks the cycle and rolls to next-due = signed + 6 months instead of reading "done" forever. Status Missing/Failed/Completed-unsigned + a "Next due on" column on-screen and in both coverage exports; also credits the previously-ignored "correlation" study type. Root cause: computeCoverageFrom marked requirements done on mere existence, no date logic. Verified live on SCAHC lab 2 (101 correlations + 11 cal-ver rows now carry a next-due). Engine-level, all facilities. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1320. GET/PUT /staff/instruments/:id/employees (transpose of the per-employee endpoints); an "Assign by Instrument" dialog lets a director pick a test system or manual test and check off who runs it. Same staff_employee_instruments join, with the 42 CFR 493.1235(a) duty-change event emitted on newly-added pairs so both orientations trigger the same reassessment. GET verified live on SCAHC lab 2. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>2026-09-24 session, Michael ("Look at San Carlos... they finished their last set of correlations (all 103) but their menu never reset").
+          <t>2026-09-24 session, Michael ("in staff we should also give the dual view when assigning coverage to test systems or manual tests").
 ---</t>
         </is>
       </c>
@@ -1421,12 +1385,12 @@
     <row r="6" ht="90" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>C40</t>
+          <t>C42</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>VeritaComp Competencies Owed derived from VeritaStaff, with gap detection (was #48)</t>
+          <t>VeritaComp coverage map (required-vs-assessed matrix, dual view)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr"/>
@@ -1434,12 +1398,12 @@
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1314 (squash 2bcb0db9). GET /api/labs/:labId/competency/owed derives each VeritaStaff testing employee's owed competencies from their assigned instruments (staff_employee_instruments -&gt; veritamap_instruments + tests), on the CLIA timeline, and flags instruments not covered by any competency program as gaps. CompetenciesOwedSection renders it on the VeritaComp landing page. Reuses the shipped bridge + suggested-method-groups match rules; no new tables. Verified live on prod with real assignment data: 2 instruments assigned to a demo staffer produced owed=2, gaps=2 (HIGH, Technical Supervisor), then reverted cleanly. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1319 (+ status layer PR #1316). /competency/owed returns per-item assessed (locked passing assessment this cycle on a covering method group) + per-employee CLIA status; CompetencyCoverageMap renders a By-employee / By-instrument matrix (Assessed / Owed / Overdue / Gap). Verified live on SCAHC lab 2 (owed 116, assessed 2, gaps 0). Completes #48 as the VeritaCheck-parity coverage map. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23/24 session, Michael ("veritacomp bases what competencies they owe (currently untrue, but needs to be true)"). Option 1 (unify roster on VeritaStaff, match instruments by id).
+          <t>2026-09-24 session, Michael ("are we building the competencies to have a coverage map, same as veritacheck?" then "build it").
 ---</t>
         </is>
       </c>
@@ -1448,12 +1412,12 @@
     <row r="7" ht="90" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>C39</t>
+          <t>C41</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>VeritaScan line items can attach or link evidence (was #46)</t>
+          <t>VeritaCheck coverage recurrence (method comparison + cal-ver/linearity + reports)</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr"/>
@@ -1461,12 +1425,12 @@
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1312 (squash a1dda93d). VeritaScan scan checklist items now show linked evidence as chips (open link, remove) plus a writer "Link evidence" affordance whose picker links an existing VeritaDC/Library document; a shortcut deep-links to the Library for new (governed) documents. Reuses the already-shipped lab_documents + document_checklist_links + coverage endpoints (URL-pointer only, no file storage, no new tables). Browser-verified live on prod (scan 23): the affordance renders and the picker opens. Closed 2026-09-24.</t>
+          <t>Closure evidence: PRs #1317 (method comparison), #1318 (cal-ver/linearity), #1321 (report Next-due columns). Periodic verification (correlation/method comparison 42 CFR 493.1281; cal-ver/linearity 42 CFR 493.1255; both 6-month) now recurs: a signed study banks the cycle and rolls to next-due = signed + 6 months instead of reading "done" forever. Status Missing/Failed/Completed-unsigned + a "Next due on" column on-screen and in both coverage exports; also credits the previously-ignored "correlation" study type. Root cause: computeCoverageFrom marked requirements done on mere existence, no date logic. Verified live on SCAHC lab 2 (101 correlations + 11 cal-ver rows now carry a next-due). Engine-level, all facilities. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>2026-09-23 session, Michael. Recurring request. Companion: cross-module evidence display on the VeritaDC policy shipped in PR #1313 (by-target cross-links surfaced in the policy View modal, browser-verified live).
+          <t>2026-09-24 session, Michael ("Look at San Carlos... they finished their last set of correlations (all 103) but their menu never reset").
 ---</t>
         </is>
       </c>
@@ -1475,12 +1439,12 @@
     <row r="8" ht="90" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>C38</t>
+          <t>C40</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>VeritaTrack calendar month cells expand to reveal hidden tasks (was #45)</t>
+          <t>VeritaComp Competencies Owed derived from VeritaStaff, with gap detection (was #48)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr"/>
@@ -1488,12 +1452,12 @@
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: VeritaTrack CalendarView month cells with more than three tasks now expand in place (chevron, "+N more" toggling to "Show less", due dates), so no task is hidden with no path to it (client/src/pages/VeritaTrackAppPage.tsx CalendarView). Shipped 2026-09-23. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1314 (squash 2bcb0db9). GET /api/labs/:labId/competency/owed derives each VeritaStaff testing employee's owed competencies from their assigned instruments (staff_employee_instruments -&gt; veritamap_instruments + tests), on the CLIA timeline, and flags instruments not covered by any competency program as gaps. CompetenciesOwedSection renders it on the VeritaComp landing page. Reuses the shipped bridge + suggested-method-groups match rules; no new tables. Verified live on prod with real assignment data: 2 instruments assigned to a demo staffer produced owed=2, gaps=2 (HIGH, Technical Supervisor), then reverted cleanly. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23 session, Michael screenshot of the VeritaTrack calendar (lab 3, September cell).
+          <t>2026-09-23/24 session, Michael ("veritacomp bases what competencies they owe (currently untrue, but needs to be true)"). Option 1 (unify roster on VeritaStaff, match instruments by id).
 ---</t>
         </is>
       </c>
@@ -1502,12 +1466,12 @@
     <row r="9" ht="90" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>C37</t>
+          <t>C39</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Long Excel column headers no longer clip CFR citations (was #44)</t>
+          <t>VeritaScan line items can attach or link evidence (was #46)</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr"/>
@@ -1515,12 +1479,12 @@
       <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. The VeritaMap export derives the header row height from the longest wrapped header via headerRowHeight(headers, colWidths) (server/routes.ts:15935) instead of a fixed 20, so "Reference Range Attestation (42 CFR 493.1253)" and the other long headers print in full. No new code this session. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1312 (squash a1dda93d). VeritaScan scan checklist items now show linked evidence as chips (open link, remove) plus a writer "Link evidence" affordance whose picker links an existing VeritaDC/Library document; a shortcut deep-links to the Library for new (governed) documents. Reuses the already-shipped lab_documents + document_checklist_links + coverage endpoints (URL-pointer only, no file storage, no new tables). Browser-verified live on prod (scan 23): the affordance renders and the picker opens. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+          <t>2026-09-23 session, Michael. Recurring request. Companion: cross-module evidence display on the VeritaDC policy shipped in PR #1313 (by-target cross-links surfaced in the policy View modal, browser-verified live).
 ---</t>
         </is>
       </c>
@@ -1529,12 +1493,12 @@
     <row r="10" ht="90" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>C36</t>
+          <t>C38</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>License stamp no longer clobbers the §6 header/footer or names the wrong lab (was #43)</t>
+          <t>VeritaTrack calendar month cells expand to reveal hidden tasks (was #45)</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr"/>
@@ -1542,12 +1506,12 @@
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. setHeaderFooter (shared/licenseExceljs.ts:155-209) now preserves an existing §6 header and appends (not overwrites) the footer left section, and customer-facing exports name the scoped lab: the VeritaScan library export reads req.scope.lab.name / clia_number (server/routes.ts:16572-16573), not the licensee. No new code this session (avoided regressing the existing fix). Closed 2026-09-24.</t>
+          <t>Closure evidence: VeritaTrack CalendarView month cells with more than three tasks now expand in place (chevron, "+N more" toggling to "Show less", due dates), so no task is hidden with no path to it (client/src/pages/VeritaTrackAppPage.tsx CalendarView). Shipped 2026-09-23. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+          <t>2026-09-23 session, Michael screenshot of the VeritaTrack calendar (lab 3, September cell).
 ---</t>
         </is>
       </c>
@@ -1556,18 +1520,72 @@
     <row r="11" ht="90" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>C34</t>
+          <t>C37</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Wire the two static-audit guards into CI (was #43)</t>
+          <t>Long Excel column headers no longer clip CFR citations (was #44)</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr"/>
       <c r="D11" s="3" t="inlineStr"/>
       <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. The VeritaMap export derives the header row height from the longest wrapped header via headerRowHeight(headers, colWidths) (server/routes.ts:15935) instead of a fixed 20, so "Reference Range Attestation (42 CFR 493.1253)" and the other long headers print in full. No new code this session. Closed 2026-09-24.</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+---</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12" ht="90" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>C36</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>License stamp no longer clobbers the §6 header/footer or names the wrong lab (was #43)</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr"/>
+      <c r="D12" s="2" t="inlineStr"/>
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. setHeaderFooter (shared/licenseExceljs.ts:155-209) now preserves an existing §6 header and appends (not overwrites) the footer left section, and customer-facing exports name the scoped lab: the VeritaScan library export reads req.scope.lab.name / clia_number (server/routes.ts:16572-16573), not the licensee. No new code this session (avoided regressing the existing fix). Closed 2026-09-24.</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+---</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13" ht="90" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>C34</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Wire the two static-audit guards into CI (was #43)</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr"/>
+      <c r="D13" s="3" t="inlineStr"/>
+      <c r="E13" s="3" t="inlineStr"/>
+      <c r="F13" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: both guards wired into the Multi-Lab Mutations Audit CI
 workflow (.github/workflows/multilab-mutations-audit.yml) as steps:
@@ -1579,24 +1597,24 @@
 (same caveat as the existing guards already in that workflow).</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr"/>
-      <c r="H11" s="3" t="inlineStr"/>
-    </row>
-    <row r="12" ht="90" customHeight="1">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="G13" s="3" t="inlineStr"/>
+      <c r="H13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14" ht="90" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>C35</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>Legacy /api/studies over-returns studies across labs (was #44)</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr"/>
-      <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="2" t="inlineStr"/>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr"/>
+      <c r="D14" s="2" t="inlineStr"/>
+      <c r="E14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: GET /api/studies now scopes its list to the active lab
 when one is resolved from the Referer (server/routes.ts), so every returned row
@@ -1606,24 +1624,24 @@
 mirroring the /api/labs/:labId/studies handler. Closed 2026-06-14.</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr"/>
-      <c r="H12" s="2" t="inlineStr"/>
-    </row>
-    <row r="13" ht="90" customHeight="1">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr"/>
+      <c r="H14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15" ht="90" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>C30</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>Verify-script convention backfill (was #41)</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr"/>
-      <c r="D13" s="3" t="inlineStr"/>
-      <c r="E13" s="3" t="inlineStr"/>
-      <c r="F13" s="3" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr"/>
+      <c r="D15" s="3" t="inlineStr"/>
+      <c r="E15" s="3" t="inlineStr"/>
+      <c r="F15" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: all 8 high-stakes math/logic commits now ship a paired
 scripts/verify-*.js (EP17 sensitivity, Deming lot-to-lot, CUMSUM+QC+multi-analyte,
@@ -1631,30 +1649,30 @@
 TEa boundary), per the strike-throughs in #41. Closed 2026-06-13.</t>
         </is>
       </c>
-      <c r="G13" s="3" t="inlineStr">
+      <c r="G15" s="3" t="inlineStr">
         <is>
           <t>scripts/audit_verify_script_coverage.py lookback, 2026-06-02; backfills
 landed 2026-06-03..06.
 ---</t>
         </is>
       </c>
-      <c r="H13" s="3" t="inlineStr"/>
-    </row>
-    <row r="14" ht="90" customHeight="1">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="H15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16" ht="90" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>C31</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>VeritaPT AAA create/update/delete silently no-op in the multi-lab UI</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr"/>
-      <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="2" t="inlineStr"/>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr"/>
+      <c r="D16" s="2" t="inlineStr"/>
+      <c r="E16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #754 (commit 92ad499) added lab-scoped POST/PUT/DELETE
 /api/labs/:labId/pt/aa-records. The UI posted to the lab-scoped path but only GET
@@ -1665,30 +1683,30 @@
 route mis-filed records to the user's default lab on multi-lab accounts).</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>2026-06-13, found during #18 Phase 3 QA;
 scripts/audit-labscoped-write-routes.mjs now guards the class.
 ---</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr"/>
-    </row>
-    <row r="15" ht="90" customHeight="1">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="H16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17" ht="90" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>C32</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>VeritaComp "Unlock assessment" false-success no-op</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr"/>
-      <c r="D15" s="3" t="inlineStr"/>
-      <c r="E15" s="3" t="inlineStr"/>
-      <c r="F15" s="3" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr"/>
+      <c r="D17" s="3" t="inlineStr"/>
+      <c r="E17" s="3" t="inlineStr"/>
+      <c r="F17" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #755 (commit 4234007) moved the unlock route to
 /api/labs/:labId/competency/assessments/:id/unlock (the path the client calls).
@@ -1699,29 +1717,29 @@
 HTML).</t>
         </is>
       </c>
-      <c r="G15" s="3" t="inlineStr">
+      <c r="G17" s="3" t="inlineStr">
         <is>
           <t>2026-06-13, found by scripts/audit-labscoped-write-routes.mjs.
 ---</t>
         </is>
       </c>
-      <c r="H15" s="3" t="inlineStr"/>
-    </row>
-    <row r="16" ht="90" customHeight="1">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="H17" s="3" t="inlineStr"/>
+    </row>
+    <row r="18" ht="90" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>C33</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>FK-cascade delete 500s + NavBar laptop-width overflow</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr"/>
-      <c r="D16" s="2" t="inlineStr"/>
-      <c r="E16" s="2" t="inlineStr"/>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr"/>
+      <c r="D18" s="2" t="inlineStr"/>
+      <c r="E18" s="2" t="inlineStr"/>
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PRs #749/#750 fixed NavBar horizontal overflow at laptop
 widths (collapse to the hamburger below 1560px); prod-verified at 1280-1920 with the
@@ -1732,57 +1750,57 @@
 500 -&gt; 200. scripts/audit-delete-cascades.mjs guards the class.</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>2026-06-13 browser QA of the A7-D4 wave + retro-QC of the 72h PR window.
 ---</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr"/>
-    </row>
-    <row r="17" ht="90" customHeight="1">
-      <c r="A17" s="3" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19" ht="90" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>C1</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>FAQ "over 25 years" -&gt; "over 23 years"</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr"/>
-      <c r="D17" s="3" t="inlineStr"/>
-      <c r="E17" s="3" t="inlineStr"/>
-      <c r="F17" s="3" t="inlineStr">
+      <c r="C19" s="3" t="inlineStr"/>
+      <c r="D19" s="3" t="inlineStr"/>
+      <c r="E19" s="3" t="inlineStr"/>
+      <c r="F19" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: client/src/pages/FAQPage.tsx line 20 reads "over
 23 years" as of 2026-05-01.</t>
         </is>
       </c>
-      <c r="G17" s="3" t="inlineStr">
+      <c r="G19" s="3" t="inlineStr">
         <is>
           <t>session 299e9a73 turn 14, ~2026-04-28.
 ---</t>
         </is>
       </c>
-      <c r="H17" s="3" t="inlineStr"/>
-    </row>
-    <row r="18" ht="90" customHeight="1">
-      <c r="A18" s="2" t="inlineStr">
+      <c r="H19" s="3" t="inlineStr"/>
+    </row>
+    <row r="20" ht="90" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>C5</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>David's VeritaQA grey-button bug (seat permissions mode)</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr"/>
-      <c r="D18" s="2" t="inlineStr"/>
-      <c r="E18" s="2" t="inlineStr"/>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr"/>
+      <c r="D20" s="2" t="inlineStr"/>
+      <c r="E20" s="2" t="inlineStr"/>
+      <c r="F20" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #10 squash-merged as commit a43fbba on
 2026-05-01 23:19 MST. Railway deploy succeeded; deployed bundle
@@ -1795,7 +1813,7 @@
 against his exact stored shape (14 of 14 expected outcomes matched).</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="G20" s="2" t="inlineStr">
         <is>
           <t>2026-05-01 David's report; veritabench + veritastock
 weren't in MODULE_LIST so seat permissions silently defaulted to
@@ -1803,75 +1821,17 @@
 ---</t>
         </is>
       </c>
-      <c r="H18" s="2" t="inlineStr"/>
-    </row>
-    <row r="19" ht="90" customHeight="1">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>C2</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>TeamPage present-tense "TJC surveyor" check</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr"/>
-      <c r="D19" s="3" t="inlineStr"/>
-      <c r="E19" s="3" t="inlineStr"/>
-      <c r="F19" s="3" t="inlineStr">
-        <is>
-          <t>Closure evidence: site-wide search confirmed all surveyor language
-is past-tense, consistent with user's 2021-2025 service. User closed
-the item in session 299e9a73 turn 4.</t>
-        </is>
-      </c>
-      <c r="G19" s="3" t="inlineStr">
-        <is>
-          <t>session 299e9a73, ~2026-04-28.
----</t>
-        </is>
-      </c>
-      <c r="H19" s="3" t="inlineStr"/>
-    </row>
-    <row r="20" ht="90" customHeight="1">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>C3</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>My Studies CSV/XLSX export (John as design partner)</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr"/>
-      <c r="D20" s="2" t="inlineStr"/>
-      <c r="E20" s="2" t="inlineStr"/>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>Closure evidence: client/src/pages/DashboardPage.tsx line 46 calls
-/api/my-studies/export. server/routes.ts line 1491 implements the
-endpoint. Pulled forward into pre-COLA per user instruction.</t>
-        </is>
-      </c>
-      <c r="G20" s="2" t="inlineStr">
-        <is>
-          <t>session 299e9a73 turn 5, ~2026-04-28.
----</t>
-        </is>
-      </c>
       <c r="H20" s="2" t="inlineStr"/>
     </row>
     <row r="21" ht="90" customHeight="1">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>C4</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Rotate GitHub PAT (because old PAT was committed in SESSION_HANDOFF files)</t>
+          <t>TeamPage present-tense "TJC surveyor" check</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr"/>
@@ -1879,8 +1839,9 @@
       <c r="E21" s="3" t="inlineStr"/>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: no ghp_* or github_pat_* patterns in current
-SESSION_HANDOFF.md or SESSION_HANDOFF-2.md as of 2026-05-01.</t>
+          <t>Closure evidence: site-wide search confirmed all surveyor language
+is past-tense, consistent with user's 2021-2025 service. User closed
+the item in session 299e9a73 turn 4.</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -1894,18 +1855,75 @@
     <row r="22" ht="90" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>C6</t>
+          <t>C3</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>VeritaPolicy service-line filtering removed (formerly #4)</t>
+          <t>My Studies CSV/XLSX export (John as design partner)</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr"/>
       <c r="D22" s="2" t="inlineStr"/>
       <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Closure evidence: client/src/pages/DashboardPage.tsx line 46 calls
+/api/my-studies/export. server/routes.ts line 1491 implements the
+endpoint. Pulled forward into pre-COLA per user instruction.</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>session 299e9a73 turn 5, ~2026-04-28.
+---</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23" ht="90" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Rotate GitHub PAT (because old PAT was committed in SESSION_HANDOFF files)</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr"/>
+      <c r="D23" s="3" t="inlineStr"/>
+      <c r="E23" s="3" t="inlineStr"/>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>Closure evidence: no ghp_* or github_pat_* patterns in current
+SESSION_HANDOFF.md or SESSION_HANDOFF-2.md as of 2026-05-01.</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>session 299e9a73, ~2026-04-28.
+---</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr"/>
+    </row>
+    <row r="24" ht="90" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>C6</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>VeritaPolicy service-line filtering removed (formerly #4)</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr"/>
+      <c r="D24" s="2" t="inlineStr"/>
+      <c r="E24" s="2" t="inlineStr"/>
+      <c r="F24" s="2" t="inlineStr">
         <is>
           <t>Closure rationale (operator decision 2026-05-10): Keep all
 VeritaPolicy rows. CFR-only references with no accreditor reference
@@ -1914,29 +1932,29 @@
 report misread the design intent.</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr">
+      <c r="G24" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H22" s="2" t="inlineStr"/>
-    </row>
-    <row r="23" ht="90" customHeight="1">
-      <c r="A23" s="3" t="inlineStr">
+      <c r="H24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25" ht="90" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
         <is>
           <t>C7</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>CLIA number format validation (formerly #13)</t>
         </is>
       </c>
-      <c r="C23" s="3" t="inlineStr"/>
-      <c r="D23" s="3" t="inlineStr"/>
-      <c r="E23" s="3" t="inlineStr"/>
-      <c r="F23" s="3" t="inlineStr">
+      <c r="C25" s="3" t="inlineStr"/>
+      <c r="D25" s="3" t="inlineStr"/>
+      <c r="E25" s="3" t="inlineStr"/>
+      <c r="F25" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: shared/validateClia.ts defines CLIA_REGEX =
 /^\d{2}D\d{7}$/ (line 24), validateClia() helper with whitespace
@@ -1947,30 +1965,30 @@
 shape exists and behaves as specified.</t>
         </is>
       </c>
-      <c r="G23" s="3" t="inlineStr">
+      <c r="G25" s="3" t="inlineStr">
         <is>
           <t>Agent verification 2026-05-10 via grep + file read.
 Operator confirmed shipped 2026-05-10.
 ---</t>
         </is>
       </c>
-      <c r="H23" s="3" t="inlineStr"/>
-    </row>
-    <row r="24" ht="90" customHeight="1">
-      <c r="A24" s="2" t="inlineStr">
+      <c r="H25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26" ht="90" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>C8</t>
         </is>
       </c>
-      <c r="B24" s="2" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t>VeritaMap lab-wide menu toggle (formerly #19)</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr"/>
-      <c r="D24" s="2" t="inlineStr"/>
-      <c r="E24" s="2" t="inlineStr"/>
-      <c r="F24" s="2" t="inlineStr">
+      <c r="C26" s="2" t="inlineStr"/>
+      <c r="D26" s="2" t="inlineStr"/>
+      <c r="E26" s="2" t="inlineStr"/>
+      <c r="F26" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: client/src/pages/VeritaMapLabwidePage.tsx
 exists and implements the labwide read-only union view. Route is
@@ -1980,59 +1998,59 @@
 parking lot plan (read-only union view, per-session toggle) shipped.</t>
         </is>
       </c>
-      <c r="G24" s="2" t="inlineStr">
+      <c r="G26" s="2" t="inlineStr">
         <is>
           <t>Agent verification 2026-05-10 via grep + file read.
 Operator confirmed shipped 2026-05-10.
 ---</t>
         </is>
       </c>
-      <c r="H24" s="2" t="inlineStr"/>
-    </row>
-    <row r="25" ht="90" customHeight="1">
-      <c r="A25" s="3" t="inlineStr">
+      <c r="H26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27" ht="90" customHeight="1">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>C9</t>
         </is>
       </c>
-      <c r="B25" s="3" t="inlineStr">
+      <c r="B27" s="3" t="inlineStr">
         <is>
           <t>Tier-1 smoke test checklist (formerly #6)</t>
         </is>
       </c>
-      <c r="C25" s="3" t="inlineStr"/>
-      <c r="D25" s="3" t="inlineStr"/>
-      <c r="E25" s="3" t="inlineStr"/>
-      <c r="F25" s="3" t="inlineStr">
+      <c r="C27" s="3" t="inlineStr"/>
+      <c r="D27" s="3" t="inlineStr"/>
+      <c r="E27" s="3" t="inlineStr"/>
+      <c r="F27" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: docs/smoke-test-tier1.md documents the Tier-1
 smoke-test process and post-deploy verification steps. Shipped via
 PR #81 as part of the 2026-05-10 wave.</t>
         </is>
       </c>
-      <c r="G25" s="3" t="inlineStr">
+      <c r="G27" s="3" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H25" s="3" t="inlineStr"/>
-    </row>
-    <row r="26" ht="90" customHeight="1">
-      <c r="A26" s="2" t="inlineStr">
+      <c r="H27" s="3" t="inlineStr"/>
+    </row>
+    <row r="28" ht="90" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>C10</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="B28" s="2" t="inlineStr">
         <is>
           <t>Per-module gating (formerly #7)</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr"/>
-      <c r="D26" s="2" t="inlineStr"/>
-      <c r="E26" s="2" t="inlineStr"/>
-      <c r="F26" s="2" t="inlineStr">
+      <c r="C28" s="2" t="inlineStr"/>
+      <c r="D28" s="2" t="inlineStr"/>
+      <c r="E28" s="2" t="inlineStr"/>
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: Client-side useIsReadOnly module keys wired
 on client/src/pages/VeritaPolicyAppPage.tsx and
@@ -2047,29 +2065,29 @@
 PR #76.</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr">
+      <c r="G28" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H26" s="2" t="inlineStr"/>
-    </row>
-    <row r="27" ht="90" customHeight="1">
-      <c r="A27" s="3" t="inlineStr">
+      <c r="H28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29" ht="90" customHeight="1">
+      <c r="A29" s="3" t="inlineStr">
         <is>
           <t>C11</t>
         </is>
       </c>
-      <c r="B27" s="3" t="inlineStr">
+      <c r="B29" s="3" t="inlineStr">
         <is>
           <t>VeritaStock shipped copy (formerly #8)</t>
         </is>
       </c>
-      <c r="C27" s="3" t="inlineStr"/>
-      <c r="D27" s="3" t="inlineStr"/>
-      <c r="E27" s="3" t="inlineStr"/>
-      <c r="F27" s="3" t="inlineStr">
+      <c r="C29" s="3" t="inlineStr"/>
+      <c r="D29" s="3" t="inlineStr"/>
+      <c r="E29" s="3" t="inlineStr"/>
+      <c r="F29" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: client/src/pages/ArticleInventoryManagementPage.tsx
 line 305 footer reads "platform that includes VeritaStock™" instead
@@ -2077,29 +2095,29 @@
 on /resources/laboratory-inventory-management. Shipped via PR #75.</t>
         </is>
       </c>
-      <c r="G27" s="3" t="inlineStr">
+      <c r="G29" s="3" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H27" s="3" t="inlineStr"/>
-    </row>
-    <row r="28" ht="90" customHeight="1">
-      <c r="A28" s="2" t="inlineStr">
+      <c r="H29" s="3" t="inlineStr"/>
+    </row>
+    <row r="30" ht="90" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>C12</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="B30" s="2" t="inlineStr">
         <is>
           <t>Admin report one-row-per-lab (formerly #14)</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr"/>
-      <c r="D28" s="2" t="inlineStr"/>
-      <c r="E28" s="2" t="inlineStr"/>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="C30" s="2" t="inlineStr"/>
+      <c r="D30" s="2" t="inlineStr"/>
+      <c r="E30" s="2" t="inlineStr"/>
+      <c r="F30" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: /api/admin/report rewritten in
 server/routes.ts (~line 595) to LEFT JOIN labs on
@@ -2114,56 +2132,56 @@
 prerequisite, not a code bug). Shipped via PR #85.</t>
         </is>
       </c>
-      <c r="G28" s="2" t="inlineStr">
+      <c r="G30" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H28" s="2" t="inlineStr"/>
-    </row>
-    <row r="29" ht="90" customHeight="1">
-      <c r="A29" s="3" t="inlineStr">
+      <c r="H30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31" ht="90" customHeight="1">
+      <c r="A31" s="3" t="inlineStr">
         <is>
           <t>C14</t>
         </is>
       </c>
-      <c r="B29" s="3" t="inlineStr">
+      <c r="B31" s="3" t="inlineStr">
         <is>
           <t>UI relabel "CLIA TEa" -&gt; "Lab-Set Internal Goal" (formerly #1)</t>
         </is>
       </c>
-      <c r="C29" s="3" t="inlineStr"/>
-      <c r="D29" s="3" t="inlineStr"/>
-      <c r="E29" s="3" t="inlineStr"/>
-      <c r="F29" s="3" t="inlineStr">
+      <c r="C31" s="3" t="inlineStr"/>
+      <c r="D31" s="3" t="inlineStr"/>
+      <c r="E31" s="3" t="inlineStr"/>
+      <c r="F31" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: Shipped across four PRs over 2026-05-10.</t>
         </is>
       </c>
-      <c r="G29" s="3" t="inlineStr">
+      <c r="G31" s="3" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H29" s="3" t="inlineStr"/>
-    </row>
-    <row r="30" ht="90" customHeight="1">
-      <c r="A30" s="2" t="inlineStr">
+      <c r="H31" s="3" t="inlineStr"/>
+    </row>
+    <row r="32" ht="90" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t>C13</t>
         </is>
       </c>
-      <c r="B30" s="2" t="inlineStr">
+      <c r="B32" s="2" t="inlineStr">
         <is>
           <t>WSLH PT vendor (formerly #15)</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr"/>
-      <c r="D30" s="2" t="inlineStr"/>
-      <c r="E30" s="2" t="inlineStr"/>
-      <c r="F30" s="2" t="inlineStr">
+      <c r="C32" s="2" t="inlineStr"/>
+      <c r="D32" s="2" t="inlineStr"/>
+      <c r="E32" s="2" t="inlineStr"/>
+      <c r="F32" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: Shipped 2026-05-10 via PR #79 (merge commit
 eeebc6e; merged after rebase to resolve a server/db.ts collision
@@ -2181,68 +2199,9 @@
 'WSLH' is the post-deploy success signal. Shipped via PR #79.</t>
         </is>
       </c>
-      <c r="G30" s="2" t="inlineStr">
+      <c r="G32" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
----</t>
-        </is>
-      </c>
-      <c r="H30" s="2" t="inlineStr"/>
-    </row>
-    <row r="31" ht="90" customHeight="1">
-      <c r="A31" s="3" t="inlineStr">
-        <is>
-          <t>C15</t>
-        </is>
-      </c>
-      <c r="B31" s="3" t="inlineStr">
-        <is>
-          <t>VeritaStock lot tracking + expiration + reorder alerts (formerly #21)</t>
-        </is>
-      </c>
-      <c r="C31" s="3" t="inlineStr"/>
-      <c r="D31" s="3" t="inlineStr"/>
-      <c r="E31" s="3" t="inlineStr"/>
-      <c r="F31" s="3" t="inlineStr">
-        <is>
-          <t>Closure evidence: VeritaStock™ shipped the bench-level inventory
-features the Perplexity competitor analysis identified as a gap:</t>
-        </is>
-      </c>
-      <c r="G31" s="3" t="inlineStr">
-        <is>
-          <t>Originally Perplexity competitor analysis 2026-05-10.
-Audit 2026-05-21 confirmed the feature set ships today.
----</t>
-        </is>
-      </c>
-      <c r="H31" s="3" t="inlineStr"/>
-    </row>
-    <row r="32" ht="90" customHeight="1">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>C16</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>PAL studies guided workflow (formerly #23)</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr"/>
-      <c r="D32" s="2" t="inlineStr"/>
-      <c r="E32" s="2" t="inlineStr"/>
-      <c r="F32" s="2" t="inlineStr">
-        <is>
-          <t>Closure evidence: VeritaCheck™ already ships the Precision /
-Accuracy / Linearity (PAL) study set under EP-protocol naming:</t>
-        </is>
-      </c>
-      <c r="G32" s="2" t="inlineStr">
-        <is>
-          <t>Originally Perplexity competitor analysis 2026-05-10.
-Audit 2026-05-21 confirmed the EP studies cover the PAL framing in
-full.
 ---</t>
         </is>
       </c>
@@ -2251,12 +2210,12 @@
     <row r="33" ht="90" customHeight="1">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>C17</t>
+          <t>C15</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>Source-grounded 21/29/45 CFR + 42 CFR 482-485 (formerly #26)</t>
+          <t>VeritaStock lot tracking + expiration + reorder alerts (formerly #21)</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr"/>
@@ -2264,35 +2223,94 @@
       <c r="E33" s="3" t="inlineStr"/>
       <c r="F33" s="3" t="inlineStr">
         <is>
+          <t>Closure evidence: VeritaStock™ shipped the bench-level inventory
+features the Perplexity competitor analysis identified as a gap:</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>Originally Perplexity competitor analysis 2026-05-10.
+Audit 2026-05-21 confirmed the feature set ships today.
+---</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr"/>
+    </row>
+    <row r="34" ht="90" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>C16</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>PAL studies guided workflow (formerly #23)</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr"/>
+      <c r="D34" s="2" t="inlineStr"/>
+      <c r="E34" s="2" t="inlineStr"/>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>Closure evidence: VeritaCheck™ already ships the Precision /
+Accuracy / Linearity (PAL) study set under EP-protocol naming:</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>Originally Perplexity competitor analysis 2026-05-10.
+Audit 2026-05-21 confirmed the EP studies cover the PAL framing in
+full.
+---</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr"/>
+    </row>
+    <row r="35" ht="90" customHeight="1">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>C17</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>Source-grounded 21/29/45 CFR + 42 CFR 482-485 (formerly #26)</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr"/>
+      <c r="D35" s="3" t="inlineStr"/>
+      <c r="E35" s="3" t="inlineStr"/>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
           <t>Closure evidence: PR #301 (commit 8c27806, merged 2026-05-21)
 source-grounded the 74 remaining non-493 entries in
 server/cfrRequirements.ts against verbatim eCFR XML. Breakdown
 shipped:</t>
         </is>
       </c>
-      <c r="G33" s="3" t="inlineStr">
+      <c r="G35" s="3" t="inlineStr">
         <is>
           <t>PR #301; tasks #18 in the in-session task tracker.
 ---</t>
         </is>
       </c>
-      <c r="H33" s="3" t="inlineStr"/>
-    </row>
-    <row r="34" ht="90" customHeight="1">
-      <c r="A34" s="2" t="inlineStr">
+      <c r="H35" s="3" t="inlineStr"/>
+    </row>
+    <row r="36" ht="90" customHeight="1">
+      <c r="A36" s="2" t="inlineStr">
         <is>
           <t>C18</t>
         </is>
       </c>
-      <c r="B34" s="2" t="inlineStr">
+      <c r="B36" s="2" t="inlineStr">
         <is>
           <t>VeritaPolicy "Non CLIA" chapter rename (formerly #3)</t>
         </is>
       </c>
-      <c r="C34" s="2" t="inlineStr"/>
-      <c r="D34" s="2" t="inlineStr"/>
-      <c r="E34" s="2" t="inlineStr"/>
-      <c r="F34" s="2" t="inlineStr">
+      <c r="C36" s="2" t="inlineStr"/>
+      <c r="D36" s="2" t="inlineStr"/>
+      <c r="E36" s="2" t="inlineStr"/>
+      <c r="F36" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #300 (commit 34d7707, merged 2026-05-21)
 renamed all 44 user-facing chapter labels in
@@ -2303,7 +2321,7 @@
 page.</t>
         </is>
       </c>
-      <c r="G34" s="2" t="inlineStr">
+      <c r="G36" s="2" t="inlineStr">
         <is>
           <t>CAP customer screenshot of the /veritapolicy chapter
 headers, 2026-05-01 evening. PR #300; tasks #17 in the in-session
@@ -2311,23 +2329,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H34" s="2" t="inlineStr"/>
-    </row>
-    <row r="35" ht="90" customHeight="1">
-      <c r="A35" s="3" t="inlineStr">
+      <c r="H36" s="2" t="inlineStr"/>
+    </row>
+    <row r="37" ht="90" customHeight="1">
+      <c r="A37" s="3" t="inlineStr">
         <is>
           <t>C19</t>
         </is>
       </c>
-      <c r="B35" s="3" t="inlineStr">
+      <c r="B37" s="3" t="inlineStr">
         <is>
           <t>VeritaStock department-scope toggle (formerly #31)</t>
         </is>
       </c>
-      <c r="C35" s="3" t="inlineStr"/>
-      <c r="D35" s="3" t="inlineStr"/>
-      <c r="E35" s="3" t="inlineStr"/>
-      <c r="F35" s="3" t="inlineStr">
+      <c r="C37" s="3" t="inlineStr"/>
+      <c r="D37" s="3" t="inlineStr"/>
+      <c r="E37" s="3" t="inlineStr"/>
+      <c r="F37" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #319 (commit d01f5fe, merged 2026-05-22)
 shipped the persistent dept-scope toggle on VeritaStockPage. A new
@@ -2338,7 +2356,7 @@
 workspace without re-filtering.</t>
         </is>
       </c>
-      <c r="G35" s="3" t="inlineStr">
+      <c r="G37" s="3" t="inlineStr">
         <is>
           <t>John, San Carlos lab, 2026-05-21. Same conversation that
 drove the vendor dropdown (PR #304), FILTERED VIEW banner (PR #305),
@@ -2346,23 +2364,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H35" s="3" t="inlineStr"/>
-    </row>
-    <row r="36" ht="90" customHeight="1">
-      <c r="A36" s="2" t="inlineStr">
+      <c r="H37" s="3" t="inlineStr"/>
+    </row>
+    <row r="38" ht="90" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
         <is>
           <t>C20</t>
         </is>
       </c>
-      <c r="B36" s="2" t="inlineStr">
+      <c r="B38" s="2" t="inlineStr">
         <is>
           <t>Primary-lab seat counting (formerly #12)</t>
         </is>
       </c>
-      <c r="C36" s="2" t="inlineStr"/>
-      <c r="D36" s="2" t="inlineStr"/>
-      <c r="E36" s="2" t="inlineStr"/>
-      <c r="F36" s="2" t="inlineStr">
+      <c r="C38" s="2" t="inlineStr"/>
+      <c r="D38" s="2" t="inlineStr"/>
+      <c r="E38" s="2" t="inlineStr"/>
+      <c r="F38" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: is_primary_lab INTEGER NOT NULL DEFAULT 0
 column was added to the lab_members table at db.ts:1276, with the
@@ -2373,7 +2391,7 @@
 is_primary_lab=1 ordering).</t>
         </is>
       </c>
-      <c r="G36" s="2" t="inlineStr">
+      <c r="G38" s="2" t="inlineStr">
         <is>
           <t>2026-05-07 multi-lab discussion. Build shipped as part
 of the Multi-Lab Tier 2 architecture work (Phase 3.x series, prior
@@ -2382,23 +2400,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H36" s="2" t="inlineStr"/>
-    </row>
-    <row r="37" ht="90" customHeight="1">
-      <c r="A37" s="3" t="inlineStr">
+      <c r="H38" s="2" t="inlineStr"/>
+    </row>
+    <row r="39" ht="90" customHeight="1">
+      <c r="A39" s="3" t="inlineStr">
         <is>
           <t>C21</t>
         </is>
       </c>
-      <c r="B37" s="3" t="inlineStr">
+      <c r="B39" s="3" t="inlineStr">
         <is>
           <t>Multi-lab pricing model — Option A (formerly #11)</t>
         </is>
       </c>
-      <c r="C37" s="3" t="inlineStr"/>
-      <c r="D37" s="3" t="inlineStr"/>
-      <c r="E37" s="3" t="inlineStr"/>
-      <c r="F37" s="3" t="inlineStr">
+      <c r="C39" s="3" t="inlineStr"/>
+      <c r="D39" s="3" t="inlineStr"/>
+      <c r="E39" s="3" t="inlineStr"/>
+      <c r="F39" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #322 (commit 0ccd925, merged 2026-05-22)
 added the customer-facing line to the pricing page that reflects
@@ -2411,7 +2429,7 @@
 Enterprise+ block, reads:</t>
         </is>
       </c>
-      <c r="G37" s="3" t="inlineStr">
+      <c r="G39" s="3" t="inlineStr">
         <is>
           <t>2026-05-07 multi-lab discussion (Lisa Veri's
 canonical-case session). PR #322 (initial build); softening PR
@@ -2420,30 +2438,30 @@
 ---</t>
         </is>
       </c>
-      <c r="H37" s="3" t="inlineStr"/>
-    </row>
-    <row r="38" ht="90" customHeight="1">
-      <c r="A38" s="2" t="inlineStr">
+      <c r="H39" s="3" t="inlineStr"/>
+    </row>
+    <row r="40" ht="90" customHeight="1">
+      <c r="A40" s="2" t="inlineStr">
         <is>
           <t>C22</t>
         </is>
       </c>
-      <c r="B38" s="2" t="inlineStr">
+      <c r="B40" s="2" t="inlineStr">
         <is>
           <t>VeritaOps cost-per-test module (formerly #10)</t>
         </is>
       </c>
-      <c r="C38" s="2" t="inlineStr"/>
-      <c r="D38" s="2" t="inlineStr"/>
-      <c r="E38" s="2" t="inlineStr"/>
-      <c r="F38" s="2" t="inlineStr">
+      <c r="C40" s="2" t="inlineStr"/>
+      <c r="D40" s="2" t="inlineStr"/>
+      <c r="E40" s="2" t="inlineStr"/>
+      <c r="F40" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: v1 of the VeritaOps Cost-Per-Reportable-Test
 (CPRT) module shipped across PR #325 through PR #330 on 2026-05-22.
 The module is feature-complete for the typical lab director workflow.</t>
         </is>
       </c>
-      <c r="G38" s="2" t="inlineStr">
+      <c r="G40" s="2" t="inlineStr">
         <is>
           <t>This thread, 2026-05-07 12:05 PM CDT, user message:
 "Parking lot: build an operations module for cost per test
@@ -2452,262 +2470,262 @@
 ---</t>
         </is>
       </c>
-      <c r="H38" s="2" t="inlineStr"/>
-    </row>
-    <row r="39" ht="90" customHeight="1">
-      <c r="A39" s="3" t="inlineStr">
+      <c r="H40" s="2" t="inlineStr"/>
+    </row>
+    <row r="41" ht="90" customHeight="1">
+      <c r="A41" s="3" t="inlineStr">
         <is>
           <t>C23</t>
         </is>
       </c>
-      <c r="B39" s="3" t="inlineStr">
+      <c r="B41" s="3" t="inlineStr">
         <is>
           <t>CCL lab name visual disambiguation in lab switcher (formerly #34)</t>
         </is>
       </c>
-      <c r="C39" s="3" t="inlineStr"/>
-      <c r="D39" s="3" t="inlineStr">
+      <c r="C41" s="3" t="inlineStr"/>
+      <c r="D41" s="3" t="inlineStr">
         <is>
           <t>XS (under 1 day, actual)</t>
         </is>
       </c>
-      <c r="E39" s="3" t="inlineStr">
+      <c r="E41" s="3" t="inlineStr">
         <is>
           <t>Low — cosmetic; only mattered when Lisa or Michael picked the wrong lab from...</t>
         </is>
       </c>
-      <c r="F39" s="3" t="inlineStr">
+      <c r="F41" s="3" t="inlineStr">
         <is>
           <t>Effort: XS (under 1 day, actual)
 Importance: Low — cosmetic; only mattered when Lisa or Michael picked the wrong lab from the dropdown.</t>
         </is>
       </c>
-      <c r="G39" s="3" t="inlineStr">
+      <c r="G41" s="3" t="inlineStr">
         <is>
           <t>flagged 2026-05-23 immediately after provisioning Lisa's CCL lab; closed 2026-05-24.
 ---</t>
         </is>
       </c>
-      <c r="H39" s="3" t="inlineStr"/>
-    </row>
-    <row r="40" ht="90" customHeight="1">
-      <c r="A40" s="2" t="inlineStr">
+      <c r="H41" s="3" t="inlineStr"/>
+    </row>
+    <row r="42" ht="90" customHeight="1">
+      <c r="A42" s="2" t="inlineStr">
         <is>
           <t>C24</t>
         </is>
       </c>
-      <c r="B40" s="2" t="inlineStr">
+      <c r="B42" s="2" t="inlineStr">
         <is>
           <t>VC Unlimited Y1/Y2 price disclosure UX (formerly #35)</t>
         </is>
       </c>
-      <c r="C40" s="2" t="inlineStr"/>
-      <c r="D40" s="2" t="inlineStr">
+      <c r="C42" s="2" t="inlineStr"/>
+      <c r="D42" s="2" t="inlineStr">
         <is>
           <t>XS (under 1 day, actual)</t>
         </is>
       </c>
-      <c r="E40" s="2" t="inlineStr">
+      <c r="E42" s="2" t="inlineStr">
         <is>
           <t>Low when shipped (proactive, no customer complaint yet) — but high if a procu...</t>
         </is>
       </c>
-      <c r="F40" s="2" t="inlineStr">
+      <c r="F42" s="2" t="inlineStr">
         <is>
           <t>Effort: XS (under 1 day, actual)
 Importance: Low when shipped (proactive, no customer complaint yet) — but high if a procurement reviewer later disputes the $499 renewal as undisclosed.</t>
         </is>
       </c>
-      <c r="G40" s="2" t="inlineStr">
+      <c r="G42" s="2" t="inlineStr">
         <is>
           <t>Pricing rebuild 2026-05-23; closed 2026-05-24 proactively before any customer dispute.
 ---</t>
         </is>
       </c>
-      <c r="H40" s="2" t="inlineStr"/>
-    </row>
-    <row r="41" ht="90" customHeight="1">
-      <c r="A41" s="3" t="inlineStr">
+      <c r="H42" s="2" t="inlineStr"/>
+    </row>
+    <row r="43" ht="90" customHeight="1">
+      <c r="A43" s="3" t="inlineStr">
         <is>
           <t>C25</t>
         </is>
       </c>
-      <c r="B41" s="3" t="inlineStr">
+      <c r="B43" s="3" t="inlineStr">
         <is>
           <t>VeritaQC Phase 1 (Levey-Jennings + Westgard live engine) (formerly #20)</t>
         </is>
       </c>
-      <c r="C41" s="3" t="inlineStr"/>
-      <c r="D41" s="3" t="inlineStr">
+      <c r="C43" s="3" t="inlineStr"/>
+      <c r="D43" s="3" t="inlineStr">
         <is>
           <t>L (about 5 days end-to-end, actual: Phase 0 schema → Phase 1A evaluator → 1B...</t>
         </is>
       </c>
-      <c r="E41" s="3" t="inlineStr">
+      <c r="E43" s="3" t="inlineStr">
         <is>
           <t>High — largest single gap vs myLabCompliance.io per Perplexity competitor ana...</t>
         </is>
       </c>
-      <c r="F41" s="3" t="inlineStr">
+      <c r="F43" s="3" t="inlineStr">
         <is>
           <t>Effort: L (about 5 days end-to-end, actual: Phase 0 schema → Phase 1A evaluator → 1B entry UI → 1C daily review → 1D monthly PDF + attestation)
 Importance: High — largest single gap vs myLabCompliance.io per Perplexity competitor analysis; promotes VeritaAssure from documentation tool to lab operations platform.</t>
         </is>
       </c>
-      <c r="G41" s="3" t="inlineStr">
+      <c r="G43" s="3" t="inlineStr">
         <is>
           <t>Perplexity competitor analysis 2026-05-10. Scoping confirmed via the build_phase1_mockup.py iterations 2026-05-24. Shipped 2026-05-25.
 ---</t>
         </is>
       </c>
-      <c r="H41" s="3" t="inlineStr"/>
-    </row>
-    <row r="42" ht="90" customHeight="1">
-      <c r="A42" s="2" t="inlineStr">
+      <c r="H43" s="3" t="inlineStr"/>
+    </row>
+    <row r="44" ht="90" customHeight="1">
+      <c r="A44" s="2" t="inlineStr">
         <is>
           <t>C26</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
+      <c r="B44" s="2" t="inlineStr">
         <is>
           <t>VeritaLab CMS-116 application support + state licensing registry (formerly #22)</t>
         </is>
       </c>
-      <c r="C42" s="2" t="inlineStr"/>
-      <c r="D42" s="2" t="inlineStr">
+      <c r="C44" s="2" t="inlineStr"/>
+      <c r="D44" s="2" t="inlineStr">
         <is>
           <t>M (1-2 weeks for v1, actual)</t>
         </is>
       </c>
-      <c r="E42" s="2" t="inlineStr">
+      <c r="E44" s="2" t="inlineStr">
         <is>
           <t>Medium — competitor parity (myLabCompliance.io) plus useful at lab startup an...</t>
         </is>
       </c>
-      <c r="F42" s="2" t="inlineStr">
+      <c r="F44" s="2" t="inlineStr">
         <is>
           <t>Effort: M (1-2 weeks for v1, actual)
 Importance: Medium — competitor parity (myLabCompliance.io) plus useful at lab startup and at certificate-type changes.</t>
         </is>
       </c>
-      <c r="G42" s="2" t="inlineStr">
+      <c r="G44" s="2" t="inlineStr">
         <is>
           <t>Perplexity competitor analysis (myLabCompliance.io), 2026-05-10. Reclassified as a VeritaLab extension 2026-05-25. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H42" s="2" t="inlineStr"/>
-    </row>
-    <row r="43" ht="90" customHeight="1">
-      <c r="A43" s="3" t="inlineStr">
+      <c r="H44" s="2" t="inlineStr"/>
+    </row>
+    <row r="45" ht="90" customHeight="1">
+      <c r="A45" s="3" t="inlineStr">
         <is>
           <t>C27</t>
         </is>
       </c>
-      <c r="B43" s="3" t="inlineStr">
+      <c r="B45" s="3" t="inlineStr">
         <is>
           <t>Active vs view-only seat split (formerly #33)</t>
         </is>
       </c>
-      <c r="C43" s="3" t="inlineStr"/>
-      <c r="D43" s="3" t="inlineStr">
+      <c r="C45" s="3" t="inlineStr"/>
+      <c r="D45" s="3" t="inlineStr">
         <is>
           <t>M (~1 week of engineering, actual: shipped in a single multi-PR session)</t>
         </is>
       </c>
-      <c r="E43" s="3" t="inlineStr">
+      <c r="E45" s="3" t="inlineStr">
         <is>
           <t>Medium — closed the gap between /pricing copy and product behavior; gives sal...</t>
         </is>
       </c>
-      <c r="F43" s="3" t="inlineStr">
+      <c r="F45" s="3" t="inlineStr">
         <is>
           <t>Effort: M (~1 week of engineering, actual: shipped in a single multi-PR session)
 Importance: Medium — closed the gap between /pricing copy and product behavior; gives sales a clean answer for "do you charge for our medical director?"</t>
         </is>
       </c>
-      <c r="G43" s="3" t="inlineStr">
+      <c r="G45" s="3" t="inlineStr">
         <is>
           <t>Pricing analysis doc Decision 3 (2026-05-21); MEDIUM scenario revised 2026-05-29 to retire the "unlimited view-only" claim. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H43" s="3" t="inlineStr"/>
-    </row>
-    <row r="44" ht="90" customHeight="1">
-      <c r="A44" s="2" t="inlineStr">
+      <c r="H45" s="3" t="inlineStr"/>
+    </row>
+    <row r="46" ht="90" customHeight="1">
+      <c r="A46" s="2" t="inlineStr">
         <is>
           <t>C28</t>
         </is>
       </c>
-      <c r="B44" s="2" t="inlineStr">
+      <c r="B46" s="2" t="inlineStr">
         <is>
           <t>"Why VeritaCheck" comparative one-pager (formerly #37)</t>
         </is>
       </c>
-      <c r="C44" s="2" t="inlineStr"/>
-      <c r="D44" s="2" t="inlineStr">
+      <c r="C46" s="2" t="inlineStr"/>
+      <c r="D46" s="2" t="inlineStr">
         <is>
           <t>S (one design pass + four claim paragraphs + PDF + matching marketing-site pa...</t>
         </is>
       </c>
-      <c r="E44" s="2" t="inlineStr">
+      <c r="E46" s="2" t="inlineStr">
         <is>
           <t>Medium — closed a positioning gap surfaced by six COLA conference attendees a...</t>
         </is>
       </c>
-      <c r="F44" s="2" t="inlineStr">
+      <c r="F46" s="2" t="inlineStr">
         <is>
           <t>Effort: S (one design pass + four claim paragraphs + PDF + matching marketing-site page, actual)
 Importance: Medium — closed a positioning gap surfaced by six COLA conference attendees attached to a legacy verification tool; converts product-quality advantage into a leave-behind Lisa can hand out.</t>
         </is>
       </c>
-      <c r="G44" s="2" t="inlineStr">
+      <c r="G46" s="2" t="inlineStr">
         <is>
           <t>2026-05-11 / 2026-05-12 conference notes review with Michael. Conference attendees (Whitehead, Odegard, Othman, Molinelli, Kyle, Allred) expressed interest in equivalent / superior product. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H44" s="2" t="inlineStr"/>
-    </row>
-    <row r="45" ht="90" customHeight="1">
-      <c r="A45" s="3" t="inlineStr">
+      <c r="H46" s="2" t="inlineStr"/>
+    </row>
+    <row r="47" ht="90" customHeight="1">
+      <c r="A47" s="3" t="inlineStr">
         <is>
           <t>C29</t>
         </is>
       </c>
-      <c r="B45" s="3" t="inlineStr">
+      <c r="B47" s="3" t="inlineStr">
         <is>
           <t>VeritaPolicy approval workflow — MediaLab functional mirror</t>
         </is>
       </c>
-      <c r="C45" s="3" t="inlineStr"/>
-      <c r="D45" s="3" t="inlineStr">
+      <c r="C47" s="3" t="inlineStr"/>
+      <c r="D47" s="3" t="inlineStr">
         <is>
           <t>XL (one focused session, 12 PRs landed)</t>
         </is>
       </c>
-      <c r="E45" s="3" t="inlineStr">
+      <c r="E47" s="3" t="inlineStr">
         <is>
           <t>High — replaces MediaLab Document Control ($752/$2,250 starting price, scalin...</t>
         </is>
       </c>
-      <c r="F45" s="3" t="inlineStr">
+      <c r="F47" s="3" t="inlineStr">
         <is>
           <t>Effort: XL (one focused session, 12 PRs landed)
 Importance: High — replaces MediaLab Document Control ($752/$2,250 starting price, scaling to $10K-$20K/yr at enterprise per Capterra public data) with an included VeritaPolicy feature; closes a real positioning gap and gives sales a direct comparator line.</t>
         </is>
       </c>
-      <c r="G45" s="3" t="inlineStr">
+      <c r="G47" s="3" t="inlineStr">
         <is>
           <t>Pricing strategy conversation 2026-05-29 (Michael: "I don't like bolt-ons; we should replicate this") → scoped 8 phases → shipped all 12 PRs in single session. Shipped 2026-05-29.
 ---</t>
         </is>
       </c>
-      <c r="H45" s="3" t="inlineStr"/>
+      <c r="H47" s="3" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H45"/>
+  <autoFilter ref="A1:H47"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
TASK: Parking-lot sync - close #49 (non-issue) + log verified-users email path (C46)
PLAN:
  1. Close #49 -> C45 (coverage math already single-source; competency cadence is a different CFR interval).
  2. Log verified-users email path -> C46 (PR #1324).
  3. Rebuild PARKING_LOT.xlsx.

Self-check:
  - #49 removed once; C45+C46 present; #50 stays open. OPEN 15 / CLOSED 46 / RETIRED 6.
  - Internal docs + script only; Gate 3 N/A.
</commit_message>
<xml_diff>
--- a/PARKING_LOT.xlsx
+++ b/PARKING_LOT.xlsx
@@ -12,8 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RETIRED" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$45</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$47</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RETIRED'!$A$1:$H$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1174,77 +1174,41 @@
     <row r="16" ht="90" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>50</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Unify the coverage/competency recurrence into one shared helper (tech debt)</t>
+          <t>Competency "assessed this cycle" uses a flat 365-day window</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr"/>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>S (a few hours) - extract "latest study/assessment -&gt; status / nextDueOn / ov...</t>
+          <t>S-M - anchor the coverage-map "assessed this cycle" to the person's actual CL...</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Low - the three paths duplicate the +6-month / signed-resets-to-missing logic...</t>
+          <t>Medium - in an employee's first year the semiannual windows differ from a fla...</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>Effort: S (a few hours) - extract "latest study/assessment -&gt; status / nextDueOn / overdue" into one helper used by method comparison, cal-ver/linearity, and the competency owed derivation.
-Importance: Low - the three paths duplicate the +6-month / signed-resets-to-missing logic. They agree today (verified), but a shared helper prevents future drift and settles the dateless-signed edge in one place. No user-facing impact; studies.date is NOT NULL so the one known divergence is unreachable in practice.</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-24 session, surfaced during the coverage-recurrence build. No live defect; hygiene.
----</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr"/>
-    </row>
-    <row r="17" ht="90" customHeight="1">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>Competency "assessed this cycle" uses a flat 365-day window</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="inlineStr"/>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>S-M - anchor the coverage-map "assessed this cycle" to the person's actual CL...</t>
-        </is>
-      </c>
-      <c r="E17" s="3" t="inlineStr">
-        <is>
-          <t>Medium - in an employee's first year the semiannual windows differ from a fla...</t>
-        </is>
-      </c>
-      <c r="F17" s="3" t="inlineStr">
         <is>
           <t>Effort: S-M - anchor the coverage-map "assessed this cycle" to the person's actual CLIA cadence (semiannual in year 1 per 42 CFR 493.1451(b)(8), annual thereafter) from staff_competency_schedules, instead of the v1 flat 365-day lookback.
 Importance: Medium - in an employee's first year the semiannual windows differ from a flat annual window, so a first-year assessment could read as current slightly longer or shorter than the true cadence. Fine for the common annual case; refine for year-1 accuracy.</t>
         </is>
       </c>
-      <c r="G17" s="3" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>2026-09-24 session, VeritaComp coverage map (#48 Phase 3) v1 simplification, noted in PR #1319.
 ---</t>
         </is>
       </c>
-      <c r="H17" s="3" t="inlineStr"/>
+      <c r="H16" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H17"/>
+  <autoFilter ref="A1:H16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1255,7 +1219,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H45"/>
+  <dimension ref="A1:H47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1313,12 +1277,12 @@
     <row r="2" ht="90" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>C44</t>
+          <t>C45</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Verify-script convention backfill (was #41) + audit matcher fix</t>
+          <t>Unify coverage/competency recurrence helper (was #49) - closed as non-issue</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr"/>
@@ -1326,12 +1290,12 @@
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: #41 was fully backfilled on 2026-06-13 (all 8 high-stakes scripts landed; see C30); it had only been mis-filed in OPEN. A 2026-09-24 re-audit initially reported 4 of 5 recent math/logic commits as missing a verify script, which was a FALSE POSITIVE: scripts/audit_verify_script_coverage.py matched only scripts/verify-*.js / .cjs, so it ignored the .mjs / .mts / .ts verify scripts the repo now ships (e.g. verify-ptcoag-multi.mts, verify-tea-criterion-format.mjs). Fixed the matcher to accept .js/.cjs/.mjs/.ts/.mts; re-run shows 5 of 5 covered, 0 debt. The convention is being followed. Closed 2026-09-24.</t>
+          <t>Closure evidence: Investigated 2026-09-24 before building. The coverage recurrence math (+6-month interval, signed-resets-to-missing, nextDueOn/overdue, isFailVerdict) is ALREADY single-source in server/veritacheckCoverage.ts (computeCoverageFrom). server/coverageReport.ts and the routes.ts coverage export do not recompute it; they consume the computed nextDueOn/overdue/status fields and apply small surface-specific presentation labels (deliberately different vocabularies per surface, so they should not be merged). The only truly identical duplicate is a one-line date formatter. The competency "owed" derivation is NOT the same cadence: competency follows the CLIA milestone schedule (initial / semiannual year 1 / annual, 42 CFR 493.1451(b)(8) and 493.1235), which is a different regulatory interval from the coverage 6-month rule (493.1281 / 493.1255) and must stay separate. No worthwhile extraction; merging the two cadences would be wrong. Closed 2026-09-24. (The year-1 competency-window refinement remains tracked separately as #50.)</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 session, "keep working" pass; audit tooling bug found + fixed.
+          <t>2026-09-24 session, "keep working" pass; scoped read-only, found no real duplication.
 ---</t>
         </is>
       </c>
@@ -1340,12 +1304,12 @@
     <row r="3" ht="90" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>C43</t>
+          <t>C46</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>VeritaStaff instrument-centric (dual) assignment view</t>
+          <t>Verified-users product-update send path (wrong-list incident fix)</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr"/>
@@ -1353,12 +1317,12 @@
       <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1320. GET/PUT /staff/instruments/:id/employees (transpose of the per-employee endpoints); an "Assign by Instrument" dialog lets a director pick a test system or manual test and check off who runs it. Same staff_employee_instruments join, with the 42 CFR 493.1235(a) duty-change event emitted on newly-added pairs so both orientations trigger the same reassessment. GET verified live on SCAHC lab 2. Closed 2026-09-24.</t>
+          <t>Closure evidence: Shipped PR #1324 (merged 4e05506a, deploy ACTIVE). New POST /api/admin/users/send targets registered VeritaAssure account holders (the users table), never the Lab Director's Briefing subscriber list. Separate explicitly-named endpoint (not a flag with a dangerous default), account-holder email framing, excludes suppressed emails and RFC-reserved test domains, CC owner, dryRun + testTo previews. Public unsubscribe now upserts a suppression row so opt-outs are honored across both audiences. Live dryRun: 49 verified-user recipients vs 673 on the Briefing list. Receipts: scripts/verify-product-update-send.mts 24/24, tsc clean, rendered sample inspected. Fixes the fallout from the 2026-09-23/24 wrong-list send (a product update went to the 675-person Briefing list). Nothing sends without Michael's explicit "send it."</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>2026-09-24 session, Michael ("in staff we should also give the dual view when assigning coverage to test systems or manual tests").
+          <t>2026-09-24 session; Michael selected this as the next build after the #41 close.
 ---</t>
         </is>
       </c>
@@ -1367,12 +1331,12 @@
     <row r="4" ht="90" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>C42</t>
+          <t>C44</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>VeritaComp coverage map (required-vs-assessed matrix, dual view)</t>
+          <t>Verify-script convention backfill (was #41) + audit matcher fix</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr"/>
@@ -1380,12 +1344,12 @@
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1319 (+ status layer PR #1316). /competency/owed returns per-item assessed (locked passing assessment this cycle on a covering method group) + per-employee CLIA status; CompetencyCoverageMap renders a By-employee / By-instrument matrix (Assessed / Owed / Overdue / Gap). Verified live on SCAHC lab 2 (owed 116, assessed 2, gaps 0). Completes #48 as the VeritaCheck-parity coverage map. Closed 2026-09-24.</t>
+          <t>Closure evidence: #41 was fully backfilled on 2026-06-13 (all 8 high-stakes scripts landed; see C30); it had only been mis-filed in OPEN. A 2026-09-24 re-audit initially reported 4 of 5 recent math/logic commits as missing a verify script, which was a FALSE POSITIVE: scripts/audit_verify_script_coverage.py matched only scripts/verify-*.js / .cjs, so it ignored the .mjs / .mts / .ts verify scripts the repo now ships (e.g. verify-ptcoag-multi.mts, verify-tea-criterion-format.mjs). Fixed the matcher to accept .js/.cjs/.mjs/.ts/.mts; re-run shows 5 of 5 covered, 0 debt. The convention is being followed. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 session, Michael ("are we building the competencies to have a coverage map, same as veritacheck?" then "build it").
+          <t>2026-09-24 session, "keep working" pass; audit tooling bug found + fixed.
 ---</t>
         </is>
       </c>
@@ -1394,12 +1358,12 @@
     <row r="5" ht="90" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>C41</t>
+          <t>C43</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>VeritaCheck coverage recurrence (method comparison + cal-ver/linearity + reports)</t>
+          <t>VeritaStaff instrument-centric (dual) assignment view</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr"/>
@@ -1407,12 +1371,12 @@
       <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: PRs #1317 (method comparison), #1318 (cal-ver/linearity), #1321 (report Next-due columns). Periodic verification (correlation/method comparison 42 CFR 493.1281; cal-ver/linearity 42 CFR 493.1255; both 6-month) now recurs: a signed study banks the cycle and rolls to next-due = signed + 6 months instead of reading "done" forever. Status Missing/Failed/Completed-unsigned + a "Next due on" column on-screen and in both coverage exports; also credits the previously-ignored "correlation" study type. Root cause: computeCoverageFrom marked requirements done on mere existence, no date logic. Verified live on SCAHC lab 2 (101 correlations + 11 cal-ver rows now carry a next-due). Engine-level, all facilities. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1320. GET/PUT /staff/instruments/:id/employees (transpose of the per-employee endpoints); an "Assign by Instrument" dialog lets a director pick a test system or manual test and check off who runs it. Same staff_employee_instruments join, with the 42 CFR 493.1235(a) duty-change event emitted on newly-added pairs so both orientations trigger the same reassessment. GET verified live on SCAHC lab 2. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>2026-09-24 session, Michael ("Look at San Carlos... they finished their last set of correlations (all 103) but their menu never reset").
+          <t>2026-09-24 session, Michael ("in staff we should also give the dual view when assigning coverage to test systems or manual tests").
 ---</t>
         </is>
       </c>
@@ -1421,12 +1385,12 @@
     <row r="6" ht="90" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>C40</t>
+          <t>C42</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>VeritaComp Competencies Owed derived from VeritaStaff, with gap detection (was #48)</t>
+          <t>VeritaComp coverage map (required-vs-assessed matrix, dual view)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr"/>
@@ -1434,12 +1398,12 @@
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1314 (squash 2bcb0db9). GET /api/labs/:labId/competency/owed derives each VeritaStaff testing employee's owed competencies from their assigned instruments (staff_employee_instruments -&gt; veritamap_instruments + tests), on the CLIA timeline, and flags instruments not covered by any competency program as gaps. CompetenciesOwedSection renders it on the VeritaComp landing page. Reuses the shipped bridge + suggested-method-groups match rules; no new tables. Verified live on prod with real assignment data: 2 instruments assigned to a demo staffer produced owed=2, gaps=2 (HIGH, Technical Supervisor), then reverted cleanly. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1319 (+ status layer PR #1316). /competency/owed returns per-item assessed (locked passing assessment this cycle on a covering method group) + per-employee CLIA status; CompetencyCoverageMap renders a By-employee / By-instrument matrix (Assessed / Owed / Overdue / Gap). Verified live on SCAHC lab 2 (owed 116, assessed 2, gaps 0). Completes #48 as the VeritaCheck-parity coverage map. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23/24 session, Michael ("veritacomp bases what competencies they owe (currently untrue, but needs to be true)"). Option 1 (unify roster on VeritaStaff, match instruments by id).
+          <t>2026-09-24 session, Michael ("are we building the competencies to have a coverage map, same as veritacheck?" then "build it").
 ---</t>
         </is>
       </c>
@@ -1448,12 +1412,12 @@
     <row r="7" ht="90" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>C39</t>
+          <t>C41</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>VeritaScan line items can attach or link evidence (was #46)</t>
+          <t>VeritaCheck coverage recurrence (method comparison + cal-ver/linearity + reports)</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr"/>
@@ -1461,12 +1425,12 @@
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1312 (squash a1dda93d). VeritaScan scan checklist items now show linked evidence as chips (open link, remove) plus a writer "Link evidence" affordance whose picker links an existing VeritaDC/Library document; a shortcut deep-links to the Library for new (governed) documents. Reuses the already-shipped lab_documents + document_checklist_links + coverage endpoints (URL-pointer only, no file storage, no new tables). Browser-verified live on prod (scan 23): the affordance renders and the picker opens. Closed 2026-09-24.</t>
+          <t>Closure evidence: PRs #1317 (method comparison), #1318 (cal-ver/linearity), #1321 (report Next-due columns). Periodic verification (correlation/method comparison 42 CFR 493.1281; cal-ver/linearity 42 CFR 493.1255; both 6-month) now recurs: a signed study banks the cycle and rolls to next-due = signed + 6 months instead of reading "done" forever. Status Missing/Failed/Completed-unsigned + a "Next due on" column on-screen and in both coverage exports; also credits the previously-ignored "correlation" study type. Root cause: computeCoverageFrom marked requirements done on mere existence, no date logic. Verified live on SCAHC lab 2 (101 correlations + 11 cal-ver rows now carry a next-due). Engine-level, all facilities. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>2026-09-23 session, Michael. Recurring request. Companion: cross-module evidence display on the VeritaDC policy shipped in PR #1313 (by-target cross-links surfaced in the policy View modal, browser-verified live).
+          <t>2026-09-24 session, Michael ("Look at San Carlos... they finished their last set of correlations (all 103) but their menu never reset").
 ---</t>
         </is>
       </c>
@@ -1475,12 +1439,12 @@
     <row r="8" ht="90" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>C38</t>
+          <t>C40</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>VeritaTrack calendar month cells expand to reveal hidden tasks (was #45)</t>
+          <t>VeritaComp Competencies Owed derived from VeritaStaff, with gap detection (was #48)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr"/>
@@ -1488,12 +1452,12 @@
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: VeritaTrack CalendarView month cells with more than three tasks now expand in place (chevron, "+N more" toggling to "Show less", due dates), so no task is hidden with no path to it (client/src/pages/VeritaTrackAppPage.tsx CalendarView). Shipped 2026-09-23. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1314 (squash 2bcb0db9). GET /api/labs/:labId/competency/owed derives each VeritaStaff testing employee's owed competencies from their assigned instruments (staff_employee_instruments -&gt; veritamap_instruments + tests), on the CLIA timeline, and flags instruments not covered by any competency program as gaps. CompetenciesOwedSection renders it on the VeritaComp landing page. Reuses the shipped bridge + suggested-method-groups match rules; no new tables. Verified live on prod with real assignment data: 2 instruments assigned to a demo staffer produced owed=2, gaps=2 (HIGH, Technical Supervisor), then reverted cleanly. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23 session, Michael screenshot of the VeritaTrack calendar (lab 3, September cell).
+          <t>2026-09-23/24 session, Michael ("veritacomp bases what competencies they owe (currently untrue, but needs to be true)"). Option 1 (unify roster on VeritaStaff, match instruments by id).
 ---</t>
         </is>
       </c>
@@ -1502,12 +1466,12 @@
     <row r="9" ht="90" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>C37</t>
+          <t>C39</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Long Excel column headers no longer clip CFR citations (was #44)</t>
+          <t>VeritaScan line items can attach or link evidence (was #46)</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr"/>
@@ -1515,12 +1479,12 @@
       <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. The VeritaMap export derives the header row height from the longest wrapped header via headerRowHeight(headers, colWidths) (server/routes.ts:15935) instead of a fixed 20, so "Reference Range Attestation (42 CFR 493.1253)" and the other long headers print in full. No new code this session. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1312 (squash a1dda93d). VeritaScan scan checklist items now show linked evidence as chips (open link, remove) plus a writer "Link evidence" affordance whose picker links an existing VeritaDC/Library document; a shortcut deep-links to the Library for new (governed) documents. Reuses the already-shipped lab_documents + document_checklist_links + coverage endpoints (URL-pointer only, no file storage, no new tables). Browser-verified live on prod (scan 23): the affordance renders and the picker opens. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+          <t>2026-09-23 session, Michael. Recurring request. Companion: cross-module evidence display on the VeritaDC policy shipped in PR #1313 (by-target cross-links surfaced in the policy View modal, browser-verified live).
 ---</t>
         </is>
       </c>
@@ -1529,12 +1493,12 @@
     <row r="10" ht="90" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>C36</t>
+          <t>C38</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>License stamp no longer clobbers the §6 header/footer or names the wrong lab (was #43)</t>
+          <t>VeritaTrack calendar month cells expand to reveal hidden tasks (was #45)</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr"/>
@@ -1542,12 +1506,12 @@
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. setHeaderFooter (shared/licenseExceljs.ts:155-209) now preserves an existing §6 header and appends (not overwrites) the footer left section, and customer-facing exports name the scoped lab: the VeritaScan library export reads req.scope.lab.name / clia_number (server/routes.ts:16572-16573), not the licensee. No new code this session (avoided regressing the existing fix). Closed 2026-09-24.</t>
+          <t>Closure evidence: VeritaTrack CalendarView month cells with more than three tasks now expand in place (chevron, "+N more" toggling to "Show less", due dates), so no task is hidden with no path to it (client/src/pages/VeritaTrackAppPage.tsx CalendarView). Shipped 2026-09-23. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+          <t>2026-09-23 session, Michael screenshot of the VeritaTrack calendar (lab 3, September cell).
 ---</t>
         </is>
       </c>
@@ -1556,18 +1520,72 @@
     <row r="11" ht="90" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>C34</t>
+          <t>C37</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Wire the two static-audit guards into CI (was #43)</t>
+          <t>Long Excel column headers no longer clip CFR citations (was #44)</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr"/>
       <c r="D11" s="3" t="inlineStr"/>
       <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. The VeritaMap export derives the header row height from the longest wrapped header via headerRowHeight(headers, colWidths) (server/routes.ts:15935) instead of a fixed 20, so "Reference Range Attestation (42 CFR 493.1253)" and the other long headers print in full. No new code this session. Closed 2026-09-24.</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+---</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12" ht="90" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>C36</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>License stamp no longer clobbers the §6 header/footer or names the wrong lab (was #43)</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr"/>
+      <c r="D12" s="2" t="inlineStr"/>
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. setHeaderFooter (shared/licenseExceljs.ts:155-209) now preserves an existing §6 header and appends (not overwrites) the footer left section, and customer-facing exports name the scoped lab: the VeritaScan library export reads req.scope.lab.name / clia_number (server/routes.ts:16572-16573), not the licensee. No new code this session (avoided regressing the existing fix). Closed 2026-09-24.</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+---</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13" ht="90" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>C34</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Wire the two static-audit guards into CI (was #43)</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr"/>
+      <c r="D13" s="3" t="inlineStr"/>
+      <c r="E13" s="3" t="inlineStr"/>
+      <c r="F13" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: both guards wired into the Multi-Lab Mutations Audit CI
 workflow (.github/workflows/multilab-mutations-audit.yml) as steps:
@@ -1579,24 +1597,24 @@
 (same caveat as the existing guards already in that workflow).</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr"/>
-      <c r="H11" s="3" t="inlineStr"/>
-    </row>
-    <row r="12" ht="90" customHeight="1">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="G13" s="3" t="inlineStr"/>
+      <c r="H13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14" ht="90" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>C35</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>Legacy /api/studies over-returns studies across labs (was #44)</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr"/>
-      <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="2" t="inlineStr"/>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr"/>
+      <c r="D14" s="2" t="inlineStr"/>
+      <c r="E14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: GET /api/studies now scopes its list to the active lab
 when one is resolved from the Referer (server/routes.ts), so every returned row
@@ -1606,24 +1624,24 @@
 mirroring the /api/labs/:labId/studies handler. Closed 2026-06-14.</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr"/>
-      <c r="H12" s="2" t="inlineStr"/>
-    </row>
-    <row r="13" ht="90" customHeight="1">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr"/>
+      <c r="H14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15" ht="90" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>C30</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>Verify-script convention backfill (was #41)</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr"/>
-      <c r="D13" s="3" t="inlineStr"/>
-      <c r="E13" s="3" t="inlineStr"/>
-      <c r="F13" s="3" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr"/>
+      <c r="D15" s="3" t="inlineStr"/>
+      <c r="E15" s="3" t="inlineStr"/>
+      <c r="F15" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: all 8 high-stakes math/logic commits now ship a paired
 scripts/verify-*.js (EP17 sensitivity, Deming lot-to-lot, CUMSUM+QC+multi-analyte,
@@ -1631,30 +1649,30 @@
 TEa boundary), per the strike-throughs in #41. Closed 2026-06-13.</t>
         </is>
       </c>
-      <c r="G13" s="3" t="inlineStr">
+      <c r="G15" s="3" t="inlineStr">
         <is>
           <t>scripts/audit_verify_script_coverage.py lookback, 2026-06-02; backfills
 landed 2026-06-03..06.
 ---</t>
         </is>
       </c>
-      <c r="H13" s="3" t="inlineStr"/>
-    </row>
-    <row r="14" ht="90" customHeight="1">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="H15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16" ht="90" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>C31</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>VeritaPT AAA create/update/delete silently no-op in the multi-lab UI</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr"/>
-      <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="2" t="inlineStr"/>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr"/>
+      <c r="D16" s="2" t="inlineStr"/>
+      <c r="E16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #754 (commit 92ad499) added lab-scoped POST/PUT/DELETE
 /api/labs/:labId/pt/aa-records. The UI posted to the lab-scoped path but only GET
@@ -1665,30 +1683,30 @@
 route mis-filed records to the user's default lab on multi-lab accounts).</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>2026-06-13, found during #18 Phase 3 QA;
 scripts/audit-labscoped-write-routes.mjs now guards the class.
 ---</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr"/>
-    </row>
-    <row r="15" ht="90" customHeight="1">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="H16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17" ht="90" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>C32</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>VeritaComp "Unlock assessment" false-success no-op</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr"/>
-      <c r="D15" s="3" t="inlineStr"/>
-      <c r="E15" s="3" t="inlineStr"/>
-      <c r="F15" s="3" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr"/>
+      <c r="D17" s="3" t="inlineStr"/>
+      <c r="E17" s="3" t="inlineStr"/>
+      <c r="F17" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #755 (commit 4234007) moved the unlock route to
 /api/labs/:labId/competency/assessments/:id/unlock (the path the client calls).
@@ -1699,29 +1717,29 @@
 HTML).</t>
         </is>
       </c>
-      <c r="G15" s="3" t="inlineStr">
+      <c r="G17" s="3" t="inlineStr">
         <is>
           <t>2026-06-13, found by scripts/audit-labscoped-write-routes.mjs.
 ---</t>
         </is>
       </c>
-      <c r="H15" s="3" t="inlineStr"/>
-    </row>
-    <row r="16" ht="90" customHeight="1">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="H17" s="3" t="inlineStr"/>
+    </row>
+    <row r="18" ht="90" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>C33</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>FK-cascade delete 500s + NavBar laptop-width overflow</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr"/>
-      <c r="D16" s="2" t="inlineStr"/>
-      <c r="E16" s="2" t="inlineStr"/>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr"/>
+      <c r="D18" s="2" t="inlineStr"/>
+      <c r="E18" s="2" t="inlineStr"/>
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PRs #749/#750 fixed NavBar horizontal overflow at laptop
 widths (collapse to the hamburger below 1560px); prod-verified at 1280-1920 with the
@@ -1732,57 +1750,57 @@
 500 -&gt; 200. scripts/audit-delete-cascades.mjs guards the class.</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>2026-06-13 browser QA of the A7-D4 wave + retro-QC of the 72h PR window.
 ---</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr"/>
-    </row>
-    <row r="17" ht="90" customHeight="1">
-      <c r="A17" s="3" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19" ht="90" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>C1</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>FAQ "over 25 years" -&gt; "over 23 years"</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr"/>
-      <c r="D17" s="3" t="inlineStr"/>
-      <c r="E17" s="3" t="inlineStr"/>
-      <c r="F17" s="3" t="inlineStr">
+      <c r="C19" s="3" t="inlineStr"/>
+      <c r="D19" s="3" t="inlineStr"/>
+      <c r="E19" s="3" t="inlineStr"/>
+      <c r="F19" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: client/src/pages/FAQPage.tsx line 20 reads "over
 23 years" as of 2026-05-01.</t>
         </is>
       </c>
-      <c r="G17" s="3" t="inlineStr">
+      <c r="G19" s="3" t="inlineStr">
         <is>
           <t>session 299e9a73 turn 14, ~2026-04-28.
 ---</t>
         </is>
       </c>
-      <c r="H17" s="3" t="inlineStr"/>
-    </row>
-    <row r="18" ht="90" customHeight="1">
-      <c r="A18" s="2" t="inlineStr">
+      <c r="H19" s="3" t="inlineStr"/>
+    </row>
+    <row r="20" ht="90" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>C5</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>David's VeritaQA grey-button bug (seat permissions mode)</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr"/>
-      <c r="D18" s="2" t="inlineStr"/>
-      <c r="E18" s="2" t="inlineStr"/>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr"/>
+      <c r="D20" s="2" t="inlineStr"/>
+      <c r="E20" s="2" t="inlineStr"/>
+      <c r="F20" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #10 squash-merged as commit a43fbba on
 2026-05-01 23:19 MST. Railway deploy succeeded; deployed bundle
@@ -1795,7 +1813,7 @@
 against his exact stored shape (14 of 14 expected outcomes matched).</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="G20" s="2" t="inlineStr">
         <is>
           <t>2026-05-01 David's report; veritabench + veritastock
 weren't in MODULE_LIST so seat permissions silently defaulted to
@@ -1803,75 +1821,17 @@
 ---</t>
         </is>
       </c>
-      <c r="H18" s="2" t="inlineStr"/>
-    </row>
-    <row r="19" ht="90" customHeight="1">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>C2</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>TeamPage present-tense "TJC surveyor" check</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr"/>
-      <c r="D19" s="3" t="inlineStr"/>
-      <c r="E19" s="3" t="inlineStr"/>
-      <c r="F19" s="3" t="inlineStr">
-        <is>
-          <t>Closure evidence: site-wide search confirmed all surveyor language
-is past-tense, consistent with user's 2021-2025 service. User closed
-the item in session 299e9a73 turn 4.</t>
-        </is>
-      </c>
-      <c r="G19" s="3" t="inlineStr">
-        <is>
-          <t>session 299e9a73, ~2026-04-28.
----</t>
-        </is>
-      </c>
-      <c r="H19" s="3" t="inlineStr"/>
-    </row>
-    <row r="20" ht="90" customHeight="1">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>C3</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>My Studies CSV/XLSX export (John as design partner)</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr"/>
-      <c r="D20" s="2" t="inlineStr"/>
-      <c r="E20" s="2" t="inlineStr"/>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>Closure evidence: client/src/pages/DashboardPage.tsx line 46 calls
-/api/my-studies/export. server/routes.ts line 1491 implements the
-endpoint. Pulled forward into pre-COLA per user instruction.</t>
-        </is>
-      </c>
-      <c r="G20" s="2" t="inlineStr">
-        <is>
-          <t>session 299e9a73 turn 5, ~2026-04-28.
----</t>
-        </is>
-      </c>
       <c r="H20" s="2" t="inlineStr"/>
     </row>
     <row r="21" ht="90" customHeight="1">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>C4</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Rotate GitHub PAT (because old PAT was committed in SESSION_HANDOFF files)</t>
+          <t>TeamPage present-tense "TJC surveyor" check</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr"/>
@@ -1879,8 +1839,9 @@
       <c r="E21" s="3" t="inlineStr"/>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: no ghp_* or github_pat_* patterns in current
-SESSION_HANDOFF.md or SESSION_HANDOFF-2.md as of 2026-05-01.</t>
+          <t>Closure evidence: site-wide search confirmed all surveyor language
+is past-tense, consistent with user's 2021-2025 service. User closed
+the item in session 299e9a73 turn 4.</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -1894,18 +1855,75 @@
     <row r="22" ht="90" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>C6</t>
+          <t>C3</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>VeritaPolicy service-line filtering removed (formerly #4)</t>
+          <t>My Studies CSV/XLSX export (John as design partner)</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr"/>
       <c r="D22" s="2" t="inlineStr"/>
       <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Closure evidence: client/src/pages/DashboardPage.tsx line 46 calls
+/api/my-studies/export. server/routes.ts line 1491 implements the
+endpoint. Pulled forward into pre-COLA per user instruction.</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>session 299e9a73 turn 5, ~2026-04-28.
+---</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23" ht="90" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Rotate GitHub PAT (because old PAT was committed in SESSION_HANDOFF files)</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr"/>
+      <c r="D23" s="3" t="inlineStr"/>
+      <c r="E23" s="3" t="inlineStr"/>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>Closure evidence: no ghp_* or github_pat_* patterns in current
+SESSION_HANDOFF.md or SESSION_HANDOFF-2.md as of 2026-05-01.</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>session 299e9a73, ~2026-04-28.
+---</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr"/>
+    </row>
+    <row r="24" ht="90" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>C6</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>VeritaPolicy service-line filtering removed (formerly #4)</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr"/>
+      <c r="D24" s="2" t="inlineStr"/>
+      <c r="E24" s="2" t="inlineStr"/>
+      <c r="F24" s="2" t="inlineStr">
         <is>
           <t>Closure rationale (operator decision 2026-05-10): Keep all
 VeritaPolicy rows. CFR-only references with no accreditor reference
@@ -1914,29 +1932,29 @@
 report misread the design intent.</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr">
+      <c r="G24" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H22" s="2" t="inlineStr"/>
-    </row>
-    <row r="23" ht="90" customHeight="1">
-      <c r="A23" s="3" t="inlineStr">
+      <c r="H24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25" ht="90" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
         <is>
           <t>C7</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>CLIA number format validation (formerly #13)</t>
         </is>
       </c>
-      <c r="C23" s="3" t="inlineStr"/>
-      <c r="D23" s="3" t="inlineStr"/>
-      <c r="E23" s="3" t="inlineStr"/>
-      <c r="F23" s="3" t="inlineStr">
+      <c r="C25" s="3" t="inlineStr"/>
+      <c r="D25" s="3" t="inlineStr"/>
+      <c r="E25" s="3" t="inlineStr"/>
+      <c r="F25" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: shared/validateClia.ts defines CLIA_REGEX =
 /^\d{2}D\d{7}$/ (line 24), validateClia() helper with whitespace
@@ -1947,30 +1965,30 @@
 shape exists and behaves as specified.</t>
         </is>
       </c>
-      <c r="G23" s="3" t="inlineStr">
+      <c r="G25" s="3" t="inlineStr">
         <is>
           <t>Agent verification 2026-05-10 via grep + file read.
 Operator confirmed shipped 2026-05-10.
 ---</t>
         </is>
       </c>
-      <c r="H23" s="3" t="inlineStr"/>
-    </row>
-    <row r="24" ht="90" customHeight="1">
-      <c r="A24" s="2" t="inlineStr">
+      <c r="H25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26" ht="90" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>C8</t>
         </is>
       </c>
-      <c r="B24" s="2" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t>VeritaMap lab-wide menu toggle (formerly #19)</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr"/>
-      <c r="D24" s="2" t="inlineStr"/>
-      <c r="E24" s="2" t="inlineStr"/>
-      <c r="F24" s="2" t="inlineStr">
+      <c r="C26" s="2" t="inlineStr"/>
+      <c r="D26" s="2" t="inlineStr"/>
+      <c r="E26" s="2" t="inlineStr"/>
+      <c r="F26" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: client/src/pages/VeritaMapLabwidePage.tsx
 exists and implements the labwide read-only union view. Route is
@@ -1980,59 +1998,59 @@
 parking lot plan (read-only union view, per-session toggle) shipped.</t>
         </is>
       </c>
-      <c r="G24" s="2" t="inlineStr">
+      <c r="G26" s="2" t="inlineStr">
         <is>
           <t>Agent verification 2026-05-10 via grep + file read.
 Operator confirmed shipped 2026-05-10.
 ---</t>
         </is>
       </c>
-      <c r="H24" s="2" t="inlineStr"/>
-    </row>
-    <row r="25" ht="90" customHeight="1">
-      <c r="A25" s="3" t="inlineStr">
+      <c r="H26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27" ht="90" customHeight="1">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>C9</t>
         </is>
       </c>
-      <c r="B25" s="3" t="inlineStr">
+      <c r="B27" s="3" t="inlineStr">
         <is>
           <t>Tier-1 smoke test checklist (formerly #6)</t>
         </is>
       </c>
-      <c r="C25" s="3" t="inlineStr"/>
-      <c r="D25" s="3" t="inlineStr"/>
-      <c r="E25" s="3" t="inlineStr"/>
-      <c r="F25" s="3" t="inlineStr">
+      <c r="C27" s="3" t="inlineStr"/>
+      <c r="D27" s="3" t="inlineStr"/>
+      <c r="E27" s="3" t="inlineStr"/>
+      <c r="F27" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: docs/smoke-test-tier1.md documents the Tier-1
 smoke-test process and post-deploy verification steps. Shipped via
 PR #81 as part of the 2026-05-10 wave.</t>
         </is>
       </c>
-      <c r="G25" s="3" t="inlineStr">
+      <c r="G27" s="3" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H25" s="3" t="inlineStr"/>
-    </row>
-    <row r="26" ht="90" customHeight="1">
-      <c r="A26" s="2" t="inlineStr">
+      <c r="H27" s="3" t="inlineStr"/>
+    </row>
+    <row r="28" ht="90" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>C10</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="B28" s="2" t="inlineStr">
         <is>
           <t>Per-module gating (formerly #7)</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr"/>
-      <c r="D26" s="2" t="inlineStr"/>
-      <c r="E26" s="2" t="inlineStr"/>
-      <c r="F26" s="2" t="inlineStr">
+      <c r="C28" s="2" t="inlineStr"/>
+      <c r="D28" s="2" t="inlineStr"/>
+      <c r="E28" s="2" t="inlineStr"/>
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: Client-side useIsReadOnly module keys wired
 on client/src/pages/VeritaPolicyAppPage.tsx and
@@ -2047,29 +2065,29 @@
 PR #76.</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr">
+      <c r="G28" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H26" s="2" t="inlineStr"/>
-    </row>
-    <row r="27" ht="90" customHeight="1">
-      <c r="A27" s="3" t="inlineStr">
+      <c r="H28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29" ht="90" customHeight="1">
+      <c r="A29" s="3" t="inlineStr">
         <is>
           <t>C11</t>
         </is>
       </c>
-      <c r="B27" s="3" t="inlineStr">
+      <c r="B29" s="3" t="inlineStr">
         <is>
           <t>VeritaStock shipped copy (formerly #8)</t>
         </is>
       </c>
-      <c r="C27" s="3" t="inlineStr"/>
-      <c r="D27" s="3" t="inlineStr"/>
-      <c r="E27" s="3" t="inlineStr"/>
-      <c r="F27" s="3" t="inlineStr">
+      <c r="C29" s="3" t="inlineStr"/>
+      <c r="D29" s="3" t="inlineStr"/>
+      <c r="E29" s="3" t="inlineStr"/>
+      <c r="F29" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: client/src/pages/ArticleInventoryManagementPage.tsx
 line 305 footer reads "platform that includes VeritaStock™" instead
@@ -2077,29 +2095,29 @@
 on /resources/laboratory-inventory-management. Shipped via PR #75.</t>
         </is>
       </c>
-      <c r="G27" s="3" t="inlineStr">
+      <c r="G29" s="3" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H27" s="3" t="inlineStr"/>
-    </row>
-    <row r="28" ht="90" customHeight="1">
-      <c r="A28" s="2" t="inlineStr">
+      <c r="H29" s="3" t="inlineStr"/>
+    </row>
+    <row r="30" ht="90" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>C12</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="B30" s="2" t="inlineStr">
         <is>
           <t>Admin report one-row-per-lab (formerly #14)</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr"/>
-      <c r="D28" s="2" t="inlineStr"/>
-      <c r="E28" s="2" t="inlineStr"/>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="C30" s="2" t="inlineStr"/>
+      <c r="D30" s="2" t="inlineStr"/>
+      <c r="E30" s="2" t="inlineStr"/>
+      <c r="F30" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: /api/admin/report rewritten in
 server/routes.ts (~line 595) to LEFT JOIN labs on
@@ -2114,56 +2132,56 @@
 prerequisite, not a code bug). Shipped via PR #85.</t>
         </is>
       </c>
-      <c r="G28" s="2" t="inlineStr">
+      <c r="G30" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H28" s="2" t="inlineStr"/>
-    </row>
-    <row r="29" ht="90" customHeight="1">
-      <c r="A29" s="3" t="inlineStr">
+      <c r="H30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31" ht="90" customHeight="1">
+      <c r="A31" s="3" t="inlineStr">
         <is>
           <t>C14</t>
         </is>
       </c>
-      <c r="B29" s="3" t="inlineStr">
+      <c r="B31" s="3" t="inlineStr">
         <is>
           <t>UI relabel "CLIA TEa" -&gt; "Lab-Set Internal Goal" (formerly #1)</t>
         </is>
       </c>
-      <c r="C29" s="3" t="inlineStr"/>
-      <c r="D29" s="3" t="inlineStr"/>
-      <c r="E29" s="3" t="inlineStr"/>
-      <c r="F29" s="3" t="inlineStr">
+      <c r="C31" s="3" t="inlineStr"/>
+      <c r="D31" s="3" t="inlineStr"/>
+      <c r="E31" s="3" t="inlineStr"/>
+      <c r="F31" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: Shipped across four PRs over 2026-05-10.</t>
         </is>
       </c>
-      <c r="G29" s="3" t="inlineStr">
+      <c r="G31" s="3" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H29" s="3" t="inlineStr"/>
-    </row>
-    <row r="30" ht="90" customHeight="1">
-      <c r="A30" s="2" t="inlineStr">
+      <c r="H31" s="3" t="inlineStr"/>
+    </row>
+    <row r="32" ht="90" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t>C13</t>
         </is>
       </c>
-      <c r="B30" s="2" t="inlineStr">
+      <c r="B32" s="2" t="inlineStr">
         <is>
           <t>WSLH PT vendor (formerly #15)</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr"/>
-      <c r="D30" s="2" t="inlineStr"/>
-      <c r="E30" s="2" t="inlineStr"/>
-      <c r="F30" s="2" t="inlineStr">
+      <c r="C32" s="2" t="inlineStr"/>
+      <c r="D32" s="2" t="inlineStr"/>
+      <c r="E32" s="2" t="inlineStr"/>
+      <c r="F32" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: Shipped 2026-05-10 via PR #79 (merge commit
 eeebc6e; merged after rebase to resolve a server/db.ts collision
@@ -2181,68 +2199,9 @@
 'WSLH' is the post-deploy success signal. Shipped via PR #79.</t>
         </is>
       </c>
-      <c r="G30" s="2" t="inlineStr">
+      <c r="G32" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
----</t>
-        </is>
-      </c>
-      <c r="H30" s="2" t="inlineStr"/>
-    </row>
-    <row r="31" ht="90" customHeight="1">
-      <c r="A31" s="3" t="inlineStr">
-        <is>
-          <t>C15</t>
-        </is>
-      </c>
-      <c r="B31" s="3" t="inlineStr">
-        <is>
-          <t>VeritaStock lot tracking + expiration + reorder alerts (formerly #21)</t>
-        </is>
-      </c>
-      <c r="C31" s="3" t="inlineStr"/>
-      <c r="D31" s="3" t="inlineStr"/>
-      <c r="E31" s="3" t="inlineStr"/>
-      <c r="F31" s="3" t="inlineStr">
-        <is>
-          <t>Closure evidence: VeritaStock™ shipped the bench-level inventory
-features the Perplexity competitor analysis identified as a gap:</t>
-        </is>
-      </c>
-      <c r="G31" s="3" t="inlineStr">
-        <is>
-          <t>Originally Perplexity competitor analysis 2026-05-10.
-Audit 2026-05-21 confirmed the feature set ships today.
----</t>
-        </is>
-      </c>
-      <c r="H31" s="3" t="inlineStr"/>
-    </row>
-    <row r="32" ht="90" customHeight="1">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>C16</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>PAL studies guided workflow (formerly #23)</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr"/>
-      <c r="D32" s="2" t="inlineStr"/>
-      <c r="E32" s="2" t="inlineStr"/>
-      <c r="F32" s="2" t="inlineStr">
-        <is>
-          <t>Closure evidence: VeritaCheck™ already ships the Precision /
-Accuracy / Linearity (PAL) study set under EP-protocol naming:</t>
-        </is>
-      </c>
-      <c r="G32" s="2" t="inlineStr">
-        <is>
-          <t>Originally Perplexity competitor analysis 2026-05-10.
-Audit 2026-05-21 confirmed the EP studies cover the PAL framing in
-full.
 ---</t>
         </is>
       </c>
@@ -2251,12 +2210,12 @@
     <row r="33" ht="90" customHeight="1">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>C17</t>
+          <t>C15</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>Source-grounded 21/29/45 CFR + 42 CFR 482-485 (formerly #26)</t>
+          <t>VeritaStock lot tracking + expiration + reorder alerts (formerly #21)</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr"/>
@@ -2264,35 +2223,94 @@
       <c r="E33" s="3" t="inlineStr"/>
       <c r="F33" s="3" t="inlineStr">
         <is>
+          <t>Closure evidence: VeritaStock™ shipped the bench-level inventory
+features the Perplexity competitor analysis identified as a gap:</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>Originally Perplexity competitor analysis 2026-05-10.
+Audit 2026-05-21 confirmed the feature set ships today.
+---</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr"/>
+    </row>
+    <row r="34" ht="90" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>C16</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>PAL studies guided workflow (formerly #23)</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr"/>
+      <c r="D34" s="2" t="inlineStr"/>
+      <c r="E34" s="2" t="inlineStr"/>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>Closure evidence: VeritaCheck™ already ships the Precision /
+Accuracy / Linearity (PAL) study set under EP-protocol naming:</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>Originally Perplexity competitor analysis 2026-05-10.
+Audit 2026-05-21 confirmed the EP studies cover the PAL framing in
+full.
+---</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr"/>
+    </row>
+    <row r="35" ht="90" customHeight="1">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>C17</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>Source-grounded 21/29/45 CFR + 42 CFR 482-485 (formerly #26)</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr"/>
+      <c r="D35" s="3" t="inlineStr"/>
+      <c r="E35" s="3" t="inlineStr"/>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
           <t>Closure evidence: PR #301 (commit 8c27806, merged 2026-05-21)
 source-grounded the 74 remaining non-493 entries in
 server/cfrRequirements.ts against verbatim eCFR XML. Breakdown
 shipped:</t>
         </is>
       </c>
-      <c r="G33" s="3" t="inlineStr">
+      <c r="G35" s="3" t="inlineStr">
         <is>
           <t>PR #301; tasks #18 in the in-session task tracker.
 ---</t>
         </is>
       </c>
-      <c r="H33" s="3" t="inlineStr"/>
-    </row>
-    <row r="34" ht="90" customHeight="1">
-      <c r="A34" s="2" t="inlineStr">
+      <c r="H35" s="3" t="inlineStr"/>
+    </row>
+    <row r="36" ht="90" customHeight="1">
+      <c r="A36" s="2" t="inlineStr">
         <is>
           <t>C18</t>
         </is>
       </c>
-      <c r="B34" s="2" t="inlineStr">
+      <c r="B36" s="2" t="inlineStr">
         <is>
           <t>VeritaPolicy "Non CLIA" chapter rename (formerly #3)</t>
         </is>
       </c>
-      <c r="C34" s="2" t="inlineStr"/>
-      <c r="D34" s="2" t="inlineStr"/>
-      <c r="E34" s="2" t="inlineStr"/>
-      <c r="F34" s="2" t="inlineStr">
+      <c r="C36" s="2" t="inlineStr"/>
+      <c r="D36" s="2" t="inlineStr"/>
+      <c r="E36" s="2" t="inlineStr"/>
+      <c r="F36" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #300 (commit 34d7707, merged 2026-05-21)
 renamed all 44 user-facing chapter labels in
@@ -2303,7 +2321,7 @@
 page.</t>
         </is>
       </c>
-      <c r="G34" s="2" t="inlineStr">
+      <c r="G36" s="2" t="inlineStr">
         <is>
           <t>CAP customer screenshot of the /veritapolicy chapter
 headers, 2026-05-01 evening. PR #300; tasks #17 in the in-session
@@ -2311,23 +2329,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H34" s="2" t="inlineStr"/>
-    </row>
-    <row r="35" ht="90" customHeight="1">
-      <c r="A35" s="3" t="inlineStr">
+      <c r="H36" s="2" t="inlineStr"/>
+    </row>
+    <row r="37" ht="90" customHeight="1">
+      <c r="A37" s="3" t="inlineStr">
         <is>
           <t>C19</t>
         </is>
       </c>
-      <c r="B35" s="3" t="inlineStr">
+      <c r="B37" s="3" t="inlineStr">
         <is>
           <t>VeritaStock department-scope toggle (formerly #31)</t>
         </is>
       </c>
-      <c r="C35" s="3" t="inlineStr"/>
-      <c r="D35" s="3" t="inlineStr"/>
-      <c r="E35" s="3" t="inlineStr"/>
-      <c r="F35" s="3" t="inlineStr">
+      <c r="C37" s="3" t="inlineStr"/>
+      <c r="D37" s="3" t="inlineStr"/>
+      <c r="E37" s="3" t="inlineStr"/>
+      <c r="F37" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #319 (commit d01f5fe, merged 2026-05-22)
 shipped the persistent dept-scope toggle on VeritaStockPage. A new
@@ -2338,7 +2356,7 @@
 workspace without re-filtering.</t>
         </is>
       </c>
-      <c r="G35" s="3" t="inlineStr">
+      <c r="G37" s="3" t="inlineStr">
         <is>
           <t>John, San Carlos lab, 2026-05-21. Same conversation that
 drove the vendor dropdown (PR #304), FILTERED VIEW banner (PR #305),
@@ -2346,23 +2364,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H35" s="3" t="inlineStr"/>
-    </row>
-    <row r="36" ht="90" customHeight="1">
-      <c r="A36" s="2" t="inlineStr">
+      <c r="H37" s="3" t="inlineStr"/>
+    </row>
+    <row r="38" ht="90" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
         <is>
           <t>C20</t>
         </is>
       </c>
-      <c r="B36" s="2" t="inlineStr">
+      <c r="B38" s="2" t="inlineStr">
         <is>
           <t>Primary-lab seat counting (formerly #12)</t>
         </is>
       </c>
-      <c r="C36" s="2" t="inlineStr"/>
-      <c r="D36" s="2" t="inlineStr"/>
-      <c r="E36" s="2" t="inlineStr"/>
-      <c r="F36" s="2" t="inlineStr">
+      <c r="C38" s="2" t="inlineStr"/>
+      <c r="D38" s="2" t="inlineStr"/>
+      <c r="E38" s="2" t="inlineStr"/>
+      <c r="F38" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: is_primary_lab INTEGER NOT NULL DEFAULT 0
 column was added to the lab_members table at db.ts:1276, with the
@@ -2373,7 +2391,7 @@
 is_primary_lab=1 ordering).</t>
         </is>
       </c>
-      <c r="G36" s="2" t="inlineStr">
+      <c r="G38" s="2" t="inlineStr">
         <is>
           <t>2026-05-07 multi-lab discussion. Build shipped as part
 of the Multi-Lab Tier 2 architecture work (Phase 3.x series, prior
@@ -2382,23 +2400,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H36" s="2" t="inlineStr"/>
-    </row>
-    <row r="37" ht="90" customHeight="1">
-      <c r="A37" s="3" t="inlineStr">
+      <c r="H38" s="2" t="inlineStr"/>
+    </row>
+    <row r="39" ht="90" customHeight="1">
+      <c r="A39" s="3" t="inlineStr">
         <is>
           <t>C21</t>
         </is>
       </c>
-      <c r="B37" s="3" t="inlineStr">
+      <c r="B39" s="3" t="inlineStr">
         <is>
           <t>Multi-lab pricing model — Option A (formerly #11)</t>
         </is>
       </c>
-      <c r="C37" s="3" t="inlineStr"/>
-      <c r="D37" s="3" t="inlineStr"/>
-      <c r="E37" s="3" t="inlineStr"/>
-      <c r="F37" s="3" t="inlineStr">
+      <c r="C39" s="3" t="inlineStr"/>
+      <c r="D39" s="3" t="inlineStr"/>
+      <c r="E39" s="3" t="inlineStr"/>
+      <c r="F39" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #322 (commit 0ccd925, merged 2026-05-22)
 added the customer-facing line to the pricing page that reflects
@@ -2411,7 +2429,7 @@
 Enterprise+ block, reads:</t>
         </is>
       </c>
-      <c r="G37" s="3" t="inlineStr">
+      <c r="G39" s="3" t="inlineStr">
         <is>
           <t>2026-05-07 multi-lab discussion (Lisa Veri's
 canonical-case session). PR #322 (initial build); softening PR
@@ -2420,30 +2438,30 @@
 ---</t>
         </is>
       </c>
-      <c r="H37" s="3" t="inlineStr"/>
-    </row>
-    <row r="38" ht="90" customHeight="1">
-      <c r="A38" s="2" t="inlineStr">
+      <c r="H39" s="3" t="inlineStr"/>
+    </row>
+    <row r="40" ht="90" customHeight="1">
+      <c r="A40" s="2" t="inlineStr">
         <is>
           <t>C22</t>
         </is>
       </c>
-      <c r="B38" s="2" t="inlineStr">
+      <c r="B40" s="2" t="inlineStr">
         <is>
           <t>VeritaOps cost-per-test module (formerly #10)</t>
         </is>
       </c>
-      <c r="C38" s="2" t="inlineStr"/>
-      <c r="D38" s="2" t="inlineStr"/>
-      <c r="E38" s="2" t="inlineStr"/>
-      <c r="F38" s="2" t="inlineStr">
+      <c r="C40" s="2" t="inlineStr"/>
+      <c r="D40" s="2" t="inlineStr"/>
+      <c r="E40" s="2" t="inlineStr"/>
+      <c r="F40" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: v1 of the VeritaOps Cost-Per-Reportable-Test
 (CPRT) module shipped across PR #325 through PR #330 on 2026-05-22.
 The module is feature-complete for the typical lab director workflow.</t>
         </is>
       </c>
-      <c r="G38" s="2" t="inlineStr">
+      <c r="G40" s="2" t="inlineStr">
         <is>
           <t>This thread, 2026-05-07 12:05 PM CDT, user message:
 "Parking lot: build an operations module for cost per test
@@ -2452,262 +2470,262 @@
 ---</t>
         </is>
       </c>
-      <c r="H38" s="2" t="inlineStr"/>
-    </row>
-    <row r="39" ht="90" customHeight="1">
-      <c r="A39" s="3" t="inlineStr">
+      <c r="H40" s="2" t="inlineStr"/>
+    </row>
+    <row r="41" ht="90" customHeight="1">
+      <c r="A41" s="3" t="inlineStr">
         <is>
           <t>C23</t>
         </is>
       </c>
-      <c r="B39" s="3" t="inlineStr">
+      <c r="B41" s="3" t="inlineStr">
         <is>
           <t>CCL lab name visual disambiguation in lab switcher (formerly #34)</t>
         </is>
       </c>
-      <c r="C39" s="3" t="inlineStr"/>
-      <c r="D39" s="3" t="inlineStr">
+      <c r="C41" s="3" t="inlineStr"/>
+      <c r="D41" s="3" t="inlineStr">
         <is>
           <t>XS (under 1 day, actual)</t>
         </is>
       </c>
-      <c r="E39" s="3" t="inlineStr">
+      <c r="E41" s="3" t="inlineStr">
         <is>
           <t>Low — cosmetic; only mattered when Lisa or Michael picked the wrong lab from...</t>
         </is>
       </c>
-      <c r="F39" s="3" t="inlineStr">
+      <c r="F41" s="3" t="inlineStr">
         <is>
           <t>Effort: XS (under 1 day, actual)
 Importance: Low — cosmetic; only mattered when Lisa or Michael picked the wrong lab from the dropdown.</t>
         </is>
       </c>
-      <c r="G39" s="3" t="inlineStr">
+      <c r="G41" s="3" t="inlineStr">
         <is>
           <t>flagged 2026-05-23 immediately after provisioning Lisa's CCL lab; closed 2026-05-24.
 ---</t>
         </is>
       </c>
-      <c r="H39" s="3" t="inlineStr"/>
-    </row>
-    <row r="40" ht="90" customHeight="1">
-      <c r="A40" s="2" t="inlineStr">
+      <c r="H41" s="3" t="inlineStr"/>
+    </row>
+    <row r="42" ht="90" customHeight="1">
+      <c r="A42" s="2" t="inlineStr">
         <is>
           <t>C24</t>
         </is>
       </c>
-      <c r="B40" s="2" t="inlineStr">
+      <c r="B42" s="2" t="inlineStr">
         <is>
           <t>VC Unlimited Y1/Y2 price disclosure UX (formerly #35)</t>
         </is>
       </c>
-      <c r="C40" s="2" t="inlineStr"/>
-      <c r="D40" s="2" t="inlineStr">
+      <c r="C42" s="2" t="inlineStr"/>
+      <c r="D42" s="2" t="inlineStr">
         <is>
           <t>XS (under 1 day, actual)</t>
         </is>
       </c>
-      <c r="E40" s="2" t="inlineStr">
+      <c r="E42" s="2" t="inlineStr">
         <is>
           <t>Low when shipped (proactive, no customer complaint yet) — but high if a procu...</t>
         </is>
       </c>
-      <c r="F40" s="2" t="inlineStr">
+      <c r="F42" s="2" t="inlineStr">
         <is>
           <t>Effort: XS (under 1 day, actual)
 Importance: Low when shipped (proactive, no customer complaint yet) — but high if a procurement reviewer later disputes the $499 renewal as undisclosed.</t>
         </is>
       </c>
-      <c r="G40" s="2" t="inlineStr">
+      <c r="G42" s="2" t="inlineStr">
         <is>
           <t>Pricing rebuild 2026-05-23; closed 2026-05-24 proactively before any customer dispute.
 ---</t>
         </is>
       </c>
-      <c r="H40" s="2" t="inlineStr"/>
-    </row>
-    <row r="41" ht="90" customHeight="1">
-      <c r="A41" s="3" t="inlineStr">
+      <c r="H42" s="2" t="inlineStr"/>
+    </row>
+    <row r="43" ht="90" customHeight="1">
+      <c r="A43" s="3" t="inlineStr">
         <is>
           <t>C25</t>
         </is>
       </c>
-      <c r="B41" s="3" t="inlineStr">
+      <c r="B43" s="3" t="inlineStr">
         <is>
           <t>VeritaQC Phase 1 (Levey-Jennings + Westgard live engine) (formerly #20)</t>
         </is>
       </c>
-      <c r="C41" s="3" t="inlineStr"/>
-      <c r="D41" s="3" t="inlineStr">
+      <c r="C43" s="3" t="inlineStr"/>
+      <c r="D43" s="3" t="inlineStr">
         <is>
           <t>L (about 5 days end-to-end, actual: Phase 0 schema → Phase 1A evaluator → 1B...</t>
         </is>
       </c>
-      <c r="E41" s="3" t="inlineStr">
+      <c r="E43" s="3" t="inlineStr">
         <is>
           <t>High — largest single gap vs myLabCompliance.io per Perplexity competitor ana...</t>
         </is>
       </c>
-      <c r="F41" s="3" t="inlineStr">
+      <c r="F43" s="3" t="inlineStr">
         <is>
           <t>Effort: L (about 5 days end-to-end, actual: Phase 0 schema → Phase 1A evaluator → 1B entry UI → 1C daily review → 1D monthly PDF + attestation)
 Importance: High — largest single gap vs myLabCompliance.io per Perplexity competitor analysis; promotes VeritaAssure from documentation tool to lab operations platform.</t>
         </is>
       </c>
-      <c r="G41" s="3" t="inlineStr">
+      <c r="G43" s="3" t="inlineStr">
         <is>
           <t>Perplexity competitor analysis 2026-05-10. Scoping confirmed via the build_phase1_mockup.py iterations 2026-05-24. Shipped 2026-05-25.
 ---</t>
         </is>
       </c>
-      <c r="H41" s="3" t="inlineStr"/>
-    </row>
-    <row r="42" ht="90" customHeight="1">
-      <c r="A42" s="2" t="inlineStr">
+      <c r="H43" s="3" t="inlineStr"/>
+    </row>
+    <row r="44" ht="90" customHeight="1">
+      <c r="A44" s="2" t="inlineStr">
         <is>
           <t>C26</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
+      <c r="B44" s="2" t="inlineStr">
         <is>
           <t>VeritaLab CMS-116 application support + state licensing registry (formerly #22)</t>
         </is>
       </c>
-      <c r="C42" s="2" t="inlineStr"/>
-      <c r="D42" s="2" t="inlineStr">
+      <c r="C44" s="2" t="inlineStr"/>
+      <c r="D44" s="2" t="inlineStr">
         <is>
           <t>M (1-2 weeks for v1, actual)</t>
         </is>
       </c>
-      <c r="E42" s="2" t="inlineStr">
+      <c r="E44" s="2" t="inlineStr">
         <is>
           <t>Medium — competitor parity (myLabCompliance.io) plus useful at lab startup an...</t>
         </is>
       </c>
-      <c r="F42" s="2" t="inlineStr">
+      <c r="F44" s="2" t="inlineStr">
         <is>
           <t>Effort: M (1-2 weeks for v1, actual)
 Importance: Medium — competitor parity (myLabCompliance.io) plus useful at lab startup and at certificate-type changes.</t>
         </is>
       </c>
-      <c r="G42" s="2" t="inlineStr">
+      <c r="G44" s="2" t="inlineStr">
         <is>
           <t>Perplexity competitor analysis (myLabCompliance.io), 2026-05-10. Reclassified as a VeritaLab extension 2026-05-25. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H42" s="2" t="inlineStr"/>
-    </row>
-    <row r="43" ht="90" customHeight="1">
-      <c r="A43" s="3" t="inlineStr">
+      <c r="H44" s="2" t="inlineStr"/>
+    </row>
+    <row r="45" ht="90" customHeight="1">
+      <c r="A45" s="3" t="inlineStr">
         <is>
           <t>C27</t>
         </is>
       </c>
-      <c r="B43" s="3" t="inlineStr">
+      <c r="B45" s="3" t="inlineStr">
         <is>
           <t>Active vs view-only seat split (formerly #33)</t>
         </is>
       </c>
-      <c r="C43" s="3" t="inlineStr"/>
-      <c r="D43" s="3" t="inlineStr">
+      <c r="C45" s="3" t="inlineStr"/>
+      <c r="D45" s="3" t="inlineStr">
         <is>
           <t>M (~1 week of engineering, actual: shipped in a single multi-PR session)</t>
         </is>
       </c>
-      <c r="E43" s="3" t="inlineStr">
+      <c r="E45" s="3" t="inlineStr">
         <is>
           <t>Medium — closed the gap between /pricing copy and product behavior; gives sal...</t>
         </is>
       </c>
-      <c r="F43" s="3" t="inlineStr">
+      <c r="F45" s="3" t="inlineStr">
         <is>
           <t>Effort: M (~1 week of engineering, actual: shipped in a single multi-PR session)
 Importance: Medium — closed the gap between /pricing copy and product behavior; gives sales a clean answer for "do you charge for our medical director?"</t>
         </is>
       </c>
-      <c r="G43" s="3" t="inlineStr">
+      <c r="G45" s="3" t="inlineStr">
         <is>
           <t>Pricing analysis doc Decision 3 (2026-05-21); MEDIUM scenario revised 2026-05-29 to retire the "unlimited view-only" claim. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H43" s="3" t="inlineStr"/>
-    </row>
-    <row r="44" ht="90" customHeight="1">
-      <c r="A44" s="2" t="inlineStr">
+      <c r="H45" s="3" t="inlineStr"/>
+    </row>
+    <row r="46" ht="90" customHeight="1">
+      <c r="A46" s="2" t="inlineStr">
         <is>
           <t>C28</t>
         </is>
       </c>
-      <c r="B44" s="2" t="inlineStr">
+      <c r="B46" s="2" t="inlineStr">
         <is>
           <t>"Why VeritaCheck" comparative one-pager (formerly #37)</t>
         </is>
       </c>
-      <c r="C44" s="2" t="inlineStr"/>
-      <c r="D44" s="2" t="inlineStr">
+      <c r="C46" s="2" t="inlineStr"/>
+      <c r="D46" s="2" t="inlineStr">
         <is>
           <t>S (one design pass + four claim paragraphs + PDF + matching marketing-site pa...</t>
         </is>
       </c>
-      <c r="E44" s="2" t="inlineStr">
+      <c r="E46" s="2" t="inlineStr">
         <is>
           <t>Medium — closed a positioning gap surfaced by six COLA conference attendees a...</t>
         </is>
       </c>
-      <c r="F44" s="2" t="inlineStr">
+      <c r="F46" s="2" t="inlineStr">
         <is>
           <t>Effort: S (one design pass + four claim paragraphs + PDF + matching marketing-site page, actual)
 Importance: Medium — closed a positioning gap surfaced by six COLA conference attendees attached to a legacy verification tool; converts product-quality advantage into a leave-behind Lisa can hand out.</t>
         </is>
       </c>
-      <c r="G44" s="2" t="inlineStr">
+      <c r="G46" s="2" t="inlineStr">
         <is>
           <t>2026-05-11 / 2026-05-12 conference notes review with Michael. Conference attendees (Whitehead, Odegard, Othman, Molinelli, Kyle, Allred) expressed interest in equivalent / superior product. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H44" s="2" t="inlineStr"/>
-    </row>
-    <row r="45" ht="90" customHeight="1">
-      <c r="A45" s="3" t="inlineStr">
+      <c r="H46" s="2" t="inlineStr"/>
+    </row>
+    <row r="47" ht="90" customHeight="1">
+      <c r="A47" s="3" t="inlineStr">
         <is>
           <t>C29</t>
         </is>
       </c>
-      <c r="B45" s="3" t="inlineStr">
+      <c r="B47" s="3" t="inlineStr">
         <is>
           <t>VeritaPolicy approval workflow — MediaLab functional mirror</t>
         </is>
       </c>
-      <c r="C45" s="3" t="inlineStr"/>
-      <c r="D45" s="3" t="inlineStr">
+      <c r="C47" s="3" t="inlineStr"/>
+      <c r="D47" s="3" t="inlineStr">
         <is>
           <t>XL (one focused session, 12 PRs landed)</t>
         </is>
       </c>
-      <c r="E45" s="3" t="inlineStr">
+      <c r="E47" s="3" t="inlineStr">
         <is>
           <t>High — replaces MediaLab Document Control ($752/$2,250 starting price, scalin...</t>
         </is>
       </c>
-      <c r="F45" s="3" t="inlineStr">
+      <c r="F47" s="3" t="inlineStr">
         <is>
           <t>Effort: XL (one focused session, 12 PRs landed)
 Importance: High — replaces MediaLab Document Control ($752/$2,250 starting price, scaling to $10K-$20K/yr at enterprise per Capterra public data) with an included VeritaPolicy feature; closes a real positioning gap and gives sales a direct comparator line.</t>
         </is>
       </c>
-      <c r="G45" s="3" t="inlineStr">
+      <c r="G47" s="3" t="inlineStr">
         <is>
           <t>Pricing strategy conversation 2026-05-29 (Michael: "I don't like bolt-ons; we should replicate this") → scoped 8 phases → shipped all 12 PRs in single session. Shipped 2026-05-29.
 ---</t>
         </is>
       </c>
-      <c r="H45" s="3" t="inlineStr"/>
+      <c r="H47" s="3" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H45"/>
+  <autoFilter ref="A1:H47"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
docs(parking-lot): log VeritaAssure optimizations 51/52; scope 36 into VeritaResponse
TASK: Log Michael's three 2026-09-28 "for later (placeholder)" VeritaAssure optimizations to the parking lot.
PLAN: Add OPEN #51 (VeritaTrack task owner + owner-scoped reminder routing) and #52 (Medical Director seat via account-grant dropdown, designate/transfer-MD block); fold the VeritaResponse internal non-conforming-event write-up direction into existing #36 as the awaited scope decision; regenerate PARKING_LOT.xlsx.
Self-check:
  - No code touched; docs + regenerated xlsx mirror only.
  - xlsx re-run reports 17 OPEN / 46 CLOSED / 6 RETIRED; #36 updated in place (not duplicated).
  - Michael's verbatim wording preserved on all three; "veritatask" mapped to VeritaTrack (no VeritaTask module exists).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PARKING_LOT.xlsx
+++ b/PARKING_LOT.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RETIRED" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$47</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RETIRED'!$A$1:$H$7</definedName>
   </definedNames>
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -933,7 +933,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Parked 2026-05-26 with a one-line scope intent. Michael indicated he will walk through the requirements in more detail in a follow-up conversation. Do not start building until that walkthrough happ...</t>
+          <t>Scoped, not started (updated 2026-09-28). Now lands in VeritaResponse per Michael's direction above; the earlier "new standalone module" framing is superseded. Do not start building until Michael g...</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -1207,8 +1207,94 @@
       </c>
       <c r="H16" s="2" t="inlineStr"/>
     </row>
+    <row r="17" ht="90" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>VeritaTrack task owner + owner-scoped reminder routing</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Open, not started. Placeholder pending build. Open questions: is the owner a staff_employee or a seat user, and how are reminder recipients currently chosen.</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>S-M (1-3 days to ~1.5 weeks) — add an owner on a VeritaTrack task, selectable...</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Medium — cuts reminder-email noise so people only get the tasks that are thei...</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Michael, verbatim (2026-09-28): "In veritatask, we should be able to assign an owner from staff that are built, then in the reminder section, we should be able to designate reminder emails only to the owner. The hem person does not need the chemistry reminders, etc." Module note: there is no VeritaTask module in the codebase; the task/reminder surface is VeritaTrack (client/src/pages/VeritaTrackAppPage.tsx), so this lands there. Today VeritaTrack tasks are not owned by a specific staff member and reminder emails are not recipient-scoped to an owner. The build adds (a) an owner selector on each task drawn from the lab's VeritaStaff roster, and (b) a reminder setting that routes the reminder email to only that owner. Confirm the current reminder recipient model before sizing.</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-28 session, Michael "for later (placeholder)" optimization #1 (relaying from the Lab Members / VeritaAssure screens).</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>Post-COLA. No customer urgency.
+---</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="90" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Medical Director seat via account-grant dropdown (designate / transfer MD)</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Open, not started. Placeholder. Confirm the current MD-seat assignment path and the one-MD-per-location enforcement point before sizing.</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>S-M (1-3 days to ~1.5 weeks) — move MD-seat assignment onto the same per-memb...</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Medium-High — the MD seat is a recurring friction point (Georgetown, SCAHC MD...</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Michael, verbatim (2026-09-28): "The way we are doing the medical director seat is silly. Why not just use the account grant dropdown to give a medical director seat. If the person is already in, then we should just be able to grant the medical director seat the same way we promote people to admin or reduce them to staff as long as we only have 1 per location. Maybe do another block like the transfer ownership block as 'designate medical director or transfer medical director'." So: fold the MD seat into the existing member role dropdown (Admin / Staff / ... + Medical Director) with a single-MD-per-lab constraint, and add a dedicated designate-or-transfer-MD block that mirrors the transfer-ownership UX for changing the MD. Cross-ref [[project_medical_director_designation]] and the seat model.</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28 session, Michael "for later (placeholder)" optimization #3 (relaying from the Lab Members screen).</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Post-COLA. No customer urgency.
+---</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H16"/>
+  <autoFilter ref="A1:H18"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
docs(parking-lot): log VeritaAssure optimizations 51/52; scope 36 into VeritaResponse (#1353)
TASK: Log Michael's 2026-09-28 for-later VeritaAssure optimizations to the parking lot.
PLAN: Add OPEN #51 (VeritaTrack task owner + owner-scoped reminders) and #52 (MD seat via account-grant dropdown); fold internal non-conforming-event write-up into #36 as the awaited scope decision; regenerate PARKING_LOT.xlsx.
Self-check: docs + xlsx only, no code; #36 updated in place not duplicated; verbatim wording preserved.
</commit_message>
<xml_diff>
--- a/PARKING_LOT.xlsx
+++ b/PARKING_LOT.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RETIRED" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$47</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RETIRED'!$A$1:$H$7</definedName>
   </definedNames>
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -933,7 +933,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Parked 2026-05-26 with a one-line scope intent. Michael indicated he will walk through the requirements in more detail in a follow-up conversation. Do not start building until that walkthrough happ...</t>
+          <t>Scoped, not started (updated 2026-09-28). Now lands in VeritaResponse per Michael's direction above; the earlier "new standalone module" framing is superseded. Do not start building until Michael g...</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -1207,8 +1207,94 @@
       </c>
       <c r="H16" s="2" t="inlineStr"/>
     </row>
+    <row r="17" ht="90" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>VeritaTrack task owner + owner-scoped reminder routing</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Open, not started. Placeholder pending build. Open questions: is the owner a staff_employee or a seat user, and how are reminder recipients currently chosen.</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>S-M (1-3 days to ~1.5 weeks) — add an owner on a VeritaTrack task, selectable...</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Medium — cuts reminder-email noise so people only get the tasks that are thei...</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Michael, verbatim (2026-09-28): "In veritatask, we should be able to assign an owner from staff that are built, then in the reminder section, we should be able to designate reminder emails only to the owner. The hem person does not need the chemistry reminders, etc." Module note: there is no VeritaTask module in the codebase; the task/reminder surface is VeritaTrack (client/src/pages/VeritaTrackAppPage.tsx), so this lands there. Today VeritaTrack tasks are not owned by a specific staff member and reminder emails are not recipient-scoped to an owner. The build adds (a) an owner selector on each task drawn from the lab's VeritaStaff roster, and (b) a reminder setting that routes the reminder email to only that owner. Confirm the current reminder recipient model before sizing.</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-28 session, Michael "for later (placeholder)" optimization #1 (relaying from the Lab Members / VeritaAssure screens).</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>Post-COLA. No customer urgency.
+---</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="90" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Medical Director seat via account-grant dropdown (designate / transfer MD)</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Open, not started. Placeholder. Confirm the current MD-seat assignment path and the one-MD-per-location enforcement point before sizing.</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>S-M (1-3 days to ~1.5 weeks) — move MD-seat assignment onto the same per-memb...</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Medium-High — the MD seat is a recurring friction point (Georgetown, SCAHC MD...</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Michael, verbatim (2026-09-28): "The way we are doing the medical director seat is silly. Why not just use the account grant dropdown to give a medical director seat. If the person is already in, then we should just be able to grant the medical director seat the same way we promote people to admin or reduce them to staff as long as we only have 1 per location. Maybe do another block like the transfer ownership block as 'designate medical director or transfer medical director'." So: fold the MD seat into the existing member role dropdown (Admin / Staff / ... + Medical Director) with a single-MD-per-lab constraint, and add a dedicated designate-or-transfer-MD block that mirrors the transfer-ownership UX for changing the MD. Cross-ref [[project_medical_director_designation]] and the seat model.</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28 session, Michael "for later (placeholder)" optimization #3 (relaying from the Lab Members screen).</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Post-COLA. No customer urgency.
+---</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H16"/>
+  <autoFilter ref="A1:H18"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
docs(parking-lot): close #18 (shipped), reclassify #17 to CLOSED (VeritaResponse live)
TASK: Per Michael, remove two shipped items mis-filed in OPEN so the list reflects reality.
PLAN: Move #18 (AAA coverage, all phases shipped) to CLOSED as C47; reclassify #17 (VeritaResponse, built and live) to CLOSED as C48 with the customer-triggered residual (renderer audit + Tier 3) noted; leave standard pointer lines in OPEN; regenerate PARKING_LOT.xlsx.
Self-check:
  - Docs + regenerated xlsx only, no code.
  - xlsx now reports OPEN 15 / CLOSED 48 / RETIRED 6 (was 17/46/6).
  - Full original scoping for both items preserved in git history; closure evidence retained in C47/C48.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PARKING_LOT.xlsx
+++ b/PARKING_LOT.xlsx
@@ -12,8 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RETIRED" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$18</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$47</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$49</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RETIRED'!$A$1:$H$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -564,6 +564,12 @@
         <is>
           <t>Pre-COLA. May 6-8 conference; Saturday + Sunday +
 Monday available before the booth.
+---
+_(item #17 reclassified to CLOSED 2026-09-28; VeritaResponse shipped and live, see C48 below)_
+---
+_(item #18 closed 2026-09-28; all phases shipped, see C47 below)_
+---
+_(item #22 closed 2026-05-28; see C26 below)_
 ---</t>
         </is>
       </c>
@@ -571,130 +577,30 @@
     <row r="3" ht="90" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>27</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>New flagship module: VeritaResponse (post-survey deficiency response)</t>
+          <t>Acquire CAP MOL (Molecular) checklist to verify 2 pending entries</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>BUILT and LIVE (this entry was stale). VeritaResponse shipped as a
-full module: findings table + CRUD + lifecycle, due-date computation, 30/60/90-day
-effectiveness monitoring (wave C3), cross-modu...</t>
+          <t>Open, blocks on operator obtaining the MOL checklist.</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>XL (6+ weeks; flagship-scale)</t>
+          <t>N/A (operator action — ~1 hour of code work once the file is in hand)</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>High — booth-validated demand at COLA Nashville; no existing module covers po...</t>
+          <t>Low — two entries total; low traffic; only matters when a customer cites a MO...</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>A new module that helps a lab manage the full lifecycle of
-responding to inspection deficiencies (CAP, TJC, COLA, CMS-2567,
-AABB), from intake of a citation through corrective-action authoring,
-supporting-evidence collection, submission tracking, and 30/60/90-day
-effectiveness verification. Pairs with VeritaCheck (find gaps before
-they cite you) and VeritaPT (prove your PT covers your menu) to
-complete the compliance lifecycle: prevent → respond → prove.</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-07 conference user request, COLA Nashville. User
-asked for thoughts and recommendations on adding a deficiency-response
-module. Online research conducted same session covering CAP, TJC,
-COLA, CMS-2567, AABB. URLs cited above.</t>
-        </is>
-      </c>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>Post-COLA. Build is multi-week regardless;
-zero rationale for any code change before the conference ends.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="90" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>18</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Unregulated analyte / Alternative Assessment (AAA) coverage — cross-module gap</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>PARTIAL as of 2026-05-10.
-- Phase 1 (VeritaScan AAA sub-block, items 169-173) CLOSED via
- PR #78 (client/src/lib/veritaScanData.ts). Item #46 retained as
- AAA gateway; new 5-item block uses ids 16...</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>S (1-3 days once #17 ships) for Phase 3 — Phases 1 and 2 already shipped.</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Medium — closes a real workflow loop (AAA failure → VeritaResponse finding) b...</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>Effort: S (1-3 days once #17 ships) for Phase 3 — Phases 1 and 2 already shipped.
-Importance: Medium — closes a real workflow loop (AAA failure → VeritaResponse finding) but only matters once #17 exists.</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>Post-COLA. Phase 1 and Phase 2 data layer
-shipped 2026-05-10.
----
-_(item #22 closed 2026-05-28; see C26 below)_
----</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="90" customHeight="1">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>27</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Acquire CAP MOL (Molecular) checklist to verify 2 pending entries</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>Open, blocks on operator obtaining the MOL checklist.</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>N/A (operator action — ~1 hour of code work once the file is in hand)</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>Low — two entries total; low traffic; only matters when a customer cites a MO...</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>PR #108 left 2 entries in server/capRequirements.ts
 flagged as unverified because the operator does not hold the CAP MOL
@@ -708,48 +614,48 @@
 The MOL module's MAS xlsx is the only one missing from that set.</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>PR #108 commit 92f9573 (closed via merge 2026-05-11),
 audit findings.</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>Post-COLA. Two entries; low traffic.
 ---</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="90" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
+    <row r="4" ht="90" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>28</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Acquire AABB Standards 35th edition + current COLA Accreditation Manual for exhaustive citation verification</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>Open, blocks on operator obtaining the gated accreditor
 manuals. Until then, AABB / COLA citations are best-effort against
 the public-source compilations.</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>N/A (operator action — ~1-2 days of audit re-run once the manuals are held)</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>High — gates #5 from reaching "exhaustively verified" status for AABB and COLA.</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>The 2026-05-11 QC audit found that VeritaScan, cfrRequirements
 cross-refs, and colaRequirements.ts cite about 180 AABB and COLA codes
@@ -769,14 +675,14 @@
  does not enumerate fully.</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>2026-05-11 QC/QA audit, documented in
 OneDrive\Lab\Regulatory\aaa Truth Master Document\PROVENANCE.md
 "Audit-coverage limits" section.</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>Post-COLA. Operator-side action item, no code
 work pending until the source documents land.
@@ -784,34 +690,34 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="90" customHeight="1">
-      <c r="A7" s="3" t="inlineStr">
+    <row r="5" ht="90" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>VeritaStock barcode scanning (full mobile scan flow)</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>Parked pending first paid commitment.
 ---</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>L (12 working days, ~3 weeks calendar)</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>High — strategic moat vs Unity Lab Services ($30K+/yr); presold as included o...</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>The remaining barcode-scanning build for VeritaStock, scoped
 during the 2026-05-20 Pfizer follow-up discussion. Order-now reorder
@@ -820,7 +726,7 @@
 Services-class inventory product.</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>2026-05-20 Pfizer follow-up session, after the order-now
 reorder document shipped (PR #286). Strategic decision documented in
@@ -831,31 +737,31 @@
 barcode scanning waits on revenue...</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr"/>
-    </row>
-    <row r="8" ht="90" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr"/>
+    </row>
+    <row r="6" ht="90" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Plain-language summary layer for verbatim CFR citations</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr"/>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr"/>
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>M (multi-day content authoring across 96 Master List rows if redesigned corre...</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>Medium — director readability win; no customer urgency.</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>server/cfrRequirements.ts carries verbatim eCFR text in
 the description field (PR #301 closed #26). The verbatim text is
@@ -864,8 +770,8 @@
 director read faster.</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr"/>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>Post-COLA. No customer urgency. Operator
 has not yet authorized a redesign attempt as of 2026-05-21.
@@ -873,29 +779,29 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="90" customHeight="1">
-      <c r="A9" s="3" t="inlineStr">
+    <row r="7" ht="90" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Lab leader community / forum (paid subscription idea)</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr"/>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr"/>
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>XL (ongoing operational commitment, not a build) as paid; S (a few days to sp...</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>Low as paid product (SWOT verdict: don't build); Medium as free lead-funnel a...</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>Operator-floated 2026-05-22: a vetted online forum for
 laboratory leaders (directors, managers, supervisors). Pricing as
@@ -908,8 +814,8 @@
 lab-leader water cooler.</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr"/>
-      <c r="H9" s="3" t="inlineStr">
+      <c r="G7" s="3" t="inlineStr"/>
+      <c r="H7" s="3" t="inlineStr">
         <is>
           <t>Post-COLA. No customer urgency.
 ---
@@ -920,39 +826,39 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="90" customHeight="1">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="8" ht="90" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>36</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>New module: laboratory non-conforming event documentation</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Scoped, not started (updated 2026-09-28). Now lands in VeritaResponse per Michael's direction above; the earlier "new standalone module" framing is superseded. Do not start building until Michael g...</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>L (initial estimate, pending Michael's scope walkthrough — likely new DB tabl...</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>High — every accredited laboratory (TJC, CAP, COLA, AABB) has to document non...</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>Build a module to document laboratory non-conforming events (NCEs). Surfaces a lab needs to capture include specimen rejection, temperature excursions, reagent issues, equipment failures, result-reporting errors, transcription errors, lost specimens, contamination events, and similar quality incidents. Full scope, target accreditor mapping, terminology preference (NCE / NCR / event / incident / occurrence), and how it should relate to the existing VeritaQC corrective-action engine and VeritaResponse deficiency tracker are TBD pending Michael's scope walkthrough.</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr"/>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>Post-COLA. No customer urgency yet, but high strategic value once defined — closes a real gap every lab has and that no other Verita module currently serves.
 ---
@@ -961,76 +867,76 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="90" customHeight="1">
-      <c r="A11" s="3" t="inlineStr">
+    <row r="9" ht="90" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>38</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>Screen-capture video: VeritaCheck method comparison in 60 seconds</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>Open. Re-parked 2026-05-27 (originally PR #117, abandoned with merge conflicts then closed-and-re-authored at current numbering). Pending operator decision on whether to record this themselves or p...</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>S for agent prep (storyboard / pre-fill / captions / checklist); ~1 hour of o...</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t>Medium — operator selected this as the highest-impact positioning artifact du...</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="F9" s="3" t="inlineStr">
         <is>
           <t>30-60 second screen recording demonstrating the "experienced lab tech figures it out in seconds" claim. From blank method-comparison study to completed PDF, no voiceover, no narration, visible cursor motion. Embed autoplay-muted on the marketing site, include in conference follow-up emails.</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="G9" s="3" t="inlineStr">
         <is>
           <t>2026-05-12 conversation. Michael selected the screen-cap video as the highest-impact positioning artifact, then asked the agent to record it. Agent does not have screen-recording capability; option parked rather than fudged.</t>
         </is>
       </c>
-      <c r="H11" s="3" t="inlineStr">
+      <c r="H9" s="3" t="inlineStr">
         <is>
           <t>Post-COLA, conference-driven.
 ---</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="90" customHeight="1">
-      <c r="A12" s="2" t="inlineStr">
+    <row r="10" ht="90" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>39</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>MediaLab parity hardening (VeritaPolicy approval workflow depth)</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Open, customer-triggered. No urgency until a prospect specifically asks for one of the listed depth items.</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>L (1-2 weeks for the high-value items; each independent feature is M)</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>Medium-High — the C29 build shipped the surface MediaLab markets but depth is...</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>The VeritaPolicy approval workflow build (C29, 2026-05-29) hit roughly 60-70% MediaLab feature surface. The following gaps remain when comparing against an enterprise MediaLab Document Control deployment:
 - Quizzes on attestations. Schema columns quiz_score and quiz_total_questions exist on policy_attestations but the quiz authoring + presentation UI was scoped out of Phase 4. MediaLab labs use 5-10 multiple-choice questions per policy to confirm comprehension, not just attestation. Adds compliance defensibility.
@@ -1040,54 +946,133 @@
 - In-browser DOCX editing. MediaLab has a structured editor that creates a Table of Contents from headings. We treat documents as...</t>
         </is>
       </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-29 QA pass after C29 shipped (qa-policy-build.js + qa-policy-ui.js: 54/54 happy path verified). Honest depth assessment surfaced by Michael's "how confident are you" question — see C29 entry for full QA receipts.</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Post-COLA. Defensive against MediaLab in head-to-head sales calls.
+---</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="90" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>VeritaQC Import Phase A: human-in-the-loop Gate 3 click-through (deferred)</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Open, awaiting Michael's 5-minute click test. Will move task #77 to completed only after he reports the user-visible result.
+---</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>XS (~5 minutes of Michael's time on a live URL).</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Low. Backend contract is fully verified via 35/35 passing offline contract ch...</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Effort: XS (~5 minutes of Michael's time on a live URL).
+Importance: Low. Backend contract is fully verified via 35/35 passing offline contract checks (scripts/verify-veritaqc-import.js) plus three live-API smoke checks against prod (candidates, preview, mappings PUT/GET) on Riverside Regional with seed lot SEED-1780436709094 (18 Glucose results). The browser-driven click was not run because Claude-in-Chrome's renderer froze repeatedly on the Radix Select inside VeritaCheckPage, not on Phase A code itself. Risk of a UX bug surviving to a customer is small but not zero.</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>task #77 stalled at Gate 3 step 8 on 2026-06-02. PR #500 squash-merged at commit 17a91ff, prod /api/health confirmed ACTIVE on that commit at 20:43 UTC.</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12" ht="90" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Outbound demo-invite messaging campaign to 1st-degree LinkedIn contacts</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Parked. Plan documented. Implementation deferred until trigger conditions met.
+---</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>L (1 week prep + 4-6 weeks of staged sends)</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>High. Converts existing warm network (~2,500 1st-degree contacts and growing...</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>A staged outbound DM campaign walking Michael's 1st-degree LinkedIn contacts through tier-segmented demo invitations for VeritaAssure. Goal: convert warmest contacts into demo conversations first, then chain into trials and paid subscriptions. Separate pipeline from COLA cohort follow-up and from content-driven inbound; all three feed the same demo funnel but originate from different warmth sources.</t>
+        </is>
+      </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29 QA pass after C29 shipped (qa-policy-build.js + qa-policy-ui.js: 54/54 happy path verified). Honest depth assessment surfaced by Michael's "how confident are you" question — see C29 entry for full QA receipts.</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>Post-COLA. Defensive against MediaLab in head-to-head sales calls.
----</t>
-        </is>
-      </c>
+          <t>2026-06-04 session, after weekly LinkedIn invite batch completion (80 sent, cap hit at #84 Victoria Allen).</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr"/>
     </row>
     <row r="13" ht="90" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>47</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>VeritaQC Import Phase A: human-in-the-loop Gate 3 click-through (deferred)</t>
+          <t>Hide sections a lab does not use from a master list, to reduce clutter (prospect-requested)</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Open, awaiting Michael's 5-minute click test. Will move task #77 to completed only after he reports the user-visible result.
+          <t>Open. Not started. Needs a one-line scope confirmation (which master list).
 ---</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>XS (~5 minutes of Michael's time on a live URL).</t>
+          <t>S-M (a few days to ~2 weeks depending on scope) — a lab-level visibility togg...</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>Low. Backend contract is fully verified via 35/35 passing offline contract ch...</t>
+          <t>Medium-High — came straight from a live prospect today as an onboarding-frict...</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Effort: XS (~5 minutes of Michael's time on a live URL).
-Importance: Low. Backend contract is fully verified via 35/35 passing offline contract checks (scripts/verify-veritaqc-import.js) plus three live-API smoke checks against prod (candidates, preview, mappings PUT/GET) on Riverside Regional with seed lot SEED-1780436709094 (18 Glucose results). The browser-driven click was not run because Claude-in-Chrome's renderer froze repeatedly on the Radix Select inside VeritaCheckPage, not on Phase A code itself. Risk of a UX bug surviving to a customer is small but not zero.</t>
+          <t>Effort: S-M (a few days to ~2 weeks depending on scope) — a lab-level visibility toggle that hides not-applicable or unused sections from a master-list view. Smaller if it is a "hide N/A" filter on the existing VeritaDC master list, larger if it also spans VeritaScan domains.
+Importance: Medium-High — came straight from a live prospect today as an onboarding-friction point; a lab that does not run a service line should not have to wade past its requirements.</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>task #77 stalled at Gate 3 step 8 on 2026-06-02. PR #500 squash-merged at commit 17a91ff, prod /api/health confirmed ACTIVE on that commit at 20:43 UTC.</t>
+          <t>2026-09-23 session, Michael relaying a prospect ask from a demo today.</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr"/>
@@ -1095,38 +1080,35 @@
     <row r="14" ht="90" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>50</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Outbound demo-invite messaging campaign to 1st-degree LinkedIn contacts</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>Parked. Plan documented. Implementation deferred until trigger conditions met.
----</t>
-        </is>
-      </c>
+          <t>Competency "assessed this cycle" uses a flat 365-day window</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr"/>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>L (1 week prep + 4-6 weeks of staged sends)</t>
+          <t>S-M - anchor the coverage-map "assessed this cycle" to the person's actual CL...</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>High. Converts existing warm network (~2,500 1st-degree contacts and growing...</t>
+          <t>Medium - in an employee's first year the semiannual windows differ from a fla...</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>A staged outbound DM campaign walking Michael's 1st-degree LinkedIn contacts through tier-segmented demo invitations for VeritaAssure. Goal: convert warmest contacts into demo conversations first, then chain into trials and paid subscriptions. Separate pipeline from COLA cohort follow-up and from content-driven inbound; all three feed the same demo funnel but originate from different warmth sources.</t>
+          <t>Effort: S-M - anchor the coverage-map "assessed this cycle" to the person's actual CLIA cadence (semiannual in year 1 per 42 CFR 493.1451(b)(8), annual thereafter) from staff_competency_schedules, instead of the v1 flat 365-day lookback.
+Importance: Medium - in an employee's first year the semiannual windows differ from a flat annual window, so a first-year assessment could read as current slightly longer or shorter than the true cadence. Fine for the common annual case; refine for year-1 accuracy.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04 session, after weekly LinkedIn invite batch completion (80 sent, cap hit at #84 Victoria Allen).</t>
+          <t>2026-09-24 session, VeritaComp coverage map (#48 Phase 3) v1 simplification, noted in PR #1319.
+---</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr"/>
@@ -1134,167 +1116,91 @@
     <row r="15" ht="90" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>51</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Hide sections a lab does not use from a master list, to reduce clutter (prospect-requested)</t>
+          <t>VeritaTrack task owner + owner-scoped reminder routing</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Open. Not started. Needs a one-line scope confirmation (which master list).
----</t>
+          <t>Open, not started. Placeholder pending build. Open questions: is the owner a staff_employee or a seat user, and how are reminder recipients currently chosen.</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>S-M (a few days to ~2 weeks depending on scope) — a lab-level visibility togg...</t>
+          <t>S-M (1-3 days to ~1.5 weeks) — add an owner on a VeritaTrack task, selectable...</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>Medium-High — came straight from a live prospect today as an onboarding-frict...</t>
+          <t>Medium — cuts reminder-email noise so people only get the tasks that are thei...</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>Effort: S-M (a few days to ~2 weeks depending on scope) — a lab-level visibility toggle that hides not-applicable or unused sections from a master-list view. Smaller if it is a "hide N/A" filter on the existing VeritaDC master list, larger if it also spans VeritaScan domains.
-Importance: Medium-High — came straight from a live prospect today as an onboarding-friction point; a lab that does not run a service line should not have to wade past its requirements.</t>
+          <t>Michael, verbatim (2026-09-28): "In veritatask, we should be able to assign an owner from staff that are built, then in the reminder section, we should be able to designate reminder emails only to the owner. The hem person does not need the chemistry reminders, etc." Module note: there is no VeritaTask module in the codebase; the task/reminder surface is VeritaTrack (client/src/pages/VeritaTrackAppPage.tsx), so this lands there. Today VeritaTrack tasks are not owned by a specific staff member and reminder emails are not recipient-scoped to an owner. The build adds (a) an owner selector on each task drawn from the lab's VeritaStaff roster, and (b) a reminder setting that routes the reminder email to only that owner. Confirm the current reminder recipient model before sizing.</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>2026-09-23 session, Michael relaying a prospect ask from a demo today.</t>
-        </is>
-      </c>
-      <c r="H15" s="3" t="inlineStr"/>
+          <t>2026-09-28 session, Michael "for later (placeholder)" optimization #1 (relaying from the Lab Members / VeritaAssure screens).</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>Post-COLA. No customer urgency.
+---</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="90" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>52</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Competency "assessed this cycle" uses a flat 365-day window</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr"/>
+          <t>Medical Director seat via account-grant dropdown (designate / transfer MD)</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Open, not started. Placeholder. Confirm the current MD-seat assignment path and the one-MD-per-location enforcement point before sizing.</t>
+        </is>
+      </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>S-M - anchor the coverage-map "assessed this cycle" to the person's actual CL...</t>
+          <t>S-M (1-3 days to ~1.5 weeks) — move MD-seat assignment onto the same per-memb...</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Medium - in an employee's first year the semiannual windows differ from a fla...</t>
+          <t>Medium-High — the MD seat is a recurring friction point (Georgetown, SCAHC MD...</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Effort: S-M - anchor the coverage-map "assessed this cycle" to the person's actual CLIA cadence (semiannual in year 1 per 42 CFR 493.1451(b)(8), annual thereafter) from staff_competency_schedules, instead of the v1 flat 365-day lookback.
-Importance: Medium - in an employee's first year the semiannual windows differ from a flat annual window, so a first-year assessment could read as current slightly longer or shorter than the true cadence. Fine for the common annual case; refine for year-1 accuracy.</t>
+          <t>Michael, verbatim (2026-09-28): "The way we are doing the medical director seat is silly. Why not just use the account grant dropdown to give a medical director seat. If the person is already in, then we should just be able to grant the medical director seat the same way we promote people to admin or reduce them to staff as long as we only have 1 per location. Maybe do another block like the transfer ownership block as 'designate medical director or transfer medical director'." So: fold the MD seat into the existing member role dropdown (Admin / Staff / ... + Medical Director) with a single-MD-per-lab constraint, and add a dedicated designate-or-transfer-MD block that mirrors the transfer-ownership UX for changing the MD. Cross-ref [[project_medical_director_designation]] and the seat model.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 session, VeritaComp coverage map (#48 Phase 3) v1 simplification, noted in PR #1319.
----</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr"/>
-    </row>
-    <row r="17" ht="90" customHeight="1">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>51</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>VeritaTrack task owner + owner-scoped reminder routing</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>Open, not started. Placeholder pending build. Open questions: is the owner a staff_employee or a seat user, and how are reminder recipients currently chosen.</t>
-        </is>
-      </c>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>S-M (1-3 days to ~1.5 weeks) — add an owner on a VeritaTrack task, selectable...</t>
-        </is>
-      </c>
-      <c r="E17" s="3" t="inlineStr">
-        <is>
-          <t>Medium — cuts reminder-email noise so people only get the tasks that are thei...</t>
-        </is>
-      </c>
-      <c r="F17" s="3" t="inlineStr">
-        <is>
-          <t>Michael, verbatim (2026-09-28): "In veritatask, we should be able to assign an owner from staff that are built, then in the reminder section, we should be able to designate reminder emails only to the owner. The hem person does not need the chemistry reminders, etc." Module note: there is no VeritaTask module in the codebase; the task/reminder surface is VeritaTrack (client/src/pages/VeritaTrackAppPage.tsx), so this lands there. Today VeritaTrack tasks are not owned by a specific staff member and reminder emails are not recipient-scoped to an owner. The build adds (a) an owner selector on each task drawn from the lab's VeritaStaff roster, and (b) a reminder setting that routes the reminder email to only that owner. Confirm the current reminder recipient model before sizing.</t>
-        </is>
-      </c>
-      <c r="G17" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-28 session, Michael "for later (placeholder)" optimization #1 (relaying from the Lab Members / VeritaAssure screens).</t>
-        </is>
-      </c>
-      <c r="H17" s="3" t="inlineStr">
+          <t>2026-09-28 session, Michael "for later (placeholder)" optimization #3 (relaying from the Lab Members screen).</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
         <is>
           <t>Post-COLA. No customer urgency.
 ---</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="90" customHeight="1">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>52</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Medical Director seat via account-grant dropdown (designate / transfer MD)</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>Open, not started. Placeholder. Confirm the current MD-seat assignment path and the one-MD-per-location enforcement point before sizing.</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>S-M (1-3 days to ~1.5 weeks) — move MD-seat assignment onto the same per-memb...</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>Medium-High — the MD seat is a recurring friction point (Georgetown, SCAHC MD...</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>Michael, verbatim (2026-09-28): "The way we are doing the medical director seat is silly. Why not just use the account grant dropdown to give a medical director seat. If the person is already in, then we should just be able to grant the medical director seat the same way we promote people to admin or reduce them to staff as long as we only have 1 per location. Maybe do another block like the transfer ownership block as 'designate medical director or transfer medical director'." So: fold the MD seat into the existing member role dropdown (Admin / Staff / ... + Medical Director) with a single-MD-per-lab constraint, and add a dedicated designate-or-transfer-MD block that mirrors the transfer-ownership UX for changing the MD. Cross-ref [[project_medical_director_designation]] and the seat model.</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 session, Michael "for later (placeholder)" optimization #3 (relaying from the Lab Members screen).</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="inlineStr">
-        <is>
-          <t>Post-COLA. No customer urgency.
----</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:H18"/>
+  <autoFilter ref="A1:H16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1305,7 +1211,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H47"/>
+  <dimension ref="A1:H49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1363,66 +1269,64 @@
     <row r="2" ht="90" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>C45</t>
+          <t>C47</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Unify coverage/competency recurrence helper (was #49) - closed as non-issue</t>
+          <t>Unregulated-analyte / Alternative Assessment (AAA) coverage (was #18)</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr"/>
-      <c r="D2" s="2" t="inlineStr"/>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>was S (Phase 3) / Importance: Medium</t>
+        </is>
+      </c>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: Investigated 2026-09-24 before building. The coverage recurrence math (+6-month interval, signed-resets-to-missing, nextDueOn/overdue, isFailVerdict) is ALREADY single-source in server/veritacheckCoverage.ts (computeCoverageFrom). server/coverageReport.ts and the routes.ts coverage export do not recompute it; they consume the computed nextDueOn/overdue/status fields and apply small surface-specific presentation labels (deliberately different vocabularies per surface, so they should not be merged). The only truly identical duplicate is a one-line date formatter. The competency "owed" derivation is NOT the same cadence: competency follows the CLIA milestone schedule (initial / semiannual year 1 / annual, 42 CFR 493.1451(b)(8) and 493.1235), which is a different regulatory interval from the coverage 6-month rule (493.1281 / 493.1255) and must stay separate. No worthwhile extraction; merging the two cadences would be wrong. Closed 2026-09-24. (The year-1 competency-window refinement remains tracked separately as #50.)</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-24 session, "keep working" pass; scoped read-only, found no real duplication.
----</t>
-        </is>
-      </c>
+          <t>Effort: was S (Phase 3) / Importance: Medium</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr"/>
       <c r="H2" s="2" t="inlineStr"/>
     </row>
     <row r="3" ht="90" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>C46</t>
+          <t>C48</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Verified-users product-update send path (wrong-list incident fix)</t>
+          <t>VeritaResponse post-survey deficiency module (was #17)</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr"/>
-      <c r="D3" s="3" t="inlineStr"/>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>was XL / Importance: High</t>
+        </is>
+      </c>
       <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: Shipped PR #1324 (merged 4e05506a, deploy ACTIVE). New POST /api/admin/users/send targets registered VeritaAssure account holders (the users table), never the Lab Director's Briefing subscriber list. Separate explicitly-named endpoint (not a flag with a dangerous default), account-holder email framing, excludes suppressed emails and RFC-reserved test domains, CC owner, dryRun + testTo previews. Public unsubscribe now upserts a suppression row so opt-outs are honored across both audiences. Live dryRun: 49 verified-user recipients vs 673 on the Briefing list. Receipts: scripts/verify-product-update-send.mts 24/24, tsc clean, rendered sample inspected. Fixes the fallout from the 2026-09-23/24 wrong-list send (a product update went to the 675-person Briefing list). Nothing sends without Michael's explicit "send it."</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-24 session; Michael selected this as the next build after the #41 close.
----</t>
-        </is>
-      </c>
+          <t>Effort: was XL / Importance: High</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr"/>
       <c r="H3" s="3" t="inlineStr"/>
     </row>
     <row r="4" ht="90" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>C44</t>
+          <t>C45</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Verify-script convention backfill (was #41) + audit matcher fix</t>
+          <t>Unify coverage/competency recurrence helper (was #49) - closed as non-issue</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr"/>
@@ -1430,12 +1334,12 @@
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: #41 was fully backfilled on 2026-06-13 (all 8 high-stakes scripts landed; see C30); it had only been mis-filed in OPEN. A 2026-09-24 re-audit initially reported 4 of 5 recent math/logic commits as missing a verify script, which was a FALSE POSITIVE: scripts/audit_verify_script_coverage.py matched only scripts/verify-*.js / .cjs, so it ignored the .mjs / .mts / .ts verify scripts the repo now ships (e.g. verify-ptcoag-multi.mts, verify-tea-criterion-format.mjs). Fixed the matcher to accept .js/.cjs/.mjs/.ts/.mts; re-run shows 5 of 5 covered, 0 debt. The convention is being followed. Closed 2026-09-24.</t>
+          <t>Closure evidence: Investigated 2026-09-24 before building. The coverage recurrence math (+6-month interval, signed-resets-to-missing, nextDueOn/overdue, isFailVerdict) is ALREADY single-source in server/veritacheckCoverage.ts (computeCoverageFrom). server/coverageReport.ts and the routes.ts coverage export do not recompute it; they consume the computed nextDueOn/overdue/status fields and apply small surface-specific presentation labels (deliberately different vocabularies per surface, so they should not be merged). The only truly identical duplicate is a one-line date formatter. The competency "owed" derivation is NOT the same cadence: competency follows the CLIA milestone schedule (initial / semiannual year 1 / annual, 42 CFR 493.1451(b)(8) and 493.1235), which is a different regulatory interval from the coverage 6-month rule (493.1281 / 493.1255) and must stay separate. No worthwhile extraction; merging the two cadences would be wrong. Closed 2026-09-24. (The year-1 competency-window refinement remains tracked separately as #50.)</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 session, "keep working" pass; audit tooling bug found + fixed.
+          <t>2026-09-24 session, "keep working" pass; scoped read-only, found no real duplication.
 ---</t>
         </is>
       </c>
@@ -1444,12 +1348,12 @@
     <row r="5" ht="90" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>C43</t>
+          <t>C46</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>VeritaStaff instrument-centric (dual) assignment view</t>
+          <t>Verified-users product-update send path (wrong-list incident fix)</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr"/>
@@ -1457,12 +1361,12 @@
       <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1320. GET/PUT /staff/instruments/:id/employees (transpose of the per-employee endpoints); an "Assign by Instrument" dialog lets a director pick a test system or manual test and check off who runs it. Same staff_employee_instruments join, with the 42 CFR 493.1235(a) duty-change event emitted on newly-added pairs so both orientations trigger the same reassessment. GET verified live on SCAHC lab 2. Closed 2026-09-24.</t>
+          <t>Closure evidence: Shipped PR #1324 (merged 4e05506a, deploy ACTIVE). New POST /api/admin/users/send targets registered VeritaAssure account holders (the users table), never the Lab Director's Briefing subscriber list. Separate explicitly-named endpoint (not a flag with a dangerous default), account-holder email framing, excludes suppressed emails and RFC-reserved test domains, CC owner, dryRun + testTo previews. Public unsubscribe now upserts a suppression row so opt-outs are honored across both audiences. Live dryRun: 49 verified-user recipients vs 673 on the Briefing list. Receipts: scripts/verify-product-update-send.mts 24/24, tsc clean, rendered sample inspected. Fixes the fallout from the 2026-09-23/24 wrong-list send (a product update went to the 675-person Briefing list). Nothing sends without Michael's explicit "send it."</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>2026-09-24 session, Michael ("in staff we should also give the dual view when assigning coverage to test systems or manual tests").
+          <t>2026-09-24 session; Michael selected this as the next build after the #41 close.
 ---</t>
         </is>
       </c>
@@ -1471,12 +1375,12 @@
     <row r="6" ht="90" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>C42</t>
+          <t>C44</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>VeritaComp coverage map (required-vs-assessed matrix, dual view)</t>
+          <t>Verify-script convention backfill (was #41) + audit matcher fix</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr"/>
@@ -1484,12 +1388,12 @@
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1319 (+ status layer PR #1316). /competency/owed returns per-item assessed (locked passing assessment this cycle on a covering method group) + per-employee CLIA status; CompetencyCoverageMap renders a By-employee / By-instrument matrix (Assessed / Owed / Overdue / Gap). Verified live on SCAHC lab 2 (owed 116, assessed 2, gaps 0). Completes #48 as the VeritaCheck-parity coverage map. Closed 2026-09-24.</t>
+          <t>Closure evidence: #41 was fully backfilled on 2026-06-13 (all 8 high-stakes scripts landed; see C30); it had only been mis-filed in OPEN. A 2026-09-24 re-audit initially reported 4 of 5 recent math/logic commits as missing a verify script, which was a FALSE POSITIVE: scripts/audit_verify_script_coverage.py matched only scripts/verify-*.js / .cjs, so it ignored the .mjs / .mts / .ts verify scripts the repo now ships (e.g. verify-ptcoag-multi.mts, verify-tea-criterion-format.mjs). Fixed the matcher to accept .js/.cjs/.mjs/.ts/.mts; re-run shows 5 of 5 covered, 0 debt. The convention is being followed. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 session, Michael ("are we building the competencies to have a coverage map, same as veritacheck?" then "build it").
+          <t>2026-09-24 session, "keep working" pass; audit tooling bug found + fixed.
 ---</t>
         </is>
       </c>
@@ -1498,12 +1402,12 @@
     <row r="7" ht="90" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>C41</t>
+          <t>C43</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>VeritaCheck coverage recurrence (method comparison + cal-ver/linearity + reports)</t>
+          <t>VeritaStaff instrument-centric (dual) assignment view</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr"/>
@@ -1511,12 +1415,12 @@
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: PRs #1317 (method comparison), #1318 (cal-ver/linearity), #1321 (report Next-due columns). Periodic verification (correlation/method comparison 42 CFR 493.1281; cal-ver/linearity 42 CFR 493.1255; both 6-month) now recurs: a signed study banks the cycle and rolls to next-due = signed + 6 months instead of reading "done" forever. Status Missing/Failed/Completed-unsigned + a "Next due on" column on-screen and in both coverage exports; also credits the previously-ignored "correlation" study type. Root cause: computeCoverageFrom marked requirements done on mere existence, no date logic. Verified live on SCAHC lab 2 (101 correlations + 11 cal-ver rows now carry a next-due). Engine-level, all facilities. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1320. GET/PUT /staff/instruments/:id/employees (transpose of the per-employee endpoints); an "Assign by Instrument" dialog lets a director pick a test system or manual test and check off who runs it. Same staff_employee_instruments join, with the 42 CFR 493.1235(a) duty-change event emitted on newly-added pairs so both orientations trigger the same reassessment. GET verified live on SCAHC lab 2. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>2026-09-24 session, Michael ("Look at San Carlos... they finished their last set of correlations (all 103) but their menu never reset").
+          <t>2026-09-24 session, Michael ("in staff we should also give the dual view when assigning coverage to test systems or manual tests").
 ---</t>
         </is>
       </c>
@@ -1525,12 +1429,12 @@
     <row r="8" ht="90" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>C40</t>
+          <t>C42</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>VeritaComp Competencies Owed derived from VeritaStaff, with gap detection (was #48)</t>
+          <t>VeritaComp coverage map (required-vs-assessed matrix, dual view)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr"/>
@@ -1538,12 +1442,12 @@
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1314 (squash 2bcb0db9). GET /api/labs/:labId/competency/owed derives each VeritaStaff testing employee's owed competencies from their assigned instruments (staff_employee_instruments -&gt; veritamap_instruments + tests), on the CLIA timeline, and flags instruments not covered by any competency program as gaps. CompetenciesOwedSection renders it on the VeritaComp landing page. Reuses the shipped bridge + suggested-method-groups match rules; no new tables. Verified live on prod with real assignment data: 2 instruments assigned to a demo staffer produced owed=2, gaps=2 (HIGH, Technical Supervisor), then reverted cleanly. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1319 (+ status layer PR #1316). /competency/owed returns per-item assessed (locked passing assessment this cycle on a covering method group) + per-employee CLIA status; CompetencyCoverageMap renders a By-employee / By-instrument matrix (Assessed / Owed / Overdue / Gap). Verified live on SCAHC lab 2 (owed 116, assessed 2, gaps 0). Completes #48 as the VeritaCheck-parity coverage map. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23/24 session, Michael ("veritacomp bases what competencies they owe (currently untrue, but needs to be true)"). Option 1 (unify roster on VeritaStaff, match instruments by id).
+          <t>2026-09-24 session, Michael ("are we building the competencies to have a coverage map, same as veritacheck?" then "build it").
 ---</t>
         </is>
       </c>
@@ -1552,12 +1456,12 @@
     <row r="9" ht="90" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>C39</t>
+          <t>C41</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>VeritaScan line items can attach or link evidence (was #46)</t>
+          <t>VeritaCheck coverage recurrence (method comparison + cal-ver/linearity + reports)</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr"/>
@@ -1565,12 +1469,12 @@
       <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1312 (squash a1dda93d). VeritaScan scan checklist items now show linked evidence as chips (open link, remove) plus a writer "Link evidence" affordance whose picker links an existing VeritaDC/Library document; a shortcut deep-links to the Library for new (governed) documents. Reuses the already-shipped lab_documents + document_checklist_links + coverage endpoints (URL-pointer only, no file storage, no new tables). Browser-verified live on prod (scan 23): the affordance renders and the picker opens. Closed 2026-09-24.</t>
+          <t>Closure evidence: PRs #1317 (method comparison), #1318 (cal-ver/linearity), #1321 (report Next-due columns). Periodic verification (correlation/method comparison 42 CFR 493.1281; cal-ver/linearity 42 CFR 493.1255; both 6-month) now recurs: a signed study banks the cycle and rolls to next-due = signed + 6 months instead of reading "done" forever. Status Missing/Failed/Completed-unsigned + a "Next due on" column on-screen and in both coverage exports; also credits the previously-ignored "correlation" study type. Root cause: computeCoverageFrom marked requirements done on mere existence, no date logic. Verified live on SCAHC lab 2 (101 correlations + 11 cal-ver rows now carry a next-due). Engine-level, all facilities. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>2026-09-23 session, Michael. Recurring request. Companion: cross-module evidence display on the VeritaDC policy shipped in PR #1313 (by-target cross-links surfaced in the policy View modal, browser-verified live).
+          <t>2026-09-24 session, Michael ("Look at San Carlos... they finished their last set of correlations (all 103) but their menu never reset").
 ---</t>
         </is>
       </c>
@@ -1579,12 +1483,12 @@
     <row r="10" ht="90" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>C38</t>
+          <t>C40</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>VeritaTrack calendar month cells expand to reveal hidden tasks (was #45)</t>
+          <t>VeritaComp Competencies Owed derived from VeritaStaff, with gap detection (was #48)</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr"/>
@@ -1592,12 +1496,12 @@
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: VeritaTrack CalendarView month cells with more than three tasks now expand in place (chevron, "+N more" toggling to "Show less", due dates), so no task is hidden with no path to it (client/src/pages/VeritaTrackAppPage.tsx CalendarView). Shipped 2026-09-23. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1314 (squash 2bcb0db9). GET /api/labs/:labId/competency/owed derives each VeritaStaff testing employee's owed competencies from their assigned instruments (staff_employee_instruments -&gt; veritamap_instruments + tests), on the CLIA timeline, and flags instruments not covered by any competency program as gaps. CompetenciesOwedSection renders it on the VeritaComp landing page. Reuses the shipped bridge + suggested-method-groups match rules; no new tables. Verified live on prod with real assignment data: 2 instruments assigned to a demo staffer produced owed=2, gaps=2 (HIGH, Technical Supervisor), then reverted cleanly. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23 session, Michael screenshot of the VeritaTrack calendar (lab 3, September cell).
+          <t>2026-09-23/24 session, Michael ("veritacomp bases what competencies they owe (currently untrue, but needs to be true)"). Option 1 (unify roster on VeritaStaff, match instruments by id).
 ---</t>
         </is>
       </c>
@@ -1606,12 +1510,12 @@
     <row r="11" ht="90" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>C37</t>
+          <t>C39</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Long Excel column headers no longer clip CFR citations (was #44)</t>
+          <t>VeritaScan line items can attach or link evidence (was #46)</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr"/>
@@ -1619,12 +1523,12 @@
       <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. The VeritaMap export derives the header row height from the longest wrapped header via headerRowHeight(headers, colWidths) (server/routes.ts:15935) instead of a fixed 20, so "Reference Range Attestation (42 CFR 493.1253)" and the other long headers print in full. No new code this session. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1312 (squash a1dda93d). VeritaScan scan checklist items now show linked evidence as chips (open link, remove) plus a writer "Link evidence" affordance whose picker links an existing VeritaDC/Library document; a shortcut deep-links to the Library for new (governed) documents. Reuses the already-shipped lab_documents + document_checklist_links + coverage endpoints (URL-pointer only, no file storage, no new tables). Browser-verified live on prod (scan 23): the affordance renders and the picker opens. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+          <t>2026-09-23 session, Michael. Recurring request. Companion: cross-module evidence display on the VeritaDC policy shipped in PR #1313 (by-target cross-links surfaced in the policy View modal, browser-verified live).
 ---</t>
         </is>
       </c>
@@ -1633,12 +1537,12 @@
     <row r="12" ht="90" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>C36</t>
+          <t>C38</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>License stamp no longer clobbers the §6 header/footer or names the wrong lab (was #43)</t>
+          <t>VeritaTrack calendar month cells expand to reveal hidden tasks (was #45)</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr"/>
@@ -1646,12 +1550,12 @@
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. setHeaderFooter (shared/licenseExceljs.ts:155-209) now preserves an existing §6 header and appends (not overwrites) the footer left section, and customer-facing exports name the scoped lab: the VeritaScan library export reads req.scope.lab.name / clia_number (server/routes.ts:16572-16573), not the licensee. No new code this session (avoided regressing the existing fix). Closed 2026-09-24.</t>
+          <t>Closure evidence: VeritaTrack CalendarView month cells with more than three tasks now expand in place (chevron, "+N more" toggling to "Show less", due dates), so no task is hidden with no path to it (client/src/pages/VeritaTrackAppPage.tsx CalendarView). Shipped 2026-09-23. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+          <t>2026-09-23 session, Michael screenshot of the VeritaTrack calendar (lab 3, September cell).
 ---</t>
         </is>
       </c>
@@ -1660,18 +1564,72 @@
     <row r="13" ht="90" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>C34</t>
+          <t>C37</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Wire the two static-audit guards into CI (was #43)</t>
+          <t>Long Excel column headers no longer clip CFR citations (was #44)</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr"/>
       <c r="D13" s="3" t="inlineStr"/>
       <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. The VeritaMap export derives the header row height from the longest wrapped header via headerRowHeight(headers, colWidths) (server/routes.ts:15935) instead of a fixed 20, so "Reference Range Attestation (42 CFR 493.1253)" and the other long headers print in full. No new code this session. Closed 2026-09-24.</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+---</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14" ht="90" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>C36</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>License stamp no longer clobbers the §6 header/footer or names the wrong lab (was #43)</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr"/>
+      <c r="D14" s="2" t="inlineStr"/>
+      <c r="E14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. setHeaderFooter (shared/licenseExceljs.ts:155-209) now preserves an existing §6 header and appends (not overwrites) the footer left section, and customer-facing exports name the scoped lab: the VeritaScan library export reads req.scope.lab.name / clia_number (server/routes.ts:16572-16573), not the licensee. No new code this session (avoided regressing the existing fix). Closed 2026-09-24.</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+---</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15" ht="90" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>C34</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Wire the two static-audit guards into CI (was #43)</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr"/>
+      <c r="D15" s="3" t="inlineStr"/>
+      <c r="E15" s="3" t="inlineStr"/>
+      <c r="F15" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: both guards wired into the Multi-Lab Mutations Audit CI
 workflow (.github/workflows/multilab-mutations-audit.yml) as steps:
@@ -1683,24 +1641,24 @@
 (same caveat as the existing guards already in that workflow).</t>
         </is>
       </c>
-      <c r="G13" s="3" t="inlineStr"/>
-      <c r="H13" s="3" t="inlineStr"/>
-    </row>
-    <row r="14" ht="90" customHeight="1">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="G15" s="3" t="inlineStr"/>
+      <c r="H15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16" ht="90" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>C35</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>Legacy /api/studies over-returns studies across labs (was #44)</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr"/>
-      <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="2" t="inlineStr"/>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr"/>
+      <c r="D16" s="2" t="inlineStr"/>
+      <c r="E16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: GET /api/studies now scopes its list to the active lab
 when one is resolved from the Referer (server/routes.ts), so every returned row
@@ -1710,24 +1668,24 @@
 mirroring the /api/labs/:labId/studies handler. Closed 2026-06-14.</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr"/>
-      <c r="H14" s="2" t="inlineStr"/>
-    </row>
-    <row r="15" ht="90" customHeight="1">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr"/>
+      <c r="H16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17" ht="90" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>C30</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>Verify-script convention backfill (was #41)</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr"/>
-      <c r="D15" s="3" t="inlineStr"/>
-      <c r="E15" s="3" t="inlineStr"/>
-      <c r="F15" s="3" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr"/>
+      <c r="D17" s="3" t="inlineStr"/>
+      <c r="E17" s="3" t="inlineStr"/>
+      <c r="F17" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: all 8 high-stakes math/logic commits now ship a paired
 scripts/verify-*.js (EP17 sensitivity, Deming lot-to-lot, CUMSUM+QC+multi-analyte,
@@ -1735,30 +1693,30 @@
 TEa boundary), per the strike-throughs in #41. Closed 2026-06-13.</t>
         </is>
       </c>
-      <c r="G15" s="3" t="inlineStr">
+      <c r="G17" s="3" t="inlineStr">
         <is>
           <t>scripts/audit_verify_script_coverage.py lookback, 2026-06-02; backfills
 landed 2026-06-03..06.
 ---</t>
         </is>
       </c>
-      <c r="H15" s="3" t="inlineStr"/>
-    </row>
-    <row r="16" ht="90" customHeight="1">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="H17" s="3" t="inlineStr"/>
+    </row>
+    <row r="18" ht="90" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>C31</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>VeritaPT AAA create/update/delete silently no-op in the multi-lab UI</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr"/>
-      <c r="D16" s="2" t="inlineStr"/>
-      <c r="E16" s="2" t="inlineStr"/>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr"/>
+      <c r="D18" s="2" t="inlineStr"/>
+      <c r="E18" s="2" t="inlineStr"/>
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #754 (commit 92ad499) added lab-scoped POST/PUT/DELETE
 /api/labs/:labId/pt/aa-records. The UI posted to the lab-scoped path but only GET
@@ -1769,30 +1727,30 @@
 route mis-filed records to the user's default lab on multi-lab accounts).</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>2026-06-13, found during #18 Phase 3 QA;
 scripts/audit-labscoped-write-routes.mjs now guards the class.
 ---</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr"/>
-    </row>
-    <row r="17" ht="90" customHeight="1">
-      <c r="A17" s="3" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19" ht="90" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>C32</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>VeritaComp "Unlock assessment" false-success no-op</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr"/>
-      <c r="D17" s="3" t="inlineStr"/>
-      <c r="E17" s="3" t="inlineStr"/>
-      <c r="F17" s="3" t="inlineStr">
+      <c r="C19" s="3" t="inlineStr"/>
+      <c r="D19" s="3" t="inlineStr"/>
+      <c r="E19" s="3" t="inlineStr"/>
+      <c r="F19" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #755 (commit 4234007) moved the unlock route to
 /api/labs/:labId/competency/assessments/:id/unlock (the path the client calls).
@@ -1803,29 +1761,29 @@
 HTML).</t>
         </is>
       </c>
-      <c r="G17" s="3" t="inlineStr">
+      <c r="G19" s="3" t="inlineStr">
         <is>
           <t>2026-06-13, found by scripts/audit-labscoped-write-routes.mjs.
 ---</t>
         </is>
       </c>
-      <c r="H17" s="3" t="inlineStr"/>
-    </row>
-    <row r="18" ht="90" customHeight="1">
-      <c r="A18" s="2" t="inlineStr">
+      <c r="H19" s="3" t="inlineStr"/>
+    </row>
+    <row r="20" ht="90" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>C33</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>FK-cascade delete 500s + NavBar laptop-width overflow</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr"/>
-      <c r="D18" s="2" t="inlineStr"/>
-      <c r="E18" s="2" t="inlineStr"/>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr"/>
+      <c r="D20" s="2" t="inlineStr"/>
+      <c r="E20" s="2" t="inlineStr"/>
+      <c r="F20" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PRs #749/#750 fixed NavBar horizontal overflow at laptop
 widths (collapse to the hamburger below 1560px); prod-verified at 1280-1920 with the
@@ -1836,57 +1794,57 @@
 500 -&gt; 200. scripts/audit-delete-cascades.mjs guards the class.</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="G20" s="2" t="inlineStr">
         <is>
           <t>2026-06-13 browser QA of the A7-D4 wave + retro-QC of the 72h PR window.
 ---</t>
         </is>
       </c>
-      <c r="H18" s="2" t="inlineStr"/>
-    </row>
-    <row r="19" ht="90" customHeight="1">
-      <c r="A19" s="3" t="inlineStr">
+      <c r="H20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21" ht="90" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>C1</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>FAQ "over 25 years" -&gt; "over 23 years"</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr"/>
-      <c r="D19" s="3" t="inlineStr"/>
-      <c r="E19" s="3" t="inlineStr"/>
-      <c r="F19" s="3" t="inlineStr">
+      <c r="C21" s="3" t="inlineStr"/>
+      <c r="D21" s="3" t="inlineStr"/>
+      <c r="E21" s="3" t="inlineStr"/>
+      <c r="F21" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: client/src/pages/FAQPage.tsx line 20 reads "over
 23 years" as of 2026-05-01.</t>
         </is>
       </c>
-      <c r="G19" s="3" t="inlineStr">
+      <c r="G21" s="3" t="inlineStr">
         <is>
           <t>session 299e9a73 turn 14, ~2026-04-28.
 ---</t>
         </is>
       </c>
-      <c r="H19" s="3" t="inlineStr"/>
-    </row>
-    <row r="20" ht="90" customHeight="1">
-      <c r="A20" s="2" t="inlineStr">
+      <c r="H21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22" ht="90" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>C5</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B22" s="2" t="inlineStr">
         <is>
           <t>David's VeritaQA grey-button bug (seat permissions mode)</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr"/>
-      <c r="D20" s="2" t="inlineStr"/>
-      <c r="E20" s="2" t="inlineStr"/>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="C22" s="2" t="inlineStr"/>
+      <c r="D22" s="2" t="inlineStr"/>
+      <c r="E22" s="2" t="inlineStr"/>
+      <c r="F22" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #10 squash-merged as commit a43fbba on
 2026-05-01 23:19 MST. Railway deploy succeeded; deployed bundle
@@ -1899,7 +1857,7 @@
 against his exact stored shape (14 of 14 expected outcomes matched).</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr">
+      <c r="G22" s="2" t="inlineStr">
         <is>
           <t>2026-05-01 David's report; veritabench + veritastock
 weren't in MODULE_LIST so seat permissions silently defaulted to
@@ -1907,75 +1865,17 @@
 ---</t>
         </is>
       </c>
-      <c r="H20" s="2" t="inlineStr"/>
-    </row>
-    <row r="21" ht="90" customHeight="1">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>C2</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>TeamPage present-tense "TJC surveyor" check</t>
-        </is>
-      </c>
-      <c r="C21" s="3" t="inlineStr"/>
-      <c r="D21" s="3" t="inlineStr"/>
-      <c r="E21" s="3" t="inlineStr"/>
-      <c r="F21" s="3" t="inlineStr">
-        <is>
-          <t>Closure evidence: site-wide search confirmed all surveyor language
-is past-tense, consistent with user's 2021-2025 service. User closed
-the item in session 299e9a73 turn 4.</t>
-        </is>
-      </c>
-      <c r="G21" s="3" t="inlineStr">
-        <is>
-          <t>session 299e9a73, ~2026-04-28.
----</t>
-        </is>
-      </c>
-      <c r="H21" s="3" t="inlineStr"/>
-    </row>
-    <row r="22" ht="90" customHeight="1">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>C3</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>My Studies CSV/XLSX export (John as design partner)</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr"/>
-      <c r="D22" s="2" t="inlineStr"/>
-      <c r="E22" s="2" t="inlineStr"/>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>Closure evidence: client/src/pages/DashboardPage.tsx line 46 calls
-/api/my-studies/export. server/routes.ts line 1491 implements the
-endpoint. Pulled forward into pre-COLA per user instruction.</t>
-        </is>
-      </c>
-      <c r="G22" s="2" t="inlineStr">
-        <is>
-          <t>session 299e9a73 turn 5, ~2026-04-28.
----</t>
-        </is>
-      </c>
       <c r="H22" s="2" t="inlineStr"/>
     </row>
     <row r="23" ht="90" customHeight="1">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>C4</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Rotate GitHub PAT (because old PAT was committed in SESSION_HANDOFF files)</t>
+          <t>TeamPage present-tense "TJC surveyor" check</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr"/>
@@ -1983,8 +1883,9 @@
       <c r="E23" s="3" t="inlineStr"/>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: no ghp_* or github_pat_* patterns in current
-SESSION_HANDOFF.md or SESSION_HANDOFF-2.md as of 2026-05-01.</t>
+          <t>Closure evidence: site-wide search confirmed all surveyor language
+is past-tense, consistent with user's 2021-2025 service. User closed
+the item in session 299e9a73 turn 4.</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -1998,18 +1899,75 @@
     <row r="24" ht="90" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>C6</t>
+          <t>C3</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>VeritaPolicy service-line filtering removed (formerly #4)</t>
+          <t>My Studies CSV/XLSX export (John as design partner)</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr"/>
       <c r="D24" s="2" t="inlineStr"/>
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Closure evidence: client/src/pages/DashboardPage.tsx line 46 calls
+/api/my-studies/export. server/routes.ts line 1491 implements the
+endpoint. Pulled forward into pre-COLA per user instruction.</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>session 299e9a73 turn 5, ~2026-04-28.
+---</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25" ht="90" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Rotate GitHub PAT (because old PAT was committed in SESSION_HANDOFF files)</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr"/>
+      <c r="D25" s="3" t="inlineStr"/>
+      <c r="E25" s="3" t="inlineStr"/>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>Closure evidence: no ghp_* or github_pat_* patterns in current
+SESSION_HANDOFF.md or SESSION_HANDOFF-2.md as of 2026-05-01.</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>session 299e9a73, ~2026-04-28.
+---</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26" ht="90" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>C6</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>VeritaPolicy service-line filtering removed (formerly #4)</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr"/>
+      <c r="D26" s="2" t="inlineStr"/>
+      <c r="E26" s="2" t="inlineStr"/>
+      <c r="F26" s="2" t="inlineStr">
         <is>
           <t>Closure rationale (operator decision 2026-05-10): Keep all
 VeritaPolicy rows. CFR-only references with no accreditor reference
@@ -2018,29 +1976,29 @@
 report misread the design intent.</t>
         </is>
       </c>
-      <c r="G24" s="2" t="inlineStr">
+      <c r="G26" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H24" s="2" t="inlineStr"/>
-    </row>
-    <row r="25" ht="90" customHeight="1">
-      <c r="A25" s="3" t="inlineStr">
+      <c r="H26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27" ht="90" customHeight="1">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>C7</t>
         </is>
       </c>
-      <c r="B25" s="3" t="inlineStr">
+      <c r="B27" s="3" t="inlineStr">
         <is>
           <t>CLIA number format validation (formerly #13)</t>
         </is>
       </c>
-      <c r="C25" s="3" t="inlineStr"/>
-      <c r="D25" s="3" t="inlineStr"/>
-      <c r="E25" s="3" t="inlineStr"/>
-      <c r="F25" s="3" t="inlineStr">
+      <c r="C27" s="3" t="inlineStr"/>
+      <c r="D27" s="3" t="inlineStr"/>
+      <c r="E27" s="3" t="inlineStr"/>
+      <c r="F27" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: shared/validateClia.ts defines CLIA_REGEX =
 /^\d{2}D\d{7}$/ (line 24), validateClia() helper with whitespace
@@ -2051,30 +2009,30 @@
 shape exists and behaves as specified.</t>
         </is>
       </c>
-      <c r="G25" s="3" t="inlineStr">
+      <c r="G27" s="3" t="inlineStr">
         <is>
           <t>Agent verification 2026-05-10 via grep + file read.
 Operator confirmed shipped 2026-05-10.
 ---</t>
         </is>
       </c>
-      <c r="H25" s="3" t="inlineStr"/>
-    </row>
-    <row r="26" ht="90" customHeight="1">
-      <c r="A26" s="2" t="inlineStr">
+      <c r="H27" s="3" t="inlineStr"/>
+    </row>
+    <row r="28" ht="90" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>C8</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="B28" s="2" t="inlineStr">
         <is>
           <t>VeritaMap lab-wide menu toggle (formerly #19)</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr"/>
-      <c r="D26" s="2" t="inlineStr"/>
-      <c r="E26" s="2" t="inlineStr"/>
-      <c r="F26" s="2" t="inlineStr">
+      <c r="C28" s="2" t="inlineStr"/>
+      <c r="D28" s="2" t="inlineStr"/>
+      <c r="E28" s="2" t="inlineStr"/>
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: client/src/pages/VeritaMapLabwidePage.tsx
 exists and implements the labwide read-only union view. Route is
@@ -2084,59 +2042,59 @@
 parking lot plan (read-only union view, per-session toggle) shipped.</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr">
+      <c r="G28" s="2" t="inlineStr">
         <is>
           <t>Agent verification 2026-05-10 via grep + file read.
 Operator confirmed shipped 2026-05-10.
 ---</t>
         </is>
       </c>
-      <c r="H26" s="2" t="inlineStr"/>
-    </row>
-    <row r="27" ht="90" customHeight="1">
-      <c r="A27" s="3" t="inlineStr">
+      <c r="H28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29" ht="90" customHeight="1">
+      <c r="A29" s="3" t="inlineStr">
         <is>
           <t>C9</t>
         </is>
       </c>
-      <c r="B27" s="3" t="inlineStr">
+      <c r="B29" s="3" t="inlineStr">
         <is>
           <t>Tier-1 smoke test checklist (formerly #6)</t>
         </is>
       </c>
-      <c r="C27" s="3" t="inlineStr"/>
-      <c r="D27" s="3" t="inlineStr"/>
-      <c r="E27" s="3" t="inlineStr"/>
-      <c r="F27" s="3" t="inlineStr">
+      <c r="C29" s="3" t="inlineStr"/>
+      <c r="D29" s="3" t="inlineStr"/>
+      <c r="E29" s="3" t="inlineStr"/>
+      <c r="F29" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: docs/smoke-test-tier1.md documents the Tier-1
 smoke-test process and post-deploy verification steps. Shipped via
 PR #81 as part of the 2026-05-10 wave.</t>
         </is>
       </c>
-      <c r="G27" s="3" t="inlineStr">
+      <c r="G29" s="3" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H27" s="3" t="inlineStr"/>
-    </row>
-    <row r="28" ht="90" customHeight="1">
-      <c r="A28" s="2" t="inlineStr">
+      <c r="H29" s="3" t="inlineStr"/>
+    </row>
+    <row r="30" ht="90" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>C10</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="B30" s="2" t="inlineStr">
         <is>
           <t>Per-module gating (formerly #7)</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr"/>
-      <c r="D28" s="2" t="inlineStr"/>
-      <c r="E28" s="2" t="inlineStr"/>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="C30" s="2" t="inlineStr"/>
+      <c r="D30" s="2" t="inlineStr"/>
+      <c r="E30" s="2" t="inlineStr"/>
+      <c r="F30" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: Client-side useIsReadOnly module keys wired
 on client/src/pages/VeritaPolicyAppPage.tsx and
@@ -2151,29 +2109,29 @@
 PR #76.</t>
         </is>
       </c>
-      <c r="G28" s="2" t="inlineStr">
+      <c r="G30" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H28" s="2" t="inlineStr"/>
-    </row>
-    <row r="29" ht="90" customHeight="1">
-      <c r="A29" s="3" t="inlineStr">
+      <c r="H30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31" ht="90" customHeight="1">
+      <c r="A31" s="3" t="inlineStr">
         <is>
           <t>C11</t>
         </is>
       </c>
-      <c r="B29" s="3" t="inlineStr">
+      <c r="B31" s="3" t="inlineStr">
         <is>
           <t>VeritaStock shipped copy (formerly #8)</t>
         </is>
       </c>
-      <c r="C29" s="3" t="inlineStr"/>
-      <c r="D29" s="3" t="inlineStr"/>
-      <c r="E29" s="3" t="inlineStr"/>
-      <c r="F29" s="3" t="inlineStr">
+      <c r="C31" s="3" t="inlineStr"/>
+      <c r="D31" s="3" t="inlineStr"/>
+      <c r="E31" s="3" t="inlineStr"/>
+      <c r="F31" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: client/src/pages/ArticleInventoryManagementPage.tsx
 line 305 footer reads "platform that includes VeritaStock™" instead
@@ -2181,29 +2139,29 @@
 on /resources/laboratory-inventory-management. Shipped via PR #75.</t>
         </is>
       </c>
-      <c r="G29" s="3" t="inlineStr">
+      <c r="G31" s="3" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H29" s="3" t="inlineStr"/>
-    </row>
-    <row r="30" ht="90" customHeight="1">
-      <c r="A30" s="2" t="inlineStr">
+      <c r="H31" s="3" t="inlineStr"/>
+    </row>
+    <row r="32" ht="90" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t>C12</t>
         </is>
       </c>
-      <c r="B30" s="2" t="inlineStr">
+      <c r="B32" s="2" t="inlineStr">
         <is>
           <t>Admin report one-row-per-lab (formerly #14)</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr"/>
-      <c r="D30" s="2" t="inlineStr"/>
-      <c r="E30" s="2" t="inlineStr"/>
-      <c r="F30" s="2" t="inlineStr">
+      <c r="C32" s="2" t="inlineStr"/>
+      <c r="D32" s="2" t="inlineStr"/>
+      <c r="E32" s="2" t="inlineStr"/>
+      <c r="F32" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: /api/admin/report rewritten in
 server/routes.ts (~line 595) to LEFT JOIN labs on
@@ -2218,56 +2176,56 @@
 prerequisite, not a code bug). Shipped via PR #85.</t>
         </is>
       </c>
-      <c r="G30" s="2" t="inlineStr">
+      <c r="G32" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H30" s="2" t="inlineStr"/>
-    </row>
-    <row r="31" ht="90" customHeight="1">
-      <c r="A31" s="3" t="inlineStr">
+      <c r="H32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33" ht="90" customHeight="1">
+      <c r="A33" s="3" t="inlineStr">
         <is>
           <t>C14</t>
         </is>
       </c>
-      <c r="B31" s="3" t="inlineStr">
+      <c r="B33" s="3" t="inlineStr">
         <is>
           <t>UI relabel "CLIA TEa" -&gt; "Lab-Set Internal Goal" (formerly #1)</t>
         </is>
       </c>
-      <c r="C31" s="3" t="inlineStr"/>
-      <c r="D31" s="3" t="inlineStr"/>
-      <c r="E31" s="3" t="inlineStr"/>
-      <c r="F31" s="3" t="inlineStr">
+      <c r="C33" s="3" t="inlineStr"/>
+      <c r="D33" s="3" t="inlineStr"/>
+      <c r="E33" s="3" t="inlineStr"/>
+      <c r="F33" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: Shipped across four PRs over 2026-05-10.</t>
         </is>
       </c>
-      <c r="G31" s="3" t="inlineStr">
+      <c r="G33" s="3" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H31" s="3" t="inlineStr"/>
-    </row>
-    <row r="32" ht="90" customHeight="1">
-      <c r="A32" s="2" t="inlineStr">
+      <c r="H33" s="3" t="inlineStr"/>
+    </row>
+    <row r="34" ht="90" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
         <is>
           <t>C13</t>
         </is>
       </c>
-      <c r="B32" s="2" t="inlineStr">
+      <c r="B34" s="2" t="inlineStr">
         <is>
           <t>WSLH PT vendor (formerly #15)</t>
         </is>
       </c>
-      <c r="C32" s="2" t="inlineStr"/>
-      <c r="D32" s="2" t="inlineStr"/>
-      <c r="E32" s="2" t="inlineStr"/>
-      <c r="F32" s="2" t="inlineStr">
+      <c r="C34" s="2" t="inlineStr"/>
+      <c r="D34" s="2" t="inlineStr"/>
+      <c r="E34" s="2" t="inlineStr"/>
+      <c r="F34" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: Shipped 2026-05-10 via PR #79 (merge commit
 eeebc6e; merged after rebase to resolve a server/db.ts collision
@@ -2285,68 +2243,9 @@
 'WSLH' is the post-deploy success signal. Shipped via PR #79.</t>
         </is>
       </c>
-      <c r="G32" s="2" t="inlineStr">
+      <c r="G34" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
----</t>
-        </is>
-      </c>
-      <c r="H32" s="2" t="inlineStr"/>
-    </row>
-    <row r="33" ht="90" customHeight="1">
-      <c r="A33" s="3" t="inlineStr">
-        <is>
-          <t>C15</t>
-        </is>
-      </c>
-      <c r="B33" s="3" t="inlineStr">
-        <is>
-          <t>VeritaStock lot tracking + expiration + reorder alerts (formerly #21)</t>
-        </is>
-      </c>
-      <c r="C33" s="3" t="inlineStr"/>
-      <c r="D33" s="3" t="inlineStr"/>
-      <c r="E33" s="3" t="inlineStr"/>
-      <c r="F33" s="3" t="inlineStr">
-        <is>
-          <t>Closure evidence: VeritaStock™ shipped the bench-level inventory
-features the Perplexity competitor analysis identified as a gap:</t>
-        </is>
-      </c>
-      <c r="G33" s="3" t="inlineStr">
-        <is>
-          <t>Originally Perplexity competitor analysis 2026-05-10.
-Audit 2026-05-21 confirmed the feature set ships today.
----</t>
-        </is>
-      </c>
-      <c r="H33" s="3" t="inlineStr"/>
-    </row>
-    <row r="34" ht="90" customHeight="1">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>C16</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>PAL studies guided workflow (formerly #23)</t>
-        </is>
-      </c>
-      <c r="C34" s="2" t="inlineStr"/>
-      <c r="D34" s="2" t="inlineStr"/>
-      <c r="E34" s="2" t="inlineStr"/>
-      <c r="F34" s="2" t="inlineStr">
-        <is>
-          <t>Closure evidence: VeritaCheck™ already ships the Precision /
-Accuracy / Linearity (PAL) study set under EP-protocol naming:</t>
-        </is>
-      </c>
-      <c r="G34" s="2" t="inlineStr">
-        <is>
-          <t>Originally Perplexity competitor analysis 2026-05-10.
-Audit 2026-05-21 confirmed the EP studies cover the PAL framing in
-full.
 ---</t>
         </is>
       </c>
@@ -2355,12 +2254,12 @@
     <row r="35" ht="90" customHeight="1">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>C17</t>
+          <t>C15</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>Source-grounded 21/29/45 CFR + 42 CFR 482-485 (formerly #26)</t>
+          <t>VeritaStock lot tracking + expiration + reorder alerts (formerly #21)</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr"/>
@@ -2368,35 +2267,94 @@
       <c r="E35" s="3" t="inlineStr"/>
       <c r="F35" s="3" t="inlineStr">
         <is>
+          <t>Closure evidence: VeritaStock™ shipped the bench-level inventory
+features the Perplexity competitor analysis identified as a gap:</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>Originally Perplexity competitor analysis 2026-05-10.
+Audit 2026-05-21 confirmed the feature set ships today.
+---</t>
+        </is>
+      </c>
+      <c r="H35" s="3" t="inlineStr"/>
+    </row>
+    <row r="36" ht="90" customHeight="1">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>C16</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>PAL studies guided workflow (formerly #23)</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr"/>
+      <c r="D36" s="2" t="inlineStr"/>
+      <c r="E36" s="2" t="inlineStr"/>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Closure evidence: VeritaCheck™ already ships the Precision /
+Accuracy / Linearity (PAL) study set under EP-protocol naming:</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>Originally Perplexity competitor analysis 2026-05-10.
+Audit 2026-05-21 confirmed the EP studies cover the PAL framing in
+full.
+---</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr"/>
+    </row>
+    <row r="37" ht="90" customHeight="1">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>C17</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>Source-grounded 21/29/45 CFR + 42 CFR 482-485 (formerly #26)</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr"/>
+      <c r="D37" s="3" t="inlineStr"/>
+      <c r="E37" s="3" t="inlineStr"/>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
           <t>Closure evidence: PR #301 (commit 8c27806, merged 2026-05-21)
 source-grounded the 74 remaining non-493 entries in
 server/cfrRequirements.ts against verbatim eCFR XML. Breakdown
 shipped:</t>
         </is>
       </c>
-      <c r="G35" s="3" t="inlineStr">
+      <c r="G37" s="3" t="inlineStr">
         <is>
           <t>PR #301; tasks #18 in the in-session task tracker.
 ---</t>
         </is>
       </c>
-      <c r="H35" s="3" t="inlineStr"/>
-    </row>
-    <row r="36" ht="90" customHeight="1">
-      <c r="A36" s="2" t="inlineStr">
+      <c r="H37" s="3" t="inlineStr"/>
+    </row>
+    <row r="38" ht="90" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
         <is>
           <t>C18</t>
         </is>
       </c>
-      <c r="B36" s="2" t="inlineStr">
+      <c r="B38" s="2" t="inlineStr">
         <is>
           <t>VeritaPolicy "Non CLIA" chapter rename (formerly #3)</t>
         </is>
       </c>
-      <c r="C36" s="2" t="inlineStr"/>
-      <c r="D36" s="2" t="inlineStr"/>
-      <c r="E36" s="2" t="inlineStr"/>
-      <c r="F36" s="2" t="inlineStr">
+      <c r="C38" s="2" t="inlineStr"/>
+      <c r="D38" s="2" t="inlineStr"/>
+      <c r="E38" s="2" t="inlineStr"/>
+      <c r="F38" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #300 (commit 34d7707, merged 2026-05-21)
 renamed all 44 user-facing chapter labels in
@@ -2407,7 +2365,7 @@
 page.</t>
         </is>
       </c>
-      <c r="G36" s="2" t="inlineStr">
+      <c r="G38" s="2" t="inlineStr">
         <is>
           <t>CAP customer screenshot of the /veritapolicy chapter
 headers, 2026-05-01 evening. PR #300; tasks #17 in the in-session
@@ -2415,23 +2373,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H36" s="2" t="inlineStr"/>
-    </row>
-    <row r="37" ht="90" customHeight="1">
-      <c r="A37" s="3" t="inlineStr">
+      <c r="H38" s="2" t="inlineStr"/>
+    </row>
+    <row r="39" ht="90" customHeight="1">
+      <c r="A39" s="3" t="inlineStr">
         <is>
           <t>C19</t>
         </is>
       </c>
-      <c r="B37" s="3" t="inlineStr">
+      <c r="B39" s="3" t="inlineStr">
         <is>
           <t>VeritaStock department-scope toggle (formerly #31)</t>
         </is>
       </c>
-      <c r="C37" s="3" t="inlineStr"/>
-      <c r="D37" s="3" t="inlineStr"/>
-      <c r="E37" s="3" t="inlineStr"/>
-      <c r="F37" s="3" t="inlineStr">
+      <c r="C39" s="3" t="inlineStr"/>
+      <c r="D39" s="3" t="inlineStr"/>
+      <c r="E39" s="3" t="inlineStr"/>
+      <c r="F39" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #319 (commit d01f5fe, merged 2026-05-22)
 shipped the persistent dept-scope toggle on VeritaStockPage. A new
@@ -2442,7 +2400,7 @@
 workspace without re-filtering.</t>
         </is>
       </c>
-      <c r="G37" s="3" t="inlineStr">
+      <c r="G39" s="3" t="inlineStr">
         <is>
           <t>John, San Carlos lab, 2026-05-21. Same conversation that
 drove the vendor dropdown (PR #304), FILTERED VIEW banner (PR #305),
@@ -2450,23 +2408,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H37" s="3" t="inlineStr"/>
-    </row>
-    <row r="38" ht="90" customHeight="1">
-      <c r="A38" s="2" t="inlineStr">
+      <c r="H39" s="3" t="inlineStr"/>
+    </row>
+    <row r="40" ht="90" customHeight="1">
+      <c r="A40" s="2" t="inlineStr">
         <is>
           <t>C20</t>
         </is>
       </c>
-      <c r="B38" s="2" t="inlineStr">
+      <c r="B40" s="2" t="inlineStr">
         <is>
           <t>Primary-lab seat counting (formerly #12)</t>
         </is>
       </c>
-      <c r="C38" s="2" t="inlineStr"/>
-      <c r="D38" s="2" t="inlineStr"/>
-      <c r="E38" s="2" t="inlineStr"/>
-      <c r="F38" s="2" t="inlineStr">
+      <c r="C40" s="2" t="inlineStr"/>
+      <c r="D40" s="2" t="inlineStr"/>
+      <c r="E40" s="2" t="inlineStr"/>
+      <c r="F40" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: is_primary_lab INTEGER NOT NULL DEFAULT 0
 column was added to the lab_members table at db.ts:1276, with the
@@ -2477,7 +2435,7 @@
 is_primary_lab=1 ordering).</t>
         </is>
       </c>
-      <c r="G38" s="2" t="inlineStr">
+      <c r="G40" s="2" t="inlineStr">
         <is>
           <t>2026-05-07 multi-lab discussion. Build shipped as part
 of the Multi-Lab Tier 2 architecture work (Phase 3.x series, prior
@@ -2486,23 +2444,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H38" s="2" t="inlineStr"/>
-    </row>
-    <row r="39" ht="90" customHeight="1">
-      <c r="A39" s="3" t="inlineStr">
+      <c r="H40" s="2" t="inlineStr"/>
+    </row>
+    <row r="41" ht="90" customHeight="1">
+      <c r="A41" s="3" t="inlineStr">
         <is>
           <t>C21</t>
         </is>
       </c>
-      <c r="B39" s="3" t="inlineStr">
+      <c r="B41" s="3" t="inlineStr">
         <is>
           <t>Multi-lab pricing model — Option A (formerly #11)</t>
         </is>
       </c>
-      <c r="C39" s="3" t="inlineStr"/>
-      <c r="D39" s="3" t="inlineStr"/>
-      <c r="E39" s="3" t="inlineStr"/>
-      <c r="F39" s="3" t="inlineStr">
+      <c r="C41" s="3" t="inlineStr"/>
+      <c r="D41" s="3" t="inlineStr"/>
+      <c r="E41" s="3" t="inlineStr"/>
+      <c r="F41" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #322 (commit 0ccd925, merged 2026-05-22)
 added the customer-facing line to the pricing page that reflects
@@ -2515,7 +2473,7 @@
 Enterprise+ block, reads:</t>
         </is>
       </c>
-      <c r="G39" s="3" t="inlineStr">
+      <c r="G41" s="3" t="inlineStr">
         <is>
           <t>2026-05-07 multi-lab discussion (Lisa Veri's
 canonical-case session). PR #322 (initial build); softening PR
@@ -2524,30 +2482,30 @@
 ---</t>
         </is>
       </c>
-      <c r="H39" s="3" t="inlineStr"/>
-    </row>
-    <row r="40" ht="90" customHeight="1">
-      <c r="A40" s="2" t="inlineStr">
+      <c r="H41" s="3" t="inlineStr"/>
+    </row>
+    <row r="42" ht="90" customHeight="1">
+      <c r="A42" s="2" t="inlineStr">
         <is>
           <t>C22</t>
         </is>
       </c>
-      <c r="B40" s="2" t="inlineStr">
+      <c r="B42" s="2" t="inlineStr">
         <is>
           <t>VeritaOps cost-per-test module (formerly #10)</t>
         </is>
       </c>
-      <c r="C40" s="2" t="inlineStr"/>
-      <c r="D40" s="2" t="inlineStr"/>
-      <c r="E40" s="2" t="inlineStr"/>
-      <c r="F40" s="2" t="inlineStr">
+      <c r="C42" s="2" t="inlineStr"/>
+      <c r="D42" s="2" t="inlineStr"/>
+      <c r="E42" s="2" t="inlineStr"/>
+      <c r="F42" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: v1 of the VeritaOps Cost-Per-Reportable-Test
 (CPRT) module shipped across PR #325 through PR #330 on 2026-05-22.
 The module is feature-complete for the typical lab director workflow.</t>
         </is>
       </c>
-      <c r="G40" s="2" t="inlineStr">
+      <c r="G42" s="2" t="inlineStr">
         <is>
           <t>This thread, 2026-05-07 12:05 PM CDT, user message:
 "Parking lot: build an operations module for cost per test
@@ -2556,262 +2514,262 @@
 ---</t>
         </is>
       </c>
-      <c r="H40" s="2" t="inlineStr"/>
-    </row>
-    <row r="41" ht="90" customHeight="1">
-      <c r="A41" s="3" t="inlineStr">
+      <c r="H42" s="2" t="inlineStr"/>
+    </row>
+    <row r="43" ht="90" customHeight="1">
+      <c r="A43" s="3" t="inlineStr">
         <is>
           <t>C23</t>
         </is>
       </c>
-      <c r="B41" s="3" t="inlineStr">
+      <c r="B43" s="3" t="inlineStr">
         <is>
           <t>CCL lab name visual disambiguation in lab switcher (formerly #34)</t>
         </is>
       </c>
-      <c r="C41" s="3" t="inlineStr"/>
-      <c r="D41" s="3" t="inlineStr">
+      <c r="C43" s="3" t="inlineStr"/>
+      <c r="D43" s="3" t="inlineStr">
         <is>
           <t>XS (under 1 day, actual)</t>
         </is>
       </c>
-      <c r="E41" s="3" t="inlineStr">
+      <c r="E43" s="3" t="inlineStr">
         <is>
           <t>Low — cosmetic; only mattered when Lisa or Michael picked the wrong lab from...</t>
         </is>
       </c>
-      <c r="F41" s="3" t="inlineStr">
+      <c r="F43" s="3" t="inlineStr">
         <is>
           <t>Effort: XS (under 1 day, actual)
 Importance: Low — cosmetic; only mattered when Lisa or Michael picked the wrong lab from the dropdown.</t>
         </is>
       </c>
-      <c r="G41" s="3" t="inlineStr">
+      <c r="G43" s="3" t="inlineStr">
         <is>
           <t>flagged 2026-05-23 immediately after provisioning Lisa's CCL lab; closed 2026-05-24.
 ---</t>
         </is>
       </c>
-      <c r="H41" s="3" t="inlineStr"/>
-    </row>
-    <row r="42" ht="90" customHeight="1">
-      <c r="A42" s="2" t="inlineStr">
+      <c r="H43" s="3" t="inlineStr"/>
+    </row>
+    <row r="44" ht="90" customHeight="1">
+      <c r="A44" s="2" t="inlineStr">
         <is>
           <t>C24</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
+      <c r="B44" s="2" t="inlineStr">
         <is>
           <t>VC Unlimited Y1/Y2 price disclosure UX (formerly #35)</t>
         </is>
       </c>
-      <c r="C42" s="2" t="inlineStr"/>
-      <c r="D42" s="2" t="inlineStr">
+      <c r="C44" s="2" t="inlineStr"/>
+      <c r="D44" s="2" t="inlineStr">
         <is>
           <t>XS (under 1 day, actual)</t>
         </is>
       </c>
-      <c r="E42" s="2" t="inlineStr">
+      <c r="E44" s="2" t="inlineStr">
         <is>
           <t>Low when shipped (proactive, no customer complaint yet) — but high if a procu...</t>
         </is>
       </c>
-      <c r="F42" s="2" t="inlineStr">
+      <c r="F44" s="2" t="inlineStr">
         <is>
           <t>Effort: XS (under 1 day, actual)
 Importance: Low when shipped (proactive, no customer complaint yet) — but high if a procurement reviewer later disputes the $499 renewal as undisclosed.</t>
         </is>
       </c>
-      <c r="G42" s="2" t="inlineStr">
+      <c r="G44" s="2" t="inlineStr">
         <is>
           <t>Pricing rebuild 2026-05-23; closed 2026-05-24 proactively before any customer dispute.
 ---</t>
         </is>
       </c>
-      <c r="H42" s="2" t="inlineStr"/>
-    </row>
-    <row r="43" ht="90" customHeight="1">
-      <c r="A43" s="3" t="inlineStr">
+      <c r="H44" s="2" t="inlineStr"/>
+    </row>
+    <row r="45" ht="90" customHeight="1">
+      <c r="A45" s="3" t="inlineStr">
         <is>
           <t>C25</t>
         </is>
       </c>
-      <c r="B43" s="3" t="inlineStr">
+      <c r="B45" s="3" t="inlineStr">
         <is>
           <t>VeritaQC Phase 1 (Levey-Jennings + Westgard live engine) (formerly #20)</t>
         </is>
       </c>
-      <c r="C43" s="3" t="inlineStr"/>
-      <c r="D43" s="3" t="inlineStr">
+      <c r="C45" s="3" t="inlineStr"/>
+      <c r="D45" s="3" t="inlineStr">
         <is>
           <t>L (about 5 days end-to-end, actual: Phase 0 schema → Phase 1A evaluator → 1B...</t>
         </is>
       </c>
-      <c r="E43" s="3" t="inlineStr">
+      <c r="E45" s="3" t="inlineStr">
         <is>
           <t>High — largest single gap vs myLabCompliance.io per Perplexity competitor ana...</t>
         </is>
       </c>
-      <c r="F43" s="3" t="inlineStr">
+      <c r="F45" s="3" t="inlineStr">
         <is>
           <t>Effort: L (about 5 days end-to-end, actual: Phase 0 schema → Phase 1A evaluator → 1B entry UI → 1C daily review → 1D monthly PDF + attestation)
 Importance: High — largest single gap vs myLabCompliance.io per Perplexity competitor analysis; promotes VeritaAssure from documentation tool to lab operations platform.</t>
         </is>
       </c>
-      <c r="G43" s="3" t="inlineStr">
+      <c r="G45" s="3" t="inlineStr">
         <is>
           <t>Perplexity competitor analysis 2026-05-10. Scoping confirmed via the build_phase1_mockup.py iterations 2026-05-24. Shipped 2026-05-25.
 ---</t>
         </is>
       </c>
-      <c r="H43" s="3" t="inlineStr"/>
-    </row>
-    <row r="44" ht="90" customHeight="1">
-      <c r="A44" s="2" t="inlineStr">
+      <c r="H45" s="3" t="inlineStr"/>
+    </row>
+    <row r="46" ht="90" customHeight="1">
+      <c r="A46" s="2" t="inlineStr">
         <is>
           <t>C26</t>
         </is>
       </c>
-      <c r="B44" s="2" t="inlineStr">
+      <c r="B46" s="2" t="inlineStr">
         <is>
           <t>VeritaLab CMS-116 application support + state licensing registry (formerly #22)</t>
         </is>
       </c>
-      <c r="C44" s="2" t="inlineStr"/>
-      <c r="D44" s="2" t="inlineStr">
+      <c r="C46" s="2" t="inlineStr"/>
+      <c r="D46" s="2" t="inlineStr">
         <is>
           <t>M (1-2 weeks for v1, actual)</t>
         </is>
       </c>
-      <c r="E44" s="2" t="inlineStr">
+      <c r="E46" s="2" t="inlineStr">
         <is>
           <t>Medium — competitor parity (myLabCompliance.io) plus useful at lab startup an...</t>
         </is>
       </c>
-      <c r="F44" s="2" t="inlineStr">
+      <c r="F46" s="2" t="inlineStr">
         <is>
           <t>Effort: M (1-2 weeks for v1, actual)
 Importance: Medium — competitor parity (myLabCompliance.io) plus useful at lab startup and at certificate-type changes.</t>
         </is>
       </c>
-      <c r="G44" s="2" t="inlineStr">
+      <c r="G46" s="2" t="inlineStr">
         <is>
           <t>Perplexity competitor analysis (myLabCompliance.io), 2026-05-10. Reclassified as a VeritaLab extension 2026-05-25. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H44" s="2" t="inlineStr"/>
-    </row>
-    <row r="45" ht="90" customHeight="1">
-      <c r="A45" s="3" t="inlineStr">
+      <c r="H46" s="2" t="inlineStr"/>
+    </row>
+    <row r="47" ht="90" customHeight="1">
+      <c r="A47" s="3" t="inlineStr">
         <is>
           <t>C27</t>
         </is>
       </c>
-      <c r="B45" s="3" t="inlineStr">
+      <c r="B47" s="3" t="inlineStr">
         <is>
           <t>Active vs view-only seat split (formerly #33)</t>
         </is>
       </c>
-      <c r="C45" s="3" t="inlineStr"/>
-      <c r="D45" s="3" t="inlineStr">
+      <c r="C47" s="3" t="inlineStr"/>
+      <c r="D47" s="3" t="inlineStr">
         <is>
           <t>M (~1 week of engineering, actual: shipped in a single multi-PR session)</t>
         </is>
       </c>
-      <c r="E45" s="3" t="inlineStr">
+      <c r="E47" s="3" t="inlineStr">
         <is>
           <t>Medium — closed the gap between /pricing copy and product behavior; gives sal...</t>
         </is>
       </c>
-      <c r="F45" s="3" t="inlineStr">
+      <c r="F47" s="3" t="inlineStr">
         <is>
           <t>Effort: M (~1 week of engineering, actual: shipped in a single multi-PR session)
 Importance: Medium — closed the gap between /pricing copy and product behavior; gives sales a clean answer for "do you charge for our medical director?"</t>
         </is>
       </c>
-      <c r="G45" s="3" t="inlineStr">
+      <c r="G47" s="3" t="inlineStr">
         <is>
           <t>Pricing analysis doc Decision 3 (2026-05-21); MEDIUM scenario revised 2026-05-29 to retire the "unlimited view-only" claim. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H45" s="3" t="inlineStr"/>
-    </row>
-    <row r="46" ht="90" customHeight="1">
-      <c r="A46" s="2" t="inlineStr">
+      <c r="H47" s="3" t="inlineStr"/>
+    </row>
+    <row r="48" ht="90" customHeight="1">
+      <c r="A48" s="2" t="inlineStr">
         <is>
           <t>C28</t>
         </is>
       </c>
-      <c r="B46" s="2" t="inlineStr">
+      <c r="B48" s="2" t="inlineStr">
         <is>
           <t>"Why VeritaCheck" comparative one-pager (formerly #37)</t>
         </is>
       </c>
-      <c r="C46" s="2" t="inlineStr"/>
-      <c r="D46" s="2" t="inlineStr">
+      <c r="C48" s="2" t="inlineStr"/>
+      <c r="D48" s="2" t="inlineStr">
         <is>
           <t>S (one design pass + four claim paragraphs + PDF + matching marketing-site pa...</t>
         </is>
       </c>
-      <c r="E46" s="2" t="inlineStr">
+      <c r="E48" s="2" t="inlineStr">
         <is>
           <t>Medium — closed a positioning gap surfaced by six COLA conference attendees a...</t>
         </is>
       </c>
-      <c r="F46" s="2" t="inlineStr">
+      <c r="F48" s="2" t="inlineStr">
         <is>
           <t>Effort: S (one design pass + four claim paragraphs + PDF + matching marketing-site page, actual)
 Importance: Medium — closed a positioning gap surfaced by six COLA conference attendees attached to a legacy verification tool; converts product-quality advantage into a leave-behind Lisa can hand out.</t>
         </is>
       </c>
-      <c r="G46" s="2" t="inlineStr">
+      <c r="G48" s="2" t="inlineStr">
         <is>
           <t>2026-05-11 / 2026-05-12 conference notes review with Michael. Conference attendees (Whitehead, Odegard, Othman, Molinelli, Kyle, Allred) expressed interest in equivalent / superior product. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H46" s="2" t="inlineStr"/>
-    </row>
-    <row r="47" ht="90" customHeight="1">
-      <c r="A47" s="3" t="inlineStr">
+      <c r="H48" s="2" t="inlineStr"/>
+    </row>
+    <row r="49" ht="90" customHeight="1">
+      <c r="A49" s="3" t="inlineStr">
         <is>
           <t>C29</t>
         </is>
       </c>
-      <c r="B47" s="3" t="inlineStr">
+      <c r="B49" s="3" t="inlineStr">
         <is>
           <t>VeritaPolicy approval workflow — MediaLab functional mirror</t>
         </is>
       </c>
-      <c r="C47" s="3" t="inlineStr"/>
-      <c r="D47" s="3" t="inlineStr">
+      <c r="C49" s="3" t="inlineStr"/>
+      <c r="D49" s="3" t="inlineStr">
         <is>
           <t>XL (one focused session, 12 PRs landed)</t>
         </is>
       </c>
-      <c r="E47" s="3" t="inlineStr">
+      <c r="E49" s="3" t="inlineStr">
         <is>
           <t>High — replaces MediaLab Document Control ($752/$2,250 starting price, scalin...</t>
         </is>
       </c>
-      <c r="F47" s="3" t="inlineStr">
+      <c r="F49" s="3" t="inlineStr">
         <is>
           <t>Effort: XL (one focused session, 12 PRs landed)
 Importance: High — replaces MediaLab Document Control ($752/$2,250 starting price, scaling to $10K-$20K/yr at enterprise per Capterra public data) with an included VeritaPolicy feature; closes a real positioning gap and gives sales a direct comparator line.</t>
         </is>
       </c>
-      <c r="G47" s="3" t="inlineStr">
+      <c r="G49" s="3" t="inlineStr">
         <is>
           <t>Pricing strategy conversation 2026-05-29 (Michael: "I don't like bolt-ons; we should replicate this") → scoped 8 phases → shipped all 12 PRs in single session. Shipped 2026-05-29.
 ---</t>
         </is>
       </c>
-      <c r="H47" s="3" t="inlineStr"/>
+      <c r="H49" s="3" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H47"/>
+  <autoFilter ref="A1:H49"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
docs(parking-lot): close #18 (shipped), reclassify #17 to CLOSED (#1354)
TASK: Remove two shipped items mis-filed in OPEN. PLAN: #18 -> C47, #17 -> C48; regenerate xlsx. Self-check: docs only, OPEN 17->15.
</commit_message>
<xml_diff>
--- a/PARKING_LOT.xlsx
+++ b/PARKING_LOT.xlsx
@@ -12,8 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RETIRED" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$18</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$47</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$49</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RETIRED'!$A$1:$H$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -564,6 +564,12 @@
         <is>
           <t>Pre-COLA. May 6-8 conference; Saturday + Sunday +
 Monday available before the booth.
+---
+_(item #17 reclassified to CLOSED 2026-09-28; VeritaResponse shipped and live, see C48 below)_
+---
+_(item #18 closed 2026-09-28; all phases shipped, see C47 below)_
+---
+_(item #22 closed 2026-05-28; see C26 below)_
 ---</t>
         </is>
       </c>
@@ -571,130 +577,30 @@
     <row r="3" ht="90" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>27</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>New flagship module: VeritaResponse (post-survey deficiency response)</t>
+          <t>Acquire CAP MOL (Molecular) checklist to verify 2 pending entries</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>BUILT and LIVE (this entry was stale). VeritaResponse shipped as a
-full module: findings table + CRUD + lifecycle, due-date computation, 30/60/90-day
-effectiveness monitoring (wave C3), cross-modu...</t>
+          <t>Open, blocks on operator obtaining the MOL checklist.</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>XL (6+ weeks; flagship-scale)</t>
+          <t>N/A (operator action — ~1 hour of code work once the file is in hand)</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>High — booth-validated demand at COLA Nashville; no existing module covers po...</t>
+          <t>Low — two entries total; low traffic; only matters when a customer cites a MO...</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>A new module that helps a lab manage the full lifecycle of
-responding to inspection deficiencies (CAP, TJC, COLA, CMS-2567,
-AABB), from intake of a citation through corrective-action authoring,
-supporting-evidence collection, submission tracking, and 30/60/90-day
-effectiveness verification. Pairs with VeritaCheck (find gaps before
-they cite you) and VeritaPT (prove your PT covers your menu) to
-complete the compliance lifecycle: prevent → respond → prove.</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-07 conference user request, COLA Nashville. User
-asked for thoughts and recommendations on adding a deficiency-response
-module. Online research conducted same session covering CAP, TJC,
-COLA, CMS-2567, AABB. URLs cited above.</t>
-        </is>
-      </c>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>Post-COLA. Build is multi-week regardless;
-zero rationale for any code change before the conference ends.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="90" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>18</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Unregulated analyte / Alternative Assessment (AAA) coverage — cross-module gap</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>PARTIAL as of 2026-05-10.
-- Phase 1 (VeritaScan AAA sub-block, items 169-173) CLOSED via
- PR #78 (client/src/lib/veritaScanData.ts). Item #46 retained as
- AAA gateway; new 5-item block uses ids 16...</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>S (1-3 days once #17 ships) for Phase 3 — Phases 1 and 2 already shipped.</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Medium — closes a real workflow loop (AAA failure → VeritaResponse finding) b...</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>Effort: S (1-3 days once #17 ships) for Phase 3 — Phases 1 and 2 already shipped.
-Importance: Medium — closes a real workflow loop (AAA failure → VeritaResponse finding) but only matters once #17 exists.</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>Post-COLA. Phase 1 and Phase 2 data layer
-shipped 2026-05-10.
----
-_(item #22 closed 2026-05-28; see C26 below)_
----</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="90" customHeight="1">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>27</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Acquire CAP MOL (Molecular) checklist to verify 2 pending entries</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>Open, blocks on operator obtaining the MOL checklist.</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>N/A (operator action — ~1 hour of code work once the file is in hand)</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>Low — two entries total; low traffic; only matters when a customer cites a MO...</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>PR #108 left 2 entries in server/capRequirements.ts
 flagged as unverified because the operator does not hold the CAP MOL
@@ -708,48 +614,48 @@
 The MOL module's MAS xlsx is the only one missing from that set.</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>PR #108 commit 92f9573 (closed via merge 2026-05-11),
 audit findings.</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>Post-COLA. Two entries; low traffic.
 ---</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="90" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
+    <row r="4" ht="90" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>28</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Acquire AABB Standards 35th edition + current COLA Accreditation Manual for exhaustive citation verification</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>Open, blocks on operator obtaining the gated accreditor
 manuals. Until then, AABB / COLA citations are best-effort against
 the public-source compilations.</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>N/A (operator action — ~1-2 days of audit re-run once the manuals are held)</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>High — gates #5 from reaching "exhaustively verified" status for AABB and COLA.</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>The 2026-05-11 QC audit found that VeritaScan, cfrRequirements
 cross-refs, and colaRequirements.ts cite about 180 AABB and COLA codes
@@ -769,14 +675,14 @@
  does not enumerate fully.</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>2026-05-11 QC/QA audit, documented in
 OneDrive\Lab\Regulatory\aaa Truth Master Document\PROVENANCE.md
 "Audit-coverage limits" section.</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>Post-COLA. Operator-side action item, no code
 work pending until the source documents land.
@@ -784,34 +690,34 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="90" customHeight="1">
-      <c r="A7" s="3" t="inlineStr">
+    <row r="5" ht="90" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>VeritaStock barcode scanning (full mobile scan flow)</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>Parked pending first paid commitment.
 ---</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>L (12 working days, ~3 weeks calendar)</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>High — strategic moat vs Unity Lab Services ($30K+/yr); presold as included o...</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>The remaining barcode-scanning build for VeritaStock, scoped
 during the 2026-05-20 Pfizer follow-up discussion. Order-now reorder
@@ -820,7 +726,7 @@
 Services-class inventory product.</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>2026-05-20 Pfizer follow-up session, after the order-now
 reorder document shipped (PR #286). Strategic decision documented in
@@ -831,31 +737,31 @@
 barcode scanning waits on revenue...</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr"/>
-    </row>
-    <row r="8" ht="90" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr"/>
+    </row>
+    <row r="6" ht="90" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Plain-language summary layer for verbatim CFR citations</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr"/>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr"/>
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>M (multi-day content authoring across 96 Master List rows if redesigned corre...</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>Medium — director readability win; no customer urgency.</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>server/cfrRequirements.ts carries verbatim eCFR text in
 the description field (PR #301 closed #26). The verbatim text is
@@ -864,8 +770,8 @@
 director read faster.</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr"/>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>Post-COLA. No customer urgency. Operator
 has not yet authorized a redesign attempt as of 2026-05-21.
@@ -873,29 +779,29 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="90" customHeight="1">
-      <c r="A9" s="3" t="inlineStr">
+    <row r="7" ht="90" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Lab leader community / forum (paid subscription idea)</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr"/>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr"/>
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>XL (ongoing operational commitment, not a build) as paid; S (a few days to sp...</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>Low as paid product (SWOT verdict: don't build); Medium as free lead-funnel a...</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>Operator-floated 2026-05-22: a vetted online forum for
 laboratory leaders (directors, managers, supervisors). Pricing as
@@ -908,8 +814,8 @@
 lab-leader water cooler.</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr"/>
-      <c r="H9" s="3" t="inlineStr">
+      <c r="G7" s="3" t="inlineStr"/>
+      <c r="H7" s="3" t="inlineStr">
         <is>
           <t>Post-COLA. No customer urgency.
 ---
@@ -920,39 +826,39 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="90" customHeight="1">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="8" ht="90" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>36</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>New module: laboratory non-conforming event documentation</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Scoped, not started (updated 2026-09-28). Now lands in VeritaResponse per Michael's direction above; the earlier "new standalone module" framing is superseded. Do not start building until Michael g...</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>L (initial estimate, pending Michael's scope walkthrough — likely new DB tabl...</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>High — every accredited laboratory (TJC, CAP, COLA, AABB) has to document non...</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>Build a module to document laboratory non-conforming events (NCEs). Surfaces a lab needs to capture include specimen rejection, temperature excursions, reagent issues, equipment failures, result-reporting errors, transcription errors, lost specimens, contamination events, and similar quality incidents. Full scope, target accreditor mapping, terminology preference (NCE / NCR / event / incident / occurrence), and how it should relate to the existing VeritaQC corrective-action engine and VeritaResponse deficiency tracker are TBD pending Michael's scope walkthrough.</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr"/>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>Post-COLA. No customer urgency yet, but high strategic value once defined — closes a real gap every lab has and that no other Verita module currently serves.
 ---
@@ -961,76 +867,76 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="90" customHeight="1">
-      <c r="A11" s="3" t="inlineStr">
+    <row r="9" ht="90" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>38</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>Screen-capture video: VeritaCheck method comparison in 60 seconds</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>Open. Re-parked 2026-05-27 (originally PR #117, abandoned with merge conflicts then closed-and-re-authored at current numbering). Pending operator decision on whether to record this themselves or p...</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>S for agent prep (storyboard / pre-fill / captions / checklist); ~1 hour of o...</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t>Medium — operator selected this as the highest-impact positioning artifact du...</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="F9" s="3" t="inlineStr">
         <is>
           <t>30-60 second screen recording demonstrating the "experienced lab tech figures it out in seconds" claim. From blank method-comparison study to completed PDF, no voiceover, no narration, visible cursor motion. Embed autoplay-muted on the marketing site, include in conference follow-up emails.</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="G9" s="3" t="inlineStr">
         <is>
           <t>2026-05-12 conversation. Michael selected the screen-cap video as the highest-impact positioning artifact, then asked the agent to record it. Agent does not have screen-recording capability; option parked rather than fudged.</t>
         </is>
       </c>
-      <c r="H11" s="3" t="inlineStr">
+      <c r="H9" s="3" t="inlineStr">
         <is>
           <t>Post-COLA, conference-driven.
 ---</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="90" customHeight="1">
-      <c r="A12" s="2" t="inlineStr">
+    <row r="10" ht="90" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>39</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>MediaLab parity hardening (VeritaPolicy approval workflow depth)</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Open, customer-triggered. No urgency until a prospect specifically asks for one of the listed depth items.</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>L (1-2 weeks for the high-value items; each independent feature is M)</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>Medium-High — the C29 build shipped the surface MediaLab markets but depth is...</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>The VeritaPolicy approval workflow build (C29, 2026-05-29) hit roughly 60-70% MediaLab feature surface. The following gaps remain when comparing against an enterprise MediaLab Document Control deployment:
 - Quizzes on attestations. Schema columns quiz_score and quiz_total_questions exist on policy_attestations but the quiz authoring + presentation UI was scoped out of Phase 4. MediaLab labs use 5-10 multiple-choice questions per policy to confirm comprehension, not just attestation. Adds compliance defensibility.
@@ -1040,54 +946,133 @@
 - In-browser DOCX editing. MediaLab has a structured editor that creates a Table of Contents from headings. We treat documents as...</t>
         </is>
       </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-29 QA pass after C29 shipped (qa-policy-build.js + qa-policy-ui.js: 54/54 happy path verified). Honest depth assessment surfaced by Michael's "how confident are you" question — see C29 entry for full QA receipts.</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Post-COLA. Defensive against MediaLab in head-to-head sales calls.
+---</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="90" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>VeritaQC Import Phase A: human-in-the-loop Gate 3 click-through (deferred)</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Open, awaiting Michael's 5-minute click test. Will move task #77 to completed only after he reports the user-visible result.
+---</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>XS (~5 minutes of Michael's time on a live URL).</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Low. Backend contract is fully verified via 35/35 passing offline contract ch...</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Effort: XS (~5 minutes of Michael's time on a live URL).
+Importance: Low. Backend contract is fully verified via 35/35 passing offline contract checks (scripts/verify-veritaqc-import.js) plus three live-API smoke checks against prod (candidates, preview, mappings PUT/GET) on Riverside Regional with seed lot SEED-1780436709094 (18 Glucose results). The browser-driven click was not run because Claude-in-Chrome's renderer froze repeatedly on the Radix Select inside VeritaCheckPage, not on Phase A code itself. Risk of a UX bug surviving to a customer is small but not zero.</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>task #77 stalled at Gate 3 step 8 on 2026-06-02. PR #500 squash-merged at commit 17a91ff, prod /api/health confirmed ACTIVE on that commit at 20:43 UTC.</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12" ht="90" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Outbound demo-invite messaging campaign to 1st-degree LinkedIn contacts</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Parked. Plan documented. Implementation deferred until trigger conditions met.
+---</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>L (1 week prep + 4-6 weeks of staged sends)</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>High. Converts existing warm network (~2,500 1st-degree contacts and growing...</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>A staged outbound DM campaign walking Michael's 1st-degree LinkedIn contacts through tier-segmented demo invitations for VeritaAssure. Goal: convert warmest contacts into demo conversations first, then chain into trials and paid subscriptions. Separate pipeline from COLA cohort follow-up and from content-driven inbound; all three feed the same demo funnel but originate from different warmth sources.</t>
+        </is>
+      </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29 QA pass after C29 shipped (qa-policy-build.js + qa-policy-ui.js: 54/54 happy path verified). Honest depth assessment surfaced by Michael's "how confident are you" question — see C29 entry for full QA receipts.</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>Post-COLA. Defensive against MediaLab in head-to-head sales calls.
----</t>
-        </is>
-      </c>
+          <t>2026-06-04 session, after weekly LinkedIn invite batch completion (80 sent, cap hit at #84 Victoria Allen).</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr"/>
     </row>
     <row r="13" ht="90" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>47</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>VeritaQC Import Phase A: human-in-the-loop Gate 3 click-through (deferred)</t>
+          <t>Hide sections a lab does not use from a master list, to reduce clutter (prospect-requested)</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Open, awaiting Michael's 5-minute click test. Will move task #77 to completed only after he reports the user-visible result.
+          <t>Open. Not started. Needs a one-line scope confirmation (which master list).
 ---</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>XS (~5 minutes of Michael's time on a live URL).</t>
+          <t>S-M (a few days to ~2 weeks depending on scope) — a lab-level visibility togg...</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>Low. Backend contract is fully verified via 35/35 passing offline contract ch...</t>
+          <t>Medium-High — came straight from a live prospect today as an onboarding-frict...</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Effort: XS (~5 minutes of Michael's time on a live URL).
-Importance: Low. Backend contract is fully verified via 35/35 passing offline contract checks (scripts/verify-veritaqc-import.js) plus three live-API smoke checks against prod (candidates, preview, mappings PUT/GET) on Riverside Regional with seed lot SEED-1780436709094 (18 Glucose results). The browser-driven click was not run because Claude-in-Chrome's renderer froze repeatedly on the Radix Select inside VeritaCheckPage, not on Phase A code itself. Risk of a UX bug surviving to a customer is small but not zero.</t>
+          <t>Effort: S-M (a few days to ~2 weeks depending on scope) — a lab-level visibility toggle that hides not-applicable or unused sections from a master-list view. Smaller if it is a "hide N/A" filter on the existing VeritaDC master list, larger if it also spans VeritaScan domains.
+Importance: Medium-High — came straight from a live prospect today as an onboarding-friction point; a lab that does not run a service line should not have to wade past its requirements.</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>task #77 stalled at Gate 3 step 8 on 2026-06-02. PR #500 squash-merged at commit 17a91ff, prod /api/health confirmed ACTIVE on that commit at 20:43 UTC.</t>
+          <t>2026-09-23 session, Michael relaying a prospect ask from a demo today.</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr"/>
@@ -1095,38 +1080,35 @@
     <row r="14" ht="90" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>50</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Outbound demo-invite messaging campaign to 1st-degree LinkedIn contacts</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>Parked. Plan documented. Implementation deferred until trigger conditions met.
----</t>
-        </is>
-      </c>
+          <t>Competency "assessed this cycle" uses a flat 365-day window</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr"/>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>L (1 week prep + 4-6 weeks of staged sends)</t>
+          <t>S-M - anchor the coverage-map "assessed this cycle" to the person's actual CL...</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>High. Converts existing warm network (~2,500 1st-degree contacts and growing...</t>
+          <t>Medium - in an employee's first year the semiannual windows differ from a fla...</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>A staged outbound DM campaign walking Michael's 1st-degree LinkedIn contacts through tier-segmented demo invitations for VeritaAssure. Goal: convert warmest contacts into demo conversations first, then chain into trials and paid subscriptions. Separate pipeline from COLA cohort follow-up and from content-driven inbound; all three feed the same demo funnel but originate from different warmth sources.</t>
+          <t>Effort: S-M - anchor the coverage-map "assessed this cycle" to the person's actual CLIA cadence (semiannual in year 1 per 42 CFR 493.1451(b)(8), annual thereafter) from staff_competency_schedules, instead of the v1 flat 365-day lookback.
+Importance: Medium - in an employee's first year the semiannual windows differ from a flat annual window, so a first-year assessment could read as current slightly longer or shorter than the true cadence. Fine for the common annual case; refine for year-1 accuracy.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04 session, after weekly LinkedIn invite batch completion (80 sent, cap hit at #84 Victoria Allen).</t>
+          <t>2026-09-24 session, VeritaComp coverage map (#48 Phase 3) v1 simplification, noted in PR #1319.
+---</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr"/>
@@ -1134,167 +1116,91 @@
     <row r="15" ht="90" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>51</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Hide sections a lab does not use from a master list, to reduce clutter (prospect-requested)</t>
+          <t>VeritaTrack task owner + owner-scoped reminder routing</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Open. Not started. Needs a one-line scope confirmation (which master list).
----</t>
+          <t>Open, not started. Placeholder pending build. Open questions: is the owner a staff_employee or a seat user, and how are reminder recipients currently chosen.</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>S-M (a few days to ~2 weeks depending on scope) — a lab-level visibility togg...</t>
+          <t>S-M (1-3 days to ~1.5 weeks) — add an owner on a VeritaTrack task, selectable...</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>Medium-High — came straight from a live prospect today as an onboarding-frict...</t>
+          <t>Medium — cuts reminder-email noise so people only get the tasks that are thei...</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>Effort: S-M (a few days to ~2 weeks depending on scope) — a lab-level visibility toggle that hides not-applicable or unused sections from a master-list view. Smaller if it is a "hide N/A" filter on the existing VeritaDC master list, larger if it also spans VeritaScan domains.
-Importance: Medium-High — came straight from a live prospect today as an onboarding-friction point; a lab that does not run a service line should not have to wade past its requirements.</t>
+          <t>Michael, verbatim (2026-09-28): "In veritatask, we should be able to assign an owner from staff that are built, then in the reminder section, we should be able to designate reminder emails only to the owner. The hem person does not need the chemistry reminders, etc." Module note: there is no VeritaTask module in the codebase; the task/reminder surface is VeritaTrack (client/src/pages/VeritaTrackAppPage.tsx), so this lands there. Today VeritaTrack tasks are not owned by a specific staff member and reminder emails are not recipient-scoped to an owner. The build adds (a) an owner selector on each task drawn from the lab's VeritaStaff roster, and (b) a reminder setting that routes the reminder email to only that owner. Confirm the current reminder recipient model before sizing.</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>2026-09-23 session, Michael relaying a prospect ask from a demo today.</t>
-        </is>
-      </c>
-      <c r="H15" s="3" t="inlineStr"/>
+          <t>2026-09-28 session, Michael "for later (placeholder)" optimization #1 (relaying from the Lab Members / VeritaAssure screens).</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>Post-COLA. No customer urgency.
+---</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="90" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>52</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Competency "assessed this cycle" uses a flat 365-day window</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr"/>
+          <t>Medical Director seat via account-grant dropdown (designate / transfer MD)</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Open, not started. Placeholder. Confirm the current MD-seat assignment path and the one-MD-per-location enforcement point before sizing.</t>
+        </is>
+      </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>S-M - anchor the coverage-map "assessed this cycle" to the person's actual CL...</t>
+          <t>S-M (1-3 days to ~1.5 weeks) — move MD-seat assignment onto the same per-memb...</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Medium - in an employee's first year the semiannual windows differ from a fla...</t>
+          <t>Medium-High — the MD seat is a recurring friction point (Georgetown, SCAHC MD...</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Effort: S-M - anchor the coverage-map "assessed this cycle" to the person's actual CLIA cadence (semiannual in year 1 per 42 CFR 493.1451(b)(8), annual thereafter) from staff_competency_schedules, instead of the v1 flat 365-day lookback.
-Importance: Medium - in an employee's first year the semiannual windows differ from a flat annual window, so a first-year assessment could read as current slightly longer or shorter than the true cadence. Fine for the common annual case; refine for year-1 accuracy.</t>
+          <t>Michael, verbatim (2026-09-28): "The way we are doing the medical director seat is silly. Why not just use the account grant dropdown to give a medical director seat. If the person is already in, then we should just be able to grant the medical director seat the same way we promote people to admin or reduce them to staff as long as we only have 1 per location. Maybe do another block like the transfer ownership block as 'designate medical director or transfer medical director'." So: fold the MD seat into the existing member role dropdown (Admin / Staff / ... + Medical Director) with a single-MD-per-lab constraint, and add a dedicated designate-or-transfer-MD block that mirrors the transfer-ownership UX for changing the MD. Cross-ref [[project_medical_director_designation]] and the seat model.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 session, VeritaComp coverage map (#48 Phase 3) v1 simplification, noted in PR #1319.
----</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr"/>
-    </row>
-    <row r="17" ht="90" customHeight="1">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>51</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>VeritaTrack task owner + owner-scoped reminder routing</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>Open, not started. Placeholder pending build. Open questions: is the owner a staff_employee or a seat user, and how are reminder recipients currently chosen.</t>
-        </is>
-      </c>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>S-M (1-3 days to ~1.5 weeks) — add an owner on a VeritaTrack task, selectable...</t>
-        </is>
-      </c>
-      <c r="E17" s="3" t="inlineStr">
-        <is>
-          <t>Medium — cuts reminder-email noise so people only get the tasks that are thei...</t>
-        </is>
-      </c>
-      <c r="F17" s="3" t="inlineStr">
-        <is>
-          <t>Michael, verbatim (2026-09-28): "In veritatask, we should be able to assign an owner from staff that are built, then in the reminder section, we should be able to designate reminder emails only to the owner. The hem person does not need the chemistry reminders, etc." Module note: there is no VeritaTask module in the codebase; the task/reminder surface is VeritaTrack (client/src/pages/VeritaTrackAppPage.tsx), so this lands there. Today VeritaTrack tasks are not owned by a specific staff member and reminder emails are not recipient-scoped to an owner. The build adds (a) an owner selector on each task drawn from the lab's VeritaStaff roster, and (b) a reminder setting that routes the reminder email to only that owner. Confirm the current reminder recipient model before sizing.</t>
-        </is>
-      </c>
-      <c r="G17" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-28 session, Michael "for later (placeholder)" optimization #1 (relaying from the Lab Members / VeritaAssure screens).</t>
-        </is>
-      </c>
-      <c r="H17" s="3" t="inlineStr">
+          <t>2026-09-28 session, Michael "for later (placeholder)" optimization #3 (relaying from the Lab Members screen).</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
         <is>
           <t>Post-COLA. No customer urgency.
 ---</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="90" customHeight="1">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>52</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Medical Director seat via account-grant dropdown (designate / transfer MD)</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>Open, not started. Placeholder. Confirm the current MD-seat assignment path and the one-MD-per-location enforcement point before sizing.</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>S-M (1-3 days to ~1.5 weeks) — move MD-seat assignment onto the same per-memb...</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>Medium-High — the MD seat is a recurring friction point (Georgetown, SCAHC MD...</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>Michael, verbatim (2026-09-28): "The way we are doing the medical director seat is silly. Why not just use the account grant dropdown to give a medical director seat. If the person is already in, then we should just be able to grant the medical director seat the same way we promote people to admin or reduce them to staff as long as we only have 1 per location. Maybe do another block like the transfer ownership block as 'designate medical director or transfer medical director'." So: fold the MD seat into the existing member role dropdown (Admin / Staff / ... + Medical Director) with a single-MD-per-lab constraint, and add a dedicated designate-or-transfer-MD block that mirrors the transfer-ownership UX for changing the MD. Cross-ref [[project_medical_director_designation]] and the seat model.</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 session, Michael "for later (placeholder)" optimization #3 (relaying from the Lab Members screen).</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="inlineStr">
-        <is>
-          <t>Post-COLA. No customer urgency.
----</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:H18"/>
+  <autoFilter ref="A1:H16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1305,7 +1211,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H47"/>
+  <dimension ref="A1:H49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1363,66 +1269,64 @@
     <row r="2" ht="90" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>C45</t>
+          <t>C47</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Unify coverage/competency recurrence helper (was #49) - closed as non-issue</t>
+          <t>Unregulated-analyte / Alternative Assessment (AAA) coverage (was #18)</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr"/>
-      <c r="D2" s="2" t="inlineStr"/>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>was S (Phase 3) / Importance: Medium</t>
+        </is>
+      </c>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: Investigated 2026-09-24 before building. The coverage recurrence math (+6-month interval, signed-resets-to-missing, nextDueOn/overdue, isFailVerdict) is ALREADY single-source in server/veritacheckCoverage.ts (computeCoverageFrom). server/coverageReport.ts and the routes.ts coverage export do not recompute it; they consume the computed nextDueOn/overdue/status fields and apply small surface-specific presentation labels (deliberately different vocabularies per surface, so they should not be merged). The only truly identical duplicate is a one-line date formatter. The competency "owed" derivation is NOT the same cadence: competency follows the CLIA milestone schedule (initial / semiannual year 1 / annual, 42 CFR 493.1451(b)(8) and 493.1235), which is a different regulatory interval from the coverage 6-month rule (493.1281 / 493.1255) and must stay separate. No worthwhile extraction; merging the two cadences would be wrong. Closed 2026-09-24. (The year-1 competency-window refinement remains tracked separately as #50.)</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-24 session, "keep working" pass; scoped read-only, found no real duplication.
----</t>
-        </is>
-      </c>
+          <t>Effort: was S (Phase 3) / Importance: Medium</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr"/>
       <c r="H2" s="2" t="inlineStr"/>
     </row>
     <row r="3" ht="90" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>C46</t>
+          <t>C48</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Verified-users product-update send path (wrong-list incident fix)</t>
+          <t>VeritaResponse post-survey deficiency module (was #17)</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr"/>
-      <c r="D3" s="3" t="inlineStr"/>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>was XL / Importance: High</t>
+        </is>
+      </c>
       <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: Shipped PR #1324 (merged 4e05506a, deploy ACTIVE). New POST /api/admin/users/send targets registered VeritaAssure account holders (the users table), never the Lab Director's Briefing subscriber list. Separate explicitly-named endpoint (not a flag with a dangerous default), account-holder email framing, excludes suppressed emails and RFC-reserved test domains, CC owner, dryRun + testTo previews. Public unsubscribe now upserts a suppression row so opt-outs are honored across both audiences. Live dryRun: 49 verified-user recipients vs 673 on the Briefing list. Receipts: scripts/verify-product-update-send.mts 24/24, tsc clean, rendered sample inspected. Fixes the fallout from the 2026-09-23/24 wrong-list send (a product update went to the 675-person Briefing list). Nothing sends without Michael's explicit "send it."</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-24 session; Michael selected this as the next build after the #41 close.
----</t>
-        </is>
-      </c>
+          <t>Effort: was XL / Importance: High</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr"/>
       <c r="H3" s="3" t="inlineStr"/>
     </row>
     <row r="4" ht="90" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>C44</t>
+          <t>C45</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Verify-script convention backfill (was #41) + audit matcher fix</t>
+          <t>Unify coverage/competency recurrence helper (was #49) - closed as non-issue</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr"/>
@@ -1430,12 +1334,12 @@
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: #41 was fully backfilled on 2026-06-13 (all 8 high-stakes scripts landed; see C30); it had only been mis-filed in OPEN. A 2026-09-24 re-audit initially reported 4 of 5 recent math/logic commits as missing a verify script, which was a FALSE POSITIVE: scripts/audit_verify_script_coverage.py matched only scripts/verify-*.js / .cjs, so it ignored the .mjs / .mts / .ts verify scripts the repo now ships (e.g. verify-ptcoag-multi.mts, verify-tea-criterion-format.mjs). Fixed the matcher to accept .js/.cjs/.mjs/.ts/.mts; re-run shows 5 of 5 covered, 0 debt. The convention is being followed. Closed 2026-09-24.</t>
+          <t>Closure evidence: Investigated 2026-09-24 before building. The coverage recurrence math (+6-month interval, signed-resets-to-missing, nextDueOn/overdue, isFailVerdict) is ALREADY single-source in server/veritacheckCoverage.ts (computeCoverageFrom). server/coverageReport.ts and the routes.ts coverage export do not recompute it; they consume the computed nextDueOn/overdue/status fields and apply small surface-specific presentation labels (deliberately different vocabularies per surface, so they should not be merged). The only truly identical duplicate is a one-line date formatter. The competency "owed" derivation is NOT the same cadence: competency follows the CLIA milestone schedule (initial / semiannual year 1 / annual, 42 CFR 493.1451(b)(8) and 493.1235), which is a different regulatory interval from the coverage 6-month rule (493.1281 / 493.1255) and must stay separate. No worthwhile extraction; merging the two cadences would be wrong. Closed 2026-09-24. (The year-1 competency-window refinement remains tracked separately as #50.)</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 session, "keep working" pass; audit tooling bug found + fixed.
+          <t>2026-09-24 session, "keep working" pass; scoped read-only, found no real duplication.
 ---</t>
         </is>
       </c>
@@ -1444,12 +1348,12 @@
     <row r="5" ht="90" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>C43</t>
+          <t>C46</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>VeritaStaff instrument-centric (dual) assignment view</t>
+          <t>Verified-users product-update send path (wrong-list incident fix)</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr"/>
@@ -1457,12 +1361,12 @@
       <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1320. GET/PUT /staff/instruments/:id/employees (transpose of the per-employee endpoints); an "Assign by Instrument" dialog lets a director pick a test system or manual test and check off who runs it. Same staff_employee_instruments join, with the 42 CFR 493.1235(a) duty-change event emitted on newly-added pairs so both orientations trigger the same reassessment. GET verified live on SCAHC lab 2. Closed 2026-09-24.</t>
+          <t>Closure evidence: Shipped PR #1324 (merged 4e05506a, deploy ACTIVE). New POST /api/admin/users/send targets registered VeritaAssure account holders (the users table), never the Lab Director's Briefing subscriber list. Separate explicitly-named endpoint (not a flag with a dangerous default), account-holder email framing, excludes suppressed emails and RFC-reserved test domains, CC owner, dryRun + testTo previews. Public unsubscribe now upserts a suppression row so opt-outs are honored across both audiences. Live dryRun: 49 verified-user recipients vs 673 on the Briefing list. Receipts: scripts/verify-product-update-send.mts 24/24, tsc clean, rendered sample inspected. Fixes the fallout from the 2026-09-23/24 wrong-list send (a product update went to the 675-person Briefing list). Nothing sends without Michael's explicit "send it."</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>2026-09-24 session, Michael ("in staff we should also give the dual view when assigning coverage to test systems or manual tests").
+          <t>2026-09-24 session; Michael selected this as the next build after the #41 close.
 ---</t>
         </is>
       </c>
@@ -1471,12 +1375,12 @@
     <row r="6" ht="90" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>C42</t>
+          <t>C44</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>VeritaComp coverage map (required-vs-assessed matrix, dual view)</t>
+          <t>Verify-script convention backfill (was #41) + audit matcher fix</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr"/>
@@ -1484,12 +1388,12 @@
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1319 (+ status layer PR #1316). /competency/owed returns per-item assessed (locked passing assessment this cycle on a covering method group) + per-employee CLIA status; CompetencyCoverageMap renders a By-employee / By-instrument matrix (Assessed / Owed / Overdue / Gap). Verified live on SCAHC lab 2 (owed 116, assessed 2, gaps 0). Completes #48 as the VeritaCheck-parity coverage map. Closed 2026-09-24.</t>
+          <t>Closure evidence: #41 was fully backfilled on 2026-06-13 (all 8 high-stakes scripts landed; see C30); it had only been mis-filed in OPEN. A 2026-09-24 re-audit initially reported 4 of 5 recent math/logic commits as missing a verify script, which was a FALSE POSITIVE: scripts/audit_verify_script_coverage.py matched only scripts/verify-*.js / .cjs, so it ignored the .mjs / .mts / .ts verify scripts the repo now ships (e.g. verify-ptcoag-multi.mts, verify-tea-criterion-format.mjs). Fixed the matcher to accept .js/.cjs/.mjs/.ts/.mts; re-run shows 5 of 5 covered, 0 debt. The convention is being followed. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 session, Michael ("are we building the competencies to have a coverage map, same as veritacheck?" then "build it").
+          <t>2026-09-24 session, "keep working" pass; audit tooling bug found + fixed.
 ---</t>
         </is>
       </c>
@@ -1498,12 +1402,12 @@
     <row r="7" ht="90" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>C41</t>
+          <t>C43</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>VeritaCheck coverage recurrence (method comparison + cal-ver/linearity + reports)</t>
+          <t>VeritaStaff instrument-centric (dual) assignment view</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr"/>
@@ -1511,12 +1415,12 @@
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: PRs #1317 (method comparison), #1318 (cal-ver/linearity), #1321 (report Next-due columns). Periodic verification (correlation/method comparison 42 CFR 493.1281; cal-ver/linearity 42 CFR 493.1255; both 6-month) now recurs: a signed study banks the cycle and rolls to next-due = signed + 6 months instead of reading "done" forever. Status Missing/Failed/Completed-unsigned + a "Next due on" column on-screen and in both coverage exports; also credits the previously-ignored "correlation" study type. Root cause: computeCoverageFrom marked requirements done on mere existence, no date logic. Verified live on SCAHC lab 2 (101 correlations + 11 cal-ver rows now carry a next-due). Engine-level, all facilities. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1320. GET/PUT /staff/instruments/:id/employees (transpose of the per-employee endpoints); an "Assign by Instrument" dialog lets a director pick a test system or manual test and check off who runs it. Same staff_employee_instruments join, with the 42 CFR 493.1235(a) duty-change event emitted on newly-added pairs so both orientations trigger the same reassessment. GET verified live on SCAHC lab 2. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>2026-09-24 session, Michael ("Look at San Carlos... they finished their last set of correlations (all 103) but their menu never reset").
+          <t>2026-09-24 session, Michael ("in staff we should also give the dual view when assigning coverage to test systems or manual tests").
 ---</t>
         </is>
       </c>
@@ -1525,12 +1429,12 @@
     <row r="8" ht="90" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>C40</t>
+          <t>C42</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>VeritaComp Competencies Owed derived from VeritaStaff, with gap detection (was #48)</t>
+          <t>VeritaComp coverage map (required-vs-assessed matrix, dual view)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr"/>
@@ -1538,12 +1442,12 @@
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1314 (squash 2bcb0db9). GET /api/labs/:labId/competency/owed derives each VeritaStaff testing employee's owed competencies from their assigned instruments (staff_employee_instruments -&gt; veritamap_instruments + tests), on the CLIA timeline, and flags instruments not covered by any competency program as gaps. CompetenciesOwedSection renders it on the VeritaComp landing page. Reuses the shipped bridge + suggested-method-groups match rules; no new tables. Verified live on prod with real assignment data: 2 instruments assigned to a demo staffer produced owed=2, gaps=2 (HIGH, Technical Supervisor), then reverted cleanly. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1319 (+ status layer PR #1316). /competency/owed returns per-item assessed (locked passing assessment this cycle on a covering method group) + per-employee CLIA status; CompetencyCoverageMap renders a By-employee / By-instrument matrix (Assessed / Owed / Overdue / Gap). Verified live on SCAHC lab 2 (owed 116, assessed 2, gaps 0). Completes #48 as the VeritaCheck-parity coverage map. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23/24 session, Michael ("veritacomp bases what competencies they owe (currently untrue, but needs to be true)"). Option 1 (unify roster on VeritaStaff, match instruments by id).
+          <t>2026-09-24 session, Michael ("are we building the competencies to have a coverage map, same as veritacheck?" then "build it").
 ---</t>
         </is>
       </c>
@@ -1552,12 +1456,12 @@
     <row r="9" ht="90" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>C39</t>
+          <t>C41</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>VeritaScan line items can attach or link evidence (was #46)</t>
+          <t>VeritaCheck coverage recurrence (method comparison + cal-ver/linearity + reports)</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr"/>
@@ -1565,12 +1469,12 @@
       <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1312 (squash a1dda93d). VeritaScan scan checklist items now show linked evidence as chips (open link, remove) plus a writer "Link evidence" affordance whose picker links an existing VeritaDC/Library document; a shortcut deep-links to the Library for new (governed) documents. Reuses the already-shipped lab_documents + document_checklist_links + coverage endpoints (URL-pointer only, no file storage, no new tables). Browser-verified live on prod (scan 23): the affordance renders and the picker opens. Closed 2026-09-24.</t>
+          <t>Closure evidence: PRs #1317 (method comparison), #1318 (cal-ver/linearity), #1321 (report Next-due columns). Periodic verification (correlation/method comparison 42 CFR 493.1281; cal-ver/linearity 42 CFR 493.1255; both 6-month) now recurs: a signed study banks the cycle and rolls to next-due = signed + 6 months instead of reading "done" forever. Status Missing/Failed/Completed-unsigned + a "Next due on" column on-screen and in both coverage exports; also credits the previously-ignored "correlation" study type. Root cause: computeCoverageFrom marked requirements done on mere existence, no date logic. Verified live on SCAHC lab 2 (101 correlations + 11 cal-ver rows now carry a next-due). Engine-level, all facilities. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>2026-09-23 session, Michael. Recurring request. Companion: cross-module evidence display on the VeritaDC policy shipped in PR #1313 (by-target cross-links surfaced in the policy View modal, browser-verified live).
+          <t>2026-09-24 session, Michael ("Look at San Carlos... they finished their last set of correlations (all 103) but their menu never reset").
 ---</t>
         </is>
       </c>
@@ -1579,12 +1483,12 @@
     <row r="10" ht="90" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>C38</t>
+          <t>C40</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>VeritaTrack calendar month cells expand to reveal hidden tasks (was #45)</t>
+          <t>VeritaComp Competencies Owed derived from VeritaStaff, with gap detection (was #48)</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr"/>
@@ -1592,12 +1496,12 @@
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: VeritaTrack CalendarView month cells with more than three tasks now expand in place (chevron, "+N more" toggling to "Show less", due dates), so no task is hidden with no path to it (client/src/pages/VeritaTrackAppPage.tsx CalendarView). Shipped 2026-09-23. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1314 (squash 2bcb0db9). GET /api/labs/:labId/competency/owed derives each VeritaStaff testing employee's owed competencies from their assigned instruments (staff_employee_instruments -&gt; veritamap_instruments + tests), on the CLIA timeline, and flags instruments not covered by any competency program as gaps. CompetenciesOwedSection renders it on the VeritaComp landing page. Reuses the shipped bridge + suggested-method-groups match rules; no new tables. Verified live on prod with real assignment data: 2 instruments assigned to a demo staffer produced owed=2, gaps=2 (HIGH, Technical Supervisor), then reverted cleanly. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23 session, Michael screenshot of the VeritaTrack calendar (lab 3, September cell).
+          <t>2026-09-23/24 session, Michael ("veritacomp bases what competencies they owe (currently untrue, but needs to be true)"). Option 1 (unify roster on VeritaStaff, match instruments by id).
 ---</t>
         </is>
       </c>
@@ -1606,12 +1510,12 @@
     <row r="11" ht="90" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>C37</t>
+          <t>C39</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Long Excel column headers no longer clip CFR citations (was #44)</t>
+          <t>VeritaScan line items can attach or link evidence (was #46)</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr"/>
@@ -1619,12 +1523,12 @@
       <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. The VeritaMap export derives the header row height from the longest wrapped header via headerRowHeight(headers, colWidths) (server/routes.ts:15935) instead of a fixed 20, so "Reference Range Attestation (42 CFR 493.1253)" and the other long headers print in full. No new code this session. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1312 (squash a1dda93d). VeritaScan scan checklist items now show linked evidence as chips (open link, remove) plus a writer "Link evidence" affordance whose picker links an existing VeritaDC/Library document; a shortcut deep-links to the Library for new (governed) documents. Reuses the already-shipped lab_documents + document_checklist_links + coverage endpoints (URL-pointer only, no file storage, no new tables). Browser-verified live on prod (scan 23): the affordance renders and the picker opens. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+          <t>2026-09-23 session, Michael. Recurring request. Companion: cross-module evidence display on the VeritaDC policy shipped in PR #1313 (by-target cross-links surfaced in the policy View modal, browser-verified live).
 ---</t>
         </is>
       </c>
@@ -1633,12 +1537,12 @@
     <row r="12" ht="90" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>C36</t>
+          <t>C38</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>License stamp no longer clobbers the §6 header/footer or names the wrong lab (was #43)</t>
+          <t>VeritaTrack calendar month cells expand to reveal hidden tasks (was #45)</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr"/>
@@ -1646,12 +1550,12 @@
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. setHeaderFooter (shared/licenseExceljs.ts:155-209) now preserves an existing §6 header and appends (not overwrites) the footer left section, and customer-facing exports name the scoped lab: the VeritaScan library export reads req.scope.lab.name / clia_number (server/routes.ts:16572-16573), not the licensee. No new code this session (avoided regressing the existing fix). Closed 2026-09-24.</t>
+          <t>Closure evidence: VeritaTrack CalendarView month cells with more than three tasks now expand in place (chevron, "+N more" toggling to "Show less", due dates), so no task is hidden with no path to it (client/src/pages/VeritaTrackAppPage.tsx CalendarView). Shipped 2026-09-23. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+          <t>2026-09-23 session, Michael screenshot of the VeritaTrack calendar (lab 3, September cell).
 ---</t>
         </is>
       </c>
@@ -1660,18 +1564,72 @@
     <row r="13" ht="90" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>C34</t>
+          <t>C37</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Wire the two static-audit guards into CI (was #43)</t>
+          <t>Long Excel column headers no longer clip CFR citations (was #44)</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr"/>
       <c r="D13" s="3" t="inlineStr"/>
       <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. The VeritaMap export derives the header row height from the longest wrapped header via headerRowHeight(headers, colWidths) (server/routes.ts:15935) instead of a fixed 20, so "Reference Range Attestation (42 CFR 493.1253)" and the other long headers print in full. No new code this session. Closed 2026-09-24.</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+---</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14" ht="90" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>C36</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>License stamp no longer clobbers the §6 header/footer or names the wrong lab (was #43)</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr"/>
+      <c r="D14" s="2" t="inlineStr"/>
+      <c r="E14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. setHeaderFooter (shared/licenseExceljs.ts:155-209) now preserves an existing §6 header and appends (not overwrites) the footer left section, and customer-facing exports name the scoped lab: the VeritaScan library export reads req.scope.lab.name / clia_number (server/routes.ts:16572-16573), not the licensee. No new code this session (avoided regressing the existing fix). Closed 2026-09-24.</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+---</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15" ht="90" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>C34</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Wire the two static-audit guards into CI (was #43)</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr"/>
+      <c r="D15" s="3" t="inlineStr"/>
+      <c r="E15" s="3" t="inlineStr"/>
+      <c r="F15" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: both guards wired into the Multi-Lab Mutations Audit CI
 workflow (.github/workflows/multilab-mutations-audit.yml) as steps:
@@ -1683,24 +1641,24 @@
 (same caveat as the existing guards already in that workflow).</t>
         </is>
       </c>
-      <c r="G13" s="3" t="inlineStr"/>
-      <c r="H13" s="3" t="inlineStr"/>
-    </row>
-    <row r="14" ht="90" customHeight="1">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="G15" s="3" t="inlineStr"/>
+      <c r="H15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16" ht="90" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>C35</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>Legacy /api/studies over-returns studies across labs (was #44)</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr"/>
-      <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="2" t="inlineStr"/>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr"/>
+      <c r="D16" s="2" t="inlineStr"/>
+      <c r="E16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: GET /api/studies now scopes its list to the active lab
 when one is resolved from the Referer (server/routes.ts), so every returned row
@@ -1710,24 +1668,24 @@
 mirroring the /api/labs/:labId/studies handler. Closed 2026-06-14.</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr"/>
-      <c r="H14" s="2" t="inlineStr"/>
-    </row>
-    <row r="15" ht="90" customHeight="1">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr"/>
+      <c r="H16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17" ht="90" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>C30</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>Verify-script convention backfill (was #41)</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr"/>
-      <c r="D15" s="3" t="inlineStr"/>
-      <c r="E15" s="3" t="inlineStr"/>
-      <c r="F15" s="3" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr"/>
+      <c r="D17" s="3" t="inlineStr"/>
+      <c r="E17" s="3" t="inlineStr"/>
+      <c r="F17" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: all 8 high-stakes math/logic commits now ship a paired
 scripts/verify-*.js (EP17 sensitivity, Deming lot-to-lot, CUMSUM+QC+multi-analyte,
@@ -1735,30 +1693,30 @@
 TEa boundary), per the strike-throughs in #41. Closed 2026-06-13.</t>
         </is>
       </c>
-      <c r="G15" s="3" t="inlineStr">
+      <c r="G17" s="3" t="inlineStr">
         <is>
           <t>scripts/audit_verify_script_coverage.py lookback, 2026-06-02; backfills
 landed 2026-06-03..06.
 ---</t>
         </is>
       </c>
-      <c r="H15" s="3" t="inlineStr"/>
-    </row>
-    <row r="16" ht="90" customHeight="1">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="H17" s="3" t="inlineStr"/>
+    </row>
+    <row r="18" ht="90" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>C31</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>VeritaPT AAA create/update/delete silently no-op in the multi-lab UI</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr"/>
-      <c r="D16" s="2" t="inlineStr"/>
-      <c r="E16" s="2" t="inlineStr"/>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr"/>
+      <c r="D18" s="2" t="inlineStr"/>
+      <c r="E18" s="2" t="inlineStr"/>
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #754 (commit 92ad499) added lab-scoped POST/PUT/DELETE
 /api/labs/:labId/pt/aa-records. The UI posted to the lab-scoped path but only GET
@@ -1769,30 +1727,30 @@
 route mis-filed records to the user's default lab on multi-lab accounts).</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>2026-06-13, found during #18 Phase 3 QA;
 scripts/audit-labscoped-write-routes.mjs now guards the class.
 ---</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr"/>
-    </row>
-    <row r="17" ht="90" customHeight="1">
-      <c r="A17" s="3" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19" ht="90" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>C32</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>VeritaComp "Unlock assessment" false-success no-op</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr"/>
-      <c r="D17" s="3" t="inlineStr"/>
-      <c r="E17" s="3" t="inlineStr"/>
-      <c r="F17" s="3" t="inlineStr">
+      <c r="C19" s="3" t="inlineStr"/>
+      <c r="D19" s="3" t="inlineStr"/>
+      <c r="E19" s="3" t="inlineStr"/>
+      <c r="F19" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #755 (commit 4234007) moved the unlock route to
 /api/labs/:labId/competency/assessments/:id/unlock (the path the client calls).
@@ -1803,29 +1761,29 @@
 HTML).</t>
         </is>
       </c>
-      <c r="G17" s="3" t="inlineStr">
+      <c r="G19" s="3" t="inlineStr">
         <is>
           <t>2026-06-13, found by scripts/audit-labscoped-write-routes.mjs.
 ---</t>
         </is>
       </c>
-      <c r="H17" s="3" t="inlineStr"/>
-    </row>
-    <row r="18" ht="90" customHeight="1">
-      <c r="A18" s="2" t="inlineStr">
+      <c r="H19" s="3" t="inlineStr"/>
+    </row>
+    <row r="20" ht="90" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>C33</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>FK-cascade delete 500s + NavBar laptop-width overflow</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr"/>
-      <c r="D18" s="2" t="inlineStr"/>
-      <c r="E18" s="2" t="inlineStr"/>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr"/>
+      <c r="D20" s="2" t="inlineStr"/>
+      <c r="E20" s="2" t="inlineStr"/>
+      <c r="F20" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PRs #749/#750 fixed NavBar horizontal overflow at laptop
 widths (collapse to the hamburger below 1560px); prod-verified at 1280-1920 with the
@@ -1836,57 +1794,57 @@
 500 -&gt; 200. scripts/audit-delete-cascades.mjs guards the class.</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="G20" s="2" t="inlineStr">
         <is>
           <t>2026-06-13 browser QA of the A7-D4 wave + retro-QC of the 72h PR window.
 ---</t>
         </is>
       </c>
-      <c r="H18" s="2" t="inlineStr"/>
-    </row>
-    <row r="19" ht="90" customHeight="1">
-      <c r="A19" s="3" t="inlineStr">
+      <c r="H20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21" ht="90" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>C1</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>FAQ "over 25 years" -&gt; "over 23 years"</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr"/>
-      <c r="D19" s="3" t="inlineStr"/>
-      <c r="E19" s="3" t="inlineStr"/>
-      <c r="F19" s="3" t="inlineStr">
+      <c r="C21" s="3" t="inlineStr"/>
+      <c r="D21" s="3" t="inlineStr"/>
+      <c r="E21" s="3" t="inlineStr"/>
+      <c r="F21" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: client/src/pages/FAQPage.tsx line 20 reads "over
 23 years" as of 2026-05-01.</t>
         </is>
       </c>
-      <c r="G19" s="3" t="inlineStr">
+      <c r="G21" s="3" t="inlineStr">
         <is>
           <t>session 299e9a73 turn 14, ~2026-04-28.
 ---</t>
         </is>
       </c>
-      <c r="H19" s="3" t="inlineStr"/>
-    </row>
-    <row r="20" ht="90" customHeight="1">
-      <c r="A20" s="2" t="inlineStr">
+      <c r="H21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22" ht="90" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>C5</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B22" s="2" t="inlineStr">
         <is>
           <t>David's VeritaQA grey-button bug (seat permissions mode)</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr"/>
-      <c r="D20" s="2" t="inlineStr"/>
-      <c r="E20" s="2" t="inlineStr"/>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="C22" s="2" t="inlineStr"/>
+      <c r="D22" s="2" t="inlineStr"/>
+      <c r="E22" s="2" t="inlineStr"/>
+      <c r="F22" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #10 squash-merged as commit a43fbba on
 2026-05-01 23:19 MST. Railway deploy succeeded; deployed bundle
@@ -1899,7 +1857,7 @@
 against his exact stored shape (14 of 14 expected outcomes matched).</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr">
+      <c r="G22" s="2" t="inlineStr">
         <is>
           <t>2026-05-01 David's report; veritabench + veritastock
 weren't in MODULE_LIST so seat permissions silently defaulted to
@@ -1907,75 +1865,17 @@
 ---</t>
         </is>
       </c>
-      <c r="H20" s="2" t="inlineStr"/>
-    </row>
-    <row r="21" ht="90" customHeight="1">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>C2</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>TeamPage present-tense "TJC surveyor" check</t>
-        </is>
-      </c>
-      <c r="C21" s="3" t="inlineStr"/>
-      <c r="D21" s="3" t="inlineStr"/>
-      <c r="E21" s="3" t="inlineStr"/>
-      <c r="F21" s="3" t="inlineStr">
-        <is>
-          <t>Closure evidence: site-wide search confirmed all surveyor language
-is past-tense, consistent with user's 2021-2025 service. User closed
-the item in session 299e9a73 turn 4.</t>
-        </is>
-      </c>
-      <c r="G21" s="3" t="inlineStr">
-        <is>
-          <t>session 299e9a73, ~2026-04-28.
----</t>
-        </is>
-      </c>
-      <c r="H21" s="3" t="inlineStr"/>
-    </row>
-    <row r="22" ht="90" customHeight="1">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>C3</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>My Studies CSV/XLSX export (John as design partner)</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr"/>
-      <c r="D22" s="2" t="inlineStr"/>
-      <c r="E22" s="2" t="inlineStr"/>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>Closure evidence: client/src/pages/DashboardPage.tsx line 46 calls
-/api/my-studies/export. server/routes.ts line 1491 implements the
-endpoint. Pulled forward into pre-COLA per user instruction.</t>
-        </is>
-      </c>
-      <c r="G22" s="2" t="inlineStr">
-        <is>
-          <t>session 299e9a73 turn 5, ~2026-04-28.
----</t>
-        </is>
-      </c>
       <c r="H22" s="2" t="inlineStr"/>
     </row>
     <row r="23" ht="90" customHeight="1">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>C4</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Rotate GitHub PAT (because old PAT was committed in SESSION_HANDOFF files)</t>
+          <t>TeamPage present-tense "TJC surveyor" check</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr"/>
@@ -1983,8 +1883,9 @@
       <c r="E23" s="3" t="inlineStr"/>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: no ghp_* or github_pat_* patterns in current
-SESSION_HANDOFF.md or SESSION_HANDOFF-2.md as of 2026-05-01.</t>
+          <t>Closure evidence: site-wide search confirmed all surveyor language
+is past-tense, consistent with user's 2021-2025 service. User closed
+the item in session 299e9a73 turn 4.</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -1998,18 +1899,75 @@
     <row r="24" ht="90" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>C6</t>
+          <t>C3</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>VeritaPolicy service-line filtering removed (formerly #4)</t>
+          <t>My Studies CSV/XLSX export (John as design partner)</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr"/>
       <c r="D24" s="2" t="inlineStr"/>
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Closure evidence: client/src/pages/DashboardPage.tsx line 46 calls
+/api/my-studies/export. server/routes.ts line 1491 implements the
+endpoint. Pulled forward into pre-COLA per user instruction.</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>session 299e9a73 turn 5, ~2026-04-28.
+---</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25" ht="90" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Rotate GitHub PAT (because old PAT was committed in SESSION_HANDOFF files)</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr"/>
+      <c r="D25" s="3" t="inlineStr"/>
+      <c r="E25" s="3" t="inlineStr"/>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>Closure evidence: no ghp_* or github_pat_* patterns in current
+SESSION_HANDOFF.md or SESSION_HANDOFF-2.md as of 2026-05-01.</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>session 299e9a73, ~2026-04-28.
+---</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26" ht="90" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>C6</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>VeritaPolicy service-line filtering removed (formerly #4)</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr"/>
+      <c r="D26" s="2" t="inlineStr"/>
+      <c r="E26" s="2" t="inlineStr"/>
+      <c r="F26" s="2" t="inlineStr">
         <is>
           <t>Closure rationale (operator decision 2026-05-10): Keep all
 VeritaPolicy rows. CFR-only references with no accreditor reference
@@ -2018,29 +1976,29 @@
 report misread the design intent.</t>
         </is>
       </c>
-      <c r="G24" s="2" t="inlineStr">
+      <c r="G26" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H24" s="2" t="inlineStr"/>
-    </row>
-    <row r="25" ht="90" customHeight="1">
-      <c r="A25" s="3" t="inlineStr">
+      <c r="H26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27" ht="90" customHeight="1">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>C7</t>
         </is>
       </c>
-      <c r="B25" s="3" t="inlineStr">
+      <c r="B27" s="3" t="inlineStr">
         <is>
           <t>CLIA number format validation (formerly #13)</t>
         </is>
       </c>
-      <c r="C25" s="3" t="inlineStr"/>
-      <c r="D25" s="3" t="inlineStr"/>
-      <c r="E25" s="3" t="inlineStr"/>
-      <c r="F25" s="3" t="inlineStr">
+      <c r="C27" s="3" t="inlineStr"/>
+      <c r="D27" s="3" t="inlineStr"/>
+      <c r="E27" s="3" t="inlineStr"/>
+      <c r="F27" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: shared/validateClia.ts defines CLIA_REGEX =
 /^\d{2}D\d{7}$/ (line 24), validateClia() helper with whitespace
@@ -2051,30 +2009,30 @@
 shape exists and behaves as specified.</t>
         </is>
       </c>
-      <c r="G25" s="3" t="inlineStr">
+      <c r="G27" s="3" t="inlineStr">
         <is>
           <t>Agent verification 2026-05-10 via grep + file read.
 Operator confirmed shipped 2026-05-10.
 ---</t>
         </is>
       </c>
-      <c r="H25" s="3" t="inlineStr"/>
-    </row>
-    <row r="26" ht="90" customHeight="1">
-      <c r="A26" s="2" t="inlineStr">
+      <c r="H27" s="3" t="inlineStr"/>
+    </row>
+    <row r="28" ht="90" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>C8</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="B28" s="2" t="inlineStr">
         <is>
           <t>VeritaMap lab-wide menu toggle (formerly #19)</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr"/>
-      <c r="D26" s="2" t="inlineStr"/>
-      <c r="E26" s="2" t="inlineStr"/>
-      <c r="F26" s="2" t="inlineStr">
+      <c r="C28" s="2" t="inlineStr"/>
+      <c r="D28" s="2" t="inlineStr"/>
+      <c r="E28" s="2" t="inlineStr"/>
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: client/src/pages/VeritaMapLabwidePage.tsx
 exists and implements the labwide read-only union view. Route is
@@ -2084,59 +2042,59 @@
 parking lot plan (read-only union view, per-session toggle) shipped.</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr">
+      <c r="G28" s="2" t="inlineStr">
         <is>
           <t>Agent verification 2026-05-10 via grep + file read.
 Operator confirmed shipped 2026-05-10.
 ---</t>
         </is>
       </c>
-      <c r="H26" s="2" t="inlineStr"/>
-    </row>
-    <row r="27" ht="90" customHeight="1">
-      <c r="A27" s="3" t="inlineStr">
+      <c r="H28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29" ht="90" customHeight="1">
+      <c r="A29" s="3" t="inlineStr">
         <is>
           <t>C9</t>
         </is>
       </c>
-      <c r="B27" s="3" t="inlineStr">
+      <c r="B29" s="3" t="inlineStr">
         <is>
           <t>Tier-1 smoke test checklist (formerly #6)</t>
         </is>
       </c>
-      <c r="C27" s="3" t="inlineStr"/>
-      <c r="D27" s="3" t="inlineStr"/>
-      <c r="E27" s="3" t="inlineStr"/>
-      <c r="F27" s="3" t="inlineStr">
+      <c r="C29" s="3" t="inlineStr"/>
+      <c r="D29" s="3" t="inlineStr"/>
+      <c r="E29" s="3" t="inlineStr"/>
+      <c r="F29" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: docs/smoke-test-tier1.md documents the Tier-1
 smoke-test process and post-deploy verification steps. Shipped via
 PR #81 as part of the 2026-05-10 wave.</t>
         </is>
       </c>
-      <c r="G27" s="3" t="inlineStr">
+      <c r="G29" s="3" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H27" s="3" t="inlineStr"/>
-    </row>
-    <row r="28" ht="90" customHeight="1">
-      <c r="A28" s="2" t="inlineStr">
+      <c r="H29" s="3" t="inlineStr"/>
+    </row>
+    <row r="30" ht="90" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>C10</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="B30" s="2" t="inlineStr">
         <is>
           <t>Per-module gating (formerly #7)</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr"/>
-      <c r="D28" s="2" t="inlineStr"/>
-      <c r="E28" s="2" t="inlineStr"/>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="C30" s="2" t="inlineStr"/>
+      <c r="D30" s="2" t="inlineStr"/>
+      <c r="E30" s="2" t="inlineStr"/>
+      <c r="F30" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: Client-side useIsReadOnly module keys wired
 on client/src/pages/VeritaPolicyAppPage.tsx and
@@ -2151,29 +2109,29 @@
 PR #76.</t>
         </is>
       </c>
-      <c r="G28" s="2" t="inlineStr">
+      <c r="G30" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H28" s="2" t="inlineStr"/>
-    </row>
-    <row r="29" ht="90" customHeight="1">
-      <c r="A29" s="3" t="inlineStr">
+      <c r="H30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31" ht="90" customHeight="1">
+      <c r="A31" s="3" t="inlineStr">
         <is>
           <t>C11</t>
         </is>
       </c>
-      <c r="B29" s="3" t="inlineStr">
+      <c r="B31" s="3" t="inlineStr">
         <is>
           <t>VeritaStock shipped copy (formerly #8)</t>
         </is>
       </c>
-      <c r="C29" s="3" t="inlineStr"/>
-      <c r="D29" s="3" t="inlineStr"/>
-      <c r="E29" s="3" t="inlineStr"/>
-      <c r="F29" s="3" t="inlineStr">
+      <c r="C31" s="3" t="inlineStr"/>
+      <c r="D31" s="3" t="inlineStr"/>
+      <c r="E31" s="3" t="inlineStr"/>
+      <c r="F31" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: client/src/pages/ArticleInventoryManagementPage.tsx
 line 305 footer reads "platform that includes VeritaStock™" instead
@@ -2181,29 +2139,29 @@
 on /resources/laboratory-inventory-management. Shipped via PR #75.</t>
         </is>
       </c>
-      <c r="G29" s="3" t="inlineStr">
+      <c r="G31" s="3" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H29" s="3" t="inlineStr"/>
-    </row>
-    <row r="30" ht="90" customHeight="1">
-      <c r="A30" s="2" t="inlineStr">
+      <c r="H31" s="3" t="inlineStr"/>
+    </row>
+    <row r="32" ht="90" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t>C12</t>
         </is>
       </c>
-      <c r="B30" s="2" t="inlineStr">
+      <c r="B32" s="2" t="inlineStr">
         <is>
           <t>Admin report one-row-per-lab (formerly #14)</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr"/>
-      <c r="D30" s="2" t="inlineStr"/>
-      <c r="E30" s="2" t="inlineStr"/>
-      <c r="F30" s="2" t="inlineStr">
+      <c r="C32" s="2" t="inlineStr"/>
+      <c r="D32" s="2" t="inlineStr"/>
+      <c r="E32" s="2" t="inlineStr"/>
+      <c r="F32" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: /api/admin/report rewritten in
 server/routes.ts (~line 595) to LEFT JOIN labs on
@@ -2218,56 +2176,56 @@
 prerequisite, not a code bug). Shipped via PR #85.</t>
         </is>
       </c>
-      <c r="G30" s="2" t="inlineStr">
+      <c r="G32" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H30" s="2" t="inlineStr"/>
-    </row>
-    <row r="31" ht="90" customHeight="1">
-      <c r="A31" s="3" t="inlineStr">
+      <c r="H32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33" ht="90" customHeight="1">
+      <c r="A33" s="3" t="inlineStr">
         <is>
           <t>C14</t>
         </is>
       </c>
-      <c r="B31" s="3" t="inlineStr">
+      <c r="B33" s="3" t="inlineStr">
         <is>
           <t>UI relabel "CLIA TEa" -&gt; "Lab-Set Internal Goal" (formerly #1)</t>
         </is>
       </c>
-      <c r="C31" s="3" t="inlineStr"/>
-      <c r="D31" s="3" t="inlineStr"/>
-      <c r="E31" s="3" t="inlineStr"/>
-      <c r="F31" s="3" t="inlineStr">
+      <c r="C33" s="3" t="inlineStr"/>
+      <c r="D33" s="3" t="inlineStr"/>
+      <c r="E33" s="3" t="inlineStr"/>
+      <c r="F33" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: Shipped across four PRs over 2026-05-10.</t>
         </is>
       </c>
-      <c r="G31" s="3" t="inlineStr">
+      <c r="G33" s="3" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H31" s="3" t="inlineStr"/>
-    </row>
-    <row r="32" ht="90" customHeight="1">
-      <c r="A32" s="2" t="inlineStr">
+      <c r="H33" s="3" t="inlineStr"/>
+    </row>
+    <row r="34" ht="90" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
         <is>
           <t>C13</t>
         </is>
       </c>
-      <c r="B32" s="2" t="inlineStr">
+      <c r="B34" s="2" t="inlineStr">
         <is>
           <t>WSLH PT vendor (formerly #15)</t>
         </is>
       </c>
-      <c r="C32" s="2" t="inlineStr"/>
-      <c r="D32" s="2" t="inlineStr"/>
-      <c r="E32" s="2" t="inlineStr"/>
-      <c r="F32" s="2" t="inlineStr">
+      <c r="C34" s="2" t="inlineStr"/>
+      <c r="D34" s="2" t="inlineStr"/>
+      <c r="E34" s="2" t="inlineStr"/>
+      <c r="F34" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: Shipped 2026-05-10 via PR #79 (merge commit
 eeebc6e; merged after rebase to resolve a server/db.ts collision
@@ -2285,68 +2243,9 @@
 'WSLH' is the post-deploy success signal. Shipped via PR #79.</t>
         </is>
       </c>
-      <c r="G32" s="2" t="inlineStr">
+      <c r="G34" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
----</t>
-        </is>
-      </c>
-      <c r="H32" s="2" t="inlineStr"/>
-    </row>
-    <row r="33" ht="90" customHeight="1">
-      <c r="A33" s="3" t="inlineStr">
-        <is>
-          <t>C15</t>
-        </is>
-      </c>
-      <c r="B33" s="3" t="inlineStr">
-        <is>
-          <t>VeritaStock lot tracking + expiration + reorder alerts (formerly #21)</t>
-        </is>
-      </c>
-      <c r="C33" s="3" t="inlineStr"/>
-      <c r="D33" s="3" t="inlineStr"/>
-      <c r="E33" s="3" t="inlineStr"/>
-      <c r="F33" s="3" t="inlineStr">
-        <is>
-          <t>Closure evidence: VeritaStock™ shipped the bench-level inventory
-features the Perplexity competitor analysis identified as a gap:</t>
-        </is>
-      </c>
-      <c r="G33" s="3" t="inlineStr">
-        <is>
-          <t>Originally Perplexity competitor analysis 2026-05-10.
-Audit 2026-05-21 confirmed the feature set ships today.
----</t>
-        </is>
-      </c>
-      <c r="H33" s="3" t="inlineStr"/>
-    </row>
-    <row r="34" ht="90" customHeight="1">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>C16</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>PAL studies guided workflow (formerly #23)</t>
-        </is>
-      </c>
-      <c r="C34" s="2" t="inlineStr"/>
-      <c r="D34" s="2" t="inlineStr"/>
-      <c r="E34" s="2" t="inlineStr"/>
-      <c r="F34" s="2" t="inlineStr">
-        <is>
-          <t>Closure evidence: VeritaCheck™ already ships the Precision /
-Accuracy / Linearity (PAL) study set under EP-protocol naming:</t>
-        </is>
-      </c>
-      <c r="G34" s="2" t="inlineStr">
-        <is>
-          <t>Originally Perplexity competitor analysis 2026-05-10.
-Audit 2026-05-21 confirmed the EP studies cover the PAL framing in
-full.
 ---</t>
         </is>
       </c>
@@ -2355,12 +2254,12 @@
     <row r="35" ht="90" customHeight="1">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>C17</t>
+          <t>C15</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>Source-grounded 21/29/45 CFR + 42 CFR 482-485 (formerly #26)</t>
+          <t>VeritaStock lot tracking + expiration + reorder alerts (formerly #21)</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr"/>
@@ -2368,35 +2267,94 @@
       <c r="E35" s="3" t="inlineStr"/>
       <c r="F35" s="3" t="inlineStr">
         <is>
+          <t>Closure evidence: VeritaStock™ shipped the bench-level inventory
+features the Perplexity competitor analysis identified as a gap:</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>Originally Perplexity competitor analysis 2026-05-10.
+Audit 2026-05-21 confirmed the feature set ships today.
+---</t>
+        </is>
+      </c>
+      <c r="H35" s="3" t="inlineStr"/>
+    </row>
+    <row r="36" ht="90" customHeight="1">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>C16</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>PAL studies guided workflow (formerly #23)</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr"/>
+      <c r="D36" s="2" t="inlineStr"/>
+      <c r="E36" s="2" t="inlineStr"/>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Closure evidence: VeritaCheck™ already ships the Precision /
+Accuracy / Linearity (PAL) study set under EP-protocol naming:</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>Originally Perplexity competitor analysis 2026-05-10.
+Audit 2026-05-21 confirmed the EP studies cover the PAL framing in
+full.
+---</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr"/>
+    </row>
+    <row r="37" ht="90" customHeight="1">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>C17</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>Source-grounded 21/29/45 CFR + 42 CFR 482-485 (formerly #26)</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr"/>
+      <c r="D37" s="3" t="inlineStr"/>
+      <c r="E37" s="3" t="inlineStr"/>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
           <t>Closure evidence: PR #301 (commit 8c27806, merged 2026-05-21)
 source-grounded the 74 remaining non-493 entries in
 server/cfrRequirements.ts against verbatim eCFR XML. Breakdown
 shipped:</t>
         </is>
       </c>
-      <c r="G35" s="3" t="inlineStr">
+      <c r="G37" s="3" t="inlineStr">
         <is>
           <t>PR #301; tasks #18 in the in-session task tracker.
 ---</t>
         </is>
       </c>
-      <c r="H35" s="3" t="inlineStr"/>
-    </row>
-    <row r="36" ht="90" customHeight="1">
-      <c r="A36" s="2" t="inlineStr">
+      <c r="H37" s="3" t="inlineStr"/>
+    </row>
+    <row r="38" ht="90" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
         <is>
           <t>C18</t>
         </is>
       </c>
-      <c r="B36" s="2" t="inlineStr">
+      <c r="B38" s="2" t="inlineStr">
         <is>
           <t>VeritaPolicy "Non CLIA" chapter rename (formerly #3)</t>
         </is>
       </c>
-      <c r="C36" s="2" t="inlineStr"/>
-      <c r="D36" s="2" t="inlineStr"/>
-      <c r="E36" s="2" t="inlineStr"/>
-      <c r="F36" s="2" t="inlineStr">
+      <c r="C38" s="2" t="inlineStr"/>
+      <c r="D38" s="2" t="inlineStr"/>
+      <c r="E38" s="2" t="inlineStr"/>
+      <c r="F38" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #300 (commit 34d7707, merged 2026-05-21)
 renamed all 44 user-facing chapter labels in
@@ -2407,7 +2365,7 @@
 page.</t>
         </is>
       </c>
-      <c r="G36" s="2" t="inlineStr">
+      <c r="G38" s="2" t="inlineStr">
         <is>
           <t>CAP customer screenshot of the /veritapolicy chapter
 headers, 2026-05-01 evening. PR #300; tasks #17 in the in-session
@@ -2415,23 +2373,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H36" s="2" t="inlineStr"/>
-    </row>
-    <row r="37" ht="90" customHeight="1">
-      <c r="A37" s="3" t="inlineStr">
+      <c r="H38" s="2" t="inlineStr"/>
+    </row>
+    <row r="39" ht="90" customHeight="1">
+      <c r="A39" s="3" t="inlineStr">
         <is>
           <t>C19</t>
         </is>
       </c>
-      <c r="B37" s="3" t="inlineStr">
+      <c r="B39" s="3" t="inlineStr">
         <is>
           <t>VeritaStock department-scope toggle (formerly #31)</t>
         </is>
       </c>
-      <c r="C37" s="3" t="inlineStr"/>
-      <c r="D37" s="3" t="inlineStr"/>
-      <c r="E37" s="3" t="inlineStr"/>
-      <c r="F37" s="3" t="inlineStr">
+      <c r="C39" s="3" t="inlineStr"/>
+      <c r="D39" s="3" t="inlineStr"/>
+      <c r="E39" s="3" t="inlineStr"/>
+      <c r="F39" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #319 (commit d01f5fe, merged 2026-05-22)
 shipped the persistent dept-scope toggle on VeritaStockPage. A new
@@ -2442,7 +2400,7 @@
 workspace without re-filtering.</t>
         </is>
       </c>
-      <c r="G37" s="3" t="inlineStr">
+      <c r="G39" s="3" t="inlineStr">
         <is>
           <t>John, San Carlos lab, 2026-05-21. Same conversation that
 drove the vendor dropdown (PR #304), FILTERED VIEW banner (PR #305),
@@ -2450,23 +2408,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H37" s="3" t="inlineStr"/>
-    </row>
-    <row r="38" ht="90" customHeight="1">
-      <c r="A38" s="2" t="inlineStr">
+      <c r="H39" s="3" t="inlineStr"/>
+    </row>
+    <row r="40" ht="90" customHeight="1">
+      <c r="A40" s="2" t="inlineStr">
         <is>
           <t>C20</t>
         </is>
       </c>
-      <c r="B38" s="2" t="inlineStr">
+      <c r="B40" s="2" t="inlineStr">
         <is>
           <t>Primary-lab seat counting (formerly #12)</t>
         </is>
       </c>
-      <c r="C38" s="2" t="inlineStr"/>
-      <c r="D38" s="2" t="inlineStr"/>
-      <c r="E38" s="2" t="inlineStr"/>
-      <c r="F38" s="2" t="inlineStr">
+      <c r="C40" s="2" t="inlineStr"/>
+      <c r="D40" s="2" t="inlineStr"/>
+      <c r="E40" s="2" t="inlineStr"/>
+      <c r="F40" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: is_primary_lab INTEGER NOT NULL DEFAULT 0
 column was added to the lab_members table at db.ts:1276, with the
@@ -2477,7 +2435,7 @@
 is_primary_lab=1 ordering).</t>
         </is>
       </c>
-      <c r="G38" s="2" t="inlineStr">
+      <c r="G40" s="2" t="inlineStr">
         <is>
           <t>2026-05-07 multi-lab discussion. Build shipped as part
 of the Multi-Lab Tier 2 architecture work (Phase 3.x series, prior
@@ -2486,23 +2444,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H38" s="2" t="inlineStr"/>
-    </row>
-    <row r="39" ht="90" customHeight="1">
-      <c r="A39" s="3" t="inlineStr">
+      <c r="H40" s="2" t="inlineStr"/>
+    </row>
+    <row r="41" ht="90" customHeight="1">
+      <c r="A41" s="3" t="inlineStr">
         <is>
           <t>C21</t>
         </is>
       </c>
-      <c r="B39" s="3" t="inlineStr">
+      <c r="B41" s="3" t="inlineStr">
         <is>
           <t>Multi-lab pricing model — Option A (formerly #11)</t>
         </is>
       </c>
-      <c r="C39" s="3" t="inlineStr"/>
-      <c r="D39" s="3" t="inlineStr"/>
-      <c r="E39" s="3" t="inlineStr"/>
-      <c r="F39" s="3" t="inlineStr">
+      <c r="C41" s="3" t="inlineStr"/>
+      <c r="D41" s="3" t="inlineStr"/>
+      <c r="E41" s="3" t="inlineStr"/>
+      <c r="F41" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #322 (commit 0ccd925, merged 2026-05-22)
 added the customer-facing line to the pricing page that reflects
@@ -2515,7 +2473,7 @@
 Enterprise+ block, reads:</t>
         </is>
       </c>
-      <c r="G39" s="3" t="inlineStr">
+      <c r="G41" s="3" t="inlineStr">
         <is>
           <t>2026-05-07 multi-lab discussion (Lisa Veri's
 canonical-case session). PR #322 (initial build); softening PR
@@ -2524,30 +2482,30 @@
 ---</t>
         </is>
       </c>
-      <c r="H39" s="3" t="inlineStr"/>
-    </row>
-    <row r="40" ht="90" customHeight="1">
-      <c r="A40" s="2" t="inlineStr">
+      <c r="H41" s="3" t="inlineStr"/>
+    </row>
+    <row r="42" ht="90" customHeight="1">
+      <c r="A42" s="2" t="inlineStr">
         <is>
           <t>C22</t>
         </is>
       </c>
-      <c r="B40" s="2" t="inlineStr">
+      <c r="B42" s="2" t="inlineStr">
         <is>
           <t>VeritaOps cost-per-test module (formerly #10)</t>
         </is>
       </c>
-      <c r="C40" s="2" t="inlineStr"/>
-      <c r="D40" s="2" t="inlineStr"/>
-      <c r="E40" s="2" t="inlineStr"/>
-      <c r="F40" s="2" t="inlineStr">
+      <c r="C42" s="2" t="inlineStr"/>
+      <c r="D42" s="2" t="inlineStr"/>
+      <c r="E42" s="2" t="inlineStr"/>
+      <c r="F42" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: v1 of the VeritaOps Cost-Per-Reportable-Test
 (CPRT) module shipped across PR #325 through PR #330 on 2026-05-22.
 The module is feature-complete for the typical lab director workflow.</t>
         </is>
       </c>
-      <c r="G40" s="2" t="inlineStr">
+      <c r="G42" s="2" t="inlineStr">
         <is>
           <t>This thread, 2026-05-07 12:05 PM CDT, user message:
 "Parking lot: build an operations module for cost per test
@@ -2556,262 +2514,262 @@
 ---</t>
         </is>
       </c>
-      <c r="H40" s="2" t="inlineStr"/>
-    </row>
-    <row r="41" ht="90" customHeight="1">
-      <c r="A41" s="3" t="inlineStr">
+      <c r="H42" s="2" t="inlineStr"/>
+    </row>
+    <row r="43" ht="90" customHeight="1">
+      <c r="A43" s="3" t="inlineStr">
         <is>
           <t>C23</t>
         </is>
       </c>
-      <c r="B41" s="3" t="inlineStr">
+      <c r="B43" s="3" t="inlineStr">
         <is>
           <t>CCL lab name visual disambiguation in lab switcher (formerly #34)</t>
         </is>
       </c>
-      <c r="C41" s="3" t="inlineStr"/>
-      <c r="D41" s="3" t="inlineStr">
+      <c r="C43" s="3" t="inlineStr"/>
+      <c r="D43" s="3" t="inlineStr">
         <is>
           <t>XS (under 1 day, actual)</t>
         </is>
       </c>
-      <c r="E41" s="3" t="inlineStr">
+      <c r="E43" s="3" t="inlineStr">
         <is>
           <t>Low — cosmetic; only mattered when Lisa or Michael picked the wrong lab from...</t>
         </is>
       </c>
-      <c r="F41" s="3" t="inlineStr">
+      <c r="F43" s="3" t="inlineStr">
         <is>
           <t>Effort: XS (under 1 day, actual)
 Importance: Low — cosmetic; only mattered when Lisa or Michael picked the wrong lab from the dropdown.</t>
         </is>
       </c>
-      <c r="G41" s="3" t="inlineStr">
+      <c r="G43" s="3" t="inlineStr">
         <is>
           <t>flagged 2026-05-23 immediately after provisioning Lisa's CCL lab; closed 2026-05-24.
 ---</t>
         </is>
       </c>
-      <c r="H41" s="3" t="inlineStr"/>
-    </row>
-    <row r="42" ht="90" customHeight="1">
-      <c r="A42" s="2" t="inlineStr">
+      <c r="H43" s="3" t="inlineStr"/>
+    </row>
+    <row r="44" ht="90" customHeight="1">
+      <c r="A44" s="2" t="inlineStr">
         <is>
           <t>C24</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
+      <c r="B44" s="2" t="inlineStr">
         <is>
           <t>VC Unlimited Y1/Y2 price disclosure UX (formerly #35)</t>
         </is>
       </c>
-      <c r="C42" s="2" t="inlineStr"/>
-      <c r="D42" s="2" t="inlineStr">
+      <c r="C44" s="2" t="inlineStr"/>
+      <c r="D44" s="2" t="inlineStr">
         <is>
           <t>XS (under 1 day, actual)</t>
         </is>
       </c>
-      <c r="E42" s="2" t="inlineStr">
+      <c r="E44" s="2" t="inlineStr">
         <is>
           <t>Low when shipped (proactive, no customer complaint yet) — but high if a procu...</t>
         </is>
       </c>
-      <c r="F42" s="2" t="inlineStr">
+      <c r="F44" s="2" t="inlineStr">
         <is>
           <t>Effort: XS (under 1 day, actual)
 Importance: Low when shipped (proactive, no customer complaint yet) — but high if a procurement reviewer later disputes the $499 renewal as undisclosed.</t>
         </is>
       </c>
-      <c r="G42" s="2" t="inlineStr">
+      <c r="G44" s="2" t="inlineStr">
         <is>
           <t>Pricing rebuild 2026-05-23; closed 2026-05-24 proactively before any customer dispute.
 ---</t>
         </is>
       </c>
-      <c r="H42" s="2" t="inlineStr"/>
-    </row>
-    <row r="43" ht="90" customHeight="1">
-      <c r="A43" s="3" t="inlineStr">
+      <c r="H44" s="2" t="inlineStr"/>
+    </row>
+    <row r="45" ht="90" customHeight="1">
+      <c r="A45" s="3" t="inlineStr">
         <is>
           <t>C25</t>
         </is>
       </c>
-      <c r="B43" s="3" t="inlineStr">
+      <c r="B45" s="3" t="inlineStr">
         <is>
           <t>VeritaQC Phase 1 (Levey-Jennings + Westgard live engine) (formerly #20)</t>
         </is>
       </c>
-      <c r="C43" s="3" t="inlineStr"/>
-      <c r="D43" s="3" t="inlineStr">
+      <c r="C45" s="3" t="inlineStr"/>
+      <c r="D45" s="3" t="inlineStr">
         <is>
           <t>L (about 5 days end-to-end, actual: Phase 0 schema → Phase 1A evaluator → 1B...</t>
         </is>
       </c>
-      <c r="E43" s="3" t="inlineStr">
+      <c r="E45" s="3" t="inlineStr">
         <is>
           <t>High — largest single gap vs myLabCompliance.io per Perplexity competitor ana...</t>
         </is>
       </c>
-      <c r="F43" s="3" t="inlineStr">
+      <c r="F45" s="3" t="inlineStr">
         <is>
           <t>Effort: L (about 5 days end-to-end, actual: Phase 0 schema → Phase 1A evaluator → 1B entry UI → 1C daily review → 1D monthly PDF + attestation)
 Importance: High — largest single gap vs myLabCompliance.io per Perplexity competitor analysis; promotes VeritaAssure from documentation tool to lab operations platform.</t>
         </is>
       </c>
-      <c r="G43" s="3" t="inlineStr">
+      <c r="G45" s="3" t="inlineStr">
         <is>
           <t>Perplexity competitor analysis 2026-05-10. Scoping confirmed via the build_phase1_mockup.py iterations 2026-05-24. Shipped 2026-05-25.
 ---</t>
         </is>
       </c>
-      <c r="H43" s="3" t="inlineStr"/>
-    </row>
-    <row r="44" ht="90" customHeight="1">
-      <c r="A44" s="2" t="inlineStr">
+      <c r="H45" s="3" t="inlineStr"/>
+    </row>
+    <row r="46" ht="90" customHeight="1">
+      <c r="A46" s="2" t="inlineStr">
         <is>
           <t>C26</t>
         </is>
       </c>
-      <c r="B44" s="2" t="inlineStr">
+      <c r="B46" s="2" t="inlineStr">
         <is>
           <t>VeritaLab CMS-116 application support + state licensing registry (formerly #22)</t>
         </is>
       </c>
-      <c r="C44" s="2" t="inlineStr"/>
-      <c r="D44" s="2" t="inlineStr">
+      <c r="C46" s="2" t="inlineStr"/>
+      <c r="D46" s="2" t="inlineStr">
         <is>
           <t>M (1-2 weeks for v1, actual)</t>
         </is>
       </c>
-      <c r="E44" s="2" t="inlineStr">
+      <c r="E46" s="2" t="inlineStr">
         <is>
           <t>Medium — competitor parity (myLabCompliance.io) plus useful at lab startup an...</t>
         </is>
       </c>
-      <c r="F44" s="2" t="inlineStr">
+      <c r="F46" s="2" t="inlineStr">
         <is>
           <t>Effort: M (1-2 weeks for v1, actual)
 Importance: Medium — competitor parity (myLabCompliance.io) plus useful at lab startup and at certificate-type changes.</t>
         </is>
       </c>
-      <c r="G44" s="2" t="inlineStr">
+      <c r="G46" s="2" t="inlineStr">
         <is>
           <t>Perplexity competitor analysis (myLabCompliance.io), 2026-05-10. Reclassified as a VeritaLab extension 2026-05-25. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H44" s="2" t="inlineStr"/>
-    </row>
-    <row r="45" ht="90" customHeight="1">
-      <c r="A45" s="3" t="inlineStr">
+      <c r="H46" s="2" t="inlineStr"/>
+    </row>
+    <row r="47" ht="90" customHeight="1">
+      <c r="A47" s="3" t="inlineStr">
         <is>
           <t>C27</t>
         </is>
       </c>
-      <c r="B45" s="3" t="inlineStr">
+      <c r="B47" s="3" t="inlineStr">
         <is>
           <t>Active vs view-only seat split (formerly #33)</t>
         </is>
       </c>
-      <c r="C45" s="3" t="inlineStr"/>
-      <c r="D45" s="3" t="inlineStr">
+      <c r="C47" s="3" t="inlineStr"/>
+      <c r="D47" s="3" t="inlineStr">
         <is>
           <t>M (~1 week of engineering, actual: shipped in a single multi-PR session)</t>
         </is>
       </c>
-      <c r="E45" s="3" t="inlineStr">
+      <c r="E47" s="3" t="inlineStr">
         <is>
           <t>Medium — closed the gap between /pricing copy and product behavior; gives sal...</t>
         </is>
       </c>
-      <c r="F45" s="3" t="inlineStr">
+      <c r="F47" s="3" t="inlineStr">
         <is>
           <t>Effort: M (~1 week of engineering, actual: shipped in a single multi-PR session)
 Importance: Medium — closed the gap between /pricing copy and product behavior; gives sales a clean answer for "do you charge for our medical director?"</t>
         </is>
       </c>
-      <c r="G45" s="3" t="inlineStr">
+      <c r="G47" s="3" t="inlineStr">
         <is>
           <t>Pricing analysis doc Decision 3 (2026-05-21); MEDIUM scenario revised 2026-05-29 to retire the "unlimited view-only" claim. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H45" s="3" t="inlineStr"/>
-    </row>
-    <row r="46" ht="90" customHeight="1">
-      <c r="A46" s="2" t="inlineStr">
+      <c r="H47" s="3" t="inlineStr"/>
+    </row>
+    <row r="48" ht="90" customHeight="1">
+      <c r="A48" s="2" t="inlineStr">
         <is>
           <t>C28</t>
         </is>
       </c>
-      <c r="B46" s="2" t="inlineStr">
+      <c r="B48" s="2" t="inlineStr">
         <is>
           <t>"Why VeritaCheck" comparative one-pager (formerly #37)</t>
         </is>
       </c>
-      <c r="C46" s="2" t="inlineStr"/>
-      <c r="D46" s="2" t="inlineStr">
+      <c r="C48" s="2" t="inlineStr"/>
+      <c r="D48" s="2" t="inlineStr">
         <is>
           <t>S (one design pass + four claim paragraphs + PDF + matching marketing-site pa...</t>
         </is>
       </c>
-      <c r="E46" s="2" t="inlineStr">
+      <c r="E48" s="2" t="inlineStr">
         <is>
           <t>Medium — closed a positioning gap surfaced by six COLA conference attendees a...</t>
         </is>
       </c>
-      <c r="F46" s="2" t="inlineStr">
+      <c r="F48" s="2" t="inlineStr">
         <is>
           <t>Effort: S (one design pass + four claim paragraphs + PDF + matching marketing-site page, actual)
 Importance: Medium — closed a positioning gap surfaced by six COLA conference attendees attached to a legacy verification tool; converts product-quality advantage into a leave-behind Lisa can hand out.</t>
         </is>
       </c>
-      <c r="G46" s="2" t="inlineStr">
+      <c r="G48" s="2" t="inlineStr">
         <is>
           <t>2026-05-11 / 2026-05-12 conference notes review with Michael. Conference attendees (Whitehead, Odegard, Othman, Molinelli, Kyle, Allred) expressed interest in equivalent / superior product. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H46" s="2" t="inlineStr"/>
-    </row>
-    <row r="47" ht="90" customHeight="1">
-      <c r="A47" s="3" t="inlineStr">
+      <c r="H48" s="2" t="inlineStr"/>
+    </row>
+    <row r="49" ht="90" customHeight="1">
+      <c r="A49" s="3" t="inlineStr">
         <is>
           <t>C29</t>
         </is>
       </c>
-      <c r="B47" s="3" t="inlineStr">
+      <c r="B49" s="3" t="inlineStr">
         <is>
           <t>VeritaPolicy approval workflow — MediaLab functional mirror</t>
         </is>
       </c>
-      <c r="C47" s="3" t="inlineStr"/>
-      <c r="D47" s="3" t="inlineStr">
+      <c r="C49" s="3" t="inlineStr"/>
+      <c r="D49" s="3" t="inlineStr">
         <is>
           <t>XL (one focused session, 12 PRs landed)</t>
         </is>
       </c>
-      <c r="E47" s="3" t="inlineStr">
+      <c r="E49" s="3" t="inlineStr">
         <is>
           <t>High — replaces MediaLab Document Control ($752/$2,250 starting price, scalin...</t>
         </is>
       </c>
-      <c r="F47" s="3" t="inlineStr">
+      <c r="F49" s="3" t="inlineStr">
         <is>
           <t>Effort: XL (one focused session, 12 PRs landed)
 Importance: High — replaces MediaLab Document Control ($752/$2,250 starting price, scaling to $10K-$20K/yr at enterprise per Capterra public data) with an included VeritaPolicy feature; closes a real positioning gap and gives sales a direct comparator line.</t>
         </is>
       </c>
-      <c r="G47" s="3" t="inlineStr">
+      <c r="G49" s="3" t="inlineStr">
         <is>
           <t>Pricing strategy conversation 2026-05-29 (Michael: "I don't like bolt-ons; we should replicate this") → scoped 8 phases → shipped all 12 PRs in single session. Shipped 2026-05-29.
 ---</t>
         </is>
       </c>
-      <c r="H47" s="3" t="inlineStr"/>
+      <c r="H49" s="3" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H47"/>
+  <autoFilter ref="A1:H49"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
docs(parking-lot): log #53 VeritaCEU free-CE provider list
TASK: Capture Jennifer Small's (Lifepoint) free continuing-education source list for the future VeritaCEU module, per Michael 2026-09-28.
PLAN: Add OPEN #53 with the provider list (API, ARUP, Cardinal, Fisher, MLO, ADLM, Siemens, Cepheid, Abbott, OneLab/CDC, BioRad, LabRoots; Whitehat Communications delivery); regenerate PARKING_LOT.xlsx.
Self-check: docs + xlsx only; source attributed; reference-only entry, not started.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PARKING_LOT.xlsx
+++ b/PARKING_LOT.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RETIRED" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$49</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RETIRED'!$A$1:$H$7</definedName>
   </definedNames>
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1199,8 +1199,52 @@
         </is>
       </c>
     </row>
+    <row r="17" ht="90" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>VeritaCEU: curated free-continuing-education provider list (seed / reference)</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Open, reference captured. Not started.</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>S (1-2 days to seed a curated provider list and surface it in VeritaCEU; XS t...</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Low-Medium — quality-of-life for VeritaCEU users (find free CE fast); not blo...</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Effort: S (1-2 days to seed a curated provider list and surface it in VeritaCEU; XS to just store the reference)
+Importance: Low-Medium — quality-of-life for VeritaCEU users (find free CE fast); not blocking any sale.</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>Jennifer Small (jennifer.small@lifepointhealth.net) email 2026-09-25, forwarded by Michael 2026-09-28 for the future CEU module.</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>Post-COLA. No customer urgency.
+---</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H16"/>
+  <autoFilter ref="A1:H17"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
TASK: log #53 VeritaCEU free-CE provider list in parking lot (#1359)
PLAN:
  1. record the VeritaCEU free-CE provider list as parking-lot item #53 for the future CEU module

Self-check:
  - docs-only change, Gate 3 N/A
  - each key at line start; Commit Message Gate passes
</commit_message>
<xml_diff>
--- a/PARKING_LOT.xlsx
+++ b/PARKING_LOT.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RETIRED" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$49</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RETIRED'!$A$1:$H$7</definedName>
   </definedNames>
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1199,8 +1199,52 @@
         </is>
       </c>
     </row>
+    <row r="17" ht="90" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>VeritaCEU: curated free-continuing-education provider list (seed / reference)</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Open, reference captured. Not started.</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>S (1-2 days to seed a curated provider list and surface it in VeritaCEU; XS t...</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Low-Medium — quality-of-life for VeritaCEU users (find free CE fast); not blo...</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Effort: S (1-2 days to seed a curated provider list and surface it in VeritaCEU; XS to just store the reference)
+Importance: Low-Medium — quality-of-life for VeritaCEU users (find free CE fast); not blocking any sale.</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>Jennifer Small (jennifer.small@lifepointhealth.net) email 2026-09-25, forwarded by Michael 2026-09-28 for the future CEU module.</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>Post-COLA. No customer urgency.
+---</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H16"/>
+  <autoFilter ref="A1:H17"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
TASK: close parking-lot #50/#51/#52 (shipped PR #1356/#1358/#1361) PLAN:   1. move #50, #51, #52 from OPEN to CLOSED (C49/C50/C51) with prod-verified evidence   2. regenerate PARKING_LOT.xlsx (OPEN 16 to 13, CLOSED +3) Self-check:   - docs-only change, Gate 3 N/A   - #52 closed as core (member picker); residual optional UX noted in C51   - keys at line start; Commit Message Gate passes
</commit_message>
<xml_diff>
--- a/PARKING_LOT.xlsx
+++ b/PARKING_LOT.xlsx
@@ -12,8 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RETIRED" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$49</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$52</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RETIRED'!$A$1:$H$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1051,7 +1051,10 @@
       <c r="C13" s="3" t="inlineStr">
         <is>
           <t>Open. Not started. Needs a one-line scope confirmation (which master list).
----</t>
+---
+_(item #50 closed 2026-09-28; shipped PR #1356, prod-verified, see C49 below)_
+---
+_(item #51 closed 2026-09-28;...</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
@@ -1080,163 +1083,41 @@
     <row r="14" ht="90" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>53</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Competency "assessed this cycle" uses a flat 365-day window</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr"/>
+          <t>VeritaCEU: curated free-continuing-education provider list (seed / reference)</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Open, reference captured. Not started.</t>
+        </is>
+      </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>S-M - anchor the coverage-map "assessed this cycle" to the person's actual CL...</t>
+          <t>S (1-2 days to seed a curated provider list and surface it in VeritaCEU; XS t...</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Medium - in an employee's first year the semiannual windows differ from a fla...</t>
+          <t>Low-Medium — quality-of-life for VeritaCEU users (find free CE fast); not blo...</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>Effort: S-M - anchor the coverage-map "assessed this cycle" to the person's actual CLIA cadence (semiannual in year 1 per 42 CFR 493.1451(b)(8), annual thereafter) from staff_competency_schedules, instead of the v1 flat 365-day lookback.
-Importance: Medium - in an employee's first year the semiannual windows differ from a flat annual window, so a first-year assessment could read as current slightly longer or shorter than the true cadence. Fine for the common annual case; refine for year-1 accuracy.</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-24 session, VeritaComp coverage map (#48 Phase 3) v1 simplification, noted in PR #1319.
----</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr"/>
-    </row>
-    <row r="15" ht="90" customHeight="1">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>51</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>VeritaTrack task owner + owner-scoped reminder routing</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>Open, not started. Placeholder pending build. Open questions: is the owner a staff_employee or a seat user, and how are reminder recipients currently chosen.</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>S-M (1-3 days to ~1.5 weeks) — add an owner on a VeritaTrack task, selectable...</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="inlineStr">
-        <is>
-          <t>Medium — cuts reminder-email noise so people only get the tasks that are thei...</t>
-        </is>
-      </c>
-      <c r="F15" s="3" t="inlineStr">
-        <is>
-          <t>Michael, verbatim (2026-09-28): "In veritatask, we should be able to assign an owner from staff that are built, then in the reminder section, we should be able to designate reminder emails only to the owner. The hem person does not need the chemistry reminders, etc." Module note: there is no VeritaTask module in the codebase; the task/reminder surface is VeritaTrack (client/src/pages/VeritaTrackAppPage.tsx), so this lands there. Today VeritaTrack tasks are not owned by a specific staff member and reminder emails are not recipient-scoped to an owner. The build adds (a) an owner selector on each task drawn from the lab's VeritaStaff roster, and (b) a reminder setting that routes the reminder email to only that owner. Confirm the current reminder recipient model before sizing.</t>
-        </is>
-      </c>
-      <c r="G15" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-28 session, Michael "for later (placeholder)" optimization #1 (relaying from the Lab Members / VeritaAssure screens).</t>
-        </is>
-      </c>
-      <c r="H15" s="3" t="inlineStr">
-        <is>
-          <t>Post-COLA. No customer urgency.
----</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="90" customHeight="1">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>52</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>Medical Director seat via account-grant dropdown (designate / transfer MD)</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Open, not started. Placeholder. Confirm the current MD-seat assignment path and the one-MD-per-location enforcement point before sizing.</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>S-M (1-3 days to ~1.5 weeks) — move MD-seat assignment onto the same per-memb...</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>Medium-High — the MD seat is a recurring friction point (Georgetown, SCAHC MD...</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>Michael, verbatim (2026-09-28): "The way we are doing the medical director seat is silly. Why not just use the account grant dropdown to give a medical director seat. If the person is already in, then we should just be able to grant the medical director seat the same way we promote people to admin or reduce them to staff as long as we only have 1 per location. Maybe do another block like the transfer ownership block as 'designate medical director or transfer medical director'." So: fold the MD seat into the existing member role dropdown (Admin / Staff / ... + Medical Director) with a single-MD-per-lab constraint, and add a dedicated designate-or-transfer-MD block that mirrors the transfer-ownership UX for changing the MD. Cross-ref [[project_medical_director_designation]] and the seat model.</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 session, Michael "for later (placeholder)" optimization #3 (relaying from the Lab Members screen).</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>Post-COLA. No customer urgency.
----</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="90" customHeight="1">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>53</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>VeritaCEU: curated free-continuing-education provider list (seed / reference)</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>Open, reference captured. Not started.</t>
-        </is>
-      </c>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>S (1-2 days to seed a curated provider list and surface it in VeritaCEU; XS t...</t>
-        </is>
-      </c>
-      <c r="E17" s="3" t="inlineStr">
-        <is>
-          <t>Low-Medium — quality-of-life for VeritaCEU users (find free CE fast); not blo...</t>
-        </is>
-      </c>
-      <c r="F17" s="3" t="inlineStr">
         <is>
           <t>Effort: S (1-2 days to seed a curated provider list and surface it in VeritaCEU; XS to just store the reference)
 Importance: Low-Medium — quality-of-life for VeritaCEU users (find free CE fast); not blocking any sale.</t>
         </is>
       </c>
-      <c r="G17" s="3" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>Jennifer Small (jennifer.small@lifepointhealth.net) email 2026-09-25, forwarded by Michael 2026-09-28 for the future CEU module.</t>
         </is>
       </c>
-      <c r="H17" s="3" t="inlineStr">
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>Post-COLA. No customer urgency.
 ---</t>
@@ -1244,7 +1125,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H17"/>
+  <autoFilter ref="A1:H14"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1255,7 +1136,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H49"/>
+  <dimension ref="A1:H52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1313,24 +1194,24 @@
     <row r="2" ht="90" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>C47</t>
+          <t>C49</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Unregulated-analyte / Alternative Assessment (AAA) coverage (was #18)</t>
+          <t>Competency "assessed this cycle" cadence-aware window (was #50)</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr"/>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>was S (Phase 3) / Importance: Medium</t>
+          <t>was S-M / Importance: Medium</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Effort: was S (Phase 3) / Importance: Medium</t>
+          <t>Effort: was S-M / Importance: Medium</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
@@ -1339,24 +1220,24 @@
     <row r="3" ht="90" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>C48</t>
+          <t>C50</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>VeritaResponse post-survey deficiency module (was #17)</t>
+          <t>VeritaTrack task owner + owner-only reminder routing (was #51)</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr"/>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>was XL / Importance: High</t>
+          <t>was S-M / Importance: Medium</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Effort: was XL / Importance: High</t>
+          <t>Effort: was S-M / Importance: Medium</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr"/>
@@ -1365,93 +1246,90 @@
     <row r="4" ht="90" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>C45</t>
+          <t>C51</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Unify coverage/competency recurrence helper (was #49) - closed as non-issue</t>
+          <t>Designate Medical Director by picking a lab member (was #52, core)</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr"/>
-      <c r="D4" s="2" t="inlineStr"/>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>was S-M / Importance: Medium-High</t>
+        </is>
+      </c>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: Investigated 2026-09-24 before building. The coverage recurrence math (+6-month interval, signed-resets-to-missing, nextDueOn/overdue, isFailVerdict) is ALREADY single-source in server/veritacheckCoverage.ts (computeCoverageFrom). server/coverageReport.ts and the routes.ts coverage export do not recompute it; they consume the computed nextDueOn/overdue/status fields and apply small surface-specific presentation labels (deliberately different vocabularies per surface, so they should not be merged). The only truly identical duplicate is a one-line date formatter. The competency "owed" derivation is NOT the same cadence: competency follows the CLIA milestone schedule (initial / semiannual year 1 / annual, 42 CFR 493.1451(b)(8) and 493.1235), which is a different regulatory interval from the coverage 6-month rule (493.1281 / 493.1255) and must stay separate. No worthwhile extraction; merging the two cadences would be wrong. Closed 2026-09-24. (The year-1 competency-window refinement remains tracked separately as #50.)</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-24 session, "keep working" pass; scoped read-only, found no real duplication.
----</t>
-        </is>
-      </c>
+          <t>Effort: was S-M / Importance: Medium-High</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr"/>
       <c r="H4" s="2" t="inlineStr"/>
     </row>
     <row r="5" ht="90" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>C46</t>
+          <t>C47</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Verified-users product-update send path (wrong-list incident fix)</t>
+          <t>Unregulated-analyte / Alternative Assessment (AAA) coverage (was #18)</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr"/>
-      <c r="D5" s="3" t="inlineStr"/>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>was S (Phase 3) / Importance: Medium</t>
+        </is>
+      </c>
       <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: Shipped PR #1324 (merged 4e05506a, deploy ACTIVE). New POST /api/admin/users/send targets registered VeritaAssure account holders (the users table), never the Lab Director's Briefing subscriber list. Separate explicitly-named endpoint (not a flag with a dangerous default), account-holder email framing, excludes suppressed emails and RFC-reserved test domains, CC owner, dryRun + testTo previews. Public unsubscribe now upserts a suppression row so opt-outs are honored across both audiences. Live dryRun: 49 verified-user recipients vs 673 on the Briefing list. Receipts: scripts/verify-product-update-send.mts 24/24, tsc clean, rendered sample inspected. Fixes the fallout from the 2026-09-23/24 wrong-list send (a product update went to the 675-person Briefing list). Nothing sends without Michael's explicit "send it."</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-24 session; Michael selected this as the next build after the #41 close.
----</t>
-        </is>
-      </c>
+          <t>Effort: was S (Phase 3) / Importance: Medium</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr"/>
       <c r="H5" s="3" t="inlineStr"/>
     </row>
     <row r="6" ht="90" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>C44</t>
+          <t>C48</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Verify-script convention backfill (was #41) + audit matcher fix</t>
+          <t>VeritaResponse post-survey deficiency module (was #17)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr"/>
-      <c r="D6" s="2" t="inlineStr"/>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>was XL / Importance: High</t>
+        </is>
+      </c>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: #41 was fully backfilled on 2026-06-13 (all 8 high-stakes scripts landed; see C30); it had only been mis-filed in OPEN. A 2026-09-24 re-audit initially reported 4 of 5 recent math/logic commits as missing a verify script, which was a FALSE POSITIVE: scripts/audit_verify_script_coverage.py matched only scripts/verify-*.js / .cjs, so it ignored the .mjs / .mts / .ts verify scripts the repo now ships (e.g. verify-ptcoag-multi.mts, verify-tea-criterion-format.mjs). Fixed the matcher to accept .js/.cjs/.mjs/.ts/.mts; re-run shows 5 of 5 covered, 0 debt. The convention is being followed. Closed 2026-09-24.</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-24 session, "keep working" pass; audit tooling bug found + fixed.
----</t>
-        </is>
-      </c>
+          <t>Effort: was XL / Importance: High</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr"/>
       <c r="H6" s="2" t="inlineStr"/>
     </row>
     <row r="7" ht="90" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>C43</t>
+          <t>C45</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>VeritaStaff instrument-centric (dual) assignment view</t>
+          <t>Unify coverage/competency recurrence helper (was #49) - closed as non-issue</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr"/>
@@ -1459,12 +1337,12 @@
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1320. GET/PUT /staff/instruments/:id/employees (transpose of the per-employee endpoints); an "Assign by Instrument" dialog lets a director pick a test system or manual test and check off who runs it. Same staff_employee_instruments join, with the 42 CFR 493.1235(a) duty-change event emitted on newly-added pairs so both orientations trigger the same reassessment. GET verified live on SCAHC lab 2. Closed 2026-09-24.</t>
+          <t>Closure evidence: Investigated 2026-09-24 before building. The coverage recurrence math (+6-month interval, signed-resets-to-missing, nextDueOn/overdue, isFailVerdict) is ALREADY single-source in server/veritacheckCoverage.ts (computeCoverageFrom). server/coverageReport.ts and the routes.ts coverage export do not recompute it; they consume the computed nextDueOn/overdue/status fields and apply small surface-specific presentation labels (deliberately different vocabularies per surface, so they should not be merged). The only truly identical duplicate is a one-line date formatter. The competency "owed" derivation is NOT the same cadence: competency follows the CLIA milestone schedule (initial / semiannual year 1 / annual, 42 CFR 493.1451(b)(8) and 493.1235), which is a different regulatory interval from the coverage 6-month rule (493.1281 / 493.1255) and must stay separate. No worthwhile extraction; merging the two cadences would be wrong. Closed 2026-09-24. (The year-1 competency-window refinement remains tracked separately as #50.)</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>2026-09-24 session, Michael ("in staff we should also give the dual view when assigning coverage to test systems or manual tests").
+          <t>2026-09-24 session, "keep working" pass; scoped read-only, found no real duplication.
 ---</t>
         </is>
       </c>
@@ -1473,12 +1351,12 @@
     <row r="8" ht="90" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>C42</t>
+          <t>C46</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>VeritaComp coverage map (required-vs-assessed matrix, dual view)</t>
+          <t>Verified-users product-update send path (wrong-list incident fix)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr"/>
@@ -1486,12 +1364,12 @@
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1319 (+ status layer PR #1316). /competency/owed returns per-item assessed (locked passing assessment this cycle on a covering method group) + per-employee CLIA status; CompetencyCoverageMap renders a By-employee / By-instrument matrix (Assessed / Owed / Overdue / Gap). Verified live on SCAHC lab 2 (owed 116, assessed 2, gaps 0). Completes #48 as the VeritaCheck-parity coverage map. Closed 2026-09-24.</t>
+          <t>Closure evidence: Shipped PR #1324 (merged 4e05506a, deploy ACTIVE). New POST /api/admin/users/send targets registered VeritaAssure account holders (the users table), never the Lab Director's Briefing subscriber list. Separate explicitly-named endpoint (not a flag with a dangerous default), account-holder email framing, excludes suppressed emails and RFC-reserved test domains, CC owner, dryRun + testTo previews. Public unsubscribe now upserts a suppression row so opt-outs are honored across both audiences. Live dryRun: 49 verified-user recipients vs 673 on the Briefing list. Receipts: scripts/verify-product-update-send.mts 24/24, tsc clean, rendered sample inspected. Fixes the fallout from the 2026-09-23/24 wrong-list send (a product update went to the 675-person Briefing list). Nothing sends without Michael's explicit "send it."</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 session, Michael ("are we building the competencies to have a coverage map, same as veritacheck?" then "build it").
+          <t>2026-09-24 session; Michael selected this as the next build after the #41 close.
 ---</t>
         </is>
       </c>
@@ -1500,12 +1378,12 @@
     <row r="9" ht="90" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>C41</t>
+          <t>C44</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>VeritaCheck coverage recurrence (method comparison + cal-ver/linearity + reports)</t>
+          <t>Verify-script convention backfill (was #41) + audit matcher fix</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr"/>
@@ -1513,12 +1391,12 @@
       <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: PRs #1317 (method comparison), #1318 (cal-ver/linearity), #1321 (report Next-due columns). Periodic verification (correlation/method comparison 42 CFR 493.1281; cal-ver/linearity 42 CFR 493.1255; both 6-month) now recurs: a signed study banks the cycle and rolls to next-due = signed + 6 months instead of reading "done" forever. Status Missing/Failed/Completed-unsigned + a "Next due on" column on-screen and in both coverage exports; also credits the previously-ignored "correlation" study type. Root cause: computeCoverageFrom marked requirements done on mere existence, no date logic. Verified live on SCAHC lab 2 (101 correlations + 11 cal-ver rows now carry a next-due). Engine-level, all facilities. Closed 2026-09-24.</t>
+          <t>Closure evidence: #41 was fully backfilled on 2026-06-13 (all 8 high-stakes scripts landed; see C30); it had only been mis-filed in OPEN. A 2026-09-24 re-audit initially reported 4 of 5 recent math/logic commits as missing a verify script, which was a FALSE POSITIVE: scripts/audit_verify_script_coverage.py matched only scripts/verify-*.js / .cjs, so it ignored the .mjs / .mts / .ts verify scripts the repo now ships (e.g. verify-ptcoag-multi.mts, verify-tea-criterion-format.mjs). Fixed the matcher to accept .js/.cjs/.mjs/.ts/.mts; re-run shows 5 of 5 covered, 0 debt. The convention is being followed. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>2026-09-24 session, Michael ("Look at San Carlos... they finished their last set of correlations (all 103) but their menu never reset").
+          <t>2026-09-24 session, "keep working" pass; audit tooling bug found + fixed.
 ---</t>
         </is>
       </c>
@@ -1527,12 +1405,12 @@
     <row r="10" ht="90" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>C40</t>
+          <t>C43</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>VeritaComp Competencies Owed derived from VeritaStaff, with gap detection (was #48)</t>
+          <t>VeritaStaff instrument-centric (dual) assignment view</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr"/>
@@ -1540,12 +1418,12 @@
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1314 (squash 2bcb0db9). GET /api/labs/:labId/competency/owed derives each VeritaStaff testing employee's owed competencies from their assigned instruments (staff_employee_instruments -&gt; veritamap_instruments + tests), on the CLIA timeline, and flags instruments not covered by any competency program as gaps. CompetenciesOwedSection renders it on the VeritaComp landing page. Reuses the shipped bridge + suggested-method-groups match rules; no new tables. Verified live on prod with real assignment data: 2 instruments assigned to a demo staffer produced owed=2, gaps=2 (HIGH, Technical Supervisor), then reverted cleanly. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1320. GET/PUT /staff/instruments/:id/employees (transpose of the per-employee endpoints); an "Assign by Instrument" dialog lets a director pick a test system or manual test and check off who runs it. Same staff_employee_instruments join, with the 42 CFR 493.1235(a) duty-change event emitted on newly-added pairs so both orientations trigger the same reassessment. GET verified live on SCAHC lab 2. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23/24 session, Michael ("veritacomp bases what competencies they owe (currently untrue, but needs to be true)"). Option 1 (unify roster on VeritaStaff, match instruments by id).
+          <t>2026-09-24 session, Michael ("in staff we should also give the dual view when assigning coverage to test systems or manual tests").
 ---</t>
         </is>
       </c>
@@ -1554,12 +1432,12 @@
     <row r="11" ht="90" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>C39</t>
+          <t>C42</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>VeritaScan line items can attach or link evidence (was #46)</t>
+          <t>VeritaComp coverage map (required-vs-assessed matrix, dual view)</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr"/>
@@ -1567,12 +1445,12 @@
       <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1312 (squash a1dda93d). VeritaScan scan checklist items now show linked evidence as chips (open link, remove) plus a writer "Link evidence" affordance whose picker links an existing VeritaDC/Library document; a shortcut deep-links to the Library for new (governed) documents. Reuses the already-shipped lab_documents + document_checklist_links + coverage endpoints (URL-pointer only, no file storage, no new tables). Browser-verified live on prod (scan 23): the affordance renders and the picker opens. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1319 (+ status layer PR #1316). /competency/owed returns per-item assessed (locked passing assessment this cycle on a covering method group) + per-employee CLIA status; CompetencyCoverageMap renders a By-employee / By-instrument matrix (Assessed / Owed / Overdue / Gap). Verified live on SCAHC lab 2 (owed 116, assessed 2, gaps 0). Completes #48 as the VeritaCheck-parity coverage map. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>2026-09-23 session, Michael. Recurring request. Companion: cross-module evidence display on the VeritaDC policy shipped in PR #1313 (by-target cross-links surfaced in the policy View modal, browser-verified live).
+          <t>2026-09-24 session, Michael ("are we building the competencies to have a coverage map, same as veritacheck?" then "build it").
 ---</t>
         </is>
       </c>
@@ -1581,12 +1459,12 @@
     <row r="12" ht="90" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>C38</t>
+          <t>C41</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>VeritaTrack calendar month cells expand to reveal hidden tasks (was #45)</t>
+          <t>VeritaCheck coverage recurrence (method comparison + cal-ver/linearity + reports)</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr"/>
@@ -1594,12 +1472,12 @@
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: VeritaTrack CalendarView month cells with more than three tasks now expand in place (chevron, "+N more" toggling to "Show less", due dates), so no task is hidden with no path to it (client/src/pages/VeritaTrackAppPage.tsx CalendarView). Shipped 2026-09-23. Closed 2026-09-24.</t>
+          <t>Closure evidence: PRs #1317 (method comparison), #1318 (cal-ver/linearity), #1321 (report Next-due columns). Periodic verification (correlation/method comparison 42 CFR 493.1281; cal-ver/linearity 42 CFR 493.1255; both 6-month) now recurs: a signed study banks the cycle and rolls to next-due = signed + 6 months instead of reading "done" forever. Status Missing/Failed/Completed-unsigned + a "Next due on" column on-screen and in both coverage exports; also credits the previously-ignored "correlation" study type. Root cause: computeCoverageFrom marked requirements done on mere existence, no date logic. Verified live on SCAHC lab 2 (101 correlations + 11 cal-ver rows now carry a next-due). Engine-level, all facilities. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23 session, Michael screenshot of the VeritaTrack calendar (lab 3, September cell).
+          <t>2026-09-24 session, Michael ("Look at San Carlos... they finished their last set of correlations (all 103) but their menu never reset").
 ---</t>
         </is>
       </c>
@@ -1608,12 +1486,12 @@
     <row r="13" ht="90" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>C37</t>
+          <t>C40</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Long Excel column headers no longer clip CFR citations (was #44)</t>
+          <t>VeritaComp Competencies Owed derived from VeritaStaff, with gap detection (was #48)</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr"/>
@@ -1621,12 +1499,12 @@
       <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. The VeritaMap export derives the header row height from the longest wrapped header via headerRowHeight(headers, colWidths) (server/routes.ts:15935) instead of a fixed 20, so "Reference Range Attestation (42 CFR 493.1253)" and the other long headers print in full. No new code this session. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1314 (squash 2bcb0db9). GET /api/labs/:labId/competency/owed derives each VeritaStaff testing employee's owed competencies from their assigned instruments (staff_employee_instruments -&gt; veritamap_instruments + tests), on the CLIA timeline, and flags instruments not covered by any competency program as gaps. CompetenciesOwedSection renders it on the VeritaComp landing page. Reuses the shipped bridge + suggested-method-groups match rules; no new tables. Verified live on prod with real assignment data: 2 instruments assigned to a demo staffer produced owed=2, gaps=2 (HIGH, Technical Supervisor), then reverted cleanly. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+          <t>2026-09-23/24 session, Michael ("veritacomp bases what competencies they owe (currently untrue, but needs to be true)"). Option 1 (unify roster on VeritaStaff, match instruments by id).
 ---</t>
         </is>
       </c>
@@ -1635,12 +1513,12 @@
     <row r="14" ht="90" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>C36</t>
+          <t>C39</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>License stamp no longer clobbers the §6 header/footer or names the wrong lab (was #43)</t>
+          <t>VeritaScan line items can attach or link evidence (was #46)</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr"/>
@@ -1648,12 +1526,12 @@
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. setHeaderFooter (shared/licenseExceljs.ts:155-209) now preserves an existing §6 header and appends (not overwrites) the footer left section, and customer-facing exports name the scoped lab: the VeritaScan library export reads req.scope.lab.name / clia_number (server/routes.ts:16572-16573), not the licensee. No new code this session (avoided regressing the existing fix). Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1312 (squash a1dda93d). VeritaScan scan checklist items now show linked evidence as chips (open link, remove) plus a writer "Link evidence" affordance whose picker links an existing VeritaDC/Library document; a shortcut deep-links to the Library for new (governed) documents. Reuses the already-shipped lab_documents + document_checklist_links + coverage endpoints (URL-pointer only, no file storage, no new tables). Browser-verified live on prod (scan 23): the affordance renders and the picker opens. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+          <t>2026-09-23 session, Michael. Recurring request. Companion: cross-module evidence display on the VeritaDC policy shipped in PR #1313 (by-target cross-links surfaced in the policy View modal, browser-verified live).
 ---</t>
         </is>
       </c>
@@ -1662,18 +1540,99 @@
     <row r="15" ht="90" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>C34</t>
+          <t>C38</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Wire the two static-audit guards into CI (was #43)</t>
+          <t>VeritaTrack calendar month cells expand to reveal hidden tasks (was #45)</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr"/>
       <c r="D15" s="3" t="inlineStr"/>
       <c r="E15" s="3" t="inlineStr"/>
       <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Closure evidence: VeritaTrack CalendarView month cells with more than three tasks now expand in place (chevron, "+N more" toggling to "Show less", due dates), so no task is hidden with no path to it (client/src/pages/VeritaTrackAppPage.tsx CalendarView). Shipped 2026-09-23. Closed 2026-09-24.</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-23 session, Michael screenshot of the VeritaTrack calendar (lab 3, September cell).
+---</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16" ht="90" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>C37</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Long Excel column headers no longer clip CFR citations (was #44)</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr"/>
+      <c r="D16" s="2" t="inlineStr"/>
+      <c r="E16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. The VeritaMap export derives the header row height from the longest wrapped header via headerRowHeight(headers, colWidths) (server/routes.ts:15935) instead of a fixed 20, so "Reference Range Attestation (42 CFR 493.1253)" and the other long headers print in full. No new code this session. Closed 2026-09-24.</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+---</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17" ht="90" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>C36</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>License stamp no longer clobbers the §6 header/footer or names the wrong lab (was #43)</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr"/>
+      <c r="D17" s="3" t="inlineStr"/>
+      <c r="E17" s="3" t="inlineStr"/>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. setHeaderFooter (shared/licenseExceljs.ts:155-209) now preserves an existing §6 header and appends (not overwrites) the footer left section, and customer-facing exports name the scoped lab: the VeritaScan library export reads req.scope.lab.name / clia_number (server/routes.ts:16572-16573), not the licensee. No new code this session (avoided regressing the existing fix). Closed 2026-09-24.</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+---</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr"/>
+    </row>
+    <row r="18" ht="90" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>C34</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Wire the two static-audit guards into CI (was #43)</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr"/>
+      <c r="D18" s="2" t="inlineStr"/>
+      <c r="E18" s="2" t="inlineStr"/>
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: both guards wired into the Multi-Lab Mutations Audit CI
 workflow (.github/workflows/multilab-mutations-audit.yml) as steps:
@@ -1685,24 +1644,24 @@
 (same caveat as the existing guards already in that workflow).</t>
         </is>
       </c>
-      <c r="G15" s="3" t="inlineStr"/>
-      <c r="H15" s="3" t="inlineStr"/>
-    </row>
-    <row r="16" ht="90" customHeight="1">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr"/>
+      <c r="H18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19" ht="90" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>C35</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>Legacy /api/studies over-returns studies across labs (was #44)</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr"/>
-      <c r="D16" s="2" t="inlineStr"/>
-      <c r="E16" s="2" t="inlineStr"/>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="C19" s="3" t="inlineStr"/>
+      <c r="D19" s="3" t="inlineStr"/>
+      <c r="E19" s="3" t="inlineStr"/>
+      <c r="F19" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: GET /api/studies now scopes its list to the active lab
 when one is resolved from the Referer (server/routes.ts), so every returned row
@@ -1712,24 +1671,24 @@
 mirroring the /api/labs/:labId/studies handler. Closed 2026-06-14.</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr"/>
-      <c r="H16" s="2" t="inlineStr"/>
-    </row>
-    <row r="17" ht="90" customHeight="1">
-      <c r="A17" s="3" t="inlineStr">
+      <c r="G19" s="3" t="inlineStr"/>
+      <c r="H19" s="3" t="inlineStr"/>
+    </row>
+    <row r="20" ht="90" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>C30</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>Verify-script convention backfill (was #41)</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr"/>
-      <c r="D17" s="3" t="inlineStr"/>
-      <c r="E17" s="3" t="inlineStr"/>
-      <c r="F17" s="3" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr"/>
+      <c r="D20" s="2" t="inlineStr"/>
+      <c r="E20" s="2" t="inlineStr"/>
+      <c r="F20" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: all 8 high-stakes math/logic commits now ship a paired
 scripts/verify-*.js (EP17 sensitivity, Deming lot-to-lot, CUMSUM+QC+multi-analyte,
@@ -1737,30 +1696,30 @@
 TEa boundary), per the strike-throughs in #41. Closed 2026-06-13.</t>
         </is>
       </c>
-      <c r="G17" s="3" t="inlineStr">
+      <c r="G20" s="2" t="inlineStr">
         <is>
           <t>scripts/audit_verify_script_coverage.py lookback, 2026-06-02; backfills
 landed 2026-06-03..06.
 ---</t>
         </is>
       </c>
-      <c r="H17" s="3" t="inlineStr"/>
-    </row>
-    <row r="18" ht="90" customHeight="1">
-      <c r="A18" s="2" t="inlineStr">
+      <c r="H20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21" ht="90" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>C31</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>VeritaPT AAA create/update/delete silently no-op in the multi-lab UI</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr"/>
-      <c r="D18" s="2" t="inlineStr"/>
-      <c r="E18" s="2" t="inlineStr"/>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="C21" s="3" t="inlineStr"/>
+      <c r="D21" s="3" t="inlineStr"/>
+      <c r="E21" s="3" t="inlineStr"/>
+      <c r="F21" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #754 (commit 92ad499) added lab-scoped POST/PUT/DELETE
 /api/labs/:labId/pt/aa-records. The UI posted to the lab-scoped path but only GET
@@ -1771,30 +1730,30 @@
 route mis-filed records to the user's default lab on multi-lab accounts).</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="G21" s="3" t="inlineStr">
         <is>
           <t>2026-06-13, found during #18 Phase 3 QA;
 scripts/audit-labscoped-write-routes.mjs now guards the class.
 ---</t>
         </is>
       </c>
-      <c r="H18" s="2" t="inlineStr"/>
-    </row>
-    <row r="19" ht="90" customHeight="1">
-      <c r="A19" s="3" t="inlineStr">
+      <c r="H21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22" ht="90" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>C32</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B22" s="2" t="inlineStr">
         <is>
           <t>VeritaComp "Unlock assessment" false-success no-op</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr"/>
-      <c r="D19" s="3" t="inlineStr"/>
-      <c r="E19" s="3" t="inlineStr"/>
-      <c r="F19" s="3" t="inlineStr">
+      <c r="C22" s="2" t="inlineStr"/>
+      <c r="D22" s="2" t="inlineStr"/>
+      <c r="E22" s="2" t="inlineStr"/>
+      <c r="F22" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #755 (commit 4234007) moved the unlock route to
 /api/labs/:labId/competency/assessments/:id/unlock (the path the client calls).
@@ -1805,29 +1764,29 @@
 HTML).</t>
         </is>
       </c>
-      <c r="G19" s="3" t="inlineStr">
+      <c r="G22" s="2" t="inlineStr">
         <is>
           <t>2026-06-13, found by scripts/audit-labscoped-write-routes.mjs.
 ---</t>
         </is>
       </c>
-      <c r="H19" s="3" t="inlineStr"/>
-    </row>
-    <row r="20" ht="90" customHeight="1">
-      <c r="A20" s="2" t="inlineStr">
+      <c r="H22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23" ht="90" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>C33</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>FK-cascade delete 500s + NavBar laptop-width overflow</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr"/>
-      <c r="D20" s="2" t="inlineStr"/>
-      <c r="E20" s="2" t="inlineStr"/>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="C23" s="3" t="inlineStr"/>
+      <c r="D23" s="3" t="inlineStr"/>
+      <c r="E23" s="3" t="inlineStr"/>
+      <c r="F23" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PRs #749/#750 fixed NavBar horizontal overflow at laptop
 widths (collapse to the hamburger below 1560px); prod-verified at 1280-1920 with the
@@ -1838,57 +1797,57 @@
 500 -&gt; 200. scripts/audit-delete-cascades.mjs guards the class.</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr">
+      <c r="G23" s="3" t="inlineStr">
         <is>
           <t>2026-06-13 browser QA of the A7-D4 wave + retro-QC of the 72h PR window.
 ---</t>
         </is>
       </c>
-      <c r="H20" s="2" t="inlineStr"/>
-    </row>
-    <row r="21" ht="90" customHeight="1">
-      <c r="A21" s="3" t="inlineStr">
+      <c r="H23" s="3" t="inlineStr"/>
+    </row>
+    <row r="24" ht="90" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>C1</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>FAQ "over 25 years" -&gt; "over 23 years"</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr"/>
-      <c r="D21" s="3" t="inlineStr"/>
-      <c r="E21" s="3" t="inlineStr"/>
-      <c r="F21" s="3" t="inlineStr">
+      <c r="C24" s="2" t="inlineStr"/>
+      <c r="D24" s="2" t="inlineStr"/>
+      <c r="E24" s="2" t="inlineStr"/>
+      <c r="F24" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: client/src/pages/FAQPage.tsx line 20 reads "over
 23 years" as of 2026-05-01.</t>
         </is>
       </c>
-      <c r="G21" s="3" t="inlineStr">
+      <c r="G24" s="2" t="inlineStr">
         <is>
           <t>session 299e9a73 turn 14, ~2026-04-28.
 ---</t>
         </is>
       </c>
-      <c r="H21" s="3" t="inlineStr"/>
-    </row>
-    <row r="22" ht="90" customHeight="1">
-      <c r="A22" s="2" t="inlineStr">
+      <c r="H24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25" ht="90" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
         <is>
           <t>C5</t>
         </is>
       </c>
-      <c r="B22" s="2" t="inlineStr">
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>David's VeritaQA grey-button bug (seat permissions mode)</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr"/>
-      <c r="D22" s="2" t="inlineStr"/>
-      <c r="E22" s="2" t="inlineStr"/>
-      <c r="F22" s="2" t="inlineStr">
+      <c r="C25" s="3" t="inlineStr"/>
+      <c r="D25" s="3" t="inlineStr"/>
+      <c r="E25" s="3" t="inlineStr"/>
+      <c r="F25" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #10 squash-merged as commit a43fbba on
 2026-05-01 23:19 MST. Railway deploy succeeded; deployed bundle
@@ -1901,7 +1860,7 @@
 against his exact stored shape (14 of 14 expected outcomes matched).</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr">
+      <c r="G25" s="3" t="inlineStr">
         <is>
           <t>2026-05-01 David's report; veritabench + veritastock
 weren't in MODULE_LIST so seat permissions silently defaulted to
@@ -1909,109 +1868,109 @@
 ---</t>
         </is>
       </c>
-      <c r="H22" s="2" t="inlineStr"/>
-    </row>
-    <row r="23" ht="90" customHeight="1">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>C2</t>
-        </is>
-      </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>TeamPage present-tense "TJC surveyor" check</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="inlineStr"/>
-      <c r="D23" s="3" t="inlineStr"/>
-      <c r="E23" s="3" t="inlineStr"/>
-      <c r="F23" s="3" t="inlineStr">
-        <is>
-          <t>Closure evidence: site-wide search confirmed all surveyor language
-is past-tense, consistent with user's 2021-2025 service. User closed
-the item in session 299e9a73 turn 4.</t>
-        </is>
-      </c>
-      <c r="G23" s="3" t="inlineStr">
-        <is>
-          <t>session 299e9a73, ~2026-04-28.
----</t>
-        </is>
-      </c>
-      <c r="H23" s="3" t="inlineStr"/>
-    </row>
-    <row r="24" ht="90" customHeight="1">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>C3</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>My Studies CSV/XLSX export (John as design partner)</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr"/>
-      <c r="D24" s="2" t="inlineStr"/>
-      <c r="E24" s="2" t="inlineStr"/>
-      <c r="F24" s="2" t="inlineStr">
-        <is>
-          <t>Closure evidence: client/src/pages/DashboardPage.tsx line 46 calls
-/api/my-studies/export. server/routes.ts line 1491 implements the
-endpoint. Pulled forward into pre-COLA per user instruction.</t>
-        </is>
-      </c>
-      <c r="G24" s="2" t="inlineStr">
-        <is>
-          <t>session 299e9a73 turn 5, ~2026-04-28.
----</t>
-        </is>
-      </c>
-      <c r="H24" s="2" t="inlineStr"/>
-    </row>
-    <row r="25" ht="90" customHeight="1">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t>C4</t>
-        </is>
-      </c>
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>Rotate GitHub PAT (because old PAT was committed in SESSION_HANDOFF files)</t>
-        </is>
-      </c>
-      <c r="C25" s="3" t="inlineStr"/>
-      <c r="D25" s="3" t="inlineStr"/>
-      <c r="E25" s="3" t="inlineStr"/>
-      <c r="F25" s="3" t="inlineStr">
-        <is>
-          <t>Closure evidence: no ghp_* or github_pat_* patterns in current
-SESSION_HANDOFF.md or SESSION_HANDOFF-2.md as of 2026-05-01.</t>
-        </is>
-      </c>
-      <c r="G25" s="3" t="inlineStr">
-        <is>
-          <t>session 299e9a73, ~2026-04-28.
----</t>
-        </is>
-      </c>
       <c r="H25" s="3" t="inlineStr"/>
     </row>
     <row r="26" ht="90" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>C6</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>VeritaPolicy service-line filtering removed (formerly #4)</t>
+          <t>TeamPage present-tense "TJC surveyor" check</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr"/>
       <c r="D26" s="2" t="inlineStr"/>
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Closure evidence: site-wide search confirmed all surveyor language
+is past-tense, consistent with user's 2021-2025 service. User closed
+the item in session 299e9a73 turn 4.</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>session 299e9a73, ~2026-04-28.
+---</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27" ht="90" customHeight="1">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>C3</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>My Studies CSV/XLSX export (John as design partner)</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr"/>
+      <c r="D27" s="3" t="inlineStr"/>
+      <c r="E27" s="3" t="inlineStr"/>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>Closure evidence: client/src/pages/DashboardPage.tsx line 46 calls
+/api/my-studies/export. server/routes.ts line 1491 implements the
+endpoint. Pulled forward into pre-COLA per user instruction.</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>session 299e9a73 turn 5, ~2026-04-28.
+---</t>
+        </is>
+      </c>
+      <c r="H27" s="3" t="inlineStr"/>
+    </row>
+    <row r="28" ht="90" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Rotate GitHub PAT (because old PAT was committed in SESSION_HANDOFF files)</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr"/>
+      <c r="D28" s="2" t="inlineStr"/>
+      <c r="E28" s="2" t="inlineStr"/>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Closure evidence: no ghp_* or github_pat_* patterns in current
+SESSION_HANDOFF.md or SESSION_HANDOFF-2.md as of 2026-05-01.</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>session 299e9a73, ~2026-04-28.
+---</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29" ht="90" customHeight="1">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>C6</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>VeritaPolicy service-line filtering removed (formerly #4)</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr"/>
+      <c r="D29" s="3" t="inlineStr"/>
+      <c r="E29" s="3" t="inlineStr"/>
+      <c r="F29" s="3" t="inlineStr">
         <is>
           <t>Closure rationale (operator decision 2026-05-10): Keep all
 VeritaPolicy rows. CFR-only references with no accreditor reference
@@ -2020,29 +1979,29 @@
 report misread the design intent.</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr">
+      <c r="G29" s="3" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H26" s="2" t="inlineStr"/>
-    </row>
-    <row r="27" ht="90" customHeight="1">
-      <c r="A27" s="3" t="inlineStr">
+      <c r="H29" s="3" t="inlineStr"/>
+    </row>
+    <row r="30" ht="90" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>C7</t>
         </is>
       </c>
-      <c r="B27" s="3" t="inlineStr">
+      <c r="B30" s="2" t="inlineStr">
         <is>
           <t>CLIA number format validation (formerly #13)</t>
         </is>
       </c>
-      <c r="C27" s="3" t="inlineStr"/>
-      <c r="D27" s="3" t="inlineStr"/>
-      <c r="E27" s="3" t="inlineStr"/>
-      <c r="F27" s="3" t="inlineStr">
+      <c r="C30" s="2" t="inlineStr"/>
+      <c r="D30" s="2" t="inlineStr"/>
+      <c r="E30" s="2" t="inlineStr"/>
+      <c r="F30" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: shared/validateClia.ts defines CLIA_REGEX =
 /^\d{2}D\d{7}$/ (line 24), validateClia() helper with whitespace
@@ -2053,30 +2012,30 @@
 shape exists and behaves as specified.</t>
         </is>
       </c>
-      <c r="G27" s="3" t="inlineStr">
+      <c r="G30" s="2" t="inlineStr">
         <is>
           <t>Agent verification 2026-05-10 via grep + file read.
 Operator confirmed shipped 2026-05-10.
 ---</t>
         </is>
       </c>
-      <c r="H27" s="3" t="inlineStr"/>
-    </row>
-    <row r="28" ht="90" customHeight="1">
-      <c r="A28" s="2" t="inlineStr">
+      <c r="H30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31" ht="90" customHeight="1">
+      <c r="A31" s="3" t="inlineStr">
         <is>
           <t>C8</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="B31" s="3" t="inlineStr">
         <is>
           <t>VeritaMap lab-wide menu toggle (formerly #19)</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr"/>
-      <c r="D28" s="2" t="inlineStr"/>
-      <c r="E28" s="2" t="inlineStr"/>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="C31" s="3" t="inlineStr"/>
+      <c r="D31" s="3" t="inlineStr"/>
+      <c r="E31" s="3" t="inlineStr"/>
+      <c r="F31" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: client/src/pages/VeritaMapLabwidePage.tsx
 exists and implements the labwide read-only union view. Route is
@@ -2086,59 +2045,59 @@
 parking lot plan (read-only union view, per-session toggle) shipped.</t>
         </is>
       </c>
-      <c r="G28" s="2" t="inlineStr">
+      <c r="G31" s="3" t="inlineStr">
         <is>
           <t>Agent verification 2026-05-10 via grep + file read.
 Operator confirmed shipped 2026-05-10.
 ---</t>
         </is>
       </c>
-      <c r="H28" s="2" t="inlineStr"/>
-    </row>
-    <row r="29" ht="90" customHeight="1">
-      <c r="A29" s="3" t="inlineStr">
+      <c r="H31" s="3" t="inlineStr"/>
+    </row>
+    <row r="32" ht="90" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t>C9</t>
         </is>
       </c>
-      <c r="B29" s="3" t="inlineStr">
+      <c r="B32" s="2" t="inlineStr">
         <is>
           <t>Tier-1 smoke test checklist (formerly #6)</t>
         </is>
       </c>
-      <c r="C29" s="3" t="inlineStr"/>
-      <c r="D29" s="3" t="inlineStr"/>
-      <c r="E29" s="3" t="inlineStr"/>
-      <c r="F29" s="3" t="inlineStr">
+      <c r="C32" s="2" t="inlineStr"/>
+      <c r="D32" s="2" t="inlineStr"/>
+      <c r="E32" s="2" t="inlineStr"/>
+      <c r="F32" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: docs/smoke-test-tier1.md documents the Tier-1
 smoke-test process and post-deploy verification steps. Shipped via
 PR #81 as part of the 2026-05-10 wave.</t>
         </is>
       </c>
-      <c r="G29" s="3" t="inlineStr">
+      <c r="G32" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H29" s="3" t="inlineStr"/>
-    </row>
-    <row r="30" ht="90" customHeight="1">
-      <c r="A30" s="2" t="inlineStr">
+      <c r="H32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33" ht="90" customHeight="1">
+      <c r="A33" s="3" t="inlineStr">
         <is>
           <t>C10</t>
         </is>
       </c>
-      <c r="B30" s="2" t="inlineStr">
+      <c r="B33" s="3" t="inlineStr">
         <is>
           <t>Per-module gating (formerly #7)</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr"/>
-      <c r="D30" s="2" t="inlineStr"/>
-      <c r="E30" s="2" t="inlineStr"/>
-      <c r="F30" s="2" t="inlineStr">
+      <c r="C33" s="3" t="inlineStr"/>
+      <c r="D33" s="3" t="inlineStr"/>
+      <c r="E33" s="3" t="inlineStr"/>
+      <c r="F33" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: Client-side useIsReadOnly module keys wired
 on client/src/pages/VeritaPolicyAppPage.tsx and
@@ -2153,29 +2112,29 @@
 PR #76.</t>
         </is>
       </c>
-      <c r="G30" s="2" t="inlineStr">
+      <c r="G33" s="3" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H30" s="2" t="inlineStr"/>
-    </row>
-    <row r="31" ht="90" customHeight="1">
-      <c r="A31" s="3" t="inlineStr">
+      <c r="H33" s="3" t="inlineStr"/>
+    </row>
+    <row r="34" ht="90" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
         <is>
           <t>C11</t>
         </is>
       </c>
-      <c r="B31" s="3" t="inlineStr">
+      <c r="B34" s="2" t="inlineStr">
         <is>
           <t>VeritaStock shipped copy (formerly #8)</t>
         </is>
       </c>
-      <c r="C31" s="3" t="inlineStr"/>
-      <c r="D31" s="3" t="inlineStr"/>
-      <c r="E31" s="3" t="inlineStr"/>
-      <c r="F31" s="3" t="inlineStr">
+      <c r="C34" s="2" t="inlineStr"/>
+      <c r="D34" s="2" t="inlineStr"/>
+      <c r="E34" s="2" t="inlineStr"/>
+      <c r="F34" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: client/src/pages/ArticleInventoryManagementPage.tsx
 line 305 footer reads "platform that includes VeritaStock™" instead
@@ -2183,29 +2142,29 @@
 on /resources/laboratory-inventory-management. Shipped via PR #75.</t>
         </is>
       </c>
-      <c r="G31" s="3" t="inlineStr">
+      <c r="G34" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H31" s="3" t="inlineStr"/>
-    </row>
-    <row r="32" ht="90" customHeight="1">
-      <c r="A32" s="2" t="inlineStr">
+      <c r="H34" s="2" t="inlineStr"/>
+    </row>
+    <row r="35" ht="90" customHeight="1">
+      <c r="A35" s="3" t="inlineStr">
         <is>
           <t>C12</t>
         </is>
       </c>
-      <c r="B32" s="2" t="inlineStr">
+      <c r="B35" s="3" t="inlineStr">
         <is>
           <t>Admin report one-row-per-lab (formerly #14)</t>
         </is>
       </c>
-      <c r="C32" s="2" t="inlineStr"/>
-      <c r="D32" s="2" t="inlineStr"/>
-      <c r="E32" s="2" t="inlineStr"/>
-      <c r="F32" s="2" t="inlineStr">
+      <c r="C35" s="3" t="inlineStr"/>
+      <c r="D35" s="3" t="inlineStr"/>
+      <c r="E35" s="3" t="inlineStr"/>
+      <c r="F35" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: /api/admin/report rewritten in
 server/routes.ts (~line 595) to LEFT JOIN labs on
@@ -2220,56 +2179,56 @@
 prerequisite, not a code bug). Shipped via PR #85.</t>
         </is>
       </c>
-      <c r="G32" s="2" t="inlineStr">
+      <c r="G35" s="3" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H32" s="2" t="inlineStr"/>
-    </row>
-    <row r="33" ht="90" customHeight="1">
-      <c r="A33" s="3" t="inlineStr">
+      <c r="H35" s="3" t="inlineStr"/>
+    </row>
+    <row r="36" ht="90" customHeight="1">
+      <c r="A36" s="2" t="inlineStr">
         <is>
           <t>C14</t>
         </is>
       </c>
-      <c r="B33" s="3" t="inlineStr">
+      <c r="B36" s="2" t="inlineStr">
         <is>
           <t>UI relabel "CLIA TEa" -&gt; "Lab-Set Internal Goal" (formerly #1)</t>
         </is>
       </c>
-      <c r="C33" s="3" t="inlineStr"/>
-      <c r="D33" s="3" t="inlineStr"/>
-      <c r="E33" s="3" t="inlineStr"/>
-      <c r="F33" s="3" t="inlineStr">
+      <c r="C36" s="2" t="inlineStr"/>
+      <c r="D36" s="2" t="inlineStr"/>
+      <c r="E36" s="2" t="inlineStr"/>
+      <c r="F36" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: Shipped across four PRs over 2026-05-10.</t>
         </is>
       </c>
-      <c r="G33" s="3" t="inlineStr">
+      <c r="G36" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H33" s="3" t="inlineStr"/>
-    </row>
-    <row r="34" ht="90" customHeight="1">
-      <c r="A34" s="2" t="inlineStr">
+      <c r="H36" s="2" t="inlineStr"/>
+    </row>
+    <row r="37" ht="90" customHeight="1">
+      <c r="A37" s="3" t="inlineStr">
         <is>
           <t>C13</t>
         </is>
       </c>
-      <c r="B34" s="2" t="inlineStr">
+      <c r="B37" s="3" t="inlineStr">
         <is>
           <t>WSLH PT vendor (formerly #15)</t>
         </is>
       </c>
-      <c r="C34" s="2" t="inlineStr"/>
-      <c r="D34" s="2" t="inlineStr"/>
-      <c r="E34" s="2" t="inlineStr"/>
-      <c r="F34" s="2" t="inlineStr">
+      <c r="C37" s="3" t="inlineStr"/>
+      <c r="D37" s="3" t="inlineStr"/>
+      <c r="E37" s="3" t="inlineStr"/>
+      <c r="F37" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: Shipped 2026-05-10 via PR #79 (merge commit
 eeebc6e; merged after rebase to resolve a server/db.ts collision
@@ -2287,64 +2246,64 @@
 'WSLH' is the post-deploy success signal. Shipped via PR #79.</t>
         </is>
       </c>
-      <c r="G34" s="2" t="inlineStr">
+      <c r="G37" s="3" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H34" s="2" t="inlineStr"/>
-    </row>
-    <row r="35" ht="90" customHeight="1">
-      <c r="A35" s="3" t="inlineStr">
+      <c r="H37" s="3" t="inlineStr"/>
+    </row>
+    <row r="38" ht="90" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
         <is>
           <t>C15</t>
         </is>
       </c>
-      <c r="B35" s="3" t="inlineStr">
+      <c r="B38" s="2" t="inlineStr">
         <is>
           <t>VeritaStock lot tracking + expiration + reorder alerts (formerly #21)</t>
         </is>
       </c>
-      <c r="C35" s="3" t="inlineStr"/>
-      <c r="D35" s="3" t="inlineStr"/>
-      <c r="E35" s="3" t="inlineStr"/>
-      <c r="F35" s="3" t="inlineStr">
+      <c r="C38" s="2" t="inlineStr"/>
+      <c r="D38" s="2" t="inlineStr"/>
+      <c r="E38" s="2" t="inlineStr"/>
+      <c r="F38" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: VeritaStock™ shipped the bench-level inventory
 features the Perplexity competitor analysis identified as a gap:</t>
         </is>
       </c>
-      <c r="G35" s="3" t="inlineStr">
+      <c r="G38" s="2" t="inlineStr">
         <is>
           <t>Originally Perplexity competitor analysis 2026-05-10.
 Audit 2026-05-21 confirmed the feature set ships today.
 ---</t>
         </is>
       </c>
-      <c r="H35" s="3" t="inlineStr"/>
-    </row>
-    <row r="36" ht="90" customHeight="1">
-      <c r="A36" s="2" t="inlineStr">
+      <c r="H38" s="2" t="inlineStr"/>
+    </row>
+    <row r="39" ht="90" customHeight="1">
+      <c r="A39" s="3" t="inlineStr">
         <is>
           <t>C16</t>
         </is>
       </c>
-      <c r="B36" s="2" t="inlineStr">
+      <c r="B39" s="3" t="inlineStr">
         <is>
           <t>PAL studies guided workflow (formerly #23)</t>
         </is>
       </c>
-      <c r="C36" s="2" t="inlineStr"/>
-      <c r="D36" s="2" t="inlineStr"/>
-      <c r="E36" s="2" t="inlineStr"/>
-      <c r="F36" s="2" t="inlineStr">
+      <c r="C39" s="3" t="inlineStr"/>
+      <c r="D39" s="3" t="inlineStr"/>
+      <c r="E39" s="3" t="inlineStr"/>
+      <c r="F39" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: VeritaCheck™ already ships the Precision /
 Accuracy / Linearity (PAL) study set under EP-protocol naming:</t>
         </is>
       </c>
-      <c r="G36" s="2" t="inlineStr">
+      <c r="G39" s="3" t="inlineStr">
         <is>
           <t>Originally Perplexity competitor analysis 2026-05-10.
 Audit 2026-05-21 confirmed the EP studies cover the PAL framing in
@@ -2352,23 +2311,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H36" s="2" t="inlineStr"/>
-    </row>
-    <row r="37" ht="90" customHeight="1">
-      <c r="A37" s="3" t="inlineStr">
+      <c r="H39" s="3" t="inlineStr"/>
+    </row>
+    <row r="40" ht="90" customHeight="1">
+      <c r="A40" s="2" t="inlineStr">
         <is>
           <t>C17</t>
         </is>
       </c>
-      <c r="B37" s="3" t="inlineStr">
+      <c r="B40" s="2" t="inlineStr">
         <is>
           <t>Source-grounded 21/29/45 CFR + 42 CFR 482-485 (formerly #26)</t>
         </is>
       </c>
-      <c r="C37" s="3" t="inlineStr"/>
-      <c r="D37" s="3" t="inlineStr"/>
-      <c r="E37" s="3" t="inlineStr"/>
-      <c r="F37" s="3" t="inlineStr">
+      <c r="C40" s="2" t="inlineStr"/>
+      <c r="D40" s="2" t="inlineStr"/>
+      <c r="E40" s="2" t="inlineStr"/>
+      <c r="F40" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #301 (commit 8c27806, merged 2026-05-21)
 source-grounded the 74 remaining non-493 entries in
@@ -2376,29 +2335,29 @@
 shipped:</t>
         </is>
       </c>
-      <c r="G37" s="3" t="inlineStr">
+      <c r="G40" s="2" t="inlineStr">
         <is>
           <t>PR #301; tasks #18 in the in-session task tracker.
 ---</t>
         </is>
       </c>
-      <c r="H37" s="3" t="inlineStr"/>
-    </row>
-    <row r="38" ht="90" customHeight="1">
-      <c r="A38" s="2" t="inlineStr">
+      <c r="H40" s="2" t="inlineStr"/>
+    </row>
+    <row r="41" ht="90" customHeight="1">
+      <c r="A41" s="3" t="inlineStr">
         <is>
           <t>C18</t>
         </is>
       </c>
-      <c r="B38" s="2" t="inlineStr">
+      <c r="B41" s="3" t="inlineStr">
         <is>
           <t>VeritaPolicy "Non CLIA" chapter rename (formerly #3)</t>
         </is>
       </c>
-      <c r="C38" s="2" t="inlineStr"/>
-      <c r="D38" s="2" t="inlineStr"/>
-      <c r="E38" s="2" t="inlineStr"/>
-      <c r="F38" s="2" t="inlineStr">
+      <c r="C41" s="3" t="inlineStr"/>
+      <c r="D41" s="3" t="inlineStr"/>
+      <c r="E41" s="3" t="inlineStr"/>
+      <c r="F41" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #300 (commit 34d7707, merged 2026-05-21)
 renamed all 44 user-facing chapter labels in
@@ -2409,7 +2368,7 @@
 page.</t>
         </is>
       </c>
-      <c r="G38" s="2" t="inlineStr">
+      <c r="G41" s="3" t="inlineStr">
         <is>
           <t>CAP customer screenshot of the /veritapolicy chapter
 headers, 2026-05-01 evening. PR #300; tasks #17 in the in-session
@@ -2417,23 +2376,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H38" s="2" t="inlineStr"/>
-    </row>
-    <row r="39" ht="90" customHeight="1">
-      <c r="A39" s="3" t="inlineStr">
+      <c r="H41" s="3" t="inlineStr"/>
+    </row>
+    <row r="42" ht="90" customHeight="1">
+      <c r="A42" s="2" t="inlineStr">
         <is>
           <t>C19</t>
         </is>
       </c>
-      <c r="B39" s="3" t="inlineStr">
+      <c r="B42" s="2" t="inlineStr">
         <is>
           <t>VeritaStock department-scope toggle (formerly #31)</t>
         </is>
       </c>
-      <c r="C39" s="3" t="inlineStr"/>
-      <c r="D39" s="3" t="inlineStr"/>
-      <c r="E39" s="3" t="inlineStr"/>
-      <c r="F39" s="3" t="inlineStr">
+      <c r="C42" s="2" t="inlineStr"/>
+      <c r="D42" s="2" t="inlineStr"/>
+      <c r="E42" s="2" t="inlineStr"/>
+      <c r="F42" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #319 (commit d01f5fe, merged 2026-05-22)
 shipped the persistent dept-scope toggle on VeritaStockPage. A new
@@ -2444,7 +2403,7 @@
 workspace without re-filtering.</t>
         </is>
       </c>
-      <c r="G39" s="3" t="inlineStr">
+      <c r="G42" s="2" t="inlineStr">
         <is>
           <t>John, San Carlos lab, 2026-05-21. Same conversation that
 drove the vendor dropdown (PR #304), FILTERED VIEW banner (PR #305),
@@ -2452,23 +2411,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H39" s="3" t="inlineStr"/>
-    </row>
-    <row r="40" ht="90" customHeight="1">
-      <c r="A40" s="2" t="inlineStr">
+      <c r="H42" s="2" t="inlineStr"/>
+    </row>
+    <row r="43" ht="90" customHeight="1">
+      <c r="A43" s="3" t="inlineStr">
         <is>
           <t>C20</t>
         </is>
       </c>
-      <c r="B40" s="2" t="inlineStr">
+      <c r="B43" s="3" t="inlineStr">
         <is>
           <t>Primary-lab seat counting (formerly #12)</t>
         </is>
       </c>
-      <c r="C40" s="2" t="inlineStr"/>
-      <c r="D40" s="2" t="inlineStr"/>
-      <c r="E40" s="2" t="inlineStr"/>
-      <c r="F40" s="2" t="inlineStr">
+      <c r="C43" s="3" t="inlineStr"/>
+      <c r="D43" s="3" t="inlineStr"/>
+      <c r="E43" s="3" t="inlineStr"/>
+      <c r="F43" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: is_primary_lab INTEGER NOT NULL DEFAULT 0
 column was added to the lab_members table at db.ts:1276, with the
@@ -2479,7 +2438,7 @@
 is_primary_lab=1 ordering).</t>
         </is>
       </c>
-      <c r="G40" s="2" t="inlineStr">
+      <c r="G43" s="3" t="inlineStr">
         <is>
           <t>2026-05-07 multi-lab discussion. Build shipped as part
 of the Multi-Lab Tier 2 architecture work (Phase 3.x series, prior
@@ -2488,23 +2447,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H40" s="2" t="inlineStr"/>
-    </row>
-    <row r="41" ht="90" customHeight="1">
-      <c r="A41" s="3" t="inlineStr">
+      <c r="H43" s="3" t="inlineStr"/>
+    </row>
+    <row r="44" ht="90" customHeight="1">
+      <c r="A44" s="2" t="inlineStr">
         <is>
           <t>C21</t>
         </is>
       </c>
-      <c r="B41" s="3" t="inlineStr">
+      <c r="B44" s="2" t="inlineStr">
         <is>
           <t>Multi-lab pricing model — Option A (formerly #11)</t>
         </is>
       </c>
-      <c r="C41" s="3" t="inlineStr"/>
-      <c r="D41" s="3" t="inlineStr"/>
-      <c r="E41" s="3" t="inlineStr"/>
-      <c r="F41" s="3" t="inlineStr">
+      <c r="C44" s="2" t="inlineStr"/>
+      <c r="D44" s="2" t="inlineStr"/>
+      <c r="E44" s="2" t="inlineStr"/>
+      <c r="F44" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #322 (commit 0ccd925, merged 2026-05-22)
 added the customer-facing line to the pricing page that reflects
@@ -2517,7 +2476,7 @@
 Enterprise+ block, reads:</t>
         </is>
       </c>
-      <c r="G41" s="3" t="inlineStr">
+      <c r="G44" s="2" t="inlineStr">
         <is>
           <t>2026-05-07 multi-lab discussion (Lisa Veri's
 canonical-case session). PR #322 (initial build); softening PR
@@ -2526,30 +2485,30 @@
 ---</t>
         </is>
       </c>
-      <c r="H41" s="3" t="inlineStr"/>
-    </row>
-    <row r="42" ht="90" customHeight="1">
-      <c r="A42" s="2" t="inlineStr">
+      <c r="H44" s="2" t="inlineStr"/>
+    </row>
+    <row r="45" ht="90" customHeight="1">
+      <c r="A45" s="3" t="inlineStr">
         <is>
           <t>C22</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
+      <c r="B45" s="3" t="inlineStr">
         <is>
           <t>VeritaOps cost-per-test module (formerly #10)</t>
         </is>
       </c>
-      <c r="C42" s="2" t="inlineStr"/>
-      <c r="D42" s="2" t="inlineStr"/>
-      <c r="E42" s="2" t="inlineStr"/>
-      <c r="F42" s="2" t="inlineStr">
+      <c r="C45" s="3" t="inlineStr"/>
+      <c r="D45" s="3" t="inlineStr"/>
+      <c r="E45" s="3" t="inlineStr"/>
+      <c r="F45" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: v1 of the VeritaOps Cost-Per-Reportable-Test
 (CPRT) module shipped across PR #325 through PR #330 on 2026-05-22.
 The module is feature-complete for the typical lab director workflow.</t>
         </is>
       </c>
-      <c r="G42" s="2" t="inlineStr">
+      <c r="G45" s="3" t="inlineStr">
         <is>
           <t>This thread, 2026-05-07 12:05 PM CDT, user message:
 "Parking lot: build an operations module for cost per test
@@ -2558,262 +2517,262 @@
 ---</t>
         </is>
       </c>
-      <c r="H42" s="2" t="inlineStr"/>
-    </row>
-    <row r="43" ht="90" customHeight="1">
-      <c r="A43" s="3" t="inlineStr">
+      <c r="H45" s="3" t="inlineStr"/>
+    </row>
+    <row r="46" ht="90" customHeight="1">
+      <c r="A46" s="2" t="inlineStr">
         <is>
           <t>C23</t>
         </is>
       </c>
-      <c r="B43" s="3" t="inlineStr">
+      <c r="B46" s="2" t="inlineStr">
         <is>
           <t>CCL lab name visual disambiguation in lab switcher (formerly #34)</t>
         </is>
       </c>
-      <c r="C43" s="3" t="inlineStr"/>
-      <c r="D43" s="3" t="inlineStr">
+      <c r="C46" s="2" t="inlineStr"/>
+      <c r="D46" s="2" t="inlineStr">
         <is>
           <t>XS (under 1 day, actual)</t>
         </is>
       </c>
-      <c r="E43" s="3" t="inlineStr">
+      <c r="E46" s="2" t="inlineStr">
         <is>
           <t>Low — cosmetic; only mattered when Lisa or Michael picked the wrong lab from...</t>
         </is>
       </c>
-      <c r="F43" s="3" t="inlineStr">
+      <c r="F46" s="2" t="inlineStr">
         <is>
           <t>Effort: XS (under 1 day, actual)
 Importance: Low — cosmetic; only mattered when Lisa or Michael picked the wrong lab from the dropdown.</t>
         </is>
       </c>
-      <c r="G43" s="3" t="inlineStr">
+      <c r="G46" s="2" t="inlineStr">
         <is>
           <t>flagged 2026-05-23 immediately after provisioning Lisa's CCL lab; closed 2026-05-24.
 ---</t>
         </is>
       </c>
-      <c r="H43" s="3" t="inlineStr"/>
-    </row>
-    <row r="44" ht="90" customHeight="1">
-      <c r="A44" s="2" t="inlineStr">
+      <c r="H46" s="2" t="inlineStr"/>
+    </row>
+    <row r="47" ht="90" customHeight="1">
+      <c r="A47" s="3" t="inlineStr">
         <is>
           <t>C24</t>
         </is>
       </c>
-      <c r="B44" s="2" t="inlineStr">
+      <c r="B47" s="3" t="inlineStr">
         <is>
           <t>VC Unlimited Y1/Y2 price disclosure UX (formerly #35)</t>
         </is>
       </c>
-      <c r="C44" s="2" t="inlineStr"/>
-      <c r="D44" s="2" t="inlineStr">
+      <c r="C47" s="3" t="inlineStr"/>
+      <c r="D47" s="3" t="inlineStr">
         <is>
           <t>XS (under 1 day, actual)</t>
         </is>
       </c>
-      <c r="E44" s="2" t="inlineStr">
+      <c r="E47" s="3" t="inlineStr">
         <is>
           <t>Low when shipped (proactive, no customer complaint yet) — but high if a procu...</t>
         </is>
       </c>
-      <c r="F44" s="2" t="inlineStr">
+      <c r="F47" s="3" t="inlineStr">
         <is>
           <t>Effort: XS (under 1 day, actual)
 Importance: Low when shipped (proactive, no customer complaint yet) — but high if a procurement reviewer later disputes the $499 renewal as undisclosed.</t>
         </is>
       </c>
-      <c r="G44" s="2" t="inlineStr">
+      <c r="G47" s="3" t="inlineStr">
         <is>
           <t>Pricing rebuild 2026-05-23; closed 2026-05-24 proactively before any customer dispute.
 ---</t>
         </is>
       </c>
-      <c r="H44" s="2" t="inlineStr"/>
-    </row>
-    <row r="45" ht="90" customHeight="1">
-      <c r="A45" s="3" t="inlineStr">
+      <c r="H47" s="3" t="inlineStr"/>
+    </row>
+    <row r="48" ht="90" customHeight="1">
+      <c r="A48" s="2" t="inlineStr">
         <is>
           <t>C25</t>
         </is>
       </c>
-      <c r="B45" s="3" t="inlineStr">
+      <c r="B48" s="2" t="inlineStr">
         <is>
           <t>VeritaQC Phase 1 (Levey-Jennings + Westgard live engine) (formerly #20)</t>
         </is>
       </c>
-      <c r="C45" s="3" t="inlineStr"/>
-      <c r="D45" s="3" t="inlineStr">
+      <c r="C48" s="2" t="inlineStr"/>
+      <c r="D48" s="2" t="inlineStr">
         <is>
           <t>L (about 5 days end-to-end, actual: Phase 0 schema → Phase 1A evaluator → 1B...</t>
         </is>
       </c>
-      <c r="E45" s="3" t="inlineStr">
+      <c r="E48" s="2" t="inlineStr">
         <is>
           <t>High — largest single gap vs myLabCompliance.io per Perplexity competitor ana...</t>
         </is>
       </c>
-      <c r="F45" s="3" t="inlineStr">
+      <c r="F48" s="2" t="inlineStr">
         <is>
           <t>Effort: L (about 5 days end-to-end, actual: Phase 0 schema → Phase 1A evaluator → 1B entry UI → 1C daily review → 1D monthly PDF + attestation)
 Importance: High — largest single gap vs myLabCompliance.io per Perplexity competitor analysis; promotes VeritaAssure from documentation tool to lab operations platform.</t>
         </is>
       </c>
-      <c r="G45" s="3" t="inlineStr">
+      <c r="G48" s="2" t="inlineStr">
         <is>
           <t>Perplexity competitor analysis 2026-05-10. Scoping confirmed via the build_phase1_mockup.py iterations 2026-05-24. Shipped 2026-05-25.
 ---</t>
         </is>
       </c>
-      <c r="H45" s="3" t="inlineStr"/>
-    </row>
-    <row r="46" ht="90" customHeight="1">
-      <c r="A46" s="2" t="inlineStr">
+      <c r="H48" s="2" t="inlineStr"/>
+    </row>
+    <row r="49" ht="90" customHeight="1">
+      <c r="A49" s="3" t="inlineStr">
         <is>
           <t>C26</t>
         </is>
       </c>
-      <c r="B46" s="2" t="inlineStr">
+      <c r="B49" s="3" t="inlineStr">
         <is>
           <t>VeritaLab CMS-116 application support + state licensing registry (formerly #22)</t>
         </is>
       </c>
-      <c r="C46" s="2" t="inlineStr"/>
-      <c r="D46" s="2" t="inlineStr">
+      <c r="C49" s="3" t="inlineStr"/>
+      <c r="D49" s="3" t="inlineStr">
         <is>
           <t>M (1-2 weeks for v1, actual)</t>
         </is>
       </c>
-      <c r="E46" s="2" t="inlineStr">
+      <c r="E49" s="3" t="inlineStr">
         <is>
           <t>Medium — competitor parity (myLabCompliance.io) plus useful at lab startup an...</t>
         </is>
       </c>
-      <c r="F46" s="2" t="inlineStr">
+      <c r="F49" s="3" t="inlineStr">
         <is>
           <t>Effort: M (1-2 weeks for v1, actual)
 Importance: Medium — competitor parity (myLabCompliance.io) plus useful at lab startup and at certificate-type changes.</t>
         </is>
       </c>
-      <c r="G46" s="2" t="inlineStr">
+      <c r="G49" s="3" t="inlineStr">
         <is>
           <t>Perplexity competitor analysis (myLabCompliance.io), 2026-05-10. Reclassified as a VeritaLab extension 2026-05-25. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H46" s="2" t="inlineStr"/>
-    </row>
-    <row r="47" ht="90" customHeight="1">
-      <c r="A47" s="3" t="inlineStr">
+      <c r="H49" s="3" t="inlineStr"/>
+    </row>
+    <row r="50" ht="90" customHeight="1">
+      <c r="A50" s="2" t="inlineStr">
         <is>
           <t>C27</t>
         </is>
       </c>
-      <c r="B47" s="3" t="inlineStr">
+      <c r="B50" s="2" t="inlineStr">
         <is>
           <t>Active vs view-only seat split (formerly #33)</t>
         </is>
       </c>
-      <c r="C47" s="3" t="inlineStr"/>
-      <c r="D47" s="3" t="inlineStr">
+      <c r="C50" s="2" t="inlineStr"/>
+      <c r="D50" s="2" t="inlineStr">
         <is>
           <t>M (~1 week of engineering, actual: shipped in a single multi-PR session)</t>
         </is>
       </c>
-      <c r="E47" s="3" t="inlineStr">
+      <c r="E50" s="2" t="inlineStr">
         <is>
           <t>Medium — closed the gap between /pricing copy and product behavior; gives sal...</t>
         </is>
       </c>
-      <c r="F47" s="3" t="inlineStr">
+      <c r="F50" s="2" t="inlineStr">
         <is>
           <t>Effort: M (~1 week of engineering, actual: shipped in a single multi-PR session)
 Importance: Medium — closed the gap between /pricing copy and product behavior; gives sales a clean answer for "do you charge for our medical director?"</t>
         </is>
       </c>
-      <c r="G47" s="3" t="inlineStr">
+      <c r="G50" s="2" t="inlineStr">
         <is>
           <t>Pricing analysis doc Decision 3 (2026-05-21); MEDIUM scenario revised 2026-05-29 to retire the "unlimited view-only" claim. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H47" s="3" t="inlineStr"/>
-    </row>
-    <row r="48" ht="90" customHeight="1">
-      <c r="A48" s="2" t="inlineStr">
+      <c r="H50" s="2" t="inlineStr"/>
+    </row>
+    <row r="51" ht="90" customHeight="1">
+      <c r="A51" s="3" t="inlineStr">
         <is>
           <t>C28</t>
         </is>
       </c>
-      <c r="B48" s="2" t="inlineStr">
+      <c r="B51" s="3" t="inlineStr">
         <is>
           <t>"Why VeritaCheck" comparative one-pager (formerly #37)</t>
         </is>
       </c>
-      <c r="C48" s="2" t="inlineStr"/>
-      <c r="D48" s="2" t="inlineStr">
+      <c r="C51" s="3" t="inlineStr"/>
+      <c r="D51" s="3" t="inlineStr">
         <is>
           <t>S (one design pass + four claim paragraphs + PDF + matching marketing-site pa...</t>
         </is>
       </c>
-      <c r="E48" s="2" t="inlineStr">
+      <c r="E51" s="3" t="inlineStr">
         <is>
           <t>Medium — closed a positioning gap surfaced by six COLA conference attendees a...</t>
         </is>
       </c>
-      <c r="F48" s="2" t="inlineStr">
+      <c r="F51" s="3" t="inlineStr">
         <is>
           <t>Effort: S (one design pass + four claim paragraphs + PDF + matching marketing-site page, actual)
 Importance: Medium — closed a positioning gap surfaced by six COLA conference attendees attached to a legacy verification tool; converts product-quality advantage into a leave-behind Lisa can hand out.</t>
         </is>
       </c>
-      <c r="G48" s="2" t="inlineStr">
+      <c r="G51" s="3" t="inlineStr">
         <is>
           <t>2026-05-11 / 2026-05-12 conference notes review with Michael. Conference attendees (Whitehead, Odegard, Othman, Molinelli, Kyle, Allred) expressed interest in equivalent / superior product. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H48" s="2" t="inlineStr"/>
-    </row>
-    <row r="49" ht="90" customHeight="1">
-      <c r="A49" s="3" t="inlineStr">
+      <c r="H51" s="3" t="inlineStr"/>
+    </row>
+    <row r="52" ht="90" customHeight="1">
+      <c r="A52" s="2" t="inlineStr">
         <is>
           <t>C29</t>
         </is>
       </c>
-      <c r="B49" s="3" t="inlineStr">
+      <c r="B52" s="2" t="inlineStr">
         <is>
           <t>VeritaPolicy approval workflow — MediaLab functional mirror</t>
         </is>
       </c>
-      <c r="C49" s="3" t="inlineStr"/>
-      <c r="D49" s="3" t="inlineStr">
+      <c r="C52" s="2" t="inlineStr"/>
+      <c r="D52" s="2" t="inlineStr">
         <is>
           <t>XL (one focused session, 12 PRs landed)</t>
         </is>
       </c>
-      <c r="E49" s="3" t="inlineStr">
+      <c r="E52" s="2" t="inlineStr">
         <is>
           <t>High — replaces MediaLab Document Control ($752/$2,250 starting price, scalin...</t>
         </is>
       </c>
-      <c r="F49" s="3" t="inlineStr">
+      <c r="F52" s="2" t="inlineStr">
         <is>
           <t>Effort: XL (one focused session, 12 PRs landed)
 Importance: High — replaces MediaLab Document Control ($752/$2,250 starting price, scaling to $10K-$20K/yr at enterprise per Capterra public data) with an included VeritaPolicy feature; closes a real positioning gap and gives sales a direct comparator line.</t>
         </is>
       </c>
-      <c r="G49" s="3" t="inlineStr">
+      <c r="G52" s="2" t="inlineStr">
         <is>
           <t>Pricing strategy conversation 2026-05-29 (Michael: "I don't like bolt-ons; we should replicate this") → scoped 8 phases → shipped all 12 PRs in single session. Shipped 2026-05-29.
 ---</t>
         </is>
       </c>
-      <c r="H49" s="3" t="inlineStr"/>
+      <c r="H52" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H49"/>
+  <autoFilter ref="A1:H52"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
TASK: close parking-lot #50/#51/#52 as shipped (#1363)
PLAN:
  1. move #50/#51/#52 from OPEN to CLOSED (C49/C50/C51) with prod-verified evidence
  2. regenerate PARKING_LOT.xlsx (OPEN 16 to 13, CLOSED +3)

Self-check:
  - docs-only, Gate 3 N/A
  - #52 closed as core member picker; residual optional UX noted in C51
  - keys at line start
</commit_message>
<xml_diff>
--- a/PARKING_LOT.xlsx
+++ b/PARKING_LOT.xlsx
@@ -12,8 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RETIRED" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$49</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$52</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RETIRED'!$A$1:$H$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1051,7 +1051,10 @@
       <c r="C13" s="3" t="inlineStr">
         <is>
           <t>Open. Not started. Needs a one-line scope confirmation (which master list).
----</t>
+---
+_(item #50 closed 2026-09-28; shipped PR #1356, prod-verified, see C49 below)_
+---
+_(item #51 closed 2026-09-28;...</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
@@ -1080,163 +1083,41 @@
     <row r="14" ht="90" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>53</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Competency "assessed this cycle" uses a flat 365-day window</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr"/>
+          <t>VeritaCEU: curated free-continuing-education provider list (seed / reference)</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Open, reference captured. Not started.</t>
+        </is>
+      </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>S-M - anchor the coverage-map "assessed this cycle" to the person's actual CL...</t>
+          <t>S (1-2 days to seed a curated provider list and surface it in VeritaCEU; XS t...</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Medium - in an employee's first year the semiannual windows differ from a fla...</t>
+          <t>Low-Medium — quality-of-life for VeritaCEU users (find free CE fast); not blo...</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>Effort: S-M - anchor the coverage-map "assessed this cycle" to the person's actual CLIA cadence (semiannual in year 1 per 42 CFR 493.1451(b)(8), annual thereafter) from staff_competency_schedules, instead of the v1 flat 365-day lookback.
-Importance: Medium - in an employee's first year the semiannual windows differ from a flat annual window, so a first-year assessment could read as current slightly longer or shorter than the true cadence. Fine for the common annual case; refine for year-1 accuracy.</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-24 session, VeritaComp coverage map (#48 Phase 3) v1 simplification, noted in PR #1319.
----</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr"/>
-    </row>
-    <row r="15" ht="90" customHeight="1">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>51</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>VeritaTrack task owner + owner-scoped reminder routing</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>Open, not started. Placeholder pending build. Open questions: is the owner a staff_employee or a seat user, and how are reminder recipients currently chosen.</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>S-M (1-3 days to ~1.5 weeks) — add an owner on a VeritaTrack task, selectable...</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="inlineStr">
-        <is>
-          <t>Medium — cuts reminder-email noise so people only get the tasks that are thei...</t>
-        </is>
-      </c>
-      <c r="F15" s="3" t="inlineStr">
-        <is>
-          <t>Michael, verbatim (2026-09-28): "In veritatask, we should be able to assign an owner from staff that are built, then in the reminder section, we should be able to designate reminder emails only to the owner. The hem person does not need the chemistry reminders, etc." Module note: there is no VeritaTask module in the codebase; the task/reminder surface is VeritaTrack (client/src/pages/VeritaTrackAppPage.tsx), so this lands there. Today VeritaTrack tasks are not owned by a specific staff member and reminder emails are not recipient-scoped to an owner. The build adds (a) an owner selector on each task drawn from the lab's VeritaStaff roster, and (b) a reminder setting that routes the reminder email to only that owner. Confirm the current reminder recipient model before sizing.</t>
-        </is>
-      </c>
-      <c r="G15" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-28 session, Michael "for later (placeholder)" optimization #1 (relaying from the Lab Members / VeritaAssure screens).</t>
-        </is>
-      </c>
-      <c r="H15" s="3" t="inlineStr">
-        <is>
-          <t>Post-COLA. No customer urgency.
----</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="90" customHeight="1">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>52</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>Medical Director seat via account-grant dropdown (designate / transfer MD)</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Open, not started. Placeholder. Confirm the current MD-seat assignment path and the one-MD-per-location enforcement point before sizing.</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>S-M (1-3 days to ~1.5 weeks) — move MD-seat assignment onto the same per-memb...</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>Medium-High — the MD seat is a recurring friction point (Georgetown, SCAHC MD...</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>Michael, verbatim (2026-09-28): "The way we are doing the medical director seat is silly. Why not just use the account grant dropdown to give a medical director seat. If the person is already in, then we should just be able to grant the medical director seat the same way we promote people to admin or reduce them to staff as long as we only have 1 per location. Maybe do another block like the transfer ownership block as 'designate medical director or transfer medical director'." So: fold the MD seat into the existing member role dropdown (Admin / Staff / ... + Medical Director) with a single-MD-per-lab constraint, and add a dedicated designate-or-transfer-MD block that mirrors the transfer-ownership UX for changing the MD. Cross-ref [[project_medical_director_designation]] and the seat model.</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 session, Michael "for later (placeholder)" optimization #3 (relaying from the Lab Members screen).</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>Post-COLA. No customer urgency.
----</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="90" customHeight="1">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>53</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>VeritaCEU: curated free-continuing-education provider list (seed / reference)</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>Open, reference captured. Not started.</t>
-        </is>
-      </c>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>S (1-2 days to seed a curated provider list and surface it in VeritaCEU; XS t...</t>
-        </is>
-      </c>
-      <c r="E17" s="3" t="inlineStr">
-        <is>
-          <t>Low-Medium — quality-of-life for VeritaCEU users (find free CE fast); not blo...</t>
-        </is>
-      </c>
-      <c r="F17" s="3" t="inlineStr">
         <is>
           <t>Effort: S (1-2 days to seed a curated provider list and surface it in VeritaCEU; XS to just store the reference)
 Importance: Low-Medium — quality-of-life for VeritaCEU users (find free CE fast); not blocking any sale.</t>
         </is>
       </c>
-      <c r="G17" s="3" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>Jennifer Small (jennifer.small@lifepointhealth.net) email 2026-09-25, forwarded by Michael 2026-09-28 for the future CEU module.</t>
         </is>
       </c>
-      <c r="H17" s="3" t="inlineStr">
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>Post-COLA. No customer urgency.
 ---</t>
@@ -1244,7 +1125,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H17"/>
+  <autoFilter ref="A1:H14"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1255,7 +1136,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H49"/>
+  <dimension ref="A1:H52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1313,24 +1194,24 @@
     <row r="2" ht="90" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>C47</t>
+          <t>C49</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Unregulated-analyte / Alternative Assessment (AAA) coverage (was #18)</t>
+          <t>Competency "assessed this cycle" cadence-aware window (was #50)</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr"/>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>was S (Phase 3) / Importance: Medium</t>
+          <t>was S-M / Importance: Medium</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Effort: was S (Phase 3) / Importance: Medium</t>
+          <t>Effort: was S-M / Importance: Medium</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
@@ -1339,24 +1220,24 @@
     <row r="3" ht="90" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>C48</t>
+          <t>C50</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>VeritaResponse post-survey deficiency module (was #17)</t>
+          <t>VeritaTrack task owner + owner-only reminder routing (was #51)</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr"/>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>was XL / Importance: High</t>
+          <t>was S-M / Importance: Medium</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Effort: was XL / Importance: High</t>
+          <t>Effort: was S-M / Importance: Medium</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr"/>
@@ -1365,93 +1246,90 @@
     <row r="4" ht="90" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>C45</t>
+          <t>C51</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Unify coverage/competency recurrence helper (was #49) - closed as non-issue</t>
+          <t>Designate Medical Director by picking a lab member (was #52, core)</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr"/>
-      <c r="D4" s="2" t="inlineStr"/>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>was S-M / Importance: Medium-High</t>
+        </is>
+      </c>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: Investigated 2026-09-24 before building. The coverage recurrence math (+6-month interval, signed-resets-to-missing, nextDueOn/overdue, isFailVerdict) is ALREADY single-source in server/veritacheckCoverage.ts (computeCoverageFrom). server/coverageReport.ts and the routes.ts coverage export do not recompute it; they consume the computed nextDueOn/overdue/status fields and apply small surface-specific presentation labels (deliberately different vocabularies per surface, so they should not be merged). The only truly identical duplicate is a one-line date formatter. The competency "owed" derivation is NOT the same cadence: competency follows the CLIA milestone schedule (initial / semiannual year 1 / annual, 42 CFR 493.1451(b)(8) and 493.1235), which is a different regulatory interval from the coverage 6-month rule (493.1281 / 493.1255) and must stay separate. No worthwhile extraction; merging the two cadences would be wrong. Closed 2026-09-24. (The year-1 competency-window refinement remains tracked separately as #50.)</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-24 session, "keep working" pass; scoped read-only, found no real duplication.
----</t>
-        </is>
-      </c>
+          <t>Effort: was S-M / Importance: Medium-High</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr"/>
       <c r="H4" s="2" t="inlineStr"/>
     </row>
     <row r="5" ht="90" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>C46</t>
+          <t>C47</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Verified-users product-update send path (wrong-list incident fix)</t>
+          <t>Unregulated-analyte / Alternative Assessment (AAA) coverage (was #18)</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr"/>
-      <c r="D5" s="3" t="inlineStr"/>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>was S (Phase 3) / Importance: Medium</t>
+        </is>
+      </c>
       <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: Shipped PR #1324 (merged 4e05506a, deploy ACTIVE). New POST /api/admin/users/send targets registered VeritaAssure account holders (the users table), never the Lab Director's Briefing subscriber list. Separate explicitly-named endpoint (not a flag with a dangerous default), account-holder email framing, excludes suppressed emails and RFC-reserved test domains, CC owner, dryRun + testTo previews. Public unsubscribe now upserts a suppression row so opt-outs are honored across both audiences. Live dryRun: 49 verified-user recipients vs 673 on the Briefing list. Receipts: scripts/verify-product-update-send.mts 24/24, tsc clean, rendered sample inspected. Fixes the fallout from the 2026-09-23/24 wrong-list send (a product update went to the 675-person Briefing list). Nothing sends without Michael's explicit "send it."</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-24 session; Michael selected this as the next build after the #41 close.
----</t>
-        </is>
-      </c>
+          <t>Effort: was S (Phase 3) / Importance: Medium</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr"/>
       <c r="H5" s="3" t="inlineStr"/>
     </row>
     <row r="6" ht="90" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>C44</t>
+          <t>C48</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Verify-script convention backfill (was #41) + audit matcher fix</t>
+          <t>VeritaResponse post-survey deficiency module (was #17)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr"/>
-      <c r="D6" s="2" t="inlineStr"/>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>was XL / Importance: High</t>
+        </is>
+      </c>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: #41 was fully backfilled on 2026-06-13 (all 8 high-stakes scripts landed; see C30); it had only been mis-filed in OPEN. A 2026-09-24 re-audit initially reported 4 of 5 recent math/logic commits as missing a verify script, which was a FALSE POSITIVE: scripts/audit_verify_script_coverage.py matched only scripts/verify-*.js / .cjs, so it ignored the .mjs / .mts / .ts verify scripts the repo now ships (e.g. verify-ptcoag-multi.mts, verify-tea-criterion-format.mjs). Fixed the matcher to accept .js/.cjs/.mjs/.ts/.mts; re-run shows 5 of 5 covered, 0 debt. The convention is being followed. Closed 2026-09-24.</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-24 session, "keep working" pass; audit tooling bug found + fixed.
----</t>
-        </is>
-      </c>
+          <t>Effort: was XL / Importance: High</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr"/>
       <c r="H6" s="2" t="inlineStr"/>
     </row>
     <row r="7" ht="90" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>C43</t>
+          <t>C45</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>VeritaStaff instrument-centric (dual) assignment view</t>
+          <t>Unify coverage/competency recurrence helper (was #49) - closed as non-issue</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr"/>
@@ -1459,12 +1337,12 @@
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1320. GET/PUT /staff/instruments/:id/employees (transpose of the per-employee endpoints); an "Assign by Instrument" dialog lets a director pick a test system or manual test and check off who runs it. Same staff_employee_instruments join, with the 42 CFR 493.1235(a) duty-change event emitted on newly-added pairs so both orientations trigger the same reassessment. GET verified live on SCAHC lab 2. Closed 2026-09-24.</t>
+          <t>Closure evidence: Investigated 2026-09-24 before building. The coverage recurrence math (+6-month interval, signed-resets-to-missing, nextDueOn/overdue, isFailVerdict) is ALREADY single-source in server/veritacheckCoverage.ts (computeCoverageFrom). server/coverageReport.ts and the routes.ts coverage export do not recompute it; they consume the computed nextDueOn/overdue/status fields and apply small surface-specific presentation labels (deliberately different vocabularies per surface, so they should not be merged). The only truly identical duplicate is a one-line date formatter. The competency "owed" derivation is NOT the same cadence: competency follows the CLIA milestone schedule (initial / semiannual year 1 / annual, 42 CFR 493.1451(b)(8) and 493.1235), which is a different regulatory interval from the coverage 6-month rule (493.1281 / 493.1255) and must stay separate. No worthwhile extraction; merging the two cadences would be wrong. Closed 2026-09-24. (The year-1 competency-window refinement remains tracked separately as #50.)</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>2026-09-24 session, Michael ("in staff we should also give the dual view when assigning coverage to test systems or manual tests").
+          <t>2026-09-24 session, "keep working" pass; scoped read-only, found no real duplication.
 ---</t>
         </is>
       </c>
@@ -1473,12 +1351,12 @@
     <row r="8" ht="90" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>C42</t>
+          <t>C46</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>VeritaComp coverage map (required-vs-assessed matrix, dual view)</t>
+          <t>Verified-users product-update send path (wrong-list incident fix)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr"/>
@@ -1486,12 +1364,12 @@
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1319 (+ status layer PR #1316). /competency/owed returns per-item assessed (locked passing assessment this cycle on a covering method group) + per-employee CLIA status; CompetencyCoverageMap renders a By-employee / By-instrument matrix (Assessed / Owed / Overdue / Gap). Verified live on SCAHC lab 2 (owed 116, assessed 2, gaps 0). Completes #48 as the VeritaCheck-parity coverage map. Closed 2026-09-24.</t>
+          <t>Closure evidence: Shipped PR #1324 (merged 4e05506a, deploy ACTIVE). New POST /api/admin/users/send targets registered VeritaAssure account holders (the users table), never the Lab Director's Briefing subscriber list. Separate explicitly-named endpoint (not a flag with a dangerous default), account-holder email framing, excludes suppressed emails and RFC-reserved test domains, CC owner, dryRun + testTo previews. Public unsubscribe now upserts a suppression row so opt-outs are honored across both audiences. Live dryRun: 49 verified-user recipients vs 673 on the Briefing list. Receipts: scripts/verify-product-update-send.mts 24/24, tsc clean, rendered sample inspected. Fixes the fallout from the 2026-09-23/24 wrong-list send (a product update went to the 675-person Briefing list). Nothing sends without Michael's explicit "send it."</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 session, Michael ("are we building the competencies to have a coverage map, same as veritacheck?" then "build it").
+          <t>2026-09-24 session; Michael selected this as the next build after the #41 close.
 ---</t>
         </is>
       </c>
@@ -1500,12 +1378,12 @@
     <row r="9" ht="90" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>C41</t>
+          <t>C44</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>VeritaCheck coverage recurrence (method comparison + cal-ver/linearity + reports)</t>
+          <t>Verify-script convention backfill (was #41) + audit matcher fix</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr"/>
@@ -1513,12 +1391,12 @@
       <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: PRs #1317 (method comparison), #1318 (cal-ver/linearity), #1321 (report Next-due columns). Periodic verification (correlation/method comparison 42 CFR 493.1281; cal-ver/linearity 42 CFR 493.1255; both 6-month) now recurs: a signed study banks the cycle and rolls to next-due = signed + 6 months instead of reading "done" forever. Status Missing/Failed/Completed-unsigned + a "Next due on" column on-screen and in both coverage exports; also credits the previously-ignored "correlation" study type. Root cause: computeCoverageFrom marked requirements done on mere existence, no date logic. Verified live on SCAHC lab 2 (101 correlations + 11 cal-ver rows now carry a next-due). Engine-level, all facilities. Closed 2026-09-24.</t>
+          <t>Closure evidence: #41 was fully backfilled on 2026-06-13 (all 8 high-stakes scripts landed; see C30); it had only been mis-filed in OPEN. A 2026-09-24 re-audit initially reported 4 of 5 recent math/logic commits as missing a verify script, which was a FALSE POSITIVE: scripts/audit_verify_script_coverage.py matched only scripts/verify-*.js / .cjs, so it ignored the .mjs / .mts / .ts verify scripts the repo now ships (e.g. verify-ptcoag-multi.mts, verify-tea-criterion-format.mjs). Fixed the matcher to accept .js/.cjs/.mjs/.ts/.mts; re-run shows 5 of 5 covered, 0 debt. The convention is being followed. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>2026-09-24 session, Michael ("Look at San Carlos... they finished their last set of correlations (all 103) but their menu never reset").
+          <t>2026-09-24 session, "keep working" pass; audit tooling bug found + fixed.
 ---</t>
         </is>
       </c>
@@ -1527,12 +1405,12 @@
     <row r="10" ht="90" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>C40</t>
+          <t>C43</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>VeritaComp Competencies Owed derived from VeritaStaff, with gap detection (was #48)</t>
+          <t>VeritaStaff instrument-centric (dual) assignment view</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr"/>
@@ -1540,12 +1418,12 @@
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1314 (squash 2bcb0db9). GET /api/labs/:labId/competency/owed derives each VeritaStaff testing employee's owed competencies from their assigned instruments (staff_employee_instruments -&gt; veritamap_instruments + tests), on the CLIA timeline, and flags instruments not covered by any competency program as gaps. CompetenciesOwedSection renders it on the VeritaComp landing page. Reuses the shipped bridge + suggested-method-groups match rules; no new tables. Verified live on prod with real assignment data: 2 instruments assigned to a demo staffer produced owed=2, gaps=2 (HIGH, Technical Supervisor), then reverted cleanly. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1320. GET/PUT /staff/instruments/:id/employees (transpose of the per-employee endpoints); an "Assign by Instrument" dialog lets a director pick a test system or manual test and check off who runs it. Same staff_employee_instruments join, with the 42 CFR 493.1235(a) duty-change event emitted on newly-added pairs so both orientations trigger the same reassessment. GET verified live on SCAHC lab 2. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23/24 session, Michael ("veritacomp bases what competencies they owe (currently untrue, but needs to be true)"). Option 1 (unify roster on VeritaStaff, match instruments by id).
+          <t>2026-09-24 session, Michael ("in staff we should also give the dual view when assigning coverage to test systems or manual tests").
 ---</t>
         </is>
       </c>
@@ -1554,12 +1432,12 @@
     <row r="11" ht="90" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>C39</t>
+          <t>C42</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>VeritaScan line items can attach or link evidence (was #46)</t>
+          <t>VeritaComp coverage map (required-vs-assessed matrix, dual view)</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr"/>
@@ -1567,12 +1445,12 @@
       <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1312 (squash a1dda93d). VeritaScan scan checklist items now show linked evidence as chips (open link, remove) plus a writer "Link evidence" affordance whose picker links an existing VeritaDC/Library document; a shortcut deep-links to the Library for new (governed) documents. Reuses the already-shipped lab_documents + document_checklist_links + coverage endpoints (URL-pointer only, no file storage, no new tables). Browser-verified live on prod (scan 23): the affordance renders and the picker opens. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1319 (+ status layer PR #1316). /competency/owed returns per-item assessed (locked passing assessment this cycle on a covering method group) + per-employee CLIA status; CompetencyCoverageMap renders a By-employee / By-instrument matrix (Assessed / Owed / Overdue / Gap). Verified live on SCAHC lab 2 (owed 116, assessed 2, gaps 0). Completes #48 as the VeritaCheck-parity coverage map. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>2026-09-23 session, Michael. Recurring request. Companion: cross-module evidence display on the VeritaDC policy shipped in PR #1313 (by-target cross-links surfaced in the policy View modal, browser-verified live).
+          <t>2026-09-24 session, Michael ("are we building the competencies to have a coverage map, same as veritacheck?" then "build it").
 ---</t>
         </is>
       </c>
@@ -1581,12 +1459,12 @@
     <row r="12" ht="90" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>C38</t>
+          <t>C41</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>VeritaTrack calendar month cells expand to reveal hidden tasks (was #45)</t>
+          <t>VeritaCheck coverage recurrence (method comparison + cal-ver/linearity + reports)</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr"/>
@@ -1594,12 +1472,12 @@
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: VeritaTrack CalendarView month cells with more than three tasks now expand in place (chevron, "+N more" toggling to "Show less", due dates), so no task is hidden with no path to it (client/src/pages/VeritaTrackAppPage.tsx CalendarView). Shipped 2026-09-23. Closed 2026-09-24.</t>
+          <t>Closure evidence: PRs #1317 (method comparison), #1318 (cal-ver/linearity), #1321 (report Next-due columns). Periodic verification (correlation/method comparison 42 CFR 493.1281; cal-ver/linearity 42 CFR 493.1255; both 6-month) now recurs: a signed study banks the cycle and rolls to next-due = signed + 6 months instead of reading "done" forever. Status Missing/Failed/Completed-unsigned + a "Next due on" column on-screen and in both coverage exports; also credits the previously-ignored "correlation" study type. Root cause: computeCoverageFrom marked requirements done on mere existence, no date logic. Verified live on SCAHC lab 2 (101 correlations + 11 cal-ver rows now carry a next-due). Engine-level, all facilities. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23 session, Michael screenshot of the VeritaTrack calendar (lab 3, September cell).
+          <t>2026-09-24 session, Michael ("Look at San Carlos... they finished their last set of correlations (all 103) but their menu never reset").
 ---</t>
         </is>
       </c>
@@ -1608,12 +1486,12 @@
     <row r="13" ht="90" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>C37</t>
+          <t>C40</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Long Excel column headers no longer clip CFR citations (was #44)</t>
+          <t>VeritaComp Competencies Owed derived from VeritaStaff, with gap detection (was #48)</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr"/>
@@ -1621,12 +1499,12 @@
       <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. The VeritaMap export derives the header row height from the longest wrapped header via headerRowHeight(headers, colWidths) (server/routes.ts:15935) instead of a fixed 20, so "Reference Range Attestation (42 CFR 493.1253)" and the other long headers print in full. No new code this session. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1314 (squash 2bcb0db9). GET /api/labs/:labId/competency/owed derives each VeritaStaff testing employee's owed competencies from their assigned instruments (staff_employee_instruments -&gt; veritamap_instruments + tests), on the CLIA timeline, and flags instruments not covered by any competency program as gaps. CompetenciesOwedSection renders it on the VeritaComp landing page. Reuses the shipped bridge + suggested-method-groups match rules; no new tables. Verified live on prod with real assignment data: 2 instruments assigned to a demo staffer produced owed=2, gaps=2 (HIGH, Technical Supervisor), then reverted cleanly. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+          <t>2026-09-23/24 session, Michael ("veritacomp bases what competencies they owe (currently untrue, but needs to be true)"). Option 1 (unify roster on VeritaStaff, match instruments by id).
 ---</t>
         </is>
       </c>
@@ -1635,12 +1513,12 @@
     <row r="14" ht="90" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>C36</t>
+          <t>C39</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>License stamp no longer clobbers the §6 header/footer or names the wrong lab (was #43)</t>
+          <t>VeritaScan line items can attach or link evidence (was #46)</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr"/>
@@ -1648,12 +1526,12 @@
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. setHeaderFooter (shared/licenseExceljs.ts:155-209) now preserves an existing §6 header and appends (not overwrites) the footer left section, and customer-facing exports name the scoped lab: the VeritaScan library export reads req.scope.lab.name / clia_number (server/routes.ts:16572-16573), not the licensee. No new code this session (avoided regressing the existing fix). Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1312 (squash a1dda93d). VeritaScan scan checklist items now show linked evidence as chips (open link, remove) plus a writer "Link evidence" affordance whose picker links an existing VeritaDC/Library document; a shortcut deep-links to the Library for new (governed) documents. Reuses the already-shipped lab_documents + document_checklist_links + coverage endpoints (URL-pointer only, no file storage, no new tables). Browser-verified live on prod (scan 23): the affordance renders and the picker opens. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+          <t>2026-09-23 session, Michael. Recurring request. Companion: cross-module evidence display on the VeritaDC policy shipped in PR #1313 (by-target cross-links surfaced in the policy View modal, browser-verified live).
 ---</t>
         </is>
       </c>
@@ -1662,18 +1540,99 @@
     <row r="15" ht="90" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>C34</t>
+          <t>C38</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Wire the two static-audit guards into CI (was #43)</t>
+          <t>VeritaTrack calendar month cells expand to reveal hidden tasks (was #45)</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr"/>
       <c r="D15" s="3" t="inlineStr"/>
       <c r="E15" s="3" t="inlineStr"/>
       <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Closure evidence: VeritaTrack CalendarView month cells with more than three tasks now expand in place (chevron, "+N more" toggling to "Show less", due dates), so no task is hidden with no path to it (client/src/pages/VeritaTrackAppPage.tsx CalendarView). Shipped 2026-09-23. Closed 2026-09-24.</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-23 session, Michael screenshot of the VeritaTrack calendar (lab 3, September cell).
+---</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16" ht="90" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>C37</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Long Excel column headers no longer clip CFR citations (was #44)</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr"/>
+      <c r="D16" s="2" t="inlineStr"/>
+      <c r="E16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. The VeritaMap export derives the header row height from the longest wrapped header via headerRowHeight(headers, colWidths) (server/routes.ts:15935) instead of a fixed 20, so "Reference Range Attestation (42 CFR 493.1253)" and the other long headers print in full. No new code this session. Closed 2026-09-24.</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+---</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17" ht="90" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>C36</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>License stamp no longer clobbers the §6 header/footer or names the wrong lab (was #43)</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr"/>
+      <c r="D17" s="3" t="inlineStr"/>
+      <c r="E17" s="3" t="inlineStr"/>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. setHeaderFooter (shared/licenseExceljs.ts:155-209) now preserves an existing §6 header and appends (not overwrites) the footer left section, and customer-facing exports name the scoped lab: the VeritaScan library export reads req.scope.lab.name / clia_number (server/routes.ts:16572-16573), not the licensee. No new code this session (avoided regressing the existing fix). Closed 2026-09-24.</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+---</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr"/>
+    </row>
+    <row r="18" ht="90" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>C34</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Wire the two static-audit guards into CI (was #43)</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr"/>
+      <c r="D18" s="2" t="inlineStr"/>
+      <c r="E18" s="2" t="inlineStr"/>
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: both guards wired into the Multi-Lab Mutations Audit CI
 workflow (.github/workflows/multilab-mutations-audit.yml) as steps:
@@ -1685,24 +1644,24 @@
 (same caveat as the existing guards already in that workflow).</t>
         </is>
       </c>
-      <c r="G15" s="3" t="inlineStr"/>
-      <c r="H15" s="3" t="inlineStr"/>
-    </row>
-    <row r="16" ht="90" customHeight="1">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr"/>
+      <c r="H18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19" ht="90" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>C35</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>Legacy /api/studies over-returns studies across labs (was #44)</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr"/>
-      <c r="D16" s="2" t="inlineStr"/>
-      <c r="E16" s="2" t="inlineStr"/>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="C19" s="3" t="inlineStr"/>
+      <c r="D19" s="3" t="inlineStr"/>
+      <c r="E19" s="3" t="inlineStr"/>
+      <c r="F19" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: GET /api/studies now scopes its list to the active lab
 when one is resolved from the Referer (server/routes.ts), so every returned row
@@ -1712,24 +1671,24 @@
 mirroring the /api/labs/:labId/studies handler. Closed 2026-06-14.</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr"/>
-      <c r="H16" s="2" t="inlineStr"/>
-    </row>
-    <row r="17" ht="90" customHeight="1">
-      <c r="A17" s="3" t="inlineStr">
+      <c r="G19" s="3" t="inlineStr"/>
+      <c r="H19" s="3" t="inlineStr"/>
+    </row>
+    <row r="20" ht="90" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>C30</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>Verify-script convention backfill (was #41)</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr"/>
-      <c r="D17" s="3" t="inlineStr"/>
-      <c r="E17" s="3" t="inlineStr"/>
-      <c r="F17" s="3" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr"/>
+      <c r="D20" s="2" t="inlineStr"/>
+      <c r="E20" s="2" t="inlineStr"/>
+      <c r="F20" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: all 8 high-stakes math/logic commits now ship a paired
 scripts/verify-*.js (EP17 sensitivity, Deming lot-to-lot, CUMSUM+QC+multi-analyte,
@@ -1737,30 +1696,30 @@
 TEa boundary), per the strike-throughs in #41. Closed 2026-06-13.</t>
         </is>
       </c>
-      <c r="G17" s="3" t="inlineStr">
+      <c r="G20" s="2" t="inlineStr">
         <is>
           <t>scripts/audit_verify_script_coverage.py lookback, 2026-06-02; backfills
 landed 2026-06-03..06.
 ---</t>
         </is>
       </c>
-      <c r="H17" s="3" t="inlineStr"/>
-    </row>
-    <row r="18" ht="90" customHeight="1">
-      <c r="A18" s="2" t="inlineStr">
+      <c r="H20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21" ht="90" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>C31</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>VeritaPT AAA create/update/delete silently no-op in the multi-lab UI</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr"/>
-      <c r="D18" s="2" t="inlineStr"/>
-      <c r="E18" s="2" t="inlineStr"/>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="C21" s="3" t="inlineStr"/>
+      <c r="D21" s="3" t="inlineStr"/>
+      <c r="E21" s="3" t="inlineStr"/>
+      <c r="F21" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #754 (commit 92ad499) added lab-scoped POST/PUT/DELETE
 /api/labs/:labId/pt/aa-records. The UI posted to the lab-scoped path but only GET
@@ -1771,30 +1730,30 @@
 route mis-filed records to the user's default lab on multi-lab accounts).</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="G21" s="3" t="inlineStr">
         <is>
           <t>2026-06-13, found during #18 Phase 3 QA;
 scripts/audit-labscoped-write-routes.mjs now guards the class.
 ---</t>
         </is>
       </c>
-      <c r="H18" s="2" t="inlineStr"/>
-    </row>
-    <row r="19" ht="90" customHeight="1">
-      <c r="A19" s="3" t="inlineStr">
+      <c r="H21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22" ht="90" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>C32</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B22" s="2" t="inlineStr">
         <is>
           <t>VeritaComp "Unlock assessment" false-success no-op</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr"/>
-      <c r="D19" s="3" t="inlineStr"/>
-      <c r="E19" s="3" t="inlineStr"/>
-      <c r="F19" s="3" t="inlineStr">
+      <c r="C22" s="2" t="inlineStr"/>
+      <c r="D22" s="2" t="inlineStr"/>
+      <c r="E22" s="2" t="inlineStr"/>
+      <c r="F22" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #755 (commit 4234007) moved the unlock route to
 /api/labs/:labId/competency/assessments/:id/unlock (the path the client calls).
@@ -1805,29 +1764,29 @@
 HTML).</t>
         </is>
       </c>
-      <c r="G19" s="3" t="inlineStr">
+      <c r="G22" s="2" t="inlineStr">
         <is>
           <t>2026-06-13, found by scripts/audit-labscoped-write-routes.mjs.
 ---</t>
         </is>
       </c>
-      <c r="H19" s="3" t="inlineStr"/>
-    </row>
-    <row r="20" ht="90" customHeight="1">
-      <c r="A20" s="2" t="inlineStr">
+      <c r="H22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23" ht="90" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>C33</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>FK-cascade delete 500s + NavBar laptop-width overflow</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr"/>
-      <c r="D20" s="2" t="inlineStr"/>
-      <c r="E20" s="2" t="inlineStr"/>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="C23" s="3" t="inlineStr"/>
+      <c r="D23" s="3" t="inlineStr"/>
+      <c r="E23" s="3" t="inlineStr"/>
+      <c r="F23" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PRs #749/#750 fixed NavBar horizontal overflow at laptop
 widths (collapse to the hamburger below 1560px); prod-verified at 1280-1920 with the
@@ -1838,57 +1797,57 @@
 500 -&gt; 200. scripts/audit-delete-cascades.mjs guards the class.</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr">
+      <c r="G23" s="3" t="inlineStr">
         <is>
           <t>2026-06-13 browser QA of the A7-D4 wave + retro-QC of the 72h PR window.
 ---</t>
         </is>
       </c>
-      <c r="H20" s="2" t="inlineStr"/>
-    </row>
-    <row r="21" ht="90" customHeight="1">
-      <c r="A21" s="3" t="inlineStr">
+      <c r="H23" s="3" t="inlineStr"/>
+    </row>
+    <row r="24" ht="90" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>C1</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>FAQ "over 25 years" -&gt; "over 23 years"</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr"/>
-      <c r="D21" s="3" t="inlineStr"/>
-      <c r="E21" s="3" t="inlineStr"/>
-      <c r="F21" s="3" t="inlineStr">
+      <c r="C24" s="2" t="inlineStr"/>
+      <c r="D24" s="2" t="inlineStr"/>
+      <c r="E24" s="2" t="inlineStr"/>
+      <c r="F24" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: client/src/pages/FAQPage.tsx line 20 reads "over
 23 years" as of 2026-05-01.</t>
         </is>
       </c>
-      <c r="G21" s="3" t="inlineStr">
+      <c r="G24" s="2" t="inlineStr">
         <is>
           <t>session 299e9a73 turn 14, ~2026-04-28.
 ---</t>
         </is>
       </c>
-      <c r="H21" s="3" t="inlineStr"/>
-    </row>
-    <row r="22" ht="90" customHeight="1">
-      <c r="A22" s="2" t="inlineStr">
+      <c r="H24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25" ht="90" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
         <is>
           <t>C5</t>
         </is>
       </c>
-      <c r="B22" s="2" t="inlineStr">
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>David's VeritaQA grey-button bug (seat permissions mode)</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr"/>
-      <c r="D22" s="2" t="inlineStr"/>
-      <c r="E22" s="2" t="inlineStr"/>
-      <c r="F22" s="2" t="inlineStr">
+      <c r="C25" s="3" t="inlineStr"/>
+      <c r="D25" s="3" t="inlineStr"/>
+      <c r="E25" s="3" t="inlineStr"/>
+      <c r="F25" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #10 squash-merged as commit a43fbba on
 2026-05-01 23:19 MST. Railway deploy succeeded; deployed bundle
@@ -1901,7 +1860,7 @@
 against his exact stored shape (14 of 14 expected outcomes matched).</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr">
+      <c r="G25" s="3" t="inlineStr">
         <is>
           <t>2026-05-01 David's report; veritabench + veritastock
 weren't in MODULE_LIST so seat permissions silently defaulted to
@@ -1909,109 +1868,109 @@
 ---</t>
         </is>
       </c>
-      <c r="H22" s="2" t="inlineStr"/>
-    </row>
-    <row r="23" ht="90" customHeight="1">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>C2</t>
-        </is>
-      </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>TeamPage present-tense "TJC surveyor" check</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="inlineStr"/>
-      <c r="D23" s="3" t="inlineStr"/>
-      <c r="E23" s="3" t="inlineStr"/>
-      <c r="F23" s="3" t="inlineStr">
-        <is>
-          <t>Closure evidence: site-wide search confirmed all surveyor language
-is past-tense, consistent with user's 2021-2025 service. User closed
-the item in session 299e9a73 turn 4.</t>
-        </is>
-      </c>
-      <c r="G23" s="3" t="inlineStr">
-        <is>
-          <t>session 299e9a73, ~2026-04-28.
----</t>
-        </is>
-      </c>
-      <c r="H23" s="3" t="inlineStr"/>
-    </row>
-    <row r="24" ht="90" customHeight="1">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>C3</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>My Studies CSV/XLSX export (John as design partner)</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr"/>
-      <c r="D24" s="2" t="inlineStr"/>
-      <c r="E24" s="2" t="inlineStr"/>
-      <c r="F24" s="2" t="inlineStr">
-        <is>
-          <t>Closure evidence: client/src/pages/DashboardPage.tsx line 46 calls
-/api/my-studies/export. server/routes.ts line 1491 implements the
-endpoint. Pulled forward into pre-COLA per user instruction.</t>
-        </is>
-      </c>
-      <c r="G24" s="2" t="inlineStr">
-        <is>
-          <t>session 299e9a73 turn 5, ~2026-04-28.
----</t>
-        </is>
-      </c>
-      <c r="H24" s="2" t="inlineStr"/>
-    </row>
-    <row r="25" ht="90" customHeight="1">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t>C4</t>
-        </is>
-      </c>
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>Rotate GitHub PAT (because old PAT was committed in SESSION_HANDOFF files)</t>
-        </is>
-      </c>
-      <c r="C25" s="3" t="inlineStr"/>
-      <c r="D25" s="3" t="inlineStr"/>
-      <c r="E25" s="3" t="inlineStr"/>
-      <c r="F25" s="3" t="inlineStr">
-        <is>
-          <t>Closure evidence: no ghp_* or github_pat_* patterns in current
-SESSION_HANDOFF.md or SESSION_HANDOFF-2.md as of 2026-05-01.</t>
-        </is>
-      </c>
-      <c r="G25" s="3" t="inlineStr">
-        <is>
-          <t>session 299e9a73, ~2026-04-28.
----</t>
-        </is>
-      </c>
       <c r="H25" s="3" t="inlineStr"/>
     </row>
     <row r="26" ht="90" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>C6</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>VeritaPolicy service-line filtering removed (formerly #4)</t>
+          <t>TeamPage present-tense "TJC surveyor" check</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr"/>
       <c r="D26" s="2" t="inlineStr"/>
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Closure evidence: site-wide search confirmed all surveyor language
+is past-tense, consistent with user's 2021-2025 service. User closed
+the item in session 299e9a73 turn 4.</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>session 299e9a73, ~2026-04-28.
+---</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27" ht="90" customHeight="1">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>C3</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>My Studies CSV/XLSX export (John as design partner)</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr"/>
+      <c r="D27" s="3" t="inlineStr"/>
+      <c r="E27" s="3" t="inlineStr"/>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>Closure evidence: client/src/pages/DashboardPage.tsx line 46 calls
+/api/my-studies/export. server/routes.ts line 1491 implements the
+endpoint. Pulled forward into pre-COLA per user instruction.</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>session 299e9a73 turn 5, ~2026-04-28.
+---</t>
+        </is>
+      </c>
+      <c r="H27" s="3" t="inlineStr"/>
+    </row>
+    <row r="28" ht="90" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Rotate GitHub PAT (because old PAT was committed in SESSION_HANDOFF files)</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr"/>
+      <c r="D28" s="2" t="inlineStr"/>
+      <c r="E28" s="2" t="inlineStr"/>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Closure evidence: no ghp_* or github_pat_* patterns in current
+SESSION_HANDOFF.md or SESSION_HANDOFF-2.md as of 2026-05-01.</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>session 299e9a73, ~2026-04-28.
+---</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29" ht="90" customHeight="1">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>C6</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>VeritaPolicy service-line filtering removed (formerly #4)</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr"/>
+      <c r="D29" s="3" t="inlineStr"/>
+      <c r="E29" s="3" t="inlineStr"/>
+      <c r="F29" s="3" t="inlineStr">
         <is>
           <t>Closure rationale (operator decision 2026-05-10): Keep all
 VeritaPolicy rows. CFR-only references with no accreditor reference
@@ -2020,29 +1979,29 @@
 report misread the design intent.</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr">
+      <c r="G29" s="3" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H26" s="2" t="inlineStr"/>
-    </row>
-    <row r="27" ht="90" customHeight="1">
-      <c r="A27" s="3" t="inlineStr">
+      <c r="H29" s="3" t="inlineStr"/>
+    </row>
+    <row r="30" ht="90" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>C7</t>
         </is>
       </c>
-      <c r="B27" s="3" t="inlineStr">
+      <c r="B30" s="2" t="inlineStr">
         <is>
           <t>CLIA number format validation (formerly #13)</t>
         </is>
       </c>
-      <c r="C27" s="3" t="inlineStr"/>
-      <c r="D27" s="3" t="inlineStr"/>
-      <c r="E27" s="3" t="inlineStr"/>
-      <c r="F27" s="3" t="inlineStr">
+      <c r="C30" s="2" t="inlineStr"/>
+      <c r="D30" s="2" t="inlineStr"/>
+      <c r="E30" s="2" t="inlineStr"/>
+      <c r="F30" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: shared/validateClia.ts defines CLIA_REGEX =
 /^\d{2}D\d{7}$/ (line 24), validateClia() helper with whitespace
@@ -2053,30 +2012,30 @@
 shape exists and behaves as specified.</t>
         </is>
       </c>
-      <c r="G27" s="3" t="inlineStr">
+      <c r="G30" s="2" t="inlineStr">
         <is>
           <t>Agent verification 2026-05-10 via grep + file read.
 Operator confirmed shipped 2026-05-10.
 ---</t>
         </is>
       </c>
-      <c r="H27" s="3" t="inlineStr"/>
-    </row>
-    <row r="28" ht="90" customHeight="1">
-      <c r="A28" s="2" t="inlineStr">
+      <c r="H30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31" ht="90" customHeight="1">
+      <c r="A31" s="3" t="inlineStr">
         <is>
           <t>C8</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="B31" s="3" t="inlineStr">
         <is>
           <t>VeritaMap lab-wide menu toggle (formerly #19)</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr"/>
-      <c r="D28" s="2" t="inlineStr"/>
-      <c r="E28" s="2" t="inlineStr"/>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="C31" s="3" t="inlineStr"/>
+      <c r="D31" s="3" t="inlineStr"/>
+      <c r="E31" s="3" t="inlineStr"/>
+      <c r="F31" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: client/src/pages/VeritaMapLabwidePage.tsx
 exists and implements the labwide read-only union view. Route is
@@ -2086,59 +2045,59 @@
 parking lot plan (read-only union view, per-session toggle) shipped.</t>
         </is>
       </c>
-      <c r="G28" s="2" t="inlineStr">
+      <c r="G31" s="3" t="inlineStr">
         <is>
           <t>Agent verification 2026-05-10 via grep + file read.
 Operator confirmed shipped 2026-05-10.
 ---</t>
         </is>
       </c>
-      <c r="H28" s="2" t="inlineStr"/>
-    </row>
-    <row r="29" ht="90" customHeight="1">
-      <c r="A29" s="3" t="inlineStr">
+      <c r="H31" s="3" t="inlineStr"/>
+    </row>
+    <row r="32" ht="90" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t>C9</t>
         </is>
       </c>
-      <c r="B29" s="3" t="inlineStr">
+      <c r="B32" s="2" t="inlineStr">
         <is>
           <t>Tier-1 smoke test checklist (formerly #6)</t>
         </is>
       </c>
-      <c r="C29" s="3" t="inlineStr"/>
-      <c r="D29" s="3" t="inlineStr"/>
-      <c r="E29" s="3" t="inlineStr"/>
-      <c r="F29" s="3" t="inlineStr">
+      <c r="C32" s="2" t="inlineStr"/>
+      <c r="D32" s="2" t="inlineStr"/>
+      <c r="E32" s="2" t="inlineStr"/>
+      <c r="F32" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: docs/smoke-test-tier1.md documents the Tier-1
 smoke-test process and post-deploy verification steps. Shipped via
 PR #81 as part of the 2026-05-10 wave.</t>
         </is>
       </c>
-      <c r="G29" s="3" t="inlineStr">
+      <c r="G32" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H29" s="3" t="inlineStr"/>
-    </row>
-    <row r="30" ht="90" customHeight="1">
-      <c r="A30" s="2" t="inlineStr">
+      <c r="H32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33" ht="90" customHeight="1">
+      <c r="A33" s="3" t="inlineStr">
         <is>
           <t>C10</t>
         </is>
       </c>
-      <c r="B30" s="2" t="inlineStr">
+      <c r="B33" s="3" t="inlineStr">
         <is>
           <t>Per-module gating (formerly #7)</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr"/>
-      <c r="D30" s="2" t="inlineStr"/>
-      <c r="E30" s="2" t="inlineStr"/>
-      <c r="F30" s="2" t="inlineStr">
+      <c r="C33" s="3" t="inlineStr"/>
+      <c r="D33" s="3" t="inlineStr"/>
+      <c r="E33" s="3" t="inlineStr"/>
+      <c r="F33" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: Client-side useIsReadOnly module keys wired
 on client/src/pages/VeritaPolicyAppPage.tsx and
@@ -2153,29 +2112,29 @@
 PR #76.</t>
         </is>
       </c>
-      <c r="G30" s="2" t="inlineStr">
+      <c r="G33" s="3" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H30" s="2" t="inlineStr"/>
-    </row>
-    <row r="31" ht="90" customHeight="1">
-      <c r="A31" s="3" t="inlineStr">
+      <c r="H33" s="3" t="inlineStr"/>
+    </row>
+    <row r="34" ht="90" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
         <is>
           <t>C11</t>
         </is>
       </c>
-      <c r="B31" s="3" t="inlineStr">
+      <c r="B34" s="2" t="inlineStr">
         <is>
           <t>VeritaStock shipped copy (formerly #8)</t>
         </is>
       </c>
-      <c r="C31" s="3" t="inlineStr"/>
-      <c r="D31" s="3" t="inlineStr"/>
-      <c r="E31" s="3" t="inlineStr"/>
-      <c r="F31" s="3" t="inlineStr">
+      <c r="C34" s="2" t="inlineStr"/>
+      <c r="D34" s="2" t="inlineStr"/>
+      <c r="E34" s="2" t="inlineStr"/>
+      <c r="F34" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: client/src/pages/ArticleInventoryManagementPage.tsx
 line 305 footer reads "platform that includes VeritaStock™" instead
@@ -2183,29 +2142,29 @@
 on /resources/laboratory-inventory-management. Shipped via PR #75.</t>
         </is>
       </c>
-      <c r="G31" s="3" t="inlineStr">
+      <c r="G34" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H31" s="3" t="inlineStr"/>
-    </row>
-    <row r="32" ht="90" customHeight="1">
-      <c r="A32" s="2" t="inlineStr">
+      <c r="H34" s="2" t="inlineStr"/>
+    </row>
+    <row r="35" ht="90" customHeight="1">
+      <c r="A35" s="3" t="inlineStr">
         <is>
           <t>C12</t>
         </is>
       </c>
-      <c r="B32" s="2" t="inlineStr">
+      <c r="B35" s="3" t="inlineStr">
         <is>
           <t>Admin report one-row-per-lab (formerly #14)</t>
         </is>
       </c>
-      <c r="C32" s="2" t="inlineStr"/>
-      <c r="D32" s="2" t="inlineStr"/>
-      <c r="E32" s="2" t="inlineStr"/>
-      <c r="F32" s="2" t="inlineStr">
+      <c r="C35" s="3" t="inlineStr"/>
+      <c r="D35" s="3" t="inlineStr"/>
+      <c r="E35" s="3" t="inlineStr"/>
+      <c r="F35" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: /api/admin/report rewritten in
 server/routes.ts (~line 595) to LEFT JOIN labs on
@@ -2220,56 +2179,56 @@
 prerequisite, not a code bug). Shipped via PR #85.</t>
         </is>
       </c>
-      <c r="G32" s="2" t="inlineStr">
+      <c r="G35" s="3" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H32" s="2" t="inlineStr"/>
-    </row>
-    <row r="33" ht="90" customHeight="1">
-      <c r="A33" s="3" t="inlineStr">
+      <c r="H35" s="3" t="inlineStr"/>
+    </row>
+    <row r="36" ht="90" customHeight="1">
+      <c r="A36" s="2" t="inlineStr">
         <is>
           <t>C14</t>
         </is>
       </c>
-      <c r="B33" s="3" t="inlineStr">
+      <c r="B36" s="2" t="inlineStr">
         <is>
           <t>UI relabel "CLIA TEa" -&gt; "Lab-Set Internal Goal" (formerly #1)</t>
         </is>
       </c>
-      <c r="C33" s="3" t="inlineStr"/>
-      <c r="D33" s="3" t="inlineStr"/>
-      <c r="E33" s="3" t="inlineStr"/>
-      <c r="F33" s="3" t="inlineStr">
+      <c r="C36" s="2" t="inlineStr"/>
+      <c r="D36" s="2" t="inlineStr"/>
+      <c r="E36" s="2" t="inlineStr"/>
+      <c r="F36" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: Shipped across four PRs over 2026-05-10.</t>
         </is>
       </c>
-      <c r="G33" s="3" t="inlineStr">
+      <c r="G36" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H33" s="3" t="inlineStr"/>
-    </row>
-    <row r="34" ht="90" customHeight="1">
-      <c r="A34" s="2" t="inlineStr">
+      <c r="H36" s="2" t="inlineStr"/>
+    </row>
+    <row r="37" ht="90" customHeight="1">
+      <c r="A37" s="3" t="inlineStr">
         <is>
           <t>C13</t>
         </is>
       </c>
-      <c r="B34" s="2" t="inlineStr">
+      <c r="B37" s="3" t="inlineStr">
         <is>
           <t>WSLH PT vendor (formerly #15)</t>
         </is>
       </c>
-      <c r="C34" s="2" t="inlineStr"/>
-      <c r="D34" s="2" t="inlineStr"/>
-      <c r="E34" s="2" t="inlineStr"/>
-      <c r="F34" s="2" t="inlineStr">
+      <c r="C37" s="3" t="inlineStr"/>
+      <c r="D37" s="3" t="inlineStr"/>
+      <c r="E37" s="3" t="inlineStr"/>
+      <c r="F37" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: Shipped 2026-05-10 via PR #79 (merge commit
 eeebc6e; merged after rebase to resolve a server/db.ts collision
@@ -2287,64 +2246,64 @@
 'WSLH' is the post-deploy success signal. Shipped via PR #79.</t>
         </is>
       </c>
-      <c r="G34" s="2" t="inlineStr">
+      <c r="G37" s="3" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H34" s="2" t="inlineStr"/>
-    </row>
-    <row r="35" ht="90" customHeight="1">
-      <c r="A35" s="3" t="inlineStr">
+      <c r="H37" s="3" t="inlineStr"/>
+    </row>
+    <row r="38" ht="90" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
         <is>
           <t>C15</t>
         </is>
       </c>
-      <c r="B35" s="3" t="inlineStr">
+      <c r="B38" s="2" t="inlineStr">
         <is>
           <t>VeritaStock lot tracking + expiration + reorder alerts (formerly #21)</t>
         </is>
       </c>
-      <c r="C35" s="3" t="inlineStr"/>
-      <c r="D35" s="3" t="inlineStr"/>
-      <c r="E35" s="3" t="inlineStr"/>
-      <c r="F35" s="3" t="inlineStr">
+      <c r="C38" s="2" t="inlineStr"/>
+      <c r="D38" s="2" t="inlineStr"/>
+      <c r="E38" s="2" t="inlineStr"/>
+      <c r="F38" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: VeritaStock™ shipped the bench-level inventory
 features the Perplexity competitor analysis identified as a gap:</t>
         </is>
       </c>
-      <c r="G35" s="3" t="inlineStr">
+      <c r="G38" s="2" t="inlineStr">
         <is>
           <t>Originally Perplexity competitor analysis 2026-05-10.
 Audit 2026-05-21 confirmed the feature set ships today.
 ---</t>
         </is>
       </c>
-      <c r="H35" s="3" t="inlineStr"/>
-    </row>
-    <row r="36" ht="90" customHeight="1">
-      <c r="A36" s="2" t="inlineStr">
+      <c r="H38" s="2" t="inlineStr"/>
+    </row>
+    <row r="39" ht="90" customHeight="1">
+      <c r="A39" s="3" t="inlineStr">
         <is>
           <t>C16</t>
         </is>
       </c>
-      <c r="B36" s="2" t="inlineStr">
+      <c r="B39" s="3" t="inlineStr">
         <is>
           <t>PAL studies guided workflow (formerly #23)</t>
         </is>
       </c>
-      <c r="C36" s="2" t="inlineStr"/>
-      <c r="D36" s="2" t="inlineStr"/>
-      <c r="E36" s="2" t="inlineStr"/>
-      <c r="F36" s="2" t="inlineStr">
+      <c r="C39" s="3" t="inlineStr"/>
+      <c r="D39" s="3" t="inlineStr"/>
+      <c r="E39" s="3" t="inlineStr"/>
+      <c r="F39" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: VeritaCheck™ already ships the Precision /
 Accuracy / Linearity (PAL) study set under EP-protocol naming:</t>
         </is>
       </c>
-      <c r="G36" s="2" t="inlineStr">
+      <c r="G39" s="3" t="inlineStr">
         <is>
           <t>Originally Perplexity competitor analysis 2026-05-10.
 Audit 2026-05-21 confirmed the EP studies cover the PAL framing in
@@ -2352,23 +2311,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H36" s="2" t="inlineStr"/>
-    </row>
-    <row r="37" ht="90" customHeight="1">
-      <c r="A37" s="3" t="inlineStr">
+      <c r="H39" s="3" t="inlineStr"/>
+    </row>
+    <row r="40" ht="90" customHeight="1">
+      <c r="A40" s="2" t="inlineStr">
         <is>
           <t>C17</t>
         </is>
       </c>
-      <c r="B37" s="3" t="inlineStr">
+      <c r="B40" s="2" t="inlineStr">
         <is>
           <t>Source-grounded 21/29/45 CFR + 42 CFR 482-485 (formerly #26)</t>
         </is>
       </c>
-      <c r="C37" s="3" t="inlineStr"/>
-      <c r="D37" s="3" t="inlineStr"/>
-      <c r="E37" s="3" t="inlineStr"/>
-      <c r="F37" s="3" t="inlineStr">
+      <c r="C40" s="2" t="inlineStr"/>
+      <c r="D40" s="2" t="inlineStr"/>
+      <c r="E40" s="2" t="inlineStr"/>
+      <c r="F40" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #301 (commit 8c27806, merged 2026-05-21)
 source-grounded the 74 remaining non-493 entries in
@@ -2376,29 +2335,29 @@
 shipped:</t>
         </is>
       </c>
-      <c r="G37" s="3" t="inlineStr">
+      <c r="G40" s="2" t="inlineStr">
         <is>
           <t>PR #301; tasks #18 in the in-session task tracker.
 ---</t>
         </is>
       </c>
-      <c r="H37" s="3" t="inlineStr"/>
-    </row>
-    <row r="38" ht="90" customHeight="1">
-      <c r="A38" s="2" t="inlineStr">
+      <c r="H40" s="2" t="inlineStr"/>
+    </row>
+    <row r="41" ht="90" customHeight="1">
+      <c r="A41" s="3" t="inlineStr">
         <is>
           <t>C18</t>
         </is>
       </c>
-      <c r="B38" s="2" t="inlineStr">
+      <c r="B41" s="3" t="inlineStr">
         <is>
           <t>VeritaPolicy "Non CLIA" chapter rename (formerly #3)</t>
         </is>
       </c>
-      <c r="C38" s="2" t="inlineStr"/>
-      <c r="D38" s="2" t="inlineStr"/>
-      <c r="E38" s="2" t="inlineStr"/>
-      <c r="F38" s="2" t="inlineStr">
+      <c r="C41" s="3" t="inlineStr"/>
+      <c r="D41" s="3" t="inlineStr"/>
+      <c r="E41" s="3" t="inlineStr"/>
+      <c r="F41" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #300 (commit 34d7707, merged 2026-05-21)
 renamed all 44 user-facing chapter labels in
@@ -2409,7 +2368,7 @@
 page.</t>
         </is>
       </c>
-      <c r="G38" s="2" t="inlineStr">
+      <c r="G41" s="3" t="inlineStr">
         <is>
           <t>CAP customer screenshot of the /veritapolicy chapter
 headers, 2026-05-01 evening. PR #300; tasks #17 in the in-session
@@ -2417,23 +2376,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H38" s="2" t="inlineStr"/>
-    </row>
-    <row r="39" ht="90" customHeight="1">
-      <c r="A39" s="3" t="inlineStr">
+      <c r="H41" s="3" t="inlineStr"/>
+    </row>
+    <row r="42" ht="90" customHeight="1">
+      <c r="A42" s="2" t="inlineStr">
         <is>
           <t>C19</t>
         </is>
       </c>
-      <c r="B39" s="3" t="inlineStr">
+      <c r="B42" s="2" t="inlineStr">
         <is>
           <t>VeritaStock department-scope toggle (formerly #31)</t>
         </is>
       </c>
-      <c r="C39" s="3" t="inlineStr"/>
-      <c r="D39" s="3" t="inlineStr"/>
-      <c r="E39" s="3" t="inlineStr"/>
-      <c r="F39" s="3" t="inlineStr">
+      <c r="C42" s="2" t="inlineStr"/>
+      <c r="D42" s="2" t="inlineStr"/>
+      <c r="E42" s="2" t="inlineStr"/>
+      <c r="F42" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #319 (commit d01f5fe, merged 2026-05-22)
 shipped the persistent dept-scope toggle on VeritaStockPage. A new
@@ -2444,7 +2403,7 @@
 workspace without re-filtering.</t>
         </is>
       </c>
-      <c r="G39" s="3" t="inlineStr">
+      <c r="G42" s="2" t="inlineStr">
         <is>
           <t>John, San Carlos lab, 2026-05-21. Same conversation that
 drove the vendor dropdown (PR #304), FILTERED VIEW banner (PR #305),
@@ -2452,23 +2411,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H39" s="3" t="inlineStr"/>
-    </row>
-    <row r="40" ht="90" customHeight="1">
-      <c r="A40" s="2" t="inlineStr">
+      <c r="H42" s="2" t="inlineStr"/>
+    </row>
+    <row r="43" ht="90" customHeight="1">
+      <c r="A43" s="3" t="inlineStr">
         <is>
           <t>C20</t>
         </is>
       </c>
-      <c r="B40" s="2" t="inlineStr">
+      <c r="B43" s="3" t="inlineStr">
         <is>
           <t>Primary-lab seat counting (formerly #12)</t>
         </is>
       </c>
-      <c r="C40" s="2" t="inlineStr"/>
-      <c r="D40" s="2" t="inlineStr"/>
-      <c r="E40" s="2" t="inlineStr"/>
-      <c r="F40" s="2" t="inlineStr">
+      <c r="C43" s="3" t="inlineStr"/>
+      <c r="D43" s="3" t="inlineStr"/>
+      <c r="E43" s="3" t="inlineStr"/>
+      <c r="F43" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: is_primary_lab INTEGER NOT NULL DEFAULT 0
 column was added to the lab_members table at db.ts:1276, with the
@@ -2479,7 +2438,7 @@
 is_primary_lab=1 ordering).</t>
         </is>
       </c>
-      <c r="G40" s="2" t="inlineStr">
+      <c r="G43" s="3" t="inlineStr">
         <is>
           <t>2026-05-07 multi-lab discussion. Build shipped as part
 of the Multi-Lab Tier 2 architecture work (Phase 3.x series, prior
@@ -2488,23 +2447,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H40" s="2" t="inlineStr"/>
-    </row>
-    <row r="41" ht="90" customHeight="1">
-      <c r="A41" s="3" t="inlineStr">
+      <c r="H43" s="3" t="inlineStr"/>
+    </row>
+    <row r="44" ht="90" customHeight="1">
+      <c r="A44" s="2" t="inlineStr">
         <is>
           <t>C21</t>
         </is>
       </c>
-      <c r="B41" s="3" t="inlineStr">
+      <c r="B44" s="2" t="inlineStr">
         <is>
           <t>Multi-lab pricing model — Option A (formerly #11)</t>
         </is>
       </c>
-      <c r="C41" s="3" t="inlineStr"/>
-      <c r="D41" s="3" t="inlineStr"/>
-      <c r="E41" s="3" t="inlineStr"/>
-      <c r="F41" s="3" t="inlineStr">
+      <c r="C44" s="2" t="inlineStr"/>
+      <c r="D44" s="2" t="inlineStr"/>
+      <c r="E44" s="2" t="inlineStr"/>
+      <c r="F44" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #322 (commit 0ccd925, merged 2026-05-22)
 added the customer-facing line to the pricing page that reflects
@@ -2517,7 +2476,7 @@
 Enterprise+ block, reads:</t>
         </is>
       </c>
-      <c r="G41" s="3" t="inlineStr">
+      <c r="G44" s="2" t="inlineStr">
         <is>
           <t>2026-05-07 multi-lab discussion (Lisa Veri's
 canonical-case session). PR #322 (initial build); softening PR
@@ -2526,30 +2485,30 @@
 ---</t>
         </is>
       </c>
-      <c r="H41" s="3" t="inlineStr"/>
-    </row>
-    <row r="42" ht="90" customHeight="1">
-      <c r="A42" s="2" t="inlineStr">
+      <c r="H44" s="2" t="inlineStr"/>
+    </row>
+    <row r="45" ht="90" customHeight="1">
+      <c r="A45" s="3" t="inlineStr">
         <is>
           <t>C22</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
+      <c r="B45" s="3" t="inlineStr">
         <is>
           <t>VeritaOps cost-per-test module (formerly #10)</t>
         </is>
       </c>
-      <c r="C42" s="2" t="inlineStr"/>
-      <c r="D42" s="2" t="inlineStr"/>
-      <c r="E42" s="2" t="inlineStr"/>
-      <c r="F42" s="2" t="inlineStr">
+      <c r="C45" s="3" t="inlineStr"/>
+      <c r="D45" s="3" t="inlineStr"/>
+      <c r="E45" s="3" t="inlineStr"/>
+      <c r="F45" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: v1 of the VeritaOps Cost-Per-Reportable-Test
 (CPRT) module shipped across PR #325 through PR #330 on 2026-05-22.
 The module is feature-complete for the typical lab director workflow.</t>
         </is>
       </c>
-      <c r="G42" s="2" t="inlineStr">
+      <c r="G45" s="3" t="inlineStr">
         <is>
           <t>This thread, 2026-05-07 12:05 PM CDT, user message:
 "Parking lot: build an operations module for cost per test
@@ -2558,262 +2517,262 @@
 ---</t>
         </is>
       </c>
-      <c r="H42" s="2" t="inlineStr"/>
-    </row>
-    <row r="43" ht="90" customHeight="1">
-      <c r="A43" s="3" t="inlineStr">
+      <c r="H45" s="3" t="inlineStr"/>
+    </row>
+    <row r="46" ht="90" customHeight="1">
+      <c r="A46" s="2" t="inlineStr">
         <is>
           <t>C23</t>
         </is>
       </c>
-      <c r="B43" s="3" t="inlineStr">
+      <c r="B46" s="2" t="inlineStr">
         <is>
           <t>CCL lab name visual disambiguation in lab switcher (formerly #34)</t>
         </is>
       </c>
-      <c r="C43" s="3" t="inlineStr"/>
-      <c r="D43" s="3" t="inlineStr">
+      <c r="C46" s="2" t="inlineStr"/>
+      <c r="D46" s="2" t="inlineStr">
         <is>
           <t>XS (under 1 day, actual)</t>
         </is>
       </c>
-      <c r="E43" s="3" t="inlineStr">
+      <c r="E46" s="2" t="inlineStr">
         <is>
           <t>Low — cosmetic; only mattered when Lisa or Michael picked the wrong lab from...</t>
         </is>
       </c>
-      <c r="F43" s="3" t="inlineStr">
+      <c r="F46" s="2" t="inlineStr">
         <is>
           <t>Effort: XS (under 1 day, actual)
 Importance: Low — cosmetic; only mattered when Lisa or Michael picked the wrong lab from the dropdown.</t>
         </is>
       </c>
-      <c r="G43" s="3" t="inlineStr">
+      <c r="G46" s="2" t="inlineStr">
         <is>
           <t>flagged 2026-05-23 immediately after provisioning Lisa's CCL lab; closed 2026-05-24.
 ---</t>
         </is>
       </c>
-      <c r="H43" s="3" t="inlineStr"/>
-    </row>
-    <row r="44" ht="90" customHeight="1">
-      <c r="A44" s="2" t="inlineStr">
+      <c r="H46" s="2" t="inlineStr"/>
+    </row>
+    <row r="47" ht="90" customHeight="1">
+      <c r="A47" s="3" t="inlineStr">
         <is>
           <t>C24</t>
         </is>
       </c>
-      <c r="B44" s="2" t="inlineStr">
+      <c r="B47" s="3" t="inlineStr">
         <is>
           <t>VC Unlimited Y1/Y2 price disclosure UX (formerly #35)</t>
         </is>
       </c>
-      <c r="C44" s="2" t="inlineStr"/>
-      <c r="D44" s="2" t="inlineStr">
+      <c r="C47" s="3" t="inlineStr"/>
+      <c r="D47" s="3" t="inlineStr">
         <is>
           <t>XS (under 1 day, actual)</t>
         </is>
       </c>
-      <c r="E44" s="2" t="inlineStr">
+      <c r="E47" s="3" t="inlineStr">
         <is>
           <t>Low when shipped (proactive, no customer complaint yet) — but high if a procu...</t>
         </is>
       </c>
-      <c r="F44" s="2" t="inlineStr">
+      <c r="F47" s="3" t="inlineStr">
         <is>
           <t>Effort: XS (under 1 day, actual)
 Importance: Low when shipped (proactive, no customer complaint yet) — but high if a procurement reviewer later disputes the $499 renewal as undisclosed.</t>
         </is>
       </c>
-      <c r="G44" s="2" t="inlineStr">
+      <c r="G47" s="3" t="inlineStr">
         <is>
           <t>Pricing rebuild 2026-05-23; closed 2026-05-24 proactively before any customer dispute.
 ---</t>
         </is>
       </c>
-      <c r="H44" s="2" t="inlineStr"/>
-    </row>
-    <row r="45" ht="90" customHeight="1">
-      <c r="A45" s="3" t="inlineStr">
+      <c r="H47" s="3" t="inlineStr"/>
+    </row>
+    <row r="48" ht="90" customHeight="1">
+      <c r="A48" s="2" t="inlineStr">
         <is>
           <t>C25</t>
         </is>
       </c>
-      <c r="B45" s="3" t="inlineStr">
+      <c r="B48" s="2" t="inlineStr">
         <is>
           <t>VeritaQC Phase 1 (Levey-Jennings + Westgard live engine) (formerly #20)</t>
         </is>
       </c>
-      <c r="C45" s="3" t="inlineStr"/>
-      <c r="D45" s="3" t="inlineStr">
+      <c r="C48" s="2" t="inlineStr"/>
+      <c r="D48" s="2" t="inlineStr">
         <is>
           <t>L (about 5 days end-to-end, actual: Phase 0 schema → Phase 1A evaluator → 1B...</t>
         </is>
       </c>
-      <c r="E45" s="3" t="inlineStr">
+      <c r="E48" s="2" t="inlineStr">
         <is>
           <t>High — largest single gap vs myLabCompliance.io per Perplexity competitor ana...</t>
         </is>
       </c>
-      <c r="F45" s="3" t="inlineStr">
+      <c r="F48" s="2" t="inlineStr">
         <is>
           <t>Effort: L (about 5 days end-to-end, actual: Phase 0 schema → Phase 1A evaluator → 1B entry UI → 1C daily review → 1D monthly PDF + attestation)
 Importance: High — largest single gap vs myLabCompliance.io per Perplexity competitor analysis; promotes VeritaAssure from documentation tool to lab operations platform.</t>
         </is>
       </c>
-      <c r="G45" s="3" t="inlineStr">
+      <c r="G48" s="2" t="inlineStr">
         <is>
           <t>Perplexity competitor analysis 2026-05-10. Scoping confirmed via the build_phase1_mockup.py iterations 2026-05-24. Shipped 2026-05-25.
 ---</t>
         </is>
       </c>
-      <c r="H45" s="3" t="inlineStr"/>
-    </row>
-    <row r="46" ht="90" customHeight="1">
-      <c r="A46" s="2" t="inlineStr">
+      <c r="H48" s="2" t="inlineStr"/>
+    </row>
+    <row r="49" ht="90" customHeight="1">
+      <c r="A49" s="3" t="inlineStr">
         <is>
           <t>C26</t>
         </is>
       </c>
-      <c r="B46" s="2" t="inlineStr">
+      <c r="B49" s="3" t="inlineStr">
         <is>
           <t>VeritaLab CMS-116 application support + state licensing registry (formerly #22)</t>
         </is>
       </c>
-      <c r="C46" s="2" t="inlineStr"/>
-      <c r="D46" s="2" t="inlineStr">
+      <c r="C49" s="3" t="inlineStr"/>
+      <c r="D49" s="3" t="inlineStr">
         <is>
           <t>M (1-2 weeks for v1, actual)</t>
         </is>
       </c>
-      <c r="E46" s="2" t="inlineStr">
+      <c r="E49" s="3" t="inlineStr">
         <is>
           <t>Medium — competitor parity (myLabCompliance.io) plus useful at lab startup an...</t>
         </is>
       </c>
-      <c r="F46" s="2" t="inlineStr">
+      <c r="F49" s="3" t="inlineStr">
         <is>
           <t>Effort: M (1-2 weeks for v1, actual)
 Importance: Medium — competitor parity (myLabCompliance.io) plus useful at lab startup and at certificate-type changes.</t>
         </is>
       </c>
-      <c r="G46" s="2" t="inlineStr">
+      <c r="G49" s="3" t="inlineStr">
         <is>
           <t>Perplexity competitor analysis (myLabCompliance.io), 2026-05-10. Reclassified as a VeritaLab extension 2026-05-25. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H46" s="2" t="inlineStr"/>
-    </row>
-    <row r="47" ht="90" customHeight="1">
-      <c r="A47" s="3" t="inlineStr">
+      <c r="H49" s="3" t="inlineStr"/>
+    </row>
+    <row r="50" ht="90" customHeight="1">
+      <c r="A50" s="2" t="inlineStr">
         <is>
           <t>C27</t>
         </is>
       </c>
-      <c r="B47" s="3" t="inlineStr">
+      <c r="B50" s="2" t="inlineStr">
         <is>
           <t>Active vs view-only seat split (formerly #33)</t>
         </is>
       </c>
-      <c r="C47" s="3" t="inlineStr"/>
-      <c r="D47" s="3" t="inlineStr">
+      <c r="C50" s="2" t="inlineStr"/>
+      <c r="D50" s="2" t="inlineStr">
         <is>
           <t>M (~1 week of engineering, actual: shipped in a single multi-PR session)</t>
         </is>
       </c>
-      <c r="E47" s="3" t="inlineStr">
+      <c r="E50" s="2" t="inlineStr">
         <is>
           <t>Medium — closed the gap between /pricing copy and product behavior; gives sal...</t>
         </is>
       </c>
-      <c r="F47" s="3" t="inlineStr">
+      <c r="F50" s="2" t="inlineStr">
         <is>
           <t>Effort: M (~1 week of engineering, actual: shipped in a single multi-PR session)
 Importance: Medium — closed the gap between /pricing copy and product behavior; gives sales a clean answer for "do you charge for our medical director?"</t>
         </is>
       </c>
-      <c r="G47" s="3" t="inlineStr">
+      <c r="G50" s="2" t="inlineStr">
         <is>
           <t>Pricing analysis doc Decision 3 (2026-05-21); MEDIUM scenario revised 2026-05-29 to retire the "unlimited view-only" claim. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H47" s="3" t="inlineStr"/>
-    </row>
-    <row r="48" ht="90" customHeight="1">
-      <c r="A48" s="2" t="inlineStr">
+      <c r="H50" s="2" t="inlineStr"/>
+    </row>
+    <row r="51" ht="90" customHeight="1">
+      <c r="A51" s="3" t="inlineStr">
         <is>
           <t>C28</t>
         </is>
       </c>
-      <c r="B48" s="2" t="inlineStr">
+      <c r="B51" s="3" t="inlineStr">
         <is>
           <t>"Why VeritaCheck" comparative one-pager (formerly #37)</t>
         </is>
       </c>
-      <c r="C48" s="2" t="inlineStr"/>
-      <c r="D48" s="2" t="inlineStr">
+      <c r="C51" s="3" t="inlineStr"/>
+      <c r="D51" s="3" t="inlineStr">
         <is>
           <t>S (one design pass + four claim paragraphs + PDF + matching marketing-site pa...</t>
         </is>
       </c>
-      <c r="E48" s="2" t="inlineStr">
+      <c r="E51" s="3" t="inlineStr">
         <is>
           <t>Medium — closed a positioning gap surfaced by six COLA conference attendees a...</t>
         </is>
       </c>
-      <c r="F48" s="2" t="inlineStr">
+      <c r="F51" s="3" t="inlineStr">
         <is>
           <t>Effort: S (one design pass + four claim paragraphs + PDF + matching marketing-site page, actual)
 Importance: Medium — closed a positioning gap surfaced by six COLA conference attendees attached to a legacy verification tool; converts product-quality advantage into a leave-behind Lisa can hand out.</t>
         </is>
       </c>
-      <c r="G48" s="2" t="inlineStr">
+      <c r="G51" s="3" t="inlineStr">
         <is>
           <t>2026-05-11 / 2026-05-12 conference notes review with Michael. Conference attendees (Whitehead, Odegard, Othman, Molinelli, Kyle, Allred) expressed interest in equivalent / superior product. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H48" s="2" t="inlineStr"/>
-    </row>
-    <row r="49" ht="90" customHeight="1">
-      <c r="A49" s="3" t="inlineStr">
+      <c r="H51" s="3" t="inlineStr"/>
+    </row>
+    <row r="52" ht="90" customHeight="1">
+      <c r="A52" s="2" t="inlineStr">
         <is>
           <t>C29</t>
         </is>
       </c>
-      <c r="B49" s="3" t="inlineStr">
+      <c r="B52" s="2" t="inlineStr">
         <is>
           <t>VeritaPolicy approval workflow — MediaLab functional mirror</t>
         </is>
       </c>
-      <c r="C49" s="3" t="inlineStr"/>
-      <c r="D49" s="3" t="inlineStr">
+      <c r="C52" s="2" t="inlineStr"/>
+      <c r="D52" s="2" t="inlineStr">
         <is>
           <t>XL (one focused session, 12 PRs landed)</t>
         </is>
       </c>
-      <c r="E49" s="3" t="inlineStr">
+      <c r="E52" s="2" t="inlineStr">
         <is>
           <t>High — replaces MediaLab Document Control ($752/$2,250 starting price, scalin...</t>
         </is>
       </c>
-      <c r="F49" s="3" t="inlineStr">
+      <c r="F52" s="2" t="inlineStr">
         <is>
           <t>Effort: XL (one focused session, 12 PRs landed)
 Importance: High — replaces MediaLab Document Control ($752/$2,250 starting price, scaling to $10K-$20K/yr at enterprise per Capterra public data) with an included VeritaPolicy feature; closes a real positioning gap and gives sales a direct comparator line.</t>
         </is>
       </c>
-      <c r="G49" s="3" t="inlineStr">
+      <c r="G52" s="2" t="inlineStr">
         <is>
           <t>Pricing strategy conversation 2026-05-29 (Michael: "I don't like bolt-ons; we should replicate this") → scoped 8 phases → shipped all 12 PRs in single session. Shipped 2026-05-29.
 ---</t>
         </is>
       </c>
-      <c r="H49" s="3" t="inlineStr"/>
+      <c r="H52" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H49"/>
+  <autoFilter ref="A1:H52"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
TASK: mark parking-lot #47 shipped (found stale during #36 verification) PLAN:   1. #47 hide-N/A master-list toggle was already merged as PR #1364; correct the stale OPEN entry   2. regenerate PARKING_LOT.xlsx to stay in sync Self-check:   - docs-only, Gate 3 N/A; verified #47 present in origin/main (d45dcc5a) before marking shipped; keys at line start
</commit_message>
<xml_diff>
--- a/PARKING_LOT.xlsx
+++ b/PARKING_LOT.xlsx
@@ -1050,11 +1050,7 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Open. Not started. Needs a one-line scope confirmation (which master list).
----
-_(item #50 closed 2026-09-28; shipped PR #1356, prod-verified, see C49 below)_
----
-_(item #51 closed 2026-09-28;...</t>
+          <t>SHIPPED (PR #1364, in origin/main; predates this session, entry was stale). Built as the VeritaDC (VeritaPolicy) Master List "Show only applicable" toggle in client/src/pages/VeritaPolicyAppPage.ts...</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">

</xml_diff>

<commit_message>
TASK: VeritaResponse internal NCE (#36) - lab-found event + MD/admin sign-off + PDF
PLAN:
  1. server: internal_nce source type + event fields + MD/owner-admin gated sign-off endpoint
  2. client: Internal event (NCE) create flow + list badge + gated sign-off button
  3. PDF: internal-NCE write-up renderer (signature block on page 1) + env-gated Playwright spec

Self-check:
  - inspection/PT paths untouched; tsc clean; pre-commit audit 0 errors; CI green 9/9
  - accreditor stays NOT NULL (internal_nce stores Other); sign-off 403s non-MD/non-owner-admin
  - Gate 3 browser verify runs on prod post-deploy per the deploy-then-verify path
</commit_message>
<xml_diff>
--- a/PARKING_LOT.xlsx
+++ b/PARKING_LOT.xlsx
@@ -1050,11 +1050,7 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Open. Not started. Needs a one-line scope confirmation (which master list).
----
-_(item #50 closed 2026-09-28; shipped PR #1356, prod-verified, see C49 below)_
----
-_(item #51 closed 2026-09-28;...</t>
+          <t>SHIPPED (PR #1364, in origin/main; predates this session, entry was stale). Built as the VeritaDC (VeritaPolicy) Master List "Show only applicable" toggle in client/src/pages/VeritaPolicyAppPage.ts...</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">

</xml_diff>

<commit_message>
TASK: move parking-lot #36 to CLOSED (C52) - VeritaResponse internal NCE shipped PLAN:   1. replace the OPEN #36 entry with a closed stub; add C52 to CLOSED with closure evidence (PR #1368, 29cc6e23, deployed, Gate-3 passed)   2. regenerate PARKING_LOT.xlsx (OPEN 13->12, CLOSED 51->52) Self-check:   - docs-only, Gate 3 N/A; #36 verified shipped this session; next C-number confirmed (max was C51); keys at line start
</commit_message>
<xml_diff>
--- a/PARKING_LOT.xlsx
+++ b/PARKING_LOT.xlsx
@@ -12,8 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RETIRED" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$52</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$53</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RETIRED'!$A$1:$H$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -822,6 +822,10 @@
 _(item #33 closed 2026-05-28; see C27 below)_
 ---
 _(items #34 and #35 closed 2026-05-24; see C23 and C24 below)_
+---
+_(item #36 closed 2026-09-29; shipped PR #1368, prod-verified, see C52 below)_
+---
+_(item #37 closed 2026-05-28; see C28 below)_
 ---</t>
         </is>
       </c>
@@ -829,40 +833,42 @@
     <row r="8" ht="90" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>38</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>New module: laboratory non-conforming event documentation</t>
+          <t>Screen-capture video: VeritaCheck method comparison in 60 seconds</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Scoped, not started (updated 2026-09-28). Now lands in VeritaResponse per Michael's direction above; the earlier "new standalone module" framing is superseded. Do not start building until Michael g...</t>
+          <t>Open. Re-parked 2026-05-27 (originally PR #117, abandoned with merge conflicts then closed-and-re-authored at current numbering). Pending operator decision on whether to record this themselves or p...</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>L (initial estimate, pending Michael's scope walkthrough — likely new DB tabl...</t>
+          <t>S for agent prep (storyboard / pre-fill / captions / checklist); ~1 hour of o...</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>High — every accredited laboratory (TJC, CAP, COLA, AABB) has to document non...</t>
+          <t>Medium — operator selected this as the highest-impact positioning artifact du...</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Build a module to document laboratory non-conforming events (NCEs). Surfaces a lab needs to capture include specimen rejection, temperature excursions, reagent issues, equipment failures, result-reporting errors, transcription errors, lost specimens, contamination events, and similar quality incidents. Full scope, target accreditor mapping, terminology preference (NCE / NCR / event / incident / occurrence), and how it should relate to the existing VeritaQC corrective-action engine and VeritaResponse deficiency tracker are TBD pending Michael's scope walkthrough.</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr"/>
+          <t>30-60 second screen recording demonstrating the "experienced lab tech figures it out in seconds" claim. From blank method-comparison study to completed PDF, no voiceover, no narration, visible cursor motion. Embed autoplay-muted on the marketing site, include in conference follow-up emails.</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-12 conversation. Michael selected the screen-cap video as the highest-impact positioning artifact, then asked the agent to record it. Agent does not have screen-recording capability; option parked rather than fudged.</t>
+        </is>
+      </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Post-COLA. No customer urgency yet, but high strategic value once defined — closes a real gap every lab has and that no other Verita module currently serves.
----
-_(item #37 closed 2026-05-28; see C28 below)_
+          <t>Post-COLA, conference-driven.
 ---</t>
         </is>
       </c>
@@ -870,73 +876,30 @@
     <row r="9" ht="90" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>39</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Screen-capture video: VeritaCheck method comparison in 60 seconds</t>
+          <t>MediaLab parity hardening (VeritaPolicy approval workflow depth)</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Open. Re-parked 2026-05-27 (originally PR #117, abandoned with merge conflicts then closed-and-re-authored at current numbering). Pending operator decision on whether to record this themselves or p...</t>
+          <t>Small-item sequence COMPLETE (items 1-5 all shipped; verified against the codebase 2026-09-29, print view PR #1367). Remaining depth items (SSO/AD, delegation, in-browser editing, per-department ro...</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>S for agent prep (storyboard / pre-fill / captions / checklist); ~1 hour of o...</t>
+          <t>L (1-2 weeks for the high-value items; each independent feature is M)</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Medium — operator selected this as the highest-impact positioning artifact du...</t>
+          <t>Medium-High — the C29 build shipped the surface MediaLab markets but depth is...</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>30-60 second screen recording demonstrating the "experienced lab tech figures it out in seconds" claim. From blank method-comparison study to completed PDF, no voiceover, no narration, visible cursor motion. Embed autoplay-muted on the marketing site, include in conference follow-up emails.</t>
-        </is>
-      </c>
-      <c r="G9" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-12 conversation. Michael selected the screen-cap video as the highest-impact positioning artifact, then asked the agent to record it. Agent does not have screen-recording capability; option parked rather than fudged.</t>
-        </is>
-      </c>
-      <c r="H9" s="3" t="inlineStr">
-        <is>
-          <t>Post-COLA, conference-driven.
----</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="90" customHeight="1">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>39</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>MediaLab parity hardening (VeritaPolicy approval workflow depth)</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Small-item sequence COMPLETE (items 1-5 all shipped; verified against the codebase 2026-09-29, print view PR #1367). Remaining depth items (SSO/AD, delegation, in-browser editing, per-department ro...</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>L (1-2 weeks for the high-value items; each independent feature is M)</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>Medium-High — the C29 build shipped the surface MediaLab markets but depth is...</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>The VeritaPolicy approval workflow build (C29, 2026-05-29) hit roughly 60-70% MediaLab feature surface. The following gaps remain when comparing against an enterprise MediaLab Document Control deployment:
 - Quizzes on attestations. Schema columns quiz_score and quiz_total_questions exist on policy_attestations but the quiz authoring + presentation UI was scoped out of Phase 4. MediaLab labs use 5-10 multiple-choice questions per policy to confirm comprehension, not just attestation. Adds compliance defensibility.
@@ -946,54 +909,93 @@
 - In-browser DOCX editing. MediaLab has a structured editor that creates a Table of Contents from headings. We treat documents as...</t>
         </is>
       </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-29 QA pass after C29 shipped (qa-policy-build.js + qa-policy-ui.js: 54/54 happy path verified). Honest depth assessment surfaced by Michael's "how confident are you" question — see C29 entry for full QA receipts.</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>Post-COLA. Defensive against MediaLab in head-to-head sales calls.
+---</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="90" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>VeritaQC Import Phase A: human-in-the-loop Gate 3 click-through (deferred)</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Open, awaiting Michael's 5-minute click test. Will move task #77 to completed only after he reports the user-visible result.
+---</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>XS (~5 minutes of Michael's time on a live URL).</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Low. Backend contract is fully verified via 35/35 passing offline contract ch...</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Effort: XS (~5 minutes of Michael's time on a live URL).
+Importance: Low. Backend contract is fully verified via 35/35 passing offline contract checks (scripts/verify-veritaqc-import.js) plus three live-API smoke checks against prod (candidates, preview, mappings PUT/GET) on Riverside Regional with seed lot SEED-1780436709094 (18 Glucose results). The browser-driven click was not run because Claude-in-Chrome's renderer froze repeatedly on the Radix Select inside VeritaCheckPage, not on Phase A code itself. Risk of a UX bug surviving to a customer is small but not zero.</t>
+        </is>
+      </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29 QA pass after C29 shipped (qa-policy-build.js + qa-policy-ui.js: 54/54 happy path verified). Honest depth assessment surfaced by Michael's "how confident are you" question — see C29 entry for full QA receipts.</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>Post-COLA. Defensive against MediaLab in head-to-head sales calls.
----</t>
-        </is>
-      </c>
+          <t>task #77 stalled at Gate 3 step 8 on 2026-06-02. PR #500 squash-merged at commit 17a91ff, prod /api/health confirmed ACTIVE on that commit at 20:43 UTC.</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr"/>
     </row>
     <row r="11" ht="90" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>42</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>VeritaQC Import Phase A: human-in-the-loop Gate 3 click-through (deferred)</t>
+          <t>Outbound demo-invite messaging campaign to 1st-degree LinkedIn contacts</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Open, awaiting Michael's 5-minute click test. Will move task #77 to completed only after he reports the user-visible result.
+          <t>Parked. Plan documented. Implementation deferred until trigger conditions met.
 ---</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>XS (~5 minutes of Michael's time on a live URL).</t>
+          <t>L (1 week prep + 4-6 weeks of staged sends)</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>Low. Backend contract is fully verified via 35/35 passing offline contract ch...</t>
+          <t>High. Converts existing warm network (~2,500 1st-degree contacts and growing...</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Effort: XS (~5 minutes of Michael's time on a live URL).
-Importance: Low. Backend contract is fully verified via 35/35 passing offline contract checks (scripts/verify-veritaqc-import.js) plus three live-API smoke checks against prod (candidates, preview, mappings PUT/GET) on Riverside Regional with seed lot SEED-1780436709094 (18 Glucose results). The browser-driven click was not run because Claude-in-Chrome's renderer froze repeatedly on the Radix Select inside VeritaCheckPage, not on Phase A code itself. Risk of a UX bug surviving to a customer is small but not zero.</t>
+          <t>A staged outbound DM campaign walking Michael's 1st-degree LinkedIn contacts through tier-segmented demo invitations for VeritaAssure. Goal: convert warmest contacts into demo conversations first, then chain into trials and paid subscriptions. Separate pipeline from COLA cohort follow-up and from content-driven inbound; all three feed the same demo funnel but originate from different warmth sources.</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>task #77 stalled at Gate 3 step 8 on 2026-06-02. PR #500 squash-merged at commit 17a91ff, prod /api/health confirmed ACTIVE on that commit at 20:43 UTC.</t>
+          <t>2026-06-04 session, after weekly LinkedIn invite batch completion (80 sent, cap hit at #84 Victoria Allen).</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr"/>
@@ -1001,38 +1003,38 @@
     <row r="12" ht="90" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>47</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Outbound demo-invite messaging campaign to 1st-degree LinkedIn contacts</t>
+          <t>Hide sections a lab does not use from a master list, to reduce clutter (prospect-requested)</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Parked. Plan documented. Implementation deferred until trigger conditions met.
----</t>
+          <t>SHIPPED (PR #1364, in origin/main; predates this session, entry was stale). Built as the VeritaDC (VeritaPolicy) Master List "Show only applicable" toggle in client/src/pages/VeritaPolicyAppPage.ts...</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>L (1 week prep + 4-6 weeks of staged sends)</t>
+          <t>S-M (a few days to ~2 weeks depending on scope) — a lab-level visibility togg...</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>High. Converts existing warm network (~2,500 1st-degree contacts and growing...</t>
+          <t>Medium-High — came straight from a live prospect today as an onboarding-frict...</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>A staged outbound DM campaign walking Michael's 1st-degree LinkedIn contacts through tier-segmented demo invitations for VeritaAssure. Goal: convert warmest contacts into demo conversations first, then chain into trials and paid subscriptions. Separate pipeline from COLA cohort follow-up and from content-driven inbound; all three feed the same demo funnel but originate from different warmth sources.</t>
+          <t>Effort: S-M (a few days to ~2 weeks depending on scope) — a lab-level visibility toggle that hides not-applicable or unused sections from a master-list view. Smaller if it is a "hide N/A" filter on the existing VeritaDC master list, larger if it also spans VeritaScan domains.
+Importance: Medium-High — came straight from a live prospect today as an onboarding-friction point; a lab that does not run a service line should not have to wade past its requirements.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04 session, after weekly LinkedIn invite batch completion (80 sent, cap hit at #84 Victoria Allen).</t>
+          <t>2026-09-23 session, Michael relaying a prospect ask from a demo today.</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr"/>
@@ -1040,80 +1042,41 @@
     <row r="13" ht="90" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>53</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Hide sections a lab does not use from a master list, to reduce clutter (prospect-requested)</t>
+          <t>VeritaCEU: curated free-continuing-education provider list (seed / reference)</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>SHIPPED (PR #1364, in origin/main; predates this session, entry was stale). Built as the VeritaDC (VeritaPolicy) Master List "Show only applicable" toggle in client/src/pages/VeritaPolicyAppPage.ts...</t>
+          <t>Open, reference captured. Not started.</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>S-M (a few days to ~2 weeks depending on scope) — a lab-level visibility togg...</t>
+          <t>S (1-2 days to seed a curated provider list and surface it in VeritaCEU; XS t...</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>Medium-High — came straight from a live prospect today as an onboarding-frict...</t>
+          <t>Low-Medium — quality-of-life for VeritaCEU users (find free CE fast); not blo...</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>Effort: S-M (a few days to ~2 weeks depending on scope) — a lab-level visibility toggle that hides not-applicable or unused sections from a master-list view. Smaller if it is a "hide N/A" filter on the existing VeritaDC master list, larger if it also spans VeritaScan domains.
-Importance: Medium-High — came straight from a live prospect today as an onboarding-friction point; a lab that does not run a service line should not have to wade past its requirements.</t>
-        </is>
-      </c>
-      <c r="G13" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-23 session, Michael relaying a prospect ask from a demo today.</t>
-        </is>
-      </c>
-      <c r="H13" s="3" t="inlineStr"/>
-    </row>
-    <row r="14" ht="90" customHeight="1">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>53</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>VeritaCEU: curated free-continuing-education provider list (seed / reference)</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>Open, reference captured. Not started.</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>S (1-2 days to seed a curated provider list and surface it in VeritaCEU; XS t...</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>Low-Medium — quality-of-life for VeritaCEU users (find free CE fast); not blo...</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>Effort: S (1-2 days to seed a curated provider list and surface it in VeritaCEU; XS to just store the reference)
 Importance: Low-Medium — quality-of-life for VeritaCEU users (find free CE fast); not blocking any sale.</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="G13" s="3" t="inlineStr">
         <is>
           <t>Jennifer Small (jennifer.small@lifepointhealth.net) email 2026-09-25, forwarded by Michael 2026-09-28 for the future CEU module.</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="H13" s="3" t="inlineStr">
         <is>
           <t>Post-COLA. No customer urgency.
 ---</t>
@@ -1121,7 +1084,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H14"/>
+  <autoFilter ref="A1:H13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1132,7 +1095,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H52"/>
+  <dimension ref="A1:H53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1190,24 +1153,24 @@
     <row r="2" ht="90" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>C49</t>
+          <t>C52</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Competency "assessed this cycle" cadence-aware window (was #50)</t>
+          <t>VeritaResponse internal NCE / non-conforming event (was #36)</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr"/>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>was S-M / Importance: Medium</t>
+          <t>was L (shipped as MEDIUM) / Importance: High</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Effort: was S-M / Importance: Medium</t>
+          <t>Effort: was L (shipped as MEDIUM) / Importance: High</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
@@ -1216,12 +1179,12 @@
     <row r="3" ht="90" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>C50</t>
+          <t>C49</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>VeritaTrack task owner + owner-only reminder routing (was #51)</t>
+          <t>Competency "assessed this cycle" cadence-aware window (was #50)</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr"/>
@@ -1242,24 +1205,24 @@
     <row r="4" ht="90" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>C51</t>
+          <t>C50</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Designate Medical Director by picking a lab member (was #52, core)</t>
+          <t>VeritaTrack task owner + owner-only reminder routing (was #51)</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr"/>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>was S-M / Importance: Medium-High</t>
+          <t>was S-M / Importance: Medium</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Effort: was S-M / Importance: Medium-High</t>
+          <t>Effort: was S-M / Importance: Medium</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr"/>
@@ -1268,24 +1231,24 @@
     <row r="5" ht="90" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>C47</t>
+          <t>C51</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Unregulated-analyte / Alternative Assessment (AAA) coverage (was #18)</t>
+          <t>Designate Medical Director by picking a lab member (was #52, core)</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr"/>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>was S (Phase 3) / Importance: Medium</t>
+          <t>was S-M / Importance: Medium-High</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Effort: was S (Phase 3) / Importance: Medium</t>
+          <t>Effort: was S-M / Importance: Medium-High</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr"/>
@@ -1294,24 +1257,24 @@
     <row r="6" ht="90" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>C48</t>
+          <t>C47</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>VeritaResponse post-survey deficiency module (was #17)</t>
+          <t>Unregulated-analyte / Alternative Assessment (AAA) coverage (was #18)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr"/>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>was XL / Importance: High</t>
+          <t>was S (Phase 3) / Importance: Medium</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Effort: was XL / Importance: High</t>
+          <t>Effort: was S (Phase 3) / Importance: Medium</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
@@ -1320,39 +1283,38 @@
     <row r="7" ht="90" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>C45</t>
+          <t>C48</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Unify coverage/competency recurrence helper (was #49) - closed as non-issue</t>
+          <t>VeritaResponse post-survey deficiency module (was #17)</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr"/>
-      <c r="D7" s="3" t="inlineStr"/>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>was XL / Importance: High</t>
+        </is>
+      </c>
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: Investigated 2026-09-24 before building. The coverage recurrence math (+6-month interval, signed-resets-to-missing, nextDueOn/overdue, isFailVerdict) is ALREADY single-source in server/veritacheckCoverage.ts (computeCoverageFrom). server/coverageReport.ts and the routes.ts coverage export do not recompute it; they consume the computed nextDueOn/overdue/status fields and apply small surface-specific presentation labels (deliberately different vocabularies per surface, so they should not be merged). The only truly identical duplicate is a one-line date formatter. The competency "owed" derivation is NOT the same cadence: competency follows the CLIA milestone schedule (initial / semiannual year 1 / annual, 42 CFR 493.1451(b)(8) and 493.1235), which is a different regulatory interval from the coverage 6-month rule (493.1281 / 493.1255) and must stay separate. No worthwhile extraction; merging the two cadences would be wrong. Closed 2026-09-24. (The year-1 competency-window refinement remains tracked separately as #50.)</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-24 session, "keep working" pass; scoped read-only, found no real duplication.
----</t>
-        </is>
-      </c>
+          <t>Effort: was XL / Importance: High</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr"/>
       <c r="H7" s="3" t="inlineStr"/>
     </row>
     <row r="8" ht="90" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>C46</t>
+          <t>C45</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Verified-users product-update send path (wrong-list incident fix)</t>
+          <t>Unify coverage/competency recurrence helper (was #49) - closed as non-issue</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr"/>
@@ -1360,12 +1322,12 @@
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: Shipped PR #1324 (merged 4e05506a, deploy ACTIVE). New POST /api/admin/users/send targets registered VeritaAssure account holders (the users table), never the Lab Director's Briefing subscriber list. Separate explicitly-named endpoint (not a flag with a dangerous default), account-holder email framing, excludes suppressed emails and RFC-reserved test domains, CC owner, dryRun + testTo previews. Public unsubscribe now upserts a suppression row so opt-outs are honored across both audiences. Live dryRun: 49 verified-user recipients vs 673 on the Briefing list. Receipts: scripts/verify-product-update-send.mts 24/24, tsc clean, rendered sample inspected. Fixes the fallout from the 2026-09-23/24 wrong-list send (a product update went to the 675-person Briefing list). Nothing sends without Michael's explicit "send it."</t>
+          <t>Closure evidence: Investigated 2026-09-24 before building. The coverage recurrence math (+6-month interval, signed-resets-to-missing, nextDueOn/overdue, isFailVerdict) is ALREADY single-source in server/veritacheckCoverage.ts (computeCoverageFrom). server/coverageReport.ts and the routes.ts coverage export do not recompute it; they consume the computed nextDueOn/overdue/status fields and apply small surface-specific presentation labels (deliberately different vocabularies per surface, so they should not be merged). The only truly identical duplicate is a one-line date formatter. The competency "owed" derivation is NOT the same cadence: competency follows the CLIA milestone schedule (initial / semiannual year 1 / annual, 42 CFR 493.1451(b)(8) and 493.1235), which is a different regulatory interval from the coverage 6-month rule (493.1281 / 493.1255) and must stay separate. No worthwhile extraction; merging the two cadences would be wrong. Closed 2026-09-24. (The year-1 competency-window refinement remains tracked separately as #50.)</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 session; Michael selected this as the next build after the #41 close.
+          <t>2026-09-24 session, "keep working" pass; scoped read-only, found no real duplication.
 ---</t>
         </is>
       </c>
@@ -1374,12 +1336,12 @@
     <row r="9" ht="90" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>C44</t>
+          <t>C46</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Verify-script convention backfill (was #41) + audit matcher fix</t>
+          <t>Verified-users product-update send path (wrong-list incident fix)</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr"/>
@@ -1387,12 +1349,12 @@
       <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: #41 was fully backfilled on 2026-06-13 (all 8 high-stakes scripts landed; see C30); it had only been mis-filed in OPEN. A 2026-09-24 re-audit initially reported 4 of 5 recent math/logic commits as missing a verify script, which was a FALSE POSITIVE: scripts/audit_verify_script_coverage.py matched only scripts/verify-*.js / .cjs, so it ignored the .mjs / .mts / .ts verify scripts the repo now ships (e.g. verify-ptcoag-multi.mts, verify-tea-criterion-format.mjs). Fixed the matcher to accept .js/.cjs/.mjs/.ts/.mts; re-run shows 5 of 5 covered, 0 debt. The convention is being followed. Closed 2026-09-24.</t>
+          <t>Closure evidence: Shipped PR #1324 (merged 4e05506a, deploy ACTIVE). New POST /api/admin/users/send targets registered VeritaAssure account holders (the users table), never the Lab Director's Briefing subscriber list. Separate explicitly-named endpoint (not a flag with a dangerous default), account-holder email framing, excludes suppressed emails and RFC-reserved test domains, CC owner, dryRun + testTo previews. Public unsubscribe now upserts a suppression row so opt-outs are honored across both audiences. Live dryRun: 49 verified-user recipients vs 673 on the Briefing list. Receipts: scripts/verify-product-update-send.mts 24/24, tsc clean, rendered sample inspected. Fixes the fallout from the 2026-09-23/24 wrong-list send (a product update went to the 675-person Briefing list). Nothing sends without Michael's explicit "send it."</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>2026-09-24 session, "keep working" pass; audit tooling bug found + fixed.
+          <t>2026-09-24 session; Michael selected this as the next build after the #41 close.
 ---</t>
         </is>
       </c>
@@ -1401,12 +1363,12 @@
     <row r="10" ht="90" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>C43</t>
+          <t>C44</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>VeritaStaff instrument-centric (dual) assignment view</t>
+          <t>Verify-script convention backfill (was #41) + audit matcher fix</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr"/>
@@ -1414,12 +1376,12 @@
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1320. GET/PUT /staff/instruments/:id/employees (transpose of the per-employee endpoints); an "Assign by Instrument" dialog lets a director pick a test system or manual test and check off who runs it. Same staff_employee_instruments join, with the 42 CFR 493.1235(a) duty-change event emitted on newly-added pairs so both orientations trigger the same reassessment. GET verified live on SCAHC lab 2. Closed 2026-09-24.</t>
+          <t>Closure evidence: #41 was fully backfilled on 2026-06-13 (all 8 high-stakes scripts landed; see C30); it had only been mis-filed in OPEN. A 2026-09-24 re-audit initially reported 4 of 5 recent math/logic commits as missing a verify script, which was a FALSE POSITIVE: scripts/audit_verify_script_coverage.py matched only scripts/verify-*.js / .cjs, so it ignored the .mjs / .mts / .ts verify scripts the repo now ships (e.g. verify-ptcoag-multi.mts, verify-tea-criterion-format.mjs). Fixed the matcher to accept .js/.cjs/.mjs/.ts/.mts; re-run shows 5 of 5 covered, 0 debt. The convention is being followed. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 session, Michael ("in staff we should also give the dual view when assigning coverage to test systems or manual tests").
+          <t>2026-09-24 session, "keep working" pass; audit tooling bug found + fixed.
 ---</t>
         </is>
       </c>
@@ -1428,12 +1390,12 @@
     <row r="11" ht="90" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>C42</t>
+          <t>C43</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>VeritaComp coverage map (required-vs-assessed matrix, dual view)</t>
+          <t>VeritaStaff instrument-centric (dual) assignment view</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr"/>
@@ -1441,12 +1403,12 @@
       <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1319 (+ status layer PR #1316). /competency/owed returns per-item assessed (locked passing assessment this cycle on a covering method group) + per-employee CLIA status; CompetencyCoverageMap renders a By-employee / By-instrument matrix (Assessed / Owed / Overdue / Gap). Verified live on SCAHC lab 2 (owed 116, assessed 2, gaps 0). Completes #48 as the VeritaCheck-parity coverage map. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1320. GET/PUT /staff/instruments/:id/employees (transpose of the per-employee endpoints); an "Assign by Instrument" dialog lets a director pick a test system or manual test and check off who runs it. Same staff_employee_instruments join, with the 42 CFR 493.1235(a) duty-change event emitted on newly-added pairs so both orientations trigger the same reassessment. GET verified live on SCAHC lab 2. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>2026-09-24 session, Michael ("are we building the competencies to have a coverage map, same as veritacheck?" then "build it").
+          <t>2026-09-24 session, Michael ("in staff we should also give the dual view when assigning coverage to test systems or manual tests").
 ---</t>
         </is>
       </c>
@@ -1455,12 +1417,12 @@
     <row r="12" ht="90" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>C41</t>
+          <t>C42</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>VeritaCheck coverage recurrence (method comparison + cal-ver/linearity + reports)</t>
+          <t>VeritaComp coverage map (required-vs-assessed matrix, dual view)</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr"/>
@@ -1468,12 +1430,12 @@
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: PRs #1317 (method comparison), #1318 (cal-ver/linearity), #1321 (report Next-due columns). Periodic verification (correlation/method comparison 42 CFR 493.1281; cal-ver/linearity 42 CFR 493.1255; both 6-month) now recurs: a signed study banks the cycle and rolls to next-due = signed + 6 months instead of reading "done" forever. Status Missing/Failed/Completed-unsigned + a "Next due on" column on-screen and in both coverage exports; also credits the previously-ignored "correlation" study type. Root cause: computeCoverageFrom marked requirements done on mere existence, no date logic. Verified live on SCAHC lab 2 (101 correlations + 11 cal-ver rows now carry a next-due). Engine-level, all facilities. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1319 (+ status layer PR #1316). /competency/owed returns per-item assessed (locked passing assessment this cycle on a covering method group) + per-employee CLIA status; CompetencyCoverageMap renders a By-employee / By-instrument matrix (Assessed / Owed / Overdue / Gap). Verified live on SCAHC lab 2 (owed 116, assessed 2, gaps 0). Completes #48 as the VeritaCheck-parity coverage map. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 session, Michael ("Look at San Carlos... they finished their last set of correlations (all 103) but their menu never reset").
+          <t>2026-09-24 session, Michael ("are we building the competencies to have a coverage map, same as veritacheck?" then "build it").
 ---</t>
         </is>
       </c>
@@ -1482,12 +1444,12 @@
     <row r="13" ht="90" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>C40</t>
+          <t>C41</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>VeritaComp Competencies Owed derived from VeritaStaff, with gap detection (was #48)</t>
+          <t>VeritaCheck coverage recurrence (method comparison + cal-ver/linearity + reports)</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr"/>
@@ -1495,12 +1457,12 @@
       <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1314 (squash 2bcb0db9). GET /api/labs/:labId/competency/owed derives each VeritaStaff testing employee's owed competencies from their assigned instruments (staff_employee_instruments -&gt; veritamap_instruments + tests), on the CLIA timeline, and flags instruments not covered by any competency program as gaps. CompetenciesOwedSection renders it on the VeritaComp landing page. Reuses the shipped bridge + suggested-method-groups match rules; no new tables. Verified live on prod with real assignment data: 2 instruments assigned to a demo staffer produced owed=2, gaps=2 (HIGH, Technical Supervisor), then reverted cleanly. Closed 2026-09-24.</t>
+          <t>Closure evidence: PRs #1317 (method comparison), #1318 (cal-ver/linearity), #1321 (report Next-due columns). Periodic verification (correlation/method comparison 42 CFR 493.1281; cal-ver/linearity 42 CFR 493.1255; both 6-month) now recurs: a signed study banks the cycle and rolls to next-due = signed + 6 months instead of reading "done" forever. Status Missing/Failed/Completed-unsigned + a "Next due on" column on-screen and in both coverage exports; also credits the previously-ignored "correlation" study type. Root cause: computeCoverageFrom marked requirements done on mere existence, no date logic. Verified live on SCAHC lab 2 (101 correlations + 11 cal-ver rows now carry a next-due). Engine-level, all facilities. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>2026-09-23/24 session, Michael ("veritacomp bases what competencies they owe (currently untrue, but needs to be true)"). Option 1 (unify roster on VeritaStaff, match instruments by id).
+          <t>2026-09-24 session, Michael ("Look at San Carlos... they finished their last set of correlations (all 103) but their menu never reset").
 ---</t>
         </is>
       </c>
@@ -1509,12 +1471,12 @@
     <row r="14" ht="90" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>C39</t>
+          <t>C40</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>VeritaScan line items can attach or link evidence (was #46)</t>
+          <t>VeritaComp Competencies Owed derived from VeritaStaff, with gap detection (was #48)</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr"/>
@@ -1522,12 +1484,12 @@
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1312 (squash a1dda93d). VeritaScan scan checklist items now show linked evidence as chips (open link, remove) plus a writer "Link evidence" affordance whose picker links an existing VeritaDC/Library document; a shortcut deep-links to the Library for new (governed) documents. Reuses the already-shipped lab_documents + document_checklist_links + coverage endpoints (URL-pointer only, no file storage, no new tables). Browser-verified live on prod (scan 23): the affordance renders and the picker opens. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1314 (squash 2bcb0db9). GET /api/labs/:labId/competency/owed derives each VeritaStaff testing employee's owed competencies from their assigned instruments (staff_employee_instruments -&gt; veritamap_instruments + tests), on the CLIA timeline, and flags instruments not covered by any competency program as gaps. CompetenciesOwedSection renders it on the VeritaComp landing page. Reuses the shipped bridge + suggested-method-groups match rules; no new tables. Verified live on prod with real assignment data: 2 instruments assigned to a demo staffer produced owed=2, gaps=2 (HIGH, Technical Supervisor), then reverted cleanly. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23 session, Michael. Recurring request. Companion: cross-module evidence display on the VeritaDC policy shipped in PR #1313 (by-target cross-links surfaced in the policy View modal, browser-verified live).
+          <t>2026-09-23/24 session, Michael ("veritacomp bases what competencies they owe (currently untrue, but needs to be true)"). Option 1 (unify roster on VeritaStaff, match instruments by id).
 ---</t>
         </is>
       </c>
@@ -1536,12 +1498,12 @@
     <row r="15" ht="90" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>C38</t>
+          <t>C39</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>VeritaTrack calendar month cells expand to reveal hidden tasks (was #45)</t>
+          <t>VeritaScan line items can attach or link evidence (was #46)</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr"/>
@@ -1549,12 +1511,12 @@
       <c r="E15" s="3" t="inlineStr"/>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: VeritaTrack CalendarView month cells with more than three tasks now expand in place (chevron, "+N more" toggling to "Show less", due dates), so no task is hidden with no path to it (client/src/pages/VeritaTrackAppPage.tsx CalendarView). Shipped 2026-09-23. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1312 (squash a1dda93d). VeritaScan scan checklist items now show linked evidence as chips (open link, remove) plus a writer "Link evidence" affordance whose picker links an existing VeritaDC/Library document; a shortcut deep-links to the Library for new (governed) documents. Reuses the already-shipped lab_documents + document_checklist_links + coverage endpoints (URL-pointer only, no file storage, no new tables). Browser-verified live on prod (scan 23): the affordance renders and the picker opens. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>2026-09-23 session, Michael screenshot of the VeritaTrack calendar (lab 3, September cell).
+          <t>2026-09-23 session, Michael. Recurring request. Companion: cross-module evidence display on the VeritaDC policy shipped in PR #1313 (by-target cross-links surfaced in the policy View modal, browser-verified live).
 ---</t>
         </is>
       </c>
@@ -1563,12 +1525,12 @@
     <row r="16" ht="90" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>C37</t>
+          <t>C38</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Long Excel column headers no longer clip CFR citations (was #44)</t>
+          <t>VeritaTrack calendar month cells expand to reveal hidden tasks (was #45)</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr"/>
@@ -1576,12 +1538,12 @@
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. The VeritaMap export derives the header row height from the longest wrapped header via headerRowHeight(headers, colWidths) (server/routes.ts:15935) instead of a fixed 20, so "Reference Range Attestation (42 CFR 493.1253)" and the other long headers print in full. No new code this session. Closed 2026-09-24.</t>
+          <t>Closure evidence: VeritaTrack CalendarView month cells with more than three tasks now expand in place (chevron, "+N more" toggling to "Show less", due dates), so no task is hidden with no path to it (client/src/pages/VeritaTrackAppPage.tsx CalendarView). Shipped 2026-09-23. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+          <t>2026-09-23 session, Michael screenshot of the VeritaTrack calendar (lab 3, September cell).
 ---</t>
         </is>
       </c>
@@ -1590,12 +1552,12 @@
     <row r="17" ht="90" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>C36</t>
+          <t>C37</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>License stamp no longer clobbers the §6 header/footer or names the wrong lab (was #43)</t>
+          <t>Long Excel column headers no longer clip CFR citations (was #44)</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr"/>
@@ -1603,7 +1565,7 @@
       <c r="E17" s="3" t="inlineStr"/>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. setHeaderFooter (shared/licenseExceljs.ts:155-209) now preserves an existing §6 header and appends (not overwrites) the footer left section, and customer-facing exports name the scoped lab: the VeritaScan library export reads req.scope.lab.name / clia_number (server/routes.ts:16572-16573), not the licensee. No new code this session (avoided regressing the existing fix). Closed 2026-09-24.</t>
+          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. The VeritaMap export derives the header row height from the longest wrapped header via headerRowHeight(headers, colWidths) (server/routes.ts:15935) instead of a fixed 20, so "Reference Range Attestation (42 CFR 493.1253)" and the other long headers print in full. No new code this session. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -1617,18 +1579,45 @@
     <row r="18" ht="90" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>C34</t>
+          <t>C36</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Wire the two static-audit guards into CI (was #43)</t>
+          <t>License stamp no longer clobbers the §6 header/footer or names the wrong lab (was #43)</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr"/>
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. setHeaderFooter (shared/licenseExceljs.ts:155-209) now preserves an existing §6 header and appends (not overwrites) the footer left section, and customer-facing exports name the scoped lab: the VeritaScan library export reads req.scope.lab.name / clia_number (server/routes.ts:16572-16573), not the licensee. No new code this session (avoided regressing the existing fix). Closed 2026-09-24.</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+---</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19" ht="90" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>C34</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Wire the two static-audit guards into CI (was #43)</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr"/>
+      <c r="D19" s="3" t="inlineStr"/>
+      <c r="E19" s="3" t="inlineStr"/>
+      <c r="F19" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: both guards wired into the Multi-Lab Mutations Audit CI
 workflow (.github/workflows/multilab-mutations-audit.yml) as steps:
@@ -1640,24 +1629,24 @@
 (same caveat as the existing guards already in that workflow).</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr"/>
-      <c r="H18" s="2" t="inlineStr"/>
-    </row>
-    <row r="19" ht="90" customHeight="1">
-      <c r="A19" s="3" t="inlineStr">
+      <c r="G19" s="3" t="inlineStr"/>
+      <c r="H19" s="3" t="inlineStr"/>
+    </row>
+    <row r="20" ht="90" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>C35</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>Legacy /api/studies over-returns studies across labs (was #44)</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr"/>
-      <c r="D19" s="3" t="inlineStr"/>
-      <c r="E19" s="3" t="inlineStr"/>
-      <c r="F19" s="3" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr"/>
+      <c r="D20" s="2" t="inlineStr"/>
+      <c r="E20" s="2" t="inlineStr"/>
+      <c r="F20" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: GET /api/studies now scopes its list to the active lab
 when one is resolved from the Referer (server/routes.ts), so every returned row
@@ -1667,24 +1656,24 @@
 mirroring the /api/labs/:labId/studies handler. Closed 2026-06-14.</t>
         </is>
       </c>
-      <c r="G19" s="3" t="inlineStr"/>
-      <c r="H19" s="3" t="inlineStr"/>
-    </row>
-    <row r="20" ht="90" customHeight="1">
-      <c r="A20" s="2" t="inlineStr">
+      <c r="G20" s="2" t="inlineStr"/>
+      <c r="H20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21" ht="90" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>C30</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>Verify-script convention backfill (was #41)</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr"/>
-      <c r="D20" s="2" t="inlineStr"/>
-      <c r="E20" s="2" t="inlineStr"/>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="C21" s="3" t="inlineStr"/>
+      <c r="D21" s="3" t="inlineStr"/>
+      <c r="E21" s="3" t="inlineStr"/>
+      <c r="F21" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: all 8 high-stakes math/logic commits now ship a paired
 scripts/verify-*.js (EP17 sensitivity, Deming lot-to-lot, CUMSUM+QC+multi-analyte,
@@ -1692,30 +1681,30 @@
 TEa boundary), per the strike-throughs in #41. Closed 2026-06-13.</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr">
+      <c r="G21" s="3" t="inlineStr">
         <is>
           <t>scripts/audit_verify_script_coverage.py lookback, 2026-06-02; backfills
 landed 2026-06-03..06.
 ---</t>
         </is>
       </c>
-      <c r="H20" s="2" t="inlineStr"/>
-    </row>
-    <row r="21" ht="90" customHeight="1">
-      <c r="A21" s="3" t="inlineStr">
+      <c r="H21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22" ht="90" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>C31</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B22" s="2" t="inlineStr">
         <is>
           <t>VeritaPT AAA create/update/delete silently no-op in the multi-lab UI</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr"/>
-      <c r="D21" s="3" t="inlineStr"/>
-      <c r="E21" s="3" t="inlineStr"/>
-      <c r="F21" s="3" t="inlineStr">
+      <c r="C22" s="2" t="inlineStr"/>
+      <c r="D22" s="2" t="inlineStr"/>
+      <c r="E22" s="2" t="inlineStr"/>
+      <c r="F22" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #754 (commit 92ad499) added lab-scoped POST/PUT/DELETE
 /api/labs/:labId/pt/aa-records. The UI posted to the lab-scoped path but only GET
@@ -1726,30 +1715,30 @@
 route mis-filed records to the user's default lab on multi-lab accounts).</t>
         </is>
       </c>
-      <c r="G21" s="3" t="inlineStr">
+      <c r="G22" s="2" t="inlineStr">
         <is>
           <t>2026-06-13, found during #18 Phase 3 QA;
 scripts/audit-labscoped-write-routes.mjs now guards the class.
 ---</t>
         </is>
       </c>
-      <c r="H21" s="3" t="inlineStr"/>
-    </row>
-    <row r="22" ht="90" customHeight="1">
-      <c r="A22" s="2" t="inlineStr">
+      <c r="H22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23" ht="90" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>C32</t>
         </is>
       </c>
-      <c r="B22" s="2" t="inlineStr">
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>VeritaComp "Unlock assessment" false-success no-op</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr"/>
-      <c r="D22" s="2" t="inlineStr"/>
-      <c r="E22" s="2" t="inlineStr"/>
-      <c r="F22" s="2" t="inlineStr">
+      <c r="C23" s="3" t="inlineStr"/>
+      <c r="D23" s="3" t="inlineStr"/>
+      <c r="E23" s="3" t="inlineStr"/>
+      <c r="F23" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #755 (commit 4234007) moved the unlock route to
 /api/labs/:labId/competency/assessments/:id/unlock (the path the client calls).
@@ -1760,29 +1749,29 @@
 HTML).</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr">
+      <c r="G23" s="3" t="inlineStr">
         <is>
           <t>2026-06-13, found by scripts/audit-labscoped-write-routes.mjs.
 ---</t>
         </is>
       </c>
-      <c r="H22" s="2" t="inlineStr"/>
-    </row>
-    <row r="23" ht="90" customHeight="1">
-      <c r="A23" s="3" t="inlineStr">
+      <c r="H23" s="3" t="inlineStr"/>
+    </row>
+    <row r="24" ht="90" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>C33</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>FK-cascade delete 500s + NavBar laptop-width overflow</t>
         </is>
       </c>
-      <c r="C23" s="3" t="inlineStr"/>
-      <c r="D23" s="3" t="inlineStr"/>
-      <c r="E23" s="3" t="inlineStr"/>
-      <c r="F23" s="3" t="inlineStr">
+      <c r="C24" s="2" t="inlineStr"/>
+      <c r="D24" s="2" t="inlineStr"/>
+      <c r="E24" s="2" t="inlineStr"/>
+      <c r="F24" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PRs #749/#750 fixed NavBar horizontal overflow at laptop
 widths (collapse to the hamburger below 1560px); prod-verified at 1280-1920 with the
@@ -1793,37 +1782,9 @@
 500 -&gt; 200. scripts/audit-delete-cascades.mjs guards the class.</t>
         </is>
       </c>
-      <c r="G23" s="3" t="inlineStr">
+      <c r="G24" s="2" t="inlineStr">
         <is>
           <t>2026-06-13 browser QA of the A7-D4 wave + retro-QC of the 72h PR window.
----</t>
-        </is>
-      </c>
-      <c r="H23" s="3" t="inlineStr"/>
-    </row>
-    <row r="24" ht="90" customHeight="1">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>C1</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>FAQ "over 25 years" -&gt; "over 23 years"</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr"/>
-      <c r="D24" s="2" t="inlineStr"/>
-      <c r="E24" s="2" t="inlineStr"/>
-      <c r="F24" s="2" t="inlineStr">
-        <is>
-          <t>Closure evidence: client/src/pages/FAQPage.tsx line 20 reads "over
-23 years" as of 2026-05-01.</t>
-        </is>
-      </c>
-      <c r="G24" s="2" t="inlineStr">
-        <is>
-          <t>session 299e9a73 turn 14, ~2026-04-28.
 ---</t>
         </is>
       </c>
@@ -1832,18 +1793,46 @@
     <row r="25" ht="90" customHeight="1">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>C5</t>
+          <t>C1</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>David's VeritaQA grey-button bug (seat permissions mode)</t>
+          <t>FAQ "over 25 years" -&gt; "over 23 years"</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr"/>
       <c r="D25" s="3" t="inlineStr"/>
       <c r="E25" s="3" t="inlineStr"/>
       <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>Closure evidence: client/src/pages/FAQPage.tsx line 20 reads "over
+23 years" as of 2026-05-01.</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>session 299e9a73 turn 14, ~2026-04-28.
+---</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26" ht="90" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>David's VeritaQA grey-button bug (seat permissions mode)</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr"/>
+      <c r="D26" s="2" t="inlineStr"/>
+      <c r="E26" s="2" t="inlineStr"/>
+      <c r="F26" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #10 squash-merged as commit a43fbba on
 2026-05-01 23:19 MST. Railway deploy succeeded; deployed bundle
@@ -1856,7 +1845,7 @@
 against his exact stored shape (14 of 14 expected outcomes matched).</t>
         </is>
       </c>
-      <c r="G25" s="3" t="inlineStr">
+      <c r="G26" s="2" t="inlineStr">
         <is>
           <t>2026-05-01 David's report; veritabench + veritastock
 weren't in MODULE_LIST so seat permissions silently defaulted to
@@ -1864,46 +1853,17 @@
 ---</t>
         </is>
       </c>
-      <c r="H25" s="3" t="inlineStr"/>
-    </row>
-    <row r="26" ht="90" customHeight="1">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>C2</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>TeamPage present-tense "TJC surveyor" check</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr"/>
-      <c r="D26" s="2" t="inlineStr"/>
-      <c r="E26" s="2" t="inlineStr"/>
-      <c r="F26" s="2" t="inlineStr">
-        <is>
-          <t>Closure evidence: site-wide search confirmed all surveyor language
-is past-tense, consistent with user's 2021-2025 service. User closed
-the item in session 299e9a73 turn 4.</t>
-        </is>
-      </c>
-      <c r="G26" s="2" t="inlineStr">
-        <is>
-          <t>session 299e9a73, ~2026-04-28.
----</t>
-        </is>
-      </c>
       <c r="H26" s="2" t="inlineStr"/>
     </row>
     <row r="27" ht="90" customHeight="1">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>C3</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>My Studies CSV/XLSX export (John as design partner)</t>
+          <t>TeamPage present-tense "TJC surveyor" check</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr"/>
@@ -1911,14 +1871,14 @@
       <c r="E27" s="3" t="inlineStr"/>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: client/src/pages/DashboardPage.tsx line 46 calls
-/api/my-studies/export. server/routes.ts line 1491 implements the
-endpoint. Pulled forward into pre-COLA per user instruction.</t>
+          <t>Closure evidence: site-wide search confirmed all surveyor language
+is past-tense, consistent with user's 2021-2025 service. User closed
+the item in session 299e9a73 turn 4.</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>session 299e9a73 turn 5, ~2026-04-28.
+          <t>session 299e9a73, ~2026-04-28.
 ---</t>
         </is>
       </c>
@@ -1927,12 +1887,12 @@
     <row r="28" ht="90" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>C4</t>
+          <t>C3</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Rotate GitHub PAT (because old PAT was committed in SESSION_HANDOFF files)</t>
+          <t>My Studies CSV/XLSX export (John as design partner)</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr"/>
@@ -1940,13 +1900,14 @@
       <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: no ghp_* or github_pat_* patterns in current
-SESSION_HANDOFF.md or SESSION_HANDOFF-2.md as of 2026-05-01.</t>
+          <t>Closure evidence: client/src/pages/DashboardPage.tsx line 46 calls
+/api/my-studies/export. server/routes.ts line 1491 implements the
+endpoint. Pulled forward into pre-COLA per user instruction.</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>session 299e9a73, ~2026-04-28.
+          <t>session 299e9a73 turn 5, ~2026-04-28.
 ---</t>
         </is>
       </c>
@@ -1955,18 +1916,46 @@
     <row r="29" ht="90" customHeight="1">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>C6</t>
+          <t>C4</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>VeritaPolicy service-line filtering removed (formerly #4)</t>
+          <t>Rotate GitHub PAT (because old PAT was committed in SESSION_HANDOFF files)</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr"/>
       <c r="D29" s="3" t="inlineStr"/>
       <c r="E29" s="3" t="inlineStr"/>
       <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>Closure evidence: no ghp_* or github_pat_* patterns in current
+SESSION_HANDOFF.md or SESSION_HANDOFF-2.md as of 2026-05-01.</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>session 299e9a73, ~2026-04-28.
+---</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr"/>
+    </row>
+    <row r="30" ht="90" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>C6</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>VeritaPolicy service-line filtering removed (formerly #4)</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr"/>
+      <c r="D30" s="2" t="inlineStr"/>
+      <c r="E30" s="2" t="inlineStr"/>
+      <c r="F30" s="2" t="inlineStr">
         <is>
           <t>Closure rationale (operator decision 2026-05-10): Keep all
 VeritaPolicy rows. CFR-only references with no accreditor reference
@@ -1975,29 +1964,29 @@
 report misread the design intent.</t>
         </is>
       </c>
-      <c r="G29" s="3" t="inlineStr">
+      <c r="G30" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H29" s="3" t="inlineStr"/>
-    </row>
-    <row r="30" ht="90" customHeight="1">
-      <c r="A30" s="2" t="inlineStr">
+      <c r="H30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31" ht="90" customHeight="1">
+      <c r="A31" s="3" t="inlineStr">
         <is>
           <t>C7</t>
         </is>
       </c>
-      <c r="B30" s="2" t="inlineStr">
+      <c r="B31" s="3" t="inlineStr">
         <is>
           <t>CLIA number format validation (formerly #13)</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr"/>
-      <c r="D30" s="2" t="inlineStr"/>
-      <c r="E30" s="2" t="inlineStr"/>
-      <c r="F30" s="2" t="inlineStr">
+      <c r="C31" s="3" t="inlineStr"/>
+      <c r="D31" s="3" t="inlineStr"/>
+      <c r="E31" s="3" t="inlineStr"/>
+      <c r="F31" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: shared/validateClia.ts defines CLIA_REGEX =
 /^\d{2}D\d{7}$/ (line 24), validateClia() helper with whitespace
@@ -2008,30 +1997,30 @@
 shape exists and behaves as specified.</t>
         </is>
       </c>
-      <c r="G30" s="2" t="inlineStr">
+      <c r="G31" s="3" t="inlineStr">
         <is>
           <t>Agent verification 2026-05-10 via grep + file read.
 Operator confirmed shipped 2026-05-10.
 ---</t>
         </is>
       </c>
-      <c r="H30" s="2" t="inlineStr"/>
-    </row>
-    <row r="31" ht="90" customHeight="1">
-      <c r="A31" s="3" t="inlineStr">
+      <c r="H31" s="3" t="inlineStr"/>
+    </row>
+    <row r="32" ht="90" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t>C8</t>
         </is>
       </c>
-      <c r="B31" s="3" t="inlineStr">
+      <c r="B32" s="2" t="inlineStr">
         <is>
           <t>VeritaMap lab-wide menu toggle (formerly #19)</t>
         </is>
       </c>
-      <c r="C31" s="3" t="inlineStr"/>
-      <c r="D31" s="3" t="inlineStr"/>
-      <c r="E31" s="3" t="inlineStr"/>
-      <c r="F31" s="3" t="inlineStr">
+      <c r="C32" s="2" t="inlineStr"/>
+      <c r="D32" s="2" t="inlineStr"/>
+      <c r="E32" s="2" t="inlineStr"/>
+      <c r="F32" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: client/src/pages/VeritaMapLabwidePage.tsx
 exists and implements the labwide read-only union view. Route is
@@ -2041,59 +2030,59 @@
 parking lot plan (read-only union view, per-session toggle) shipped.</t>
         </is>
       </c>
-      <c r="G31" s="3" t="inlineStr">
+      <c r="G32" s="2" t="inlineStr">
         <is>
           <t>Agent verification 2026-05-10 via grep + file read.
 Operator confirmed shipped 2026-05-10.
 ---</t>
         </is>
       </c>
-      <c r="H31" s="3" t="inlineStr"/>
-    </row>
-    <row r="32" ht="90" customHeight="1">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>C9</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>Tier-1 smoke test checklist (formerly #6)</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr"/>
-      <c r="D32" s="2" t="inlineStr"/>
-      <c r="E32" s="2" t="inlineStr"/>
-      <c r="F32" s="2" t="inlineStr">
-        <is>
-          <t>Closure evidence: docs/smoke-test-tier1.md documents the Tier-1
-smoke-test process and post-deploy verification steps. Shipped via
-PR #81 as part of the 2026-05-10 wave.</t>
-        </is>
-      </c>
-      <c r="G32" s="2" t="inlineStr">
-        <is>
-          <t>Operator instruction 2026-05-10 in this session.
----</t>
-        </is>
-      </c>
       <c r="H32" s="2" t="inlineStr"/>
     </row>
     <row r="33" ht="90" customHeight="1">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>C10</t>
+          <t>C9</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>Per-module gating (formerly #7)</t>
+          <t>Tier-1 smoke test checklist (formerly #6)</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr"/>
       <c r="D33" s="3" t="inlineStr"/>
       <c r="E33" s="3" t="inlineStr"/>
       <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>Closure evidence: docs/smoke-test-tier1.md documents the Tier-1
+smoke-test process and post-deploy verification steps. Shipped via
+PR #81 as part of the 2026-05-10 wave.</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>Operator instruction 2026-05-10 in this session.
+---</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr"/>
+    </row>
+    <row r="34" ht="90" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>C10</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Per-module gating (formerly #7)</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr"/>
+      <c r="D34" s="2" t="inlineStr"/>
+      <c r="E34" s="2" t="inlineStr"/>
+      <c r="F34" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: Client-side useIsReadOnly module keys wired
 on client/src/pages/VeritaPolicyAppPage.tsx and
@@ -2108,29 +2097,29 @@
 PR #76.</t>
         </is>
       </c>
-      <c r="G33" s="3" t="inlineStr">
+      <c r="G34" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H33" s="3" t="inlineStr"/>
-    </row>
-    <row r="34" ht="90" customHeight="1">
-      <c r="A34" s="2" t="inlineStr">
+      <c r="H34" s="2" t="inlineStr"/>
+    </row>
+    <row r="35" ht="90" customHeight="1">
+      <c r="A35" s="3" t="inlineStr">
         <is>
           <t>C11</t>
         </is>
       </c>
-      <c r="B34" s="2" t="inlineStr">
+      <c r="B35" s="3" t="inlineStr">
         <is>
           <t>VeritaStock shipped copy (formerly #8)</t>
         </is>
       </c>
-      <c r="C34" s="2" t="inlineStr"/>
-      <c r="D34" s="2" t="inlineStr"/>
-      <c r="E34" s="2" t="inlineStr"/>
-      <c r="F34" s="2" t="inlineStr">
+      <c r="C35" s="3" t="inlineStr"/>
+      <c r="D35" s="3" t="inlineStr"/>
+      <c r="E35" s="3" t="inlineStr"/>
+      <c r="F35" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: client/src/pages/ArticleInventoryManagementPage.tsx
 line 305 footer reads "platform that includes VeritaStock™" instead
@@ -2138,29 +2127,29 @@
 on /resources/laboratory-inventory-management. Shipped via PR #75.</t>
         </is>
       </c>
-      <c r="G34" s="2" t="inlineStr">
+      <c r="G35" s="3" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H34" s="2" t="inlineStr"/>
-    </row>
-    <row r="35" ht="90" customHeight="1">
-      <c r="A35" s="3" t="inlineStr">
+      <c r="H35" s="3" t="inlineStr"/>
+    </row>
+    <row r="36" ht="90" customHeight="1">
+      <c r="A36" s="2" t="inlineStr">
         <is>
           <t>C12</t>
         </is>
       </c>
-      <c r="B35" s="3" t="inlineStr">
+      <c r="B36" s="2" t="inlineStr">
         <is>
           <t>Admin report one-row-per-lab (formerly #14)</t>
         </is>
       </c>
-      <c r="C35" s="3" t="inlineStr"/>
-      <c r="D35" s="3" t="inlineStr"/>
-      <c r="E35" s="3" t="inlineStr"/>
-      <c r="F35" s="3" t="inlineStr">
+      <c r="C36" s="2" t="inlineStr"/>
+      <c r="D36" s="2" t="inlineStr"/>
+      <c r="E36" s="2" t="inlineStr"/>
+      <c r="F36" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: /api/admin/report rewritten in
 server/routes.ts (~line 595) to LEFT JOIN labs on
@@ -2175,33 +2164,6 @@
 prerequisite, not a code bug). Shipped via PR #85.</t>
         </is>
       </c>
-      <c r="G35" s="3" t="inlineStr">
-        <is>
-          <t>Operator instruction 2026-05-10 in this session.
----</t>
-        </is>
-      </c>
-      <c r="H35" s="3" t="inlineStr"/>
-    </row>
-    <row r="36" ht="90" customHeight="1">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>C14</t>
-        </is>
-      </c>
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t>UI relabel "CLIA TEa" -&gt; "Lab-Set Internal Goal" (formerly #1)</t>
-        </is>
-      </c>
-      <c r="C36" s="2" t="inlineStr"/>
-      <c r="D36" s="2" t="inlineStr"/>
-      <c r="E36" s="2" t="inlineStr"/>
-      <c r="F36" s="2" t="inlineStr">
-        <is>
-          <t>Closure evidence: Shipped across four PRs over 2026-05-10.</t>
-        </is>
-      </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
@@ -2213,18 +2175,45 @@
     <row r="37" ht="90" customHeight="1">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>C13</t>
+          <t>C14</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>WSLH PT vendor (formerly #15)</t>
+          <t>UI relabel "CLIA TEa" -&gt; "Lab-Set Internal Goal" (formerly #1)</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr"/>
       <c r="D37" s="3" t="inlineStr"/>
       <c r="E37" s="3" t="inlineStr"/>
       <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>Closure evidence: Shipped across four PRs over 2026-05-10.</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>Operator instruction 2026-05-10 in this session.
+---</t>
+        </is>
+      </c>
+      <c r="H37" s="3" t="inlineStr"/>
+    </row>
+    <row r="38" ht="90" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>C13</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>WSLH PT vendor (formerly #15)</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr"/>
+      <c r="D38" s="2" t="inlineStr"/>
+      <c r="E38" s="2" t="inlineStr"/>
+      <c r="F38" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: Shipped 2026-05-10 via PR #79 (merge commit
 eeebc6e; merged after rebase to resolve a server/db.ts collision
@@ -2242,38 +2231,9 @@
 'WSLH' is the post-deploy success signal. Shipped via PR #79.</t>
         </is>
       </c>
-      <c r="G37" s="3" t="inlineStr">
+      <c r="G38" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
----</t>
-        </is>
-      </c>
-      <c r="H37" s="3" t="inlineStr"/>
-    </row>
-    <row r="38" ht="90" customHeight="1">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>C15</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>VeritaStock lot tracking + expiration + reorder alerts (formerly #21)</t>
-        </is>
-      </c>
-      <c r="C38" s="2" t="inlineStr"/>
-      <c r="D38" s="2" t="inlineStr"/>
-      <c r="E38" s="2" t="inlineStr"/>
-      <c r="F38" s="2" t="inlineStr">
-        <is>
-          <t>Closure evidence: VeritaStock™ shipped the bench-level inventory
-features the Perplexity competitor analysis identified as a gap:</t>
-        </is>
-      </c>
-      <c r="G38" s="2" t="inlineStr">
-        <is>
-          <t>Originally Perplexity competitor analysis 2026-05-10.
-Audit 2026-05-21 confirmed the feature set ships today.
 ---</t>
         </is>
       </c>
@@ -2282,12 +2242,12 @@
     <row r="39" ht="90" customHeight="1">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>C16</t>
+          <t>C15</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>PAL studies guided workflow (formerly #23)</t>
+          <t>VeritaStock lot tracking + expiration + reorder alerts (formerly #21)</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr"/>
@@ -2295,15 +2255,14 @@
       <c r="E39" s="3" t="inlineStr"/>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: VeritaCheck™ already ships the Precision /
-Accuracy / Linearity (PAL) study set under EP-protocol naming:</t>
+          <t>Closure evidence: VeritaStock™ shipped the bench-level inventory
+features the Perplexity competitor analysis identified as a gap:</t>
         </is>
       </c>
       <c r="G39" s="3" t="inlineStr">
         <is>
           <t>Originally Perplexity competitor analysis 2026-05-10.
-Audit 2026-05-21 confirmed the EP studies cover the PAL framing in
-full.
+Audit 2026-05-21 confirmed the feature set ships today.
 ---</t>
         </is>
       </c>
@@ -2312,12 +2271,12 @@
     <row r="40" ht="90" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>C17</t>
+          <t>C16</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Source-grounded 21/29/45 CFR + 42 CFR 482-485 (formerly #26)</t>
+          <t>PAL studies guided workflow (formerly #23)</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr"/>
@@ -2325,35 +2284,65 @@
       <c r="E40" s="2" t="inlineStr"/>
       <c r="F40" s="2" t="inlineStr">
         <is>
+          <t>Closure evidence: VeritaCheck™ already ships the Precision /
+Accuracy / Linearity (PAL) study set under EP-protocol naming:</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>Originally Perplexity competitor analysis 2026-05-10.
+Audit 2026-05-21 confirmed the EP studies cover the PAL framing in
+full.
+---</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr"/>
+    </row>
+    <row r="41" ht="90" customHeight="1">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>C17</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>Source-grounded 21/29/45 CFR + 42 CFR 482-485 (formerly #26)</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr"/>
+      <c r="D41" s="3" t="inlineStr"/>
+      <c r="E41" s="3" t="inlineStr"/>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
           <t>Closure evidence: PR #301 (commit 8c27806, merged 2026-05-21)
 source-grounded the 74 remaining non-493 entries in
 server/cfrRequirements.ts against verbatim eCFR XML. Breakdown
 shipped:</t>
         </is>
       </c>
-      <c r="G40" s="2" t="inlineStr">
+      <c r="G41" s="3" t="inlineStr">
         <is>
           <t>PR #301; tasks #18 in the in-session task tracker.
 ---</t>
         </is>
       </c>
-      <c r="H40" s="2" t="inlineStr"/>
-    </row>
-    <row r="41" ht="90" customHeight="1">
-      <c r="A41" s="3" t="inlineStr">
+      <c r="H41" s="3" t="inlineStr"/>
+    </row>
+    <row r="42" ht="90" customHeight="1">
+      <c r="A42" s="2" t="inlineStr">
         <is>
           <t>C18</t>
         </is>
       </c>
-      <c r="B41" s="3" t="inlineStr">
+      <c r="B42" s="2" t="inlineStr">
         <is>
           <t>VeritaPolicy "Non CLIA" chapter rename (formerly #3)</t>
         </is>
       </c>
-      <c r="C41" s="3" t="inlineStr"/>
-      <c r="D41" s="3" t="inlineStr"/>
-      <c r="E41" s="3" t="inlineStr"/>
-      <c r="F41" s="3" t="inlineStr">
+      <c r="C42" s="2" t="inlineStr"/>
+      <c r="D42" s="2" t="inlineStr"/>
+      <c r="E42" s="2" t="inlineStr"/>
+      <c r="F42" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #300 (commit 34d7707, merged 2026-05-21)
 renamed all 44 user-facing chapter labels in
@@ -2364,7 +2353,7 @@
 page.</t>
         </is>
       </c>
-      <c r="G41" s="3" t="inlineStr">
+      <c r="G42" s="2" t="inlineStr">
         <is>
           <t>CAP customer screenshot of the /veritapolicy chapter
 headers, 2026-05-01 evening. PR #300; tasks #17 in the in-session
@@ -2372,23 +2361,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H41" s="3" t="inlineStr"/>
-    </row>
-    <row r="42" ht="90" customHeight="1">
-      <c r="A42" s="2" t="inlineStr">
+      <c r="H42" s="2" t="inlineStr"/>
+    </row>
+    <row r="43" ht="90" customHeight="1">
+      <c r="A43" s="3" t="inlineStr">
         <is>
           <t>C19</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
+      <c r="B43" s="3" t="inlineStr">
         <is>
           <t>VeritaStock department-scope toggle (formerly #31)</t>
         </is>
       </c>
-      <c r="C42" s="2" t="inlineStr"/>
-      <c r="D42" s="2" t="inlineStr"/>
-      <c r="E42" s="2" t="inlineStr"/>
-      <c r="F42" s="2" t="inlineStr">
+      <c r="C43" s="3" t="inlineStr"/>
+      <c r="D43" s="3" t="inlineStr"/>
+      <c r="E43" s="3" t="inlineStr"/>
+      <c r="F43" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #319 (commit d01f5fe, merged 2026-05-22)
 shipped the persistent dept-scope toggle on VeritaStockPage. A new
@@ -2399,7 +2388,7 @@
 workspace without re-filtering.</t>
         </is>
       </c>
-      <c r="G42" s="2" t="inlineStr">
+      <c r="G43" s="3" t="inlineStr">
         <is>
           <t>John, San Carlos lab, 2026-05-21. Same conversation that
 drove the vendor dropdown (PR #304), FILTERED VIEW banner (PR #305),
@@ -2407,23 +2396,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H42" s="2" t="inlineStr"/>
-    </row>
-    <row r="43" ht="90" customHeight="1">
-      <c r="A43" s="3" t="inlineStr">
+      <c r="H43" s="3" t="inlineStr"/>
+    </row>
+    <row r="44" ht="90" customHeight="1">
+      <c r="A44" s="2" t="inlineStr">
         <is>
           <t>C20</t>
         </is>
       </c>
-      <c r="B43" s="3" t="inlineStr">
+      <c r="B44" s="2" t="inlineStr">
         <is>
           <t>Primary-lab seat counting (formerly #12)</t>
         </is>
       </c>
-      <c r="C43" s="3" t="inlineStr"/>
-      <c r="D43" s="3" t="inlineStr"/>
-      <c r="E43" s="3" t="inlineStr"/>
-      <c r="F43" s="3" t="inlineStr">
+      <c r="C44" s="2" t="inlineStr"/>
+      <c r="D44" s="2" t="inlineStr"/>
+      <c r="E44" s="2" t="inlineStr"/>
+      <c r="F44" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: is_primary_lab INTEGER NOT NULL DEFAULT 0
 column was added to the lab_members table at db.ts:1276, with the
@@ -2434,7 +2423,7 @@
 is_primary_lab=1 ordering).</t>
         </is>
       </c>
-      <c r="G43" s="3" t="inlineStr">
+      <c r="G44" s="2" t="inlineStr">
         <is>
           <t>2026-05-07 multi-lab discussion. Build shipped as part
 of the Multi-Lab Tier 2 architecture work (Phase 3.x series, prior
@@ -2443,23 +2432,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H43" s="3" t="inlineStr"/>
-    </row>
-    <row r="44" ht="90" customHeight="1">
-      <c r="A44" s="2" t="inlineStr">
+      <c r="H44" s="2" t="inlineStr"/>
+    </row>
+    <row r="45" ht="90" customHeight="1">
+      <c r="A45" s="3" t="inlineStr">
         <is>
           <t>C21</t>
         </is>
       </c>
-      <c r="B44" s="2" t="inlineStr">
+      <c r="B45" s="3" t="inlineStr">
         <is>
           <t>Multi-lab pricing model — Option A (formerly #11)</t>
         </is>
       </c>
-      <c r="C44" s="2" t="inlineStr"/>
-      <c r="D44" s="2" t="inlineStr"/>
-      <c r="E44" s="2" t="inlineStr"/>
-      <c r="F44" s="2" t="inlineStr">
+      <c r="C45" s="3" t="inlineStr"/>
+      <c r="D45" s="3" t="inlineStr"/>
+      <c r="E45" s="3" t="inlineStr"/>
+      <c r="F45" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #322 (commit 0ccd925, merged 2026-05-22)
 added the customer-facing line to the pricing page that reflects
@@ -2472,7 +2461,7 @@
 Enterprise+ block, reads:</t>
         </is>
       </c>
-      <c r="G44" s="2" t="inlineStr">
+      <c r="G45" s="3" t="inlineStr">
         <is>
           <t>2026-05-07 multi-lab discussion (Lisa Veri's
 canonical-case session). PR #322 (initial build); softening PR
@@ -2481,30 +2470,30 @@
 ---</t>
         </is>
       </c>
-      <c r="H44" s="2" t="inlineStr"/>
-    </row>
-    <row r="45" ht="90" customHeight="1">
-      <c r="A45" s="3" t="inlineStr">
+      <c r="H45" s="3" t="inlineStr"/>
+    </row>
+    <row r="46" ht="90" customHeight="1">
+      <c r="A46" s="2" t="inlineStr">
         <is>
           <t>C22</t>
         </is>
       </c>
-      <c r="B45" s="3" t="inlineStr">
+      <c r="B46" s="2" t="inlineStr">
         <is>
           <t>VeritaOps cost-per-test module (formerly #10)</t>
         </is>
       </c>
-      <c r="C45" s="3" t="inlineStr"/>
-      <c r="D45" s="3" t="inlineStr"/>
-      <c r="E45" s="3" t="inlineStr"/>
-      <c r="F45" s="3" t="inlineStr">
+      <c r="C46" s="2" t="inlineStr"/>
+      <c r="D46" s="2" t="inlineStr"/>
+      <c r="E46" s="2" t="inlineStr"/>
+      <c r="F46" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: v1 of the VeritaOps Cost-Per-Reportable-Test
 (CPRT) module shipped across PR #325 through PR #330 on 2026-05-22.
 The module is feature-complete for the typical lab director workflow.</t>
         </is>
       </c>
-      <c r="G45" s="3" t="inlineStr">
+      <c r="G46" s="2" t="inlineStr">
         <is>
           <t>This thread, 2026-05-07 12:05 PM CDT, user message:
 "Parking lot: build an operations module for cost per test
@@ -2513,262 +2502,262 @@
 ---</t>
         </is>
       </c>
-      <c r="H45" s="3" t="inlineStr"/>
-    </row>
-    <row r="46" ht="90" customHeight="1">
-      <c r="A46" s="2" t="inlineStr">
+      <c r="H46" s="2" t="inlineStr"/>
+    </row>
+    <row r="47" ht="90" customHeight="1">
+      <c r="A47" s="3" t="inlineStr">
         <is>
           <t>C23</t>
         </is>
       </c>
-      <c r="B46" s="2" t="inlineStr">
+      <c r="B47" s="3" t="inlineStr">
         <is>
           <t>CCL lab name visual disambiguation in lab switcher (formerly #34)</t>
         </is>
       </c>
-      <c r="C46" s="2" t="inlineStr"/>
-      <c r="D46" s="2" t="inlineStr">
+      <c r="C47" s="3" t="inlineStr"/>
+      <c r="D47" s="3" t="inlineStr">
         <is>
           <t>XS (under 1 day, actual)</t>
         </is>
       </c>
-      <c r="E46" s="2" t="inlineStr">
+      <c r="E47" s="3" t="inlineStr">
         <is>
           <t>Low — cosmetic; only mattered when Lisa or Michael picked the wrong lab from...</t>
         </is>
       </c>
-      <c r="F46" s="2" t="inlineStr">
+      <c r="F47" s="3" t="inlineStr">
         <is>
           <t>Effort: XS (under 1 day, actual)
 Importance: Low — cosmetic; only mattered when Lisa or Michael picked the wrong lab from the dropdown.</t>
         </is>
       </c>
-      <c r="G46" s="2" t="inlineStr">
+      <c r="G47" s="3" t="inlineStr">
         <is>
           <t>flagged 2026-05-23 immediately after provisioning Lisa's CCL lab; closed 2026-05-24.
 ---</t>
         </is>
       </c>
-      <c r="H46" s="2" t="inlineStr"/>
-    </row>
-    <row r="47" ht="90" customHeight="1">
-      <c r="A47" s="3" t="inlineStr">
+      <c r="H47" s="3" t="inlineStr"/>
+    </row>
+    <row r="48" ht="90" customHeight="1">
+      <c r="A48" s="2" t="inlineStr">
         <is>
           <t>C24</t>
         </is>
       </c>
-      <c r="B47" s="3" t="inlineStr">
+      <c r="B48" s="2" t="inlineStr">
         <is>
           <t>VC Unlimited Y1/Y2 price disclosure UX (formerly #35)</t>
         </is>
       </c>
-      <c r="C47" s="3" t="inlineStr"/>
-      <c r="D47" s="3" t="inlineStr">
+      <c r="C48" s="2" t="inlineStr"/>
+      <c r="D48" s="2" t="inlineStr">
         <is>
           <t>XS (under 1 day, actual)</t>
         </is>
       </c>
-      <c r="E47" s="3" t="inlineStr">
+      <c r="E48" s="2" t="inlineStr">
         <is>
           <t>Low when shipped (proactive, no customer complaint yet) — but high if a procu...</t>
         </is>
       </c>
-      <c r="F47" s="3" t="inlineStr">
+      <c r="F48" s="2" t="inlineStr">
         <is>
           <t>Effort: XS (under 1 day, actual)
 Importance: Low when shipped (proactive, no customer complaint yet) — but high if a procurement reviewer later disputes the $499 renewal as undisclosed.</t>
         </is>
       </c>
-      <c r="G47" s="3" t="inlineStr">
+      <c r="G48" s="2" t="inlineStr">
         <is>
           <t>Pricing rebuild 2026-05-23; closed 2026-05-24 proactively before any customer dispute.
 ---</t>
         </is>
       </c>
-      <c r="H47" s="3" t="inlineStr"/>
-    </row>
-    <row r="48" ht="90" customHeight="1">
-      <c r="A48" s="2" t="inlineStr">
+      <c r="H48" s="2" t="inlineStr"/>
+    </row>
+    <row r="49" ht="90" customHeight="1">
+      <c r="A49" s="3" t="inlineStr">
         <is>
           <t>C25</t>
         </is>
       </c>
-      <c r="B48" s="2" t="inlineStr">
+      <c r="B49" s="3" t="inlineStr">
         <is>
           <t>VeritaQC Phase 1 (Levey-Jennings + Westgard live engine) (formerly #20)</t>
         </is>
       </c>
-      <c r="C48" s="2" t="inlineStr"/>
-      <c r="D48" s="2" t="inlineStr">
+      <c r="C49" s="3" t="inlineStr"/>
+      <c r="D49" s="3" t="inlineStr">
         <is>
           <t>L (about 5 days end-to-end, actual: Phase 0 schema → Phase 1A evaluator → 1B...</t>
         </is>
       </c>
-      <c r="E48" s="2" t="inlineStr">
+      <c r="E49" s="3" t="inlineStr">
         <is>
           <t>High — largest single gap vs myLabCompliance.io per Perplexity competitor ana...</t>
         </is>
       </c>
-      <c r="F48" s="2" t="inlineStr">
+      <c r="F49" s="3" t="inlineStr">
         <is>
           <t>Effort: L (about 5 days end-to-end, actual: Phase 0 schema → Phase 1A evaluator → 1B entry UI → 1C daily review → 1D monthly PDF + attestation)
 Importance: High — largest single gap vs myLabCompliance.io per Perplexity competitor analysis; promotes VeritaAssure from documentation tool to lab operations platform.</t>
         </is>
       </c>
-      <c r="G48" s="2" t="inlineStr">
+      <c r="G49" s="3" t="inlineStr">
         <is>
           <t>Perplexity competitor analysis 2026-05-10. Scoping confirmed via the build_phase1_mockup.py iterations 2026-05-24. Shipped 2026-05-25.
 ---</t>
         </is>
       </c>
-      <c r="H48" s="2" t="inlineStr"/>
-    </row>
-    <row r="49" ht="90" customHeight="1">
-      <c r="A49" s="3" t="inlineStr">
+      <c r="H49" s="3" t="inlineStr"/>
+    </row>
+    <row r="50" ht="90" customHeight="1">
+      <c r="A50" s="2" t="inlineStr">
         <is>
           <t>C26</t>
         </is>
       </c>
-      <c r="B49" s="3" t="inlineStr">
+      <c r="B50" s="2" t="inlineStr">
         <is>
           <t>VeritaLab CMS-116 application support + state licensing registry (formerly #22)</t>
         </is>
       </c>
-      <c r="C49" s="3" t="inlineStr"/>
-      <c r="D49" s="3" t="inlineStr">
+      <c r="C50" s="2" t="inlineStr"/>
+      <c r="D50" s="2" t="inlineStr">
         <is>
           <t>M (1-2 weeks for v1, actual)</t>
         </is>
       </c>
-      <c r="E49" s="3" t="inlineStr">
+      <c r="E50" s="2" t="inlineStr">
         <is>
           <t>Medium — competitor parity (myLabCompliance.io) plus useful at lab startup an...</t>
         </is>
       </c>
-      <c r="F49" s="3" t="inlineStr">
+      <c r="F50" s="2" t="inlineStr">
         <is>
           <t>Effort: M (1-2 weeks for v1, actual)
 Importance: Medium — competitor parity (myLabCompliance.io) plus useful at lab startup and at certificate-type changes.</t>
         </is>
       </c>
-      <c r="G49" s="3" t="inlineStr">
+      <c r="G50" s="2" t="inlineStr">
         <is>
           <t>Perplexity competitor analysis (myLabCompliance.io), 2026-05-10. Reclassified as a VeritaLab extension 2026-05-25. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H49" s="3" t="inlineStr"/>
-    </row>
-    <row r="50" ht="90" customHeight="1">
-      <c r="A50" s="2" t="inlineStr">
+      <c r="H50" s="2" t="inlineStr"/>
+    </row>
+    <row r="51" ht="90" customHeight="1">
+      <c r="A51" s="3" t="inlineStr">
         <is>
           <t>C27</t>
         </is>
       </c>
-      <c r="B50" s="2" t="inlineStr">
+      <c r="B51" s="3" t="inlineStr">
         <is>
           <t>Active vs view-only seat split (formerly #33)</t>
         </is>
       </c>
-      <c r="C50" s="2" t="inlineStr"/>
-      <c r="D50" s="2" t="inlineStr">
+      <c r="C51" s="3" t="inlineStr"/>
+      <c r="D51" s="3" t="inlineStr">
         <is>
           <t>M (~1 week of engineering, actual: shipped in a single multi-PR session)</t>
         </is>
       </c>
-      <c r="E50" s="2" t="inlineStr">
+      <c r="E51" s="3" t="inlineStr">
         <is>
           <t>Medium — closed the gap between /pricing copy and product behavior; gives sal...</t>
         </is>
       </c>
-      <c r="F50" s="2" t="inlineStr">
+      <c r="F51" s="3" t="inlineStr">
         <is>
           <t>Effort: M (~1 week of engineering, actual: shipped in a single multi-PR session)
 Importance: Medium — closed the gap between /pricing copy and product behavior; gives sales a clean answer for "do you charge for our medical director?"</t>
         </is>
       </c>
-      <c r="G50" s="2" t="inlineStr">
+      <c r="G51" s="3" t="inlineStr">
         <is>
           <t>Pricing analysis doc Decision 3 (2026-05-21); MEDIUM scenario revised 2026-05-29 to retire the "unlimited view-only" claim. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H50" s="2" t="inlineStr"/>
-    </row>
-    <row r="51" ht="90" customHeight="1">
-      <c r="A51" s="3" t="inlineStr">
+      <c r="H51" s="3" t="inlineStr"/>
+    </row>
+    <row r="52" ht="90" customHeight="1">
+      <c r="A52" s="2" t="inlineStr">
         <is>
           <t>C28</t>
         </is>
       </c>
-      <c r="B51" s="3" t="inlineStr">
+      <c r="B52" s="2" t="inlineStr">
         <is>
           <t>"Why VeritaCheck" comparative one-pager (formerly #37)</t>
         </is>
       </c>
-      <c r="C51" s="3" t="inlineStr"/>
-      <c r="D51" s="3" t="inlineStr">
+      <c r="C52" s="2" t="inlineStr"/>
+      <c r="D52" s="2" t="inlineStr">
         <is>
           <t>S (one design pass + four claim paragraphs + PDF + matching marketing-site pa...</t>
         </is>
       </c>
-      <c r="E51" s="3" t="inlineStr">
+      <c r="E52" s="2" t="inlineStr">
         <is>
           <t>Medium — closed a positioning gap surfaced by six COLA conference attendees a...</t>
         </is>
       </c>
-      <c r="F51" s="3" t="inlineStr">
+      <c r="F52" s="2" t="inlineStr">
         <is>
           <t>Effort: S (one design pass + four claim paragraphs + PDF + matching marketing-site page, actual)
 Importance: Medium — closed a positioning gap surfaced by six COLA conference attendees attached to a legacy verification tool; converts product-quality advantage into a leave-behind Lisa can hand out.</t>
         </is>
       </c>
-      <c r="G51" s="3" t="inlineStr">
+      <c r="G52" s="2" t="inlineStr">
         <is>
           <t>2026-05-11 / 2026-05-12 conference notes review with Michael. Conference attendees (Whitehead, Odegard, Othman, Molinelli, Kyle, Allred) expressed interest in equivalent / superior product. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H51" s="3" t="inlineStr"/>
-    </row>
-    <row r="52" ht="90" customHeight="1">
-      <c r="A52" s="2" t="inlineStr">
+      <c r="H52" s="2" t="inlineStr"/>
+    </row>
+    <row r="53" ht="90" customHeight="1">
+      <c r="A53" s="3" t="inlineStr">
         <is>
           <t>C29</t>
         </is>
       </c>
-      <c r="B52" s="2" t="inlineStr">
+      <c r="B53" s="3" t="inlineStr">
         <is>
           <t>VeritaPolicy approval workflow — MediaLab functional mirror</t>
         </is>
       </c>
-      <c r="C52" s="2" t="inlineStr"/>
-      <c r="D52" s="2" t="inlineStr">
+      <c r="C53" s="3" t="inlineStr"/>
+      <c r="D53" s="3" t="inlineStr">
         <is>
           <t>XL (one focused session, 12 PRs landed)</t>
         </is>
       </c>
-      <c r="E52" s="2" t="inlineStr">
+      <c r="E53" s="3" t="inlineStr">
         <is>
           <t>High — replaces MediaLab Document Control ($752/$2,250 starting price, scalin...</t>
         </is>
       </c>
-      <c r="F52" s="2" t="inlineStr">
+      <c r="F53" s="3" t="inlineStr">
         <is>
           <t>Effort: XL (one focused session, 12 PRs landed)
 Importance: High — replaces MediaLab Document Control ($752/$2,250 starting price, scaling to $10K-$20K/yr at enterprise per Capterra public data) with an included VeritaPolicy feature; closes a real positioning gap and gives sales a direct comparator line.</t>
         </is>
       </c>
-      <c r="G52" s="2" t="inlineStr">
+      <c r="G53" s="3" t="inlineStr">
         <is>
           <t>Pricing strategy conversation 2026-05-29 (Michael: "I don't like bolt-ons; we should replicate this") → scoped 8 phases → shipped all 12 PRs in single session. Shipped 2026-05-29.
 ---</t>
         </is>
       </c>
-      <c r="H52" s="2" t="inlineStr"/>
+      <c r="H53" s="3" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H52"/>
+  <autoFilter ref="A1:H53"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
TASK: Move parking-lot #36 to CLOSED (C52) after VeritaResponse internal NCE shipped
PLAN: Update PARKING_LOT.md and PARKING_LOT.xlsx to reflect #36 (VeritaResponse internal NCE) shipped: move #36 from OPEN to CLOSED as C52 with the PR reference. Docs-only bookkeeping.
Self-check: docs-only, no code paths touched; xlsx regenerated from the tracked script; validate gate green on PR.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PARKING_LOT.xlsx
+++ b/PARKING_LOT.xlsx
@@ -12,8 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RETIRED" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$52</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$53</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RETIRED'!$A$1:$H$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -822,6 +822,10 @@
 _(item #33 closed 2026-05-28; see C27 below)_
 ---
 _(items #34 and #35 closed 2026-05-24; see C23 and C24 below)_
+---
+_(item #36 closed 2026-09-29; shipped PR #1368, prod-verified, see C52 below)_
+---
+_(item #37 closed 2026-05-28; see C28 below)_
 ---</t>
         </is>
       </c>
@@ -829,40 +833,42 @@
     <row r="8" ht="90" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>38</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>New module: laboratory non-conforming event documentation</t>
+          <t>Screen-capture video: VeritaCheck method comparison in 60 seconds</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Scoped, not started (updated 2026-09-28). Now lands in VeritaResponse per Michael's direction above; the earlier "new standalone module" framing is superseded. Do not start building until Michael g...</t>
+          <t>Open. Re-parked 2026-05-27 (originally PR #117, abandoned with merge conflicts then closed-and-re-authored at current numbering). Pending operator decision on whether to record this themselves or p...</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>L (initial estimate, pending Michael's scope walkthrough — likely new DB tabl...</t>
+          <t>S for agent prep (storyboard / pre-fill / captions / checklist); ~1 hour of o...</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>High — every accredited laboratory (TJC, CAP, COLA, AABB) has to document non...</t>
+          <t>Medium — operator selected this as the highest-impact positioning artifact du...</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Build a module to document laboratory non-conforming events (NCEs). Surfaces a lab needs to capture include specimen rejection, temperature excursions, reagent issues, equipment failures, result-reporting errors, transcription errors, lost specimens, contamination events, and similar quality incidents. Full scope, target accreditor mapping, terminology preference (NCE / NCR / event / incident / occurrence), and how it should relate to the existing VeritaQC corrective-action engine and VeritaResponse deficiency tracker are TBD pending Michael's scope walkthrough.</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr"/>
+          <t>30-60 second screen recording demonstrating the "experienced lab tech figures it out in seconds" claim. From blank method-comparison study to completed PDF, no voiceover, no narration, visible cursor motion. Embed autoplay-muted on the marketing site, include in conference follow-up emails.</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-12 conversation. Michael selected the screen-cap video as the highest-impact positioning artifact, then asked the agent to record it. Agent does not have screen-recording capability; option parked rather than fudged.</t>
+        </is>
+      </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Post-COLA. No customer urgency yet, but high strategic value once defined — closes a real gap every lab has and that no other Verita module currently serves.
----
-_(item #37 closed 2026-05-28; see C28 below)_
+          <t>Post-COLA, conference-driven.
 ---</t>
         </is>
       </c>
@@ -870,73 +876,30 @@
     <row r="9" ht="90" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>39</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Screen-capture video: VeritaCheck method comparison in 60 seconds</t>
+          <t>MediaLab parity hardening (VeritaPolicy approval workflow depth)</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Open. Re-parked 2026-05-27 (originally PR #117, abandoned with merge conflicts then closed-and-re-authored at current numbering). Pending operator decision on whether to record this themselves or p...</t>
+          <t>Small-item sequence COMPLETE (items 1-5 all shipped; verified against the codebase 2026-09-29, print view PR #1367). Remaining depth items (SSO/AD, delegation, in-browser editing, per-department ro...</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>S for agent prep (storyboard / pre-fill / captions / checklist); ~1 hour of o...</t>
+          <t>L (1-2 weeks for the high-value items; each independent feature is M)</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Medium — operator selected this as the highest-impact positioning artifact du...</t>
+          <t>Medium-High — the C29 build shipped the surface MediaLab markets but depth is...</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>30-60 second screen recording demonstrating the "experienced lab tech figures it out in seconds" claim. From blank method-comparison study to completed PDF, no voiceover, no narration, visible cursor motion. Embed autoplay-muted on the marketing site, include in conference follow-up emails.</t>
-        </is>
-      </c>
-      <c r="G9" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-12 conversation. Michael selected the screen-cap video as the highest-impact positioning artifact, then asked the agent to record it. Agent does not have screen-recording capability; option parked rather than fudged.</t>
-        </is>
-      </c>
-      <c r="H9" s="3" t="inlineStr">
-        <is>
-          <t>Post-COLA, conference-driven.
----</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="90" customHeight="1">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>39</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>MediaLab parity hardening (VeritaPolicy approval workflow depth)</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Small-item sequence COMPLETE (items 1-5 all shipped; verified against the codebase 2026-09-29, print view PR #1367). Remaining depth items (SSO/AD, delegation, in-browser editing, per-department ro...</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>L (1-2 weeks for the high-value items; each independent feature is M)</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>Medium-High — the C29 build shipped the surface MediaLab markets but depth is...</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>The VeritaPolicy approval workflow build (C29, 2026-05-29) hit roughly 60-70% MediaLab feature surface. The following gaps remain when comparing against an enterprise MediaLab Document Control deployment:
 - Quizzes on attestations. Schema columns quiz_score and quiz_total_questions exist on policy_attestations but the quiz authoring + presentation UI was scoped out of Phase 4. MediaLab labs use 5-10 multiple-choice questions per policy to confirm comprehension, not just attestation. Adds compliance defensibility.
@@ -946,54 +909,93 @@
 - In-browser DOCX editing. MediaLab has a structured editor that creates a Table of Contents from headings. We treat documents as...</t>
         </is>
       </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-29 QA pass after C29 shipped (qa-policy-build.js + qa-policy-ui.js: 54/54 happy path verified). Honest depth assessment surfaced by Michael's "how confident are you" question — see C29 entry for full QA receipts.</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>Post-COLA. Defensive against MediaLab in head-to-head sales calls.
+---</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="90" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>VeritaQC Import Phase A: human-in-the-loop Gate 3 click-through (deferred)</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Open, awaiting Michael's 5-minute click test. Will move task #77 to completed only after he reports the user-visible result.
+---</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>XS (~5 minutes of Michael's time on a live URL).</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Low. Backend contract is fully verified via 35/35 passing offline contract ch...</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Effort: XS (~5 minutes of Michael's time on a live URL).
+Importance: Low. Backend contract is fully verified via 35/35 passing offline contract checks (scripts/verify-veritaqc-import.js) plus three live-API smoke checks against prod (candidates, preview, mappings PUT/GET) on Riverside Regional with seed lot SEED-1780436709094 (18 Glucose results). The browser-driven click was not run because Claude-in-Chrome's renderer froze repeatedly on the Radix Select inside VeritaCheckPage, not on Phase A code itself. Risk of a UX bug surviving to a customer is small but not zero.</t>
+        </is>
+      </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29 QA pass after C29 shipped (qa-policy-build.js + qa-policy-ui.js: 54/54 happy path verified). Honest depth assessment surfaced by Michael's "how confident are you" question — see C29 entry for full QA receipts.</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>Post-COLA. Defensive against MediaLab in head-to-head sales calls.
----</t>
-        </is>
-      </c>
+          <t>task #77 stalled at Gate 3 step 8 on 2026-06-02. PR #500 squash-merged at commit 17a91ff, prod /api/health confirmed ACTIVE on that commit at 20:43 UTC.</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr"/>
     </row>
     <row r="11" ht="90" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>42</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>VeritaQC Import Phase A: human-in-the-loop Gate 3 click-through (deferred)</t>
+          <t>Outbound demo-invite messaging campaign to 1st-degree LinkedIn contacts</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Open, awaiting Michael's 5-minute click test. Will move task #77 to completed only after he reports the user-visible result.
+          <t>Parked. Plan documented. Implementation deferred until trigger conditions met.
 ---</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>XS (~5 minutes of Michael's time on a live URL).</t>
+          <t>L (1 week prep + 4-6 weeks of staged sends)</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>Low. Backend contract is fully verified via 35/35 passing offline contract ch...</t>
+          <t>High. Converts existing warm network (~2,500 1st-degree contacts and growing...</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Effort: XS (~5 minutes of Michael's time on a live URL).
-Importance: Low. Backend contract is fully verified via 35/35 passing offline contract checks (scripts/verify-veritaqc-import.js) plus three live-API smoke checks against prod (candidates, preview, mappings PUT/GET) on Riverside Regional with seed lot SEED-1780436709094 (18 Glucose results). The browser-driven click was not run because Claude-in-Chrome's renderer froze repeatedly on the Radix Select inside VeritaCheckPage, not on Phase A code itself. Risk of a UX bug surviving to a customer is small but not zero.</t>
+          <t>A staged outbound DM campaign walking Michael's 1st-degree LinkedIn contacts through tier-segmented demo invitations for VeritaAssure. Goal: convert warmest contacts into demo conversations first, then chain into trials and paid subscriptions. Separate pipeline from COLA cohort follow-up and from content-driven inbound; all three feed the same demo funnel but originate from different warmth sources.</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>task #77 stalled at Gate 3 step 8 on 2026-06-02. PR #500 squash-merged at commit 17a91ff, prod /api/health confirmed ACTIVE on that commit at 20:43 UTC.</t>
+          <t>2026-06-04 session, after weekly LinkedIn invite batch completion (80 sent, cap hit at #84 Victoria Allen).</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr"/>
@@ -1001,38 +1003,38 @@
     <row r="12" ht="90" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>47</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Outbound demo-invite messaging campaign to 1st-degree LinkedIn contacts</t>
+          <t>Hide sections a lab does not use from a master list, to reduce clutter (prospect-requested)</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Parked. Plan documented. Implementation deferred until trigger conditions met.
----</t>
+          <t>SHIPPED (PR #1364, in origin/main; predates this session, entry was stale). Built as the VeritaDC (VeritaPolicy) Master List "Show only applicable" toggle in client/src/pages/VeritaPolicyAppPage.ts...</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>L (1 week prep + 4-6 weeks of staged sends)</t>
+          <t>S-M (a few days to ~2 weeks depending on scope) — a lab-level visibility togg...</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>High. Converts existing warm network (~2,500 1st-degree contacts and growing...</t>
+          <t>Medium-High — came straight from a live prospect today as an onboarding-frict...</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>A staged outbound DM campaign walking Michael's 1st-degree LinkedIn contacts through tier-segmented demo invitations for VeritaAssure. Goal: convert warmest contacts into demo conversations first, then chain into trials and paid subscriptions. Separate pipeline from COLA cohort follow-up and from content-driven inbound; all three feed the same demo funnel but originate from different warmth sources.</t>
+          <t>Effort: S-M (a few days to ~2 weeks depending on scope) — a lab-level visibility toggle that hides not-applicable or unused sections from a master-list view. Smaller if it is a "hide N/A" filter on the existing VeritaDC master list, larger if it also spans VeritaScan domains.
+Importance: Medium-High — came straight from a live prospect today as an onboarding-friction point; a lab that does not run a service line should not have to wade past its requirements.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04 session, after weekly LinkedIn invite batch completion (80 sent, cap hit at #84 Victoria Allen).</t>
+          <t>2026-09-23 session, Michael relaying a prospect ask from a demo today.</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr"/>
@@ -1040,80 +1042,41 @@
     <row r="13" ht="90" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>53</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Hide sections a lab does not use from a master list, to reduce clutter (prospect-requested)</t>
+          <t>VeritaCEU: curated free-continuing-education provider list (seed / reference)</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>SHIPPED (PR #1364, in origin/main; predates this session, entry was stale). Built as the VeritaDC (VeritaPolicy) Master List "Show only applicable" toggle in client/src/pages/VeritaPolicyAppPage.ts...</t>
+          <t>Open, reference captured. Not started.</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>S-M (a few days to ~2 weeks depending on scope) — a lab-level visibility togg...</t>
+          <t>S (1-2 days to seed a curated provider list and surface it in VeritaCEU; XS t...</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>Medium-High — came straight from a live prospect today as an onboarding-frict...</t>
+          <t>Low-Medium — quality-of-life for VeritaCEU users (find free CE fast); not blo...</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>Effort: S-M (a few days to ~2 weeks depending on scope) — a lab-level visibility toggle that hides not-applicable or unused sections from a master-list view. Smaller if it is a "hide N/A" filter on the existing VeritaDC master list, larger if it also spans VeritaScan domains.
-Importance: Medium-High — came straight from a live prospect today as an onboarding-friction point; a lab that does not run a service line should not have to wade past its requirements.</t>
-        </is>
-      </c>
-      <c r="G13" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-23 session, Michael relaying a prospect ask from a demo today.</t>
-        </is>
-      </c>
-      <c r="H13" s="3" t="inlineStr"/>
-    </row>
-    <row r="14" ht="90" customHeight="1">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>53</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>VeritaCEU: curated free-continuing-education provider list (seed / reference)</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>Open, reference captured. Not started.</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>S (1-2 days to seed a curated provider list and surface it in VeritaCEU; XS t...</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>Low-Medium — quality-of-life for VeritaCEU users (find free CE fast); not blo...</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>Effort: S (1-2 days to seed a curated provider list and surface it in VeritaCEU; XS to just store the reference)
 Importance: Low-Medium — quality-of-life for VeritaCEU users (find free CE fast); not blocking any sale.</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="G13" s="3" t="inlineStr">
         <is>
           <t>Jennifer Small (jennifer.small@lifepointhealth.net) email 2026-09-25, forwarded by Michael 2026-09-28 for the future CEU module.</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="H13" s="3" t="inlineStr">
         <is>
           <t>Post-COLA. No customer urgency.
 ---</t>
@@ -1121,7 +1084,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H14"/>
+  <autoFilter ref="A1:H13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1132,7 +1095,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H52"/>
+  <dimension ref="A1:H53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1190,24 +1153,24 @@
     <row r="2" ht="90" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>C49</t>
+          <t>C52</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Competency "assessed this cycle" cadence-aware window (was #50)</t>
+          <t>VeritaResponse internal NCE / non-conforming event (was #36)</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr"/>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>was S-M / Importance: Medium</t>
+          <t>was L (shipped as MEDIUM) / Importance: High</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Effort: was S-M / Importance: Medium</t>
+          <t>Effort: was L (shipped as MEDIUM) / Importance: High</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
@@ -1216,12 +1179,12 @@
     <row r="3" ht="90" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>C50</t>
+          <t>C49</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>VeritaTrack task owner + owner-only reminder routing (was #51)</t>
+          <t>Competency "assessed this cycle" cadence-aware window (was #50)</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr"/>
@@ -1242,24 +1205,24 @@
     <row r="4" ht="90" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>C51</t>
+          <t>C50</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Designate Medical Director by picking a lab member (was #52, core)</t>
+          <t>VeritaTrack task owner + owner-only reminder routing (was #51)</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr"/>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>was S-M / Importance: Medium-High</t>
+          <t>was S-M / Importance: Medium</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Effort: was S-M / Importance: Medium-High</t>
+          <t>Effort: was S-M / Importance: Medium</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr"/>
@@ -1268,24 +1231,24 @@
     <row r="5" ht="90" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>C47</t>
+          <t>C51</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Unregulated-analyte / Alternative Assessment (AAA) coverage (was #18)</t>
+          <t>Designate Medical Director by picking a lab member (was #52, core)</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr"/>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>was S (Phase 3) / Importance: Medium</t>
+          <t>was S-M / Importance: Medium-High</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Effort: was S (Phase 3) / Importance: Medium</t>
+          <t>Effort: was S-M / Importance: Medium-High</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr"/>
@@ -1294,24 +1257,24 @@
     <row r="6" ht="90" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>C48</t>
+          <t>C47</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>VeritaResponse post-survey deficiency module (was #17)</t>
+          <t>Unregulated-analyte / Alternative Assessment (AAA) coverage (was #18)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr"/>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>was XL / Importance: High</t>
+          <t>was S (Phase 3) / Importance: Medium</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Effort: was XL / Importance: High</t>
+          <t>Effort: was S (Phase 3) / Importance: Medium</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
@@ -1320,39 +1283,38 @@
     <row r="7" ht="90" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>C45</t>
+          <t>C48</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Unify coverage/competency recurrence helper (was #49) - closed as non-issue</t>
+          <t>VeritaResponse post-survey deficiency module (was #17)</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr"/>
-      <c r="D7" s="3" t="inlineStr"/>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>was XL / Importance: High</t>
+        </is>
+      </c>
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: Investigated 2026-09-24 before building. The coverage recurrence math (+6-month interval, signed-resets-to-missing, nextDueOn/overdue, isFailVerdict) is ALREADY single-source in server/veritacheckCoverage.ts (computeCoverageFrom). server/coverageReport.ts and the routes.ts coverage export do not recompute it; they consume the computed nextDueOn/overdue/status fields and apply small surface-specific presentation labels (deliberately different vocabularies per surface, so they should not be merged). The only truly identical duplicate is a one-line date formatter. The competency "owed" derivation is NOT the same cadence: competency follows the CLIA milestone schedule (initial / semiannual year 1 / annual, 42 CFR 493.1451(b)(8) and 493.1235), which is a different regulatory interval from the coverage 6-month rule (493.1281 / 493.1255) and must stay separate. No worthwhile extraction; merging the two cadences would be wrong. Closed 2026-09-24. (The year-1 competency-window refinement remains tracked separately as #50.)</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-24 session, "keep working" pass; scoped read-only, found no real duplication.
----</t>
-        </is>
-      </c>
+          <t>Effort: was XL / Importance: High</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr"/>
       <c r="H7" s="3" t="inlineStr"/>
     </row>
     <row r="8" ht="90" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>C46</t>
+          <t>C45</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Verified-users product-update send path (wrong-list incident fix)</t>
+          <t>Unify coverage/competency recurrence helper (was #49) - closed as non-issue</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr"/>
@@ -1360,12 +1322,12 @@
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: Shipped PR #1324 (merged 4e05506a, deploy ACTIVE). New POST /api/admin/users/send targets registered VeritaAssure account holders (the users table), never the Lab Director's Briefing subscriber list. Separate explicitly-named endpoint (not a flag with a dangerous default), account-holder email framing, excludes suppressed emails and RFC-reserved test domains, CC owner, dryRun + testTo previews. Public unsubscribe now upserts a suppression row so opt-outs are honored across both audiences. Live dryRun: 49 verified-user recipients vs 673 on the Briefing list. Receipts: scripts/verify-product-update-send.mts 24/24, tsc clean, rendered sample inspected. Fixes the fallout from the 2026-09-23/24 wrong-list send (a product update went to the 675-person Briefing list). Nothing sends without Michael's explicit "send it."</t>
+          <t>Closure evidence: Investigated 2026-09-24 before building. The coverage recurrence math (+6-month interval, signed-resets-to-missing, nextDueOn/overdue, isFailVerdict) is ALREADY single-source in server/veritacheckCoverage.ts (computeCoverageFrom). server/coverageReport.ts and the routes.ts coverage export do not recompute it; they consume the computed nextDueOn/overdue/status fields and apply small surface-specific presentation labels (deliberately different vocabularies per surface, so they should not be merged). The only truly identical duplicate is a one-line date formatter. The competency "owed" derivation is NOT the same cadence: competency follows the CLIA milestone schedule (initial / semiannual year 1 / annual, 42 CFR 493.1451(b)(8) and 493.1235), which is a different regulatory interval from the coverage 6-month rule (493.1281 / 493.1255) and must stay separate. No worthwhile extraction; merging the two cadences would be wrong. Closed 2026-09-24. (The year-1 competency-window refinement remains tracked separately as #50.)</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 session; Michael selected this as the next build after the #41 close.
+          <t>2026-09-24 session, "keep working" pass; scoped read-only, found no real duplication.
 ---</t>
         </is>
       </c>
@@ -1374,12 +1336,12 @@
     <row r="9" ht="90" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>C44</t>
+          <t>C46</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Verify-script convention backfill (was #41) + audit matcher fix</t>
+          <t>Verified-users product-update send path (wrong-list incident fix)</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr"/>
@@ -1387,12 +1349,12 @@
       <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: #41 was fully backfilled on 2026-06-13 (all 8 high-stakes scripts landed; see C30); it had only been mis-filed in OPEN. A 2026-09-24 re-audit initially reported 4 of 5 recent math/logic commits as missing a verify script, which was a FALSE POSITIVE: scripts/audit_verify_script_coverage.py matched only scripts/verify-*.js / .cjs, so it ignored the .mjs / .mts / .ts verify scripts the repo now ships (e.g. verify-ptcoag-multi.mts, verify-tea-criterion-format.mjs). Fixed the matcher to accept .js/.cjs/.mjs/.ts/.mts; re-run shows 5 of 5 covered, 0 debt. The convention is being followed. Closed 2026-09-24.</t>
+          <t>Closure evidence: Shipped PR #1324 (merged 4e05506a, deploy ACTIVE). New POST /api/admin/users/send targets registered VeritaAssure account holders (the users table), never the Lab Director's Briefing subscriber list. Separate explicitly-named endpoint (not a flag with a dangerous default), account-holder email framing, excludes suppressed emails and RFC-reserved test domains, CC owner, dryRun + testTo previews. Public unsubscribe now upserts a suppression row so opt-outs are honored across both audiences. Live dryRun: 49 verified-user recipients vs 673 on the Briefing list. Receipts: scripts/verify-product-update-send.mts 24/24, tsc clean, rendered sample inspected. Fixes the fallout from the 2026-09-23/24 wrong-list send (a product update went to the 675-person Briefing list). Nothing sends without Michael's explicit "send it."</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>2026-09-24 session, "keep working" pass; audit tooling bug found + fixed.
+          <t>2026-09-24 session; Michael selected this as the next build after the #41 close.
 ---</t>
         </is>
       </c>
@@ -1401,12 +1363,12 @@
     <row r="10" ht="90" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>C43</t>
+          <t>C44</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>VeritaStaff instrument-centric (dual) assignment view</t>
+          <t>Verify-script convention backfill (was #41) + audit matcher fix</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr"/>
@@ -1414,12 +1376,12 @@
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1320. GET/PUT /staff/instruments/:id/employees (transpose of the per-employee endpoints); an "Assign by Instrument" dialog lets a director pick a test system or manual test and check off who runs it. Same staff_employee_instruments join, with the 42 CFR 493.1235(a) duty-change event emitted on newly-added pairs so both orientations trigger the same reassessment. GET verified live on SCAHC lab 2. Closed 2026-09-24.</t>
+          <t>Closure evidence: #41 was fully backfilled on 2026-06-13 (all 8 high-stakes scripts landed; see C30); it had only been mis-filed in OPEN. A 2026-09-24 re-audit initially reported 4 of 5 recent math/logic commits as missing a verify script, which was a FALSE POSITIVE: scripts/audit_verify_script_coverage.py matched only scripts/verify-*.js / .cjs, so it ignored the .mjs / .mts / .ts verify scripts the repo now ships (e.g. verify-ptcoag-multi.mts, verify-tea-criterion-format.mjs). Fixed the matcher to accept .js/.cjs/.mjs/.ts/.mts; re-run shows 5 of 5 covered, 0 debt. The convention is being followed. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 session, Michael ("in staff we should also give the dual view when assigning coverage to test systems or manual tests").
+          <t>2026-09-24 session, "keep working" pass; audit tooling bug found + fixed.
 ---</t>
         </is>
       </c>
@@ -1428,12 +1390,12 @@
     <row r="11" ht="90" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>C42</t>
+          <t>C43</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>VeritaComp coverage map (required-vs-assessed matrix, dual view)</t>
+          <t>VeritaStaff instrument-centric (dual) assignment view</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr"/>
@@ -1441,12 +1403,12 @@
       <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1319 (+ status layer PR #1316). /competency/owed returns per-item assessed (locked passing assessment this cycle on a covering method group) + per-employee CLIA status; CompetencyCoverageMap renders a By-employee / By-instrument matrix (Assessed / Owed / Overdue / Gap). Verified live on SCAHC lab 2 (owed 116, assessed 2, gaps 0). Completes #48 as the VeritaCheck-parity coverage map. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1320. GET/PUT /staff/instruments/:id/employees (transpose of the per-employee endpoints); an "Assign by Instrument" dialog lets a director pick a test system or manual test and check off who runs it. Same staff_employee_instruments join, with the 42 CFR 493.1235(a) duty-change event emitted on newly-added pairs so both orientations trigger the same reassessment. GET verified live on SCAHC lab 2. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>2026-09-24 session, Michael ("are we building the competencies to have a coverage map, same as veritacheck?" then "build it").
+          <t>2026-09-24 session, Michael ("in staff we should also give the dual view when assigning coverage to test systems or manual tests").
 ---</t>
         </is>
       </c>
@@ -1455,12 +1417,12 @@
     <row r="12" ht="90" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>C41</t>
+          <t>C42</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>VeritaCheck coverage recurrence (method comparison + cal-ver/linearity + reports)</t>
+          <t>VeritaComp coverage map (required-vs-assessed matrix, dual view)</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr"/>
@@ -1468,12 +1430,12 @@
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: PRs #1317 (method comparison), #1318 (cal-ver/linearity), #1321 (report Next-due columns). Periodic verification (correlation/method comparison 42 CFR 493.1281; cal-ver/linearity 42 CFR 493.1255; both 6-month) now recurs: a signed study banks the cycle and rolls to next-due = signed + 6 months instead of reading "done" forever. Status Missing/Failed/Completed-unsigned + a "Next due on" column on-screen and in both coverage exports; also credits the previously-ignored "correlation" study type. Root cause: computeCoverageFrom marked requirements done on mere existence, no date logic. Verified live on SCAHC lab 2 (101 correlations + 11 cal-ver rows now carry a next-due). Engine-level, all facilities. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1319 (+ status layer PR #1316). /competency/owed returns per-item assessed (locked passing assessment this cycle on a covering method group) + per-employee CLIA status; CompetencyCoverageMap renders a By-employee / By-instrument matrix (Assessed / Owed / Overdue / Gap). Verified live on SCAHC lab 2 (owed 116, assessed 2, gaps 0). Completes #48 as the VeritaCheck-parity coverage map. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 session, Michael ("Look at San Carlos... they finished their last set of correlations (all 103) but their menu never reset").
+          <t>2026-09-24 session, Michael ("are we building the competencies to have a coverage map, same as veritacheck?" then "build it").
 ---</t>
         </is>
       </c>
@@ -1482,12 +1444,12 @@
     <row r="13" ht="90" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>C40</t>
+          <t>C41</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>VeritaComp Competencies Owed derived from VeritaStaff, with gap detection (was #48)</t>
+          <t>VeritaCheck coverage recurrence (method comparison + cal-ver/linearity + reports)</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr"/>
@@ -1495,12 +1457,12 @@
       <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1314 (squash 2bcb0db9). GET /api/labs/:labId/competency/owed derives each VeritaStaff testing employee's owed competencies from their assigned instruments (staff_employee_instruments -&gt; veritamap_instruments + tests), on the CLIA timeline, and flags instruments not covered by any competency program as gaps. CompetenciesOwedSection renders it on the VeritaComp landing page. Reuses the shipped bridge + suggested-method-groups match rules; no new tables. Verified live on prod with real assignment data: 2 instruments assigned to a demo staffer produced owed=2, gaps=2 (HIGH, Technical Supervisor), then reverted cleanly. Closed 2026-09-24.</t>
+          <t>Closure evidence: PRs #1317 (method comparison), #1318 (cal-ver/linearity), #1321 (report Next-due columns). Periodic verification (correlation/method comparison 42 CFR 493.1281; cal-ver/linearity 42 CFR 493.1255; both 6-month) now recurs: a signed study banks the cycle and rolls to next-due = signed + 6 months instead of reading "done" forever. Status Missing/Failed/Completed-unsigned + a "Next due on" column on-screen and in both coverage exports; also credits the previously-ignored "correlation" study type. Root cause: computeCoverageFrom marked requirements done on mere existence, no date logic. Verified live on SCAHC lab 2 (101 correlations + 11 cal-ver rows now carry a next-due). Engine-level, all facilities. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>2026-09-23/24 session, Michael ("veritacomp bases what competencies they owe (currently untrue, but needs to be true)"). Option 1 (unify roster on VeritaStaff, match instruments by id).
+          <t>2026-09-24 session, Michael ("Look at San Carlos... they finished their last set of correlations (all 103) but their menu never reset").
 ---</t>
         </is>
       </c>
@@ -1509,12 +1471,12 @@
     <row r="14" ht="90" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>C39</t>
+          <t>C40</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>VeritaScan line items can attach or link evidence (was #46)</t>
+          <t>VeritaComp Competencies Owed derived from VeritaStaff, with gap detection (was #48)</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr"/>
@@ -1522,12 +1484,12 @@
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1312 (squash a1dda93d). VeritaScan scan checklist items now show linked evidence as chips (open link, remove) plus a writer "Link evidence" affordance whose picker links an existing VeritaDC/Library document; a shortcut deep-links to the Library for new (governed) documents. Reuses the already-shipped lab_documents + document_checklist_links + coverage endpoints (URL-pointer only, no file storage, no new tables). Browser-verified live on prod (scan 23): the affordance renders and the picker opens. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1314 (squash 2bcb0db9). GET /api/labs/:labId/competency/owed derives each VeritaStaff testing employee's owed competencies from their assigned instruments (staff_employee_instruments -&gt; veritamap_instruments + tests), on the CLIA timeline, and flags instruments not covered by any competency program as gaps. CompetenciesOwedSection renders it on the VeritaComp landing page. Reuses the shipped bridge + suggested-method-groups match rules; no new tables. Verified live on prod with real assignment data: 2 instruments assigned to a demo staffer produced owed=2, gaps=2 (HIGH, Technical Supervisor), then reverted cleanly. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23 session, Michael. Recurring request. Companion: cross-module evidence display on the VeritaDC policy shipped in PR #1313 (by-target cross-links surfaced in the policy View modal, browser-verified live).
+          <t>2026-09-23/24 session, Michael ("veritacomp bases what competencies they owe (currently untrue, but needs to be true)"). Option 1 (unify roster on VeritaStaff, match instruments by id).
 ---</t>
         </is>
       </c>
@@ -1536,12 +1498,12 @@
     <row r="15" ht="90" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>C38</t>
+          <t>C39</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>VeritaTrack calendar month cells expand to reveal hidden tasks (was #45)</t>
+          <t>VeritaScan line items can attach or link evidence (was #46)</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr"/>
@@ -1549,12 +1511,12 @@
       <c r="E15" s="3" t="inlineStr"/>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: VeritaTrack CalendarView month cells with more than three tasks now expand in place (chevron, "+N more" toggling to "Show less", due dates), so no task is hidden with no path to it (client/src/pages/VeritaTrackAppPage.tsx CalendarView). Shipped 2026-09-23. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1312 (squash a1dda93d). VeritaScan scan checklist items now show linked evidence as chips (open link, remove) plus a writer "Link evidence" affordance whose picker links an existing VeritaDC/Library document; a shortcut deep-links to the Library for new (governed) documents. Reuses the already-shipped lab_documents + document_checklist_links + coverage endpoints (URL-pointer only, no file storage, no new tables). Browser-verified live on prod (scan 23): the affordance renders and the picker opens. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>2026-09-23 session, Michael screenshot of the VeritaTrack calendar (lab 3, September cell).
+          <t>2026-09-23 session, Michael. Recurring request. Companion: cross-module evidence display on the VeritaDC policy shipped in PR #1313 (by-target cross-links surfaced in the policy View modal, browser-verified live).
 ---</t>
         </is>
       </c>
@@ -1563,12 +1525,12 @@
     <row r="16" ht="90" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>C37</t>
+          <t>C38</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Long Excel column headers no longer clip CFR citations (was #44)</t>
+          <t>VeritaTrack calendar month cells expand to reveal hidden tasks (was #45)</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr"/>
@@ -1576,12 +1538,12 @@
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. The VeritaMap export derives the header row height from the longest wrapped header via headerRowHeight(headers, colWidths) (server/routes.ts:15935) instead of a fixed 20, so "Reference Range Attestation (42 CFR 493.1253)" and the other long headers print in full. No new code this session. Closed 2026-09-24.</t>
+          <t>Closure evidence: VeritaTrack CalendarView month cells with more than three tasks now expand in place (chevron, "+N more" toggling to "Show less", due dates), so no task is hidden with no path to it (client/src/pages/VeritaTrackAppPage.tsx CalendarView). Shipped 2026-09-23. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+          <t>2026-09-23 session, Michael screenshot of the VeritaTrack calendar (lab 3, September cell).
 ---</t>
         </is>
       </c>
@@ -1590,12 +1552,12 @@
     <row r="17" ht="90" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>C36</t>
+          <t>C37</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>License stamp no longer clobbers the §6 header/footer or names the wrong lab (was #43)</t>
+          <t>Long Excel column headers no longer clip CFR citations (was #44)</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr"/>
@@ -1603,7 +1565,7 @@
       <c r="E17" s="3" t="inlineStr"/>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. setHeaderFooter (shared/licenseExceljs.ts:155-209) now preserves an existing §6 header and appends (not overwrites) the footer left section, and customer-facing exports name the scoped lab: the VeritaScan library export reads req.scope.lab.name / clia_number (server/routes.ts:16572-16573), not the licensee. No new code this session (avoided regressing the existing fix). Closed 2026-09-24.</t>
+          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. The VeritaMap export derives the header row height from the longest wrapped header via headerRowHeight(headers, colWidths) (server/routes.ts:15935) instead of a fixed 20, so "Reference Range Attestation (42 CFR 493.1253)" and the other long headers print in full. No new code this session. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -1617,18 +1579,45 @@
     <row r="18" ht="90" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>C34</t>
+          <t>C36</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Wire the two static-audit guards into CI (was #43)</t>
+          <t>License stamp no longer clobbers the §6 header/footer or names the wrong lab (was #43)</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr"/>
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. setHeaderFooter (shared/licenseExceljs.ts:155-209) now preserves an existing §6 header and appends (not overwrites) the footer left section, and customer-facing exports name the scoped lab: the VeritaScan library export reads req.scope.lab.name / clia_number (server/routes.ts:16572-16573), not the licensee. No new code this session (avoided regressing the existing fix). Closed 2026-09-24.</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+---</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19" ht="90" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>C34</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Wire the two static-audit guards into CI (was #43)</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr"/>
+      <c r="D19" s="3" t="inlineStr"/>
+      <c r="E19" s="3" t="inlineStr"/>
+      <c r="F19" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: both guards wired into the Multi-Lab Mutations Audit CI
 workflow (.github/workflows/multilab-mutations-audit.yml) as steps:
@@ -1640,24 +1629,24 @@
 (same caveat as the existing guards already in that workflow).</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr"/>
-      <c r="H18" s="2" t="inlineStr"/>
-    </row>
-    <row r="19" ht="90" customHeight="1">
-      <c r="A19" s="3" t="inlineStr">
+      <c r="G19" s="3" t="inlineStr"/>
+      <c r="H19" s="3" t="inlineStr"/>
+    </row>
+    <row r="20" ht="90" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>C35</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>Legacy /api/studies over-returns studies across labs (was #44)</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr"/>
-      <c r="D19" s="3" t="inlineStr"/>
-      <c r="E19" s="3" t="inlineStr"/>
-      <c r="F19" s="3" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr"/>
+      <c r="D20" s="2" t="inlineStr"/>
+      <c r="E20" s="2" t="inlineStr"/>
+      <c r="F20" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: GET /api/studies now scopes its list to the active lab
 when one is resolved from the Referer (server/routes.ts), so every returned row
@@ -1667,24 +1656,24 @@
 mirroring the /api/labs/:labId/studies handler. Closed 2026-06-14.</t>
         </is>
       </c>
-      <c r="G19" s="3" t="inlineStr"/>
-      <c r="H19" s="3" t="inlineStr"/>
-    </row>
-    <row r="20" ht="90" customHeight="1">
-      <c r="A20" s="2" t="inlineStr">
+      <c r="G20" s="2" t="inlineStr"/>
+      <c r="H20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21" ht="90" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>C30</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>Verify-script convention backfill (was #41)</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr"/>
-      <c r="D20" s="2" t="inlineStr"/>
-      <c r="E20" s="2" t="inlineStr"/>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="C21" s="3" t="inlineStr"/>
+      <c r="D21" s="3" t="inlineStr"/>
+      <c r="E21" s="3" t="inlineStr"/>
+      <c r="F21" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: all 8 high-stakes math/logic commits now ship a paired
 scripts/verify-*.js (EP17 sensitivity, Deming lot-to-lot, CUMSUM+QC+multi-analyte,
@@ -1692,30 +1681,30 @@
 TEa boundary), per the strike-throughs in #41. Closed 2026-06-13.</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr">
+      <c r="G21" s="3" t="inlineStr">
         <is>
           <t>scripts/audit_verify_script_coverage.py lookback, 2026-06-02; backfills
 landed 2026-06-03..06.
 ---</t>
         </is>
       </c>
-      <c r="H20" s="2" t="inlineStr"/>
-    </row>
-    <row r="21" ht="90" customHeight="1">
-      <c r="A21" s="3" t="inlineStr">
+      <c r="H21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22" ht="90" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>C31</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B22" s="2" t="inlineStr">
         <is>
           <t>VeritaPT AAA create/update/delete silently no-op in the multi-lab UI</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr"/>
-      <c r="D21" s="3" t="inlineStr"/>
-      <c r="E21" s="3" t="inlineStr"/>
-      <c r="F21" s="3" t="inlineStr">
+      <c r="C22" s="2" t="inlineStr"/>
+      <c r="D22" s="2" t="inlineStr"/>
+      <c r="E22" s="2" t="inlineStr"/>
+      <c r="F22" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #754 (commit 92ad499) added lab-scoped POST/PUT/DELETE
 /api/labs/:labId/pt/aa-records. The UI posted to the lab-scoped path but only GET
@@ -1726,30 +1715,30 @@
 route mis-filed records to the user's default lab on multi-lab accounts).</t>
         </is>
       </c>
-      <c r="G21" s="3" t="inlineStr">
+      <c r="G22" s="2" t="inlineStr">
         <is>
           <t>2026-06-13, found during #18 Phase 3 QA;
 scripts/audit-labscoped-write-routes.mjs now guards the class.
 ---</t>
         </is>
       </c>
-      <c r="H21" s="3" t="inlineStr"/>
-    </row>
-    <row r="22" ht="90" customHeight="1">
-      <c r="A22" s="2" t="inlineStr">
+      <c r="H22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23" ht="90" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>C32</t>
         </is>
       </c>
-      <c r="B22" s="2" t="inlineStr">
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>VeritaComp "Unlock assessment" false-success no-op</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr"/>
-      <c r="D22" s="2" t="inlineStr"/>
-      <c r="E22" s="2" t="inlineStr"/>
-      <c r="F22" s="2" t="inlineStr">
+      <c r="C23" s="3" t="inlineStr"/>
+      <c r="D23" s="3" t="inlineStr"/>
+      <c r="E23" s="3" t="inlineStr"/>
+      <c r="F23" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #755 (commit 4234007) moved the unlock route to
 /api/labs/:labId/competency/assessments/:id/unlock (the path the client calls).
@@ -1760,29 +1749,29 @@
 HTML).</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr">
+      <c r="G23" s="3" t="inlineStr">
         <is>
           <t>2026-06-13, found by scripts/audit-labscoped-write-routes.mjs.
 ---</t>
         </is>
       </c>
-      <c r="H22" s="2" t="inlineStr"/>
-    </row>
-    <row r="23" ht="90" customHeight="1">
-      <c r="A23" s="3" t="inlineStr">
+      <c r="H23" s="3" t="inlineStr"/>
+    </row>
+    <row r="24" ht="90" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>C33</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>FK-cascade delete 500s + NavBar laptop-width overflow</t>
         </is>
       </c>
-      <c r="C23" s="3" t="inlineStr"/>
-      <c r="D23" s="3" t="inlineStr"/>
-      <c r="E23" s="3" t="inlineStr"/>
-      <c r="F23" s="3" t="inlineStr">
+      <c r="C24" s="2" t="inlineStr"/>
+      <c r="D24" s="2" t="inlineStr"/>
+      <c r="E24" s="2" t="inlineStr"/>
+      <c r="F24" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PRs #749/#750 fixed NavBar horizontal overflow at laptop
 widths (collapse to the hamburger below 1560px); prod-verified at 1280-1920 with the
@@ -1793,37 +1782,9 @@
 500 -&gt; 200. scripts/audit-delete-cascades.mjs guards the class.</t>
         </is>
       </c>
-      <c r="G23" s="3" t="inlineStr">
+      <c r="G24" s="2" t="inlineStr">
         <is>
           <t>2026-06-13 browser QA of the A7-D4 wave + retro-QC of the 72h PR window.
----</t>
-        </is>
-      </c>
-      <c r="H23" s="3" t="inlineStr"/>
-    </row>
-    <row r="24" ht="90" customHeight="1">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>C1</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>FAQ "over 25 years" -&gt; "over 23 years"</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr"/>
-      <c r="D24" s="2" t="inlineStr"/>
-      <c r="E24" s="2" t="inlineStr"/>
-      <c r="F24" s="2" t="inlineStr">
-        <is>
-          <t>Closure evidence: client/src/pages/FAQPage.tsx line 20 reads "over
-23 years" as of 2026-05-01.</t>
-        </is>
-      </c>
-      <c r="G24" s="2" t="inlineStr">
-        <is>
-          <t>session 299e9a73 turn 14, ~2026-04-28.
 ---</t>
         </is>
       </c>
@@ -1832,18 +1793,46 @@
     <row r="25" ht="90" customHeight="1">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>C5</t>
+          <t>C1</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>David's VeritaQA grey-button bug (seat permissions mode)</t>
+          <t>FAQ "over 25 years" -&gt; "over 23 years"</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr"/>
       <c r="D25" s="3" t="inlineStr"/>
       <c r="E25" s="3" t="inlineStr"/>
       <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>Closure evidence: client/src/pages/FAQPage.tsx line 20 reads "over
+23 years" as of 2026-05-01.</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>session 299e9a73 turn 14, ~2026-04-28.
+---</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26" ht="90" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>David's VeritaQA grey-button bug (seat permissions mode)</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr"/>
+      <c r="D26" s="2" t="inlineStr"/>
+      <c r="E26" s="2" t="inlineStr"/>
+      <c r="F26" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #10 squash-merged as commit a43fbba on
 2026-05-01 23:19 MST. Railway deploy succeeded; deployed bundle
@@ -1856,7 +1845,7 @@
 against his exact stored shape (14 of 14 expected outcomes matched).</t>
         </is>
       </c>
-      <c r="G25" s="3" t="inlineStr">
+      <c r="G26" s="2" t="inlineStr">
         <is>
           <t>2026-05-01 David's report; veritabench + veritastock
 weren't in MODULE_LIST so seat permissions silently defaulted to
@@ -1864,46 +1853,17 @@
 ---</t>
         </is>
       </c>
-      <c r="H25" s="3" t="inlineStr"/>
-    </row>
-    <row r="26" ht="90" customHeight="1">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>C2</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>TeamPage present-tense "TJC surveyor" check</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr"/>
-      <c r="D26" s="2" t="inlineStr"/>
-      <c r="E26" s="2" t="inlineStr"/>
-      <c r="F26" s="2" t="inlineStr">
-        <is>
-          <t>Closure evidence: site-wide search confirmed all surveyor language
-is past-tense, consistent with user's 2021-2025 service. User closed
-the item in session 299e9a73 turn 4.</t>
-        </is>
-      </c>
-      <c r="G26" s="2" t="inlineStr">
-        <is>
-          <t>session 299e9a73, ~2026-04-28.
----</t>
-        </is>
-      </c>
       <c r="H26" s="2" t="inlineStr"/>
     </row>
     <row r="27" ht="90" customHeight="1">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>C3</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>My Studies CSV/XLSX export (John as design partner)</t>
+          <t>TeamPage present-tense "TJC surveyor" check</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr"/>
@@ -1911,14 +1871,14 @@
       <c r="E27" s="3" t="inlineStr"/>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: client/src/pages/DashboardPage.tsx line 46 calls
-/api/my-studies/export. server/routes.ts line 1491 implements the
-endpoint. Pulled forward into pre-COLA per user instruction.</t>
+          <t>Closure evidence: site-wide search confirmed all surveyor language
+is past-tense, consistent with user's 2021-2025 service. User closed
+the item in session 299e9a73 turn 4.</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>session 299e9a73 turn 5, ~2026-04-28.
+          <t>session 299e9a73, ~2026-04-28.
 ---</t>
         </is>
       </c>
@@ -1927,12 +1887,12 @@
     <row r="28" ht="90" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>C4</t>
+          <t>C3</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Rotate GitHub PAT (because old PAT was committed in SESSION_HANDOFF files)</t>
+          <t>My Studies CSV/XLSX export (John as design partner)</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr"/>
@@ -1940,13 +1900,14 @@
       <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: no ghp_* or github_pat_* patterns in current
-SESSION_HANDOFF.md or SESSION_HANDOFF-2.md as of 2026-05-01.</t>
+          <t>Closure evidence: client/src/pages/DashboardPage.tsx line 46 calls
+/api/my-studies/export. server/routes.ts line 1491 implements the
+endpoint. Pulled forward into pre-COLA per user instruction.</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>session 299e9a73, ~2026-04-28.
+          <t>session 299e9a73 turn 5, ~2026-04-28.
 ---</t>
         </is>
       </c>
@@ -1955,18 +1916,46 @@
     <row r="29" ht="90" customHeight="1">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>C6</t>
+          <t>C4</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>VeritaPolicy service-line filtering removed (formerly #4)</t>
+          <t>Rotate GitHub PAT (because old PAT was committed in SESSION_HANDOFF files)</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr"/>
       <c r="D29" s="3" t="inlineStr"/>
       <c r="E29" s="3" t="inlineStr"/>
       <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>Closure evidence: no ghp_* or github_pat_* patterns in current
+SESSION_HANDOFF.md or SESSION_HANDOFF-2.md as of 2026-05-01.</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>session 299e9a73, ~2026-04-28.
+---</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr"/>
+    </row>
+    <row r="30" ht="90" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>C6</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>VeritaPolicy service-line filtering removed (formerly #4)</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr"/>
+      <c r="D30" s="2" t="inlineStr"/>
+      <c r="E30" s="2" t="inlineStr"/>
+      <c r="F30" s="2" t="inlineStr">
         <is>
           <t>Closure rationale (operator decision 2026-05-10): Keep all
 VeritaPolicy rows. CFR-only references with no accreditor reference
@@ -1975,29 +1964,29 @@
 report misread the design intent.</t>
         </is>
       </c>
-      <c r="G29" s="3" t="inlineStr">
+      <c r="G30" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H29" s="3" t="inlineStr"/>
-    </row>
-    <row r="30" ht="90" customHeight="1">
-      <c r="A30" s="2" t="inlineStr">
+      <c r="H30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31" ht="90" customHeight="1">
+      <c r="A31" s="3" t="inlineStr">
         <is>
           <t>C7</t>
         </is>
       </c>
-      <c r="B30" s="2" t="inlineStr">
+      <c r="B31" s="3" t="inlineStr">
         <is>
           <t>CLIA number format validation (formerly #13)</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr"/>
-      <c r="D30" s="2" t="inlineStr"/>
-      <c r="E30" s="2" t="inlineStr"/>
-      <c r="F30" s="2" t="inlineStr">
+      <c r="C31" s="3" t="inlineStr"/>
+      <c r="D31" s="3" t="inlineStr"/>
+      <c r="E31" s="3" t="inlineStr"/>
+      <c r="F31" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: shared/validateClia.ts defines CLIA_REGEX =
 /^\d{2}D\d{7}$/ (line 24), validateClia() helper with whitespace
@@ -2008,30 +1997,30 @@
 shape exists and behaves as specified.</t>
         </is>
       </c>
-      <c r="G30" s="2" t="inlineStr">
+      <c r="G31" s="3" t="inlineStr">
         <is>
           <t>Agent verification 2026-05-10 via grep + file read.
 Operator confirmed shipped 2026-05-10.
 ---</t>
         </is>
       </c>
-      <c r="H30" s="2" t="inlineStr"/>
-    </row>
-    <row r="31" ht="90" customHeight="1">
-      <c r="A31" s="3" t="inlineStr">
+      <c r="H31" s="3" t="inlineStr"/>
+    </row>
+    <row r="32" ht="90" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t>C8</t>
         </is>
       </c>
-      <c r="B31" s="3" t="inlineStr">
+      <c r="B32" s="2" t="inlineStr">
         <is>
           <t>VeritaMap lab-wide menu toggle (formerly #19)</t>
         </is>
       </c>
-      <c r="C31" s="3" t="inlineStr"/>
-      <c r="D31" s="3" t="inlineStr"/>
-      <c r="E31" s="3" t="inlineStr"/>
-      <c r="F31" s="3" t="inlineStr">
+      <c r="C32" s="2" t="inlineStr"/>
+      <c r="D32" s="2" t="inlineStr"/>
+      <c r="E32" s="2" t="inlineStr"/>
+      <c r="F32" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: client/src/pages/VeritaMapLabwidePage.tsx
 exists and implements the labwide read-only union view. Route is
@@ -2041,59 +2030,59 @@
 parking lot plan (read-only union view, per-session toggle) shipped.</t>
         </is>
       </c>
-      <c r="G31" s="3" t="inlineStr">
+      <c r="G32" s="2" t="inlineStr">
         <is>
           <t>Agent verification 2026-05-10 via grep + file read.
 Operator confirmed shipped 2026-05-10.
 ---</t>
         </is>
       </c>
-      <c r="H31" s="3" t="inlineStr"/>
-    </row>
-    <row r="32" ht="90" customHeight="1">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>C9</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>Tier-1 smoke test checklist (formerly #6)</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr"/>
-      <c r="D32" s="2" t="inlineStr"/>
-      <c r="E32" s="2" t="inlineStr"/>
-      <c r="F32" s="2" t="inlineStr">
-        <is>
-          <t>Closure evidence: docs/smoke-test-tier1.md documents the Tier-1
-smoke-test process and post-deploy verification steps. Shipped via
-PR #81 as part of the 2026-05-10 wave.</t>
-        </is>
-      </c>
-      <c r="G32" s="2" t="inlineStr">
-        <is>
-          <t>Operator instruction 2026-05-10 in this session.
----</t>
-        </is>
-      </c>
       <c r="H32" s="2" t="inlineStr"/>
     </row>
     <row r="33" ht="90" customHeight="1">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>C10</t>
+          <t>C9</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>Per-module gating (formerly #7)</t>
+          <t>Tier-1 smoke test checklist (formerly #6)</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr"/>
       <c r="D33" s="3" t="inlineStr"/>
       <c r="E33" s="3" t="inlineStr"/>
       <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>Closure evidence: docs/smoke-test-tier1.md documents the Tier-1
+smoke-test process and post-deploy verification steps. Shipped via
+PR #81 as part of the 2026-05-10 wave.</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>Operator instruction 2026-05-10 in this session.
+---</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr"/>
+    </row>
+    <row r="34" ht="90" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>C10</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Per-module gating (formerly #7)</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr"/>
+      <c r="D34" s="2" t="inlineStr"/>
+      <c r="E34" s="2" t="inlineStr"/>
+      <c r="F34" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: Client-side useIsReadOnly module keys wired
 on client/src/pages/VeritaPolicyAppPage.tsx and
@@ -2108,29 +2097,29 @@
 PR #76.</t>
         </is>
       </c>
-      <c r="G33" s="3" t="inlineStr">
+      <c r="G34" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H33" s="3" t="inlineStr"/>
-    </row>
-    <row r="34" ht="90" customHeight="1">
-      <c r="A34" s="2" t="inlineStr">
+      <c r="H34" s="2" t="inlineStr"/>
+    </row>
+    <row r="35" ht="90" customHeight="1">
+      <c r="A35" s="3" t="inlineStr">
         <is>
           <t>C11</t>
         </is>
       </c>
-      <c r="B34" s="2" t="inlineStr">
+      <c r="B35" s="3" t="inlineStr">
         <is>
           <t>VeritaStock shipped copy (formerly #8)</t>
         </is>
       </c>
-      <c r="C34" s="2" t="inlineStr"/>
-      <c r="D34" s="2" t="inlineStr"/>
-      <c r="E34" s="2" t="inlineStr"/>
-      <c r="F34" s="2" t="inlineStr">
+      <c r="C35" s="3" t="inlineStr"/>
+      <c r="D35" s="3" t="inlineStr"/>
+      <c r="E35" s="3" t="inlineStr"/>
+      <c r="F35" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: client/src/pages/ArticleInventoryManagementPage.tsx
 line 305 footer reads "platform that includes VeritaStock™" instead
@@ -2138,29 +2127,29 @@
 on /resources/laboratory-inventory-management. Shipped via PR #75.</t>
         </is>
       </c>
-      <c r="G34" s="2" t="inlineStr">
+      <c r="G35" s="3" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H34" s="2" t="inlineStr"/>
-    </row>
-    <row r="35" ht="90" customHeight="1">
-      <c r="A35" s="3" t="inlineStr">
+      <c r="H35" s="3" t="inlineStr"/>
+    </row>
+    <row r="36" ht="90" customHeight="1">
+      <c r="A36" s="2" t="inlineStr">
         <is>
           <t>C12</t>
         </is>
       </c>
-      <c r="B35" s="3" t="inlineStr">
+      <c r="B36" s="2" t="inlineStr">
         <is>
           <t>Admin report one-row-per-lab (formerly #14)</t>
         </is>
       </c>
-      <c r="C35" s="3" t="inlineStr"/>
-      <c r="D35" s="3" t="inlineStr"/>
-      <c r="E35" s="3" t="inlineStr"/>
-      <c r="F35" s="3" t="inlineStr">
+      <c r="C36" s="2" t="inlineStr"/>
+      <c r="D36" s="2" t="inlineStr"/>
+      <c r="E36" s="2" t="inlineStr"/>
+      <c r="F36" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: /api/admin/report rewritten in
 server/routes.ts (~line 595) to LEFT JOIN labs on
@@ -2175,33 +2164,6 @@
 prerequisite, not a code bug). Shipped via PR #85.</t>
         </is>
       </c>
-      <c r="G35" s="3" t="inlineStr">
-        <is>
-          <t>Operator instruction 2026-05-10 in this session.
----</t>
-        </is>
-      </c>
-      <c r="H35" s="3" t="inlineStr"/>
-    </row>
-    <row r="36" ht="90" customHeight="1">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>C14</t>
-        </is>
-      </c>
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t>UI relabel "CLIA TEa" -&gt; "Lab-Set Internal Goal" (formerly #1)</t>
-        </is>
-      </c>
-      <c r="C36" s="2" t="inlineStr"/>
-      <c r="D36" s="2" t="inlineStr"/>
-      <c r="E36" s="2" t="inlineStr"/>
-      <c r="F36" s="2" t="inlineStr">
-        <is>
-          <t>Closure evidence: Shipped across four PRs over 2026-05-10.</t>
-        </is>
-      </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
@@ -2213,18 +2175,45 @@
     <row r="37" ht="90" customHeight="1">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>C13</t>
+          <t>C14</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>WSLH PT vendor (formerly #15)</t>
+          <t>UI relabel "CLIA TEa" -&gt; "Lab-Set Internal Goal" (formerly #1)</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr"/>
       <c r="D37" s="3" t="inlineStr"/>
       <c r="E37" s="3" t="inlineStr"/>
       <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>Closure evidence: Shipped across four PRs over 2026-05-10.</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>Operator instruction 2026-05-10 in this session.
+---</t>
+        </is>
+      </c>
+      <c r="H37" s="3" t="inlineStr"/>
+    </row>
+    <row r="38" ht="90" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>C13</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>WSLH PT vendor (formerly #15)</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr"/>
+      <c r="D38" s="2" t="inlineStr"/>
+      <c r="E38" s="2" t="inlineStr"/>
+      <c r="F38" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: Shipped 2026-05-10 via PR #79 (merge commit
 eeebc6e; merged after rebase to resolve a server/db.ts collision
@@ -2242,38 +2231,9 @@
 'WSLH' is the post-deploy success signal. Shipped via PR #79.</t>
         </is>
       </c>
-      <c r="G37" s="3" t="inlineStr">
+      <c r="G38" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
----</t>
-        </is>
-      </c>
-      <c r="H37" s="3" t="inlineStr"/>
-    </row>
-    <row r="38" ht="90" customHeight="1">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>C15</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>VeritaStock lot tracking + expiration + reorder alerts (formerly #21)</t>
-        </is>
-      </c>
-      <c r="C38" s="2" t="inlineStr"/>
-      <c r="D38" s="2" t="inlineStr"/>
-      <c r="E38" s="2" t="inlineStr"/>
-      <c r="F38" s="2" t="inlineStr">
-        <is>
-          <t>Closure evidence: VeritaStock™ shipped the bench-level inventory
-features the Perplexity competitor analysis identified as a gap:</t>
-        </is>
-      </c>
-      <c r="G38" s="2" t="inlineStr">
-        <is>
-          <t>Originally Perplexity competitor analysis 2026-05-10.
-Audit 2026-05-21 confirmed the feature set ships today.
 ---</t>
         </is>
       </c>
@@ -2282,12 +2242,12 @@
     <row r="39" ht="90" customHeight="1">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>C16</t>
+          <t>C15</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>PAL studies guided workflow (formerly #23)</t>
+          <t>VeritaStock lot tracking + expiration + reorder alerts (formerly #21)</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr"/>
@@ -2295,15 +2255,14 @@
       <c r="E39" s="3" t="inlineStr"/>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: VeritaCheck™ already ships the Precision /
-Accuracy / Linearity (PAL) study set under EP-protocol naming:</t>
+          <t>Closure evidence: VeritaStock™ shipped the bench-level inventory
+features the Perplexity competitor analysis identified as a gap:</t>
         </is>
       </c>
       <c r="G39" s="3" t="inlineStr">
         <is>
           <t>Originally Perplexity competitor analysis 2026-05-10.
-Audit 2026-05-21 confirmed the EP studies cover the PAL framing in
-full.
+Audit 2026-05-21 confirmed the feature set ships today.
 ---</t>
         </is>
       </c>
@@ -2312,12 +2271,12 @@
     <row r="40" ht="90" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>C17</t>
+          <t>C16</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Source-grounded 21/29/45 CFR + 42 CFR 482-485 (formerly #26)</t>
+          <t>PAL studies guided workflow (formerly #23)</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr"/>
@@ -2325,35 +2284,65 @@
       <c r="E40" s="2" t="inlineStr"/>
       <c r="F40" s="2" t="inlineStr">
         <is>
+          <t>Closure evidence: VeritaCheck™ already ships the Precision /
+Accuracy / Linearity (PAL) study set under EP-protocol naming:</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>Originally Perplexity competitor analysis 2026-05-10.
+Audit 2026-05-21 confirmed the EP studies cover the PAL framing in
+full.
+---</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr"/>
+    </row>
+    <row r="41" ht="90" customHeight="1">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>C17</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>Source-grounded 21/29/45 CFR + 42 CFR 482-485 (formerly #26)</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr"/>
+      <c r="D41" s="3" t="inlineStr"/>
+      <c r="E41" s="3" t="inlineStr"/>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
           <t>Closure evidence: PR #301 (commit 8c27806, merged 2026-05-21)
 source-grounded the 74 remaining non-493 entries in
 server/cfrRequirements.ts against verbatim eCFR XML. Breakdown
 shipped:</t>
         </is>
       </c>
-      <c r="G40" s="2" t="inlineStr">
+      <c r="G41" s="3" t="inlineStr">
         <is>
           <t>PR #301; tasks #18 in the in-session task tracker.
 ---</t>
         </is>
       </c>
-      <c r="H40" s="2" t="inlineStr"/>
-    </row>
-    <row r="41" ht="90" customHeight="1">
-      <c r="A41" s="3" t="inlineStr">
+      <c r="H41" s="3" t="inlineStr"/>
+    </row>
+    <row r="42" ht="90" customHeight="1">
+      <c r="A42" s="2" t="inlineStr">
         <is>
           <t>C18</t>
         </is>
       </c>
-      <c r="B41" s="3" t="inlineStr">
+      <c r="B42" s="2" t="inlineStr">
         <is>
           <t>VeritaPolicy "Non CLIA" chapter rename (formerly #3)</t>
         </is>
       </c>
-      <c r="C41" s="3" t="inlineStr"/>
-      <c r="D41" s="3" t="inlineStr"/>
-      <c r="E41" s="3" t="inlineStr"/>
-      <c r="F41" s="3" t="inlineStr">
+      <c r="C42" s="2" t="inlineStr"/>
+      <c r="D42" s="2" t="inlineStr"/>
+      <c r="E42" s="2" t="inlineStr"/>
+      <c r="F42" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #300 (commit 34d7707, merged 2026-05-21)
 renamed all 44 user-facing chapter labels in
@@ -2364,7 +2353,7 @@
 page.</t>
         </is>
       </c>
-      <c r="G41" s="3" t="inlineStr">
+      <c r="G42" s="2" t="inlineStr">
         <is>
           <t>CAP customer screenshot of the /veritapolicy chapter
 headers, 2026-05-01 evening. PR #300; tasks #17 in the in-session
@@ -2372,23 +2361,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H41" s="3" t="inlineStr"/>
-    </row>
-    <row r="42" ht="90" customHeight="1">
-      <c r="A42" s="2" t="inlineStr">
+      <c r="H42" s="2" t="inlineStr"/>
+    </row>
+    <row r="43" ht="90" customHeight="1">
+      <c r="A43" s="3" t="inlineStr">
         <is>
           <t>C19</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
+      <c r="B43" s="3" t="inlineStr">
         <is>
           <t>VeritaStock department-scope toggle (formerly #31)</t>
         </is>
       </c>
-      <c r="C42" s="2" t="inlineStr"/>
-      <c r="D42" s="2" t="inlineStr"/>
-      <c r="E42" s="2" t="inlineStr"/>
-      <c r="F42" s="2" t="inlineStr">
+      <c r="C43" s="3" t="inlineStr"/>
+      <c r="D43" s="3" t="inlineStr"/>
+      <c r="E43" s="3" t="inlineStr"/>
+      <c r="F43" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #319 (commit d01f5fe, merged 2026-05-22)
 shipped the persistent dept-scope toggle on VeritaStockPage. A new
@@ -2399,7 +2388,7 @@
 workspace without re-filtering.</t>
         </is>
       </c>
-      <c r="G42" s="2" t="inlineStr">
+      <c r="G43" s="3" t="inlineStr">
         <is>
           <t>John, San Carlos lab, 2026-05-21. Same conversation that
 drove the vendor dropdown (PR #304), FILTERED VIEW banner (PR #305),
@@ -2407,23 +2396,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H42" s="2" t="inlineStr"/>
-    </row>
-    <row r="43" ht="90" customHeight="1">
-      <c r="A43" s="3" t="inlineStr">
+      <c r="H43" s="3" t="inlineStr"/>
+    </row>
+    <row r="44" ht="90" customHeight="1">
+      <c r="A44" s="2" t="inlineStr">
         <is>
           <t>C20</t>
         </is>
       </c>
-      <c r="B43" s="3" t="inlineStr">
+      <c r="B44" s="2" t="inlineStr">
         <is>
           <t>Primary-lab seat counting (formerly #12)</t>
         </is>
       </c>
-      <c r="C43" s="3" t="inlineStr"/>
-      <c r="D43" s="3" t="inlineStr"/>
-      <c r="E43" s="3" t="inlineStr"/>
-      <c r="F43" s="3" t="inlineStr">
+      <c r="C44" s="2" t="inlineStr"/>
+      <c r="D44" s="2" t="inlineStr"/>
+      <c r="E44" s="2" t="inlineStr"/>
+      <c r="F44" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: is_primary_lab INTEGER NOT NULL DEFAULT 0
 column was added to the lab_members table at db.ts:1276, with the
@@ -2434,7 +2423,7 @@
 is_primary_lab=1 ordering).</t>
         </is>
       </c>
-      <c r="G43" s="3" t="inlineStr">
+      <c r="G44" s="2" t="inlineStr">
         <is>
           <t>2026-05-07 multi-lab discussion. Build shipped as part
 of the Multi-Lab Tier 2 architecture work (Phase 3.x series, prior
@@ -2443,23 +2432,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H43" s="3" t="inlineStr"/>
-    </row>
-    <row r="44" ht="90" customHeight="1">
-      <c r="A44" s="2" t="inlineStr">
+      <c r="H44" s="2" t="inlineStr"/>
+    </row>
+    <row r="45" ht="90" customHeight="1">
+      <c r="A45" s="3" t="inlineStr">
         <is>
           <t>C21</t>
         </is>
       </c>
-      <c r="B44" s="2" t="inlineStr">
+      <c r="B45" s="3" t="inlineStr">
         <is>
           <t>Multi-lab pricing model — Option A (formerly #11)</t>
         </is>
       </c>
-      <c r="C44" s="2" t="inlineStr"/>
-      <c r="D44" s="2" t="inlineStr"/>
-      <c r="E44" s="2" t="inlineStr"/>
-      <c r="F44" s="2" t="inlineStr">
+      <c r="C45" s="3" t="inlineStr"/>
+      <c r="D45" s="3" t="inlineStr"/>
+      <c r="E45" s="3" t="inlineStr"/>
+      <c r="F45" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #322 (commit 0ccd925, merged 2026-05-22)
 added the customer-facing line to the pricing page that reflects
@@ -2472,7 +2461,7 @@
 Enterprise+ block, reads:</t>
         </is>
       </c>
-      <c r="G44" s="2" t="inlineStr">
+      <c r="G45" s="3" t="inlineStr">
         <is>
           <t>2026-05-07 multi-lab discussion (Lisa Veri's
 canonical-case session). PR #322 (initial build); softening PR
@@ -2481,30 +2470,30 @@
 ---</t>
         </is>
       </c>
-      <c r="H44" s="2" t="inlineStr"/>
-    </row>
-    <row r="45" ht="90" customHeight="1">
-      <c r="A45" s="3" t="inlineStr">
+      <c r="H45" s="3" t="inlineStr"/>
+    </row>
+    <row r="46" ht="90" customHeight="1">
+      <c r="A46" s="2" t="inlineStr">
         <is>
           <t>C22</t>
         </is>
       </c>
-      <c r="B45" s="3" t="inlineStr">
+      <c r="B46" s="2" t="inlineStr">
         <is>
           <t>VeritaOps cost-per-test module (formerly #10)</t>
         </is>
       </c>
-      <c r="C45" s="3" t="inlineStr"/>
-      <c r="D45" s="3" t="inlineStr"/>
-      <c r="E45" s="3" t="inlineStr"/>
-      <c r="F45" s="3" t="inlineStr">
+      <c r="C46" s="2" t="inlineStr"/>
+      <c r="D46" s="2" t="inlineStr"/>
+      <c r="E46" s="2" t="inlineStr"/>
+      <c r="F46" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: v1 of the VeritaOps Cost-Per-Reportable-Test
 (CPRT) module shipped across PR #325 through PR #330 on 2026-05-22.
 The module is feature-complete for the typical lab director workflow.</t>
         </is>
       </c>
-      <c r="G45" s="3" t="inlineStr">
+      <c r="G46" s="2" t="inlineStr">
         <is>
           <t>This thread, 2026-05-07 12:05 PM CDT, user message:
 "Parking lot: build an operations module for cost per test
@@ -2513,262 +2502,262 @@
 ---</t>
         </is>
       </c>
-      <c r="H45" s="3" t="inlineStr"/>
-    </row>
-    <row r="46" ht="90" customHeight="1">
-      <c r="A46" s="2" t="inlineStr">
+      <c r="H46" s="2" t="inlineStr"/>
+    </row>
+    <row r="47" ht="90" customHeight="1">
+      <c r="A47" s="3" t="inlineStr">
         <is>
           <t>C23</t>
         </is>
       </c>
-      <c r="B46" s="2" t="inlineStr">
+      <c r="B47" s="3" t="inlineStr">
         <is>
           <t>CCL lab name visual disambiguation in lab switcher (formerly #34)</t>
         </is>
       </c>
-      <c r="C46" s="2" t="inlineStr"/>
-      <c r="D46" s="2" t="inlineStr">
+      <c r="C47" s="3" t="inlineStr"/>
+      <c r="D47" s="3" t="inlineStr">
         <is>
           <t>XS (under 1 day, actual)</t>
         </is>
       </c>
-      <c r="E46" s="2" t="inlineStr">
+      <c r="E47" s="3" t="inlineStr">
         <is>
           <t>Low — cosmetic; only mattered when Lisa or Michael picked the wrong lab from...</t>
         </is>
       </c>
-      <c r="F46" s="2" t="inlineStr">
+      <c r="F47" s="3" t="inlineStr">
         <is>
           <t>Effort: XS (under 1 day, actual)
 Importance: Low — cosmetic; only mattered when Lisa or Michael picked the wrong lab from the dropdown.</t>
         </is>
       </c>
-      <c r="G46" s="2" t="inlineStr">
+      <c r="G47" s="3" t="inlineStr">
         <is>
           <t>flagged 2026-05-23 immediately after provisioning Lisa's CCL lab; closed 2026-05-24.
 ---</t>
         </is>
       </c>
-      <c r="H46" s="2" t="inlineStr"/>
-    </row>
-    <row r="47" ht="90" customHeight="1">
-      <c r="A47" s="3" t="inlineStr">
+      <c r="H47" s="3" t="inlineStr"/>
+    </row>
+    <row r="48" ht="90" customHeight="1">
+      <c r="A48" s="2" t="inlineStr">
         <is>
           <t>C24</t>
         </is>
       </c>
-      <c r="B47" s="3" t="inlineStr">
+      <c r="B48" s="2" t="inlineStr">
         <is>
           <t>VC Unlimited Y1/Y2 price disclosure UX (formerly #35)</t>
         </is>
       </c>
-      <c r="C47" s="3" t="inlineStr"/>
-      <c r="D47" s="3" t="inlineStr">
+      <c r="C48" s="2" t="inlineStr"/>
+      <c r="D48" s="2" t="inlineStr">
         <is>
           <t>XS (under 1 day, actual)</t>
         </is>
       </c>
-      <c r="E47" s="3" t="inlineStr">
+      <c r="E48" s="2" t="inlineStr">
         <is>
           <t>Low when shipped (proactive, no customer complaint yet) — but high if a procu...</t>
         </is>
       </c>
-      <c r="F47" s="3" t="inlineStr">
+      <c r="F48" s="2" t="inlineStr">
         <is>
           <t>Effort: XS (under 1 day, actual)
 Importance: Low when shipped (proactive, no customer complaint yet) — but high if a procurement reviewer later disputes the $499 renewal as undisclosed.</t>
         </is>
       </c>
-      <c r="G47" s="3" t="inlineStr">
+      <c r="G48" s="2" t="inlineStr">
         <is>
           <t>Pricing rebuild 2026-05-23; closed 2026-05-24 proactively before any customer dispute.
 ---</t>
         </is>
       </c>
-      <c r="H47" s="3" t="inlineStr"/>
-    </row>
-    <row r="48" ht="90" customHeight="1">
-      <c r="A48" s="2" t="inlineStr">
+      <c r="H48" s="2" t="inlineStr"/>
+    </row>
+    <row r="49" ht="90" customHeight="1">
+      <c r="A49" s="3" t="inlineStr">
         <is>
           <t>C25</t>
         </is>
       </c>
-      <c r="B48" s="2" t="inlineStr">
+      <c r="B49" s="3" t="inlineStr">
         <is>
           <t>VeritaQC Phase 1 (Levey-Jennings + Westgard live engine) (formerly #20)</t>
         </is>
       </c>
-      <c r="C48" s="2" t="inlineStr"/>
-      <c r="D48" s="2" t="inlineStr">
+      <c r="C49" s="3" t="inlineStr"/>
+      <c r="D49" s="3" t="inlineStr">
         <is>
           <t>L (about 5 days end-to-end, actual: Phase 0 schema → Phase 1A evaluator → 1B...</t>
         </is>
       </c>
-      <c r="E48" s="2" t="inlineStr">
+      <c r="E49" s="3" t="inlineStr">
         <is>
           <t>High — largest single gap vs myLabCompliance.io per Perplexity competitor ana...</t>
         </is>
       </c>
-      <c r="F48" s="2" t="inlineStr">
+      <c r="F49" s="3" t="inlineStr">
         <is>
           <t>Effort: L (about 5 days end-to-end, actual: Phase 0 schema → Phase 1A evaluator → 1B entry UI → 1C daily review → 1D monthly PDF + attestation)
 Importance: High — largest single gap vs myLabCompliance.io per Perplexity competitor analysis; promotes VeritaAssure from documentation tool to lab operations platform.</t>
         </is>
       </c>
-      <c r="G48" s="2" t="inlineStr">
+      <c r="G49" s="3" t="inlineStr">
         <is>
           <t>Perplexity competitor analysis 2026-05-10. Scoping confirmed via the build_phase1_mockup.py iterations 2026-05-24. Shipped 2026-05-25.
 ---</t>
         </is>
       </c>
-      <c r="H48" s="2" t="inlineStr"/>
-    </row>
-    <row r="49" ht="90" customHeight="1">
-      <c r="A49" s="3" t="inlineStr">
+      <c r="H49" s="3" t="inlineStr"/>
+    </row>
+    <row r="50" ht="90" customHeight="1">
+      <c r="A50" s="2" t="inlineStr">
         <is>
           <t>C26</t>
         </is>
       </c>
-      <c r="B49" s="3" t="inlineStr">
+      <c r="B50" s="2" t="inlineStr">
         <is>
           <t>VeritaLab CMS-116 application support + state licensing registry (formerly #22)</t>
         </is>
       </c>
-      <c r="C49" s="3" t="inlineStr"/>
-      <c r="D49" s="3" t="inlineStr">
+      <c r="C50" s="2" t="inlineStr"/>
+      <c r="D50" s="2" t="inlineStr">
         <is>
           <t>M (1-2 weeks for v1, actual)</t>
         </is>
       </c>
-      <c r="E49" s="3" t="inlineStr">
+      <c r="E50" s="2" t="inlineStr">
         <is>
           <t>Medium — competitor parity (myLabCompliance.io) plus useful at lab startup an...</t>
         </is>
       </c>
-      <c r="F49" s="3" t="inlineStr">
+      <c r="F50" s="2" t="inlineStr">
         <is>
           <t>Effort: M (1-2 weeks for v1, actual)
 Importance: Medium — competitor parity (myLabCompliance.io) plus useful at lab startup and at certificate-type changes.</t>
         </is>
       </c>
-      <c r="G49" s="3" t="inlineStr">
+      <c r="G50" s="2" t="inlineStr">
         <is>
           <t>Perplexity competitor analysis (myLabCompliance.io), 2026-05-10. Reclassified as a VeritaLab extension 2026-05-25. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H49" s="3" t="inlineStr"/>
-    </row>
-    <row r="50" ht="90" customHeight="1">
-      <c r="A50" s="2" t="inlineStr">
+      <c r="H50" s="2" t="inlineStr"/>
+    </row>
+    <row r="51" ht="90" customHeight="1">
+      <c r="A51" s="3" t="inlineStr">
         <is>
           <t>C27</t>
         </is>
       </c>
-      <c r="B50" s="2" t="inlineStr">
+      <c r="B51" s="3" t="inlineStr">
         <is>
           <t>Active vs view-only seat split (formerly #33)</t>
         </is>
       </c>
-      <c r="C50" s="2" t="inlineStr"/>
-      <c r="D50" s="2" t="inlineStr">
+      <c r="C51" s="3" t="inlineStr"/>
+      <c r="D51" s="3" t="inlineStr">
         <is>
           <t>M (~1 week of engineering, actual: shipped in a single multi-PR session)</t>
         </is>
       </c>
-      <c r="E50" s="2" t="inlineStr">
+      <c r="E51" s="3" t="inlineStr">
         <is>
           <t>Medium — closed the gap between /pricing copy and product behavior; gives sal...</t>
         </is>
       </c>
-      <c r="F50" s="2" t="inlineStr">
+      <c r="F51" s="3" t="inlineStr">
         <is>
           <t>Effort: M (~1 week of engineering, actual: shipped in a single multi-PR session)
 Importance: Medium — closed the gap between /pricing copy and product behavior; gives sales a clean answer for "do you charge for our medical director?"</t>
         </is>
       </c>
-      <c r="G50" s="2" t="inlineStr">
+      <c r="G51" s="3" t="inlineStr">
         <is>
           <t>Pricing analysis doc Decision 3 (2026-05-21); MEDIUM scenario revised 2026-05-29 to retire the "unlimited view-only" claim. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H50" s="2" t="inlineStr"/>
-    </row>
-    <row r="51" ht="90" customHeight="1">
-      <c r="A51" s="3" t="inlineStr">
+      <c r="H51" s="3" t="inlineStr"/>
+    </row>
+    <row r="52" ht="90" customHeight="1">
+      <c r="A52" s="2" t="inlineStr">
         <is>
           <t>C28</t>
         </is>
       </c>
-      <c r="B51" s="3" t="inlineStr">
+      <c r="B52" s="2" t="inlineStr">
         <is>
           <t>"Why VeritaCheck" comparative one-pager (formerly #37)</t>
         </is>
       </c>
-      <c r="C51" s="3" t="inlineStr"/>
-      <c r="D51" s="3" t="inlineStr">
+      <c r="C52" s="2" t="inlineStr"/>
+      <c r="D52" s="2" t="inlineStr">
         <is>
           <t>S (one design pass + four claim paragraphs + PDF + matching marketing-site pa...</t>
         </is>
       </c>
-      <c r="E51" s="3" t="inlineStr">
+      <c r="E52" s="2" t="inlineStr">
         <is>
           <t>Medium — closed a positioning gap surfaced by six COLA conference attendees a...</t>
         </is>
       </c>
-      <c r="F51" s="3" t="inlineStr">
+      <c r="F52" s="2" t="inlineStr">
         <is>
           <t>Effort: S (one design pass + four claim paragraphs + PDF + matching marketing-site page, actual)
 Importance: Medium — closed a positioning gap surfaced by six COLA conference attendees attached to a legacy verification tool; converts product-quality advantage into a leave-behind Lisa can hand out.</t>
         </is>
       </c>
-      <c r="G51" s="3" t="inlineStr">
+      <c r="G52" s="2" t="inlineStr">
         <is>
           <t>2026-05-11 / 2026-05-12 conference notes review with Michael. Conference attendees (Whitehead, Odegard, Othman, Molinelli, Kyle, Allred) expressed interest in equivalent / superior product. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H51" s="3" t="inlineStr"/>
-    </row>
-    <row r="52" ht="90" customHeight="1">
-      <c r="A52" s="2" t="inlineStr">
+      <c r="H52" s="2" t="inlineStr"/>
+    </row>
+    <row r="53" ht="90" customHeight="1">
+      <c r="A53" s="3" t="inlineStr">
         <is>
           <t>C29</t>
         </is>
       </c>
-      <c r="B52" s="2" t="inlineStr">
+      <c r="B53" s="3" t="inlineStr">
         <is>
           <t>VeritaPolicy approval workflow — MediaLab functional mirror</t>
         </is>
       </c>
-      <c r="C52" s="2" t="inlineStr"/>
-      <c r="D52" s="2" t="inlineStr">
+      <c r="C53" s="3" t="inlineStr"/>
+      <c r="D53" s="3" t="inlineStr">
         <is>
           <t>XL (one focused session, 12 PRs landed)</t>
         </is>
       </c>
-      <c r="E52" s="2" t="inlineStr">
+      <c r="E53" s="3" t="inlineStr">
         <is>
           <t>High — replaces MediaLab Document Control ($752/$2,250 starting price, scalin...</t>
         </is>
       </c>
-      <c r="F52" s="2" t="inlineStr">
+      <c r="F53" s="3" t="inlineStr">
         <is>
           <t>Effort: XL (one focused session, 12 PRs landed)
 Importance: High — replaces MediaLab Document Control ($752/$2,250 starting price, scaling to $10K-$20K/yr at enterprise per Capterra public data) with an included VeritaPolicy feature; closes a real positioning gap and gives sales a direct comparator line.</t>
         </is>
       </c>
-      <c r="G52" s="2" t="inlineStr">
+      <c r="G53" s="3" t="inlineStr">
         <is>
           <t>Pricing strategy conversation 2026-05-29 (Michael: "I don't like bolt-ons; we should replicate this") → scoped 8 phases → shipped all 12 PRs in single session. Shipped 2026-05-29.
 ---</t>
         </is>
       </c>
-      <c r="H52" s="2" t="inlineStr"/>
+      <c r="H53" s="3" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H52"/>
+  <autoFilter ref="A1:H53"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
TASK: Parking lot: add items 54-56 (VeritaTrack quarterly-display bug, VeritaScan custom questions, VeritaQC out-of-2SD entry flag) PLAN:   1. Add OPEN entries 54/55/56 to PARKING_LOT.md in the Effort/Importance format   2. Regenerate PARKING_LOT.xlsx via scripts/build_parking_lot_xlsx.py (OPEN 15 / CLOSED 52 / RETIRED 6)
Self-check:
  - both files committed together so the xlsx mirror does not drift from the markdown
  - each entry carries Effort, Importance, paragraph, Source, Status; inserted before the CLOSED section
  - internal doc only, Gate 3 N/A

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PARKING_LOT.xlsx
+++ b/PARKING_LOT.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RETIRED" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$53</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RETIRED'!$A$1:$H$7</definedName>
   </definedNames>
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1083,8 +1083,140 @@
         </is>
       </c>
     </row>
+    <row r="14" ht="90" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>VeritaTrack: quarterly task loads as monthly until re-saved (frequency display/state bug)</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Open, not started. Needs reproduction in Michael's lab first.</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>S (1-3 days: reproduce, find where the task-create frequency is stored vs ren...</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Medium — data-integrity/UX. A task entered as quarterly that shows as monthly...</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Effort: S (1-3 days: reproduce, find where the task-create frequency is stored vs rendered on the list, fix the load/display path)
+Importance: Medium — data-integrity/UX. A task entered as quarterly that shows as monthly on the tracker until someone re-saves it can drive the wrong due cadence and false "overdue" signals; silent and easy to miss.</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Michael, 2026-10-01 (parking lot).</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Either; small.
+---</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="90" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>VeritaScan: let sites add their own custom questions</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Open, not started. Needs a short design decision on scoring treatment.</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>M (1-2 weeks: a per-lab custom-question model, admin UI to author them, inclu...</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Medium-High — site-requested flexibility and a differentiator; lets a lab ext...</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Effort: M (1-2 weeks: a per-lab custom-question model, admin UI to author them, inclusion in the scan run + scoring/readiness, and export rendering)
+Importance: Medium-High — site-requested flexibility and a differentiator; lets a lab extend the standardized scan with its own internal checks without us hard-coding them.</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>Michael, 2026-10-01 (parking lot).</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>Post-COLA unless a named prospect asks.
+---</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="90" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>VeritaQC: flag/popup when a datapoint is outside +/- 2 SD at entry</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Open, not started.</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>S-M (3 days to ~1.5 weeks: compute mean/SD context at entry, warn when |z| &gt;...</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>High — patient-safety/usability gap. Right now an out-of-2SD control result i...</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Effort: S-M (3 days to ~1.5 weeks: compute mean/SD context at entry, warn when |z| &gt; 2, surface an inline flag + a confirm/acknowledge prompt; reuse the existing LJ/Westgard evaluation)
+Importance: High — patient-safety/usability gap. Right now an out-of-2SD control result is accepted silently; unless the tech scrolls to the Levey-Jennings chart they have no idea it was out, so a real QC excursion can be missed at the moment it matters.</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Michael, 2026-10-01 (parking lot).</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Either; strong quality-of-life + safety win.
+---</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H13"/>
+  <autoFilter ref="A1:H16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
TASK: Parking lot items 54-56 (VeritaTrack freq bug, VeritaScan custom Qs, VeritaQC 2SD flag)
PLAN:
  1. Add OPEN entries 54/55/56 to PARKING_LOT.md
  2. Regenerate PARKING_LOT.xlsx

Self-check:
  - both files committed together; internal doc only (Gate 3 N/A)
</commit_message>
<xml_diff>
--- a/PARKING_LOT.xlsx
+++ b/PARKING_LOT.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RETIRED" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$53</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RETIRED'!$A$1:$H$7</definedName>
   </definedNames>
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1083,8 +1083,140 @@
         </is>
       </c>
     </row>
+    <row r="14" ht="90" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>VeritaTrack: quarterly task loads as monthly until re-saved (frequency display/state bug)</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Open, not started. Needs reproduction in Michael's lab first.</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>S (1-3 days: reproduce, find where the task-create frequency is stored vs ren...</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Medium — data-integrity/UX. A task entered as quarterly that shows as monthly...</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Effort: S (1-3 days: reproduce, find where the task-create frequency is stored vs rendered on the list, fix the load/display path)
+Importance: Medium — data-integrity/UX. A task entered as quarterly that shows as monthly on the tracker until someone re-saves it can drive the wrong due cadence and false "overdue" signals; silent and easy to miss.</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Michael, 2026-10-01 (parking lot).</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Either; small.
+---</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="90" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>VeritaScan: let sites add their own custom questions</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Open, not started. Needs a short design decision on scoring treatment.</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>M (1-2 weeks: a per-lab custom-question model, admin UI to author them, inclu...</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Medium-High — site-requested flexibility and a differentiator; lets a lab ext...</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Effort: M (1-2 weeks: a per-lab custom-question model, admin UI to author them, inclusion in the scan run + scoring/readiness, and export rendering)
+Importance: Medium-High — site-requested flexibility and a differentiator; lets a lab extend the standardized scan with its own internal checks without us hard-coding them.</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>Michael, 2026-10-01 (parking lot).</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>Post-COLA unless a named prospect asks.
+---</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="90" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>VeritaQC: flag/popup when a datapoint is outside +/- 2 SD at entry</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Open, not started.</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>S-M (3 days to ~1.5 weeks: compute mean/SD context at entry, warn when |z| &gt;...</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>High — patient-safety/usability gap. Right now an out-of-2SD control result i...</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Effort: S-M (3 days to ~1.5 weeks: compute mean/SD context at entry, warn when |z| &gt; 2, surface an inline flag + a confirm/acknowledge prompt; reuse the existing LJ/Westgard evaluation)
+Importance: High — patient-safety/usability gap. Right now an out-of-2SD control result is accepted silently; unless the tech scrolls to the Levey-Jennings chart they have no idea it was out, so a real QC excursion can be missed at the moment it matters.</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Michael, 2026-10-01 (parking lot).</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Either; strong quality-of-life + safety win.
+---</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H13"/>
+  <autoFilter ref="A1:H16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
TASK: Close parking-lot #54, #55, #56 (shipped 2026-10-01) and sync the xlsx
PLAN:
  1. Move #54 (VeritaTrack frequency), #56 (VeritaQC at-entry warning), and #55
     (VeritaScan custom questions, 4 phases) from OPEN to CLOSED with PR evidence.
  2. Re-run scripts/build_parking_lot_xlsx.py so the Excel mirror matches.

Self-check:
  - All three are merged to main (PRs #1402, #1403, #1404/#1405/#1406/#1407).
  - xlsx regenerated from the edited md (CLOSED now 55 entries).
  - Internal doc change; Gate 3 N/A.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PARKING_LOT.xlsx
+++ b/PARKING_LOT.xlsx
@@ -12,8 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RETIRED" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$56</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RETIRED'!$A$1:$H$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1083,140 +1083,8 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="90" customHeight="1">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>54</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>VeritaTrack: quarterly task loads as monthly until re-saved (frequency display/state bug)</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>Open, not started. Needs reproduction in Michael's lab first.</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>S (1-3 days: reproduce, find where the task-create frequency is stored vs ren...</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>Medium — data-integrity/UX. A task entered as quarterly that shows as monthly...</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>Effort: S (1-3 days: reproduce, find where the task-create frequency is stored vs rendered on the list, fix the load/display path)
-Importance: Medium — data-integrity/UX. A task entered as quarterly that shows as monthly on the tracker until someone re-saves it can drive the wrong due cadence and false "overdue" signals; silent and easy to miss.</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>Michael, 2026-10-01 (parking lot).</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>Either; small.
----</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="90" customHeight="1">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>55</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>VeritaScan: let sites add their own custom questions</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>Open, not started. Needs a short design decision on scoring treatment.</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>M (1-2 weeks: a per-lab custom-question model, admin UI to author them, inclu...</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="inlineStr">
-        <is>
-          <t>Medium-High — site-requested flexibility and a differentiator; lets a lab ext...</t>
-        </is>
-      </c>
-      <c r="F15" s="3" t="inlineStr">
-        <is>
-          <t>Effort: M (1-2 weeks: a per-lab custom-question model, admin UI to author them, inclusion in the scan run + scoring/readiness, and export rendering)
-Importance: Medium-High — site-requested flexibility and a differentiator; lets a lab extend the standardized scan with its own internal checks without us hard-coding them.</t>
-        </is>
-      </c>
-      <c r="G15" s="3" t="inlineStr">
-        <is>
-          <t>Michael, 2026-10-01 (parking lot).</t>
-        </is>
-      </c>
-      <c r="H15" s="3" t="inlineStr">
-        <is>
-          <t>Post-COLA unless a named prospect asks.
----</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="90" customHeight="1">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>56</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>VeritaQC: flag/popup when a datapoint is outside +/- 2 SD at entry</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Open, not started.</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>S-M (3 days to ~1.5 weeks: compute mean/SD context at entry, warn when |z| &gt;...</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>High — patient-safety/usability gap. Right now an out-of-2SD control result i...</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>Effort: S-M (3 days to ~1.5 weeks: compute mean/SD context at entry, warn when |z| &gt; 2, surface an inline flag + a confirm/acknowledge prompt; reuse the existing LJ/Westgard evaluation)
-Importance: High — patient-safety/usability gap. Right now an out-of-2SD control result is accepted silently; unless the tech scrolls to the Levey-Jennings chart they have no idea it was out, so a real QC excursion can be missed at the moment it matters.</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>Michael, 2026-10-01 (parking lot).</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>Either; strong quality-of-life + safety win.
----</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:H16"/>
+  <autoFilter ref="A1:H13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1227,7 +1095,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H53"/>
+  <dimension ref="A1:H56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1285,24 +1153,24 @@
     <row r="2" ht="90" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>C52</t>
+          <t>C55</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>VeritaResponse internal NCE / non-conforming event (was #36)</t>
+          <t>VeritaScan: let sites add their own custom questions (was #55)</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr"/>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>was L (shipped as MEDIUM) / Importance: High</t>
+          <t>was M / Importance: Medium-High</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Effort: was L (shipped as MEDIUM) / Importance: High</t>
+          <t>Effort: was M / Importance: Medium-High</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
@@ -1311,24 +1179,24 @@
     <row r="3" ht="90" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>C49</t>
+          <t>C54</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Competency "assessed this cycle" cadence-aware window (was #50)</t>
+          <t>VeritaQC: at-entry warning when a QC point is outside 2 SD (was #56)</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr"/>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>was S-M / Importance: Medium</t>
+          <t>was S-M (shipped S) / Importance: High</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Effort: was S-M / Importance: Medium</t>
+          <t>Effort: was S-M (shipped S) / Importance: High</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr"/>
@@ -1337,24 +1205,24 @@
     <row r="4" ht="90" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>C50</t>
+          <t>C53</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>VeritaTrack task owner + owner-only reminder routing (was #51)</t>
+          <t>VeritaTrack: quarterly task loaded as monthly until re-saved (was #54)</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr"/>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>was S-M / Importance: Medium</t>
+          <t>was S / Importance: Medium</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Effort: was S-M / Importance: Medium</t>
+          <t>Effort: was S / Importance: Medium</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr"/>
@@ -1363,24 +1231,24 @@
     <row r="5" ht="90" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>C51</t>
+          <t>C52</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Designate Medical Director by picking a lab member (was #52, core)</t>
+          <t>VeritaResponse internal NCE / non-conforming event (was #36)</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr"/>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>was S-M / Importance: Medium-High</t>
+          <t>was L (shipped as MEDIUM) / Importance: High</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Effort: was S-M / Importance: Medium-High</t>
+          <t>Effort: was L (shipped as MEDIUM) / Importance: High</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr"/>
@@ -1389,24 +1257,24 @@
     <row r="6" ht="90" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>C47</t>
+          <t>C49</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Unregulated-analyte / Alternative Assessment (AAA) coverage (was #18)</t>
+          <t>Competency "assessed this cycle" cadence-aware window (was #50)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr"/>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>was S (Phase 3) / Importance: Medium</t>
+          <t>was S-M / Importance: Medium</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Effort: was S (Phase 3) / Importance: Medium</t>
+          <t>Effort: was S-M / Importance: Medium</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
@@ -1415,24 +1283,24 @@
     <row r="7" ht="90" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>C48</t>
+          <t>C50</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>VeritaResponse post-survey deficiency module (was #17)</t>
+          <t>VeritaTrack task owner + owner-only reminder routing (was #51)</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr"/>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>was XL / Importance: High</t>
+          <t>was S-M / Importance: Medium</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Effort: was XL / Importance: High</t>
+          <t>Effort: was S-M / Importance: Medium</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr"/>
@@ -1441,93 +1309,90 @@
     <row r="8" ht="90" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>C45</t>
+          <t>C51</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Unify coverage/competency recurrence helper (was #49) - closed as non-issue</t>
+          <t>Designate Medical Director by picking a lab member (was #52, core)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr"/>
-      <c r="D8" s="2" t="inlineStr"/>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>was S-M / Importance: Medium-High</t>
+        </is>
+      </c>
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: Investigated 2026-09-24 before building. The coverage recurrence math (+6-month interval, signed-resets-to-missing, nextDueOn/overdue, isFailVerdict) is ALREADY single-source in server/veritacheckCoverage.ts (computeCoverageFrom). server/coverageReport.ts and the routes.ts coverage export do not recompute it; they consume the computed nextDueOn/overdue/status fields and apply small surface-specific presentation labels (deliberately different vocabularies per surface, so they should not be merged). The only truly identical duplicate is a one-line date formatter. The competency "owed" derivation is NOT the same cadence: competency follows the CLIA milestone schedule (initial / semiannual year 1 / annual, 42 CFR 493.1451(b)(8) and 493.1235), which is a different regulatory interval from the coverage 6-month rule (493.1281 / 493.1255) and must stay separate. No worthwhile extraction; merging the two cadences would be wrong. Closed 2026-09-24. (The year-1 competency-window refinement remains tracked separately as #50.)</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-24 session, "keep working" pass; scoped read-only, found no real duplication.
----</t>
-        </is>
-      </c>
+          <t>Effort: was S-M / Importance: Medium-High</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr"/>
       <c r="H8" s="2" t="inlineStr"/>
     </row>
     <row r="9" ht="90" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>C46</t>
+          <t>C47</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Verified-users product-update send path (wrong-list incident fix)</t>
+          <t>Unregulated-analyte / Alternative Assessment (AAA) coverage (was #18)</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr"/>
-      <c r="D9" s="3" t="inlineStr"/>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>was S (Phase 3) / Importance: Medium</t>
+        </is>
+      </c>
       <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: Shipped PR #1324 (merged 4e05506a, deploy ACTIVE). New POST /api/admin/users/send targets registered VeritaAssure account holders (the users table), never the Lab Director's Briefing subscriber list. Separate explicitly-named endpoint (not a flag with a dangerous default), account-holder email framing, excludes suppressed emails and RFC-reserved test domains, CC owner, dryRun + testTo previews. Public unsubscribe now upserts a suppression row so opt-outs are honored across both audiences. Live dryRun: 49 verified-user recipients vs 673 on the Briefing list. Receipts: scripts/verify-product-update-send.mts 24/24, tsc clean, rendered sample inspected. Fixes the fallout from the 2026-09-23/24 wrong-list send (a product update went to the 675-person Briefing list). Nothing sends without Michael's explicit "send it."</t>
-        </is>
-      </c>
-      <c r="G9" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-24 session; Michael selected this as the next build after the #41 close.
----</t>
-        </is>
-      </c>
+          <t>Effort: was S (Phase 3) / Importance: Medium</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr"/>
       <c r="H9" s="3" t="inlineStr"/>
     </row>
     <row r="10" ht="90" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>C44</t>
+          <t>C48</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Verify-script convention backfill (was #41) + audit matcher fix</t>
+          <t>VeritaResponse post-survey deficiency module (was #17)</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr"/>
-      <c r="D10" s="2" t="inlineStr"/>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>was XL / Importance: High</t>
+        </is>
+      </c>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: #41 was fully backfilled on 2026-06-13 (all 8 high-stakes scripts landed; see C30); it had only been mis-filed in OPEN. A 2026-09-24 re-audit initially reported 4 of 5 recent math/logic commits as missing a verify script, which was a FALSE POSITIVE: scripts/audit_verify_script_coverage.py matched only scripts/verify-*.js / .cjs, so it ignored the .mjs / .mts / .ts verify scripts the repo now ships (e.g. verify-ptcoag-multi.mts, verify-tea-criterion-format.mjs). Fixed the matcher to accept .js/.cjs/.mjs/.ts/.mts; re-run shows 5 of 5 covered, 0 debt. The convention is being followed. Closed 2026-09-24.</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-24 session, "keep working" pass; audit tooling bug found + fixed.
----</t>
-        </is>
-      </c>
+          <t>Effort: was XL / Importance: High</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr"/>
       <c r="H10" s="2" t="inlineStr"/>
     </row>
     <row r="11" ht="90" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>C43</t>
+          <t>C45</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>VeritaStaff instrument-centric (dual) assignment view</t>
+          <t>Unify coverage/competency recurrence helper (was #49) - closed as non-issue</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr"/>
@@ -1535,12 +1400,12 @@
       <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1320. GET/PUT /staff/instruments/:id/employees (transpose of the per-employee endpoints); an "Assign by Instrument" dialog lets a director pick a test system or manual test and check off who runs it. Same staff_employee_instruments join, with the 42 CFR 493.1235(a) duty-change event emitted on newly-added pairs so both orientations trigger the same reassessment. GET verified live on SCAHC lab 2. Closed 2026-09-24.</t>
+          <t>Closure evidence: Investigated 2026-09-24 before building. The coverage recurrence math (+6-month interval, signed-resets-to-missing, nextDueOn/overdue, isFailVerdict) is ALREADY single-source in server/veritacheckCoverage.ts (computeCoverageFrom). server/coverageReport.ts and the routes.ts coverage export do not recompute it; they consume the computed nextDueOn/overdue/status fields and apply small surface-specific presentation labels (deliberately different vocabularies per surface, so they should not be merged). The only truly identical duplicate is a one-line date formatter. The competency "owed" derivation is NOT the same cadence: competency follows the CLIA milestone schedule (initial / semiannual year 1 / annual, 42 CFR 493.1451(b)(8) and 493.1235), which is a different regulatory interval from the coverage 6-month rule (493.1281 / 493.1255) and must stay separate. No worthwhile extraction; merging the two cadences would be wrong. Closed 2026-09-24. (The year-1 competency-window refinement remains tracked separately as #50.)</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>2026-09-24 session, Michael ("in staff we should also give the dual view when assigning coverage to test systems or manual tests").
+          <t>2026-09-24 session, "keep working" pass; scoped read-only, found no real duplication.
 ---</t>
         </is>
       </c>
@@ -1549,12 +1414,12 @@
     <row r="12" ht="90" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>C42</t>
+          <t>C46</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>VeritaComp coverage map (required-vs-assessed matrix, dual view)</t>
+          <t>Verified-users product-update send path (wrong-list incident fix)</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr"/>
@@ -1562,12 +1427,12 @@
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1319 (+ status layer PR #1316). /competency/owed returns per-item assessed (locked passing assessment this cycle on a covering method group) + per-employee CLIA status; CompetencyCoverageMap renders a By-employee / By-instrument matrix (Assessed / Owed / Overdue / Gap). Verified live on SCAHC lab 2 (owed 116, assessed 2, gaps 0). Completes #48 as the VeritaCheck-parity coverage map. Closed 2026-09-24.</t>
+          <t>Closure evidence: Shipped PR #1324 (merged 4e05506a, deploy ACTIVE). New POST /api/admin/users/send targets registered VeritaAssure account holders (the users table), never the Lab Director's Briefing subscriber list. Separate explicitly-named endpoint (not a flag with a dangerous default), account-holder email framing, excludes suppressed emails and RFC-reserved test domains, CC owner, dryRun + testTo previews. Public unsubscribe now upserts a suppression row so opt-outs are honored across both audiences. Live dryRun: 49 verified-user recipients vs 673 on the Briefing list. Receipts: scripts/verify-product-update-send.mts 24/24, tsc clean, rendered sample inspected. Fixes the fallout from the 2026-09-23/24 wrong-list send (a product update went to the 675-person Briefing list). Nothing sends without Michael's explicit "send it."</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 session, Michael ("are we building the competencies to have a coverage map, same as veritacheck?" then "build it").
+          <t>2026-09-24 session; Michael selected this as the next build after the #41 close.
 ---</t>
         </is>
       </c>
@@ -1576,12 +1441,12 @@
     <row r="13" ht="90" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>C41</t>
+          <t>C44</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>VeritaCheck coverage recurrence (method comparison + cal-ver/linearity + reports)</t>
+          <t>Verify-script convention backfill (was #41) + audit matcher fix</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr"/>
@@ -1589,12 +1454,12 @@
       <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: PRs #1317 (method comparison), #1318 (cal-ver/linearity), #1321 (report Next-due columns). Periodic verification (correlation/method comparison 42 CFR 493.1281; cal-ver/linearity 42 CFR 493.1255; both 6-month) now recurs: a signed study banks the cycle and rolls to next-due = signed + 6 months instead of reading "done" forever. Status Missing/Failed/Completed-unsigned + a "Next due on" column on-screen and in both coverage exports; also credits the previously-ignored "correlation" study type. Root cause: computeCoverageFrom marked requirements done on mere existence, no date logic. Verified live on SCAHC lab 2 (101 correlations + 11 cal-ver rows now carry a next-due). Engine-level, all facilities. Closed 2026-09-24.</t>
+          <t>Closure evidence: #41 was fully backfilled on 2026-06-13 (all 8 high-stakes scripts landed; see C30); it had only been mis-filed in OPEN. A 2026-09-24 re-audit initially reported 4 of 5 recent math/logic commits as missing a verify script, which was a FALSE POSITIVE: scripts/audit_verify_script_coverage.py matched only scripts/verify-*.js / .cjs, so it ignored the .mjs / .mts / .ts verify scripts the repo now ships (e.g. verify-ptcoag-multi.mts, verify-tea-criterion-format.mjs). Fixed the matcher to accept .js/.cjs/.mjs/.ts/.mts; re-run shows 5 of 5 covered, 0 debt. The convention is being followed. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>2026-09-24 session, Michael ("Look at San Carlos... they finished their last set of correlations (all 103) but their menu never reset").
+          <t>2026-09-24 session, "keep working" pass; audit tooling bug found + fixed.
 ---</t>
         </is>
       </c>
@@ -1603,12 +1468,12 @@
     <row r="14" ht="90" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>C40</t>
+          <t>C43</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>VeritaComp Competencies Owed derived from VeritaStaff, with gap detection (was #48)</t>
+          <t>VeritaStaff instrument-centric (dual) assignment view</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr"/>
@@ -1616,12 +1481,12 @@
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1314 (squash 2bcb0db9). GET /api/labs/:labId/competency/owed derives each VeritaStaff testing employee's owed competencies from their assigned instruments (staff_employee_instruments -&gt; veritamap_instruments + tests), on the CLIA timeline, and flags instruments not covered by any competency program as gaps. CompetenciesOwedSection renders it on the VeritaComp landing page. Reuses the shipped bridge + suggested-method-groups match rules; no new tables. Verified live on prod with real assignment data: 2 instruments assigned to a demo staffer produced owed=2, gaps=2 (HIGH, Technical Supervisor), then reverted cleanly. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1320. GET/PUT /staff/instruments/:id/employees (transpose of the per-employee endpoints); an "Assign by Instrument" dialog lets a director pick a test system or manual test and check off who runs it. Same staff_employee_instruments join, with the 42 CFR 493.1235(a) duty-change event emitted on newly-added pairs so both orientations trigger the same reassessment. GET verified live on SCAHC lab 2. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23/24 session, Michael ("veritacomp bases what competencies they owe (currently untrue, but needs to be true)"). Option 1 (unify roster on VeritaStaff, match instruments by id).
+          <t>2026-09-24 session, Michael ("in staff we should also give the dual view when assigning coverage to test systems or manual tests").
 ---</t>
         </is>
       </c>
@@ -1630,12 +1495,12 @@
     <row r="15" ht="90" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>C39</t>
+          <t>C42</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>VeritaScan line items can attach or link evidence (was #46)</t>
+          <t>VeritaComp coverage map (required-vs-assessed matrix, dual view)</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr"/>
@@ -1643,12 +1508,12 @@
       <c r="E15" s="3" t="inlineStr"/>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1312 (squash a1dda93d). VeritaScan scan checklist items now show linked evidence as chips (open link, remove) plus a writer "Link evidence" affordance whose picker links an existing VeritaDC/Library document; a shortcut deep-links to the Library for new (governed) documents. Reuses the already-shipped lab_documents + document_checklist_links + coverage endpoints (URL-pointer only, no file storage, no new tables). Browser-verified live on prod (scan 23): the affordance renders and the picker opens. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1319 (+ status layer PR #1316). /competency/owed returns per-item assessed (locked passing assessment this cycle on a covering method group) + per-employee CLIA status; CompetencyCoverageMap renders a By-employee / By-instrument matrix (Assessed / Owed / Overdue / Gap). Verified live on SCAHC lab 2 (owed 116, assessed 2, gaps 0). Completes #48 as the VeritaCheck-parity coverage map. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>2026-09-23 session, Michael. Recurring request. Companion: cross-module evidence display on the VeritaDC policy shipped in PR #1313 (by-target cross-links surfaced in the policy View modal, browser-verified live).
+          <t>2026-09-24 session, Michael ("are we building the competencies to have a coverage map, same as veritacheck?" then "build it").
 ---</t>
         </is>
       </c>
@@ -1657,12 +1522,12 @@
     <row r="16" ht="90" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>C38</t>
+          <t>C41</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>VeritaTrack calendar month cells expand to reveal hidden tasks (was #45)</t>
+          <t>VeritaCheck coverage recurrence (method comparison + cal-ver/linearity + reports)</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr"/>
@@ -1670,12 +1535,12 @@
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: VeritaTrack CalendarView month cells with more than three tasks now expand in place (chevron, "+N more" toggling to "Show less", due dates), so no task is hidden with no path to it (client/src/pages/VeritaTrackAppPage.tsx CalendarView). Shipped 2026-09-23. Closed 2026-09-24.</t>
+          <t>Closure evidence: PRs #1317 (method comparison), #1318 (cal-ver/linearity), #1321 (report Next-due columns). Periodic verification (correlation/method comparison 42 CFR 493.1281; cal-ver/linearity 42 CFR 493.1255; both 6-month) now recurs: a signed study banks the cycle and rolls to next-due = signed + 6 months instead of reading "done" forever. Status Missing/Failed/Completed-unsigned + a "Next due on" column on-screen and in both coverage exports; also credits the previously-ignored "correlation" study type. Root cause: computeCoverageFrom marked requirements done on mere existence, no date logic. Verified live on SCAHC lab 2 (101 correlations + 11 cal-ver rows now carry a next-due). Engine-level, all facilities. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23 session, Michael screenshot of the VeritaTrack calendar (lab 3, September cell).
+          <t>2026-09-24 session, Michael ("Look at San Carlos... they finished their last set of correlations (all 103) but their menu never reset").
 ---</t>
         </is>
       </c>
@@ -1684,12 +1549,12 @@
     <row r="17" ht="90" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>C37</t>
+          <t>C40</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Long Excel column headers no longer clip CFR citations (was #44)</t>
+          <t>VeritaComp Competencies Owed derived from VeritaStaff, with gap detection (was #48)</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr"/>
@@ -1697,12 +1562,12 @@
       <c r="E17" s="3" t="inlineStr"/>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. The VeritaMap export derives the header row height from the longest wrapped header via headerRowHeight(headers, colWidths) (server/routes.ts:15935) instead of a fixed 20, so "Reference Range Attestation (42 CFR 493.1253)" and the other long headers print in full. No new code this session. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1314 (squash 2bcb0db9). GET /api/labs/:labId/competency/owed derives each VeritaStaff testing employee's owed competencies from their assigned instruments (staff_employee_instruments -&gt; veritamap_instruments + tests), on the CLIA timeline, and flags instruments not covered by any competency program as gaps. CompetenciesOwedSection renders it on the VeritaComp landing page. Reuses the shipped bridge + suggested-method-groups match rules; no new tables. Verified live on prod with real assignment data: 2 instruments assigned to a demo staffer produced owed=2, gaps=2 (HIGH, Technical Supervisor), then reverted cleanly. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+          <t>2026-09-23/24 session, Michael ("veritacomp bases what competencies they owe (currently untrue, but needs to be true)"). Option 1 (unify roster on VeritaStaff, match instruments by id).
 ---</t>
         </is>
       </c>
@@ -1711,12 +1576,12 @@
     <row r="18" ht="90" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>C36</t>
+          <t>C39</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>License stamp no longer clobbers the §6 header/footer or names the wrong lab (was #43)</t>
+          <t>VeritaScan line items can attach or link evidence (was #46)</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr"/>
@@ -1724,12 +1589,12 @@
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. setHeaderFooter (shared/licenseExceljs.ts:155-209) now preserves an existing §6 header and appends (not overwrites) the footer left section, and customer-facing exports name the scoped lab: the VeritaScan library export reads req.scope.lab.name / clia_number (server/routes.ts:16572-16573), not the licensee. No new code this session (avoided regressing the existing fix). Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1312 (squash a1dda93d). VeritaScan scan checklist items now show linked evidence as chips (open link, remove) plus a writer "Link evidence" affordance whose picker links an existing VeritaDC/Library document; a shortcut deep-links to the Library for new (governed) documents. Reuses the already-shipped lab_documents + document_checklist_links + coverage endpoints (URL-pointer only, no file storage, no new tables). Browser-verified live on prod (scan 23): the affordance renders and the picker opens. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+          <t>2026-09-23 session, Michael. Recurring request. Companion: cross-module evidence display on the VeritaDC policy shipped in PR #1313 (by-target cross-links surfaced in the policy View modal, browser-verified live).
 ---</t>
         </is>
       </c>
@@ -1738,18 +1603,99 @@
     <row r="19" ht="90" customHeight="1">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>C34</t>
+          <t>C38</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Wire the two static-audit guards into CI (was #43)</t>
+          <t>VeritaTrack calendar month cells expand to reveal hidden tasks (was #45)</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr"/>
       <c r="D19" s="3" t="inlineStr"/>
       <c r="E19" s="3" t="inlineStr"/>
       <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Closure evidence: VeritaTrack CalendarView month cells with more than three tasks now expand in place (chevron, "+N more" toggling to "Show less", due dates), so no task is hidden with no path to it (client/src/pages/VeritaTrackAppPage.tsx CalendarView). Shipped 2026-09-23. Closed 2026-09-24.</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-23 session, Michael screenshot of the VeritaTrack calendar (lab 3, September cell).
+---</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr"/>
+    </row>
+    <row r="20" ht="90" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>C37</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Long Excel column headers no longer clip CFR citations (was #44)</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr"/>
+      <c r="D20" s="2" t="inlineStr"/>
+      <c r="E20" s="2" t="inlineStr"/>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. The VeritaMap export derives the header row height from the longest wrapped header via headerRowHeight(headers, colWidths) (server/routes.ts:15935) instead of a fixed 20, so "Reference Range Attestation (42 CFR 493.1253)" and the other long headers print in full. No new code this session. Closed 2026-09-24.</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+---</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21" ht="90" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>C36</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>License stamp no longer clobbers the §6 header/footer or names the wrong lab (was #43)</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr"/>
+      <c r="D21" s="3" t="inlineStr"/>
+      <c r="E21" s="3" t="inlineStr"/>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. setHeaderFooter (shared/licenseExceljs.ts:155-209) now preserves an existing §6 header and appends (not overwrites) the footer left section, and customer-facing exports name the scoped lab: the VeritaScan library export reads req.scope.lab.name / clia_number (server/routes.ts:16572-16573), not the licensee. No new code this session (avoided regressing the existing fix). Closed 2026-09-24.</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+---</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22" ht="90" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>C34</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Wire the two static-audit guards into CI (was #43)</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr"/>
+      <c r="D22" s="2" t="inlineStr"/>
+      <c r="E22" s="2" t="inlineStr"/>
+      <c r="F22" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: both guards wired into the Multi-Lab Mutations Audit CI
 workflow (.github/workflows/multilab-mutations-audit.yml) as steps:
@@ -1761,24 +1707,24 @@
 (same caveat as the existing guards already in that workflow).</t>
         </is>
       </c>
-      <c r="G19" s="3" t="inlineStr"/>
-      <c r="H19" s="3" t="inlineStr"/>
-    </row>
-    <row r="20" ht="90" customHeight="1">
-      <c r="A20" s="2" t="inlineStr">
+      <c r="G22" s="2" t="inlineStr"/>
+      <c r="H22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23" ht="90" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>C35</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>Legacy /api/studies over-returns studies across labs (was #44)</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr"/>
-      <c r="D20" s="2" t="inlineStr"/>
-      <c r="E20" s="2" t="inlineStr"/>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="C23" s="3" t="inlineStr"/>
+      <c r="D23" s="3" t="inlineStr"/>
+      <c r="E23" s="3" t="inlineStr"/>
+      <c r="F23" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: GET /api/studies now scopes its list to the active lab
 when one is resolved from the Referer (server/routes.ts), so every returned row
@@ -1788,24 +1734,24 @@
 mirroring the /api/labs/:labId/studies handler. Closed 2026-06-14.</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr"/>
-      <c r="H20" s="2" t="inlineStr"/>
-    </row>
-    <row r="21" ht="90" customHeight="1">
-      <c r="A21" s="3" t="inlineStr">
+      <c r="G23" s="3" t="inlineStr"/>
+      <c r="H23" s="3" t="inlineStr"/>
+    </row>
+    <row r="24" ht="90" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>C30</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>Verify-script convention backfill (was #41)</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr"/>
-      <c r="D21" s="3" t="inlineStr"/>
-      <c r="E21" s="3" t="inlineStr"/>
-      <c r="F21" s="3" t="inlineStr">
+      <c r="C24" s="2" t="inlineStr"/>
+      <c r="D24" s="2" t="inlineStr"/>
+      <c r="E24" s="2" t="inlineStr"/>
+      <c r="F24" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: all 8 high-stakes math/logic commits now ship a paired
 scripts/verify-*.js (EP17 sensitivity, Deming lot-to-lot, CUMSUM+QC+multi-analyte,
@@ -1813,30 +1759,30 @@
 TEa boundary), per the strike-throughs in #41. Closed 2026-06-13.</t>
         </is>
       </c>
-      <c r="G21" s="3" t="inlineStr">
+      <c r="G24" s="2" t="inlineStr">
         <is>
           <t>scripts/audit_verify_script_coverage.py lookback, 2026-06-02; backfills
 landed 2026-06-03..06.
 ---</t>
         </is>
       </c>
-      <c r="H21" s="3" t="inlineStr"/>
-    </row>
-    <row r="22" ht="90" customHeight="1">
-      <c r="A22" s="2" t="inlineStr">
+      <c r="H24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25" ht="90" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
         <is>
           <t>C31</t>
         </is>
       </c>
-      <c r="B22" s="2" t="inlineStr">
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>VeritaPT AAA create/update/delete silently no-op in the multi-lab UI</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr"/>
-      <c r="D22" s="2" t="inlineStr"/>
-      <c r="E22" s="2" t="inlineStr"/>
-      <c r="F22" s="2" t="inlineStr">
+      <c r="C25" s="3" t="inlineStr"/>
+      <c r="D25" s="3" t="inlineStr"/>
+      <c r="E25" s="3" t="inlineStr"/>
+      <c r="F25" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #754 (commit 92ad499) added lab-scoped POST/PUT/DELETE
 /api/labs/:labId/pt/aa-records. The UI posted to the lab-scoped path but only GET
@@ -1847,30 +1793,30 @@
 route mis-filed records to the user's default lab on multi-lab accounts).</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr">
+      <c r="G25" s="3" t="inlineStr">
         <is>
           <t>2026-06-13, found during #18 Phase 3 QA;
 scripts/audit-labscoped-write-routes.mjs now guards the class.
 ---</t>
         </is>
       </c>
-      <c r="H22" s="2" t="inlineStr"/>
-    </row>
-    <row r="23" ht="90" customHeight="1">
-      <c r="A23" s="3" t="inlineStr">
+      <c r="H25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26" ht="90" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>C32</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t>VeritaComp "Unlock assessment" false-success no-op</t>
         </is>
       </c>
-      <c r="C23" s="3" t="inlineStr"/>
-      <c r="D23" s="3" t="inlineStr"/>
-      <c r="E23" s="3" t="inlineStr"/>
-      <c r="F23" s="3" t="inlineStr">
+      <c r="C26" s="2" t="inlineStr"/>
+      <c r="D26" s="2" t="inlineStr"/>
+      <c r="E26" s="2" t="inlineStr"/>
+      <c r="F26" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #755 (commit 4234007) moved the unlock route to
 /api/labs/:labId/competency/assessments/:id/unlock (the path the client calls).
@@ -1881,29 +1827,29 @@
 HTML).</t>
         </is>
       </c>
-      <c r="G23" s="3" t="inlineStr">
+      <c r="G26" s="2" t="inlineStr">
         <is>
           <t>2026-06-13, found by scripts/audit-labscoped-write-routes.mjs.
 ---</t>
         </is>
       </c>
-      <c r="H23" s="3" t="inlineStr"/>
-    </row>
-    <row r="24" ht="90" customHeight="1">
-      <c r="A24" s="2" t="inlineStr">
+      <c r="H26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27" ht="90" customHeight="1">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>C33</t>
         </is>
       </c>
-      <c r="B24" s="2" t="inlineStr">
+      <c r="B27" s="3" t="inlineStr">
         <is>
           <t>FK-cascade delete 500s + NavBar laptop-width overflow</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr"/>
-      <c r="D24" s="2" t="inlineStr"/>
-      <c r="E24" s="2" t="inlineStr"/>
-      <c r="F24" s="2" t="inlineStr">
+      <c r="C27" s="3" t="inlineStr"/>
+      <c r="D27" s="3" t="inlineStr"/>
+      <c r="E27" s="3" t="inlineStr"/>
+      <c r="F27" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PRs #749/#750 fixed NavBar horizontal overflow at laptop
 widths (collapse to the hamburger below 1560px); prod-verified at 1280-1920 with the
@@ -1914,57 +1860,57 @@
 500 -&gt; 200. scripts/audit-delete-cascades.mjs guards the class.</t>
         </is>
       </c>
-      <c r="G24" s="2" t="inlineStr">
+      <c r="G27" s="3" t="inlineStr">
         <is>
           <t>2026-06-13 browser QA of the A7-D4 wave + retro-QC of the 72h PR window.
 ---</t>
         </is>
       </c>
-      <c r="H24" s="2" t="inlineStr"/>
-    </row>
-    <row r="25" ht="90" customHeight="1">
-      <c r="A25" s="3" t="inlineStr">
+      <c r="H27" s="3" t="inlineStr"/>
+    </row>
+    <row r="28" ht="90" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>C1</t>
         </is>
       </c>
-      <c r="B25" s="3" t="inlineStr">
+      <c r="B28" s="2" t="inlineStr">
         <is>
           <t>FAQ "over 25 years" -&gt; "over 23 years"</t>
         </is>
       </c>
-      <c r="C25" s="3" t="inlineStr"/>
-      <c r="D25" s="3" t="inlineStr"/>
-      <c r="E25" s="3" t="inlineStr"/>
-      <c r="F25" s="3" t="inlineStr">
+      <c r="C28" s="2" t="inlineStr"/>
+      <c r="D28" s="2" t="inlineStr"/>
+      <c r="E28" s="2" t="inlineStr"/>
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: client/src/pages/FAQPage.tsx line 20 reads "over
 23 years" as of 2026-05-01.</t>
         </is>
       </c>
-      <c r="G25" s="3" t="inlineStr">
+      <c r="G28" s="2" t="inlineStr">
         <is>
           <t>session 299e9a73 turn 14, ~2026-04-28.
 ---</t>
         </is>
       </c>
-      <c r="H25" s="3" t="inlineStr"/>
-    </row>
-    <row r="26" ht="90" customHeight="1">
-      <c r="A26" s="2" t="inlineStr">
+      <c r="H28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29" ht="90" customHeight="1">
+      <c r="A29" s="3" t="inlineStr">
         <is>
           <t>C5</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="B29" s="3" t="inlineStr">
         <is>
           <t>David's VeritaQA grey-button bug (seat permissions mode)</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr"/>
-      <c r="D26" s="2" t="inlineStr"/>
-      <c r="E26" s="2" t="inlineStr"/>
-      <c r="F26" s="2" t="inlineStr">
+      <c r="C29" s="3" t="inlineStr"/>
+      <c r="D29" s="3" t="inlineStr"/>
+      <c r="E29" s="3" t="inlineStr"/>
+      <c r="F29" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #10 squash-merged as commit a43fbba on
 2026-05-01 23:19 MST. Railway deploy succeeded; deployed bundle
@@ -1977,7 +1923,7 @@
 against his exact stored shape (14 of 14 expected outcomes matched).</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr">
+      <c r="G29" s="3" t="inlineStr">
         <is>
           <t>2026-05-01 David's report; veritabench + veritastock
 weren't in MODULE_LIST so seat permissions silently defaulted to
@@ -1985,109 +1931,109 @@
 ---</t>
         </is>
       </c>
-      <c r="H26" s="2" t="inlineStr"/>
-    </row>
-    <row r="27" ht="90" customHeight="1">
-      <c r="A27" s="3" t="inlineStr">
-        <is>
-          <t>C2</t>
-        </is>
-      </c>
-      <c r="B27" s="3" t="inlineStr">
-        <is>
-          <t>TeamPage present-tense "TJC surveyor" check</t>
-        </is>
-      </c>
-      <c r="C27" s="3" t="inlineStr"/>
-      <c r="D27" s="3" t="inlineStr"/>
-      <c r="E27" s="3" t="inlineStr"/>
-      <c r="F27" s="3" t="inlineStr">
-        <is>
-          <t>Closure evidence: site-wide search confirmed all surveyor language
-is past-tense, consistent with user's 2021-2025 service. User closed
-the item in session 299e9a73 turn 4.</t>
-        </is>
-      </c>
-      <c r="G27" s="3" t="inlineStr">
-        <is>
-          <t>session 299e9a73, ~2026-04-28.
----</t>
-        </is>
-      </c>
-      <c r="H27" s="3" t="inlineStr"/>
-    </row>
-    <row r="28" ht="90" customHeight="1">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>C3</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>My Studies CSV/XLSX export (John as design partner)</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="inlineStr"/>
-      <c r="D28" s="2" t="inlineStr"/>
-      <c r="E28" s="2" t="inlineStr"/>
-      <c r="F28" s="2" t="inlineStr">
-        <is>
-          <t>Closure evidence: client/src/pages/DashboardPage.tsx line 46 calls
-/api/my-studies/export. server/routes.ts line 1491 implements the
-endpoint. Pulled forward into pre-COLA per user instruction.</t>
-        </is>
-      </c>
-      <c r="G28" s="2" t="inlineStr">
-        <is>
-          <t>session 299e9a73 turn 5, ~2026-04-28.
----</t>
-        </is>
-      </c>
-      <c r="H28" s="2" t="inlineStr"/>
-    </row>
-    <row r="29" ht="90" customHeight="1">
-      <c r="A29" s="3" t="inlineStr">
-        <is>
-          <t>C4</t>
-        </is>
-      </c>
-      <c r="B29" s="3" t="inlineStr">
-        <is>
-          <t>Rotate GitHub PAT (because old PAT was committed in SESSION_HANDOFF files)</t>
-        </is>
-      </c>
-      <c r="C29" s="3" t="inlineStr"/>
-      <c r="D29" s="3" t="inlineStr"/>
-      <c r="E29" s="3" t="inlineStr"/>
-      <c r="F29" s="3" t="inlineStr">
-        <is>
-          <t>Closure evidence: no ghp_* or github_pat_* patterns in current
-SESSION_HANDOFF.md or SESSION_HANDOFF-2.md as of 2026-05-01.</t>
-        </is>
-      </c>
-      <c r="G29" s="3" t="inlineStr">
-        <is>
-          <t>session 299e9a73, ~2026-04-28.
----</t>
-        </is>
-      </c>
       <c r="H29" s="3" t="inlineStr"/>
     </row>
     <row r="30" ht="90" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>C6</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>VeritaPolicy service-line filtering removed (formerly #4)</t>
+          <t>TeamPage present-tense "TJC surveyor" check</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr"/>
       <c r="D30" s="2" t="inlineStr"/>
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Closure evidence: site-wide search confirmed all surveyor language
+is past-tense, consistent with user's 2021-2025 service. User closed
+the item in session 299e9a73 turn 4.</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>session 299e9a73, ~2026-04-28.
+---</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31" ht="90" customHeight="1">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>C3</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>My Studies CSV/XLSX export (John as design partner)</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr"/>
+      <c r="D31" s="3" t="inlineStr"/>
+      <c r="E31" s="3" t="inlineStr"/>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>Closure evidence: client/src/pages/DashboardPage.tsx line 46 calls
+/api/my-studies/export. server/routes.ts line 1491 implements the
+endpoint. Pulled forward into pre-COLA per user instruction.</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>session 299e9a73 turn 5, ~2026-04-28.
+---</t>
+        </is>
+      </c>
+      <c r="H31" s="3" t="inlineStr"/>
+    </row>
+    <row r="32" ht="90" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Rotate GitHub PAT (because old PAT was committed in SESSION_HANDOFF files)</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr"/>
+      <c r="D32" s="2" t="inlineStr"/>
+      <c r="E32" s="2" t="inlineStr"/>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Closure evidence: no ghp_* or github_pat_* patterns in current
+SESSION_HANDOFF.md or SESSION_HANDOFF-2.md as of 2026-05-01.</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>session 299e9a73, ~2026-04-28.
+---</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33" ht="90" customHeight="1">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>C6</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>VeritaPolicy service-line filtering removed (formerly #4)</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr"/>
+      <c r="D33" s="3" t="inlineStr"/>
+      <c r="E33" s="3" t="inlineStr"/>
+      <c r="F33" s="3" t="inlineStr">
         <is>
           <t>Closure rationale (operator decision 2026-05-10): Keep all
 VeritaPolicy rows. CFR-only references with no accreditor reference
@@ -2096,29 +2042,29 @@
 report misread the design intent.</t>
         </is>
       </c>
-      <c r="G30" s="2" t="inlineStr">
+      <c r="G33" s="3" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H30" s="2" t="inlineStr"/>
-    </row>
-    <row r="31" ht="90" customHeight="1">
-      <c r="A31" s="3" t="inlineStr">
+      <c r="H33" s="3" t="inlineStr"/>
+    </row>
+    <row r="34" ht="90" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
         <is>
           <t>C7</t>
         </is>
       </c>
-      <c r="B31" s="3" t="inlineStr">
+      <c r="B34" s="2" t="inlineStr">
         <is>
           <t>CLIA number format validation (formerly #13)</t>
         </is>
       </c>
-      <c r="C31" s="3" t="inlineStr"/>
-      <c r="D31" s="3" t="inlineStr"/>
-      <c r="E31" s="3" t="inlineStr"/>
-      <c r="F31" s="3" t="inlineStr">
+      <c r="C34" s="2" t="inlineStr"/>
+      <c r="D34" s="2" t="inlineStr"/>
+      <c r="E34" s="2" t="inlineStr"/>
+      <c r="F34" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: shared/validateClia.ts defines CLIA_REGEX =
 /^\d{2}D\d{7}$/ (line 24), validateClia() helper with whitespace
@@ -2129,30 +2075,30 @@
 shape exists and behaves as specified.</t>
         </is>
       </c>
-      <c r="G31" s="3" t="inlineStr">
+      <c r="G34" s="2" t="inlineStr">
         <is>
           <t>Agent verification 2026-05-10 via grep + file read.
 Operator confirmed shipped 2026-05-10.
 ---</t>
         </is>
       </c>
-      <c r="H31" s="3" t="inlineStr"/>
-    </row>
-    <row r="32" ht="90" customHeight="1">
-      <c r="A32" s="2" t="inlineStr">
+      <c r="H34" s="2" t="inlineStr"/>
+    </row>
+    <row r="35" ht="90" customHeight="1">
+      <c r="A35" s="3" t="inlineStr">
         <is>
           <t>C8</t>
         </is>
       </c>
-      <c r="B32" s="2" t="inlineStr">
+      <c r="B35" s="3" t="inlineStr">
         <is>
           <t>VeritaMap lab-wide menu toggle (formerly #19)</t>
         </is>
       </c>
-      <c r="C32" s="2" t="inlineStr"/>
-      <c r="D32" s="2" t="inlineStr"/>
-      <c r="E32" s="2" t="inlineStr"/>
-      <c r="F32" s="2" t="inlineStr">
+      <c r="C35" s="3" t="inlineStr"/>
+      <c r="D35" s="3" t="inlineStr"/>
+      <c r="E35" s="3" t="inlineStr"/>
+      <c r="F35" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: client/src/pages/VeritaMapLabwidePage.tsx
 exists and implements the labwide read-only union view. Route is
@@ -2162,59 +2108,59 @@
 parking lot plan (read-only union view, per-session toggle) shipped.</t>
         </is>
       </c>
-      <c r="G32" s="2" t="inlineStr">
+      <c r="G35" s="3" t="inlineStr">
         <is>
           <t>Agent verification 2026-05-10 via grep + file read.
 Operator confirmed shipped 2026-05-10.
 ---</t>
         </is>
       </c>
-      <c r="H32" s="2" t="inlineStr"/>
-    </row>
-    <row r="33" ht="90" customHeight="1">
-      <c r="A33" s="3" t="inlineStr">
+      <c r="H35" s="3" t="inlineStr"/>
+    </row>
+    <row r="36" ht="90" customHeight="1">
+      <c r="A36" s="2" t="inlineStr">
         <is>
           <t>C9</t>
         </is>
       </c>
-      <c r="B33" s="3" t="inlineStr">
+      <c r="B36" s="2" t="inlineStr">
         <is>
           <t>Tier-1 smoke test checklist (formerly #6)</t>
         </is>
       </c>
-      <c r="C33" s="3" t="inlineStr"/>
-      <c r="D33" s="3" t="inlineStr"/>
-      <c r="E33" s="3" t="inlineStr"/>
-      <c r="F33" s="3" t="inlineStr">
+      <c r="C36" s="2" t="inlineStr"/>
+      <c r="D36" s="2" t="inlineStr"/>
+      <c r="E36" s="2" t="inlineStr"/>
+      <c r="F36" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: docs/smoke-test-tier1.md documents the Tier-1
 smoke-test process and post-deploy verification steps. Shipped via
 PR #81 as part of the 2026-05-10 wave.</t>
         </is>
       </c>
-      <c r="G33" s="3" t="inlineStr">
+      <c r="G36" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H33" s="3" t="inlineStr"/>
-    </row>
-    <row r="34" ht="90" customHeight="1">
-      <c r="A34" s="2" t="inlineStr">
+      <c r="H36" s="2" t="inlineStr"/>
+    </row>
+    <row r="37" ht="90" customHeight="1">
+      <c r="A37" s="3" t="inlineStr">
         <is>
           <t>C10</t>
         </is>
       </c>
-      <c r="B34" s="2" t="inlineStr">
+      <c r="B37" s="3" t="inlineStr">
         <is>
           <t>Per-module gating (formerly #7)</t>
         </is>
       </c>
-      <c r="C34" s="2" t="inlineStr"/>
-      <c r="D34" s="2" t="inlineStr"/>
-      <c r="E34" s="2" t="inlineStr"/>
-      <c r="F34" s="2" t="inlineStr">
+      <c r="C37" s="3" t="inlineStr"/>
+      <c r="D37" s="3" t="inlineStr"/>
+      <c r="E37" s="3" t="inlineStr"/>
+      <c r="F37" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: Client-side useIsReadOnly module keys wired
 on client/src/pages/VeritaPolicyAppPage.tsx and
@@ -2229,29 +2175,29 @@
 PR #76.</t>
         </is>
       </c>
-      <c r="G34" s="2" t="inlineStr">
+      <c r="G37" s="3" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H34" s="2" t="inlineStr"/>
-    </row>
-    <row r="35" ht="90" customHeight="1">
-      <c r="A35" s="3" t="inlineStr">
+      <c r="H37" s="3" t="inlineStr"/>
+    </row>
+    <row r="38" ht="90" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
         <is>
           <t>C11</t>
         </is>
       </c>
-      <c r="B35" s="3" t="inlineStr">
+      <c r="B38" s="2" t="inlineStr">
         <is>
           <t>VeritaStock shipped copy (formerly #8)</t>
         </is>
       </c>
-      <c r="C35" s="3" t="inlineStr"/>
-      <c r="D35" s="3" t="inlineStr"/>
-      <c r="E35" s="3" t="inlineStr"/>
-      <c r="F35" s="3" t="inlineStr">
+      <c r="C38" s="2" t="inlineStr"/>
+      <c r="D38" s="2" t="inlineStr"/>
+      <c r="E38" s="2" t="inlineStr"/>
+      <c r="F38" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: client/src/pages/ArticleInventoryManagementPage.tsx
 line 305 footer reads "platform that includes VeritaStock™" instead
@@ -2259,29 +2205,29 @@
 on /resources/laboratory-inventory-management. Shipped via PR #75.</t>
         </is>
       </c>
-      <c r="G35" s="3" t="inlineStr">
+      <c r="G38" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H35" s="3" t="inlineStr"/>
-    </row>
-    <row r="36" ht="90" customHeight="1">
-      <c r="A36" s="2" t="inlineStr">
+      <c r="H38" s="2" t="inlineStr"/>
+    </row>
+    <row r="39" ht="90" customHeight="1">
+      <c r="A39" s="3" t="inlineStr">
         <is>
           <t>C12</t>
         </is>
       </c>
-      <c r="B36" s="2" t="inlineStr">
+      <c r="B39" s="3" t="inlineStr">
         <is>
           <t>Admin report one-row-per-lab (formerly #14)</t>
         </is>
       </c>
-      <c r="C36" s="2" t="inlineStr"/>
-      <c r="D36" s="2" t="inlineStr"/>
-      <c r="E36" s="2" t="inlineStr"/>
-      <c r="F36" s="2" t="inlineStr">
+      <c r="C39" s="3" t="inlineStr"/>
+      <c r="D39" s="3" t="inlineStr"/>
+      <c r="E39" s="3" t="inlineStr"/>
+      <c r="F39" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: /api/admin/report rewritten in
 server/routes.ts (~line 595) to LEFT JOIN labs on
@@ -2296,56 +2242,56 @@
 prerequisite, not a code bug). Shipped via PR #85.</t>
         </is>
       </c>
-      <c r="G36" s="2" t="inlineStr">
+      <c r="G39" s="3" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H36" s="2" t="inlineStr"/>
-    </row>
-    <row r="37" ht="90" customHeight="1">
-      <c r="A37" s="3" t="inlineStr">
+      <c r="H39" s="3" t="inlineStr"/>
+    </row>
+    <row r="40" ht="90" customHeight="1">
+      <c r="A40" s="2" t="inlineStr">
         <is>
           <t>C14</t>
         </is>
       </c>
-      <c r="B37" s="3" t="inlineStr">
+      <c r="B40" s="2" t="inlineStr">
         <is>
           <t>UI relabel "CLIA TEa" -&gt; "Lab-Set Internal Goal" (formerly #1)</t>
         </is>
       </c>
-      <c r="C37" s="3" t="inlineStr"/>
-      <c r="D37" s="3" t="inlineStr"/>
-      <c r="E37" s="3" t="inlineStr"/>
-      <c r="F37" s="3" t="inlineStr">
+      <c r="C40" s="2" t="inlineStr"/>
+      <c r="D40" s="2" t="inlineStr"/>
+      <c r="E40" s="2" t="inlineStr"/>
+      <c r="F40" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: Shipped across four PRs over 2026-05-10.</t>
         </is>
       </c>
-      <c r="G37" s="3" t="inlineStr">
+      <c r="G40" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H37" s="3" t="inlineStr"/>
-    </row>
-    <row r="38" ht="90" customHeight="1">
-      <c r="A38" s="2" t="inlineStr">
+      <c r="H40" s="2" t="inlineStr"/>
+    </row>
+    <row r="41" ht="90" customHeight="1">
+      <c r="A41" s="3" t="inlineStr">
         <is>
           <t>C13</t>
         </is>
       </c>
-      <c r="B38" s="2" t="inlineStr">
+      <c r="B41" s="3" t="inlineStr">
         <is>
           <t>WSLH PT vendor (formerly #15)</t>
         </is>
       </c>
-      <c r="C38" s="2" t="inlineStr"/>
-      <c r="D38" s="2" t="inlineStr"/>
-      <c r="E38" s="2" t="inlineStr"/>
-      <c r="F38" s="2" t="inlineStr">
+      <c r="C41" s="3" t="inlineStr"/>
+      <c r="D41" s="3" t="inlineStr"/>
+      <c r="E41" s="3" t="inlineStr"/>
+      <c r="F41" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: Shipped 2026-05-10 via PR #79 (merge commit
 eeebc6e; merged after rebase to resolve a server/db.ts collision
@@ -2363,64 +2309,64 @@
 'WSLH' is the post-deploy success signal. Shipped via PR #79.</t>
         </is>
       </c>
-      <c r="G38" s="2" t="inlineStr">
+      <c r="G41" s="3" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H38" s="2" t="inlineStr"/>
-    </row>
-    <row r="39" ht="90" customHeight="1">
-      <c r="A39" s="3" t="inlineStr">
+      <c r="H41" s="3" t="inlineStr"/>
+    </row>
+    <row r="42" ht="90" customHeight="1">
+      <c r="A42" s="2" t="inlineStr">
         <is>
           <t>C15</t>
         </is>
       </c>
-      <c r="B39" s="3" t="inlineStr">
+      <c r="B42" s="2" t="inlineStr">
         <is>
           <t>VeritaStock lot tracking + expiration + reorder alerts (formerly #21)</t>
         </is>
       </c>
-      <c r="C39" s="3" t="inlineStr"/>
-      <c r="D39" s="3" t="inlineStr"/>
-      <c r="E39" s="3" t="inlineStr"/>
-      <c r="F39" s="3" t="inlineStr">
+      <c r="C42" s="2" t="inlineStr"/>
+      <c r="D42" s="2" t="inlineStr"/>
+      <c r="E42" s="2" t="inlineStr"/>
+      <c r="F42" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: VeritaStock™ shipped the bench-level inventory
 features the Perplexity competitor analysis identified as a gap:</t>
         </is>
       </c>
-      <c r="G39" s="3" t="inlineStr">
+      <c r="G42" s="2" t="inlineStr">
         <is>
           <t>Originally Perplexity competitor analysis 2026-05-10.
 Audit 2026-05-21 confirmed the feature set ships today.
 ---</t>
         </is>
       </c>
-      <c r="H39" s="3" t="inlineStr"/>
-    </row>
-    <row r="40" ht="90" customHeight="1">
-      <c r="A40" s="2" t="inlineStr">
+      <c r="H42" s="2" t="inlineStr"/>
+    </row>
+    <row r="43" ht="90" customHeight="1">
+      <c r="A43" s="3" t="inlineStr">
         <is>
           <t>C16</t>
         </is>
       </c>
-      <c r="B40" s="2" t="inlineStr">
+      <c r="B43" s="3" t="inlineStr">
         <is>
           <t>PAL studies guided workflow (formerly #23)</t>
         </is>
       </c>
-      <c r="C40" s="2" t="inlineStr"/>
-      <c r="D40" s="2" t="inlineStr"/>
-      <c r="E40" s="2" t="inlineStr"/>
-      <c r="F40" s="2" t="inlineStr">
+      <c r="C43" s="3" t="inlineStr"/>
+      <c r="D43" s="3" t="inlineStr"/>
+      <c r="E43" s="3" t="inlineStr"/>
+      <c r="F43" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: VeritaCheck™ already ships the Precision /
 Accuracy / Linearity (PAL) study set under EP-protocol naming:</t>
         </is>
       </c>
-      <c r="G40" s="2" t="inlineStr">
+      <c r="G43" s="3" t="inlineStr">
         <is>
           <t>Originally Perplexity competitor analysis 2026-05-10.
 Audit 2026-05-21 confirmed the EP studies cover the PAL framing in
@@ -2428,23 +2374,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H40" s="2" t="inlineStr"/>
-    </row>
-    <row r="41" ht="90" customHeight="1">
-      <c r="A41" s="3" t="inlineStr">
+      <c r="H43" s="3" t="inlineStr"/>
+    </row>
+    <row r="44" ht="90" customHeight="1">
+      <c r="A44" s="2" t="inlineStr">
         <is>
           <t>C17</t>
         </is>
       </c>
-      <c r="B41" s="3" t="inlineStr">
+      <c r="B44" s="2" t="inlineStr">
         <is>
           <t>Source-grounded 21/29/45 CFR + 42 CFR 482-485 (formerly #26)</t>
         </is>
       </c>
-      <c r="C41" s="3" t="inlineStr"/>
-      <c r="D41" s="3" t="inlineStr"/>
-      <c r="E41" s="3" t="inlineStr"/>
-      <c r="F41" s="3" t="inlineStr">
+      <c r="C44" s="2" t="inlineStr"/>
+      <c r="D44" s="2" t="inlineStr"/>
+      <c r="E44" s="2" t="inlineStr"/>
+      <c r="F44" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #301 (commit 8c27806, merged 2026-05-21)
 source-grounded the 74 remaining non-493 entries in
@@ -2452,29 +2398,29 @@
 shipped:</t>
         </is>
       </c>
-      <c r="G41" s="3" t="inlineStr">
+      <c r="G44" s="2" t="inlineStr">
         <is>
           <t>PR #301; tasks #18 in the in-session task tracker.
 ---</t>
         </is>
       </c>
-      <c r="H41" s="3" t="inlineStr"/>
-    </row>
-    <row r="42" ht="90" customHeight="1">
-      <c r="A42" s="2" t="inlineStr">
+      <c r="H44" s="2" t="inlineStr"/>
+    </row>
+    <row r="45" ht="90" customHeight="1">
+      <c r="A45" s="3" t="inlineStr">
         <is>
           <t>C18</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
+      <c r="B45" s="3" t="inlineStr">
         <is>
           <t>VeritaPolicy "Non CLIA" chapter rename (formerly #3)</t>
         </is>
       </c>
-      <c r="C42" s="2" t="inlineStr"/>
-      <c r="D42" s="2" t="inlineStr"/>
-      <c r="E42" s="2" t="inlineStr"/>
-      <c r="F42" s="2" t="inlineStr">
+      <c r="C45" s="3" t="inlineStr"/>
+      <c r="D45" s="3" t="inlineStr"/>
+      <c r="E45" s="3" t="inlineStr"/>
+      <c r="F45" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #300 (commit 34d7707, merged 2026-05-21)
 renamed all 44 user-facing chapter labels in
@@ -2485,7 +2431,7 @@
 page.</t>
         </is>
       </c>
-      <c r="G42" s="2" t="inlineStr">
+      <c r="G45" s="3" t="inlineStr">
         <is>
           <t>CAP customer screenshot of the /veritapolicy chapter
 headers, 2026-05-01 evening. PR #300; tasks #17 in the in-session
@@ -2493,23 +2439,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H42" s="2" t="inlineStr"/>
-    </row>
-    <row r="43" ht="90" customHeight="1">
-      <c r="A43" s="3" t="inlineStr">
+      <c r="H45" s="3" t="inlineStr"/>
+    </row>
+    <row r="46" ht="90" customHeight="1">
+      <c r="A46" s="2" t="inlineStr">
         <is>
           <t>C19</t>
         </is>
       </c>
-      <c r="B43" s="3" t="inlineStr">
+      <c r="B46" s="2" t="inlineStr">
         <is>
           <t>VeritaStock department-scope toggle (formerly #31)</t>
         </is>
       </c>
-      <c r="C43" s="3" t="inlineStr"/>
-      <c r="D43" s="3" t="inlineStr"/>
-      <c r="E43" s="3" t="inlineStr"/>
-      <c r="F43" s="3" t="inlineStr">
+      <c r="C46" s="2" t="inlineStr"/>
+      <c r="D46" s="2" t="inlineStr"/>
+      <c r="E46" s="2" t="inlineStr"/>
+      <c r="F46" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #319 (commit d01f5fe, merged 2026-05-22)
 shipped the persistent dept-scope toggle on VeritaStockPage. A new
@@ -2520,7 +2466,7 @@
 workspace without re-filtering.</t>
         </is>
       </c>
-      <c r="G43" s="3" t="inlineStr">
+      <c r="G46" s="2" t="inlineStr">
         <is>
           <t>John, San Carlos lab, 2026-05-21. Same conversation that
 drove the vendor dropdown (PR #304), FILTERED VIEW banner (PR #305),
@@ -2528,23 +2474,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H43" s="3" t="inlineStr"/>
-    </row>
-    <row r="44" ht="90" customHeight="1">
-      <c r="A44" s="2" t="inlineStr">
+      <c r="H46" s="2" t="inlineStr"/>
+    </row>
+    <row r="47" ht="90" customHeight="1">
+      <c r="A47" s="3" t="inlineStr">
         <is>
           <t>C20</t>
         </is>
       </c>
-      <c r="B44" s="2" t="inlineStr">
+      <c r="B47" s="3" t="inlineStr">
         <is>
           <t>Primary-lab seat counting (formerly #12)</t>
         </is>
       </c>
-      <c r="C44" s="2" t="inlineStr"/>
-      <c r="D44" s="2" t="inlineStr"/>
-      <c r="E44" s="2" t="inlineStr"/>
-      <c r="F44" s="2" t="inlineStr">
+      <c r="C47" s="3" t="inlineStr"/>
+      <c r="D47" s="3" t="inlineStr"/>
+      <c r="E47" s="3" t="inlineStr"/>
+      <c r="F47" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: is_primary_lab INTEGER NOT NULL DEFAULT 0
 column was added to the lab_members table at db.ts:1276, with the
@@ -2555,7 +2501,7 @@
 is_primary_lab=1 ordering).</t>
         </is>
       </c>
-      <c r="G44" s="2" t="inlineStr">
+      <c r="G47" s="3" t="inlineStr">
         <is>
           <t>2026-05-07 multi-lab discussion. Build shipped as part
 of the Multi-Lab Tier 2 architecture work (Phase 3.x series, prior
@@ -2564,23 +2510,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H44" s="2" t="inlineStr"/>
-    </row>
-    <row r="45" ht="90" customHeight="1">
-      <c r="A45" s="3" t="inlineStr">
+      <c r="H47" s="3" t="inlineStr"/>
+    </row>
+    <row r="48" ht="90" customHeight="1">
+      <c r="A48" s="2" t="inlineStr">
         <is>
           <t>C21</t>
         </is>
       </c>
-      <c r="B45" s="3" t="inlineStr">
+      <c r="B48" s="2" t="inlineStr">
         <is>
           <t>Multi-lab pricing model — Option A (formerly #11)</t>
         </is>
       </c>
-      <c r="C45" s="3" t="inlineStr"/>
-      <c r="D45" s="3" t="inlineStr"/>
-      <c r="E45" s="3" t="inlineStr"/>
-      <c r="F45" s="3" t="inlineStr">
+      <c r="C48" s="2" t="inlineStr"/>
+      <c r="D48" s="2" t="inlineStr"/>
+      <c r="E48" s="2" t="inlineStr"/>
+      <c r="F48" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #322 (commit 0ccd925, merged 2026-05-22)
 added the customer-facing line to the pricing page that reflects
@@ -2593,7 +2539,7 @@
 Enterprise+ block, reads:</t>
         </is>
       </c>
-      <c r="G45" s="3" t="inlineStr">
+      <c r="G48" s="2" t="inlineStr">
         <is>
           <t>2026-05-07 multi-lab discussion (Lisa Veri's
 canonical-case session). PR #322 (initial build); softening PR
@@ -2602,30 +2548,30 @@
 ---</t>
         </is>
       </c>
-      <c r="H45" s="3" t="inlineStr"/>
-    </row>
-    <row r="46" ht="90" customHeight="1">
-      <c r="A46" s="2" t="inlineStr">
+      <c r="H48" s="2" t="inlineStr"/>
+    </row>
+    <row r="49" ht="90" customHeight="1">
+      <c r="A49" s="3" t="inlineStr">
         <is>
           <t>C22</t>
         </is>
       </c>
-      <c r="B46" s="2" t="inlineStr">
+      <c r="B49" s="3" t="inlineStr">
         <is>
           <t>VeritaOps cost-per-test module (formerly #10)</t>
         </is>
       </c>
-      <c r="C46" s="2" t="inlineStr"/>
-      <c r="D46" s="2" t="inlineStr"/>
-      <c r="E46" s="2" t="inlineStr"/>
-      <c r="F46" s="2" t="inlineStr">
+      <c r="C49" s="3" t="inlineStr"/>
+      <c r="D49" s="3" t="inlineStr"/>
+      <c r="E49" s="3" t="inlineStr"/>
+      <c r="F49" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: v1 of the VeritaOps Cost-Per-Reportable-Test
 (CPRT) module shipped across PR #325 through PR #330 on 2026-05-22.
 The module is feature-complete for the typical lab director workflow.</t>
         </is>
       </c>
-      <c r="G46" s="2" t="inlineStr">
+      <c r="G49" s="3" t="inlineStr">
         <is>
           <t>This thread, 2026-05-07 12:05 PM CDT, user message:
 "Parking lot: build an operations module for cost per test
@@ -2634,262 +2580,262 @@
 ---</t>
         </is>
       </c>
-      <c r="H46" s="2" t="inlineStr"/>
-    </row>
-    <row r="47" ht="90" customHeight="1">
-      <c r="A47" s="3" t="inlineStr">
+      <c r="H49" s="3" t="inlineStr"/>
+    </row>
+    <row r="50" ht="90" customHeight="1">
+      <c r="A50" s="2" t="inlineStr">
         <is>
           <t>C23</t>
         </is>
       </c>
-      <c r="B47" s="3" t="inlineStr">
+      <c r="B50" s="2" t="inlineStr">
         <is>
           <t>CCL lab name visual disambiguation in lab switcher (formerly #34)</t>
         </is>
       </c>
-      <c r="C47" s="3" t="inlineStr"/>
-      <c r="D47" s="3" t="inlineStr">
+      <c r="C50" s="2" t="inlineStr"/>
+      <c r="D50" s="2" t="inlineStr">
         <is>
           <t>XS (under 1 day, actual)</t>
         </is>
       </c>
-      <c r="E47" s="3" t="inlineStr">
+      <c r="E50" s="2" t="inlineStr">
         <is>
           <t>Low — cosmetic; only mattered when Lisa or Michael picked the wrong lab from...</t>
         </is>
       </c>
-      <c r="F47" s="3" t="inlineStr">
+      <c r="F50" s="2" t="inlineStr">
         <is>
           <t>Effort: XS (under 1 day, actual)
 Importance: Low — cosmetic; only mattered when Lisa or Michael picked the wrong lab from the dropdown.</t>
         </is>
       </c>
-      <c r="G47" s="3" t="inlineStr">
+      <c r="G50" s="2" t="inlineStr">
         <is>
           <t>flagged 2026-05-23 immediately after provisioning Lisa's CCL lab; closed 2026-05-24.
 ---</t>
         </is>
       </c>
-      <c r="H47" s="3" t="inlineStr"/>
-    </row>
-    <row r="48" ht="90" customHeight="1">
-      <c r="A48" s="2" t="inlineStr">
+      <c r="H50" s="2" t="inlineStr"/>
+    </row>
+    <row r="51" ht="90" customHeight="1">
+      <c r="A51" s="3" t="inlineStr">
         <is>
           <t>C24</t>
         </is>
       </c>
-      <c r="B48" s="2" t="inlineStr">
+      <c r="B51" s="3" t="inlineStr">
         <is>
           <t>VC Unlimited Y1/Y2 price disclosure UX (formerly #35)</t>
         </is>
       </c>
-      <c r="C48" s="2" t="inlineStr"/>
-      <c r="D48" s="2" t="inlineStr">
+      <c r="C51" s="3" t="inlineStr"/>
+      <c r="D51" s="3" t="inlineStr">
         <is>
           <t>XS (under 1 day, actual)</t>
         </is>
       </c>
-      <c r="E48" s="2" t="inlineStr">
+      <c r="E51" s="3" t="inlineStr">
         <is>
           <t>Low when shipped (proactive, no customer complaint yet) — but high if a procu...</t>
         </is>
       </c>
-      <c r="F48" s="2" t="inlineStr">
+      <c r="F51" s="3" t="inlineStr">
         <is>
           <t>Effort: XS (under 1 day, actual)
 Importance: Low when shipped (proactive, no customer complaint yet) — but high if a procurement reviewer later disputes the $499 renewal as undisclosed.</t>
         </is>
       </c>
-      <c r="G48" s="2" t="inlineStr">
+      <c r="G51" s="3" t="inlineStr">
         <is>
           <t>Pricing rebuild 2026-05-23; closed 2026-05-24 proactively before any customer dispute.
 ---</t>
         </is>
       </c>
-      <c r="H48" s="2" t="inlineStr"/>
-    </row>
-    <row r="49" ht="90" customHeight="1">
-      <c r="A49" s="3" t="inlineStr">
+      <c r="H51" s="3" t="inlineStr"/>
+    </row>
+    <row r="52" ht="90" customHeight="1">
+      <c r="A52" s="2" t="inlineStr">
         <is>
           <t>C25</t>
         </is>
       </c>
-      <c r="B49" s="3" t="inlineStr">
+      <c r="B52" s="2" t="inlineStr">
         <is>
           <t>VeritaQC Phase 1 (Levey-Jennings + Westgard live engine) (formerly #20)</t>
         </is>
       </c>
-      <c r="C49" s="3" t="inlineStr"/>
-      <c r="D49" s="3" t="inlineStr">
+      <c r="C52" s="2" t="inlineStr"/>
+      <c r="D52" s="2" t="inlineStr">
         <is>
           <t>L (about 5 days end-to-end, actual: Phase 0 schema → Phase 1A evaluator → 1B...</t>
         </is>
       </c>
-      <c r="E49" s="3" t="inlineStr">
+      <c r="E52" s="2" t="inlineStr">
         <is>
           <t>High — largest single gap vs myLabCompliance.io per Perplexity competitor ana...</t>
         </is>
       </c>
-      <c r="F49" s="3" t="inlineStr">
+      <c r="F52" s="2" t="inlineStr">
         <is>
           <t>Effort: L (about 5 days end-to-end, actual: Phase 0 schema → Phase 1A evaluator → 1B entry UI → 1C daily review → 1D monthly PDF + attestation)
 Importance: High — largest single gap vs myLabCompliance.io per Perplexity competitor analysis; promotes VeritaAssure from documentation tool to lab operations platform.</t>
         </is>
       </c>
-      <c r="G49" s="3" t="inlineStr">
+      <c r="G52" s="2" t="inlineStr">
         <is>
           <t>Perplexity competitor analysis 2026-05-10. Scoping confirmed via the build_phase1_mockup.py iterations 2026-05-24. Shipped 2026-05-25.
 ---</t>
         </is>
       </c>
-      <c r="H49" s="3" t="inlineStr"/>
-    </row>
-    <row r="50" ht="90" customHeight="1">
-      <c r="A50" s="2" t="inlineStr">
+      <c r="H52" s="2" t="inlineStr"/>
+    </row>
+    <row r="53" ht="90" customHeight="1">
+      <c r="A53" s="3" t="inlineStr">
         <is>
           <t>C26</t>
         </is>
       </c>
-      <c r="B50" s="2" t="inlineStr">
+      <c r="B53" s="3" t="inlineStr">
         <is>
           <t>VeritaLab CMS-116 application support + state licensing registry (formerly #22)</t>
         </is>
       </c>
-      <c r="C50" s="2" t="inlineStr"/>
-      <c r="D50" s="2" t="inlineStr">
+      <c r="C53" s="3" t="inlineStr"/>
+      <c r="D53" s="3" t="inlineStr">
         <is>
           <t>M (1-2 weeks for v1, actual)</t>
         </is>
       </c>
-      <c r="E50" s="2" t="inlineStr">
+      <c r="E53" s="3" t="inlineStr">
         <is>
           <t>Medium — competitor parity (myLabCompliance.io) plus useful at lab startup an...</t>
         </is>
       </c>
-      <c r="F50" s="2" t="inlineStr">
+      <c r="F53" s="3" t="inlineStr">
         <is>
           <t>Effort: M (1-2 weeks for v1, actual)
 Importance: Medium — competitor parity (myLabCompliance.io) plus useful at lab startup and at certificate-type changes.</t>
         </is>
       </c>
-      <c r="G50" s="2" t="inlineStr">
+      <c r="G53" s="3" t="inlineStr">
         <is>
           <t>Perplexity competitor analysis (myLabCompliance.io), 2026-05-10. Reclassified as a VeritaLab extension 2026-05-25. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H50" s="2" t="inlineStr"/>
-    </row>
-    <row r="51" ht="90" customHeight="1">
-      <c r="A51" s="3" t="inlineStr">
+      <c r="H53" s="3" t="inlineStr"/>
+    </row>
+    <row r="54" ht="90" customHeight="1">
+      <c r="A54" s="2" t="inlineStr">
         <is>
           <t>C27</t>
         </is>
       </c>
-      <c r="B51" s="3" t="inlineStr">
+      <c r="B54" s="2" t="inlineStr">
         <is>
           <t>Active vs view-only seat split (formerly #33)</t>
         </is>
       </c>
-      <c r="C51" s="3" t="inlineStr"/>
-      <c r="D51" s="3" t="inlineStr">
+      <c r="C54" s="2" t="inlineStr"/>
+      <c r="D54" s="2" t="inlineStr">
         <is>
           <t>M (~1 week of engineering, actual: shipped in a single multi-PR session)</t>
         </is>
       </c>
-      <c r="E51" s="3" t="inlineStr">
+      <c r="E54" s="2" t="inlineStr">
         <is>
           <t>Medium — closed the gap between /pricing copy and product behavior; gives sal...</t>
         </is>
       </c>
-      <c r="F51" s="3" t="inlineStr">
+      <c r="F54" s="2" t="inlineStr">
         <is>
           <t>Effort: M (~1 week of engineering, actual: shipped in a single multi-PR session)
 Importance: Medium — closed the gap between /pricing copy and product behavior; gives sales a clean answer for "do you charge for our medical director?"</t>
         </is>
       </c>
-      <c r="G51" s="3" t="inlineStr">
+      <c r="G54" s="2" t="inlineStr">
         <is>
           <t>Pricing analysis doc Decision 3 (2026-05-21); MEDIUM scenario revised 2026-05-29 to retire the "unlimited view-only" claim. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H51" s="3" t="inlineStr"/>
-    </row>
-    <row r="52" ht="90" customHeight="1">
-      <c r="A52" s="2" t="inlineStr">
+      <c r="H54" s="2" t="inlineStr"/>
+    </row>
+    <row r="55" ht="90" customHeight="1">
+      <c r="A55" s="3" t="inlineStr">
         <is>
           <t>C28</t>
         </is>
       </c>
-      <c r="B52" s="2" t="inlineStr">
+      <c r="B55" s="3" t="inlineStr">
         <is>
           <t>"Why VeritaCheck" comparative one-pager (formerly #37)</t>
         </is>
       </c>
-      <c r="C52" s="2" t="inlineStr"/>
-      <c r="D52" s="2" t="inlineStr">
+      <c r="C55" s="3" t="inlineStr"/>
+      <c r="D55" s="3" t="inlineStr">
         <is>
           <t>S (one design pass + four claim paragraphs + PDF + matching marketing-site pa...</t>
         </is>
       </c>
-      <c r="E52" s="2" t="inlineStr">
+      <c r="E55" s="3" t="inlineStr">
         <is>
           <t>Medium — closed a positioning gap surfaced by six COLA conference attendees a...</t>
         </is>
       </c>
-      <c r="F52" s="2" t="inlineStr">
+      <c r="F55" s="3" t="inlineStr">
         <is>
           <t>Effort: S (one design pass + four claim paragraphs + PDF + matching marketing-site page, actual)
 Importance: Medium — closed a positioning gap surfaced by six COLA conference attendees attached to a legacy verification tool; converts product-quality advantage into a leave-behind Lisa can hand out.</t>
         </is>
       </c>
-      <c r="G52" s="2" t="inlineStr">
+      <c r="G55" s="3" t="inlineStr">
         <is>
           <t>2026-05-11 / 2026-05-12 conference notes review with Michael. Conference attendees (Whitehead, Odegard, Othman, Molinelli, Kyle, Allred) expressed interest in equivalent / superior product. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H52" s="2" t="inlineStr"/>
-    </row>
-    <row r="53" ht="90" customHeight="1">
-      <c r="A53" s="3" t="inlineStr">
+      <c r="H55" s="3" t="inlineStr"/>
+    </row>
+    <row r="56" ht="90" customHeight="1">
+      <c r="A56" s="2" t="inlineStr">
         <is>
           <t>C29</t>
         </is>
       </c>
-      <c r="B53" s="3" t="inlineStr">
+      <c r="B56" s="2" t="inlineStr">
         <is>
           <t>VeritaPolicy approval workflow — MediaLab functional mirror</t>
         </is>
       </c>
-      <c r="C53" s="3" t="inlineStr"/>
-      <c r="D53" s="3" t="inlineStr">
+      <c r="C56" s="2" t="inlineStr"/>
+      <c r="D56" s="2" t="inlineStr">
         <is>
           <t>XL (one focused session, 12 PRs landed)</t>
         </is>
       </c>
-      <c r="E53" s="3" t="inlineStr">
+      <c r="E56" s="2" t="inlineStr">
         <is>
           <t>High — replaces MediaLab Document Control ($752/$2,250 starting price, scalin...</t>
         </is>
       </c>
-      <c r="F53" s="3" t="inlineStr">
+      <c r="F56" s="2" t="inlineStr">
         <is>
           <t>Effort: XL (one focused session, 12 PRs landed)
 Importance: High — replaces MediaLab Document Control ($752/$2,250 starting price, scaling to $10K-$20K/yr at enterprise per Capterra public data) with an included VeritaPolicy feature; closes a real positioning gap and gives sales a direct comparator line.</t>
         </is>
       </c>
-      <c r="G53" s="3" t="inlineStr">
+      <c r="G56" s="2" t="inlineStr">
         <is>
           <t>Pricing strategy conversation 2026-05-29 (Michael: "I don't like bolt-ons; we should replicate this") → scoped 8 phases → shipped all 12 PRs in single session. Shipped 2026-05-29.
 ---</t>
         </is>
       </c>
-      <c r="H53" s="3" t="inlineStr"/>
+      <c r="H56" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H53"/>
+  <autoFilter ref="A1:H56"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
TASK: Close parking-lot #54, #55, #56 (shipped) and sync xlsx
PLAN:
  1. Move #54, #55, #56 from OPEN to CLOSED with PR evidence.
  2. Re-sync PARKING_LOT.xlsx.

Self-check:
  - All three merged to main and live on prod (5ae6c0bb).
  - Internal doc change; Gate 3 N/A.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PARKING_LOT.xlsx
+++ b/PARKING_LOT.xlsx
@@ -12,8 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RETIRED" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$56</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RETIRED'!$A$1:$H$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1083,140 +1083,8 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="90" customHeight="1">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>54</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>VeritaTrack: quarterly task loads as monthly until re-saved (frequency display/state bug)</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>Open, not started. Needs reproduction in Michael's lab first.</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>S (1-3 days: reproduce, find where the task-create frequency is stored vs ren...</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>Medium — data-integrity/UX. A task entered as quarterly that shows as monthly...</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>Effort: S (1-3 days: reproduce, find where the task-create frequency is stored vs rendered on the list, fix the load/display path)
-Importance: Medium — data-integrity/UX. A task entered as quarterly that shows as monthly on the tracker until someone re-saves it can drive the wrong due cadence and false "overdue" signals; silent and easy to miss.</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>Michael, 2026-10-01 (parking lot).</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>Either; small.
----</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="90" customHeight="1">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>55</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>VeritaScan: let sites add their own custom questions</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>Open, not started. Needs a short design decision on scoring treatment.</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>M (1-2 weeks: a per-lab custom-question model, admin UI to author them, inclu...</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="inlineStr">
-        <is>
-          <t>Medium-High — site-requested flexibility and a differentiator; lets a lab ext...</t>
-        </is>
-      </c>
-      <c r="F15" s="3" t="inlineStr">
-        <is>
-          <t>Effort: M (1-2 weeks: a per-lab custom-question model, admin UI to author them, inclusion in the scan run + scoring/readiness, and export rendering)
-Importance: Medium-High — site-requested flexibility and a differentiator; lets a lab extend the standardized scan with its own internal checks without us hard-coding them.</t>
-        </is>
-      </c>
-      <c r="G15" s="3" t="inlineStr">
-        <is>
-          <t>Michael, 2026-10-01 (parking lot).</t>
-        </is>
-      </c>
-      <c r="H15" s="3" t="inlineStr">
-        <is>
-          <t>Post-COLA unless a named prospect asks.
----</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="90" customHeight="1">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>56</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>VeritaQC: flag/popup when a datapoint is outside +/- 2 SD at entry</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Open, not started.</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>S-M (3 days to ~1.5 weeks: compute mean/SD context at entry, warn when |z| &gt;...</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>High — patient-safety/usability gap. Right now an out-of-2SD control result i...</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>Effort: S-M (3 days to ~1.5 weeks: compute mean/SD context at entry, warn when |z| &gt; 2, surface an inline flag + a confirm/acknowledge prompt; reuse the existing LJ/Westgard evaluation)
-Importance: High — patient-safety/usability gap. Right now an out-of-2SD control result is accepted silently; unless the tech scrolls to the Levey-Jennings chart they have no idea it was out, so a real QC excursion can be missed at the moment it matters.</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>Michael, 2026-10-01 (parking lot).</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>Either; strong quality-of-life + safety win.
----</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:H16"/>
+  <autoFilter ref="A1:H13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1227,7 +1095,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H53"/>
+  <dimension ref="A1:H56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1285,24 +1153,24 @@
     <row r="2" ht="90" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>C52</t>
+          <t>C55</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>VeritaResponse internal NCE / non-conforming event (was #36)</t>
+          <t>VeritaScan: let sites add their own custom questions (was #55)</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr"/>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>was L (shipped as MEDIUM) / Importance: High</t>
+          <t>was M / Importance: Medium-High</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Effort: was L (shipped as MEDIUM) / Importance: High</t>
+          <t>Effort: was M / Importance: Medium-High</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
@@ -1311,24 +1179,24 @@
     <row r="3" ht="90" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>C49</t>
+          <t>C54</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Competency "assessed this cycle" cadence-aware window (was #50)</t>
+          <t>VeritaQC: at-entry warning when a QC point is outside 2 SD (was #56)</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr"/>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>was S-M / Importance: Medium</t>
+          <t>was S-M (shipped S) / Importance: High</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Effort: was S-M / Importance: Medium</t>
+          <t>Effort: was S-M (shipped S) / Importance: High</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr"/>
@@ -1337,24 +1205,24 @@
     <row r="4" ht="90" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>C50</t>
+          <t>C53</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>VeritaTrack task owner + owner-only reminder routing (was #51)</t>
+          <t>VeritaTrack: quarterly task loaded as monthly until re-saved (was #54)</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr"/>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>was S-M / Importance: Medium</t>
+          <t>was S / Importance: Medium</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Effort: was S-M / Importance: Medium</t>
+          <t>Effort: was S / Importance: Medium</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr"/>
@@ -1363,24 +1231,24 @@
     <row r="5" ht="90" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>C51</t>
+          <t>C52</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Designate Medical Director by picking a lab member (was #52, core)</t>
+          <t>VeritaResponse internal NCE / non-conforming event (was #36)</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr"/>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>was S-M / Importance: Medium-High</t>
+          <t>was L (shipped as MEDIUM) / Importance: High</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Effort: was S-M / Importance: Medium-High</t>
+          <t>Effort: was L (shipped as MEDIUM) / Importance: High</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr"/>
@@ -1389,24 +1257,24 @@
     <row r="6" ht="90" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>C47</t>
+          <t>C49</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Unregulated-analyte / Alternative Assessment (AAA) coverage (was #18)</t>
+          <t>Competency "assessed this cycle" cadence-aware window (was #50)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr"/>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>was S (Phase 3) / Importance: Medium</t>
+          <t>was S-M / Importance: Medium</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Effort: was S (Phase 3) / Importance: Medium</t>
+          <t>Effort: was S-M / Importance: Medium</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
@@ -1415,24 +1283,24 @@
     <row r="7" ht="90" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>C48</t>
+          <t>C50</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>VeritaResponse post-survey deficiency module (was #17)</t>
+          <t>VeritaTrack task owner + owner-only reminder routing (was #51)</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr"/>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>was XL / Importance: High</t>
+          <t>was S-M / Importance: Medium</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Effort: was XL / Importance: High</t>
+          <t>Effort: was S-M / Importance: Medium</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr"/>
@@ -1441,93 +1309,90 @@
     <row r="8" ht="90" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>C45</t>
+          <t>C51</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Unify coverage/competency recurrence helper (was #49) - closed as non-issue</t>
+          <t>Designate Medical Director by picking a lab member (was #52, core)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr"/>
-      <c r="D8" s="2" t="inlineStr"/>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>was S-M / Importance: Medium-High</t>
+        </is>
+      </c>
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: Investigated 2026-09-24 before building. The coverage recurrence math (+6-month interval, signed-resets-to-missing, nextDueOn/overdue, isFailVerdict) is ALREADY single-source in server/veritacheckCoverage.ts (computeCoverageFrom). server/coverageReport.ts and the routes.ts coverage export do not recompute it; they consume the computed nextDueOn/overdue/status fields and apply small surface-specific presentation labels (deliberately different vocabularies per surface, so they should not be merged). The only truly identical duplicate is a one-line date formatter. The competency "owed" derivation is NOT the same cadence: competency follows the CLIA milestone schedule (initial / semiannual year 1 / annual, 42 CFR 493.1451(b)(8) and 493.1235), which is a different regulatory interval from the coverage 6-month rule (493.1281 / 493.1255) and must stay separate. No worthwhile extraction; merging the two cadences would be wrong. Closed 2026-09-24. (The year-1 competency-window refinement remains tracked separately as #50.)</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-24 session, "keep working" pass; scoped read-only, found no real duplication.
----</t>
-        </is>
-      </c>
+          <t>Effort: was S-M / Importance: Medium-High</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr"/>
       <c r="H8" s="2" t="inlineStr"/>
     </row>
     <row r="9" ht="90" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>C46</t>
+          <t>C47</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Verified-users product-update send path (wrong-list incident fix)</t>
+          <t>Unregulated-analyte / Alternative Assessment (AAA) coverage (was #18)</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr"/>
-      <c r="D9" s="3" t="inlineStr"/>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>was S (Phase 3) / Importance: Medium</t>
+        </is>
+      </c>
       <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: Shipped PR #1324 (merged 4e05506a, deploy ACTIVE). New POST /api/admin/users/send targets registered VeritaAssure account holders (the users table), never the Lab Director's Briefing subscriber list. Separate explicitly-named endpoint (not a flag with a dangerous default), account-holder email framing, excludes suppressed emails and RFC-reserved test domains, CC owner, dryRun + testTo previews. Public unsubscribe now upserts a suppression row so opt-outs are honored across both audiences. Live dryRun: 49 verified-user recipients vs 673 on the Briefing list. Receipts: scripts/verify-product-update-send.mts 24/24, tsc clean, rendered sample inspected. Fixes the fallout from the 2026-09-23/24 wrong-list send (a product update went to the 675-person Briefing list). Nothing sends without Michael's explicit "send it."</t>
-        </is>
-      </c>
-      <c r="G9" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-24 session; Michael selected this as the next build after the #41 close.
----</t>
-        </is>
-      </c>
+          <t>Effort: was S (Phase 3) / Importance: Medium</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr"/>
       <c r="H9" s="3" t="inlineStr"/>
     </row>
     <row r="10" ht="90" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>C44</t>
+          <t>C48</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Verify-script convention backfill (was #41) + audit matcher fix</t>
+          <t>VeritaResponse post-survey deficiency module (was #17)</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr"/>
-      <c r="D10" s="2" t="inlineStr"/>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>was XL / Importance: High</t>
+        </is>
+      </c>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: #41 was fully backfilled on 2026-06-13 (all 8 high-stakes scripts landed; see C30); it had only been mis-filed in OPEN. A 2026-09-24 re-audit initially reported 4 of 5 recent math/logic commits as missing a verify script, which was a FALSE POSITIVE: scripts/audit_verify_script_coverage.py matched only scripts/verify-*.js / .cjs, so it ignored the .mjs / .mts / .ts verify scripts the repo now ships (e.g. verify-ptcoag-multi.mts, verify-tea-criterion-format.mjs). Fixed the matcher to accept .js/.cjs/.mjs/.ts/.mts; re-run shows 5 of 5 covered, 0 debt. The convention is being followed. Closed 2026-09-24.</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-24 session, "keep working" pass; audit tooling bug found + fixed.
----</t>
-        </is>
-      </c>
+          <t>Effort: was XL / Importance: High</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr"/>
       <c r="H10" s="2" t="inlineStr"/>
     </row>
     <row r="11" ht="90" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>C43</t>
+          <t>C45</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>VeritaStaff instrument-centric (dual) assignment view</t>
+          <t>Unify coverage/competency recurrence helper (was #49) - closed as non-issue</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr"/>
@@ -1535,12 +1400,12 @@
       <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1320. GET/PUT /staff/instruments/:id/employees (transpose of the per-employee endpoints); an "Assign by Instrument" dialog lets a director pick a test system or manual test and check off who runs it. Same staff_employee_instruments join, with the 42 CFR 493.1235(a) duty-change event emitted on newly-added pairs so both orientations trigger the same reassessment. GET verified live on SCAHC lab 2. Closed 2026-09-24.</t>
+          <t>Closure evidence: Investigated 2026-09-24 before building. The coverage recurrence math (+6-month interval, signed-resets-to-missing, nextDueOn/overdue, isFailVerdict) is ALREADY single-source in server/veritacheckCoverage.ts (computeCoverageFrom). server/coverageReport.ts and the routes.ts coverage export do not recompute it; they consume the computed nextDueOn/overdue/status fields and apply small surface-specific presentation labels (deliberately different vocabularies per surface, so they should not be merged). The only truly identical duplicate is a one-line date formatter. The competency "owed" derivation is NOT the same cadence: competency follows the CLIA milestone schedule (initial / semiannual year 1 / annual, 42 CFR 493.1451(b)(8) and 493.1235), which is a different regulatory interval from the coverage 6-month rule (493.1281 / 493.1255) and must stay separate. No worthwhile extraction; merging the two cadences would be wrong. Closed 2026-09-24. (The year-1 competency-window refinement remains tracked separately as #50.)</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>2026-09-24 session, Michael ("in staff we should also give the dual view when assigning coverage to test systems or manual tests").
+          <t>2026-09-24 session, "keep working" pass; scoped read-only, found no real duplication.
 ---</t>
         </is>
       </c>
@@ -1549,12 +1414,12 @@
     <row r="12" ht="90" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>C42</t>
+          <t>C46</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>VeritaComp coverage map (required-vs-assessed matrix, dual view)</t>
+          <t>Verified-users product-update send path (wrong-list incident fix)</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr"/>
@@ -1562,12 +1427,12 @@
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1319 (+ status layer PR #1316). /competency/owed returns per-item assessed (locked passing assessment this cycle on a covering method group) + per-employee CLIA status; CompetencyCoverageMap renders a By-employee / By-instrument matrix (Assessed / Owed / Overdue / Gap). Verified live on SCAHC lab 2 (owed 116, assessed 2, gaps 0). Completes #48 as the VeritaCheck-parity coverage map. Closed 2026-09-24.</t>
+          <t>Closure evidence: Shipped PR #1324 (merged 4e05506a, deploy ACTIVE). New POST /api/admin/users/send targets registered VeritaAssure account holders (the users table), never the Lab Director's Briefing subscriber list. Separate explicitly-named endpoint (not a flag with a dangerous default), account-holder email framing, excludes suppressed emails and RFC-reserved test domains, CC owner, dryRun + testTo previews. Public unsubscribe now upserts a suppression row so opt-outs are honored across both audiences. Live dryRun: 49 verified-user recipients vs 673 on the Briefing list. Receipts: scripts/verify-product-update-send.mts 24/24, tsc clean, rendered sample inspected. Fixes the fallout from the 2026-09-23/24 wrong-list send (a product update went to the 675-person Briefing list). Nothing sends without Michael's explicit "send it."</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 session, Michael ("are we building the competencies to have a coverage map, same as veritacheck?" then "build it").
+          <t>2026-09-24 session; Michael selected this as the next build after the #41 close.
 ---</t>
         </is>
       </c>
@@ -1576,12 +1441,12 @@
     <row r="13" ht="90" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>C41</t>
+          <t>C44</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>VeritaCheck coverage recurrence (method comparison + cal-ver/linearity + reports)</t>
+          <t>Verify-script convention backfill (was #41) + audit matcher fix</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr"/>
@@ -1589,12 +1454,12 @@
       <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: PRs #1317 (method comparison), #1318 (cal-ver/linearity), #1321 (report Next-due columns). Periodic verification (correlation/method comparison 42 CFR 493.1281; cal-ver/linearity 42 CFR 493.1255; both 6-month) now recurs: a signed study banks the cycle and rolls to next-due = signed + 6 months instead of reading "done" forever. Status Missing/Failed/Completed-unsigned + a "Next due on" column on-screen and in both coverage exports; also credits the previously-ignored "correlation" study type. Root cause: computeCoverageFrom marked requirements done on mere existence, no date logic. Verified live on SCAHC lab 2 (101 correlations + 11 cal-ver rows now carry a next-due). Engine-level, all facilities. Closed 2026-09-24.</t>
+          <t>Closure evidence: #41 was fully backfilled on 2026-06-13 (all 8 high-stakes scripts landed; see C30); it had only been mis-filed in OPEN. A 2026-09-24 re-audit initially reported 4 of 5 recent math/logic commits as missing a verify script, which was a FALSE POSITIVE: scripts/audit_verify_script_coverage.py matched only scripts/verify-*.js / .cjs, so it ignored the .mjs / .mts / .ts verify scripts the repo now ships (e.g. verify-ptcoag-multi.mts, verify-tea-criterion-format.mjs). Fixed the matcher to accept .js/.cjs/.mjs/.ts/.mts; re-run shows 5 of 5 covered, 0 debt. The convention is being followed. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>2026-09-24 session, Michael ("Look at San Carlos... they finished their last set of correlations (all 103) but their menu never reset").
+          <t>2026-09-24 session, "keep working" pass; audit tooling bug found + fixed.
 ---</t>
         </is>
       </c>
@@ -1603,12 +1468,12 @@
     <row r="14" ht="90" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>C40</t>
+          <t>C43</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>VeritaComp Competencies Owed derived from VeritaStaff, with gap detection (was #48)</t>
+          <t>VeritaStaff instrument-centric (dual) assignment view</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr"/>
@@ -1616,12 +1481,12 @@
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1314 (squash 2bcb0db9). GET /api/labs/:labId/competency/owed derives each VeritaStaff testing employee's owed competencies from their assigned instruments (staff_employee_instruments -&gt; veritamap_instruments + tests), on the CLIA timeline, and flags instruments not covered by any competency program as gaps. CompetenciesOwedSection renders it on the VeritaComp landing page. Reuses the shipped bridge + suggested-method-groups match rules; no new tables. Verified live on prod with real assignment data: 2 instruments assigned to a demo staffer produced owed=2, gaps=2 (HIGH, Technical Supervisor), then reverted cleanly. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1320. GET/PUT /staff/instruments/:id/employees (transpose of the per-employee endpoints); an "Assign by Instrument" dialog lets a director pick a test system or manual test and check off who runs it. Same staff_employee_instruments join, with the 42 CFR 493.1235(a) duty-change event emitted on newly-added pairs so both orientations trigger the same reassessment. GET verified live on SCAHC lab 2. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23/24 session, Michael ("veritacomp bases what competencies they owe (currently untrue, but needs to be true)"). Option 1 (unify roster on VeritaStaff, match instruments by id).
+          <t>2026-09-24 session, Michael ("in staff we should also give the dual view when assigning coverage to test systems or manual tests").
 ---</t>
         </is>
       </c>
@@ -1630,12 +1495,12 @@
     <row r="15" ht="90" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>C39</t>
+          <t>C42</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>VeritaScan line items can attach or link evidence (was #46)</t>
+          <t>VeritaComp coverage map (required-vs-assessed matrix, dual view)</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr"/>
@@ -1643,12 +1508,12 @@
       <c r="E15" s="3" t="inlineStr"/>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1312 (squash a1dda93d). VeritaScan scan checklist items now show linked evidence as chips (open link, remove) plus a writer "Link evidence" affordance whose picker links an existing VeritaDC/Library document; a shortcut deep-links to the Library for new (governed) documents. Reuses the already-shipped lab_documents + document_checklist_links + coverage endpoints (URL-pointer only, no file storage, no new tables). Browser-verified live on prod (scan 23): the affordance renders and the picker opens. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1319 (+ status layer PR #1316). /competency/owed returns per-item assessed (locked passing assessment this cycle on a covering method group) + per-employee CLIA status; CompetencyCoverageMap renders a By-employee / By-instrument matrix (Assessed / Owed / Overdue / Gap). Verified live on SCAHC lab 2 (owed 116, assessed 2, gaps 0). Completes #48 as the VeritaCheck-parity coverage map. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>2026-09-23 session, Michael. Recurring request. Companion: cross-module evidence display on the VeritaDC policy shipped in PR #1313 (by-target cross-links surfaced in the policy View modal, browser-verified live).
+          <t>2026-09-24 session, Michael ("are we building the competencies to have a coverage map, same as veritacheck?" then "build it").
 ---</t>
         </is>
       </c>
@@ -1657,12 +1522,12 @@
     <row r="16" ht="90" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>C38</t>
+          <t>C41</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>VeritaTrack calendar month cells expand to reveal hidden tasks (was #45)</t>
+          <t>VeritaCheck coverage recurrence (method comparison + cal-ver/linearity + reports)</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr"/>
@@ -1670,12 +1535,12 @@
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: VeritaTrack CalendarView month cells with more than three tasks now expand in place (chevron, "+N more" toggling to "Show less", due dates), so no task is hidden with no path to it (client/src/pages/VeritaTrackAppPage.tsx CalendarView). Shipped 2026-09-23. Closed 2026-09-24.</t>
+          <t>Closure evidence: PRs #1317 (method comparison), #1318 (cal-ver/linearity), #1321 (report Next-due columns). Periodic verification (correlation/method comparison 42 CFR 493.1281; cal-ver/linearity 42 CFR 493.1255; both 6-month) now recurs: a signed study banks the cycle and rolls to next-due = signed + 6 months instead of reading "done" forever. Status Missing/Failed/Completed-unsigned + a "Next due on" column on-screen and in both coverage exports; also credits the previously-ignored "correlation" study type. Root cause: computeCoverageFrom marked requirements done on mere existence, no date logic. Verified live on SCAHC lab 2 (101 correlations + 11 cal-ver rows now carry a next-due). Engine-level, all facilities. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23 session, Michael screenshot of the VeritaTrack calendar (lab 3, September cell).
+          <t>2026-09-24 session, Michael ("Look at San Carlos... they finished their last set of correlations (all 103) but their menu never reset").
 ---</t>
         </is>
       </c>
@@ -1684,12 +1549,12 @@
     <row r="17" ht="90" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>C37</t>
+          <t>C40</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Long Excel column headers no longer clip CFR citations (was #44)</t>
+          <t>VeritaComp Competencies Owed derived from VeritaStaff, with gap detection (was #48)</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr"/>
@@ -1697,12 +1562,12 @@
       <c r="E17" s="3" t="inlineStr"/>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. The VeritaMap export derives the header row height from the longest wrapped header via headerRowHeight(headers, colWidths) (server/routes.ts:15935) instead of a fixed 20, so "Reference Range Attestation (42 CFR 493.1253)" and the other long headers print in full. No new code this session. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1314 (squash 2bcb0db9). GET /api/labs/:labId/competency/owed derives each VeritaStaff testing employee's owed competencies from their assigned instruments (staff_employee_instruments -&gt; veritamap_instruments + tests), on the CLIA timeline, and flags instruments not covered by any competency program as gaps. CompetenciesOwedSection renders it on the VeritaComp landing page. Reuses the shipped bridge + suggested-method-groups match rules; no new tables. Verified live on prod with real assignment data: 2 instruments assigned to a demo staffer produced owed=2, gaps=2 (HIGH, Technical Supervisor), then reverted cleanly. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+          <t>2026-09-23/24 session, Michael ("veritacomp bases what competencies they owe (currently untrue, but needs to be true)"). Option 1 (unify roster on VeritaStaff, match instruments by id).
 ---</t>
         </is>
       </c>
@@ -1711,12 +1576,12 @@
     <row r="18" ht="90" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>C36</t>
+          <t>C39</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>License stamp no longer clobbers the §6 header/footer or names the wrong lab (was #43)</t>
+          <t>VeritaScan line items can attach or link evidence (was #46)</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr"/>
@@ -1724,12 +1589,12 @@
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. setHeaderFooter (shared/licenseExceljs.ts:155-209) now preserves an existing §6 header and appends (not overwrites) the footer left section, and customer-facing exports name the scoped lab: the VeritaScan library export reads req.scope.lab.name / clia_number (server/routes.ts:16572-16573), not the licensee. No new code this session (avoided regressing the existing fix). Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1312 (squash a1dda93d). VeritaScan scan checklist items now show linked evidence as chips (open link, remove) plus a writer "Link evidence" affordance whose picker links an existing VeritaDC/Library document; a shortcut deep-links to the Library for new (governed) documents. Reuses the already-shipped lab_documents + document_checklist_links + coverage endpoints (URL-pointer only, no file storage, no new tables). Browser-verified live on prod (scan 23): the affordance renders and the picker opens. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+          <t>2026-09-23 session, Michael. Recurring request. Companion: cross-module evidence display on the VeritaDC policy shipped in PR #1313 (by-target cross-links surfaced in the policy View modal, browser-verified live).
 ---</t>
         </is>
       </c>
@@ -1738,18 +1603,99 @@
     <row r="19" ht="90" customHeight="1">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>C34</t>
+          <t>C38</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Wire the two static-audit guards into CI (was #43)</t>
+          <t>VeritaTrack calendar month cells expand to reveal hidden tasks (was #45)</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr"/>
       <c r="D19" s="3" t="inlineStr"/>
       <c r="E19" s="3" t="inlineStr"/>
       <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Closure evidence: VeritaTrack CalendarView month cells with more than three tasks now expand in place (chevron, "+N more" toggling to "Show less", due dates), so no task is hidden with no path to it (client/src/pages/VeritaTrackAppPage.tsx CalendarView). Shipped 2026-09-23. Closed 2026-09-24.</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-23 session, Michael screenshot of the VeritaTrack calendar (lab 3, September cell).
+---</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr"/>
+    </row>
+    <row r="20" ht="90" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>C37</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Long Excel column headers no longer clip CFR citations (was #44)</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr"/>
+      <c r="D20" s="2" t="inlineStr"/>
+      <c r="E20" s="2" t="inlineStr"/>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. The VeritaMap export derives the header row height from the longest wrapped header via headerRowHeight(headers, colWidths) (server/routes.ts:15935) instead of a fixed 20, so "Reference Range Attestation (42 CFR 493.1253)" and the other long headers print in full. No new code this session. Closed 2026-09-24.</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+---</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21" ht="90" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>C36</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>License stamp no longer clobbers the §6 header/footer or names the wrong lab (was #43)</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr"/>
+      <c r="D21" s="3" t="inlineStr"/>
+      <c r="E21" s="3" t="inlineStr"/>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. setHeaderFooter (shared/licenseExceljs.ts:155-209) now preserves an existing §6 header and appends (not overwrites) the footer left section, and customer-facing exports name the scoped lab: the VeritaScan library export reads req.scope.lab.name / clia_number (server/routes.ts:16572-16573), not the licensee. No new code this session (avoided regressing the existing fix). Closed 2026-09-24.</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+---</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22" ht="90" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>C34</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Wire the two static-audit guards into CI (was #43)</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr"/>
+      <c r="D22" s="2" t="inlineStr"/>
+      <c r="E22" s="2" t="inlineStr"/>
+      <c r="F22" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: both guards wired into the Multi-Lab Mutations Audit CI
 workflow (.github/workflows/multilab-mutations-audit.yml) as steps:
@@ -1761,24 +1707,24 @@
 (same caveat as the existing guards already in that workflow).</t>
         </is>
       </c>
-      <c r="G19" s="3" t="inlineStr"/>
-      <c r="H19" s="3" t="inlineStr"/>
-    </row>
-    <row r="20" ht="90" customHeight="1">
-      <c r="A20" s="2" t="inlineStr">
+      <c r="G22" s="2" t="inlineStr"/>
+      <c r="H22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23" ht="90" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>C35</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>Legacy /api/studies over-returns studies across labs (was #44)</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr"/>
-      <c r="D20" s="2" t="inlineStr"/>
-      <c r="E20" s="2" t="inlineStr"/>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="C23" s="3" t="inlineStr"/>
+      <c r="D23" s="3" t="inlineStr"/>
+      <c r="E23" s="3" t="inlineStr"/>
+      <c r="F23" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: GET /api/studies now scopes its list to the active lab
 when one is resolved from the Referer (server/routes.ts), so every returned row
@@ -1788,24 +1734,24 @@
 mirroring the /api/labs/:labId/studies handler. Closed 2026-06-14.</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr"/>
-      <c r="H20" s="2" t="inlineStr"/>
-    </row>
-    <row r="21" ht="90" customHeight="1">
-      <c r="A21" s="3" t="inlineStr">
+      <c r="G23" s="3" t="inlineStr"/>
+      <c r="H23" s="3" t="inlineStr"/>
+    </row>
+    <row r="24" ht="90" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>C30</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>Verify-script convention backfill (was #41)</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr"/>
-      <c r="D21" s="3" t="inlineStr"/>
-      <c r="E21" s="3" t="inlineStr"/>
-      <c r="F21" s="3" t="inlineStr">
+      <c r="C24" s="2" t="inlineStr"/>
+      <c r="D24" s="2" t="inlineStr"/>
+      <c r="E24" s="2" t="inlineStr"/>
+      <c r="F24" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: all 8 high-stakes math/logic commits now ship a paired
 scripts/verify-*.js (EP17 sensitivity, Deming lot-to-lot, CUMSUM+QC+multi-analyte,
@@ -1813,30 +1759,30 @@
 TEa boundary), per the strike-throughs in #41. Closed 2026-06-13.</t>
         </is>
       </c>
-      <c r="G21" s="3" t="inlineStr">
+      <c r="G24" s="2" t="inlineStr">
         <is>
           <t>scripts/audit_verify_script_coverage.py lookback, 2026-06-02; backfills
 landed 2026-06-03..06.
 ---</t>
         </is>
       </c>
-      <c r="H21" s="3" t="inlineStr"/>
-    </row>
-    <row r="22" ht="90" customHeight="1">
-      <c r="A22" s="2" t="inlineStr">
+      <c r="H24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25" ht="90" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
         <is>
           <t>C31</t>
         </is>
       </c>
-      <c r="B22" s="2" t="inlineStr">
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>VeritaPT AAA create/update/delete silently no-op in the multi-lab UI</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr"/>
-      <c r="D22" s="2" t="inlineStr"/>
-      <c r="E22" s="2" t="inlineStr"/>
-      <c r="F22" s="2" t="inlineStr">
+      <c r="C25" s="3" t="inlineStr"/>
+      <c r="D25" s="3" t="inlineStr"/>
+      <c r="E25" s="3" t="inlineStr"/>
+      <c r="F25" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #754 (commit 92ad499) added lab-scoped POST/PUT/DELETE
 /api/labs/:labId/pt/aa-records. The UI posted to the lab-scoped path but only GET
@@ -1847,30 +1793,30 @@
 route mis-filed records to the user's default lab on multi-lab accounts).</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr">
+      <c r="G25" s="3" t="inlineStr">
         <is>
           <t>2026-06-13, found during #18 Phase 3 QA;
 scripts/audit-labscoped-write-routes.mjs now guards the class.
 ---</t>
         </is>
       </c>
-      <c r="H22" s="2" t="inlineStr"/>
-    </row>
-    <row r="23" ht="90" customHeight="1">
-      <c r="A23" s="3" t="inlineStr">
+      <c r="H25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26" ht="90" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>C32</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t>VeritaComp "Unlock assessment" false-success no-op</t>
         </is>
       </c>
-      <c r="C23" s="3" t="inlineStr"/>
-      <c r="D23" s="3" t="inlineStr"/>
-      <c r="E23" s="3" t="inlineStr"/>
-      <c r="F23" s="3" t="inlineStr">
+      <c r="C26" s="2" t="inlineStr"/>
+      <c r="D26" s="2" t="inlineStr"/>
+      <c r="E26" s="2" t="inlineStr"/>
+      <c r="F26" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #755 (commit 4234007) moved the unlock route to
 /api/labs/:labId/competency/assessments/:id/unlock (the path the client calls).
@@ -1881,29 +1827,29 @@
 HTML).</t>
         </is>
       </c>
-      <c r="G23" s="3" t="inlineStr">
+      <c r="G26" s="2" t="inlineStr">
         <is>
           <t>2026-06-13, found by scripts/audit-labscoped-write-routes.mjs.
 ---</t>
         </is>
       </c>
-      <c r="H23" s="3" t="inlineStr"/>
-    </row>
-    <row r="24" ht="90" customHeight="1">
-      <c r="A24" s="2" t="inlineStr">
+      <c r="H26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27" ht="90" customHeight="1">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>C33</t>
         </is>
       </c>
-      <c r="B24" s="2" t="inlineStr">
+      <c r="B27" s="3" t="inlineStr">
         <is>
           <t>FK-cascade delete 500s + NavBar laptop-width overflow</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr"/>
-      <c r="D24" s="2" t="inlineStr"/>
-      <c r="E24" s="2" t="inlineStr"/>
-      <c r="F24" s="2" t="inlineStr">
+      <c r="C27" s="3" t="inlineStr"/>
+      <c r="D27" s="3" t="inlineStr"/>
+      <c r="E27" s="3" t="inlineStr"/>
+      <c r="F27" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PRs #749/#750 fixed NavBar horizontal overflow at laptop
 widths (collapse to the hamburger below 1560px); prod-verified at 1280-1920 with the
@@ -1914,57 +1860,57 @@
 500 -&gt; 200. scripts/audit-delete-cascades.mjs guards the class.</t>
         </is>
       </c>
-      <c r="G24" s="2" t="inlineStr">
+      <c r="G27" s="3" t="inlineStr">
         <is>
           <t>2026-06-13 browser QA of the A7-D4 wave + retro-QC of the 72h PR window.
 ---</t>
         </is>
       </c>
-      <c r="H24" s="2" t="inlineStr"/>
-    </row>
-    <row r="25" ht="90" customHeight="1">
-      <c r="A25" s="3" t="inlineStr">
+      <c r="H27" s="3" t="inlineStr"/>
+    </row>
+    <row r="28" ht="90" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>C1</t>
         </is>
       </c>
-      <c r="B25" s="3" t="inlineStr">
+      <c r="B28" s="2" t="inlineStr">
         <is>
           <t>FAQ "over 25 years" -&gt; "over 23 years"</t>
         </is>
       </c>
-      <c r="C25" s="3" t="inlineStr"/>
-      <c r="D25" s="3" t="inlineStr"/>
-      <c r="E25" s="3" t="inlineStr"/>
-      <c r="F25" s="3" t="inlineStr">
+      <c r="C28" s="2" t="inlineStr"/>
+      <c r="D28" s="2" t="inlineStr"/>
+      <c r="E28" s="2" t="inlineStr"/>
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: client/src/pages/FAQPage.tsx line 20 reads "over
 23 years" as of 2026-05-01.</t>
         </is>
       </c>
-      <c r="G25" s="3" t="inlineStr">
+      <c r="G28" s="2" t="inlineStr">
         <is>
           <t>session 299e9a73 turn 14, ~2026-04-28.
 ---</t>
         </is>
       </c>
-      <c r="H25" s="3" t="inlineStr"/>
-    </row>
-    <row r="26" ht="90" customHeight="1">
-      <c r="A26" s="2" t="inlineStr">
+      <c r="H28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29" ht="90" customHeight="1">
+      <c r="A29" s="3" t="inlineStr">
         <is>
           <t>C5</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="B29" s="3" t="inlineStr">
         <is>
           <t>David's VeritaQA grey-button bug (seat permissions mode)</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr"/>
-      <c r="D26" s="2" t="inlineStr"/>
-      <c r="E26" s="2" t="inlineStr"/>
-      <c r="F26" s="2" t="inlineStr">
+      <c r="C29" s="3" t="inlineStr"/>
+      <c r="D29" s="3" t="inlineStr"/>
+      <c r="E29" s="3" t="inlineStr"/>
+      <c r="F29" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #10 squash-merged as commit a43fbba on
 2026-05-01 23:19 MST. Railway deploy succeeded; deployed bundle
@@ -1977,7 +1923,7 @@
 against his exact stored shape (14 of 14 expected outcomes matched).</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr">
+      <c r="G29" s="3" t="inlineStr">
         <is>
           <t>2026-05-01 David's report; veritabench + veritastock
 weren't in MODULE_LIST so seat permissions silently defaulted to
@@ -1985,109 +1931,109 @@
 ---</t>
         </is>
       </c>
-      <c r="H26" s="2" t="inlineStr"/>
-    </row>
-    <row r="27" ht="90" customHeight="1">
-      <c r="A27" s="3" t="inlineStr">
-        <is>
-          <t>C2</t>
-        </is>
-      </c>
-      <c r="B27" s="3" t="inlineStr">
-        <is>
-          <t>TeamPage present-tense "TJC surveyor" check</t>
-        </is>
-      </c>
-      <c r="C27" s="3" t="inlineStr"/>
-      <c r="D27" s="3" t="inlineStr"/>
-      <c r="E27" s="3" t="inlineStr"/>
-      <c r="F27" s="3" t="inlineStr">
-        <is>
-          <t>Closure evidence: site-wide search confirmed all surveyor language
-is past-tense, consistent with user's 2021-2025 service. User closed
-the item in session 299e9a73 turn 4.</t>
-        </is>
-      </c>
-      <c r="G27" s="3" t="inlineStr">
-        <is>
-          <t>session 299e9a73, ~2026-04-28.
----</t>
-        </is>
-      </c>
-      <c r="H27" s="3" t="inlineStr"/>
-    </row>
-    <row r="28" ht="90" customHeight="1">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>C3</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>My Studies CSV/XLSX export (John as design partner)</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="inlineStr"/>
-      <c r="D28" s="2" t="inlineStr"/>
-      <c r="E28" s="2" t="inlineStr"/>
-      <c r="F28" s="2" t="inlineStr">
-        <is>
-          <t>Closure evidence: client/src/pages/DashboardPage.tsx line 46 calls
-/api/my-studies/export. server/routes.ts line 1491 implements the
-endpoint. Pulled forward into pre-COLA per user instruction.</t>
-        </is>
-      </c>
-      <c r="G28" s="2" t="inlineStr">
-        <is>
-          <t>session 299e9a73 turn 5, ~2026-04-28.
----</t>
-        </is>
-      </c>
-      <c r="H28" s="2" t="inlineStr"/>
-    </row>
-    <row r="29" ht="90" customHeight="1">
-      <c r="A29" s="3" t="inlineStr">
-        <is>
-          <t>C4</t>
-        </is>
-      </c>
-      <c r="B29" s="3" t="inlineStr">
-        <is>
-          <t>Rotate GitHub PAT (because old PAT was committed in SESSION_HANDOFF files)</t>
-        </is>
-      </c>
-      <c r="C29" s="3" t="inlineStr"/>
-      <c r="D29" s="3" t="inlineStr"/>
-      <c r="E29" s="3" t="inlineStr"/>
-      <c r="F29" s="3" t="inlineStr">
-        <is>
-          <t>Closure evidence: no ghp_* or github_pat_* patterns in current
-SESSION_HANDOFF.md or SESSION_HANDOFF-2.md as of 2026-05-01.</t>
-        </is>
-      </c>
-      <c r="G29" s="3" t="inlineStr">
-        <is>
-          <t>session 299e9a73, ~2026-04-28.
----</t>
-        </is>
-      </c>
       <c r="H29" s="3" t="inlineStr"/>
     </row>
     <row r="30" ht="90" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>C6</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>VeritaPolicy service-line filtering removed (formerly #4)</t>
+          <t>TeamPage present-tense "TJC surveyor" check</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr"/>
       <c r="D30" s="2" t="inlineStr"/>
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Closure evidence: site-wide search confirmed all surveyor language
+is past-tense, consistent with user's 2021-2025 service. User closed
+the item in session 299e9a73 turn 4.</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>session 299e9a73, ~2026-04-28.
+---</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31" ht="90" customHeight="1">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>C3</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>My Studies CSV/XLSX export (John as design partner)</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr"/>
+      <c r="D31" s="3" t="inlineStr"/>
+      <c r="E31" s="3" t="inlineStr"/>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>Closure evidence: client/src/pages/DashboardPage.tsx line 46 calls
+/api/my-studies/export. server/routes.ts line 1491 implements the
+endpoint. Pulled forward into pre-COLA per user instruction.</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>session 299e9a73 turn 5, ~2026-04-28.
+---</t>
+        </is>
+      </c>
+      <c r="H31" s="3" t="inlineStr"/>
+    </row>
+    <row r="32" ht="90" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Rotate GitHub PAT (because old PAT was committed in SESSION_HANDOFF files)</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr"/>
+      <c r="D32" s="2" t="inlineStr"/>
+      <c r="E32" s="2" t="inlineStr"/>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Closure evidence: no ghp_* or github_pat_* patterns in current
+SESSION_HANDOFF.md or SESSION_HANDOFF-2.md as of 2026-05-01.</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>session 299e9a73, ~2026-04-28.
+---</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33" ht="90" customHeight="1">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>C6</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>VeritaPolicy service-line filtering removed (formerly #4)</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr"/>
+      <c r="D33" s="3" t="inlineStr"/>
+      <c r="E33" s="3" t="inlineStr"/>
+      <c r="F33" s="3" t="inlineStr">
         <is>
           <t>Closure rationale (operator decision 2026-05-10): Keep all
 VeritaPolicy rows. CFR-only references with no accreditor reference
@@ -2096,29 +2042,29 @@
 report misread the design intent.</t>
         </is>
       </c>
-      <c r="G30" s="2" t="inlineStr">
+      <c r="G33" s="3" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H30" s="2" t="inlineStr"/>
-    </row>
-    <row r="31" ht="90" customHeight="1">
-      <c r="A31" s="3" t="inlineStr">
+      <c r="H33" s="3" t="inlineStr"/>
+    </row>
+    <row r="34" ht="90" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
         <is>
           <t>C7</t>
         </is>
       </c>
-      <c r="B31" s="3" t="inlineStr">
+      <c r="B34" s="2" t="inlineStr">
         <is>
           <t>CLIA number format validation (formerly #13)</t>
         </is>
       </c>
-      <c r="C31" s="3" t="inlineStr"/>
-      <c r="D31" s="3" t="inlineStr"/>
-      <c r="E31" s="3" t="inlineStr"/>
-      <c r="F31" s="3" t="inlineStr">
+      <c r="C34" s="2" t="inlineStr"/>
+      <c r="D34" s="2" t="inlineStr"/>
+      <c r="E34" s="2" t="inlineStr"/>
+      <c r="F34" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: shared/validateClia.ts defines CLIA_REGEX =
 /^\d{2}D\d{7}$/ (line 24), validateClia() helper with whitespace
@@ -2129,30 +2075,30 @@
 shape exists and behaves as specified.</t>
         </is>
       </c>
-      <c r="G31" s="3" t="inlineStr">
+      <c r="G34" s="2" t="inlineStr">
         <is>
           <t>Agent verification 2026-05-10 via grep + file read.
 Operator confirmed shipped 2026-05-10.
 ---</t>
         </is>
       </c>
-      <c r="H31" s="3" t="inlineStr"/>
-    </row>
-    <row r="32" ht="90" customHeight="1">
-      <c r="A32" s="2" t="inlineStr">
+      <c r="H34" s="2" t="inlineStr"/>
+    </row>
+    <row r="35" ht="90" customHeight="1">
+      <c r="A35" s="3" t="inlineStr">
         <is>
           <t>C8</t>
         </is>
       </c>
-      <c r="B32" s="2" t="inlineStr">
+      <c r="B35" s="3" t="inlineStr">
         <is>
           <t>VeritaMap lab-wide menu toggle (formerly #19)</t>
         </is>
       </c>
-      <c r="C32" s="2" t="inlineStr"/>
-      <c r="D32" s="2" t="inlineStr"/>
-      <c r="E32" s="2" t="inlineStr"/>
-      <c r="F32" s="2" t="inlineStr">
+      <c r="C35" s="3" t="inlineStr"/>
+      <c r="D35" s="3" t="inlineStr"/>
+      <c r="E35" s="3" t="inlineStr"/>
+      <c r="F35" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: client/src/pages/VeritaMapLabwidePage.tsx
 exists and implements the labwide read-only union view. Route is
@@ -2162,59 +2108,59 @@
 parking lot plan (read-only union view, per-session toggle) shipped.</t>
         </is>
       </c>
-      <c r="G32" s="2" t="inlineStr">
+      <c r="G35" s="3" t="inlineStr">
         <is>
           <t>Agent verification 2026-05-10 via grep + file read.
 Operator confirmed shipped 2026-05-10.
 ---</t>
         </is>
       </c>
-      <c r="H32" s="2" t="inlineStr"/>
-    </row>
-    <row r="33" ht="90" customHeight="1">
-      <c r="A33" s="3" t="inlineStr">
+      <c r="H35" s="3" t="inlineStr"/>
+    </row>
+    <row r="36" ht="90" customHeight="1">
+      <c r="A36" s="2" t="inlineStr">
         <is>
           <t>C9</t>
         </is>
       </c>
-      <c r="B33" s="3" t="inlineStr">
+      <c r="B36" s="2" t="inlineStr">
         <is>
           <t>Tier-1 smoke test checklist (formerly #6)</t>
         </is>
       </c>
-      <c r="C33" s="3" t="inlineStr"/>
-      <c r="D33" s="3" t="inlineStr"/>
-      <c r="E33" s="3" t="inlineStr"/>
-      <c r="F33" s="3" t="inlineStr">
+      <c r="C36" s="2" t="inlineStr"/>
+      <c r="D36" s="2" t="inlineStr"/>
+      <c r="E36" s="2" t="inlineStr"/>
+      <c r="F36" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: docs/smoke-test-tier1.md documents the Tier-1
 smoke-test process and post-deploy verification steps. Shipped via
 PR #81 as part of the 2026-05-10 wave.</t>
         </is>
       </c>
-      <c r="G33" s="3" t="inlineStr">
+      <c r="G36" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H33" s="3" t="inlineStr"/>
-    </row>
-    <row r="34" ht="90" customHeight="1">
-      <c r="A34" s="2" t="inlineStr">
+      <c r="H36" s="2" t="inlineStr"/>
+    </row>
+    <row r="37" ht="90" customHeight="1">
+      <c r="A37" s="3" t="inlineStr">
         <is>
           <t>C10</t>
         </is>
       </c>
-      <c r="B34" s="2" t="inlineStr">
+      <c r="B37" s="3" t="inlineStr">
         <is>
           <t>Per-module gating (formerly #7)</t>
         </is>
       </c>
-      <c r="C34" s="2" t="inlineStr"/>
-      <c r="D34" s="2" t="inlineStr"/>
-      <c r="E34" s="2" t="inlineStr"/>
-      <c r="F34" s="2" t="inlineStr">
+      <c r="C37" s="3" t="inlineStr"/>
+      <c r="D37" s="3" t="inlineStr"/>
+      <c r="E37" s="3" t="inlineStr"/>
+      <c r="F37" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: Client-side useIsReadOnly module keys wired
 on client/src/pages/VeritaPolicyAppPage.tsx and
@@ -2229,29 +2175,29 @@
 PR #76.</t>
         </is>
       </c>
-      <c r="G34" s="2" t="inlineStr">
+      <c r="G37" s="3" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H34" s="2" t="inlineStr"/>
-    </row>
-    <row r="35" ht="90" customHeight="1">
-      <c r="A35" s="3" t="inlineStr">
+      <c r="H37" s="3" t="inlineStr"/>
+    </row>
+    <row r="38" ht="90" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
         <is>
           <t>C11</t>
         </is>
       </c>
-      <c r="B35" s="3" t="inlineStr">
+      <c r="B38" s="2" t="inlineStr">
         <is>
           <t>VeritaStock shipped copy (formerly #8)</t>
         </is>
       </c>
-      <c r="C35" s="3" t="inlineStr"/>
-      <c r="D35" s="3" t="inlineStr"/>
-      <c r="E35" s="3" t="inlineStr"/>
-      <c r="F35" s="3" t="inlineStr">
+      <c r="C38" s="2" t="inlineStr"/>
+      <c r="D38" s="2" t="inlineStr"/>
+      <c r="E38" s="2" t="inlineStr"/>
+      <c r="F38" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: client/src/pages/ArticleInventoryManagementPage.tsx
 line 305 footer reads "platform that includes VeritaStock™" instead
@@ -2259,29 +2205,29 @@
 on /resources/laboratory-inventory-management. Shipped via PR #75.</t>
         </is>
       </c>
-      <c r="G35" s="3" t="inlineStr">
+      <c r="G38" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H35" s="3" t="inlineStr"/>
-    </row>
-    <row r="36" ht="90" customHeight="1">
-      <c r="A36" s="2" t="inlineStr">
+      <c r="H38" s="2" t="inlineStr"/>
+    </row>
+    <row r="39" ht="90" customHeight="1">
+      <c r="A39" s="3" t="inlineStr">
         <is>
           <t>C12</t>
         </is>
       </c>
-      <c r="B36" s="2" t="inlineStr">
+      <c r="B39" s="3" t="inlineStr">
         <is>
           <t>Admin report one-row-per-lab (formerly #14)</t>
         </is>
       </c>
-      <c r="C36" s="2" t="inlineStr"/>
-      <c r="D36" s="2" t="inlineStr"/>
-      <c r="E36" s="2" t="inlineStr"/>
-      <c r="F36" s="2" t="inlineStr">
+      <c r="C39" s="3" t="inlineStr"/>
+      <c r="D39" s="3" t="inlineStr"/>
+      <c r="E39" s="3" t="inlineStr"/>
+      <c r="F39" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: /api/admin/report rewritten in
 server/routes.ts (~line 595) to LEFT JOIN labs on
@@ -2296,56 +2242,56 @@
 prerequisite, not a code bug). Shipped via PR #85.</t>
         </is>
       </c>
-      <c r="G36" s="2" t="inlineStr">
+      <c r="G39" s="3" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H36" s="2" t="inlineStr"/>
-    </row>
-    <row r="37" ht="90" customHeight="1">
-      <c r="A37" s="3" t="inlineStr">
+      <c r="H39" s="3" t="inlineStr"/>
+    </row>
+    <row r="40" ht="90" customHeight="1">
+      <c r="A40" s="2" t="inlineStr">
         <is>
           <t>C14</t>
         </is>
       </c>
-      <c r="B37" s="3" t="inlineStr">
+      <c r="B40" s="2" t="inlineStr">
         <is>
           <t>UI relabel "CLIA TEa" -&gt; "Lab-Set Internal Goal" (formerly #1)</t>
         </is>
       </c>
-      <c r="C37" s="3" t="inlineStr"/>
-      <c r="D37" s="3" t="inlineStr"/>
-      <c r="E37" s="3" t="inlineStr"/>
-      <c r="F37" s="3" t="inlineStr">
+      <c r="C40" s="2" t="inlineStr"/>
+      <c r="D40" s="2" t="inlineStr"/>
+      <c r="E40" s="2" t="inlineStr"/>
+      <c r="F40" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: Shipped across four PRs over 2026-05-10.</t>
         </is>
       </c>
-      <c r="G37" s="3" t="inlineStr">
+      <c r="G40" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H37" s="3" t="inlineStr"/>
-    </row>
-    <row r="38" ht="90" customHeight="1">
-      <c r="A38" s="2" t="inlineStr">
+      <c r="H40" s="2" t="inlineStr"/>
+    </row>
+    <row r="41" ht="90" customHeight="1">
+      <c r="A41" s="3" t="inlineStr">
         <is>
           <t>C13</t>
         </is>
       </c>
-      <c r="B38" s="2" t="inlineStr">
+      <c r="B41" s="3" t="inlineStr">
         <is>
           <t>WSLH PT vendor (formerly #15)</t>
         </is>
       </c>
-      <c r="C38" s="2" t="inlineStr"/>
-      <c r="D38" s="2" t="inlineStr"/>
-      <c r="E38" s="2" t="inlineStr"/>
-      <c r="F38" s="2" t="inlineStr">
+      <c r="C41" s="3" t="inlineStr"/>
+      <c r="D41" s="3" t="inlineStr"/>
+      <c r="E41" s="3" t="inlineStr"/>
+      <c r="F41" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: Shipped 2026-05-10 via PR #79 (merge commit
 eeebc6e; merged after rebase to resolve a server/db.ts collision
@@ -2363,64 +2309,64 @@
 'WSLH' is the post-deploy success signal. Shipped via PR #79.</t>
         </is>
       </c>
-      <c r="G38" s="2" t="inlineStr">
+      <c r="G41" s="3" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H38" s="2" t="inlineStr"/>
-    </row>
-    <row r="39" ht="90" customHeight="1">
-      <c r="A39" s="3" t="inlineStr">
+      <c r="H41" s="3" t="inlineStr"/>
+    </row>
+    <row r="42" ht="90" customHeight="1">
+      <c r="A42" s="2" t="inlineStr">
         <is>
           <t>C15</t>
         </is>
       </c>
-      <c r="B39" s="3" t="inlineStr">
+      <c r="B42" s="2" t="inlineStr">
         <is>
           <t>VeritaStock lot tracking + expiration + reorder alerts (formerly #21)</t>
         </is>
       </c>
-      <c r="C39" s="3" t="inlineStr"/>
-      <c r="D39" s="3" t="inlineStr"/>
-      <c r="E39" s="3" t="inlineStr"/>
-      <c r="F39" s="3" t="inlineStr">
+      <c r="C42" s="2" t="inlineStr"/>
+      <c r="D42" s="2" t="inlineStr"/>
+      <c r="E42" s="2" t="inlineStr"/>
+      <c r="F42" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: VeritaStock™ shipped the bench-level inventory
 features the Perplexity competitor analysis identified as a gap:</t>
         </is>
       </c>
-      <c r="G39" s="3" t="inlineStr">
+      <c r="G42" s="2" t="inlineStr">
         <is>
           <t>Originally Perplexity competitor analysis 2026-05-10.
 Audit 2026-05-21 confirmed the feature set ships today.
 ---</t>
         </is>
       </c>
-      <c r="H39" s="3" t="inlineStr"/>
-    </row>
-    <row r="40" ht="90" customHeight="1">
-      <c r="A40" s="2" t="inlineStr">
+      <c r="H42" s="2" t="inlineStr"/>
+    </row>
+    <row r="43" ht="90" customHeight="1">
+      <c r="A43" s="3" t="inlineStr">
         <is>
           <t>C16</t>
         </is>
       </c>
-      <c r="B40" s="2" t="inlineStr">
+      <c r="B43" s="3" t="inlineStr">
         <is>
           <t>PAL studies guided workflow (formerly #23)</t>
         </is>
       </c>
-      <c r="C40" s="2" t="inlineStr"/>
-      <c r="D40" s="2" t="inlineStr"/>
-      <c r="E40" s="2" t="inlineStr"/>
-      <c r="F40" s="2" t="inlineStr">
+      <c r="C43" s="3" t="inlineStr"/>
+      <c r="D43" s="3" t="inlineStr"/>
+      <c r="E43" s="3" t="inlineStr"/>
+      <c r="F43" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: VeritaCheck™ already ships the Precision /
 Accuracy / Linearity (PAL) study set under EP-protocol naming:</t>
         </is>
       </c>
-      <c r="G40" s="2" t="inlineStr">
+      <c r="G43" s="3" t="inlineStr">
         <is>
           <t>Originally Perplexity competitor analysis 2026-05-10.
 Audit 2026-05-21 confirmed the EP studies cover the PAL framing in
@@ -2428,23 +2374,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H40" s="2" t="inlineStr"/>
-    </row>
-    <row r="41" ht="90" customHeight="1">
-      <c r="A41" s="3" t="inlineStr">
+      <c r="H43" s="3" t="inlineStr"/>
+    </row>
+    <row r="44" ht="90" customHeight="1">
+      <c r="A44" s="2" t="inlineStr">
         <is>
           <t>C17</t>
         </is>
       </c>
-      <c r="B41" s="3" t="inlineStr">
+      <c r="B44" s="2" t="inlineStr">
         <is>
           <t>Source-grounded 21/29/45 CFR + 42 CFR 482-485 (formerly #26)</t>
         </is>
       </c>
-      <c r="C41" s="3" t="inlineStr"/>
-      <c r="D41" s="3" t="inlineStr"/>
-      <c r="E41" s="3" t="inlineStr"/>
-      <c r="F41" s="3" t="inlineStr">
+      <c r="C44" s="2" t="inlineStr"/>
+      <c r="D44" s="2" t="inlineStr"/>
+      <c r="E44" s="2" t="inlineStr"/>
+      <c r="F44" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #301 (commit 8c27806, merged 2026-05-21)
 source-grounded the 74 remaining non-493 entries in
@@ -2452,29 +2398,29 @@
 shipped:</t>
         </is>
       </c>
-      <c r="G41" s="3" t="inlineStr">
+      <c r="G44" s="2" t="inlineStr">
         <is>
           <t>PR #301; tasks #18 in the in-session task tracker.
 ---</t>
         </is>
       </c>
-      <c r="H41" s="3" t="inlineStr"/>
-    </row>
-    <row r="42" ht="90" customHeight="1">
-      <c r="A42" s="2" t="inlineStr">
+      <c r="H44" s="2" t="inlineStr"/>
+    </row>
+    <row r="45" ht="90" customHeight="1">
+      <c r="A45" s="3" t="inlineStr">
         <is>
           <t>C18</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
+      <c r="B45" s="3" t="inlineStr">
         <is>
           <t>VeritaPolicy "Non CLIA" chapter rename (formerly #3)</t>
         </is>
       </c>
-      <c r="C42" s="2" t="inlineStr"/>
-      <c r="D42" s="2" t="inlineStr"/>
-      <c r="E42" s="2" t="inlineStr"/>
-      <c r="F42" s="2" t="inlineStr">
+      <c r="C45" s="3" t="inlineStr"/>
+      <c r="D45" s="3" t="inlineStr"/>
+      <c r="E45" s="3" t="inlineStr"/>
+      <c r="F45" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #300 (commit 34d7707, merged 2026-05-21)
 renamed all 44 user-facing chapter labels in
@@ -2485,7 +2431,7 @@
 page.</t>
         </is>
       </c>
-      <c r="G42" s="2" t="inlineStr">
+      <c r="G45" s="3" t="inlineStr">
         <is>
           <t>CAP customer screenshot of the /veritapolicy chapter
 headers, 2026-05-01 evening. PR #300; tasks #17 in the in-session
@@ -2493,23 +2439,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H42" s="2" t="inlineStr"/>
-    </row>
-    <row r="43" ht="90" customHeight="1">
-      <c r="A43" s="3" t="inlineStr">
+      <c r="H45" s="3" t="inlineStr"/>
+    </row>
+    <row r="46" ht="90" customHeight="1">
+      <c r="A46" s="2" t="inlineStr">
         <is>
           <t>C19</t>
         </is>
       </c>
-      <c r="B43" s="3" t="inlineStr">
+      <c r="B46" s="2" t="inlineStr">
         <is>
           <t>VeritaStock department-scope toggle (formerly #31)</t>
         </is>
       </c>
-      <c r="C43" s="3" t="inlineStr"/>
-      <c r="D43" s="3" t="inlineStr"/>
-      <c r="E43" s="3" t="inlineStr"/>
-      <c r="F43" s="3" t="inlineStr">
+      <c r="C46" s="2" t="inlineStr"/>
+      <c r="D46" s="2" t="inlineStr"/>
+      <c r="E46" s="2" t="inlineStr"/>
+      <c r="F46" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #319 (commit d01f5fe, merged 2026-05-22)
 shipped the persistent dept-scope toggle on VeritaStockPage. A new
@@ -2520,7 +2466,7 @@
 workspace without re-filtering.</t>
         </is>
       </c>
-      <c r="G43" s="3" t="inlineStr">
+      <c r="G46" s="2" t="inlineStr">
         <is>
           <t>John, San Carlos lab, 2026-05-21. Same conversation that
 drove the vendor dropdown (PR #304), FILTERED VIEW banner (PR #305),
@@ -2528,23 +2474,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H43" s="3" t="inlineStr"/>
-    </row>
-    <row r="44" ht="90" customHeight="1">
-      <c r="A44" s="2" t="inlineStr">
+      <c r="H46" s="2" t="inlineStr"/>
+    </row>
+    <row r="47" ht="90" customHeight="1">
+      <c r="A47" s="3" t="inlineStr">
         <is>
           <t>C20</t>
         </is>
       </c>
-      <c r="B44" s="2" t="inlineStr">
+      <c r="B47" s="3" t="inlineStr">
         <is>
           <t>Primary-lab seat counting (formerly #12)</t>
         </is>
       </c>
-      <c r="C44" s="2" t="inlineStr"/>
-      <c r="D44" s="2" t="inlineStr"/>
-      <c r="E44" s="2" t="inlineStr"/>
-      <c r="F44" s="2" t="inlineStr">
+      <c r="C47" s="3" t="inlineStr"/>
+      <c r="D47" s="3" t="inlineStr"/>
+      <c r="E47" s="3" t="inlineStr"/>
+      <c r="F47" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: is_primary_lab INTEGER NOT NULL DEFAULT 0
 column was added to the lab_members table at db.ts:1276, with the
@@ -2555,7 +2501,7 @@
 is_primary_lab=1 ordering).</t>
         </is>
       </c>
-      <c r="G44" s="2" t="inlineStr">
+      <c r="G47" s="3" t="inlineStr">
         <is>
           <t>2026-05-07 multi-lab discussion. Build shipped as part
 of the Multi-Lab Tier 2 architecture work (Phase 3.x series, prior
@@ -2564,23 +2510,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H44" s="2" t="inlineStr"/>
-    </row>
-    <row r="45" ht="90" customHeight="1">
-      <c r="A45" s="3" t="inlineStr">
+      <c r="H47" s="3" t="inlineStr"/>
+    </row>
+    <row r="48" ht="90" customHeight="1">
+      <c r="A48" s="2" t="inlineStr">
         <is>
           <t>C21</t>
         </is>
       </c>
-      <c r="B45" s="3" t="inlineStr">
+      <c r="B48" s="2" t="inlineStr">
         <is>
           <t>Multi-lab pricing model — Option A (formerly #11)</t>
         </is>
       </c>
-      <c r="C45" s="3" t="inlineStr"/>
-      <c r="D45" s="3" t="inlineStr"/>
-      <c r="E45" s="3" t="inlineStr"/>
-      <c r="F45" s="3" t="inlineStr">
+      <c r="C48" s="2" t="inlineStr"/>
+      <c r="D48" s="2" t="inlineStr"/>
+      <c r="E48" s="2" t="inlineStr"/>
+      <c r="F48" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #322 (commit 0ccd925, merged 2026-05-22)
 added the customer-facing line to the pricing page that reflects
@@ -2593,7 +2539,7 @@
 Enterprise+ block, reads:</t>
         </is>
       </c>
-      <c r="G45" s="3" t="inlineStr">
+      <c r="G48" s="2" t="inlineStr">
         <is>
           <t>2026-05-07 multi-lab discussion (Lisa Veri's
 canonical-case session). PR #322 (initial build); softening PR
@@ -2602,30 +2548,30 @@
 ---</t>
         </is>
       </c>
-      <c r="H45" s="3" t="inlineStr"/>
-    </row>
-    <row r="46" ht="90" customHeight="1">
-      <c r="A46" s="2" t="inlineStr">
+      <c r="H48" s="2" t="inlineStr"/>
+    </row>
+    <row r="49" ht="90" customHeight="1">
+      <c r="A49" s="3" t="inlineStr">
         <is>
           <t>C22</t>
         </is>
       </c>
-      <c r="B46" s="2" t="inlineStr">
+      <c r="B49" s="3" t="inlineStr">
         <is>
           <t>VeritaOps cost-per-test module (formerly #10)</t>
         </is>
       </c>
-      <c r="C46" s="2" t="inlineStr"/>
-      <c r="D46" s="2" t="inlineStr"/>
-      <c r="E46" s="2" t="inlineStr"/>
-      <c r="F46" s="2" t="inlineStr">
+      <c r="C49" s="3" t="inlineStr"/>
+      <c r="D49" s="3" t="inlineStr"/>
+      <c r="E49" s="3" t="inlineStr"/>
+      <c r="F49" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: v1 of the VeritaOps Cost-Per-Reportable-Test
 (CPRT) module shipped across PR #325 through PR #330 on 2026-05-22.
 The module is feature-complete for the typical lab director workflow.</t>
         </is>
       </c>
-      <c r="G46" s="2" t="inlineStr">
+      <c r="G49" s="3" t="inlineStr">
         <is>
           <t>This thread, 2026-05-07 12:05 PM CDT, user message:
 "Parking lot: build an operations module for cost per test
@@ -2634,262 +2580,262 @@
 ---</t>
         </is>
       </c>
-      <c r="H46" s="2" t="inlineStr"/>
-    </row>
-    <row r="47" ht="90" customHeight="1">
-      <c r="A47" s="3" t="inlineStr">
+      <c r="H49" s="3" t="inlineStr"/>
+    </row>
+    <row r="50" ht="90" customHeight="1">
+      <c r="A50" s="2" t="inlineStr">
         <is>
           <t>C23</t>
         </is>
       </c>
-      <c r="B47" s="3" t="inlineStr">
+      <c r="B50" s="2" t="inlineStr">
         <is>
           <t>CCL lab name visual disambiguation in lab switcher (formerly #34)</t>
         </is>
       </c>
-      <c r="C47" s="3" t="inlineStr"/>
-      <c r="D47" s="3" t="inlineStr">
+      <c r="C50" s="2" t="inlineStr"/>
+      <c r="D50" s="2" t="inlineStr">
         <is>
           <t>XS (under 1 day, actual)</t>
         </is>
       </c>
-      <c r="E47" s="3" t="inlineStr">
+      <c r="E50" s="2" t="inlineStr">
         <is>
           <t>Low — cosmetic; only mattered when Lisa or Michael picked the wrong lab from...</t>
         </is>
       </c>
-      <c r="F47" s="3" t="inlineStr">
+      <c r="F50" s="2" t="inlineStr">
         <is>
           <t>Effort: XS (under 1 day, actual)
 Importance: Low — cosmetic; only mattered when Lisa or Michael picked the wrong lab from the dropdown.</t>
         </is>
       </c>
-      <c r="G47" s="3" t="inlineStr">
+      <c r="G50" s="2" t="inlineStr">
         <is>
           <t>flagged 2026-05-23 immediately after provisioning Lisa's CCL lab; closed 2026-05-24.
 ---</t>
         </is>
       </c>
-      <c r="H47" s="3" t="inlineStr"/>
-    </row>
-    <row r="48" ht="90" customHeight="1">
-      <c r="A48" s="2" t="inlineStr">
+      <c r="H50" s="2" t="inlineStr"/>
+    </row>
+    <row r="51" ht="90" customHeight="1">
+      <c r="A51" s="3" t="inlineStr">
         <is>
           <t>C24</t>
         </is>
       </c>
-      <c r="B48" s="2" t="inlineStr">
+      <c r="B51" s="3" t="inlineStr">
         <is>
           <t>VC Unlimited Y1/Y2 price disclosure UX (formerly #35)</t>
         </is>
       </c>
-      <c r="C48" s="2" t="inlineStr"/>
-      <c r="D48" s="2" t="inlineStr">
+      <c r="C51" s="3" t="inlineStr"/>
+      <c r="D51" s="3" t="inlineStr">
         <is>
           <t>XS (under 1 day, actual)</t>
         </is>
       </c>
-      <c r="E48" s="2" t="inlineStr">
+      <c r="E51" s="3" t="inlineStr">
         <is>
           <t>Low when shipped (proactive, no customer complaint yet) — but high if a procu...</t>
         </is>
       </c>
-      <c r="F48" s="2" t="inlineStr">
+      <c r="F51" s="3" t="inlineStr">
         <is>
           <t>Effort: XS (under 1 day, actual)
 Importance: Low when shipped (proactive, no customer complaint yet) — but high if a procurement reviewer later disputes the $499 renewal as undisclosed.</t>
         </is>
       </c>
-      <c r="G48" s="2" t="inlineStr">
+      <c r="G51" s="3" t="inlineStr">
         <is>
           <t>Pricing rebuild 2026-05-23; closed 2026-05-24 proactively before any customer dispute.
 ---</t>
         </is>
       </c>
-      <c r="H48" s="2" t="inlineStr"/>
-    </row>
-    <row r="49" ht="90" customHeight="1">
-      <c r="A49" s="3" t="inlineStr">
+      <c r="H51" s="3" t="inlineStr"/>
+    </row>
+    <row r="52" ht="90" customHeight="1">
+      <c r="A52" s="2" t="inlineStr">
         <is>
           <t>C25</t>
         </is>
       </c>
-      <c r="B49" s="3" t="inlineStr">
+      <c r="B52" s="2" t="inlineStr">
         <is>
           <t>VeritaQC Phase 1 (Levey-Jennings + Westgard live engine) (formerly #20)</t>
         </is>
       </c>
-      <c r="C49" s="3" t="inlineStr"/>
-      <c r="D49" s="3" t="inlineStr">
+      <c r="C52" s="2" t="inlineStr"/>
+      <c r="D52" s="2" t="inlineStr">
         <is>
           <t>L (about 5 days end-to-end, actual: Phase 0 schema → Phase 1A evaluator → 1B...</t>
         </is>
       </c>
-      <c r="E49" s="3" t="inlineStr">
+      <c r="E52" s="2" t="inlineStr">
         <is>
           <t>High — largest single gap vs myLabCompliance.io per Perplexity competitor ana...</t>
         </is>
       </c>
-      <c r="F49" s="3" t="inlineStr">
+      <c r="F52" s="2" t="inlineStr">
         <is>
           <t>Effort: L (about 5 days end-to-end, actual: Phase 0 schema → Phase 1A evaluator → 1B entry UI → 1C daily review → 1D monthly PDF + attestation)
 Importance: High — largest single gap vs myLabCompliance.io per Perplexity competitor analysis; promotes VeritaAssure from documentation tool to lab operations platform.</t>
         </is>
       </c>
-      <c r="G49" s="3" t="inlineStr">
+      <c r="G52" s="2" t="inlineStr">
         <is>
           <t>Perplexity competitor analysis 2026-05-10. Scoping confirmed via the build_phase1_mockup.py iterations 2026-05-24. Shipped 2026-05-25.
 ---</t>
         </is>
       </c>
-      <c r="H49" s="3" t="inlineStr"/>
-    </row>
-    <row r="50" ht="90" customHeight="1">
-      <c r="A50" s="2" t="inlineStr">
+      <c r="H52" s="2" t="inlineStr"/>
+    </row>
+    <row r="53" ht="90" customHeight="1">
+      <c r="A53" s="3" t="inlineStr">
         <is>
           <t>C26</t>
         </is>
       </c>
-      <c r="B50" s="2" t="inlineStr">
+      <c r="B53" s="3" t="inlineStr">
         <is>
           <t>VeritaLab CMS-116 application support + state licensing registry (formerly #22)</t>
         </is>
       </c>
-      <c r="C50" s="2" t="inlineStr"/>
-      <c r="D50" s="2" t="inlineStr">
+      <c r="C53" s="3" t="inlineStr"/>
+      <c r="D53" s="3" t="inlineStr">
         <is>
           <t>M (1-2 weeks for v1, actual)</t>
         </is>
       </c>
-      <c r="E50" s="2" t="inlineStr">
+      <c r="E53" s="3" t="inlineStr">
         <is>
           <t>Medium — competitor parity (myLabCompliance.io) plus useful at lab startup an...</t>
         </is>
       </c>
-      <c r="F50" s="2" t="inlineStr">
+      <c r="F53" s="3" t="inlineStr">
         <is>
           <t>Effort: M (1-2 weeks for v1, actual)
 Importance: Medium — competitor parity (myLabCompliance.io) plus useful at lab startup and at certificate-type changes.</t>
         </is>
       </c>
-      <c r="G50" s="2" t="inlineStr">
+      <c r="G53" s="3" t="inlineStr">
         <is>
           <t>Perplexity competitor analysis (myLabCompliance.io), 2026-05-10. Reclassified as a VeritaLab extension 2026-05-25. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H50" s="2" t="inlineStr"/>
-    </row>
-    <row r="51" ht="90" customHeight="1">
-      <c r="A51" s="3" t="inlineStr">
+      <c r="H53" s="3" t="inlineStr"/>
+    </row>
+    <row r="54" ht="90" customHeight="1">
+      <c r="A54" s="2" t="inlineStr">
         <is>
           <t>C27</t>
         </is>
       </c>
-      <c r="B51" s="3" t="inlineStr">
+      <c r="B54" s="2" t="inlineStr">
         <is>
           <t>Active vs view-only seat split (formerly #33)</t>
         </is>
       </c>
-      <c r="C51" s="3" t="inlineStr"/>
-      <c r="D51" s="3" t="inlineStr">
+      <c r="C54" s="2" t="inlineStr"/>
+      <c r="D54" s="2" t="inlineStr">
         <is>
           <t>M (~1 week of engineering, actual: shipped in a single multi-PR session)</t>
         </is>
       </c>
-      <c r="E51" s="3" t="inlineStr">
+      <c r="E54" s="2" t="inlineStr">
         <is>
           <t>Medium — closed the gap between /pricing copy and product behavior; gives sal...</t>
         </is>
       </c>
-      <c r="F51" s="3" t="inlineStr">
+      <c r="F54" s="2" t="inlineStr">
         <is>
           <t>Effort: M (~1 week of engineering, actual: shipped in a single multi-PR session)
 Importance: Medium — closed the gap between /pricing copy and product behavior; gives sales a clean answer for "do you charge for our medical director?"</t>
         </is>
       </c>
-      <c r="G51" s="3" t="inlineStr">
+      <c r="G54" s="2" t="inlineStr">
         <is>
           <t>Pricing analysis doc Decision 3 (2026-05-21); MEDIUM scenario revised 2026-05-29 to retire the "unlimited view-only" claim. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H51" s="3" t="inlineStr"/>
-    </row>
-    <row r="52" ht="90" customHeight="1">
-      <c r="A52" s="2" t="inlineStr">
+      <c r="H54" s="2" t="inlineStr"/>
+    </row>
+    <row r="55" ht="90" customHeight="1">
+      <c r="A55" s="3" t="inlineStr">
         <is>
           <t>C28</t>
         </is>
       </c>
-      <c r="B52" s="2" t="inlineStr">
+      <c r="B55" s="3" t="inlineStr">
         <is>
           <t>"Why VeritaCheck" comparative one-pager (formerly #37)</t>
         </is>
       </c>
-      <c r="C52" s="2" t="inlineStr"/>
-      <c r="D52" s="2" t="inlineStr">
+      <c r="C55" s="3" t="inlineStr"/>
+      <c r="D55" s="3" t="inlineStr">
         <is>
           <t>S (one design pass + four claim paragraphs + PDF + matching marketing-site pa...</t>
         </is>
       </c>
-      <c r="E52" s="2" t="inlineStr">
+      <c r="E55" s="3" t="inlineStr">
         <is>
           <t>Medium — closed a positioning gap surfaced by six COLA conference attendees a...</t>
         </is>
       </c>
-      <c r="F52" s="2" t="inlineStr">
+      <c r="F55" s="3" t="inlineStr">
         <is>
           <t>Effort: S (one design pass + four claim paragraphs + PDF + matching marketing-site page, actual)
 Importance: Medium — closed a positioning gap surfaced by six COLA conference attendees attached to a legacy verification tool; converts product-quality advantage into a leave-behind Lisa can hand out.</t>
         </is>
       </c>
-      <c r="G52" s="2" t="inlineStr">
+      <c r="G55" s="3" t="inlineStr">
         <is>
           <t>2026-05-11 / 2026-05-12 conference notes review with Michael. Conference attendees (Whitehead, Odegard, Othman, Molinelli, Kyle, Allred) expressed interest in equivalent / superior product. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H52" s="2" t="inlineStr"/>
-    </row>
-    <row r="53" ht="90" customHeight="1">
-      <c r="A53" s="3" t="inlineStr">
+      <c r="H55" s="3" t="inlineStr"/>
+    </row>
+    <row r="56" ht="90" customHeight="1">
+      <c r="A56" s="2" t="inlineStr">
         <is>
           <t>C29</t>
         </is>
       </c>
-      <c r="B53" s="3" t="inlineStr">
+      <c r="B56" s="2" t="inlineStr">
         <is>
           <t>VeritaPolicy approval workflow — MediaLab functional mirror</t>
         </is>
       </c>
-      <c r="C53" s="3" t="inlineStr"/>
-      <c r="D53" s="3" t="inlineStr">
+      <c r="C56" s="2" t="inlineStr"/>
+      <c r="D56" s="2" t="inlineStr">
         <is>
           <t>XL (one focused session, 12 PRs landed)</t>
         </is>
       </c>
-      <c r="E53" s="3" t="inlineStr">
+      <c r="E56" s="2" t="inlineStr">
         <is>
           <t>High — replaces MediaLab Document Control ($752/$2,250 starting price, scalin...</t>
         </is>
       </c>
-      <c r="F53" s="3" t="inlineStr">
+      <c r="F56" s="2" t="inlineStr">
         <is>
           <t>Effort: XL (one focused session, 12 PRs landed)
 Importance: High — replaces MediaLab Document Control ($752/$2,250 starting price, scaling to $10K-$20K/yr at enterprise per Capterra public data) with an included VeritaPolicy feature; closes a real positioning gap and gives sales a direct comparator line.</t>
         </is>
       </c>
-      <c r="G53" s="3" t="inlineStr">
+      <c r="G56" s="2" t="inlineStr">
         <is>
           <t>Pricing strategy conversation 2026-05-29 (Michael: "I don't like bolt-ons; we should replicate this") → scoped 8 phases → shipped all 12 PRs in single session. Shipped 2026-05-29.
 ---</t>
         </is>
       </c>
-      <c r="H53" s="3" t="inlineStr"/>
+      <c r="H56" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H53"/>
+  <autoFilter ref="A1:H56"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
TASK: Close shipped-but-stale parking-lot items #53 and #47; sync xlsx
PLAN:
  1. #53 (VeritaCEU free-CE directory) -> C56, shipped as VeritaCEU phase 2 (#1410).
  2. #47 (hide unused sections) -> C57, shipped PR #1364; entry was stale.
  3. Re-run build_parking_lot_xlsx.py.

Self-check:
  - Both verified shipped/live; internal doc change; Gate 3 N/A.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PARKING_LOT.xlsx
+++ b/PARKING_LOT.xlsx
@@ -12,8 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RETIRED" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$58</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RETIRED'!$A$1:$H$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -975,7 +975,10 @@
       <c r="C11" s="3" t="inlineStr">
         <is>
           <t>Parked. Plan documented. Implementation deferred until trigger conditions met.
----</t>
+---
+_(item #50 closed 2026-09-28; shipped PR #1356, prod-verified, see C49 below)_
+---
+_(item #51 closed 2026-09-2...</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -1000,91 +1003,8 @@
       </c>
       <c r="H11" s="3" t="inlineStr"/>
     </row>
-    <row r="12" ht="90" customHeight="1">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>47</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Hide sections a lab does not use from a master list, to reduce clutter (prospect-requested)</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>SHIPPED (PR #1364, in origin/main; predates this session, entry was stale). Built as the VeritaDC (VeritaPolicy) Master List "Show only applicable" toggle in client/src/pages/VeritaPolicyAppPage.ts...</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>S-M (a few days to ~2 weeks depending on scope) — a lab-level visibility togg...</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>Medium-High — came straight from a live prospect today as an onboarding-frict...</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>Effort: S-M (a few days to ~2 weeks depending on scope) — a lab-level visibility toggle that hides not-applicable or unused sections from a master-list view. Smaller if it is a "hide N/A" filter on the existing VeritaDC master list, larger if it also spans VeritaScan domains.
-Importance: Medium-High — came straight from a live prospect today as an onboarding-friction point; a lab that does not run a service line should not have to wade past its requirements.</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-23 session, Michael relaying a prospect ask from a demo today.</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr"/>
-    </row>
-    <row r="13" ht="90" customHeight="1">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>53</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>VeritaCEU: curated free-continuing-education provider list (seed / reference)</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>Open, reference captured. Not started.</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>S (1-2 days to seed a curated provider list and surface it in VeritaCEU; XS t...</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>Low-Medium — quality-of-life for VeritaCEU users (find free CE fast); not blo...</t>
-        </is>
-      </c>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>Effort: S (1-2 days to seed a curated provider list and surface it in VeritaCEU; XS to just store the reference)
-Importance: Low-Medium — quality-of-life for VeritaCEU users (find free CE fast); not blocking any sale.</t>
-        </is>
-      </c>
-      <c r="G13" s="3" t="inlineStr">
-        <is>
-          <t>Jennifer Small (jennifer.small@lifepointhealth.net) email 2026-09-25, forwarded by Michael 2026-09-28 for the future CEU module.</t>
-        </is>
-      </c>
-      <c r="H13" s="3" t="inlineStr">
-        <is>
-          <t>Post-COLA. No customer urgency.
----</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:H13"/>
+  <autoFilter ref="A1:H11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1095,7 +1015,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H56"/>
+  <dimension ref="A1:H58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1153,24 +1073,24 @@
     <row r="2" ht="90" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>C55</t>
+          <t>C57</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>VeritaScan: let sites add their own custom questions (was #55)</t>
+          <t>Hide sections a lab does not use from a master list (was #47)</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr"/>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>was M / Importance: Medium-High</t>
+          <t>was S-M / Importance: Medium-High (prospect-requested)</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Effort: was M / Importance: Medium-High</t>
+          <t>Effort: was S-M / Importance: Medium-High (prospect-requested)</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
@@ -1179,24 +1099,24 @@
     <row r="3" ht="90" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>C54</t>
+          <t>C56</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>VeritaQC: at-entry warning when a QC point is outside 2 SD (was #56)</t>
+          <t>VeritaCEU: curated free continuing-education provider list (was #53)</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr"/>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>was S-M (shipped S) / Importance: High</t>
+          <t>was S / Importance: Low-Medium</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Effort: was S-M (shipped S) / Importance: High</t>
+          <t>Effort: was S / Importance: Low-Medium</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr"/>
@@ -1205,24 +1125,24 @@
     <row r="4" ht="90" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>C53</t>
+          <t>C55</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>VeritaTrack: quarterly task loaded as monthly until re-saved (was #54)</t>
+          <t>VeritaScan: let sites add their own custom questions (was #55)</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr"/>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>was S / Importance: Medium</t>
+          <t>was M / Importance: Medium-High</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Effort: was S / Importance: Medium</t>
+          <t>Effort: was M / Importance: Medium-High</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr"/>
@@ -1231,24 +1151,24 @@
     <row r="5" ht="90" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>C52</t>
+          <t>C54</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>VeritaResponse internal NCE / non-conforming event (was #36)</t>
+          <t>VeritaQC: at-entry warning when a QC point is outside 2 SD (was #56)</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr"/>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>was L (shipped as MEDIUM) / Importance: High</t>
+          <t>was S-M (shipped S) / Importance: High</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Effort: was L (shipped as MEDIUM) / Importance: High</t>
+          <t>Effort: was S-M (shipped S) / Importance: High</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr"/>
@@ -1257,24 +1177,24 @@
     <row r="6" ht="90" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>C49</t>
+          <t>C53</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Competency "assessed this cycle" cadence-aware window (was #50)</t>
+          <t>VeritaTrack: quarterly task loaded as monthly until re-saved (was #54)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr"/>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>was S-M / Importance: Medium</t>
+          <t>was S / Importance: Medium</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Effort: was S-M / Importance: Medium</t>
+          <t>Effort: was S / Importance: Medium</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
@@ -1283,24 +1203,24 @@
     <row r="7" ht="90" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>C50</t>
+          <t>C52</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>VeritaTrack task owner + owner-only reminder routing (was #51)</t>
+          <t>VeritaResponse internal NCE / non-conforming event (was #36)</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr"/>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>was S-M / Importance: Medium</t>
+          <t>was L (shipped as MEDIUM) / Importance: High</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Effort: was S-M / Importance: Medium</t>
+          <t>Effort: was L (shipped as MEDIUM) / Importance: High</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr"/>
@@ -1309,24 +1229,24 @@
     <row r="8" ht="90" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>C51</t>
+          <t>C49</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Designate Medical Director by picking a lab member (was #52, core)</t>
+          <t>Competency "assessed this cycle" cadence-aware window (was #50)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr"/>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>was S-M / Importance: Medium-High</t>
+          <t>was S-M / Importance: Medium</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Effort: was S-M / Importance: Medium-High</t>
+          <t>Effort: was S-M / Importance: Medium</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
@@ -1335,24 +1255,24 @@
     <row r="9" ht="90" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>C47</t>
+          <t>C50</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Unregulated-analyte / Alternative Assessment (AAA) coverage (was #18)</t>
+          <t>VeritaTrack task owner + owner-only reminder routing (was #51)</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr"/>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>was S (Phase 3) / Importance: Medium</t>
+          <t>was S-M / Importance: Medium</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Effort: was S (Phase 3) / Importance: Medium</t>
+          <t>Effort: was S-M / Importance: Medium</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr"/>
@@ -1361,24 +1281,24 @@
     <row r="10" ht="90" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>C48</t>
+          <t>C51</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>VeritaResponse post-survey deficiency module (was #17)</t>
+          <t>Designate Medical Director by picking a lab member (was #52, core)</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr"/>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>was XL / Importance: High</t>
+          <t>was S-M / Importance: Medium-High</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Effort: was XL / Importance: High</t>
+          <t>Effort: was S-M / Importance: Medium-High</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
@@ -1387,66 +1307,64 @@
     <row r="11" ht="90" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>C45</t>
+          <t>C47</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Unify coverage/competency recurrence helper (was #49) - closed as non-issue</t>
+          <t>Unregulated-analyte / Alternative Assessment (AAA) coverage (was #18)</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr"/>
-      <c r="D11" s="3" t="inlineStr"/>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>was S (Phase 3) / Importance: Medium</t>
+        </is>
+      </c>
       <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: Investigated 2026-09-24 before building. The coverage recurrence math (+6-month interval, signed-resets-to-missing, nextDueOn/overdue, isFailVerdict) is ALREADY single-source in server/veritacheckCoverage.ts (computeCoverageFrom). server/coverageReport.ts and the routes.ts coverage export do not recompute it; they consume the computed nextDueOn/overdue/status fields and apply small surface-specific presentation labels (deliberately different vocabularies per surface, so they should not be merged). The only truly identical duplicate is a one-line date formatter. The competency "owed" derivation is NOT the same cadence: competency follows the CLIA milestone schedule (initial / semiannual year 1 / annual, 42 CFR 493.1451(b)(8) and 493.1235), which is a different regulatory interval from the coverage 6-month rule (493.1281 / 493.1255) and must stay separate. No worthwhile extraction; merging the two cadences would be wrong. Closed 2026-09-24. (The year-1 competency-window refinement remains tracked separately as #50.)</t>
-        </is>
-      </c>
-      <c r="G11" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-24 session, "keep working" pass; scoped read-only, found no real duplication.
----</t>
-        </is>
-      </c>
+          <t>Effort: was S (Phase 3) / Importance: Medium</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr"/>
       <c r="H11" s="3" t="inlineStr"/>
     </row>
     <row r="12" ht="90" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>C46</t>
+          <t>C48</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Verified-users product-update send path (wrong-list incident fix)</t>
+          <t>VeritaResponse post-survey deficiency module (was #17)</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr"/>
-      <c r="D12" s="2" t="inlineStr"/>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>was XL / Importance: High</t>
+        </is>
+      </c>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: Shipped PR #1324 (merged 4e05506a, deploy ACTIVE). New POST /api/admin/users/send targets registered VeritaAssure account holders (the users table), never the Lab Director's Briefing subscriber list. Separate explicitly-named endpoint (not a flag with a dangerous default), account-holder email framing, excludes suppressed emails and RFC-reserved test domains, CC owner, dryRun + testTo previews. Public unsubscribe now upserts a suppression row so opt-outs are honored across both audiences. Live dryRun: 49 verified-user recipients vs 673 on the Briefing list. Receipts: scripts/verify-product-update-send.mts 24/24, tsc clean, rendered sample inspected. Fixes the fallout from the 2026-09-23/24 wrong-list send (a product update went to the 675-person Briefing list). Nothing sends without Michael's explicit "send it."</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-24 session; Michael selected this as the next build after the #41 close.
----</t>
-        </is>
-      </c>
+          <t>Effort: was XL / Importance: High</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr"/>
       <c r="H12" s="2" t="inlineStr"/>
     </row>
     <row r="13" ht="90" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>C44</t>
+          <t>C45</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Verify-script convention backfill (was #41) + audit matcher fix</t>
+          <t>Unify coverage/competency recurrence helper (was #49) - closed as non-issue</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr"/>
@@ -1454,12 +1372,12 @@
       <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: #41 was fully backfilled on 2026-06-13 (all 8 high-stakes scripts landed; see C30); it had only been mis-filed in OPEN. A 2026-09-24 re-audit initially reported 4 of 5 recent math/logic commits as missing a verify script, which was a FALSE POSITIVE: scripts/audit_verify_script_coverage.py matched only scripts/verify-*.js / .cjs, so it ignored the .mjs / .mts / .ts verify scripts the repo now ships (e.g. verify-ptcoag-multi.mts, verify-tea-criterion-format.mjs). Fixed the matcher to accept .js/.cjs/.mjs/.ts/.mts; re-run shows 5 of 5 covered, 0 debt. The convention is being followed. Closed 2026-09-24.</t>
+          <t>Closure evidence: Investigated 2026-09-24 before building. The coverage recurrence math (+6-month interval, signed-resets-to-missing, nextDueOn/overdue, isFailVerdict) is ALREADY single-source in server/veritacheckCoverage.ts (computeCoverageFrom). server/coverageReport.ts and the routes.ts coverage export do not recompute it; they consume the computed nextDueOn/overdue/status fields and apply small surface-specific presentation labels (deliberately different vocabularies per surface, so they should not be merged). The only truly identical duplicate is a one-line date formatter. The competency "owed" derivation is NOT the same cadence: competency follows the CLIA milestone schedule (initial / semiannual year 1 / annual, 42 CFR 493.1451(b)(8) and 493.1235), which is a different regulatory interval from the coverage 6-month rule (493.1281 / 493.1255) and must stay separate. No worthwhile extraction; merging the two cadences would be wrong. Closed 2026-09-24. (The year-1 competency-window refinement remains tracked separately as #50.)</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>2026-09-24 session, "keep working" pass; audit tooling bug found + fixed.
+          <t>2026-09-24 session, "keep working" pass; scoped read-only, found no real duplication.
 ---</t>
         </is>
       </c>
@@ -1468,12 +1386,12 @@
     <row r="14" ht="90" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>C43</t>
+          <t>C46</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>VeritaStaff instrument-centric (dual) assignment view</t>
+          <t>Verified-users product-update send path (wrong-list incident fix)</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr"/>
@@ -1481,12 +1399,12 @@
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1320. GET/PUT /staff/instruments/:id/employees (transpose of the per-employee endpoints); an "Assign by Instrument" dialog lets a director pick a test system or manual test and check off who runs it. Same staff_employee_instruments join, with the 42 CFR 493.1235(a) duty-change event emitted on newly-added pairs so both orientations trigger the same reassessment. GET verified live on SCAHC lab 2. Closed 2026-09-24.</t>
+          <t>Closure evidence: Shipped PR #1324 (merged 4e05506a, deploy ACTIVE). New POST /api/admin/users/send targets registered VeritaAssure account holders (the users table), never the Lab Director's Briefing subscriber list. Separate explicitly-named endpoint (not a flag with a dangerous default), account-holder email framing, excludes suppressed emails and RFC-reserved test domains, CC owner, dryRun + testTo previews. Public unsubscribe now upserts a suppression row so opt-outs are honored across both audiences. Live dryRun: 49 verified-user recipients vs 673 on the Briefing list. Receipts: scripts/verify-product-update-send.mts 24/24, tsc clean, rendered sample inspected. Fixes the fallout from the 2026-09-23/24 wrong-list send (a product update went to the 675-person Briefing list). Nothing sends without Michael's explicit "send it."</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 session, Michael ("in staff we should also give the dual view when assigning coverage to test systems or manual tests").
+          <t>2026-09-24 session; Michael selected this as the next build after the #41 close.
 ---</t>
         </is>
       </c>
@@ -1495,12 +1413,12 @@
     <row r="15" ht="90" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>C42</t>
+          <t>C44</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>VeritaComp coverage map (required-vs-assessed matrix, dual view)</t>
+          <t>Verify-script convention backfill (was #41) + audit matcher fix</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr"/>
@@ -1508,12 +1426,12 @@
       <c r="E15" s="3" t="inlineStr"/>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1319 (+ status layer PR #1316). /competency/owed returns per-item assessed (locked passing assessment this cycle on a covering method group) + per-employee CLIA status; CompetencyCoverageMap renders a By-employee / By-instrument matrix (Assessed / Owed / Overdue / Gap). Verified live on SCAHC lab 2 (owed 116, assessed 2, gaps 0). Completes #48 as the VeritaCheck-parity coverage map. Closed 2026-09-24.</t>
+          <t>Closure evidence: #41 was fully backfilled on 2026-06-13 (all 8 high-stakes scripts landed; see C30); it had only been mis-filed in OPEN. A 2026-09-24 re-audit initially reported 4 of 5 recent math/logic commits as missing a verify script, which was a FALSE POSITIVE: scripts/audit_verify_script_coverage.py matched only scripts/verify-*.js / .cjs, so it ignored the .mjs / .mts / .ts verify scripts the repo now ships (e.g. verify-ptcoag-multi.mts, verify-tea-criterion-format.mjs). Fixed the matcher to accept .js/.cjs/.mjs/.ts/.mts; re-run shows 5 of 5 covered, 0 debt. The convention is being followed. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>2026-09-24 session, Michael ("are we building the competencies to have a coverage map, same as veritacheck?" then "build it").
+          <t>2026-09-24 session, "keep working" pass; audit tooling bug found + fixed.
 ---</t>
         </is>
       </c>
@@ -1522,12 +1440,12 @@
     <row r="16" ht="90" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>C41</t>
+          <t>C43</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>VeritaCheck coverage recurrence (method comparison + cal-ver/linearity + reports)</t>
+          <t>VeritaStaff instrument-centric (dual) assignment view</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr"/>
@@ -1535,12 +1453,12 @@
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: PRs #1317 (method comparison), #1318 (cal-ver/linearity), #1321 (report Next-due columns). Periodic verification (correlation/method comparison 42 CFR 493.1281; cal-ver/linearity 42 CFR 493.1255; both 6-month) now recurs: a signed study banks the cycle and rolls to next-due = signed + 6 months instead of reading "done" forever. Status Missing/Failed/Completed-unsigned + a "Next due on" column on-screen and in both coverage exports; also credits the previously-ignored "correlation" study type. Root cause: computeCoverageFrom marked requirements done on mere existence, no date logic. Verified live on SCAHC lab 2 (101 correlations + 11 cal-ver rows now carry a next-due). Engine-level, all facilities. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1320. GET/PUT /staff/instruments/:id/employees (transpose of the per-employee endpoints); an "Assign by Instrument" dialog lets a director pick a test system or manual test and check off who runs it. Same staff_employee_instruments join, with the 42 CFR 493.1235(a) duty-change event emitted on newly-added pairs so both orientations trigger the same reassessment. GET verified live on SCAHC lab 2. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 session, Michael ("Look at San Carlos... they finished their last set of correlations (all 103) but their menu never reset").
+          <t>2026-09-24 session, Michael ("in staff we should also give the dual view when assigning coverage to test systems or manual tests").
 ---</t>
         </is>
       </c>
@@ -1549,12 +1467,12 @@
     <row r="17" ht="90" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>C40</t>
+          <t>C42</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>VeritaComp Competencies Owed derived from VeritaStaff, with gap detection (was #48)</t>
+          <t>VeritaComp coverage map (required-vs-assessed matrix, dual view)</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr"/>
@@ -1562,12 +1480,12 @@
       <c r="E17" s="3" t="inlineStr"/>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1314 (squash 2bcb0db9). GET /api/labs/:labId/competency/owed derives each VeritaStaff testing employee's owed competencies from their assigned instruments (staff_employee_instruments -&gt; veritamap_instruments + tests), on the CLIA timeline, and flags instruments not covered by any competency program as gaps. CompetenciesOwedSection renders it on the VeritaComp landing page. Reuses the shipped bridge + suggested-method-groups match rules; no new tables. Verified live on prod with real assignment data: 2 instruments assigned to a demo staffer produced owed=2, gaps=2 (HIGH, Technical Supervisor), then reverted cleanly. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1319 (+ status layer PR #1316). /competency/owed returns per-item assessed (locked passing assessment this cycle on a covering method group) + per-employee CLIA status; CompetencyCoverageMap renders a By-employee / By-instrument matrix (Assessed / Owed / Overdue / Gap). Verified live on SCAHC lab 2 (owed 116, assessed 2, gaps 0). Completes #48 as the VeritaCheck-parity coverage map. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>2026-09-23/24 session, Michael ("veritacomp bases what competencies they owe (currently untrue, but needs to be true)"). Option 1 (unify roster on VeritaStaff, match instruments by id).
+          <t>2026-09-24 session, Michael ("are we building the competencies to have a coverage map, same as veritacheck?" then "build it").
 ---</t>
         </is>
       </c>
@@ -1576,12 +1494,12 @@
     <row r="18" ht="90" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>C39</t>
+          <t>C41</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>VeritaScan line items can attach or link evidence (was #46)</t>
+          <t>VeritaCheck coverage recurrence (method comparison + cal-ver/linearity + reports)</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr"/>
@@ -1589,12 +1507,12 @@
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1312 (squash a1dda93d). VeritaScan scan checklist items now show linked evidence as chips (open link, remove) plus a writer "Link evidence" affordance whose picker links an existing VeritaDC/Library document; a shortcut deep-links to the Library for new (governed) documents. Reuses the already-shipped lab_documents + document_checklist_links + coverage endpoints (URL-pointer only, no file storage, no new tables). Browser-verified live on prod (scan 23): the affordance renders and the picker opens. Closed 2026-09-24.</t>
+          <t>Closure evidence: PRs #1317 (method comparison), #1318 (cal-ver/linearity), #1321 (report Next-due columns). Periodic verification (correlation/method comparison 42 CFR 493.1281; cal-ver/linearity 42 CFR 493.1255; both 6-month) now recurs: a signed study banks the cycle and rolls to next-due = signed + 6 months instead of reading "done" forever. Status Missing/Failed/Completed-unsigned + a "Next due on" column on-screen and in both coverage exports; also credits the previously-ignored "correlation" study type. Root cause: computeCoverageFrom marked requirements done on mere existence, no date logic. Verified live on SCAHC lab 2 (101 correlations + 11 cal-ver rows now carry a next-due). Engine-level, all facilities. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23 session, Michael. Recurring request. Companion: cross-module evidence display on the VeritaDC policy shipped in PR #1313 (by-target cross-links surfaced in the policy View modal, browser-verified live).
+          <t>2026-09-24 session, Michael ("Look at San Carlos... they finished their last set of correlations (all 103) but their menu never reset").
 ---</t>
         </is>
       </c>
@@ -1603,12 +1521,12 @@
     <row r="19" ht="90" customHeight="1">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>C38</t>
+          <t>C40</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>VeritaTrack calendar month cells expand to reveal hidden tasks (was #45)</t>
+          <t>VeritaComp Competencies Owed derived from VeritaStaff, with gap detection (was #48)</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr"/>
@@ -1616,12 +1534,12 @@
       <c r="E19" s="3" t="inlineStr"/>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: VeritaTrack CalendarView month cells with more than three tasks now expand in place (chevron, "+N more" toggling to "Show less", due dates), so no task is hidden with no path to it (client/src/pages/VeritaTrackAppPage.tsx CalendarView). Shipped 2026-09-23. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1314 (squash 2bcb0db9). GET /api/labs/:labId/competency/owed derives each VeritaStaff testing employee's owed competencies from their assigned instruments (staff_employee_instruments -&gt; veritamap_instruments + tests), on the CLIA timeline, and flags instruments not covered by any competency program as gaps. CompetenciesOwedSection renders it on the VeritaComp landing page. Reuses the shipped bridge + suggested-method-groups match rules; no new tables. Verified live on prod with real assignment data: 2 instruments assigned to a demo staffer produced owed=2, gaps=2 (HIGH, Technical Supervisor), then reverted cleanly. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>2026-09-23 session, Michael screenshot of the VeritaTrack calendar (lab 3, September cell).
+          <t>2026-09-23/24 session, Michael ("veritacomp bases what competencies they owe (currently untrue, but needs to be true)"). Option 1 (unify roster on VeritaStaff, match instruments by id).
 ---</t>
         </is>
       </c>
@@ -1630,12 +1548,12 @@
     <row r="20" ht="90" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>C37</t>
+          <t>C39</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Long Excel column headers no longer clip CFR citations (was #44)</t>
+          <t>VeritaScan line items can attach or link evidence (was #46)</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr"/>
@@ -1643,12 +1561,12 @@
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. The VeritaMap export derives the header row height from the longest wrapped header via headerRowHeight(headers, colWidths) (server/routes.ts:15935) instead of a fixed 20, so "Reference Range Attestation (42 CFR 493.1253)" and the other long headers print in full. No new code this session. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1312 (squash a1dda93d). VeritaScan scan checklist items now show linked evidence as chips (open link, remove) plus a writer "Link evidence" affordance whose picker links an existing VeritaDC/Library document; a shortcut deep-links to the Library for new (governed) documents. Reuses the already-shipped lab_documents + document_checklist_links + coverage endpoints (URL-pointer only, no file storage, no new tables). Browser-verified live on prod (scan 23): the affordance renders and the picker opens. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+          <t>2026-09-23 session, Michael. Recurring request. Companion: cross-module evidence display on the VeritaDC policy shipped in PR #1313 (by-target cross-links surfaced in the policy View modal, browser-verified live).
 ---</t>
         </is>
       </c>
@@ -1657,12 +1575,12 @@
     <row r="21" ht="90" customHeight="1">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>C36</t>
+          <t>C38</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>License stamp no longer clobbers the §6 header/footer or names the wrong lab (was #43)</t>
+          <t>VeritaTrack calendar month cells expand to reveal hidden tasks (was #45)</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr"/>
@@ -1670,12 +1588,12 @@
       <c r="E21" s="3" t="inlineStr"/>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. setHeaderFooter (shared/licenseExceljs.ts:155-209) now preserves an existing §6 header and appends (not overwrites) the footer left section, and customer-facing exports name the scoped lab: the VeritaScan library export reads req.scope.lab.name / clia_number (server/routes.ts:16572-16573), not the licensee. No new code this session (avoided regressing the existing fix). Closed 2026-09-24.</t>
+          <t>Closure evidence: VeritaTrack CalendarView month cells with more than three tasks now expand in place (chevron, "+N more" toggling to "Show less", due dates), so no task is hidden with no path to it (client/src/pages/VeritaTrackAppPage.tsx CalendarView). Shipped 2026-09-23. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+          <t>2026-09-23 session, Michael screenshot of the VeritaTrack calendar (lab 3, September cell).
 ---</t>
         </is>
       </c>
@@ -1684,18 +1602,72 @@
     <row r="22" ht="90" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>C34</t>
+          <t>C37</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Wire the two static-audit guards into CI (was #43)</t>
+          <t>Long Excel column headers no longer clip CFR citations (was #44)</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr"/>
       <c r="D22" s="2" t="inlineStr"/>
       <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. The VeritaMap export derives the header row height from the longest wrapped header via headerRowHeight(headers, colWidths) (server/routes.ts:15935) instead of a fixed 20, so "Reference Range Attestation (42 CFR 493.1253)" and the other long headers print in full. No new code this session. Closed 2026-09-24.</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+---</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23" ht="90" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>C36</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>License stamp no longer clobbers the §6 header/footer or names the wrong lab (was #43)</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr"/>
+      <c r="D23" s="3" t="inlineStr"/>
+      <c r="E23" s="3" t="inlineStr"/>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. setHeaderFooter (shared/licenseExceljs.ts:155-209) now preserves an existing §6 header and appends (not overwrites) the footer left section, and customer-facing exports name the scoped lab: the VeritaScan library export reads req.scope.lab.name / clia_number (server/routes.ts:16572-16573), not the licensee. No new code this session (avoided regressing the existing fix). Closed 2026-09-24.</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+---</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr"/>
+    </row>
+    <row r="24" ht="90" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>C34</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Wire the two static-audit guards into CI (was #43)</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr"/>
+      <c r="D24" s="2" t="inlineStr"/>
+      <c r="E24" s="2" t="inlineStr"/>
+      <c r="F24" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: both guards wired into the Multi-Lab Mutations Audit CI
 workflow (.github/workflows/multilab-mutations-audit.yml) as steps:
@@ -1707,24 +1679,24 @@
 (same caveat as the existing guards already in that workflow).</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr"/>
-      <c r="H22" s="2" t="inlineStr"/>
-    </row>
-    <row r="23" ht="90" customHeight="1">
-      <c r="A23" s="3" t="inlineStr">
+      <c r="G24" s="2" t="inlineStr"/>
+      <c r="H24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25" ht="90" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
         <is>
           <t>C35</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>Legacy /api/studies over-returns studies across labs (was #44)</t>
         </is>
       </c>
-      <c r="C23" s="3" t="inlineStr"/>
-      <c r="D23" s="3" t="inlineStr"/>
-      <c r="E23" s="3" t="inlineStr"/>
-      <c r="F23" s="3" t="inlineStr">
+      <c r="C25" s="3" t="inlineStr"/>
+      <c r="D25" s="3" t="inlineStr"/>
+      <c r="E25" s="3" t="inlineStr"/>
+      <c r="F25" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: GET /api/studies now scopes its list to the active lab
 when one is resolved from the Referer (server/routes.ts), so every returned row
@@ -1734,24 +1706,24 @@
 mirroring the /api/labs/:labId/studies handler. Closed 2026-06-14.</t>
         </is>
       </c>
-      <c r="G23" s="3" t="inlineStr"/>
-      <c r="H23" s="3" t="inlineStr"/>
-    </row>
-    <row r="24" ht="90" customHeight="1">
-      <c r="A24" s="2" t="inlineStr">
+      <c r="G25" s="3" t="inlineStr"/>
+      <c r="H25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26" ht="90" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>C30</t>
         </is>
       </c>
-      <c r="B24" s="2" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t>Verify-script convention backfill (was #41)</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr"/>
-      <c r="D24" s="2" t="inlineStr"/>
-      <c r="E24" s="2" t="inlineStr"/>
-      <c r="F24" s="2" t="inlineStr">
+      <c r="C26" s="2" t="inlineStr"/>
+      <c r="D26" s="2" t="inlineStr"/>
+      <c r="E26" s="2" t="inlineStr"/>
+      <c r="F26" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: all 8 high-stakes math/logic commits now ship a paired
 scripts/verify-*.js (EP17 sensitivity, Deming lot-to-lot, CUMSUM+QC+multi-analyte,
@@ -1759,30 +1731,30 @@
 TEa boundary), per the strike-throughs in #41. Closed 2026-06-13.</t>
         </is>
       </c>
-      <c r="G24" s="2" t="inlineStr">
+      <c r="G26" s="2" t="inlineStr">
         <is>
           <t>scripts/audit_verify_script_coverage.py lookback, 2026-06-02; backfills
 landed 2026-06-03..06.
 ---</t>
         </is>
       </c>
-      <c r="H24" s="2" t="inlineStr"/>
-    </row>
-    <row r="25" ht="90" customHeight="1">
-      <c r="A25" s="3" t="inlineStr">
+      <c r="H26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27" ht="90" customHeight="1">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>C31</t>
         </is>
       </c>
-      <c r="B25" s="3" t="inlineStr">
+      <c r="B27" s="3" t="inlineStr">
         <is>
           <t>VeritaPT AAA create/update/delete silently no-op in the multi-lab UI</t>
         </is>
       </c>
-      <c r="C25" s="3" t="inlineStr"/>
-      <c r="D25" s="3" t="inlineStr"/>
-      <c r="E25" s="3" t="inlineStr"/>
-      <c r="F25" s="3" t="inlineStr">
+      <c r="C27" s="3" t="inlineStr"/>
+      <c r="D27" s="3" t="inlineStr"/>
+      <c r="E27" s="3" t="inlineStr"/>
+      <c r="F27" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #754 (commit 92ad499) added lab-scoped POST/PUT/DELETE
 /api/labs/:labId/pt/aa-records. The UI posted to the lab-scoped path but only GET
@@ -1793,30 +1765,30 @@
 route mis-filed records to the user's default lab on multi-lab accounts).</t>
         </is>
       </c>
-      <c r="G25" s="3" t="inlineStr">
+      <c r="G27" s="3" t="inlineStr">
         <is>
           <t>2026-06-13, found during #18 Phase 3 QA;
 scripts/audit-labscoped-write-routes.mjs now guards the class.
 ---</t>
         </is>
       </c>
-      <c r="H25" s="3" t="inlineStr"/>
-    </row>
-    <row r="26" ht="90" customHeight="1">
-      <c r="A26" s="2" t="inlineStr">
+      <c r="H27" s="3" t="inlineStr"/>
+    </row>
+    <row r="28" ht="90" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>C32</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="B28" s="2" t="inlineStr">
         <is>
           <t>VeritaComp "Unlock assessment" false-success no-op</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr"/>
-      <c r="D26" s="2" t="inlineStr"/>
-      <c r="E26" s="2" t="inlineStr"/>
-      <c r="F26" s="2" t="inlineStr">
+      <c r="C28" s="2" t="inlineStr"/>
+      <c r="D28" s="2" t="inlineStr"/>
+      <c r="E28" s="2" t="inlineStr"/>
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #755 (commit 4234007) moved the unlock route to
 /api/labs/:labId/competency/assessments/:id/unlock (the path the client calls).
@@ -1827,29 +1799,29 @@
 HTML).</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr">
+      <c r="G28" s="2" t="inlineStr">
         <is>
           <t>2026-06-13, found by scripts/audit-labscoped-write-routes.mjs.
 ---</t>
         </is>
       </c>
-      <c r="H26" s="2" t="inlineStr"/>
-    </row>
-    <row r="27" ht="90" customHeight="1">
-      <c r="A27" s="3" t="inlineStr">
+      <c r="H28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29" ht="90" customHeight="1">
+      <c r="A29" s="3" t="inlineStr">
         <is>
           <t>C33</t>
         </is>
       </c>
-      <c r="B27" s="3" t="inlineStr">
+      <c r="B29" s="3" t="inlineStr">
         <is>
           <t>FK-cascade delete 500s + NavBar laptop-width overflow</t>
         </is>
       </c>
-      <c r="C27" s="3" t="inlineStr"/>
-      <c r="D27" s="3" t="inlineStr"/>
-      <c r="E27" s="3" t="inlineStr"/>
-      <c r="F27" s="3" t="inlineStr">
+      <c r="C29" s="3" t="inlineStr"/>
+      <c r="D29" s="3" t="inlineStr"/>
+      <c r="E29" s="3" t="inlineStr"/>
+      <c r="F29" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PRs #749/#750 fixed NavBar horizontal overflow at laptop
 widths (collapse to the hamburger below 1560px); prod-verified at 1280-1920 with the
@@ -1860,57 +1832,57 @@
 500 -&gt; 200. scripts/audit-delete-cascades.mjs guards the class.</t>
         </is>
       </c>
-      <c r="G27" s="3" t="inlineStr">
+      <c r="G29" s="3" t="inlineStr">
         <is>
           <t>2026-06-13 browser QA of the A7-D4 wave + retro-QC of the 72h PR window.
 ---</t>
         </is>
       </c>
-      <c r="H27" s="3" t="inlineStr"/>
-    </row>
-    <row r="28" ht="90" customHeight="1">
-      <c r="A28" s="2" t="inlineStr">
+      <c r="H29" s="3" t="inlineStr"/>
+    </row>
+    <row r="30" ht="90" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>C1</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="B30" s="2" t="inlineStr">
         <is>
           <t>FAQ "over 25 years" -&gt; "over 23 years"</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr"/>
-      <c r="D28" s="2" t="inlineStr"/>
-      <c r="E28" s="2" t="inlineStr"/>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="C30" s="2" t="inlineStr"/>
+      <c r="D30" s="2" t="inlineStr"/>
+      <c r="E30" s="2" t="inlineStr"/>
+      <c r="F30" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: client/src/pages/FAQPage.tsx line 20 reads "over
 23 years" as of 2026-05-01.</t>
         </is>
       </c>
-      <c r="G28" s="2" t="inlineStr">
+      <c r="G30" s="2" t="inlineStr">
         <is>
           <t>session 299e9a73 turn 14, ~2026-04-28.
 ---</t>
         </is>
       </c>
-      <c r="H28" s="2" t="inlineStr"/>
-    </row>
-    <row r="29" ht="90" customHeight="1">
-      <c r="A29" s="3" t="inlineStr">
+      <c r="H30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31" ht="90" customHeight="1">
+      <c r="A31" s="3" t="inlineStr">
         <is>
           <t>C5</t>
         </is>
       </c>
-      <c r="B29" s="3" t="inlineStr">
+      <c r="B31" s="3" t="inlineStr">
         <is>
           <t>David's VeritaQA grey-button bug (seat permissions mode)</t>
         </is>
       </c>
-      <c r="C29" s="3" t="inlineStr"/>
-      <c r="D29" s="3" t="inlineStr"/>
-      <c r="E29" s="3" t="inlineStr"/>
-      <c r="F29" s="3" t="inlineStr">
+      <c r="C31" s="3" t="inlineStr"/>
+      <c r="D31" s="3" t="inlineStr"/>
+      <c r="E31" s="3" t="inlineStr"/>
+      <c r="F31" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #10 squash-merged as commit a43fbba on
 2026-05-01 23:19 MST. Railway deploy succeeded; deployed bundle
@@ -1923,7 +1895,7 @@
 against his exact stored shape (14 of 14 expected outcomes matched).</t>
         </is>
       </c>
-      <c r="G29" s="3" t="inlineStr">
+      <c r="G31" s="3" t="inlineStr">
         <is>
           <t>2026-05-01 David's report; veritabench + veritastock
 weren't in MODULE_LIST so seat permissions silently defaulted to
@@ -1931,75 +1903,17 @@
 ---</t>
         </is>
       </c>
-      <c r="H29" s="3" t="inlineStr"/>
-    </row>
-    <row r="30" ht="90" customHeight="1">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>C2</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>TeamPage present-tense "TJC surveyor" check</t>
-        </is>
-      </c>
-      <c r="C30" s="2" t="inlineStr"/>
-      <c r="D30" s="2" t="inlineStr"/>
-      <c r="E30" s="2" t="inlineStr"/>
-      <c r="F30" s="2" t="inlineStr">
-        <is>
-          <t>Closure evidence: site-wide search confirmed all surveyor language
-is past-tense, consistent with user's 2021-2025 service. User closed
-the item in session 299e9a73 turn 4.</t>
-        </is>
-      </c>
-      <c r="G30" s="2" t="inlineStr">
-        <is>
-          <t>session 299e9a73, ~2026-04-28.
----</t>
-        </is>
-      </c>
-      <c r="H30" s="2" t="inlineStr"/>
-    </row>
-    <row r="31" ht="90" customHeight="1">
-      <c r="A31" s="3" t="inlineStr">
-        <is>
-          <t>C3</t>
-        </is>
-      </c>
-      <c r="B31" s="3" t="inlineStr">
-        <is>
-          <t>My Studies CSV/XLSX export (John as design partner)</t>
-        </is>
-      </c>
-      <c r="C31" s="3" t="inlineStr"/>
-      <c r="D31" s="3" t="inlineStr"/>
-      <c r="E31" s="3" t="inlineStr"/>
-      <c r="F31" s="3" t="inlineStr">
-        <is>
-          <t>Closure evidence: client/src/pages/DashboardPage.tsx line 46 calls
-/api/my-studies/export. server/routes.ts line 1491 implements the
-endpoint. Pulled forward into pre-COLA per user instruction.</t>
-        </is>
-      </c>
-      <c r="G31" s="3" t="inlineStr">
-        <is>
-          <t>session 299e9a73 turn 5, ~2026-04-28.
----</t>
-        </is>
-      </c>
       <c r="H31" s="3" t="inlineStr"/>
     </row>
     <row r="32" ht="90" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>C4</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Rotate GitHub PAT (because old PAT was committed in SESSION_HANDOFF files)</t>
+          <t>TeamPage present-tense "TJC surveyor" check</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr"/>
@@ -2007,8 +1921,9 @@
       <c r="E32" s="2" t="inlineStr"/>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: no ghp_* or github_pat_* patterns in current
-SESSION_HANDOFF.md or SESSION_HANDOFF-2.md as of 2026-05-01.</t>
+          <t>Closure evidence: site-wide search confirmed all surveyor language
+is past-tense, consistent with user's 2021-2025 service. User closed
+the item in session 299e9a73 turn 4.</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -2022,18 +1937,75 @@
     <row r="33" ht="90" customHeight="1">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>C6</t>
+          <t>C3</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>VeritaPolicy service-line filtering removed (formerly #4)</t>
+          <t>My Studies CSV/XLSX export (John as design partner)</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr"/>
       <c r="D33" s="3" t="inlineStr"/>
       <c r="E33" s="3" t="inlineStr"/>
       <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>Closure evidence: client/src/pages/DashboardPage.tsx line 46 calls
+/api/my-studies/export. server/routes.ts line 1491 implements the
+endpoint. Pulled forward into pre-COLA per user instruction.</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>session 299e9a73 turn 5, ~2026-04-28.
+---</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr"/>
+    </row>
+    <row r="34" ht="90" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Rotate GitHub PAT (because old PAT was committed in SESSION_HANDOFF files)</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr"/>
+      <c r="D34" s="2" t="inlineStr"/>
+      <c r="E34" s="2" t="inlineStr"/>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>Closure evidence: no ghp_* or github_pat_* patterns in current
+SESSION_HANDOFF.md or SESSION_HANDOFF-2.md as of 2026-05-01.</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>session 299e9a73, ~2026-04-28.
+---</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr"/>
+    </row>
+    <row r="35" ht="90" customHeight="1">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>C6</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>VeritaPolicy service-line filtering removed (formerly #4)</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr"/>
+      <c r="D35" s="3" t="inlineStr"/>
+      <c r="E35" s="3" t="inlineStr"/>
+      <c r="F35" s="3" t="inlineStr">
         <is>
           <t>Closure rationale (operator decision 2026-05-10): Keep all
 VeritaPolicy rows. CFR-only references with no accreditor reference
@@ -2042,29 +2014,29 @@
 report misread the design intent.</t>
         </is>
       </c>
-      <c r="G33" s="3" t="inlineStr">
+      <c r="G35" s="3" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H33" s="3" t="inlineStr"/>
-    </row>
-    <row r="34" ht="90" customHeight="1">
-      <c r="A34" s="2" t="inlineStr">
+      <c r="H35" s="3" t="inlineStr"/>
+    </row>
+    <row r="36" ht="90" customHeight="1">
+      <c r="A36" s="2" t="inlineStr">
         <is>
           <t>C7</t>
         </is>
       </c>
-      <c r="B34" s="2" t="inlineStr">
+      <c r="B36" s="2" t="inlineStr">
         <is>
           <t>CLIA number format validation (formerly #13)</t>
         </is>
       </c>
-      <c r="C34" s="2" t="inlineStr"/>
-      <c r="D34" s="2" t="inlineStr"/>
-      <c r="E34" s="2" t="inlineStr"/>
-      <c r="F34" s="2" t="inlineStr">
+      <c r="C36" s="2" t="inlineStr"/>
+      <c r="D36" s="2" t="inlineStr"/>
+      <c r="E36" s="2" t="inlineStr"/>
+      <c r="F36" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: shared/validateClia.ts defines CLIA_REGEX =
 /^\d{2}D\d{7}$/ (line 24), validateClia() helper with whitespace
@@ -2075,30 +2047,30 @@
 shape exists and behaves as specified.</t>
         </is>
       </c>
-      <c r="G34" s="2" t="inlineStr">
+      <c r="G36" s="2" t="inlineStr">
         <is>
           <t>Agent verification 2026-05-10 via grep + file read.
 Operator confirmed shipped 2026-05-10.
 ---</t>
         </is>
       </c>
-      <c r="H34" s="2" t="inlineStr"/>
-    </row>
-    <row r="35" ht="90" customHeight="1">
-      <c r="A35" s="3" t="inlineStr">
+      <c r="H36" s="2" t="inlineStr"/>
+    </row>
+    <row r="37" ht="90" customHeight="1">
+      <c r="A37" s="3" t="inlineStr">
         <is>
           <t>C8</t>
         </is>
       </c>
-      <c r="B35" s="3" t="inlineStr">
+      <c r="B37" s="3" t="inlineStr">
         <is>
           <t>VeritaMap lab-wide menu toggle (formerly #19)</t>
         </is>
       </c>
-      <c r="C35" s="3" t="inlineStr"/>
-      <c r="D35" s="3" t="inlineStr"/>
-      <c r="E35" s="3" t="inlineStr"/>
-      <c r="F35" s="3" t="inlineStr">
+      <c r="C37" s="3" t="inlineStr"/>
+      <c r="D37" s="3" t="inlineStr"/>
+      <c r="E37" s="3" t="inlineStr"/>
+      <c r="F37" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: client/src/pages/VeritaMapLabwidePage.tsx
 exists and implements the labwide read-only union view. Route is
@@ -2108,59 +2080,59 @@
 parking lot plan (read-only union view, per-session toggle) shipped.</t>
         </is>
       </c>
-      <c r="G35" s="3" t="inlineStr">
+      <c r="G37" s="3" t="inlineStr">
         <is>
           <t>Agent verification 2026-05-10 via grep + file read.
 Operator confirmed shipped 2026-05-10.
 ---</t>
         </is>
       </c>
-      <c r="H35" s="3" t="inlineStr"/>
-    </row>
-    <row r="36" ht="90" customHeight="1">
-      <c r="A36" s="2" t="inlineStr">
+      <c r="H37" s="3" t="inlineStr"/>
+    </row>
+    <row r="38" ht="90" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
         <is>
           <t>C9</t>
         </is>
       </c>
-      <c r="B36" s="2" t="inlineStr">
+      <c r="B38" s="2" t="inlineStr">
         <is>
           <t>Tier-1 smoke test checklist (formerly #6)</t>
         </is>
       </c>
-      <c r="C36" s="2" t="inlineStr"/>
-      <c r="D36" s="2" t="inlineStr"/>
-      <c r="E36" s="2" t="inlineStr"/>
-      <c r="F36" s="2" t="inlineStr">
+      <c r="C38" s="2" t="inlineStr"/>
+      <c r="D38" s="2" t="inlineStr"/>
+      <c r="E38" s="2" t="inlineStr"/>
+      <c r="F38" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: docs/smoke-test-tier1.md documents the Tier-1
 smoke-test process and post-deploy verification steps. Shipped via
 PR #81 as part of the 2026-05-10 wave.</t>
         </is>
       </c>
-      <c r="G36" s="2" t="inlineStr">
+      <c r="G38" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H36" s="2" t="inlineStr"/>
-    </row>
-    <row r="37" ht="90" customHeight="1">
-      <c r="A37" s="3" t="inlineStr">
+      <c r="H38" s="2" t="inlineStr"/>
+    </row>
+    <row r="39" ht="90" customHeight="1">
+      <c r="A39" s="3" t="inlineStr">
         <is>
           <t>C10</t>
         </is>
       </c>
-      <c r="B37" s="3" t="inlineStr">
+      <c r="B39" s="3" t="inlineStr">
         <is>
           <t>Per-module gating (formerly #7)</t>
         </is>
       </c>
-      <c r="C37" s="3" t="inlineStr"/>
-      <c r="D37" s="3" t="inlineStr"/>
-      <c r="E37" s="3" t="inlineStr"/>
-      <c r="F37" s="3" t="inlineStr">
+      <c r="C39" s="3" t="inlineStr"/>
+      <c r="D39" s="3" t="inlineStr"/>
+      <c r="E39" s="3" t="inlineStr"/>
+      <c r="F39" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: Client-side useIsReadOnly module keys wired
 on client/src/pages/VeritaPolicyAppPage.tsx and
@@ -2175,29 +2147,29 @@
 PR #76.</t>
         </is>
       </c>
-      <c r="G37" s="3" t="inlineStr">
+      <c r="G39" s="3" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H37" s="3" t="inlineStr"/>
-    </row>
-    <row r="38" ht="90" customHeight="1">
-      <c r="A38" s="2" t="inlineStr">
+      <c r="H39" s="3" t="inlineStr"/>
+    </row>
+    <row r="40" ht="90" customHeight="1">
+      <c r="A40" s="2" t="inlineStr">
         <is>
           <t>C11</t>
         </is>
       </c>
-      <c r="B38" s="2" t="inlineStr">
+      <c r="B40" s="2" t="inlineStr">
         <is>
           <t>VeritaStock shipped copy (formerly #8)</t>
         </is>
       </c>
-      <c r="C38" s="2" t="inlineStr"/>
-      <c r="D38" s="2" t="inlineStr"/>
-      <c r="E38" s="2" t="inlineStr"/>
-      <c r="F38" s="2" t="inlineStr">
+      <c r="C40" s="2" t="inlineStr"/>
+      <c r="D40" s="2" t="inlineStr"/>
+      <c r="E40" s="2" t="inlineStr"/>
+      <c r="F40" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: client/src/pages/ArticleInventoryManagementPage.tsx
 line 305 footer reads "platform that includes VeritaStock™" instead
@@ -2205,29 +2177,29 @@
 on /resources/laboratory-inventory-management. Shipped via PR #75.</t>
         </is>
       </c>
-      <c r="G38" s="2" t="inlineStr">
+      <c r="G40" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H38" s="2" t="inlineStr"/>
-    </row>
-    <row r="39" ht="90" customHeight="1">
-      <c r="A39" s="3" t="inlineStr">
+      <c r="H40" s="2" t="inlineStr"/>
+    </row>
+    <row r="41" ht="90" customHeight="1">
+      <c r="A41" s="3" t="inlineStr">
         <is>
           <t>C12</t>
         </is>
       </c>
-      <c r="B39" s="3" t="inlineStr">
+      <c r="B41" s="3" t="inlineStr">
         <is>
           <t>Admin report one-row-per-lab (formerly #14)</t>
         </is>
       </c>
-      <c r="C39" s="3" t="inlineStr"/>
-      <c r="D39" s="3" t="inlineStr"/>
-      <c r="E39" s="3" t="inlineStr"/>
-      <c r="F39" s="3" t="inlineStr">
+      <c r="C41" s="3" t="inlineStr"/>
+      <c r="D41" s="3" t="inlineStr"/>
+      <c r="E41" s="3" t="inlineStr"/>
+      <c r="F41" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: /api/admin/report rewritten in
 server/routes.ts (~line 595) to LEFT JOIN labs on
@@ -2242,56 +2214,56 @@
 prerequisite, not a code bug). Shipped via PR #85.</t>
         </is>
       </c>
-      <c r="G39" s="3" t="inlineStr">
+      <c r="G41" s="3" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H39" s="3" t="inlineStr"/>
-    </row>
-    <row r="40" ht="90" customHeight="1">
-      <c r="A40" s="2" t="inlineStr">
+      <c r="H41" s="3" t="inlineStr"/>
+    </row>
+    <row r="42" ht="90" customHeight="1">
+      <c r="A42" s="2" t="inlineStr">
         <is>
           <t>C14</t>
         </is>
       </c>
-      <c r="B40" s="2" t="inlineStr">
+      <c r="B42" s="2" t="inlineStr">
         <is>
           <t>UI relabel "CLIA TEa" -&gt; "Lab-Set Internal Goal" (formerly #1)</t>
         </is>
       </c>
-      <c r="C40" s="2" t="inlineStr"/>
-      <c r="D40" s="2" t="inlineStr"/>
-      <c r="E40" s="2" t="inlineStr"/>
-      <c r="F40" s="2" t="inlineStr">
+      <c r="C42" s="2" t="inlineStr"/>
+      <c r="D42" s="2" t="inlineStr"/>
+      <c r="E42" s="2" t="inlineStr"/>
+      <c r="F42" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: Shipped across four PRs over 2026-05-10.</t>
         </is>
       </c>
-      <c r="G40" s="2" t="inlineStr">
+      <c r="G42" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H40" s="2" t="inlineStr"/>
-    </row>
-    <row r="41" ht="90" customHeight="1">
-      <c r="A41" s="3" t="inlineStr">
+      <c r="H42" s="2" t="inlineStr"/>
+    </row>
+    <row r="43" ht="90" customHeight="1">
+      <c r="A43" s="3" t="inlineStr">
         <is>
           <t>C13</t>
         </is>
       </c>
-      <c r="B41" s="3" t="inlineStr">
+      <c r="B43" s="3" t="inlineStr">
         <is>
           <t>WSLH PT vendor (formerly #15)</t>
         </is>
       </c>
-      <c r="C41" s="3" t="inlineStr"/>
-      <c r="D41" s="3" t="inlineStr"/>
-      <c r="E41" s="3" t="inlineStr"/>
-      <c r="F41" s="3" t="inlineStr">
+      <c r="C43" s="3" t="inlineStr"/>
+      <c r="D43" s="3" t="inlineStr"/>
+      <c r="E43" s="3" t="inlineStr"/>
+      <c r="F43" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: Shipped 2026-05-10 via PR #79 (merge commit
 eeebc6e; merged after rebase to resolve a server/db.ts collision
@@ -2309,68 +2281,9 @@
 'WSLH' is the post-deploy success signal. Shipped via PR #79.</t>
         </is>
       </c>
-      <c r="G41" s="3" t="inlineStr">
+      <c r="G43" s="3" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
----</t>
-        </is>
-      </c>
-      <c r="H41" s="3" t="inlineStr"/>
-    </row>
-    <row r="42" ht="90" customHeight="1">
-      <c r="A42" s="2" t="inlineStr">
-        <is>
-          <t>C15</t>
-        </is>
-      </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>VeritaStock lot tracking + expiration + reorder alerts (formerly #21)</t>
-        </is>
-      </c>
-      <c r="C42" s="2" t="inlineStr"/>
-      <c r="D42" s="2" t="inlineStr"/>
-      <c r="E42" s="2" t="inlineStr"/>
-      <c r="F42" s="2" t="inlineStr">
-        <is>
-          <t>Closure evidence: VeritaStock™ shipped the bench-level inventory
-features the Perplexity competitor analysis identified as a gap:</t>
-        </is>
-      </c>
-      <c r="G42" s="2" t="inlineStr">
-        <is>
-          <t>Originally Perplexity competitor analysis 2026-05-10.
-Audit 2026-05-21 confirmed the feature set ships today.
----</t>
-        </is>
-      </c>
-      <c r="H42" s="2" t="inlineStr"/>
-    </row>
-    <row r="43" ht="90" customHeight="1">
-      <c r="A43" s="3" t="inlineStr">
-        <is>
-          <t>C16</t>
-        </is>
-      </c>
-      <c r="B43" s="3" t="inlineStr">
-        <is>
-          <t>PAL studies guided workflow (formerly #23)</t>
-        </is>
-      </c>
-      <c r="C43" s="3" t="inlineStr"/>
-      <c r="D43" s="3" t="inlineStr"/>
-      <c r="E43" s="3" t="inlineStr"/>
-      <c r="F43" s="3" t="inlineStr">
-        <is>
-          <t>Closure evidence: VeritaCheck™ already ships the Precision /
-Accuracy / Linearity (PAL) study set under EP-protocol naming:</t>
-        </is>
-      </c>
-      <c r="G43" s="3" t="inlineStr">
-        <is>
-          <t>Originally Perplexity competitor analysis 2026-05-10.
-Audit 2026-05-21 confirmed the EP studies cover the PAL framing in
-full.
 ---</t>
         </is>
       </c>
@@ -2379,12 +2292,12 @@
     <row r="44" ht="90" customHeight="1">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>C17</t>
+          <t>C15</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Source-grounded 21/29/45 CFR + 42 CFR 482-485 (formerly #26)</t>
+          <t>VeritaStock lot tracking + expiration + reorder alerts (formerly #21)</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr"/>
@@ -2392,35 +2305,94 @@
       <c r="E44" s="2" t="inlineStr"/>
       <c r="F44" s="2" t="inlineStr">
         <is>
+          <t>Closure evidence: VeritaStock™ shipped the bench-level inventory
+features the Perplexity competitor analysis identified as a gap:</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>Originally Perplexity competitor analysis 2026-05-10.
+Audit 2026-05-21 confirmed the feature set ships today.
+---</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr"/>
+    </row>
+    <row r="45" ht="90" customHeight="1">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>C16</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>PAL studies guided workflow (formerly #23)</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr"/>
+      <c r="D45" s="3" t="inlineStr"/>
+      <c r="E45" s="3" t="inlineStr"/>
+      <c r="F45" s="3" t="inlineStr">
+        <is>
+          <t>Closure evidence: VeritaCheck™ already ships the Precision /
+Accuracy / Linearity (PAL) study set under EP-protocol naming:</t>
+        </is>
+      </c>
+      <c r="G45" s="3" t="inlineStr">
+        <is>
+          <t>Originally Perplexity competitor analysis 2026-05-10.
+Audit 2026-05-21 confirmed the EP studies cover the PAL framing in
+full.
+---</t>
+        </is>
+      </c>
+      <c r="H45" s="3" t="inlineStr"/>
+    </row>
+    <row r="46" ht="90" customHeight="1">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>C17</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Source-grounded 21/29/45 CFR + 42 CFR 482-485 (formerly #26)</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr"/>
+      <c r="D46" s="2" t="inlineStr"/>
+      <c r="E46" s="2" t="inlineStr"/>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
           <t>Closure evidence: PR #301 (commit 8c27806, merged 2026-05-21)
 source-grounded the 74 remaining non-493 entries in
 server/cfrRequirements.ts against verbatim eCFR XML. Breakdown
 shipped:</t>
         </is>
       </c>
-      <c r="G44" s="2" t="inlineStr">
+      <c r="G46" s="2" t="inlineStr">
         <is>
           <t>PR #301; tasks #18 in the in-session task tracker.
 ---</t>
         </is>
       </c>
-      <c r="H44" s="2" t="inlineStr"/>
-    </row>
-    <row r="45" ht="90" customHeight="1">
-      <c r="A45" s="3" t="inlineStr">
+      <c r="H46" s="2" t="inlineStr"/>
+    </row>
+    <row r="47" ht="90" customHeight="1">
+      <c r="A47" s="3" t="inlineStr">
         <is>
           <t>C18</t>
         </is>
       </c>
-      <c r="B45" s="3" t="inlineStr">
+      <c r="B47" s="3" t="inlineStr">
         <is>
           <t>VeritaPolicy "Non CLIA" chapter rename (formerly #3)</t>
         </is>
       </c>
-      <c r="C45" s="3" t="inlineStr"/>
-      <c r="D45" s="3" t="inlineStr"/>
-      <c r="E45" s="3" t="inlineStr"/>
-      <c r="F45" s="3" t="inlineStr">
+      <c r="C47" s="3" t="inlineStr"/>
+      <c r="D47" s="3" t="inlineStr"/>
+      <c r="E47" s="3" t="inlineStr"/>
+      <c r="F47" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #300 (commit 34d7707, merged 2026-05-21)
 renamed all 44 user-facing chapter labels in
@@ -2431,7 +2403,7 @@
 page.</t>
         </is>
       </c>
-      <c r="G45" s="3" t="inlineStr">
+      <c r="G47" s="3" t="inlineStr">
         <is>
           <t>CAP customer screenshot of the /veritapolicy chapter
 headers, 2026-05-01 evening. PR #300; tasks #17 in the in-session
@@ -2439,23 +2411,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H45" s="3" t="inlineStr"/>
-    </row>
-    <row r="46" ht="90" customHeight="1">
-      <c r="A46" s="2" t="inlineStr">
+      <c r="H47" s="3" t="inlineStr"/>
+    </row>
+    <row r="48" ht="90" customHeight="1">
+      <c r="A48" s="2" t="inlineStr">
         <is>
           <t>C19</t>
         </is>
       </c>
-      <c r="B46" s="2" t="inlineStr">
+      <c r="B48" s="2" t="inlineStr">
         <is>
           <t>VeritaStock department-scope toggle (formerly #31)</t>
         </is>
       </c>
-      <c r="C46" s="2" t="inlineStr"/>
-      <c r="D46" s="2" t="inlineStr"/>
-      <c r="E46" s="2" t="inlineStr"/>
-      <c r="F46" s="2" t="inlineStr">
+      <c r="C48" s="2" t="inlineStr"/>
+      <c r="D48" s="2" t="inlineStr"/>
+      <c r="E48" s="2" t="inlineStr"/>
+      <c r="F48" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #319 (commit d01f5fe, merged 2026-05-22)
 shipped the persistent dept-scope toggle on VeritaStockPage. A new
@@ -2466,7 +2438,7 @@
 workspace without re-filtering.</t>
         </is>
       </c>
-      <c r="G46" s="2" t="inlineStr">
+      <c r="G48" s="2" t="inlineStr">
         <is>
           <t>John, San Carlos lab, 2026-05-21. Same conversation that
 drove the vendor dropdown (PR #304), FILTERED VIEW banner (PR #305),
@@ -2474,23 +2446,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H46" s="2" t="inlineStr"/>
-    </row>
-    <row r="47" ht="90" customHeight="1">
-      <c r="A47" s="3" t="inlineStr">
+      <c r="H48" s="2" t="inlineStr"/>
+    </row>
+    <row r="49" ht="90" customHeight="1">
+      <c r="A49" s="3" t="inlineStr">
         <is>
           <t>C20</t>
         </is>
       </c>
-      <c r="B47" s="3" t="inlineStr">
+      <c r="B49" s="3" t="inlineStr">
         <is>
           <t>Primary-lab seat counting (formerly #12)</t>
         </is>
       </c>
-      <c r="C47" s="3" t="inlineStr"/>
-      <c r="D47" s="3" t="inlineStr"/>
-      <c r="E47" s="3" t="inlineStr"/>
-      <c r="F47" s="3" t="inlineStr">
+      <c r="C49" s="3" t="inlineStr"/>
+      <c r="D49" s="3" t="inlineStr"/>
+      <c r="E49" s="3" t="inlineStr"/>
+      <c r="F49" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: is_primary_lab INTEGER NOT NULL DEFAULT 0
 column was added to the lab_members table at db.ts:1276, with the
@@ -2501,7 +2473,7 @@
 is_primary_lab=1 ordering).</t>
         </is>
       </c>
-      <c r="G47" s="3" t="inlineStr">
+      <c r="G49" s="3" t="inlineStr">
         <is>
           <t>2026-05-07 multi-lab discussion. Build shipped as part
 of the Multi-Lab Tier 2 architecture work (Phase 3.x series, prior
@@ -2510,23 +2482,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H47" s="3" t="inlineStr"/>
-    </row>
-    <row r="48" ht="90" customHeight="1">
-      <c r="A48" s="2" t="inlineStr">
+      <c r="H49" s="3" t="inlineStr"/>
+    </row>
+    <row r="50" ht="90" customHeight="1">
+      <c r="A50" s="2" t="inlineStr">
         <is>
           <t>C21</t>
         </is>
       </c>
-      <c r="B48" s="2" t="inlineStr">
+      <c r="B50" s="2" t="inlineStr">
         <is>
           <t>Multi-lab pricing model — Option A (formerly #11)</t>
         </is>
       </c>
-      <c r="C48" s="2" t="inlineStr"/>
-      <c r="D48" s="2" t="inlineStr"/>
-      <c r="E48" s="2" t="inlineStr"/>
-      <c r="F48" s="2" t="inlineStr">
+      <c r="C50" s="2" t="inlineStr"/>
+      <c r="D50" s="2" t="inlineStr"/>
+      <c r="E50" s="2" t="inlineStr"/>
+      <c r="F50" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #322 (commit 0ccd925, merged 2026-05-22)
 added the customer-facing line to the pricing page that reflects
@@ -2539,7 +2511,7 @@
 Enterprise+ block, reads:</t>
         </is>
       </c>
-      <c r="G48" s="2" t="inlineStr">
+      <c r="G50" s="2" t="inlineStr">
         <is>
           <t>2026-05-07 multi-lab discussion (Lisa Veri's
 canonical-case session). PR #322 (initial build); softening PR
@@ -2548,30 +2520,30 @@
 ---</t>
         </is>
       </c>
-      <c r="H48" s="2" t="inlineStr"/>
-    </row>
-    <row r="49" ht="90" customHeight="1">
-      <c r="A49" s="3" t="inlineStr">
+      <c r="H50" s="2" t="inlineStr"/>
+    </row>
+    <row r="51" ht="90" customHeight="1">
+      <c r="A51" s="3" t="inlineStr">
         <is>
           <t>C22</t>
         </is>
       </c>
-      <c r="B49" s="3" t="inlineStr">
+      <c r="B51" s="3" t="inlineStr">
         <is>
           <t>VeritaOps cost-per-test module (formerly #10)</t>
         </is>
       </c>
-      <c r="C49" s="3" t="inlineStr"/>
-      <c r="D49" s="3" t="inlineStr"/>
-      <c r="E49" s="3" t="inlineStr"/>
-      <c r="F49" s="3" t="inlineStr">
+      <c r="C51" s="3" t="inlineStr"/>
+      <c r="D51" s="3" t="inlineStr"/>
+      <c r="E51" s="3" t="inlineStr"/>
+      <c r="F51" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: v1 of the VeritaOps Cost-Per-Reportable-Test
 (CPRT) module shipped across PR #325 through PR #330 on 2026-05-22.
 The module is feature-complete for the typical lab director workflow.</t>
         </is>
       </c>
-      <c r="G49" s="3" t="inlineStr">
+      <c r="G51" s="3" t="inlineStr">
         <is>
           <t>This thread, 2026-05-07 12:05 PM CDT, user message:
 "Parking lot: build an operations module for cost per test
@@ -2580,262 +2552,262 @@
 ---</t>
         </is>
       </c>
-      <c r="H49" s="3" t="inlineStr"/>
-    </row>
-    <row r="50" ht="90" customHeight="1">
-      <c r="A50" s="2" t="inlineStr">
+      <c r="H51" s="3" t="inlineStr"/>
+    </row>
+    <row r="52" ht="90" customHeight="1">
+      <c r="A52" s="2" t="inlineStr">
         <is>
           <t>C23</t>
         </is>
       </c>
-      <c r="B50" s="2" t="inlineStr">
+      <c r="B52" s="2" t="inlineStr">
         <is>
           <t>CCL lab name visual disambiguation in lab switcher (formerly #34)</t>
         </is>
       </c>
-      <c r="C50" s="2" t="inlineStr"/>
-      <c r="D50" s="2" t="inlineStr">
+      <c r="C52" s="2" t="inlineStr"/>
+      <c r="D52" s="2" t="inlineStr">
         <is>
           <t>XS (under 1 day, actual)</t>
         </is>
       </c>
-      <c r="E50" s="2" t="inlineStr">
+      <c r="E52" s="2" t="inlineStr">
         <is>
           <t>Low — cosmetic; only mattered when Lisa or Michael picked the wrong lab from...</t>
         </is>
       </c>
-      <c r="F50" s="2" t="inlineStr">
+      <c r="F52" s="2" t="inlineStr">
         <is>
           <t>Effort: XS (under 1 day, actual)
 Importance: Low — cosmetic; only mattered when Lisa or Michael picked the wrong lab from the dropdown.</t>
         </is>
       </c>
-      <c r="G50" s="2" t="inlineStr">
+      <c r="G52" s="2" t="inlineStr">
         <is>
           <t>flagged 2026-05-23 immediately after provisioning Lisa's CCL lab; closed 2026-05-24.
 ---</t>
         </is>
       </c>
-      <c r="H50" s="2" t="inlineStr"/>
-    </row>
-    <row r="51" ht="90" customHeight="1">
-      <c r="A51" s="3" t="inlineStr">
+      <c r="H52" s="2" t="inlineStr"/>
+    </row>
+    <row r="53" ht="90" customHeight="1">
+      <c r="A53" s="3" t="inlineStr">
         <is>
           <t>C24</t>
         </is>
       </c>
-      <c r="B51" s="3" t="inlineStr">
+      <c r="B53" s="3" t="inlineStr">
         <is>
           <t>VC Unlimited Y1/Y2 price disclosure UX (formerly #35)</t>
         </is>
       </c>
-      <c r="C51" s="3" t="inlineStr"/>
-      <c r="D51" s="3" t="inlineStr">
+      <c r="C53" s="3" t="inlineStr"/>
+      <c r="D53" s="3" t="inlineStr">
         <is>
           <t>XS (under 1 day, actual)</t>
         </is>
       </c>
-      <c r="E51" s="3" t="inlineStr">
+      <c r="E53" s="3" t="inlineStr">
         <is>
           <t>Low when shipped (proactive, no customer complaint yet) — but high if a procu...</t>
         </is>
       </c>
-      <c r="F51" s="3" t="inlineStr">
+      <c r="F53" s="3" t="inlineStr">
         <is>
           <t>Effort: XS (under 1 day, actual)
 Importance: Low when shipped (proactive, no customer complaint yet) — but high if a procurement reviewer later disputes the $499 renewal as undisclosed.</t>
         </is>
       </c>
-      <c r="G51" s="3" t="inlineStr">
+      <c r="G53" s="3" t="inlineStr">
         <is>
           <t>Pricing rebuild 2026-05-23; closed 2026-05-24 proactively before any customer dispute.
 ---</t>
         </is>
       </c>
-      <c r="H51" s="3" t="inlineStr"/>
-    </row>
-    <row r="52" ht="90" customHeight="1">
-      <c r="A52" s="2" t="inlineStr">
+      <c r="H53" s="3" t="inlineStr"/>
+    </row>
+    <row r="54" ht="90" customHeight="1">
+      <c r="A54" s="2" t="inlineStr">
         <is>
           <t>C25</t>
         </is>
       </c>
-      <c r="B52" s="2" t="inlineStr">
+      <c r="B54" s="2" t="inlineStr">
         <is>
           <t>VeritaQC Phase 1 (Levey-Jennings + Westgard live engine) (formerly #20)</t>
         </is>
       </c>
-      <c r="C52" s="2" t="inlineStr"/>
-      <c r="D52" s="2" t="inlineStr">
+      <c r="C54" s="2" t="inlineStr"/>
+      <c r="D54" s="2" t="inlineStr">
         <is>
           <t>L (about 5 days end-to-end, actual: Phase 0 schema → Phase 1A evaluator → 1B...</t>
         </is>
       </c>
-      <c r="E52" s="2" t="inlineStr">
+      <c r="E54" s="2" t="inlineStr">
         <is>
           <t>High — largest single gap vs myLabCompliance.io per Perplexity competitor ana...</t>
         </is>
       </c>
-      <c r="F52" s="2" t="inlineStr">
+      <c r="F54" s="2" t="inlineStr">
         <is>
           <t>Effort: L (about 5 days end-to-end, actual: Phase 0 schema → Phase 1A evaluator → 1B entry UI → 1C daily review → 1D monthly PDF + attestation)
 Importance: High — largest single gap vs myLabCompliance.io per Perplexity competitor analysis; promotes VeritaAssure from documentation tool to lab operations platform.</t>
         </is>
       </c>
-      <c r="G52" s="2" t="inlineStr">
+      <c r="G54" s="2" t="inlineStr">
         <is>
           <t>Perplexity competitor analysis 2026-05-10. Scoping confirmed via the build_phase1_mockup.py iterations 2026-05-24. Shipped 2026-05-25.
 ---</t>
         </is>
       </c>
-      <c r="H52" s="2" t="inlineStr"/>
-    </row>
-    <row r="53" ht="90" customHeight="1">
-      <c r="A53" s="3" t="inlineStr">
+      <c r="H54" s="2" t="inlineStr"/>
+    </row>
+    <row r="55" ht="90" customHeight="1">
+      <c r="A55" s="3" t="inlineStr">
         <is>
           <t>C26</t>
         </is>
       </c>
-      <c r="B53" s="3" t="inlineStr">
+      <c r="B55" s="3" t="inlineStr">
         <is>
           <t>VeritaLab CMS-116 application support + state licensing registry (formerly #22)</t>
         </is>
       </c>
-      <c r="C53" s="3" t="inlineStr"/>
-      <c r="D53" s="3" t="inlineStr">
+      <c r="C55" s="3" t="inlineStr"/>
+      <c r="D55" s="3" t="inlineStr">
         <is>
           <t>M (1-2 weeks for v1, actual)</t>
         </is>
       </c>
-      <c r="E53" s="3" t="inlineStr">
+      <c r="E55" s="3" t="inlineStr">
         <is>
           <t>Medium — competitor parity (myLabCompliance.io) plus useful at lab startup an...</t>
         </is>
       </c>
-      <c r="F53" s="3" t="inlineStr">
+      <c r="F55" s="3" t="inlineStr">
         <is>
           <t>Effort: M (1-2 weeks for v1, actual)
 Importance: Medium — competitor parity (myLabCompliance.io) plus useful at lab startup and at certificate-type changes.</t>
         </is>
       </c>
-      <c r="G53" s="3" t="inlineStr">
+      <c r="G55" s="3" t="inlineStr">
         <is>
           <t>Perplexity competitor analysis (myLabCompliance.io), 2026-05-10. Reclassified as a VeritaLab extension 2026-05-25. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H53" s="3" t="inlineStr"/>
-    </row>
-    <row r="54" ht="90" customHeight="1">
-      <c r="A54" s="2" t="inlineStr">
+      <c r="H55" s="3" t="inlineStr"/>
+    </row>
+    <row r="56" ht="90" customHeight="1">
+      <c r="A56" s="2" t="inlineStr">
         <is>
           <t>C27</t>
         </is>
       </c>
-      <c r="B54" s="2" t="inlineStr">
+      <c r="B56" s="2" t="inlineStr">
         <is>
           <t>Active vs view-only seat split (formerly #33)</t>
         </is>
       </c>
-      <c r="C54" s="2" t="inlineStr"/>
-      <c r="D54" s="2" t="inlineStr">
+      <c r="C56" s="2" t="inlineStr"/>
+      <c r="D56" s="2" t="inlineStr">
         <is>
           <t>M (~1 week of engineering, actual: shipped in a single multi-PR session)</t>
         </is>
       </c>
-      <c r="E54" s="2" t="inlineStr">
+      <c r="E56" s="2" t="inlineStr">
         <is>
           <t>Medium — closed the gap between /pricing copy and product behavior; gives sal...</t>
         </is>
       </c>
-      <c r="F54" s="2" t="inlineStr">
+      <c r="F56" s="2" t="inlineStr">
         <is>
           <t>Effort: M (~1 week of engineering, actual: shipped in a single multi-PR session)
 Importance: Medium — closed the gap between /pricing copy and product behavior; gives sales a clean answer for "do you charge for our medical director?"</t>
         </is>
       </c>
-      <c r="G54" s="2" t="inlineStr">
+      <c r="G56" s="2" t="inlineStr">
         <is>
           <t>Pricing analysis doc Decision 3 (2026-05-21); MEDIUM scenario revised 2026-05-29 to retire the "unlimited view-only" claim. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H54" s="2" t="inlineStr"/>
-    </row>
-    <row r="55" ht="90" customHeight="1">
-      <c r="A55" s="3" t="inlineStr">
+      <c r="H56" s="2" t="inlineStr"/>
+    </row>
+    <row r="57" ht="90" customHeight="1">
+      <c r="A57" s="3" t="inlineStr">
         <is>
           <t>C28</t>
         </is>
       </c>
-      <c r="B55" s="3" t="inlineStr">
+      <c r="B57" s="3" t="inlineStr">
         <is>
           <t>"Why VeritaCheck" comparative one-pager (formerly #37)</t>
         </is>
       </c>
-      <c r="C55" s="3" t="inlineStr"/>
-      <c r="D55" s="3" t="inlineStr">
+      <c r="C57" s="3" t="inlineStr"/>
+      <c r="D57" s="3" t="inlineStr">
         <is>
           <t>S (one design pass + four claim paragraphs + PDF + matching marketing-site pa...</t>
         </is>
       </c>
-      <c r="E55" s="3" t="inlineStr">
+      <c r="E57" s="3" t="inlineStr">
         <is>
           <t>Medium — closed a positioning gap surfaced by six COLA conference attendees a...</t>
         </is>
       </c>
-      <c r="F55" s="3" t="inlineStr">
+      <c r="F57" s="3" t="inlineStr">
         <is>
           <t>Effort: S (one design pass + four claim paragraphs + PDF + matching marketing-site page, actual)
 Importance: Medium — closed a positioning gap surfaced by six COLA conference attendees attached to a legacy verification tool; converts product-quality advantage into a leave-behind Lisa can hand out.</t>
         </is>
       </c>
-      <c r="G55" s="3" t="inlineStr">
+      <c r="G57" s="3" t="inlineStr">
         <is>
           <t>2026-05-11 / 2026-05-12 conference notes review with Michael. Conference attendees (Whitehead, Odegard, Othman, Molinelli, Kyle, Allred) expressed interest in equivalent / superior product. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H55" s="3" t="inlineStr"/>
-    </row>
-    <row r="56" ht="90" customHeight="1">
-      <c r="A56" s="2" t="inlineStr">
+      <c r="H57" s="3" t="inlineStr"/>
+    </row>
+    <row r="58" ht="90" customHeight="1">
+      <c r="A58" s="2" t="inlineStr">
         <is>
           <t>C29</t>
         </is>
       </c>
-      <c r="B56" s="2" t="inlineStr">
+      <c r="B58" s="2" t="inlineStr">
         <is>
           <t>VeritaPolicy approval workflow — MediaLab functional mirror</t>
         </is>
       </c>
-      <c r="C56" s="2" t="inlineStr"/>
-      <c r="D56" s="2" t="inlineStr">
+      <c r="C58" s="2" t="inlineStr"/>
+      <c r="D58" s="2" t="inlineStr">
         <is>
           <t>XL (one focused session, 12 PRs landed)</t>
         </is>
       </c>
-      <c r="E56" s="2" t="inlineStr">
+      <c r="E58" s="2" t="inlineStr">
         <is>
           <t>High — replaces MediaLab Document Control ($752/$2,250 starting price, scalin...</t>
         </is>
       </c>
-      <c r="F56" s="2" t="inlineStr">
+      <c r="F58" s="2" t="inlineStr">
         <is>
           <t>Effort: XL (one focused session, 12 PRs landed)
 Importance: High — replaces MediaLab Document Control ($752/$2,250 starting price, scaling to $10K-$20K/yr at enterprise per Capterra public data) with an included VeritaPolicy feature; closes a real positioning gap and gives sales a direct comparator line.</t>
         </is>
       </c>
-      <c r="G56" s="2" t="inlineStr">
+      <c r="G58" s="2" t="inlineStr">
         <is>
           <t>Pricing strategy conversation 2026-05-29 (Michael: "I don't like bolt-ons; we should replicate this") → scoped 8 phases → shipped all 12 PRs in single session. Shipped 2026-05-29.
 ---</t>
         </is>
       </c>
-      <c r="H56" s="2" t="inlineStr"/>
+      <c r="H58" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H56"/>
+  <autoFilter ref="A1:H58"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
TASK: Parking lot - Manual Differential complexity shows Moderate in VeritaMap, should be High
PLAN:
  1. Add OPEN item #58 (Effort XS, Importance High) per the parking-lot format
  2. Regenerate PARKING_LOT.xlsx from the markdown source

Self-check:
  - Gate 3 N/A (internal parking-lot doc, no code)
  - PARKING_LOT.xlsx regenerated from PARKING_LOT.md in the same commit
  - likely root cause noted (instrument-menu seed default); fix path = set-complexity admin endpoint

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PARKING_LOT.xlsx
+++ b/PARKING_LOT.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RETIRED" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$58</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RETIRED'!$A$1:$H$7</definedName>
   </definedNames>
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1003,8 +1003,39 @@
       </c>
       <c r="H11" s="3" t="inlineStr"/>
     </row>
+    <row r="12" ht="90" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Manual Differential complexity is MODERATE in VeritaMap, should be HIGH</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr"/>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>XS (under 1 day)</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>High — a wrong complexity under-applies HIGH-complexity requirements, produci...</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Effort: XS (under 1 day)
+Importance: High — a wrong complexity under-applies HIGH-complexity requirements, producing a false readiness picture and regulatory exposure.</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr"/>
+      <c r="H12" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H11"/>
+  <autoFilter ref="A1:H12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
TASK: Update parking lot - add items 43 (finding-closure signer confirm) + 44 (inventory Excel refresh); clarify #39 delegation note; regen xlsx PLAN:   1. Add OPEN #43 (confirm the finding-closure signer policy after the Phase 2 tightening) and #44 (regenerate the access-inventory Excel with the corrected MD persona).   2. Clarify that #39's "delegation" is VeritaPolicy approval-workflow delegation, distinct from the Letter of Delegation feature shipped this session (#1442-1445).   3. Regenerate PARKING_LOT.xlsx (OPEN 12 / CLOSED 57 / RETIRED 6). Self-check:   - xlsx regenerated from the markdown source; counts match; both committed together per the sync rule.   - Gate 3 N/A (internal documentation).   - No entries deleted; #39 amended with a dated note, not overwritten.
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PARKING_LOT.xlsx
+++ b/PARKING_LOT.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RETIRED" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$58</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RETIRED'!$A$1:$H$7</definedName>
   </definedNames>
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1003,8 +1003,86 @@
       </c>
       <c r="H11" s="3" t="inlineStr"/>
     </row>
+    <row r="12" ht="90" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Confirm the finding-closure signer policy (non-MD admins now blocked)</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Open, awaiting operator confirmation. Reverting is a one-line change (re-add the owner/admin path in the findings/:id/signoff handler) if admins should retain finding closure.
+---</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>XS (a yes/no decision; ~15 min to loosen the gate if reversed).</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Medium — changes who can close VeritaResponse findings in production; affects...</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Item 5 Phase 2 tightened VeritaResponse finding closure from "any owner / admin / edit-seat" to "the designated medical director, a delegated designee holding finding-closure for the lab's complexity, or the account owner as a logged break-glass override." This is live on prod (#1443). It follows the agreed MD-or-designee model (QB=1), and the same gate now guards QC period-review co-sign. It has not been confirmed against real customer workflows: if any lab relies on non-MD admins closing findings, they now need a Letter of Delegation, or the gate must be loosened.</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>this session, delegation feature build (2026-10-04). Flagged repeatedly in-session; awaiting explicit operator sign-off.</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13" ht="90" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Regenerate the 119-function access-inventory Excel with the corrected MD persona</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Open, low priority. Offered to Michael; skippable if the sweep was a one-off working artifact.
+---</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>XS (~15 min to re-run the sweep harness and re-deliver).</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Low — the harness and the shipped fixes are correct; only the recorded Excel'...</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>The full-inventory 4-login access sweep (VeritaAssure_Function_Inventory.xlsx) was first generated with the medical-director test persona mis-seeded as a seatless member, which over-flagged its column. The harness was then corrected to seat the MD as the active writer it actually is (scripts/qa-sweep/inventory-sweep.ts). The delivered Excel still shows the old md results; re-running reclassifies the md-artifact flags down to the real findings, which were already fixed in PR A (#1441). Only worth doing if the sheet gets filed or shared externally.</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>this session, QA sweep (2026-10-03 to 2026-10-04).</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H11"/>
+  <autoFilter ref="A1:H13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
TASK: Update parking lot - add #43/#44, clarify #39, regen xlsx
PLAN:
  1. Add OPEN #43 (finding-closure signer confirm) and #44 (inventory Excel refresh).
  2. Clarify that #39 delegation is VeritaPolicy approval-workflow delegation.
  3. Regenerate PARKING_LOT.xlsx (OPEN 12 / CLOSED 57 / RETIRED 6).

Self-check:
  - xlsx regenerated from the markdown source; both committed together per the sync rule.
  - Gate 3 N/A (internal documentation).
  - No entries deleted; #39 amended with a dated note.
</commit_message>
<xml_diff>
--- a/PARKING_LOT.xlsx
+++ b/PARKING_LOT.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RETIRED" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$58</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RETIRED'!$A$1:$H$7</definedName>
   </definedNames>
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1003,8 +1003,86 @@
       </c>
       <c r="H11" s="3" t="inlineStr"/>
     </row>
+    <row r="12" ht="90" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Confirm the finding-closure signer policy (non-MD admins now blocked)</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Open, awaiting operator confirmation. Reverting is a one-line change (re-add the owner/admin path in the findings/:id/signoff handler) if admins should retain finding closure.
+---</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>XS (a yes/no decision; ~15 min to loosen the gate if reversed).</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Medium — changes who can close VeritaResponse findings in production; affects...</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Item 5 Phase 2 tightened VeritaResponse finding closure from "any owner / admin / edit-seat" to "the designated medical director, a delegated designee holding finding-closure for the lab's complexity, or the account owner as a logged break-glass override." This is live on prod (#1443). It follows the agreed MD-or-designee model (QB=1), and the same gate now guards QC period-review co-sign. It has not been confirmed against real customer workflows: if any lab relies on non-MD admins closing findings, they now need a Letter of Delegation, or the gate must be loosened.</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>this session, delegation feature build (2026-10-04). Flagged repeatedly in-session; awaiting explicit operator sign-off.</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13" ht="90" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Regenerate the 119-function access-inventory Excel with the corrected MD persona</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Open, low priority. Offered to Michael; skippable if the sweep was a one-off working artifact.
+---</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>XS (~15 min to re-run the sweep harness and re-deliver).</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Low — the harness and the shipped fixes are correct; only the recorded Excel'...</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>The full-inventory 4-login access sweep (VeritaAssure_Function_Inventory.xlsx) was first generated with the medical-director test persona mis-seeded as a seatless member, which over-flagged its column. The harness was then corrected to seat the MD as the active writer it actually is (scripts/qa-sweep/inventory-sweep.ts). The delivered Excel still shows the old md results; re-running reclassifies the md-artifact flags down to the real findings, which were already fixed in PR A (#1441). Only worth doing if the sheet gets filed or shared externally.</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>this session, QA sweep (2026-10-03 to 2026-10-04).</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H11"/>
+  <autoFilter ref="A1:H13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
TASK: Parking lot - close #45 (VeritaDC per-document attestation tracker) as C58; regen xlsx PLAN:   1. Add CLOSED entry C58 for the VeritaDC attestation tracker + My Documents rename (shipped PRs #1447/#1449, browser-verified).   2. Regenerate PARKING_LOT.xlsx (CLOSED 57 -> 58; OPEN unchanged at 12). Self-check:   - xlsx regenerated from the markdown source; both committed together per the sync rule.   - Gate 3 N/A (internal documentation).   - Closure cites the shipped PRs + the browser verification + the date-fix follow-up.
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PARKING_LOT.xlsx
+++ b/PARKING_LOT.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$58</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$59</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RETIRED'!$A$1:$H$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1093,7 +1093,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H58"/>
+  <dimension ref="A1:H59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1151,24 +1151,24 @@
     <row r="2" ht="90" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>C57</t>
+          <t>C58</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Hide sections a lab does not use from a master list (was #47)</t>
+          <t>VeritaDC per-document attestation tracker + "My Documents" rename (built as #45)</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr"/>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>was S-M / Importance: Medium-High (prospect-requested)</t>
+          <t>was M / Importance: Medium-High</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Effort: was S-M / Importance: Medium-High (prospect-requested)</t>
+          <t>Effort: was M / Importance: Medium-High</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
@@ -1177,24 +1177,24 @@
     <row r="3" ht="90" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>C56</t>
+          <t>C57</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>VeritaCEU: curated free continuing-education provider list (was #53)</t>
+          <t>Hide sections a lab does not use from a master list (was #47)</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr"/>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>was S / Importance: Low-Medium</t>
+          <t>was S-M / Importance: Medium-High (prospect-requested)</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Effort: was S / Importance: Low-Medium</t>
+          <t>Effort: was S-M / Importance: Medium-High (prospect-requested)</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr"/>
@@ -1203,24 +1203,24 @@
     <row r="4" ht="90" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>C55</t>
+          <t>C56</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>VeritaScan: let sites add their own custom questions (was #55)</t>
+          <t>VeritaCEU: curated free continuing-education provider list (was #53)</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr"/>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>was M / Importance: Medium-High</t>
+          <t>was S / Importance: Low-Medium</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Effort: was M / Importance: Medium-High</t>
+          <t>Effort: was S / Importance: Low-Medium</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr"/>
@@ -1229,24 +1229,24 @@
     <row r="5" ht="90" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>C54</t>
+          <t>C55</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>VeritaQC: at-entry warning when a QC point is outside 2 SD (was #56)</t>
+          <t>VeritaScan: let sites add their own custom questions (was #55)</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr"/>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>was S-M (shipped S) / Importance: High</t>
+          <t>was M / Importance: Medium-High</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Effort: was S-M (shipped S) / Importance: High</t>
+          <t>Effort: was M / Importance: Medium-High</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr"/>
@@ -1255,24 +1255,24 @@
     <row r="6" ht="90" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>C53</t>
+          <t>C54</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>VeritaTrack: quarterly task loaded as monthly until re-saved (was #54)</t>
+          <t>VeritaQC: at-entry warning when a QC point is outside 2 SD (was #56)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr"/>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>was S / Importance: Medium</t>
+          <t>was S-M (shipped S) / Importance: High</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Effort: was S / Importance: Medium</t>
+          <t>Effort: was S-M (shipped S) / Importance: High</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
@@ -1281,24 +1281,24 @@
     <row r="7" ht="90" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>C52</t>
+          <t>C53</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>VeritaResponse internal NCE / non-conforming event (was #36)</t>
+          <t>VeritaTrack: quarterly task loaded as monthly until re-saved (was #54)</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr"/>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>was L (shipped as MEDIUM) / Importance: High</t>
+          <t>was S / Importance: Medium</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Effort: was L (shipped as MEDIUM) / Importance: High</t>
+          <t>Effort: was S / Importance: Medium</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr"/>
@@ -1307,24 +1307,24 @@
     <row r="8" ht="90" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>C49</t>
+          <t>C52</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Competency "assessed this cycle" cadence-aware window (was #50)</t>
+          <t>VeritaResponse internal NCE / non-conforming event (was #36)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr"/>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>was S-M / Importance: Medium</t>
+          <t>was L (shipped as MEDIUM) / Importance: High</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Effort: was S-M / Importance: Medium</t>
+          <t>Effort: was L (shipped as MEDIUM) / Importance: High</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
@@ -1333,12 +1333,12 @@
     <row r="9" ht="90" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>C50</t>
+          <t>C49</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>VeritaTrack task owner + owner-only reminder routing (was #51)</t>
+          <t>Competency "assessed this cycle" cadence-aware window (was #50)</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr"/>
@@ -1359,24 +1359,24 @@
     <row r="10" ht="90" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>C51</t>
+          <t>C50</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Designate Medical Director by picking a lab member (was #52, core)</t>
+          <t>VeritaTrack task owner + owner-only reminder routing (was #51)</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr"/>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>was S-M / Importance: Medium-High</t>
+          <t>was S-M / Importance: Medium</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Effort: was S-M / Importance: Medium-High</t>
+          <t>Effort: was S-M / Importance: Medium</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
@@ -1385,24 +1385,24 @@
     <row r="11" ht="90" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>C47</t>
+          <t>C51</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Unregulated-analyte / Alternative Assessment (AAA) coverage (was #18)</t>
+          <t>Designate Medical Director by picking a lab member (was #52, core)</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr"/>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>was S (Phase 3) / Importance: Medium</t>
+          <t>was S-M / Importance: Medium-High</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Effort: was S (Phase 3) / Importance: Medium</t>
+          <t>Effort: was S-M / Importance: Medium-High</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr"/>
@@ -1411,24 +1411,24 @@
     <row r="12" ht="90" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>C48</t>
+          <t>C47</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>VeritaResponse post-survey deficiency module (was #17)</t>
+          <t>Unregulated-analyte / Alternative Assessment (AAA) coverage (was #18)</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr"/>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>was XL / Importance: High</t>
+          <t>was S (Phase 3) / Importance: Medium</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Effort: was XL / Importance: High</t>
+          <t>Effort: was S (Phase 3) / Importance: Medium</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr"/>
@@ -1437,39 +1437,38 @@
     <row r="13" ht="90" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>C45</t>
+          <t>C48</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Unify coverage/competency recurrence helper (was #49) - closed as non-issue</t>
+          <t>VeritaResponse post-survey deficiency module (was #17)</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr"/>
-      <c r="D13" s="3" t="inlineStr"/>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>was XL / Importance: High</t>
+        </is>
+      </c>
       <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: Investigated 2026-09-24 before building. The coverage recurrence math (+6-month interval, signed-resets-to-missing, nextDueOn/overdue, isFailVerdict) is ALREADY single-source in server/veritacheckCoverage.ts (computeCoverageFrom). server/coverageReport.ts and the routes.ts coverage export do not recompute it; they consume the computed nextDueOn/overdue/status fields and apply small surface-specific presentation labels (deliberately different vocabularies per surface, so they should not be merged). The only truly identical duplicate is a one-line date formatter. The competency "owed" derivation is NOT the same cadence: competency follows the CLIA milestone schedule (initial / semiannual year 1 / annual, 42 CFR 493.1451(b)(8) and 493.1235), which is a different regulatory interval from the coverage 6-month rule (493.1281 / 493.1255) and must stay separate. No worthwhile extraction; merging the two cadences would be wrong. Closed 2026-09-24. (The year-1 competency-window refinement remains tracked separately as #50.)</t>
-        </is>
-      </c>
-      <c r="G13" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-24 session, "keep working" pass; scoped read-only, found no real duplication.
----</t>
-        </is>
-      </c>
+          <t>Effort: was XL / Importance: High</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr"/>
       <c r="H13" s="3" t="inlineStr"/>
     </row>
     <row r="14" ht="90" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>C46</t>
+          <t>C45</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Verified-users product-update send path (wrong-list incident fix)</t>
+          <t>Unify coverage/competency recurrence helper (was #49) - closed as non-issue</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr"/>
@@ -1477,12 +1476,12 @@
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: Shipped PR #1324 (merged 4e05506a, deploy ACTIVE). New POST /api/admin/users/send targets registered VeritaAssure account holders (the users table), never the Lab Director's Briefing subscriber list. Separate explicitly-named endpoint (not a flag with a dangerous default), account-holder email framing, excludes suppressed emails and RFC-reserved test domains, CC owner, dryRun + testTo previews. Public unsubscribe now upserts a suppression row so opt-outs are honored across both audiences. Live dryRun: 49 verified-user recipients vs 673 on the Briefing list. Receipts: scripts/verify-product-update-send.mts 24/24, tsc clean, rendered sample inspected. Fixes the fallout from the 2026-09-23/24 wrong-list send (a product update went to the 675-person Briefing list). Nothing sends without Michael's explicit "send it."</t>
+          <t>Closure evidence: Investigated 2026-09-24 before building. The coverage recurrence math (+6-month interval, signed-resets-to-missing, nextDueOn/overdue, isFailVerdict) is ALREADY single-source in server/veritacheckCoverage.ts (computeCoverageFrom). server/coverageReport.ts and the routes.ts coverage export do not recompute it; they consume the computed nextDueOn/overdue/status fields and apply small surface-specific presentation labels (deliberately different vocabularies per surface, so they should not be merged). The only truly identical duplicate is a one-line date formatter. The competency "owed" derivation is NOT the same cadence: competency follows the CLIA milestone schedule (initial / semiannual year 1 / annual, 42 CFR 493.1451(b)(8) and 493.1235), which is a different regulatory interval from the coverage 6-month rule (493.1281 / 493.1255) and must stay separate. No worthwhile extraction; merging the two cadences would be wrong. Closed 2026-09-24. (The year-1 competency-window refinement remains tracked separately as #50.)</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 session; Michael selected this as the next build after the #41 close.
+          <t>2026-09-24 session, "keep working" pass; scoped read-only, found no real duplication.
 ---</t>
         </is>
       </c>
@@ -1491,12 +1490,12 @@
     <row r="15" ht="90" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>C44</t>
+          <t>C46</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Verify-script convention backfill (was #41) + audit matcher fix</t>
+          <t>Verified-users product-update send path (wrong-list incident fix)</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr"/>
@@ -1504,12 +1503,12 @@
       <c r="E15" s="3" t="inlineStr"/>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: #41 was fully backfilled on 2026-06-13 (all 8 high-stakes scripts landed; see C30); it had only been mis-filed in OPEN. A 2026-09-24 re-audit initially reported 4 of 5 recent math/logic commits as missing a verify script, which was a FALSE POSITIVE: scripts/audit_verify_script_coverage.py matched only scripts/verify-*.js / .cjs, so it ignored the .mjs / .mts / .ts verify scripts the repo now ships (e.g. verify-ptcoag-multi.mts, verify-tea-criterion-format.mjs). Fixed the matcher to accept .js/.cjs/.mjs/.ts/.mts; re-run shows 5 of 5 covered, 0 debt. The convention is being followed. Closed 2026-09-24.</t>
+          <t>Closure evidence: Shipped PR #1324 (merged 4e05506a, deploy ACTIVE). New POST /api/admin/users/send targets registered VeritaAssure account holders (the users table), never the Lab Director's Briefing subscriber list. Separate explicitly-named endpoint (not a flag with a dangerous default), account-holder email framing, excludes suppressed emails and RFC-reserved test domains, CC owner, dryRun + testTo previews. Public unsubscribe now upserts a suppression row so opt-outs are honored across both audiences. Live dryRun: 49 verified-user recipients vs 673 on the Briefing list. Receipts: scripts/verify-product-update-send.mts 24/24, tsc clean, rendered sample inspected. Fixes the fallout from the 2026-09-23/24 wrong-list send (a product update went to the 675-person Briefing list). Nothing sends without Michael's explicit "send it."</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>2026-09-24 session, "keep working" pass; audit tooling bug found + fixed.
+          <t>2026-09-24 session; Michael selected this as the next build after the #41 close.
 ---</t>
         </is>
       </c>
@@ -1518,12 +1517,12 @@
     <row r="16" ht="90" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>C43</t>
+          <t>C44</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>VeritaStaff instrument-centric (dual) assignment view</t>
+          <t>Verify-script convention backfill (was #41) + audit matcher fix</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr"/>
@@ -1531,12 +1530,12 @@
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1320. GET/PUT /staff/instruments/:id/employees (transpose of the per-employee endpoints); an "Assign by Instrument" dialog lets a director pick a test system or manual test and check off who runs it. Same staff_employee_instruments join, with the 42 CFR 493.1235(a) duty-change event emitted on newly-added pairs so both orientations trigger the same reassessment. GET verified live on SCAHC lab 2. Closed 2026-09-24.</t>
+          <t>Closure evidence: #41 was fully backfilled on 2026-06-13 (all 8 high-stakes scripts landed; see C30); it had only been mis-filed in OPEN. A 2026-09-24 re-audit initially reported 4 of 5 recent math/logic commits as missing a verify script, which was a FALSE POSITIVE: scripts/audit_verify_script_coverage.py matched only scripts/verify-*.js / .cjs, so it ignored the .mjs / .mts / .ts verify scripts the repo now ships (e.g. verify-ptcoag-multi.mts, verify-tea-criterion-format.mjs). Fixed the matcher to accept .js/.cjs/.mjs/.ts/.mts; re-run shows 5 of 5 covered, 0 debt. The convention is being followed. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 session, Michael ("in staff we should also give the dual view when assigning coverage to test systems or manual tests").
+          <t>2026-09-24 session, "keep working" pass; audit tooling bug found + fixed.
 ---</t>
         </is>
       </c>
@@ -1545,12 +1544,12 @@
     <row r="17" ht="90" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>C42</t>
+          <t>C43</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>VeritaComp coverage map (required-vs-assessed matrix, dual view)</t>
+          <t>VeritaStaff instrument-centric (dual) assignment view</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr"/>
@@ -1558,12 +1557,12 @@
       <c r="E17" s="3" t="inlineStr"/>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1319 (+ status layer PR #1316). /competency/owed returns per-item assessed (locked passing assessment this cycle on a covering method group) + per-employee CLIA status; CompetencyCoverageMap renders a By-employee / By-instrument matrix (Assessed / Owed / Overdue / Gap). Verified live on SCAHC lab 2 (owed 116, assessed 2, gaps 0). Completes #48 as the VeritaCheck-parity coverage map. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1320. GET/PUT /staff/instruments/:id/employees (transpose of the per-employee endpoints); an "Assign by Instrument" dialog lets a director pick a test system or manual test and check off who runs it. Same staff_employee_instruments join, with the 42 CFR 493.1235(a) duty-change event emitted on newly-added pairs so both orientations trigger the same reassessment. GET verified live on SCAHC lab 2. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>2026-09-24 session, Michael ("are we building the competencies to have a coverage map, same as veritacheck?" then "build it").
+          <t>2026-09-24 session, Michael ("in staff we should also give the dual view when assigning coverage to test systems or manual tests").
 ---</t>
         </is>
       </c>
@@ -1572,12 +1571,12 @@
     <row r="18" ht="90" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>C41</t>
+          <t>C42</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>VeritaCheck coverage recurrence (method comparison + cal-ver/linearity + reports)</t>
+          <t>VeritaComp coverage map (required-vs-assessed matrix, dual view)</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr"/>
@@ -1585,12 +1584,12 @@
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: PRs #1317 (method comparison), #1318 (cal-ver/linearity), #1321 (report Next-due columns). Periodic verification (correlation/method comparison 42 CFR 493.1281; cal-ver/linearity 42 CFR 493.1255; both 6-month) now recurs: a signed study banks the cycle and rolls to next-due = signed + 6 months instead of reading "done" forever. Status Missing/Failed/Completed-unsigned + a "Next due on" column on-screen and in both coverage exports; also credits the previously-ignored "correlation" study type. Root cause: computeCoverageFrom marked requirements done on mere existence, no date logic. Verified live on SCAHC lab 2 (101 correlations + 11 cal-ver rows now carry a next-due). Engine-level, all facilities. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1319 (+ status layer PR #1316). /competency/owed returns per-item assessed (locked passing assessment this cycle on a covering method group) + per-employee CLIA status; CompetencyCoverageMap renders a By-employee / By-instrument matrix (Assessed / Owed / Overdue / Gap). Verified live on SCAHC lab 2 (owed 116, assessed 2, gaps 0). Completes #48 as the VeritaCheck-parity coverage map. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 session, Michael ("Look at San Carlos... they finished their last set of correlations (all 103) but their menu never reset").
+          <t>2026-09-24 session, Michael ("are we building the competencies to have a coverage map, same as veritacheck?" then "build it").
 ---</t>
         </is>
       </c>
@@ -1599,12 +1598,12 @@
     <row r="19" ht="90" customHeight="1">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>C40</t>
+          <t>C41</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>VeritaComp Competencies Owed derived from VeritaStaff, with gap detection (was #48)</t>
+          <t>VeritaCheck coverage recurrence (method comparison + cal-ver/linearity + reports)</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr"/>
@@ -1612,12 +1611,12 @@
       <c r="E19" s="3" t="inlineStr"/>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1314 (squash 2bcb0db9). GET /api/labs/:labId/competency/owed derives each VeritaStaff testing employee's owed competencies from their assigned instruments (staff_employee_instruments -&gt; veritamap_instruments + tests), on the CLIA timeline, and flags instruments not covered by any competency program as gaps. CompetenciesOwedSection renders it on the VeritaComp landing page. Reuses the shipped bridge + suggested-method-groups match rules; no new tables. Verified live on prod with real assignment data: 2 instruments assigned to a demo staffer produced owed=2, gaps=2 (HIGH, Technical Supervisor), then reverted cleanly. Closed 2026-09-24.</t>
+          <t>Closure evidence: PRs #1317 (method comparison), #1318 (cal-ver/linearity), #1321 (report Next-due columns). Periodic verification (correlation/method comparison 42 CFR 493.1281; cal-ver/linearity 42 CFR 493.1255; both 6-month) now recurs: a signed study banks the cycle and rolls to next-due = signed + 6 months instead of reading "done" forever. Status Missing/Failed/Completed-unsigned + a "Next due on" column on-screen and in both coverage exports; also credits the previously-ignored "correlation" study type. Root cause: computeCoverageFrom marked requirements done on mere existence, no date logic. Verified live on SCAHC lab 2 (101 correlations + 11 cal-ver rows now carry a next-due). Engine-level, all facilities. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>2026-09-23/24 session, Michael ("veritacomp bases what competencies they owe (currently untrue, but needs to be true)"). Option 1 (unify roster on VeritaStaff, match instruments by id).
+          <t>2026-09-24 session, Michael ("Look at San Carlos... they finished their last set of correlations (all 103) but their menu never reset").
 ---</t>
         </is>
       </c>
@@ -1626,12 +1625,12 @@
     <row r="20" ht="90" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>C39</t>
+          <t>C40</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>VeritaScan line items can attach or link evidence (was #46)</t>
+          <t>VeritaComp Competencies Owed derived from VeritaStaff, with gap detection (was #48)</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr"/>
@@ -1639,12 +1638,12 @@
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1312 (squash a1dda93d). VeritaScan scan checklist items now show linked evidence as chips (open link, remove) plus a writer "Link evidence" affordance whose picker links an existing VeritaDC/Library document; a shortcut deep-links to the Library for new (governed) documents. Reuses the already-shipped lab_documents + document_checklist_links + coverage endpoints (URL-pointer only, no file storage, no new tables). Browser-verified live on prod (scan 23): the affordance renders and the picker opens. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1314 (squash 2bcb0db9). GET /api/labs/:labId/competency/owed derives each VeritaStaff testing employee's owed competencies from their assigned instruments (staff_employee_instruments -&gt; veritamap_instruments + tests), on the CLIA timeline, and flags instruments not covered by any competency program as gaps. CompetenciesOwedSection renders it on the VeritaComp landing page. Reuses the shipped bridge + suggested-method-groups match rules; no new tables. Verified live on prod with real assignment data: 2 instruments assigned to a demo staffer produced owed=2, gaps=2 (HIGH, Technical Supervisor), then reverted cleanly. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23 session, Michael. Recurring request. Companion: cross-module evidence display on the VeritaDC policy shipped in PR #1313 (by-target cross-links surfaced in the policy View modal, browser-verified live).
+          <t>2026-09-23/24 session, Michael ("veritacomp bases what competencies they owe (currently untrue, but needs to be true)"). Option 1 (unify roster on VeritaStaff, match instruments by id).
 ---</t>
         </is>
       </c>
@@ -1653,12 +1652,12 @@
     <row r="21" ht="90" customHeight="1">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>C38</t>
+          <t>C39</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>VeritaTrack calendar month cells expand to reveal hidden tasks (was #45)</t>
+          <t>VeritaScan line items can attach or link evidence (was #46)</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr"/>
@@ -1666,12 +1665,12 @@
       <c r="E21" s="3" t="inlineStr"/>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: VeritaTrack CalendarView month cells with more than three tasks now expand in place (chevron, "+N more" toggling to "Show less", due dates), so no task is hidden with no path to it (client/src/pages/VeritaTrackAppPage.tsx CalendarView). Shipped 2026-09-23. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1312 (squash a1dda93d). VeritaScan scan checklist items now show linked evidence as chips (open link, remove) plus a writer "Link evidence" affordance whose picker links an existing VeritaDC/Library document; a shortcut deep-links to the Library for new (governed) documents. Reuses the already-shipped lab_documents + document_checklist_links + coverage endpoints (URL-pointer only, no file storage, no new tables). Browser-verified live on prod (scan 23): the affordance renders and the picker opens. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>2026-09-23 session, Michael screenshot of the VeritaTrack calendar (lab 3, September cell).
+          <t>2026-09-23 session, Michael. Recurring request. Companion: cross-module evidence display on the VeritaDC policy shipped in PR #1313 (by-target cross-links surfaced in the policy View modal, browser-verified live).
 ---</t>
         </is>
       </c>
@@ -1680,12 +1679,12 @@
     <row r="22" ht="90" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>C37</t>
+          <t>C38</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Long Excel column headers no longer clip CFR citations (was #44)</t>
+          <t>VeritaTrack calendar month cells expand to reveal hidden tasks (was #45)</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr"/>
@@ -1693,12 +1692,12 @@
       <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. The VeritaMap export derives the header row height from the longest wrapped header via headerRowHeight(headers, colWidths) (server/routes.ts:15935) instead of a fixed 20, so "Reference Range Attestation (42 CFR 493.1253)" and the other long headers print in full. No new code this session. Closed 2026-09-24.</t>
+          <t>Closure evidence: VeritaTrack CalendarView month cells with more than three tasks now expand in place (chevron, "+N more" toggling to "Show less", due dates), so no task is hidden with no path to it (client/src/pages/VeritaTrackAppPage.tsx CalendarView). Shipped 2026-09-23. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+          <t>2026-09-23 session, Michael screenshot of the VeritaTrack calendar (lab 3, September cell).
 ---</t>
         </is>
       </c>
@@ -1707,12 +1706,12 @@
     <row r="23" ht="90" customHeight="1">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>C36</t>
+          <t>C37</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>License stamp no longer clobbers the §6 header/footer or names the wrong lab (was #43)</t>
+          <t>Long Excel column headers no longer clip CFR citations (was #44)</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr"/>
@@ -1720,7 +1719,7 @@
       <c r="E23" s="3" t="inlineStr"/>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. setHeaderFooter (shared/licenseExceljs.ts:155-209) now preserves an existing §6 header and appends (not overwrites) the footer left section, and customer-facing exports name the scoped lab: the VeritaScan library export reads req.scope.lab.name / clia_number (server/routes.ts:16572-16573), not the licensee. No new code this session (avoided regressing the existing fix). Closed 2026-09-24.</t>
+          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. The VeritaMap export derives the header row height from the longest wrapped header via headerRowHeight(headers, colWidths) (server/routes.ts:15935) instead of a fixed 20, so "Reference Range Attestation (42 CFR 493.1253)" and the other long headers print in full. No new code this session. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -1734,18 +1733,45 @@
     <row r="24" ht="90" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>C34</t>
+          <t>C36</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Wire the two static-audit guards into CI (was #43)</t>
+          <t>License stamp no longer clobbers the §6 header/footer or names the wrong lab (was #43)</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr"/>
       <c r="D24" s="2" t="inlineStr"/>
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. setHeaderFooter (shared/licenseExceljs.ts:155-209) now preserves an existing §6 header and appends (not overwrites) the footer left section, and customer-facing exports name the scoped lab: the VeritaScan library export reads req.scope.lab.name / clia_number (server/routes.ts:16572-16573), not the licensee. No new code this session (avoided regressing the existing fix). Closed 2026-09-24.</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+---</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25" ht="90" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>C34</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Wire the two static-audit guards into CI (was #43)</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr"/>
+      <c r="D25" s="3" t="inlineStr"/>
+      <c r="E25" s="3" t="inlineStr"/>
+      <c r="F25" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: both guards wired into the Multi-Lab Mutations Audit CI
 workflow (.github/workflows/multilab-mutations-audit.yml) as steps:
@@ -1757,24 +1783,24 @@
 (same caveat as the existing guards already in that workflow).</t>
         </is>
       </c>
-      <c r="G24" s="2" t="inlineStr"/>
-      <c r="H24" s="2" t="inlineStr"/>
-    </row>
-    <row r="25" ht="90" customHeight="1">
-      <c r="A25" s="3" t="inlineStr">
+      <c r="G25" s="3" t="inlineStr"/>
+      <c r="H25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26" ht="90" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>C35</t>
         </is>
       </c>
-      <c r="B25" s="3" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t>Legacy /api/studies over-returns studies across labs (was #44)</t>
         </is>
       </c>
-      <c r="C25" s="3" t="inlineStr"/>
-      <c r="D25" s="3" t="inlineStr"/>
-      <c r="E25" s="3" t="inlineStr"/>
-      <c r="F25" s="3" t="inlineStr">
+      <c r="C26" s="2" t="inlineStr"/>
+      <c r="D26" s="2" t="inlineStr"/>
+      <c r="E26" s="2" t="inlineStr"/>
+      <c r="F26" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: GET /api/studies now scopes its list to the active lab
 when one is resolved from the Referer (server/routes.ts), so every returned row
@@ -1784,24 +1810,24 @@
 mirroring the /api/labs/:labId/studies handler. Closed 2026-06-14.</t>
         </is>
       </c>
-      <c r="G25" s="3" t="inlineStr"/>
-      <c r="H25" s="3" t="inlineStr"/>
-    </row>
-    <row r="26" ht="90" customHeight="1">
-      <c r="A26" s="2" t="inlineStr">
+      <c r="G26" s="2" t="inlineStr"/>
+      <c r="H26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27" ht="90" customHeight="1">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>C30</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="B27" s="3" t="inlineStr">
         <is>
           <t>Verify-script convention backfill (was #41)</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr"/>
-      <c r="D26" s="2" t="inlineStr"/>
-      <c r="E26" s="2" t="inlineStr"/>
-      <c r="F26" s="2" t="inlineStr">
+      <c r="C27" s="3" t="inlineStr"/>
+      <c r="D27" s="3" t="inlineStr"/>
+      <c r="E27" s="3" t="inlineStr"/>
+      <c r="F27" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: all 8 high-stakes math/logic commits now ship a paired
 scripts/verify-*.js (EP17 sensitivity, Deming lot-to-lot, CUMSUM+QC+multi-analyte,
@@ -1809,30 +1835,30 @@
 TEa boundary), per the strike-throughs in #41. Closed 2026-06-13.</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr">
+      <c r="G27" s="3" t="inlineStr">
         <is>
           <t>scripts/audit_verify_script_coverage.py lookback, 2026-06-02; backfills
 landed 2026-06-03..06.
 ---</t>
         </is>
       </c>
-      <c r="H26" s="2" t="inlineStr"/>
-    </row>
-    <row r="27" ht="90" customHeight="1">
-      <c r="A27" s="3" t="inlineStr">
+      <c r="H27" s="3" t="inlineStr"/>
+    </row>
+    <row r="28" ht="90" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>C31</t>
         </is>
       </c>
-      <c r="B27" s="3" t="inlineStr">
+      <c r="B28" s="2" t="inlineStr">
         <is>
           <t>VeritaPT AAA create/update/delete silently no-op in the multi-lab UI</t>
         </is>
       </c>
-      <c r="C27" s="3" t="inlineStr"/>
-      <c r="D27" s="3" t="inlineStr"/>
-      <c r="E27" s="3" t="inlineStr"/>
-      <c r="F27" s="3" t="inlineStr">
+      <c r="C28" s="2" t="inlineStr"/>
+      <c r="D28" s="2" t="inlineStr"/>
+      <c r="E28" s="2" t="inlineStr"/>
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #754 (commit 92ad499) added lab-scoped POST/PUT/DELETE
 /api/labs/:labId/pt/aa-records. The UI posted to the lab-scoped path but only GET
@@ -1843,30 +1869,30 @@
 route mis-filed records to the user's default lab on multi-lab accounts).</t>
         </is>
       </c>
-      <c r="G27" s="3" t="inlineStr">
+      <c r="G28" s="2" t="inlineStr">
         <is>
           <t>2026-06-13, found during #18 Phase 3 QA;
 scripts/audit-labscoped-write-routes.mjs now guards the class.
 ---</t>
         </is>
       </c>
-      <c r="H27" s="3" t="inlineStr"/>
-    </row>
-    <row r="28" ht="90" customHeight="1">
-      <c r="A28" s="2" t="inlineStr">
+      <c r="H28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29" ht="90" customHeight="1">
+      <c r="A29" s="3" t="inlineStr">
         <is>
           <t>C32</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="B29" s="3" t="inlineStr">
         <is>
           <t>VeritaComp "Unlock assessment" false-success no-op</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr"/>
-      <c r="D28" s="2" t="inlineStr"/>
-      <c r="E28" s="2" t="inlineStr"/>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="C29" s="3" t="inlineStr"/>
+      <c r="D29" s="3" t="inlineStr"/>
+      <c r="E29" s="3" t="inlineStr"/>
+      <c r="F29" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #755 (commit 4234007) moved the unlock route to
 /api/labs/:labId/competency/assessments/:id/unlock (the path the client calls).
@@ -1877,29 +1903,29 @@
 HTML).</t>
         </is>
       </c>
-      <c r="G28" s="2" t="inlineStr">
+      <c r="G29" s="3" t="inlineStr">
         <is>
           <t>2026-06-13, found by scripts/audit-labscoped-write-routes.mjs.
 ---</t>
         </is>
       </c>
-      <c r="H28" s="2" t="inlineStr"/>
-    </row>
-    <row r="29" ht="90" customHeight="1">
-      <c r="A29" s="3" t="inlineStr">
+      <c r="H29" s="3" t="inlineStr"/>
+    </row>
+    <row r="30" ht="90" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>C33</t>
         </is>
       </c>
-      <c r="B29" s="3" t="inlineStr">
+      <c r="B30" s="2" t="inlineStr">
         <is>
           <t>FK-cascade delete 500s + NavBar laptop-width overflow</t>
         </is>
       </c>
-      <c r="C29" s="3" t="inlineStr"/>
-      <c r="D29" s="3" t="inlineStr"/>
-      <c r="E29" s="3" t="inlineStr"/>
-      <c r="F29" s="3" t="inlineStr">
+      <c r="C30" s="2" t="inlineStr"/>
+      <c r="D30" s="2" t="inlineStr"/>
+      <c r="E30" s="2" t="inlineStr"/>
+      <c r="F30" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PRs #749/#750 fixed NavBar horizontal overflow at laptop
 widths (collapse to the hamburger below 1560px); prod-verified at 1280-1920 with the
@@ -1910,37 +1936,9 @@
 500 -&gt; 200. scripts/audit-delete-cascades.mjs guards the class.</t>
         </is>
       </c>
-      <c r="G29" s="3" t="inlineStr">
+      <c r="G30" s="2" t="inlineStr">
         <is>
           <t>2026-06-13 browser QA of the A7-D4 wave + retro-QC of the 72h PR window.
----</t>
-        </is>
-      </c>
-      <c r="H29" s="3" t="inlineStr"/>
-    </row>
-    <row r="30" ht="90" customHeight="1">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>C1</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>FAQ "over 25 years" -&gt; "over 23 years"</t>
-        </is>
-      </c>
-      <c r="C30" s="2" t="inlineStr"/>
-      <c r="D30" s="2" t="inlineStr"/>
-      <c r="E30" s="2" t="inlineStr"/>
-      <c r="F30" s="2" t="inlineStr">
-        <is>
-          <t>Closure evidence: client/src/pages/FAQPage.tsx line 20 reads "over
-23 years" as of 2026-05-01.</t>
-        </is>
-      </c>
-      <c r="G30" s="2" t="inlineStr">
-        <is>
-          <t>session 299e9a73 turn 14, ~2026-04-28.
 ---</t>
         </is>
       </c>
@@ -1949,18 +1947,46 @@
     <row r="31" ht="90" customHeight="1">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>C5</t>
+          <t>C1</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>David's VeritaQA grey-button bug (seat permissions mode)</t>
+          <t>FAQ "over 25 years" -&gt; "over 23 years"</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr"/>
       <c r="D31" s="3" t="inlineStr"/>
       <c r="E31" s="3" t="inlineStr"/>
       <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>Closure evidence: client/src/pages/FAQPage.tsx line 20 reads "over
+23 years" as of 2026-05-01.</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>session 299e9a73 turn 14, ~2026-04-28.
+---</t>
+        </is>
+      </c>
+      <c r="H31" s="3" t="inlineStr"/>
+    </row>
+    <row r="32" ht="90" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>David's VeritaQA grey-button bug (seat permissions mode)</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr"/>
+      <c r="D32" s="2" t="inlineStr"/>
+      <c r="E32" s="2" t="inlineStr"/>
+      <c r="F32" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #10 squash-merged as commit a43fbba on
 2026-05-01 23:19 MST. Railway deploy succeeded; deployed bundle
@@ -1973,7 +1999,7 @@
 against his exact stored shape (14 of 14 expected outcomes matched).</t>
         </is>
       </c>
-      <c r="G31" s="3" t="inlineStr">
+      <c r="G32" s="2" t="inlineStr">
         <is>
           <t>2026-05-01 David's report; veritabench + veritastock
 weren't in MODULE_LIST so seat permissions silently defaulted to
@@ -1981,46 +2007,17 @@
 ---</t>
         </is>
       </c>
-      <c r="H31" s="3" t="inlineStr"/>
-    </row>
-    <row r="32" ht="90" customHeight="1">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>C2</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>TeamPage present-tense "TJC surveyor" check</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr"/>
-      <c r="D32" s="2" t="inlineStr"/>
-      <c r="E32" s="2" t="inlineStr"/>
-      <c r="F32" s="2" t="inlineStr">
-        <is>
-          <t>Closure evidence: site-wide search confirmed all surveyor language
-is past-tense, consistent with user's 2021-2025 service. User closed
-the item in session 299e9a73 turn 4.</t>
-        </is>
-      </c>
-      <c r="G32" s="2" t="inlineStr">
-        <is>
-          <t>session 299e9a73, ~2026-04-28.
----</t>
-        </is>
-      </c>
       <c r="H32" s="2" t="inlineStr"/>
     </row>
     <row r="33" ht="90" customHeight="1">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>C3</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>My Studies CSV/XLSX export (John as design partner)</t>
+          <t>TeamPage present-tense "TJC surveyor" check</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr"/>
@@ -2028,14 +2025,14 @@
       <c r="E33" s="3" t="inlineStr"/>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: client/src/pages/DashboardPage.tsx line 46 calls
-/api/my-studies/export. server/routes.ts line 1491 implements the
-endpoint. Pulled forward into pre-COLA per user instruction.</t>
+          <t>Closure evidence: site-wide search confirmed all surveyor language
+is past-tense, consistent with user's 2021-2025 service. User closed
+the item in session 299e9a73 turn 4.</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>session 299e9a73 turn 5, ~2026-04-28.
+          <t>session 299e9a73, ~2026-04-28.
 ---</t>
         </is>
       </c>
@@ -2044,12 +2041,12 @@
     <row r="34" ht="90" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>C4</t>
+          <t>C3</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Rotate GitHub PAT (because old PAT was committed in SESSION_HANDOFF files)</t>
+          <t>My Studies CSV/XLSX export (John as design partner)</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr"/>
@@ -2057,13 +2054,14 @@
       <c r="E34" s="2" t="inlineStr"/>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: no ghp_* or github_pat_* patterns in current
-SESSION_HANDOFF.md or SESSION_HANDOFF-2.md as of 2026-05-01.</t>
+          <t>Closure evidence: client/src/pages/DashboardPage.tsx line 46 calls
+/api/my-studies/export. server/routes.ts line 1491 implements the
+endpoint. Pulled forward into pre-COLA per user instruction.</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>session 299e9a73, ~2026-04-28.
+          <t>session 299e9a73 turn 5, ~2026-04-28.
 ---</t>
         </is>
       </c>
@@ -2072,18 +2070,46 @@
     <row r="35" ht="90" customHeight="1">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>C6</t>
+          <t>C4</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>VeritaPolicy service-line filtering removed (formerly #4)</t>
+          <t>Rotate GitHub PAT (because old PAT was committed in SESSION_HANDOFF files)</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr"/>
       <c r="D35" s="3" t="inlineStr"/>
       <c r="E35" s="3" t="inlineStr"/>
       <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>Closure evidence: no ghp_* or github_pat_* patterns in current
+SESSION_HANDOFF.md or SESSION_HANDOFF-2.md as of 2026-05-01.</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>session 299e9a73, ~2026-04-28.
+---</t>
+        </is>
+      </c>
+      <c r="H35" s="3" t="inlineStr"/>
+    </row>
+    <row r="36" ht="90" customHeight="1">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>C6</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>VeritaPolicy service-line filtering removed (formerly #4)</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr"/>
+      <c r="D36" s="2" t="inlineStr"/>
+      <c r="E36" s="2" t="inlineStr"/>
+      <c r="F36" s="2" t="inlineStr">
         <is>
           <t>Closure rationale (operator decision 2026-05-10): Keep all
 VeritaPolicy rows. CFR-only references with no accreditor reference
@@ -2092,29 +2118,29 @@
 report misread the design intent.</t>
         </is>
       </c>
-      <c r="G35" s="3" t="inlineStr">
+      <c r="G36" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H35" s="3" t="inlineStr"/>
-    </row>
-    <row r="36" ht="90" customHeight="1">
-      <c r="A36" s="2" t="inlineStr">
+      <c r="H36" s="2" t="inlineStr"/>
+    </row>
+    <row r="37" ht="90" customHeight="1">
+      <c r="A37" s="3" t="inlineStr">
         <is>
           <t>C7</t>
         </is>
       </c>
-      <c r="B36" s="2" t="inlineStr">
+      <c r="B37" s="3" t="inlineStr">
         <is>
           <t>CLIA number format validation (formerly #13)</t>
         </is>
       </c>
-      <c r="C36" s="2" t="inlineStr"/>
-      <c r="D36" s="2" t="inlineStr"/>
-      <c r="E36" s="2" t="inlineStr"/>
-      <c r="F36" s="2" t="inlineStr">
+      <c r="C37" s="3" t="inlineStr"/>
+      <c r="D37" s="3" t="inlineStr"/>
+      <c r="E37" s="3" t="inlineStr"/>
+      <c r="F37" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: shared/validateClia.ts defines CLIA_REGEX =
 /^\d{2}D\d{7}$/ (line 24), validateClia() helper with whitespace
@@ -2125,30 +2151,30 @@
 shape exists and behaves as specified.</t>
         </is>
       </c>
-      <c r="G36" s="2" t="inlineStr">
+      <c r="G37" s="3" t="inlineStr">
         <is>
           <t>Agent verification 2026-05-10 via grep + file read.
 Operator confirmed shipped 2026-05-10.
 ---</t>
         </is>
       </c>
-      <c r="H36" s="2" t="inlineStr"/>
-    </row>
-    <row r="37" ht="90" customHeight="1">
-      <c r="A37" s="3" t="inlineStr">
+      <c r="H37" s="3" t="inlineStr"/>
+    </row>
+    <row r="38" ht="90" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
         <is>
           <t>C8</t>
         </is>
       </c>
-      <c r="B37" s="3" t="inlineStr">
+      <c r="B38" s="2" t="inlineStr">
         <is>
           <t>VeritaMap lab-wide menu toggle (formerly #19)</t>
         </is>
       </c>
-      <c r="C37" s="3" t="inlineStr"/>
-      <c r="D37" s="3" t="inlineStr"/>
-      <c r="E37" s="3" t="inlineStr"/>
-      <c r="F37" s="3" t="inlineStr">
+      <c r="C38" s="2" t="inlineStr"/>
+      <c r="D38" s="2" t="inlineStr"/>
+      <c r="E38" s="2" t="inlineStr"/>
+      <c r="F38" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: client/src/pages/VeritaMapLabwidePage.tsx
 exists and implements the labwide read-only union view. Route is
@@ -2158,59 +2184,59 @@
 parking lot plan (read-only union view, per-session toggle) shipped.</t>
         </is>
       </c>
-      <c r="G37" s="3" t="inlineStr">
+      <c r="G38" s="2" t="inlineStr">
         <is>
           <t>Agent verification 2026-05-10 via grep + file read.
 Operator confirmed shipped 2026-05-10.
 ---</t>
         </is>
       </c>
-      <c r="H37" s="3" t="inlineStr"/>
-    </row>
-    <row r="38" ht="90" customHeight="1">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>C9</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>Tier-1 smoke test checklist (formerly #6)</t>
-        </is>
-      </c>
-      <c r="C38" s="2" t="inlineStr"/>
-      <c r="D38" s="2" t="inlineStr"/>
-      <c r="E38" s="2" t="inlineStr"/>
-      <c r="F38" s="2" t="inlineStr">
-        <is>
-          <t>Closure evidence: docs/smoke-test-tier1.md documents the Tier-1
-smoke-test process and post-deploy verification steps. Shipped via
-PR #81 as part of the 2026-05-10 wave.</t>
-        </is>
-      </c>
-      <c r="G38" s="2" t="inlineStr">
-        <is>
-          <t>Operator instruction 2026-05-10 in this session.
----</t>
-        </is>
-      </c>
       <c r="H38" s="2" t="inlineStr"/>
     </row>
     <row r="39" ht="90" customHeight="1">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>C10</t>
+          <t>C9</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>Per-module gating (formerly #7)</t>
+          <t>Tier-1 smoke test checklist (formerly #6)</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr"/>
       <c r="D39" s="3" t="inlineStr"/>
       <c r="E39" s="3" t="inlineStr"/>
       <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>Closure evidence: docs/smoke-test-tier1.md documents the Tier-1
+smoke-test process and post-deploy verification steps. Shipped via
+PR #81 as part of the 2026-05-10 wave.</t>
+        </is>
+      </c>
+      <c r="G39" s="3" t="inlineStr">
+        <is>
+          <t>Operator instruction 2026-05-10 in this session.
+---</t>
+        </is>
+      </c>
+      <c r="H39" s="3" t="inlineStr"/>
+    </row>
+    <row r="40" ht="90" customHeight="1">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>C10</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Per-module gating (formerly #7)</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr"/>
+      <c r="D40" s="2" t="inlineStr"/>
+      <c r="E40" s="2" t="inlineStr"/>
+      <c r="F40" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: Client-side useIsReadOnly module keys wired
 on client/src/pages/VeritaPolicyAppPage.tsx and
@@ -2225,29 +2251,29 @@
 PR #76.</t>
         </is>
       </c>
-      <c r="G39" s="3" t="inlineStr">
+      <c r="G40" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H39" s="3" t="inlineStr"/>
-    </row>
-    <row r="40" ht="90" customHeight="1">
-      <c r="A40" s="2" t="inlineStr">
+      <c r="H40" s="2" t="inlineStr"/>
+    </row>
+    <row r="41" ht="90" customHeight="1">
+      <c r="A41" s="3" t="inlineStr">
         <is>
           <t>C11</t>
         </is>
       </c>
-      <c r="B40" s="2" t="inlineStr">
+      <c r="B41" s="3" t="inlineStr">
         <is>
           <t>VeritaStock shipped copy (formerly #8)</t>
         </is>
       </c>
-      <c r="C40" s="2" t="inlineStr"/>
-      <c r="D40" s="2" t="inlineStr"/>
-      <c r="E40" s="2" t="inlineStr"/>
-      <c r="F40" s="2" t="inlineStr">
+      <c r="C41" s="3" t="inlineStr"/>
+      <c r="D41" s="3" t="inlineStr"/>
+      <c r="E41" s="3" t="inlineStr"/>
+      <c r="F41" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: client/src/pages/ArticleInventoryManagementPage.tsx
 line 305 footer reads "platform that includes VeritaStock™" instead
@@ -2255,29 +2281,29 @@
 on /resources/laboratory-inventory-management. Shipped via PR #75.</t>
         </is>
       </c>
-      <c r="G40" s="2" t="inlineStr">
+      <c r="G41" s="3" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H40" s="2" t="inlineStr"/>
-    </row>
-    <row r="41" ht="90" customHeight="1">
-      <c r="A41" s="3" t="inlineStr">
+      <c r="H41" s="3" t="inlineStr"/>
+    </row>
+    <row r="42" ht="90" customHeight="1">
+      <c r="A42" s="2" t="inlineStr">
         <is>
           <t>C12</t>
         </is>
       </c>
-      <c r="B41" s="3" t="inlineStr">
+      <c r="B42" s="2" t="inlineStr">
         <is>
           <t>Admin report one-row-per-lab (formerly #14)</t>
         </is>
       </c>
-      <c r="C41" s="3" t="inlineStr"/>
-      <c r="D41" s="3" t="inlineStr"/>
-      <c r="E41" s="3" t="inlineStr"/>
-      <c r="F41" s="3" t="inlineStr">
+      <c r="C42" s="2" t="inlineStr"/>
+      <c r="D42" s="2" t="inlineStr"/>
+      <c r="E42" s="2" t="inlineStr"/>
+      <c r="F42" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: /api/admin/report rewritten in
 server/routes.ts (~line 595) to LEFT JOIN labs on
@@ -2292,33 +2318,6 @@
 prerequisite, not a code bug). Shipped via PR #85.</t>
         </is>
       </c>
-      <c r="G41" s="3" t="inlineStr">
-        <is>
-          <t>Operator instruction 2026-05-10 in this session.
----</t>
-        </is>
-      </c>
-      <c r="H41" s="3" t="inlineStr"/>
-    </row>
-    <row r="42" ht="90" customHeight="1">
-      <c r="A42" s="2" t="inlineStr">
-        <is>
-          <t>C14</t>
-        </is>
-      </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>UI relabel "CLIA TEa" -&gt; "Lab-Set Internal Goal" (formerly #1)</t>
-        </is>
-      </c>
-      <c r="C42" s="2" t="inlineStr"/>
-      <c r="D42" s="2" t="inlineStr"/>
-      <c r="E42" s="2" t="inlineStr"/>
-      <c r="F42" s="2" t="inlineStr">
-        <is>
-          <t>Closure evidence: Shipped across four PRs over 2026-05-10.</t>
-        </is>
-      </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
@@ -2330,18 +2329,45 @@
     <row r="43" ht="90" customHeight="1">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>C13</t>
+          <t>C14</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>WSLH PT vendor (formerly #15)</t>
+          <t>UI relabel "CLIA TEa" -&gt; "Lab-Set Internal Goal" (formerly #1)</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr"/>
       <c r="D43" s="3" t="inlineStr"/>
       <c r="E43" s="3" t="inlineStr"/>
       <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>Closure evidence: Shipped across four PRs over 2026-05-10.</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="inlineStr">
+        <is>
+          <t>Operator instruction 2026-05-10 in this session.
+---</t>
+        </is>
+      </c>
+      <c r="H43" s="3" t="inlineStr"/>
+    </row>
+    <row r="44" ht="90" customHeight="1">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>C13</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>WSLH PT vendor (formerly #15)</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr"/>
+      <c r="D44" s="2" t="inlineStr"/>
+      <c r="E44" s="2" t="inlineStr"/>
+      <c r="F44" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: Shipped 2026-05-10 via PR #79 (merge commit
 eeebc6e; merged after rebase to resolve a server/db.ts collision
@@ -2359,38 +2385,9 @@
 'WSLH' is the post-deploy success signal. Shipped via PR #79.</t>
         </is>
       </c>
-      <c r="G43" s="3" t="inlineStr">
+      <c r="G44" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
----</t>
-        </is>
-      </c>
-      <c r="H43" s="3" t="inlineStr"/>
-    </row>
-    <row r="44" ht="90" customHeight="1">
-      <c r="A44" s="2" t="inlineStr">
-        <is>
-          <t>C15</t>
-        </is>
-      </c>
-      <c r="B44" s="2" t="inlineStr">
-        <is>
-          <t>VeritaStock lot tracking + expiration + reorder alerts (formerly #21)</t>
-        </is>
-      </c>
-      <c r="C44" s="2" t="inlineStr"/>
-      <c r="D44" s="2" t="inlineStr"/>
-      <c r="E44" s="2" t="inlineStr"/>
-      <c r="F44" s="2" t="inlineStr">
-        <is>
-          <t>Closure evidence: VeritaStock™ shipped the bench-level inventory
-features the Perplexity competitor analysis identified as a gap:</t>
-        </is>
-      </c>
-      <c r="G44" s="2" t="inlineStr">
-        <is>
-          <t>Originally Perplexity competitor analysis 2026-05-10.
-Audit 2026-05-21 confirmed the feature set ships today.
 ---</t>
         </is>
       </c>
@@ -2399,12 +2396,12 @@
     <row r="45" ht="90" customHeight="1">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>C16</t>
+          <t>C15</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>PAL studies guided workflow (formerly #23)</t>
+          <t>VeritaStock lot tracking + expiration + reorder alerts (formerly #21)</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr"/>
@@ -2412,15 +2409,14 @@
       <c r="E45" s="3" t="inlineStr"/>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: VeritaCheck™ already ships the Precision /
-Accuracy / Linearity (PAL) study set under EP-protocol naming:</t>
+          <t>Closure evidence: VeritaStock™ shipped the bench-level inventory
+features the Perplexity competitor analysis identified as a gap:</t>
         </is>
       </c>
       <c r="G45" s="3" t="inlineStr">
         <is>
           <t>Originally Perplexity competitor analysis 2026-05-10.
-Audit 2026-05-21 confirmed the EP studies cover the PAL framing in
-full.
+Audit 2026-05-21 confirmed the feature set ships today.
 ---</t>
         </is>
       </c>
@@ -2429,12 +2425,12 @@
     <row r="46" ht="90" customHeight="1">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>C17</t>
+          <t>C16</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Source-grounded 21/29/45 CFR + 42 CFR 482-485 (formerly #26)</t>
+          <t>PAL studies guided workflow (formerly #23)</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr"/>
@@ -2442,35 +2438,65 @@
       <c r="E46" s="2" t="inlineStr"/>
       <c r="F46" s="2" t="inlineStr">
         <is>
+          <t>Closure evidence: VeritaCheck™ already ships the Precision /
+Accuracy / Linearity (PAL) study set under EP-protocol naming:</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>Originally Perplexity competitor analysis 2026-05-10.
+Audit 2026-05-21 confirmed the EP studies cover the PAL framing in
+full.
+---</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr"/>
+    </row>
+    <row r="47" ht="90" customHeight="1">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>C17</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>Source-grounded 21/29/45 CFR + 42 CFR 482-485 (formerly #26)</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr"/>
+      <c r="D47" s="3" t="inlineStr"/>
+      <c r="E47" s="3" t="inlineStr"/>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
           <t>Closure evidence: PR #301 (commit 8c27806, merged 2026-05-21)
 source-grounded the 74 remaining non-493 entries in
 server/cfrRequirements.ts against verbatim eCFR XML. Breakdown
 shipped:</t>
         </is>
       </c>
-      <c r="G46" s="2" t="inlineStr">
+      <c r="G47" s="3" t="inlineStr">
         <is>
           <t>PR #301; tasks #18 in the in-session task tracker.
 ---</t>
         </is>
       </c>
-      <c r="H46" s="2" t="inlineStr"/>
-    </row>
-    <row r="47" ht="90" customHeight="1">
-      <c r="A47" s="3" t="inlineStr">
+      <c r="H47" s="3" t="inlineStr"/>
+    </row>
+    <row r="48" ht="90" customHeight="1">
+      <c r="A48" s="2" t="inlineStr">
         <is>
           <t>C18</t>
         </is>
       </c>
-      <c r="B47" s="3" t="inlineStr">
+      <c r="B48" s="2" t="inlineStr">
         <is>
           <t>VeritaPolicy "Non CLIA" chapter rename (formerly #3)</t>
         </is>
       </c>
-      <c r="C47" s="3" t="inlineStr"/>
-      <c r="D47" s="3" t="inlineStr"/>
-      <c r="E47" s="3" t="inlineStr"/>
-      <c r="F47" s="3" t="inlineStr">
+      <c r="C48" s="2" t="inlineStr"/>
+      <c r="D48" s="2" t="inlineStr"/>
+      <c r="E48" s="2" t="inlineStr"/>
+      <c r="F48" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #300 (commit 34d7707, merged 2026-05-21)
 renamed all 44 user-facing chapter labels in
@@ -2481,7 +2507,7 @@
 page.</t>
         </is>
       </c>
-      <c r="G47" s="3" t="inlineStr">
+      <c r="G48" s="2" t="inlineStr">
         <is>
           <t>CAP customer screenshot of the /veritapolicy chapter
 headers, 2026-05-01 evening. PR #300; tasks #17 in the in-session
@@ -2489,23 +2515,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H47" s="3" t="inlineStr"/>
-    </row>
-    <row r="48" ht="90" customHeight="1">
-      <c r="A48" s="2" t="inlineStr">
+      <c r="H48" s="2" t="inlineStr"/>
+    </row>
+    <row r="49" ht="90" customHeight="1">
+      <c r="A49" s="3" t="inlineStr">
         <is>
           <t>C19</t>
         </is>
       </c>
-      <c r="B48" s="2" t="inlineStr">
+      <c r="B49" s="3" t="inlineStr">
         <is>
           <t>VeritaStock department-scope toggle (formerly #31)</t>
         </is>
       </c>
-      <c r="C48" s="2" t="inlineStr"/>
-      <c r="D48" s="2" t="inlineStr"/>
-      <c r="E48" s="2" t="inlineStr"/>
-      <c r="F48" s="2" t="inlineStr">
+      <c r="C49" s="3" t="inlineStr"/>
+      <c r="D49" s="3" t="inlineStr"/>
+      <c r="E49" s="3" t="inlineStr"/>
+      <c r="F49" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #319 (commit d01f5fe, merged 2026-05-22)
 shipped the persistent dept-scope toggle on VeritaStockPage. A new
@@ -2516,7 +2542,7 @@
 workspace without re-filtering.</t>
         </is>
       </c>
-      <c r="G48" s="2" t="inlineStr">
+      <c r="G49" s="3" t="inlineStr">
         <is>
           <t>John, San Carlos lab, 2026-05-21. Same conversation that
 drove the vendor dropdown (PR #304), FILTERED VIEW banner (PR #305),
@@ -2524,23 +2550,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H48" s="2" t="inlineStr"/>
-    </row>
-    <row r="49" ht="90" customHeight="1">
-      <c r="A49" s="3" t="inlineStr">
+      <c r="H49" s="3" t="inlineStr"/>
+    </row>
+    <row r="50" ht="90" customHeight="1">
+      <c r="A50" s="2" t="inlineStr">
         <is>
           <t>C20</t>
         </is>
       </c>
-      <c r="B49" s="3" t="inlineStr">
+      <c r="B50" s="2" t="inlineStr">
         <is>
           <t>Primary-lab seat counting (formerly #12)</t>
         </is>
       </c>
-      <c r="C49" s="3" t="inlineStr"/>
-      <c r="D49" s="3" t="inlineStr"/>
-      <c r="E49" s="3" t="inlineStr"/>
-      <c r="F49" s="3" t="inlineStr">
+      <c r="C50" s="2" t="inlineStr"/>
+      <c r="D50" s="2" t="inlineStr"/>
+      <c r="E50" s="2" t="inlineStr"/>
+      <c r="F50" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: is_primary_lab INTEGER NOT NULL DEFAULT 0
 column was added to the lab_members table at db.ts:1276, with the
@@ -2551,7 +2577,7 @@
 is_primary_lab=1 ordering).</t>
         </is>
       </c>
-      <c r="G49" s="3" t="inlineStr">
+      <c r="G50" s="2" t="inlineStr">
         <is>
           <t>2026-05-07 multi-lab discussion. Build shipped as part
 of the Multi-Lab Tier 2 architecture work (Phase 3.x series, prior
@@ -2560,23 +2586,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H49" s="3" t="inlineStr"/>
-    </row>
-    <row r="50" ht="90" customHeight="1">
-      <c r="A50" s="2" t="inlineStr">
+      <c r="H50" s="2" t="inlineStr"/>
+    </row>
+    <row r="51" ht="90" customHeight="1">
+      <c r="A51" s="3" t="inlineStr">
         <is>
           <t>C21</t>
         </is>
       </c>
-      <c r="B50" s="2" t="inlineStr">
+      <c r="B51" s="3" t="inlineStr">
         <is>
           <t>Multi-lab pricing model — Option A (formerly #11)</t>
         </is>
       </c>
-      <c r="C50" s="2" t="inlineStr"/>
-      <c r="D50" s="2" t="inlineStr"/>
-      <c r="E50" s="2" t="inlineStr"/>
-      <c r="F50" s="2" t="inlineStr">
+      <c r="C51" s="3" t="inlineStr"/>
+      <c r="D51" s="3" t="inlineStr"/>
+      <c r="E51" s="3" t="inlineStr"/>
+      <c r="F51" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #322 (commit 0ccd925, merged 2026-05-22)
 added the customer-facing line to the pricing page that reflects
@@ -2589,7 +2615,7 @@
 Enterprise+ block, reads:</t>
         </is>
       </c>
-      <c r="G50" s="2" t="inlineStr">
+      <c r="G51" s="3" t="inlineStr">
         <is>
           <t>2026-05-07 multi-lab discussion (Lisa Veri's
 canonical-case session). PR #322 (initial build); softening PR
@@ -2598,30 +2624,30 @@
 ---</t>
         </is>
       </c>
-      <c r="H50" s="2" t="inlineStr"/>
-    </row>
-    <row r="51" ht="90" customHeight="1">
-      <c r="A51" s="3" t="inlineStr">
+      <c r="H51" s="3" t="inlineStr"/>
+    </row>
+    <row r="52" ht="90" customHeight="1">
+      <c r="A52" s="2" t="inlineStr">
         <is>
           <t>C22</t>
         </is>
       </c>
-      <c r="B51" s="3" t="inlineStr">
+      <c r="B52" s="2" t="inlineStr">
         <is>
           <t>VeritaOps cost-per-test module (formerly #10)</t>
         </is>
       </c>
-      <c r="C51" s="3" t="inlineStr"/>
-      <c r="D51" s="3" t="inlineStr"/>
-      <c r="E51" s="3" t="inlineStr"/>
-      <c r="F51" s="3" t="inlineStr">
+      <c r="C52" s="2" t="inlineStr"/>
+      <c r="D52" s="2" t="inlineStr"/>
+      <c r="E52" s="2" t="inlineStr"/>
+      <c r="F52" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: v1 of the VeritaOps Cost-Per-Reportable-Test
 (CPRT) module shipped across PR #325 through PR #330 on 2026-05-22.
 The module is feature-complete for the typical lab director workflow.</t>
         </is>
       </c>
-      <c r="G51" s="3" t="inlineStr">
+      <c r="G52" s="2" t="inlineStr">
         <is>
           <t>This thread, 2026-05-07 12:05 PM CDT, user message:
 "Parking lot: build an operations module for cost per test
@@ -2630,262 +2656,262 @@
 ---</t>
         </is>
       </c>
-      <c r="H51" s="3" t="inlineStr"/>
-    </row>
-    <row r="52" ht="90" customHeight="1">
-      <c r="A52" s="2" t="inlineStr">
+      <c r="H52" s="2" t="inlineStr"/>
+    </row>
+    <row r="53" ht="90" customHeight="1">
+      <c r="A53" s="3" t="inlineStr">
         <is>
           <t>C23</t>
         </is>
       </c>
-      <c r="B52" s="2" t="inlineStr">
+      <c r="B53" s="3" t="inlineStr">
         <is>
           <t>CCL lab name visual disambiguation in lab switcher (formerly #34)</t>
         </is>
       </c>
-      <c r="C52" s="2" t="inlineStr"/>
-      <c r="D52" s="2" t="inlineStr">
+      <c r="C53" s="3" t="inlineStr"/>
+      <c r="D53" s="3" t="inlineStr">
         <is>
           <t>XS (under 1 day, actual)</t>
         </is>
       </c>
-      <c r="E52" s="2" t="inlineStr">
+      <c r="E53" s="3" t="inlineStr">
         <is>
           <t>Low — cosmetic; only mattered when Lisa or Michael picked the wrong lab from...</t>
         </is>
       </c>
-      <c r="F52" s="2" t="inlineStr">
+      <c r="F53" s="3" t="inlineStr">
         <is>
           <t>Effort: XS (under 1 day, actual)
 Importance: Low — cosmetic; only mattered when Lisa or Michael picked the wrong lab from the dropdown.</t>
         </is>
       </c>
-      <c r="G52" s="2" t="inlineStr">
+      <c r="G53" s="3" t="inlineStr">
         <is>
           <t>flagged 2026-05-23 immediately after provisioning Lisa's CCL lab; closed 2026-05-24.
 ---</t>
         </is>
       </c>
-      <c r="H52" s="2" t="inlineStr"/>
-    </row>
-    <row r="53" ht="90" customHeight="1">
-      <c r="A53" s="3" t="inlineStr">
+      <c r="H53" s="3" t="inlineStr"/>
+    </row>
+    <row r="54" ht="90" customHeight="1">
+      <c r="A54" s="2" t="inlineStr">
         <is>
           <t>C24</t>
         </is>
       </c>
-      <c r="B53" s="3" t="inlineStr">
+      <c r="B54" s="2" t="inlineStr">
         <is>
           <t>VC Unlimited Y1/Y2 price disclosure UX (formerly #35)</t>
         </is>
       </c>
-      <c r="C53" s="3" t="inlineStr"/>
-      <c r="D53" s="3" t="inlineStr">
+      <c r="C54" s="2" t="inlineStr"/>
+      <c r="D54" s="2" t="inlineStr">
         <is>
           <t>XS (under 1 day, actual)</t>
         </is>
       </c>
-      <c r="E53" s="3" t="inlineStr">
+      <c r="E54" s="2" t="inlineStr">
         <is>
           <t>Low when shipped (proactive, no customer complaint yet) — but high if a procu...</t>
         </is>
       </c>
-      <c r="F53" s="3" t="inlineStr">
+      <c r="F54" s="2" t="inlineStr">
         <is>
           <t>Effort: XS (under 1 day, actual)
 Importance: Low when shipped (proactive, no customer complaint yet) — but high if a procurement reviewer later disputes the $499 renewal as undisclosed.</t>
         </is>
       </c>
-      <c r="G53" s="3" t="inlineStr">
+      <c r="G54" s="2" t="inlineStr">
         <is>
           <t>Pricing rebuild 2026-05-23; closed 2026-05-24 proactively before any customer dispute.
 ---</t>
         </is>
       </c>
-      <c r="H53" s="3" t="inlineStr"/>
-    </row>
-    <row r="54" ht="90" customHeight="1">
-      <c r="A54" s="2" t="inlineStr">
+      <c r="H54" s="2" t="inlineStr"/>
+    </row>
+    <row r="55" ht="90" customHeight="1">
+      <c r="A55" s="3" t="inlineStr">
         <is>
           <t>C25</t>
         </is>
       </c>
-      <c r="B54" s="2" t="inlineStr">
+      <c r="B55" s="3" t="inlineStr">
         <is>
           <t>VeritaQC Phase 1 (Levey-Jennings + Westgard live engine) (formerly #20)</t>
         </is>
       </c>
-      <c r="C54" s="2" t="inlineStr"/>
-      <c r="D54" s="2" t="inlineStr">
+      <c r="C55" s="3" t="inlineStr"/>
+      <c r="D55" s="3" t="inlineStr">
         <is>
           <t>L (about 5 days end-to-end, actual: Phase 0 schema → Phase 1A evaluator → 1B...</t>
         </is>
       </c>
-      <c r="E54" s="2" t="inlineStr">
+      <c r="E55" s="3" t="inlineStr">
         <is>
           <t>High — largest single gap vs myLabCompliance.io per Perplexity competitor ana...</t>
         </is>
       </c>
-      <c r="F54" s="2" t="inlineStr">
+      <c r="F55" s="3" t="inlineStr">
         <is>
           <t>Effort: L (about 5 days end-to-end, actual: Phase 0 schema → Phase 1A evaluator → 1B entry UI → 1C daily review → 1D monthly PDF + attestation)
 Importance: High — largest single gap vs myLabCompliance.io per Perplexity competitor analysis; promotes VeritaAssure from documentation tool to lab operations platform.</t>
         </is>
       </c>
-      <c r="G54" s="2" t="inlineStr">
+      <c r="G55" s="3" t="inlineStr">
         <is>
           <t>Perplexity competitor analysis 2026-05-10. Scoping confirmed via the build_phase1_mockup.py iterations 2026-05-24. Shipped 2026-05-25.
 ---</t>
         </is>
       </c>
-      <c r="H54" s="2" t="inlineStr"/>
-    </row>
-    <row r="55" ht="90" customHeight="1">
-      <c r="A55" s="3" t="inlineStr">
+      <c r="H55" s="3" t="inlineStr"/>
+    </row>
+    <row r="56" ht="90" customHeight="1">
+      <c r="A56" s="2" t="inlineStr">
         <is>
           <t>C26</t>
         </is>
       </c>
-      <c r="B55" s="3" t="inlineStr">
+      <c r="B56" s="2" t="inlineStr">
         <is>
           <t>VeritaLab CMS-116 application support + state licensing registry (formerly #22)</t>
         </is>
       </c>
-      <c r="C55" s="3" t="inlineStr"/>
-      <c r="D55" s="3" t="inlineStr">
+      <c r="C56" s="2" t="inlineStr"/>
+      <c r="D56" s="2" t="inlineStr">
         <is>
           <t>M (1-2 weeks for v1, actual)</t>
         </is>
       </c>
-      <c r="E55" s="3" t="inlineStr">
+      <c r="E56" s="2" t="inlineStr">
         <is>
           <t>Medium — competitor parity (myLabCompliance.io) plus useful at lab startup an...</t>
         </is>
       </c>
-      <c r="F55" s="3" t="inlineStr">
+      <c r="F56" s="2" t="inlineStr">
         <is>
           <t>Effort: M (1-2 weeks for v1, actual)
 Importance: Medium — competitor parity (myLabCompliance.io) plus useful at lab startup and at certificate-type changes.</t>
         </is>
       </c>
-      <c r="G55" s="3" t="inlineStr">
+      <c r="G56" s="2" t="inlineStr">
         <is>
           <t>Perplexity competitor analysis (myLabCompliance.io), 2026-05-10. Reclassified as a VeritaLab extension 2026-05-25. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H55" s="3" t="inlineStr"/>
-    </row>
-    <row r="56" ht="90" customHeight="1">
-      <c r="A56" s="2" t="inlineStr">
+      <c r="H56" s="2" t="inlineStr"/>
+    </row>
+    <row r="57" ht="90" customHeight="1">
+      <c r="A57" s="3" t="inlineStr">
         <is>
           <t>C27</t>
         </is>
       </c>
-      <c r="B56" s="2" t="inlineStr">
+      <c r="B57" s="3" t="inlineStr">
         <is>
           <t>Active vs view-only seat split (formerly #33)</t>
         </is>
       </c>
-      <c r="C56" s="2" t="inlineStr"/>
-      <c r="D56" s="2" t="inlineStr">
+      <c r="C57" s="3" t="inlineStr"/>
+      <c r="D57" s="3" t="inlineStr">
         <is>
           <t>M (~1 week of engineering, actual: shipped in a single multi-PR session)</t>
         </is>
       </c>
-      <c r="E56" s="2" t="inlineStr">
+      <c r="E57" s="3" t="inlineStr">
         <is>
           <t>Medium — closed the gap between /pricing copy and product behavior; gives sal...</t>
         </is>
       </c>
-      <c r="F56" s="2" t="inlineStr">
+      <c r="F57" s="3" t="inlineStr">
         <is>
           <t>Effort: M (~1 week of engineering, actual: shipped in a single multi-PR session)
 Importance: Medium — closed the gap between /pricing copy and product behavior; gives sales a clean answer for "do you charge for our medical director?"</t>
         </is>
       </c>
-      <c r="G56" s="2" t="inlineStr">
+      <c r="G57" s="3" t="inlineStr">
         <is>
           <t>Pricing analysis doc Decision 3 (2026-05-21); MEDIUM scenario revised 2026-05-29 to retire the "unlimited view-only" claim. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H56" s="2" t="inlineStr"/>
-    </row>
-    <row r="57" ht="90" customHeight="1">
-      <c r="A57" s="3" t="inlineStr">
+      <c r="H57" s="3" t="inlineStr"/>
+    </row>
+    <row r="58" ht="90" customHeight="1">
+      <c r="A58" s="2" t="inlineStr">
         <is>
           <t>C28</t>
         </is>
       </c>
-      <c r="B57" s="3" t="inlineStr">
+      <c r="B58" s="2" t="inlineStr">
         <is>
           <t>"Why VeritaCheck" comparative one-pager (formerly #37)</t>
         </is>
       </c>
-      <c r="C57" s="3" t="inlineStr"/>
-      <c r="D57" s="3" t="inlineStr">
+      <c r="C58" s="2" t="inlineStr"/>
+      <c r="D58" s="2" t="inlineStr">
         <is>
           <t>S (one design pass + four claim paragraphs + PDF + matching marketing-site pa...</t>
         </is>
       </c>
-      <c r="E57" s="3" t="inlineStr">
+      <c r="E58" s="2" t="inlineStr">
         <is>
           <t>Medium — closed a positioning gap surfaced by six COLA conference attendees a...</t>
         </is>
       </c>
-      <c r="F57" s="3" t="inlineStr">
+      <c r="F58" s="2" t="inlineStr">
         <is>
           <t>Effort: S (one design pass + four claim paragraphs + PDF + matching marketing-site page, actual)
 Importance: Medium — closed a positioning gap surfaced by six COLA conference attendees attached to a legacy verification tool; converts product-quality advantage into a leave-behind Lisa can hand out.</t>
         </is>
       </c>
-      <c r="G57" s="3" t="inlineStr">
+      <c r="G58" s="2" t="inlineStr">
         <is>
           <t>2026-05-11 / 2026-05-12 conference notes review with Michael. Conference attendees (Whitehead, Odegard, Othman, Molinelli, Kyle, Allred) expressed interest in equivalent / superior product. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H57" s="3" t="inlineStr"/>
-    </row>
-    <row r="58" ht="90" customHeight="1">
-      <c r="A58" s="2" t="inlineStr">
+      <c r="H58" s="2" t="inlineStr"/>
+    </row>
+    <row r="59" ht="90" customHeight="1">
+      <c r="A59" s="3" t="inlineStr">
         <is>
           <t>C29</t>
         </is>
       </c>
-      <c r="B58" s="2" t="inlineStr">
+      <c r="B59" s="3" t="inlineStr">
         <is>
           <t>VeritaPolicy approval workflow — MediaLab functional mirror</t>
         </is>
       </c>
-      <c r="C58" s="2" t="inlineStr"/>
-      <c r="D58" s="2" t="inlineStr">
+      <c r="C59" s="3" t="inlineStr"/>
+      <c r="D59" s="3" t="inlineStr">
         <is>
           <t>XL (one focused session, 12 PRs landed)</t>
         </is>
       </c>
-      <c r="E58" s="2" t="inlineStr">
+      <c r="E59" s="3" t="inlineStr">
         <is>
           <t>High — replaces MediaLab Document Control ($752/$2,250 starting price, scalin...</t>
         </is>
       </c>
-      <c r="F58" s="2" t="inlineStr">
+      <c r="F59" s="3" t="inlineStr">
         <is>
           <t>Effort: XL (one focused session, 12 PRs landed)
 Importance: High — replaces MediaLab Document Control ($752/$2,250 starting price, scaling to $10K-$20K/yr at enterprise per Capterra public data) with an included VeritaPolicy feature; closes a real positioning gap and gives sales a direct comparator line.</t>
         </is>
       </c>
-      <c r="G58" s="2" t="inlineStr">
+      <c r="G59" s="3" t="inlineStr">
         <is>
           <t>Pricing strategy conversation 2026-05-29 (Michael: "I don't like bolt-ons; we should replicate this") → scoped 8 phases → shipped all 12 PRs in single session. Shipped 2026-05-29.
 ---</t>
         </is>
       </c>
-      <c r="H58" s="2" t="inlineStr"/>
+      <c r="H59" s="3" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H58"/>
+  <autoFilter ref="A1:H59"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
TASK: Parking lot - close #45 (VeritaDC attestation tracker) as C58; regen xlsx
PLAN:
  1. Add CLOSED entry C58 (VeritaDC attestation tracker + My Documents rename; shipped #1447/#1449).
  2. Regenerate PARKING_LOT.xlsx.

Self-check:
  - md + xlsx committed together per the sync rule.
  - Gate 3 N/A (internal documentation).
</commit_message>
<xml_diff>
--- a/PARKING_LOT.xlsx
+++ b/PARKING_LOT.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$58</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$59</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RETIRED'!$A$1:$H$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1093,7 +1093,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H58"/>
+  <dimension ref="A1:H59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1151,24 +1151,24 @@
     <row r="2" ht="90" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>C57</t>
+          <t>C58</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Hide sections a lab does not use from a master list (was #47)</t>
+          <t>VeritaDC per-document attestation tracker + "My Documents" rename (built as #45)</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr"/>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>was S-M / Importance: Medium-High (prospect-requested)</t>
+          <t>was M / Importance: Medium-High</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Effort: was S-M / Importance: Medium-High (prospect-requested)</t>
+          <t>Effort: was M / Importance: Medium-High</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
@@ -1177,24 +1177,24 @@
     <row r="3" ht="90" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>C56</t>
+          <t>C57</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>VeritaCEU: curated free continuing-education provider list (was #53)</t>
+          <t>Hide sections a lab does not use from a master list (was #47)</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr"/>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>was S / Importance: Low-Medium</t>
+          <t>was S-M / Importance: Medium-High (prospect-requested)</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Effort: was S / Importance: Low-Medium</t>
+          <t>Effort: was S-M / Importance: Medium-High (prospect-requested)</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr"/>
@@ -1203,24 +1203,24 @@
     <row r="4" ht="90" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>C55</t>
+          <t>C56</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>VeritaScan: let sites add their own custom questions (was #55)</t>
+          <t>VeritaCEU: curated free continuing-education provider list (was #53)</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr"/>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>was M / Importance: Medium-High</t>
+          <t>was S / Importance: Low-Medium</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Effort: was M / Importance: Medium-High</t>
+          <t>Effort: was S / Importance: Low-Medium</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr"/>
@@ -1229,24 +1229,24 @@
     <row r="5" ht="90" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>C54</t>
+          <t>C55</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>VeritaQC: at-entry warning when a QC point is outside 2 SD (was #56)</t>
+          <t>VeritaScan: let sites add their own custom questions (was #55)</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr"/>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>was S-M (shipped S) / Importance: High</t>
+          <t>was M / Importance: Medium-High</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Effort: was S-M (shipped S) / Importance: High</t>
+          <t>Effort: was M / Importance: Medium-High</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr"/>
@@ -1255,24 +1255,24 @@
     <row r="6" ht="90" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>C53</t>
+          <t>C54</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>VeritaTrack: quarterly task loaded as monthly until re-saved (was #54)</t>
+          <t>VeritaQC: at-entry warning when a QC point is outside 2 SD (was #56)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr"/>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>was S / Importance: Medium</t>
+          <t>was S-M (shipped S) / Importance: High</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Effort: was S / Importance: Medium</t>
+          <t>Effort: was S-M (shipped S) / Importance: High</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
@@ -1281,24 +1281,24 @@
     <row r="7" ht="90" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>C52</t>
+          <t>C53</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>VeritaResponse internal NCE / non-conforming event (was #36)</t>
+          <t>VeritaTrack: quarterly task loaded as monthly until re-saved (was #54)</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr"/>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>was L (shipped as MEDIUM) / Importance: High</t>
+          <t>was S / Importance: Medium</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Effort: was L (shipped as MEDIUM) / Importance: High</t>
+          <t>Effort: was S / Importance: Medium</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr"/>
@@ -1307,24 +1307,24 @@
     <row r="8" ht="90" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>C49</t>
+          <t>C52</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Competency "assessed this cycle" cadence-aware window (was #50)</t>
+          <t>VeritaResponse internal NCE / non-conforming event (was #36)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr"/>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>was S-M / Importance: Medium</t>
+          <t>was L (shipped as MEDIUM) / Importance: High</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Effort: was S-M / Importance: Medium</t>
+          <t>Effort: was L (shipped as MEDIUM) / Importance: High</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
@@ -1333,12 +1333,12 @@
     <row r="9" ht="90" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>C50</t>
+          <t>C49</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>VeritaTrack task owner + owner-only reminder routing (was #51)</t>
+          <t>Competency "assessed this cycle" cadence-aware window (was #50)</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr"/>
@@ -1359,24 +1359,24 @@
     <row r="10" ht="90" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>C51</t>
+          <t>C50</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Designate Medical Director by picking a lab member (was #52, core)</t>
+          <t>VeritaTrack task owner + owner-only reminder routing (was #51)</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr"/>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>was S-M / Importance: Medium-High</t>
+          <t>was S-M / Importance: Medium</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Effort: was S-M / Importance: Medium-High</t>
+          <t>Effort: was S-M / Importance: Medium</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
@@ -1385,24 +1385,24 @@
     <row r="11" ht="90" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>C47</t>
+          <t>C51</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Unregulated-analyte / Alternative Assessment (AAA) coverage (was #18)</t>
+          <t>Designate Medical Director by picking a lab member (was #52, core)</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr"/>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>was S (Phase 3) / Importance: Medium</t>
+          <t>was S-M / Importance: Medium-High</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Effort: was S (Phase 3) / Importance: Medium</t>
+          <t>Effort: was S-M / Importance: Medium-High</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr"/>
@@ -1411,24 +1411,24 @@
     <row r="12" ht="90" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>C48</t>
+          <t>C47</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>VeritaResponse post-survey deficiency module (was #17)</t>
+          <t>Unregulated-analyte / Alternative Assessment (AAA) coverage (was #18)</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr"/>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>was XL / Importance: High</t>
+          <t>was S (Phase 3) / Importance: Medium</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Effort: was XL / Importance: High</t>
+          <t>Effort: was S (Phase 3) / Importance: Medium</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr"/>
@@ -1437,39 +1437,38 @@
     <row r="13" ht="90" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>C45</t>
+          <t>C48</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Unify coverage/competency recurrence helper (was #49) - closed as non-issue</t>
+          <t>VeritaResponse post-survey deficiency module (was #17)</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr"/>
-      <c r="D13" s="3" t="inlineStr"/>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>was XL / Importance: High</t>
+        </is>
+      </c>
       <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: Investigated 2026-09-24 before building. The coverage recurrence math (+6-month interval, signed-resets-to-missing, nextDueOn/overdue, isFailVerdict) is ALREADY single-source in server/veritacheckCoverage.ts (computeCoverageFrom). server/coverageReport.ts and the routes.ts coverage export do not recompute it; they consume the computed nextDueOn/overdue/status fields and apply small surface-specific presentation labels (deliberately different vocabularies per surface, so they should not be merged). The only truly identical duplicate is a one-line date formatter. The competency "owed" derivation is NOT the same cadence: competency follows the CLIA milestone schedule (initial / semiannual year 1 / annual, 42 CFR 493.1451(b)(8) and 493.1235), which is a different regulatory interval from the coverage 6-month rule (493.1281 / 493.1255) and must stay separate. No worthwhile extraction; merging the two cadences would be wrong. Closed 2026-09-24. (The year-1 competency-window refinement remains tracked separately as #50.)</t>
-        </is>
-      </c>
-      <c r="G13" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-24 session, "keep working" pass; scoped read-only, found no real duplication.
----</t>
-        </is>
-      </c>
+          <t>Effort: was XL / Importance: High</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr"/>
       <c r="H13" s="3" t="inlineStr"/>
     </row>
     <row r="14" ht="90" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>C46</t>
+          <t>C45</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Verified-users product-update send path (wrong-list incident fix)</t>
+          <t>Unify coverage/competency recurrence helper (was #49) - closed as non-issue</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr"/>
@@ -1477,12 +1476,12 @@
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: Shipped PR #1324 (merged 4e05506a, deploy ACTIVE). New POST /api/admin/users/send targets registered VeritaAssure account holders (the users table), never the Lab Director's Briefing subscriber list. Separate explicitly-named endpoint (not a flag with a dangerous default), account-holder email framing, excludes suppressed emails and RFC-reserved test domains, CC owner, dryRun + testTo previews. Public unsubscribe now upserts a suppression row so opt-outs are honored across both audiences. Live dryRun: 49 verified-user recipients vs 673 on the Briefing list. Receipts: scripts/verify-product-update-send.mts 24/24, tsc clean, rendered sample inspected. Fixes the fallout from the 2026-09-23/24 wrong-list send (a product update went to the 675-person Briefing list). Nothing sends without Michael's explicit "send it."</t>
+          <t>Closure evidence: Investigated 2026-09-24 before building. The coverage recurrence math (+6-month interval, signed-resets-to-missing, nextDueOn/overdue, isFailVerdict) is ALREADY single-source in server/veritacheckCoverage.ts (computeCoverageFrom). server/coverageReport.ts and the routes.ts coverage export do not recompute it; they consume the computed nextDueOn/overdue/status fields and apply small surface-specific presentation labels (deliberately different vocabularies per surface, so they should not be merged). The only truly identical duplicate is a one-line date formatter. The competency "owed" derivation is NOT the same cadence: competency follows the CLIA milestone schedule (initial / semiannual year 1 / annual, 42 CFR 493.1451(b)(8) and 493.1235), which is a different regulatory interval from the coverage 6-month rule (493.1281 / 493.1255) and must stay separate. No worthwhile extraction; merging the two cadences would be wrong. Closed 2026-09-24. (The year-1 competency-window refinement remains tracked separately as #50.)</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 session; Michael selected this as the next build after the #41 close.
+          <t>2026-09-24 session, "keep working" pass; scoped read-only, found no real duplication.
 ---</t>
         </is>
       </c>
@@ -1491,12 +1490,12 @@
     <row r="15" ht="90" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>C44</t>
+          <t>C46</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Verify-script convention backfill (was #41) + audit matcher fix</t>
+          <t>Verified-users product-update send path (wrong-list incident fix)</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr"/>
@@ -1504,12 +1503,12 @@
       <c r="E15" s="3" t="inlineStr"/>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: #41 was fully backfilled on 2026-06-13 (all 8 high-stakes scripts landed; see C30); it had only been mis-filed in OPEN. A 2026-09-24 re-audit initially reported 4 of 5 recent math/logic commits as missing a verify script, which was a FALSE POSITIVE: scripts/audit_verify_script_coverage.py matched only scripts/verify-*.js / .cjs, so it ignored the .mjs / .mts / .ts verify scripts the repo now ships (e.g. verify-ptcoag-multi.mts, verify-tea-criterion-format.mjs). Fixed the matcher to accept .js/.cjs/.mjs/.ts/.mts; re-run shows 5 of 5 covered, 0 debt. The convention is being followed. Closed 2026-09-24.</t>
+          <t>Closure evidence: Shipped PR #1324 (merged 4e05506a, deploy ACTIVE). New POST /api/admin/users/send targets registered VeritaAssure account holders (the users table), never the Lab Director's Briefing subscriber list. Separate explicitly-named endpoint (not a flag with a dangerous default), account-holder email framing, excludes suppressed emails and RFC-reserved test domains, CC owner, dryRun + testTo previews. Public unsubscribe now upserts a suppression row so opt-outs are honored across both audiences. Live dryRun: 49 verified-user recipients vs 673 on the Briefing list. Receipts: scripts/verify-product-update-send.mts 24/24, tsc clean, rendered sample inspected. Fixes the fallout from the 2026-09-23/24 wrong-list send (a product update went to the 675-person Briefing list). Nothing sends without Michael's explicit "send it."</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>2026-09-24 session, "keep working" pass; audit tooling bug found + fixed.
+          <t>2026-09-24 session; Michael selected this as the next build after the #41 close.
 ---</t>
         </is>
       </c>
@@ -1518,12 +1517,12 @@
     <row r="16" ht="90" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>C43</t>
+          <t>C44</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>VeritaStaff instrument-centric (dual) assignment view</t>
+          <t>Verify-script convention backfill (was #41) + audit matcher fix</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr"/>
@@ -1531,12 +1530,12 @@
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1320. GET/PUT /staff/instruments/:id/employees (transpose of the per-employee endpoints); an "Assign by Instrument" dialog lets a director pick a test system or manual test and check off who runs it. Same staff_employee_instruments join, with the 42 CFR 493.1235(a) duty-change event emitted on newly-added pairs so both orientations trigger the same reassessment. GET verified live on SCAHC lab 2. Closed 2026-09-24.</t>
+          <t>Closure evidence: #41 was fully backfilled on 2026-06-13 (all 8 high-stakes scripts landed; see C30); it had only been mis-filed in OPEN. A 2026-09-24 re-audit initially reported 4 of 5 recent math/logic commits as missing a verify script, which was a FALSE POSITIVE: scripts/audit_verify_script_coverage.py matched only scripts/verify-*.js / .cjs, so it ignored the .mjs / .mts / .ts verify scripts the repo now ships (e.g. verify-ptcoag-multi.mts, verify-tea-criterion-format.mjs). Fixed the matcher to accept .js/.cjs/.mjs/.ts/.mts; re-run shows 5 of 5 covered, 0 debt. The convention is being followed. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 session, Michael ("in staff we should also give the dual view when assigning coverage to test systems or manual tests").
+          <t>2026-09-24 session, "keep working" pass; audit tooling bug found + fixed.
 ---</t>
         </is>
       </c>
@@ -1545,12 +1544,12 @@
     <row r="17" ht="90" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>C42</t>
+          <t>C43</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>VeritaComp coverage map (required-vs-assessed matrix, dual view)</t>
+          <t>VeritaStaff instrument-centric (dual) assignment view</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr"/>
@@ -1558,12 +1557,12 @@
       <c r="E17" s="3" t="inlineStr"/>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1319 (+ status layer PR #1316). /competency/owed returns per-item assessed (locked passing assessment this cycle on a covering method group) + per-employee CLIA status; CompetencyCoverageMap renders a By-employee / By-instrument matrix (Assessed / Owed / Overdue / Gap). Verified live on SCAHC lab 2 (owed 116, assessed 2, gaps 0). Completes #48 as the VeritaCheck-parity coverage map. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1320. GET/PUT /staff/instruments/:id/employees (transpose of the per-employee endpoints); an "Assign by Instrument" dialog lets a director pick a test system or manual test and check off who runs it. Same staff_employee_instruments join, with the 42 CFR 493.1235(a) duty-change event emitted on newly-added pairs so both orientations trigger the same reassessment. GET verified live on SCAHC lab 2. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>2026-09-24 session, Michael ("are we building the competencies to have a coverage map, same as veritacheck?" then "build it").
+          <t>2026-09-24 session, Michael ("in staff we should also give the dual view when assigning coverage to test systems or manual tests").
 ---</t>
         </is>
       </c>
@@ -1572,12 +1571,12 @@
     <row r="18" ht="90" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>C41</t>
+          <t>C42</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>VeritaCheck coverage recurrence (method comparison + cal-ver/linearity + reports)</t>
+          <t>VeritaComp coverage map (required-vs-assessed matrix, dual view)</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr"/>
@@ -1585,12 +1584,12 @@
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: PRs #1317 (method comparison), #1318 (cal-ver/linearity), #1321 (report Next-due columns). Periodic verification (correlation/method comparison 42 CFR 493.1281; cal-ver/linearity 42 CFR 493.1255; both 6-month) now recurs: a signed study banks the cycle and rolls to next-due = signed + 6 months instead of reading "done" forever. Status Missing/Failed/Completed-unsigned + a "Next due on" column on-screen and in both coverage exports; also credits the previously-ignored "correlation" study type. Root cause: computeCoverageFrom marked requirements done on mere existence, no date logic. Verified live on SCAHC lab 2 (101 correlations + 11 cal-ver rows now carry a next-due). Engine-level, all facilities. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1319 (+ status layer PR #1316). /competency/owed returns per-item assessed (locked passing assessment this cycle on a covering method group) + per-employee CLIA status; CompetencyCoverageMap renders a By-employee / By-instrument matrix (Assessed / Owed / Overdue / Gap). Verified live on SCAHC lab 2 (owed 116, assessed 2, gaps 0). Completes #48 as the VeritaCheck-parity coverage map. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 session, Michael ("Look at San Carlos... they finished their last set of correlations (all 103) but their menu never reset").
+          <t>2026-09-24 session, Michael ("are we building the competencies to have a coverage map, same as veritacheck?" then "build it").
 ---</t>
         </is>
       </c>
@@ -1599,12 +1598,12 @@
     <row r="19" ht="90" customHeight="1">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>C40</t>
+          <t>C41</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>VeritaComp Competencies Owed derived from VeritaStaff, with gap detection (was #48)</t>
+          <t>VeritaCheck coverage recurrence (method comparison + cal-ver/linearity + reports)</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr"/>
@@ -1612,12 +1611,12 @@
       <c r="E19" s="3" t="inlineStr"/>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1314 (squash 2bcb0db9). GET /api/labs/:labId/competency/owed derives each VeritaStaff testing employee's owed competencies from their assigned instruments (staff_employee_instruments -&gt; veritamap_instruments + tests), on the CLIA timeline, and flags instruments not covered by any competency program as gaps. CompetenciesOwedSection renders it on the VeritaComp landing page. Reuses the shipped bridge + suggested-method-groups match rules; no new tables. Verified live on prod with real assignment data: 2 instruments assigned to a demo staffer produced owed=2, gaps=2 (HIGH, Technical Supervisor), then reverted cleanly. Closed 2026-09-24.</t>
+          <t>Closure evidence: PRs #1317 (method comparison), #1318 (cal-ver/linearity), #1321 (report Next-due columns). Periodic verification (correlation/method comparison 42 CFR 493.1281; cal-ver/linearity 42 CFR 493.1255; both 6-month) now recurs: a signed study banks the cycle and rolls to next-due = signed + 6 months instead of reading "done" forever. Status Missing/Failed/Completed-unsigned + a "Next due on" column on-screen and in both coverage exports; also credits the previously-ignored "correlation" study type. Root cause: computeCoverageFrom marked requirements done on mere existence, no date logic. Verified live on SCAHC lab 2 (101 correlations + 11 cal-ver rows now carry a next-due). Engine-level, all facilities. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>2026-09-23/24 session, Michael ("veritacomp bases what competencies they owe (currently untrue, but needs to be true)"). Option 1 (unify roster on VeritaStaff, match instruments by id).
+          <t>2026-09-24 session, Michael ("Look at San Carlos... they finished their last set of correlations (all 103) but their menu never reset").
 ---</t>
         </is>
       </c>
@@ -1626,12 +1625,12 @@
     <row r="20" ht="90" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>C39</t>
+          <t>C40</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>VeritaScan line items can attach or link evidence (was #46)</t>
+          <t>VeritaComp Competencies Owed derived from VeritaStaff, with gap detection (was #48)</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr"/>
@@ -1639,12 +1638,12 @@
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1312 (squash a1dda93d). VeritaScan scan checklist items now show linked evidence as chips (open link, remove) plus a writer "Link evidence" affordance whose picker links an existing VeritaDC/Library document; a shortcut deep-links to the Library for new (governed) documents. Reuses the already-shipped lab_documents + document_checklist_links + coverage endpoints (URL-pointer only, no file storage, no new tables). Browser-verified live on prod (scan 23): the affordance renders and the picker opens. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1314 (squash 2bcb0db9). GET /api/labs/:labId/competency/owed derives each VeritaStaff testing employee's owed competencies from their assigned instruments (staff_employee_instruments -&gt; veritamap_instruments + tests), on the CLIA timeline, and flags instruments not covered by any competency program as gaps. CompetenciesOwedSection renders it on the VeritaComp landing page. Reuses the shipped bridge + suggested-method-groups match rules; no new tables. Verified live on prod with real assignment data: 2 instruments assigned to a demo staffer produced owed=2, gaps=2 (HIGH, Technical Supervisor), then reverted cleanly. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23 session, Michael. Recurring request. Companion: cross-module evidence display on the VeritaDC policy shipped in PR #1313 (by-target cross-links surfaced in the policy View modal, browser-verified live).
+          <t>2026-09-23/24 session, Michael ("veritacomp bases what competencies they owe (currently untrue, but needs to be true)"). Option 1 (unify roster on VeritaStaff, match instruments by id).
 ---</t>
         </is>
       </c>
@@ -1653,12 +1652,12 @@
     <row r="21" ht="90" customHeight="1">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>C38</t>
+          <t>C39</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>VeritaTrack calendar month cells expand to reveal hidden tasks (was #45)</t>
+          <t>VeritaScan line items can attach or link evidence (was #46)</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr"/>
@@ -1666,12 +1665,12 @@
       <c r="E21" s="3" t="inlineStr"/>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: VeritaTrack CalendarView month cells with more than three tasks now expand in place (chevron, "+N more" toggling to "Show less", due dates), so no task is hidden with no path to it (client/src/pages/VeritaTrackAppPage.tsx CalendarView). Shipped 2026-09-23. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1312 (squash a1dda93d). VeritaScan scan checklist items now show linked evidence as chips (open link, remove) plus a writer "Link evidence" affordance whose picker links an existing VeritaDC/Library document; a shortcut deep-links to the Library for new (governed) documents. Reuses the already-shipped lab_documents + document_checklist_links + coverage endpoints (URL-pointer only, no file storage, no new tables). Browser-verified live on prod (scan 23): the affordance renders and the picker opens. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>2026-09-23 session, Michael screenshot of the VeritaTrack calendar (lab 3, September cell).
+          <t>2026-09-23 session, Michael. Recurring request. Companion: cross-module evidence display on the VeritaDC policy shipped in PR #1313 (by-target cross-links surfaced in the policy View modal, browser-verified live).
 ---</t>
         </is>
       </c>
@@ -1680,12 +1679,12 @@
     <row r="22" ht="90" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>C37</t>
+          <t>C38</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Long Excel column headers no longer clip CFR citations (was #44)</t>
+          <t>VeritaTrack calendar month cells expand to reveal hidden tasks (was #45)</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr"/>
@@ -1693,12 +1692,12 @@
       <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. The VeritaMap export derives the header row height from the longest wrapped header via headerRowHeight(headers, colWidths) (server/routes.ts:15935) instead of a fixed 20, so "Reference Range Attestation (42 CFR 493.1253)" and the other long headers print in full. No new code this session. Closed 2026-09-24.</t>
+          <t>Closure evidence: VeritaTrack CalendarView month cells with more than three tasks now expand in place (chevron, "+N more" toggling to "Show less", due dates), so no task is hidden with no path to it (client/src/pages/VeritaTrackAppPage.tsx CalendarView). Shipped 2026-09-23. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+          <t>2026-09-23 session, Michael screenshot of the VeritaTrack calendar (lab 3, September cell).
 ---</t>
         </is>
       </c>
@@ -1707,12 +1706,12 @@
     <row r="23" ht="90" customHeight="1">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>C36</t>
+          <t>C37</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>License stamp no longer clobbers the §6 header/footer or names the wrong lab (was #43)</t>
+          <t>Long Excel column headers no longer clip CFR citations (was #44)</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr"/>
@@ -1720,7 +1719,7 @@
       <c r="E23" s="3" t="inlineStr"/>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. setHeaderFooter (shared/licenseExceljs.ts:155-209) now preserves an existing §6 header and appends (not overwrites) the footer left section, and customer-facing exports name the scoped lab: the VeritaScan library export reads req.scope.lab.name / clia_number (server/routes.ts:16572-16573), not the licensee. No new code this session (avoided regressing the existing fix). Closed 2026-09-24.</t>
+          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. The VeritaMap export derives the header row height from the longest wrapped header via headerRowHeight(headers, colWidths) (server/routes.ts:15935) instead of a fixed 20, so "Reference Range Attestation (42 CFR 493.1253)" and the other long headers print in full. No new code this session. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -1734,18 +1733,45 @@
     <row r="24" ht="90" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>C34</t>
+          <t>C36</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Wire the two static-audit guards into CI (was #43)</t>
+          <t>License stamp no longer clobbers the §6 header/footer or names the wrong lab (was #43)</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr"/>
       <c r="D24" s="2" t="inlineStr"/>
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. setHeaderFooter (shared/licenseExceljs.ts:155-209) now preserves an existing §6 header and appends (not overwrites) the footer left section, and customer-facing exports name the scoped lab: the VeritaScan library export reads req.scope.lab.name / clia_number (server/routes.ts:16572-16573), not the licensee. No new code this session (avoided regressing the existing fix). Closed 2026-09-24.</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+---</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25" ht="90" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>C34</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Wire the two static-audit guards into CI (was #43)</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr"/>
+      <c r="D25" s="3" t="inlineStr"/>
+      <c r="E25" s="3" t="inlineStr"/>
+      <c r="F25" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: both guards wired into the Multi-Lab Mutations Audit CI
 workflow (.github/workflows/multilab-mutations-audit.yml) as steps:
@@ -1757,24 +1783,24 @@
 (same caveat as the existing guards already in that workflow).</t>
         </is>
       </c>
-      <c r="G24" s="2" t="inlineStr"/>
-      <c r="H24" s="2" t="inlineStr"/>
-    </row>
-    <row r="25" ht="90" customHeight="1">
-      <c r="A25" s="3" t="inlineStr">
+      <c r="G25" s="3" t="inlineStr"/>
+      <c r="H25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26" ht="90" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>C35</t>
         </is>
       </c>
-      <c r="B25" s="3" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t>Legacy /api/studies over-returns studies across labs (was #44)</t>
         </is>
       </c>
-      <c r="C25" s="3" t="inlineStr"/>
-      <c r="D25" s="3" t="inlineStr"/>
-      <c r="E25" s="3" t="inlineStr"/>
-      <c r="F25" s="3" t="inlineStr">
+      <c r="C26" s="2" t="inlineStr"/>
+      <c r="D26" s="2" t="inlineStr"/>
+      <c r="E26" s="2" t="inlineStr"/>
+      <c r="F26" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: GET /api/studies now scopes its list to the active lab
 when one is resolved from the Referer (server/routes.ts), so every returned row
@@ -1784,24 +1810,24 @@
 mirroring the /api/labs/:labId/studies handler. Closed 2026-06-14.</t>
         </is>
       </c>
-      <c r="G25" s="3" t="inlineStr"/>
-      <c r="H25" s="3" t="inlineStr"/>
-    </row>
-    <row r="26" ht="90" customHeight="1">
-      <c r="A26" s="2" t="inlineStr">
+      <c r="G26" s="2" t="inlineStr"/>
+      <c r="H26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27" ht="90" customHeight="1">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>C30</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="B27" s="3" t="inlineStr">
         <is>
           <t>Verify-script convention backfill (was #41)</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr"/>
-      <c r="D26" s="2" t="inlineStr"/>
-      <c r="E26" s="2" t="inlineStr"/>
-      <c r="F26" s="2" t="inlineStr">
+      <c r="C27" s="3" t="inlineStr"/>
+      <c r="D27" s="3" t="inlineStr"/>
+      <c r="E27" s="3" t="inlineStr"/>
+      <c r="F27" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: all 8 high-stakes math/logic commits now ship a paired
 scripts/verify-*.js (EP17 sensitivity, Deming lot-to-lot, CUMSUM+QC+multi-analyte,
@@ -1809,30 +1835,30 @@
 TEa boundary), per the strike-throughs in #41. Closed 2026-06-13.</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr">
+      <c r="G27" s="3" t="inlineStr">
         <is>
           <t>scripts/audit_verify_script_coverage.py lookback, 2026-06-02; backfills
 landed 2026-06-03..06.
 ---</t>
         </is>
       </c>
-      <c r="H26" s="2" t="inlineStr"/>
-    </row>
-    <row r="27" ht="90" customHeight="1">
-      <c r="A27" s="3" t="inlineStr">
+      <c r="H27" s="3" t="inlineStr"/>
+    </row>
+    <row r="28" ht="90" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>C31</t>
         </is>
       </c>
-      <c r="B27" s="3" t="inlineStr">
+      <c r="B28" s="2" t="inlineStr">
         <is>
           <t>VeritaPT AAA create/update/delete silently no-op in the multi-lab UI</t>
         </is>
       </c>
-      <c r="C27" s="3" t="inlineStr"/>
-      <c r="D27" s="3" t="inlineStr"/>
-      <c r="E27" s="3" t="inlineStr"/>
-      <c r="F27" s="3" t="inlineStr">
+      <c r="C28" s="2" t="inlineStr"/>
+      <c r="D28" s="2" t="inlineStr"/>
+      <c r="E28" s="2" t="inlineStr"/>
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #754 (commit 92ad499) added lab-scoped POST/PUT/DELETE
 /api/labs/:labId/pt/aa-records. The UI posted to the lab-scoped path but only GET
@@ -1843,30 +1869,30 @@
 route mis-filed records to the user's default lab on multi-lab accounts).</t>
         </is>
       </c>
-      <c r="G27" s="3" t="inlineStr">
+      <c r="G28" s="2" t="inlineStr">
         <is>
           <t>2026-06-13, found during #18 Phase 3 QA;
 scripts/audit-labscoped-write-routes.mjs now guards the class.
 ---</t>
         </is>
       </c>
-      <c r="H27" s="3" t="inlineStr"/>
-    </row>
-    <row r="28" ht="90" customHeight="1">
-      <c r="A28" s="2" t="inlineStr">
+      <c r="H28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29" ht="90" customHeight="1">
+      <c r="A29" s="3" t="inlineStr">
         <is>
           <t>C32</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="B29" s="3" t="inlineStr">
         <is>
           <t>VeritaComp "Unlock assessment" false-success no-op</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr"/>
-      <c r="D28" s="2" t="inlineStr"/>
-      <c r="E28" s="2" t="inlineStr"/>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="C29" s="3" t="inlineStr"/>
+      <c r="D29" s="3" t="inlineStr"/>
+      <c r="E29" s="3" t="inlineStr"/>
+      <c r="F29" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #755 (commit 4234007) moved the unlock route to
 /api/labs/:labId/competency/assessments/:id/unlock (the path the client calls).
@@ -1877,29 +1903,29 @@
 HTML).</t>
         </is>
       </c>
-      <c r="G28" s="2" t="inlineStr">
+      <c r="G29" s="3" t="inlineStr">
         <is>
           <t>2026-06-13, found by scripts/audit-labscoped-write-routes.mjs.
 ---</t>
         </is>
       </c>
-      <c r="H28" s="2" t="inlineStr"/>
-    </row>
-    <row r="29" ht="90" customHeight="1">
-      <c r="A29" s="3" t="inlineStr">
+      <c r="H29" s="3" t="inlineStr"/>
+    </row>
+    <row r="30" ht="90" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>C33</t>
         </is>
       </c>
-      <c r="B29" s="3" t="inlineStr">
+      <c r="B30" s="2" t="inlineStr">
         <is>
           <t>FK-cascade delete 500s + NavBar laptop-width overflow</t>
         </is>
       </c>
-      <c r="C29" s="3" t="inlineStr"/>
-      <c r="D29" s="3" t="inlineStr"/>
-      <c r="E29" s="3" t="inlineStr"/>
-      <c r="F29" s="3" t="inlineStr">
+      <c r="C30" s="2" t="inlineStr"/>
+      <c r="D30" s="2" t="inlineStr"/>
+      <c r="E30" s="2" t="inlineStr"/>
+      <c r="F30" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PRs #749/#750 fixed NavBar horizontal overflow at laptop
 widths (collapse to the hamburger below 1560px); prod-verified at 1280-1920 with the
@@ -1910,37 +1936,9 @@
 500 -&gt; 200. scripts/audit-delete-cascades.mjs guards the class.</t>
         </is>
       </c>
-      <c r="G29" s="3" t="inlineStr">
+      <c r="G30" s="2" t="inlineStr">
         <is>
           <t>2026-06-13 browser QA of the A7-D4 wave + retro-QC of the 72h PR window.
----</t>
-        </is>
-      </c>
-      <c r="H29" s="3" t="inlineStr"/>
-    </row>
-    <row r="30" ht="90" customHeight="1">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>C1</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>FAQ "over 25 years" -&gt; "over 23 years"</t>
-        </is>
-      </c>
-      <c r="C30" s="2" t="inlineStr"/>
-      <c r="D30" s="2" t="inlineStr"/>
-      <c r="E30" s="2" t="inlineStr"/>
-      <c r="F30" s="2" t="inlineStr">
-        <is>
-          <t>Closure evidence: client/src/pages/FAQPage.tsx line 20 reads "over
-23 years" as of 2026-05-01.</t>
-        </is>
-      </c>
-      <c r="G30" s="2" t="inlineStr">
-        <is>
-          <t>session 299e9a73 turn 14, ~2026-04-28.
 ---</t>
         </is>
       </c>
@@ -1949,18 +1947,46 @@
     <row r="31" ht="90" customHeight="1">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>C5</t>
+          <t>C1</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>David's VeritaQA grey-button bug (seat permissions mode)</t>
+          <t>FAQ "over 25 years" -&gt; "over 23 years"</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr"/>
       <c r="D31" s="3" t="inlineStr"/>
       <c r="E31" s="3" t="inlineStr"/>
       <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>Closure evidence: client/src/pages/FAQPage.tsx line 20 reads "over
+23 years" as of 2026-05-01.</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>session 299e9a73 turn 14, ~2026-04-28.
+---</t>
+        </is>
+      </c>
+      <c r="H31" s="3" t="inlineStr"/>
+    </row>
+    <row r="32" ht="90" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>David's VeritaQA grey-button bug (seat permissions mode)</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr"/>
+      <c r="D32" s="2" t="inlineStr"/>
+      <c r="E32" s="2" t="inlineStr"/>
+      <c r="F32" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #10 squash-merged as commit a43fbba on
 2026-05-01 23:19 MST. Railway deploy succeeded; deployed bundle
@@ -1973,7 +1999,7 @@
 against his exact stored shape (14 of 14 expected outcomes matched).</t>
         </is>
       </c>
-      <c r="G31" s="3" t="inlineStr">
+      <c r="G32" s="2" t="inlineStr">
         <is>
           <t>2026-05-01 David's report; veritabench + veritastock
 weren't in MODULE_LIST so seat permissions silently defaulted to
@@ -1981,46 +2007,17 @@
 ---</t>
         </is>
       </c>
-      <c r="H31" s="3" t="inlineStr"/>
-    </row>
-    <row r="32" ht="90" customHeight="1">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>C2</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>TeamPage present-tense "TJC surveyor" check</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr"/>
-      <c r="D32" s="2" t="inlineStr"/>
-      <c r="E32" s="2" t="inlineStr"/>
-      <c r="F32" s="2" t="inlineStr">
-        <is>
-          <t>Closure evidence: site-wide search confirmed all surveyor language
-is past-tense, consistent with user's 2021-2025 service. User closed
-the item in session 299e9a73 turn 4.</t>
-        </is>
-      </c>
-      <c r="G32" s="2" t="inlineStr">
-        <is>
-          <t>session 299e9a73, ~2026-04-28.
----</t>
-        </is>
-      </c>
       <c r="H32" s="2" t="inlineStr"/>
     </row>
     <row r="33" ht="90" customHeight="1">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>C3</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>My Studies CSV/XLSX export (John as design partner)</t>
+          <t>TeamPage present-tense "TJC surveyor" check</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr"/>
@@ -2028,14 +2025,14 @@
       <c r="E33" s="3" t="inlineStr"/>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: client/src/pages/DashboardPage.tsx line 46 calls
-/api/my-studies/export. server/routes.ts line 1491 implements the
-endpoint. Pulled forward into pre-COLA per user instruction.</t>
+          <t>Closure evidence: site-wide search confirmed all surveyor language
+is past-tense, consistent with user's 2021-2025 service. User closed
+the item in session 299e9a73 turn 4.</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>session 299e9a73 turn 5, ~2026-04-28.
+          <t>session 299e9a73, ~2026-04-28.
 ---</t>
         </is>
       </c>
@@ -2044,12 +2041,12 @@
     <row r="34" ht="90" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>C4</t>
+          <t>C3</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Rotate GitHub PAT (because old PAT was committed in SESSION_HANDOFF files)</t>
+          <t>My Studies CSV/XLSX export (John as design partner)</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr"/>
@@ -2057,13 +2054,14 @@
       <c r="E34" s="2" t="inlineStr"/>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: no ghp_* or github_pat_* patterns in current
-SESSION_HANDOFF.md or SESSION_HANDOFF-2.md as of 2026-05-01.</t>
+          <t>Closure evidence: client/src/pages/DashboardPage.tsx line 46 calls
+/api/my-studies/export. server/routes.ts line 1491 implements the
+endpoint. Pulled forward into pre-COLA per user instruction.</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>session 299e9a73, ~2026-04-28.
+          <t>session 299e9a73 turn 5, ~2026-04-28.
 ---</t>
         </is>
       </c>
@@ -2072,18 +2070,46 @@
     <row r="35" ht="90" customHeight="1">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>C6</t>
+          <t>C4</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>VeritaPolicy service-line filtering removed (formerly #4)</t>
+          <t>Rotate GitHub PAT (because old PAT was committed in SESSION_HANDOFF files)</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr"/>
       <c r="D35" s="3" t="inlineStr"/>
       <c r="E35" s="3" t="inlineStr"/>
       <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>Closure evidence: no ghp_* or github_pat_* patterns in current
+SESSION_HANDOFF.md or SESSION_HANDOFF-2.md as of 2026-05-01.</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>session 299e9a73, ~2026-04-28.
+---</t>
+        </is>
+      </c>
+      <c r="H35" s="3" t="inlineStr"/>
+    </row>
+    <row r="36" ht="90" customHeight="1">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>C6</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>VeritaPolicy service-line filtering removed (formerly #4)</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr"/>
+      <c r="D36" s="2" t="inlineStr"/>
+      <c r="E36" s="2" t="inlineStr"/>
+      <c r="F36" s="2" t="inlineStr">
         <is>
           <t>Closure rationale (operator decision 2026-05-10): Keep all
 VeritaPolicy rows. CFR-only references with no accreditor reference
@@ -2092,29 +2118,29 @@
 report misread the design intent.</t>
         </is>
       </c>
-      <c r="G35" s="3" t="inlineStr">
+      <c r="G36" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H35" s="3" t="inlineStr"/>
-    </row>
-    <row r="36" ht="90" customHeight="1">
-      <c r="A36" s="2" t="inlineStr">
+      <c r="H36" s="2" t="inlineStr"/>
+    </row>
+    <row r="37" ht="90" customHeight="1">
+      <c r="A37" s="3" t="inlineStr">
         <is>
           <t>C7</t>
         </is>
       </c>
-      <c r="B36" s="2" t="inlineStr">
+      <c r="B37" s="3" t="inlineStr">
         <is>
           <t>CLIA number format validation (formerly #13)</t>
         </is>
       </c>
-      <c r="C36" s="2" t="inlineStr"/>
-      <c r="D36" s="2" t="inlineStr"/>
-      <c r="E36" s="2" t="inlineStr"/>
-      <c r="F36" s="2" t="inlineStr">
+      <c r="C37" s="3" t="inlineStr"/>
+      <c r="D37" s="3" t="inlineStr"/>
+      <c r="E37" s="3" t="inlineStr"/>
+      <c r="F37" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: shared/validateClia.ts defines CLIA_REGEX =
 /^\d{2}D\d{7}$/ (line 24), validateClia() helper with whitespace
@@ -2125,30 +2151,30 @@
 shape exists and behaves as specified.</t>
         </is>
       </c>
-      <c r="G36" s="2" t="inlineStr">
+      <c r="G37" s="3" t="inlineStr">
         <is>
           <t>Agent verification 2026-05-10 via grep + file read.
 Operator confirmed shipped 2026-05-10.
 ---</t>
         </is>
       </c>
-      <c r="H36" s="2" t="inlineStr"/>
-    </row>
-    <row r="37" ht="90" customHeight="1">
-      <c r="A37" s="3" t="inlineStr">
+      <c r="H37" s="3" t="inlineStr"/>
+    </row>
+    <row r="38" ht="90" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
         <is>
           <t>C8</t>
         </is>
       </c>
-      <c r="B37" s="3" t="inlineStr">
+      <c r="B38" s="2" t="inlineStr">
         <is>
           <t>VeritaMap lab-wide menu toggle (formerly #19)</t>
         </is>
       </c>
-      <c r="C37" s="3" t="inlineStr"/>
-      <c r="D37" s="3" t="inlineStr"/>
-      <c r="E37" s="3" t="inlineStr"/>
-      <c r="F37" s="3" t="inlineStr">
+      <c r="C38" s="2" t="inlineStr"/>
+      <c r="D38" s="2" t="inlineStr"/>
+      <c r="E38" s="2" t="inlineStr"/>
+      <c r="F38" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: client/src/pages/VeritaMapLabwidePage.tsx
 exists and implements the labwide read-only union view. Route is
@@ -2158,59 +2184,59 @@
 parking lot plan (read-only union view, per-session toggle) shipped.</t>
         </is>
       </c>
-      <c r="G37" s="3" t="inlineStr">
+      <c r="G38" s="2" t="inlineStr">
         <is>
           <t>Agent verification 2026-05-10 via grep + file read.
 Operator confirmed shipped 2026-05-10.
 ---</t>
         </is>
       </c>
-      <c r="H37" s="3" t="inlineStr"/>
-    </row>
-    <row r="38" ht="90" customHeight="1">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>C9</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>Tier-1 smoke test checklist (formerly #6)</t>
-        </is>
-      </c>
-      <c r="C38" s="2" t="inlineStr"/>
-      <c r="D38" s="2" t="inlineStr"/>
-      <c r="E38" s="2" t="inlineStr"/>
-      <c r="F38" s="2" t="inlineStr">
-        <is>
-          <t>Closure evidence: docs/smoke-test-tier1.md documents the Tier-1
-smoke-test process and post-deploy verification steps. Shipped via
-PR #81 as part of the 2026-05-10 wave.</t>
-        </is>
-      </c>
-      <c r="G38" s="2" t="inlineStr">
-        <is>
-          <t>Operator instruction 2026-05-10 in this session.
----</t>
-        </is>
-      </c>
       <c r="H38" s="2" t="inlineStr"/>
     </row>
     <row r="39" ht="90" customHeight="1">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>C10</t>
+          <t>C9</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>Per-module gating (formerly #7)</t>
+          <t>Tier-1 smoke test checklist (formerly #6)</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr"/>
       <c r="D39" s="3" t="inlineStr"/>
       <c r="E39" s="3" t="inlineStr"/>
       <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>Closure evidence: docs/smoke-test-tier1.md documents the Tier-1
+smoke-test process and post-deploy verification steps. Shipped via
+PR #81 as part of the 2026-05-10 wave.</t>
+        </is>
+      </c>
+      <c r="G39" s="3" t="inlineStr">
+        <is>
+          <t>Operator instruction 2026-05-10 in this session.
+---</t>
+        </is>
+      </c>
+      <c r="H39" s="3" t="inlineStr"/>
+    </row>
+    <row r="40" ht="90" customHeight="1">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>C10</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Per-module gating (formerly #7)</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr"/>
+      <c r="D40" s="2" t="inlineStr"/>
+      <c r="E40" s="2" t="inlineStr"/>
+      <c r="F40" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: Client-side useIsReadOnly module keys wired
 on client/src/pages/VeritaPolicyAppPage.tsx and
@@ -2225,29 +2251,29 @@
 PR #76.</t>
         </is>
       </c>
-      <c r="G39" s="3" t="inlineStr">
+      <c r="G40" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H39" s="3" t="inlineStr"/>
-    </row>
-    <row r="40" ht="90" customHeight="1">
-      <c r="A40" s="2" t="inlineStr">
+      <c r="H40" s="2" t="inlineStr"/>
+    </row>
+    <row r="41" ht="90" customHeight="1">
+      <c r="A41" s="3" t="inlineStr">
         <is>
           <t>C11</t>
         </is>
       </c>
-      <c r="B40" s="2" t="inlineStr">
+      <c r="B41" s="3" t="inlineStr">
         <is>
           <t>VeritaStock shipped copy (formerly #8)</t>
         </is>
       </c>
-      <c r="C40" s="2" t="inlineStr"/>
-      <c r="D40" s="2" t="inlineStr"/>
-      <c r="E40" s="2" t="inlineStr"/>
-      <c r="F40" s="2" t="inlineStr">
+      <c r="C41" s="3" t="inlineStr"/>
+      <c r="D41" s="3" t="inlineStr"/>
+      <c r="E41" s="3" t="inlineStr"/>
+      <c r="F41" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: client/src/pages/ArticleInventoryManagementPage.tsx
 line 305 footer reads "platform that includes VeritaStock™" instead
@@ -2255,29 +2281,29 @@
 on /resources/laboratory-inventory-management. Shipped via PR #75.</t>
         </is>
       </c>
-      <c r="G40" s="2" t="inlineStr">
+      <c r="G41" s="3" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H40" s="2" t="inlineStr"/>
-    </row>
-    <row r="41" ht="90" customHeight="1">
-      <c r="A41" s="3" t="inlineStr">
+      <c r="H41" s="3" t="inlineStr"/>
+    </row>
+    <row r="42" ht="90" customHeight="1">
+      <c r="A42" s="2" t="inlineStr">
         <is>
           <t>C12</t>
         </is>
       </c>
-      <c r="B41" s="3" t="inlineStr">
+      <c r="B42" s="2" t="inlineStr">
         <is>
           <t>Admin report one-row-per-lab (formerly #14)</t>
         </is>
       </c>
-      <c r="C41" s="3" t="inlineStr"/>
-      <c r="D41" s="3" t="inlineStr"/>
-      <c r="E41" s="3" t="inlineStr"/>
-      <c r="F41" s="3" t="inlineStr">
+      <c r="C42" s="2" t="inlineStr"/>
+      <c r="D42" s="2" t="inlineStr"/>
+      <c r="E42" s="2" t="inlineStr"/>
+      <c r="F42" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: /api/admin/report rewritten in
 server/routes.ts (~line 595) to LEFT JOIN labs on
@@ -2292,33 +2318,6 @@
 prerequisite, not a code bug). Shipped via PR #85.</t>
         </is>
       </c>
-      <c r="G41" s="3" t="inlineStr">
-        <is>
-          <t>Operator instruction 2026-05-10 in this session.
----</t>
-        </is>
-      </c>
-      <c r="H41" s="3" t="inlineStr"/>
-    </row>
-    <row r="42" ht="90" customHeight="1">
-      <c r="A42" s="2" t="inlineStr">
-        <is>
-          <t>C14</t>
-        </is>
-      </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>UI relabel "CLIA TEa" -&gt; "Lab-Set Internal Goal" (formerly #1)</t>
-        </is>
-      </c>
-      <c r="C42" s="2" t="inlineStr"/>
-      <c r="D42" s="2" t="inlineStr"/>
-      <c r="E42" s="2" t="inlineStr"/>
-      <c r="F42" s="2" t="inlineStr">
-        <is>
-          <t>Closure evidence: Shipped across four PRs over 2026-05-10.</t>
-        </is>
-      </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
@@ -2330,18 +2329,45 @@
     <row r="43" ht="90" customHeight="1">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>C13</t>
+          <t>C14</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>WSLH PT vendor (formerly #15)</t>
+          <t>UI relabel "CLIA TEa" -&gt; "Lab-Set Internal Goal" (formerly #1)</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr"/>
       <c r="D43" s="3" t="inlineStr"/>
       <c r="E43" s="3" t="inlineStr"/>
       <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>Closure evidence: Shipped across four PRs over 2026-05-10.</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="inlineStr">
+        <is>
+          <t>Operator instruction 2026-05-10 in this session.
+---</t>
+        </is>
+      </c>
+      <c r="H43" s="3" t="inlineStr"/>
+    </row>
+    <row r="44" ht="90" customHeight="1">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>C13</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>WSLH PT vendor (formerly #15)</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr"/>
+      <c r="D44" s="2" t="inlineStr"/>
+      <c r="E44" s="2" t="inlineStr"/>
+      <c r="F44" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: Shipped 2026-05-10 via PR #79 (merge commit
 eeebc6e; merged after rebase to resolve a server/db.ts collision
@@ -2359,38 +2385,9 @@
 'WSLH' is the post-deploy success signal. Shipped via PR #79.</t>
         </is>
       </c>
-      <c r="G43" s="3" t="inlineStr">
+      <c r="G44" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
----</t>
-        </is>
-      </c>
-      <c r="H43" s="3" t="inlineStr"/>
-    </row>
-    <row r="44" ht="90" customHeight="1">
-      <c r="A44" s="2" t="inlineStr">
-        <is>
-          <t>C15</t>
-        </is>
-      </c>
-      <c r="B44" s="2" t="inlineStr">
-        <is>
-          <t>VeritaStock lot tracking + expiration + reorder alerts (formerly #21)</t>
-        </is>
-      </c>
-      <c r="C44" s="2" t="inlineStr"/>
-      <c r="D44" s="2" t="inlineStr"/>
-      <c r="E44" s="2" t="inlineStr"/>
-      <c r="F44" s="2" t="inlineStr">
-        <is>
-          <t>Closure evidence: VeritaStock™ shipped the bench-level inventory
-features the Perplexity competitor analysis identified as a gap:</t>
-        </is>
-      </c>
-      <c r="G44" s="2" t="inlineStr">
-        <is>
-          <t>Originally Perplexity competitor analysis 2026-05-10.
-Audit 2026-05-21 confirmed the feature set ships today.
 ---</t>
         </is>
       </c>
@@ -2399,12 +2396,12 @@
     <row r="45" ht="90" customHeight="1">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>C16</t>
+          <t>C15</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>PAL studies guided workflow (formerly #23)</t>
+          <t>VeritaStock lot tracking + expiration + reorder alerts (formerly #21)</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr"/>
@@ -2412,15 +2409,14 @@
       <c r="E45" s="3" t="inlineStr"/>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: VeritaCheck™ already ships the Precision /
-Accuracy / Linearity (PAL) study set under EP-protocol naming:</t>
+          <t>Closure evidence: VeritaStock™ shipped the bench-level inventory
+features the Perplexity competitor analysis identified as a gap:</t>
         </is>
       </c>
       <c r="G45" s="3" t="inlineStr">
         <is>
           <t>Originally Perplexity competitor analysis 2026-05-10.
-Audit 2026-05-21 confirmed the EP studies cover the PAL framing in
-full.
+Audit 2026-05-21 confirmed the feature set ships today.
 ---</t>
         </is>
       </c>
@@ -2429,12 +2425,12 @@
     <row r="46" ht="90" customHeight="1">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>C17</t>
+          <t>C16</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Source-grounded 21/29/45 CFR + 42 CFR 482-485 (formerly #26)</t>
+          <t>PAL studies guided workflow (formerly #23)</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr"/>
@@ -2442,35 +2438,65 @@
       <c r="E46" s="2" t="inlineStr"/>
       <c r="F46" s="2" t="inlineStr">
         <is>
+          <t>Closure evidence: VeritaCheck™ already ships the Precision /
+Accuracy / Linearity (PAL) study set under EP-protocol naming:</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>Originally Perplexity competitor analysis 2026-05-10.
+Audit 2026-05-21 confirmed the EP studies cover the PAL framing in
+full.
+---</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr"/>
+    </row>
+    <row r="47" ht="90" customHeight="1">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>C17</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>Source-grounded 21/29/45 CFR + 42 CFR 482-485 (formerly #26)</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr"/>
+      <c r="D47" s="3" t="inlineStr"/>
+      <c r="E47" s="3" t="inlineStr"/>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
           <t>Closure evidence: PR #301 (commit 8c27806, merged 2026-05-21)
 source-grounded the 74 remaining non-493 entries in
 server/cfrRequirements.ts against verbatim eCFR XML. Breakdown
 shipped:</t>
         </is>
       </c>
-      <c r="G46" s="2" t="inlineStr">
+      <c r="G47" s="3" t="inlineStr">
         <is>
           <t>PR #301; tasks #18 in the in-session task tracker.
 ---</t>
         </is>
       </c>
-      <c r="H46" s="2" t="inlineStr"/>
-    </row>
-    <row r="47" ht="90" customHeight="1">
-      <c r="A47" s="3" t="inlineStr">
+      <c r="H47" s="3" t="inlineStr"/>
+    </row>
+    <row r="48" ht="90" customHeight="1">
+      <c r="A48" s="2" t="inlineStr">
         <is>
           <t>C18</t>
         </is>
       </c>
-      <c r="B47" s="3" t="inlineStr">
+      <c r="B48" s="2" t="inlineStr">
         <is>
           <t>VeritaPolicy "Non CLIA" chapter rename (formerly #3)</t>
         </is>
       </c>
-      <c r="C47" s="3" t="inlineStr"/>
-      <c r="D47" s="3" t="inlineStr"/>
-      <c r="E47" s="3" t="inlineStr"/>
-      <c r="F47" s="3" t="inlineStr">
+      <c r="C48" s="2" t="inlineStr"/>
+      <c r="D48" s="2" t="inlineStr"/>
+      <c r="E48" s="2" t="inlineStr"/>
+      <c r="F48" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #300 (commit 34d7707, merged 2026-05-21)
 renamed all 44 user-facing chapter labels in
@@ -2481,7 +2507,7 @@
 page.</t>
         </is>
       </c>
-      <c r="G47" s="3" t="inlineStr">
+      <c r="G48" s="2" t="inlineStr">
         <is>
           <t>CAP customer screenshot of the /veritapolicy chapter
 headers, 2026-05-01 evening. PR #300; tasks #17 in the in-session
@@ -2489,23 +2515,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H47" s="3" t="inlineStr"/>
-    </row>
-    <row r="48" ht="90" customHeight="1">
-      <c r="A48" s="2" t="inlineStr">
+      <c r="H48" s="2" t="inlineStr"/>
+    </row>
+    <row r="49" ht="90" customHeight="1">
+      <c r="A49" s="3" t="inlineStr">
         <is>
           <t>C19</t>
         </is>
       </c>
-      <c r="B48" s="2" t="inlineStr">
+      <c r="B49" s="3" t="inlineStr">
         <is>
           <t>VeritaStock department-scope toggle (formerly #31)</t>
         </is>
       </c>
-      <c r="C48" s="2" t="inlineStr"/>
-      <c r="D48" s="2" t="inlineStr"/>
-      <c r="E48" s="2" t="inlineStr"/>
-      <c r="F48" s="2" t="inlineStr">
+      <c r="C49" s="3" t="inlineStr"/>
+      <c r="D49" s="3" t="inlineStr"/>
+      <c r="E49" s="3" t="inlineStr"/>
+      <c r="F49" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #319 (commit d01f5fe, merged 2026-05-22)
 shipped the persistent dept-scope toggle on VeritaStockPage. A new
@@ -2516,7 +2542,7 @@
 workspace without re-filtering.</t>
         </is>
       </c>
-      <c r="G48" s="2" t="inlineStr">
+      <c r="G49" s="3" t="inlineStr">
         <is>
           <t>John, San Carlos lab, 2026-05-21. Same conversation that
 drove the vendor dropdown (PR #304), FILTERED VIEW banner (PR #305),
@@ -2524,23 +2550,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H48" s="2" t="inlineStr"/>
-    </row>
-    <row r="49" ht="90" customHeight="1">
-      <c r="A49" s="3" t="inlineStr">
+      <c r="H49" s="3" t="inlineStr"/>
+    </row>
+    <row r="50" ht="90" customHeight="1">
+      <c r="A50" s="2" t="inlineStr">
         <is>
           <t>C20</t>
         </is>
       </c>
-      <c r="B49" s="3" t="inlineStr">
+      <c r="B50" s="2" t="inlineStr">
         <is>
           <t>Primary-lab seat counting (formerly #12)</t>
         </is>
       </c>
-      <c r="C49" s="3" t="inlineStr"/>
-      <c r="D49" s="3" t="inlineStr"/>
-      <c r="E49" s="3" t="inlineStr"/>
-      <c r="F49" s="3" t="inlineStr">
+      <c r="C50" s="2" t="inlineStr"/>
+      <c r="D50" s="2" t="inlineStr"/>
+      <c r="E50" s="2" t="inlineStr"/>
+      <c r="F50" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: is_primary_lab INTEGER NOT NULL DEFAULT 0
 column was added to the lab_members table at db.ts:1276, with the
@@ -2551,7 +2577,7 @@
 is_primary_lab=1 ordering).</t>
         </is>
       </c>
-      <c r="G49" s="3" t="inlineStr">
+      <c r="G50" s="2" t="inlineStr">
         <is>
           <t>2026-05-07 multi-lab discussion. Build shipped as part
 of the Multi-Lab Tier 2 architecture work (Phase 3.x series, prior
@@ -2560,23 +2586,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H49" s="3" t="inlineStr"/>
-    </row>
-    <row r="50" ht="90" customHeight="1">
-      <c r="A50" s="2" t="inlineStr">
+      <c r="H50" s="2" t="inlineStr"/>
+    </row>
+    <row r="51" ht="90" customHeight="1">
+      <c r="A51" s="3" t="inlineStr">
         <is>
           <t>C21</t>
         </is>
       </c>
-      <c r="B50" s="2" t="inlineStr">
+      <c r="B51" s="3" t="inlineStr">
         <is>
           <t>Multi-lab pricing model — Option A (formerly #11)</t>
         </is>
       </c>
-      <c r="C50" s="2" t="inlineStr"/>
-      <c r="D50" s="2" t="inlineStr"/>
-      <c r="E50" s="2" t="inlineStr"/>
-      <c r="F50" s="2" t="inlineStr">
+      <c r="C51" s="3" t="inlineStr"/>
+      <c r="D51" s="3" t="inlineStr"/>
+      <c r="E51" s="3" t="inlineStr"/>
+      <c r="F51" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #322 (commit 0ccd925, merged 2026-05-22)
 added the customer-facing line to the pricing page that reflects
@@ -2589,7 +2615,7 @@
 Enterprise+ block, reads:</t>
         </is>
       </c>
-      <c r="G50" s="2" t="inlineStr">
+      <c r="G51" s="3" t="inlineStr">
         <is>
           <t>2026-05-07 multi-lab discussion (Lisa Veri's
 canonical-case session). PR #322 (initial build); softening PR
@@ -2598,30 +2624,30 @@
 ---</t>
         </is>
       </c>
-      <c r="H50" s="2" t="inlineStr"/>
-    </row>
-    <row r="51" ht="90" customHeight="1">
-      <c r="A51" s="3" t="inlineStr">
+      <c r="H51" s="3" t="inlineStr"/>
+    </row>
+    <row r="52" ht="90" customHeight="1">
+      <c r="A52" s="2" t="inlineStr">
         <is>
           <t>C22</t>
         </is>
       </c>
-      <c r="B51" s="3" t="inlineStr">
+      <c r="B52" s="2" t="inlineStr">
         <is>
           <t>VeritaOps cost-per-test module (formerly #10)</t>
         </is>
       </c>
-      <c r="C51" s="3" t="inlineStr"/>
-      <c r="D51" s="3" t="inlineStr"/>
-      <c r="E51" s="3" t="inlineStr"/>
-      <c r="F51" s="3" t="inlineStr">
+      <c r="C52" s="2" t="inlineStr"/>
+      <c r="D52" s="2" t="inlineStr"/>
+      <c r="E52" s="2" t="inlineStr"/>
+      <c r="F52" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: v1 of the VeritaOps Cost-Per-Reportable-Test
 (CPRT) module shipped across PR #325 through PR #330 on 2026-05-22.
 The module is feature-complete for the typical lab director workflow.</t>
         </is>
       </c>
-      <c r="G51" s="3" t="inlineStr">
+      <c r="G52" s="2" t="inlineStr">
         <is>
           <t>This thread, 2026-05-07 12:05 PM CDT, user message:
 "Parking lot: build an operations module for cost per test
@@ -2630,262 +2656,262 @@
 ---</t>
         </is>
       </c>
-      <c r="H51" s="3" t="inlineStr"/>
-    </row>
-    <row r="52" ht="90" customHeight="1">
-      <c r="A52" s="2" t="inlineStr">
+      <c r="H52" s="2" t="inlineStr"/>
+    </row>
+    <row r="53" ht="90" customHeight="1">
+      <c r="A53" s="3" t="inlineStr">
         <is>
           <t>C23</t>
         </is>
       </c>
-      <c r="B52" s="2" t="inlineStr">
+      <c r="B53" s="3" t="inlineStr">
         <is>
           <t>CCL lab name visual disambiguation in lab switcher (formerly #34)</t>
         </is>
       </c>
-      <c r="C52" s="2" t="inlineStr"/>
-      <c r="D52" s="2" t="inlineStr">
+      <c r="C53" s="3" t="inlineStr"/>
+      <c r="D53" s="3" t="inlineStr">
         <is>
           <t>XS (under 1 day, actual)</t>
         </is>
       </c>
-      <c r="E52" s="2" t="inlineStr">
+      <c r="E53" s="3" t="inlineStr">
         <is>
           <t>Low — cosmetic; only mattered when Lisa or Michael picked the wrong lab from...</t>
         </is>
       </c>
-      <c r="F52" s="2" t="inlineStr">
+      <c r="F53" s="3" t="inlineStr">
         <is>
           <t>Effort: XS (under 1 day, actual)
 Importance: Low — cosmetic; only mattered when Lisa or Michael picked the wrong lab from the dropdown.</t>
         </is>
       </c>
-      <c r="G52" s="2" t="inlineStr">
+      <c r="G53" s="3" t="inlineStr">
         <is>
           <t>flagged 2026-05-23 immediately after provisioning Lisa's CCL lab; closed 2026-05-24.
 ---</t>
         </is>
       </c>
-      <c r="H52" s="2" t="inlineStr"/>
-    </row>
-    <row r="53" ht="90" customHeight="1">
-      <c r="A53" s="3" t="inlineStr">
+      <c r="H53" s="3" t="inlineStr"/>
+    </row>
+    <row r="54" ht="90" customHeight="1">
+      <c r="A54" s="2" t="inlineStr">
         <is>
           <t>C24</t>
         </is>
       </c>
-      <c r="B53" s="3" t="inlineStr">
+      <c r="B54" s="2" t="inlineStr">
         <is>
           <t>VC Unlimited Y1/Y2 price disclosure UX (formerly #35)</t>
         </is>
       </c>
-      <c r="C53" s="3" t="inlineStr"/>
-      <c r="D53" s="3" t="inlineStr">
+      <c r="C54" s="2" t="inlineStr"/>
+      <c r="D54" s="2" t="inlineStr">
         <is>
           <t>XS (under 1 day, actual)</t>
         </is>
       </c>
-      <c r="E53" s="3" t="inlineStr">
+      <c r="E54" s="2" t="inlineStr">
         <is>
           <t>Low when shipped (proactive, no customer complaint yet) — but high if a procu...</t>
         </is>
       </c>
-      <c r="F53" s="3" t="inlineStr">
+      <c r="F54" s="2" t="inlineStr">
         <is>
           <t>Effort: XS (under 1 day, actual)
 Importance: Low when shipped (proactive, no customer complaint yet) — but high if a procurement reviewer later disputes the $499 renewal as undisclosed.</t>
         </is>
       </c>
-      <c r="G53" s="3" t="inlineStr">
+      <c r="G54" s="2" t="inlineStr">
         <is>
           <t>Pricing rebuild 2026-05-23; closed 2026-05-24 proactively before any customer dispute.
 ---</t>
         </is>
       </c>
-      <c r="H53" s="3" t="inlineStr"/>
-    </row>
-    <row r="54" ht="90" customHeight="1">
-      <c r="A54" s="2" t="inlineStr">
+      <c r="H54" s="2" t="inlineStr"/>
+    </row>
+    <row r="55" ht="90" customHeight="1">
+      <c r="A55" s="3" t="inlineStr">
         <is>
           <t>C25</t>
         </is>
       </c>
-      <c r="B54" s="2" t="inlineStr">
+      <c r="B55" s="3" t="inlineStr">
         <is>
           <t>VeritaQC Phase 1 (Levey-Jennings + Westgard live engine) (formerly #20)</t>
         </is>
       </c>
-      <c r="C54" s="2" t="inlineStr"/>
-      <c r="D54" s="2" t="inlineStr">
+      <c r="C55" s="3" t="inlineStr"/>
+      <c r="D55" s="3" t="inlineStr">
         <is>
           <t>L (about 5 days end-to-end, actual: Phase 0 schema → Phase 1A evaluator → 1B...</t>
         </is>
       </c>
-      <c r="E54" s="2" t="inlineStr">
+      <c r="E55" s="3" t="inlineStr">
         <is>
           <t>High — largest single gap vs myLabCompliance.io per Perplexity competitor ana...</t>
         </is>
       </c>
-      <c r="F54" s="2" t="inlineStr">
+      <c r="F55" s="3" t="inlineStr">
         <is>
           <t>Effort: L (about 5 days end-to-end, actual: Phase 0 schema → Phase 1A evaluator → 1B entry UI → 1C daily review → 1D monthly PDF + attestation)
 Importance: High — largest single gap vs myLabCompliance.io per Perplexity competitor analysis; promotes VeritaAssure from documentation tool to lab operations platform.</t>
         </is>
       </c>
-      <c r="G54" s="2" t="inlineStr">
+      <c r="G55" s="3" t="inlineStr">
         <is>
           <t>Perplexity competitor analysis 2026-05-10. Scoping confirmed via the build_phase1_mockup.py iterations 2026-05-24. Shipped 2026-05-25.
 ---</t>
         </is>
       </c>
-      <c r="H54" s="2" t="inlineStr"/>
-    </row>
-    <row r="55" ht="90" customHeight="1">
-      <c r="A55" s="3" t="inlineStr">
+      <c r="H55" s="3" t="inlineStr"/>
+    </row>
+    <row r="56" ht="90" customHeight="1">
+      <c r="A56" s="2" t="inlineStr">
         <is>
           <t>C26</t>
         </is>
       </c>
-      <c r="B55" s="3" t="inlineStr">
+      <c r="B56" s="2" t="inlineStr">
         <is>
           <t>VeritaLab CMS-116 application support + state licensing registry (formerly #22)</t>
         </is>
       </c>
-      <c r="C55" s="3" t="inlineStr"/>
-      <c r="D55" s="3" t="inlineStr">
+      <c r="C56" s="2" t="inlineStr"/>
+      <c r="D56" s="2" t="inlineStr">
         <is>
           <t>M (1-2 weeks for v1, actual)</t>
         </is>
       </c>
-      <c r="E55" s="3" t="inlineStr">
+      <c r="E56" s="2" t="inlineStr">
         <is>
           <t>Medium — competitor parity (myLabCompliance.io) plus useful at lab startup an...</t>
         </is>
       </c>
-      <c r="F55" s="3" t="inlineStr">
+      <c r="F56" s="2" t="inlineStr">
         <is>
           <t>Effort: M (1-2 weeks for v1, actual)
 Importance: Medium — competitor parity (myLabCompliance.io) plus useful at lab startup and at certificate-type changes.</t>
         </is>
       </c>
-      <c r="G55" s="3" t="inlineStr">
+      <c r="G56" s="2" t="inlineStr">
         <is>
           <t>Perplexity competitor analysis (myLabCompliance.io), 2026-05-10. Reclassified as a VeritaLab extension 2026-05-25. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H55" s="3" t="inlineStr"/>
-    </row>
-    <row r="56" ht="90" customHeight="1">
-      <c r="A56" s="2" t="inlineStr">
+      <c r="H56" s="2" t="inlineStr"/>
+    </row>
+    <row r="57" ht="90" customHeight="1">
+      <c r="A57" s="3" t="inlineStr">
         <is>
           <t>C27</t>
         </is>
       </c>
-      <c r="B56" s="2" t="inlineStr">
+      <c r="B57" s="3" t="inlineStr">
         <is>
           <t>Active vs view-only seat split (formerly #33)</t>
         </is>
       </c>
-      <c r="C56" s="2" t="inlineStr"/>
-      <c r="D56" s="2" t="inlineStr">
+      <c r="C57" s="3" t="inlineStr"/>
+      <c r="D57" s="3" t="inlineStr">
         <is>
           <t>M (~1 week of engineering, actual: shipped in a single multi-PR session)</t>
         </is>
       </c>
-      <c r="E56" s="2" t="inlineStr">
+      <c r="E57" s="3" t="inlineStr">
         <is>
           <t>Medium — closed the gap between /pricing copy and product behavior; gives sal...</t>
         </is>
       </c>
-      <c r="F56" s="2" t="inlineStr">
+      <c r="F57" s="3" t="inlineStr">
         <is>
           <t>Effort: M (~1 week of engineering, actual: shipped in a single multi-PR session)
 Importance: Medium — closed the gap between /pricing copy and product behavior; gives sales a clean answer for "do you charge for our medical director?"</t>
         </is>
       </c>
-      <c r="G56" s="2" t="inlineStr">
+      <c r="G57" s="3" t="inlineStr">
         <is>
           <t>Pricing analysis doc Decision 3 (2026-05-21); MEDIUM scenario revised 2026-05-29 to retire the "unlimited view-only" claim. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H56" s="2" t="inlineStr"/>
-    </row>
-    <row r="57" ht="90" customHeight="1">
-      <c r="A57" s="3" t="inlineStr">
+      <c r="H57" s="3" t="inlineStr"/>
+    </row>
+    <row r="58" ht="90" customHeight="1">
+      <c r="A58" s="2" t="inlineStr">
         <is>
           <t>C28</t>
         </is>
       </c>
-      <c r="B57" s="3" t="inlineStr">
+      <c r="B58" s="2" t="inlineStr">
         <is>
           <t>"Why VeritaCheck" comparative one-pager (formerly #37)</t>
         </is>
       </c>
-      <c r="C57" s="3" t="inlineStr"/>
-      <c r="D57" s="3" t="inlineStr">
+      <c r="C58" s="2" t="inlineStr"/>
+      <c r="D58" s="2" t="inlineStr">
         <is>
           <t>S (one design pass + four claim paragraphs + PDF + matching marketing-site pa...</t>
         </is>
       </c>
-      <c r="E57" s="3" t="inlineStr">
+      <c r="E58" s="2" t="inlineStr">
         <is>
           <t>Medium — closed a positioning gap surfaced by six COLA conference attendees a...</t>
         </is>
       </c>
-      <c r="F57" s="3" t="inlineStr">
+      <c r="F58" s="2" t="inlineStr">
         <is>
           <t>Effort: S (one design pass + four claim paragraphs + PDF + matching marketing-site page, actual)
 Importance: Medium — closed a positioning gap surfaced by six COLA conference attendees attached to a legacy verification tool; converts product-quality advantage into a leave-behind Lisa can hand out.</t>
         </is>
       </c>
-      <c r="G57" s="3" t="inlineStr">
+      <c r="G58" s="2" t="inlineStr">
         <is>
           <t>2026-05-11 / 2026-05-12 conference notes review with Michael. Conference attendees (Whitehead, Odegard, Othman, Molinelli, Kyle, Allred) expressed interest in equivalent / superior product. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H57" s="3" t="inlineStr"/>
-    </row>
-    <row r="58" ht="90" customHeight="1">
-      <c r="A58" s="2" t="inlineStr">
+      <c r="H58" s="2" t="inlineStr"/>
+    </row>
+    <row r="59" ht="90" customHeight="1">
+      <c r="A59" s="3" t="inlineStr">
         <is>
           <t>C29</t>
         </is>
       </c>
-      <c r="B58" s="2" t="inlineStr">
+      <c r="B59" s="3" t="inlineStr">
         <is>
           <t>VeritaPolicy approval workflow — MediaLab functional mirror</t>
         </is>
       </c>
-      <c r="C58" s="2" t="inlineStr"/>
-      <c r="D58" s="2" t="inlineStr">
+      <c r="C59" s="3" t="inlineStr"/>
+      <c r="D59" s="3" t="inlineStr">
         <is>
           <t>XL (one focused session, 12 PRs landed)</t>
         </is>
       </c>
-      <c r="E58" s="2" t="inlineStr">
+      <c r="E59" s="3" t="inlineStr">
         <is>
           <t>High — replaces MediaLab Document Control ($752/$2,250 starting price, scalin...</t>
         </is>
       </c>
-      <c r="F58" s="2" t="inlineStr">
+      <c r="F59" s="3" t="inlineStr">
         <is>
           <t>Effort: XL (one focused session, 12 PRs landed)
 Importance: High — replaces MediaLab Document Control ($752/$2,250 starting price, scaling to $10K-$20K/yr at enterprise per Capterra public data) with an included VeritaPolicy feature; closes a real positioning gap and gives sales a direct comparator line.</t>
         </is>
       </c>
-      <c r="G58" s="2" t="inlineStr">
+      <c r="G59" s="3" t="inlineStr">
         <is>
           <t>Pricing strategy conversation 2026-05-29 (Michael: "I don't like bolt-ons; we should replicate this") → scoped 8 phases → shipped all 12 PRs in single session. Shipped 2026-05-29.
 ---</t>
         </is>
       </c>
-      <c r="H58" s="2" t="inlineStr"/>
+      <c r="H59" s="3" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H58"/>
+  <autoFilter ref="A1:H59"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
TASK: Parking lot - close #43 as C59 (keep finding-closure MD/designee/owner-only); regen xlsx PLAN:   1. Record the operator decision to keep VeritaResponse finding closure restricted to MD / designee / owner-override; move #43 from OPEN to CLOSED as C59.   2. Regenerate PARKING_LOT.xlsx (OPEN 12 -> 11; CLOSED 58 -> 59). Self-check:   - No code change: prod already enforces this (shipped #1443/#1444); this records the confirmation only.   - md + xlsx committed together per the sync rule.   - Gate 3 N/A (internal documentation).
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PARKING_LOT.xlsx
+++ b/PARKING_LOT.xlsx
@@ -12,8 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RETIRED" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$59</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$60</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RETIRED'!$A$1:$H$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1006,83 +1006,44 @@
     <row r="12" ht="90" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>44</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Confirm the finding-closure signer policy (non-MD admins now blocked)</t>
+          <t>Regenerate the 119-function access-inventory Excel with the corrected MD persona</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Open, awaiting operator confirmation. Reverting is a one-line change (re-add the owner/admin path in the findings/:id/signoff handler) if admins should retain finding closure.
+          <t>Open, low priority. Offered to Michael; skippable if the sweep was a one-off working artifact.
 ---</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>XS (a yes/no decision; ~15 min to loosen the gate if reversed).</t>
+          <t>XS (~15 min to re-run the sweep harness and re-deliver).</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Medium — changes who can close VeritaResponse findings in production; affects...</t>
+          <t>Low — the harness and the shipped fixes are correct; only the recorded Excel'...</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Item 5 Phase 2 tightened VeritaResponse finding closure from "any owner / admin / edit-seat" to "the designated medical director, a delegated designee holding finding-closure for the lab's complexity, or the account owner as a logged break-glass override." This is live on prod (#1443). It follows the agreed MD-or-designee model (QB=1), and the same gate now guards QC period-review co-sign. It has not been confirmed against real customer workflows: if any lab relies on non-MD admins closing findings, they now need a Letter of Delegation, or the gate must be loosened.</t>
+          <t>The full-inventory 4-login access sweep (VeritaAssure_Function_Inventory.xlsx) was first generated with the medical-director test persona mis-seeded as a seatless member, which over-flagged its column. The harness was then corrected to seat the MD as the active writer it actually is (scripts/qa-sweep/inventory-sweep.ts). The delivered Excel still shows the old md results; re-running reclassifies the md-artifact flags down to the real findings, which were already fixed in PR A (#1441). Only worth doing if the sheet gets filed or shared externally.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>this session, delegation feature build (2026-10-04). Flagged repeatedly in-session; awaiting explicit operator sign-off.</t>
+          <t>this session, QA sweep (2026-10-03 to 2026-10-04).</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr"/>
     </row>
-    <row r="13" ht="90" customHeight="1">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>44</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>Regenerate the 119-function access-inventory Excel with the corrected MD persona</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>Open, low priority. Offered to Michael; skippable if the sweep was a one-off working artifact.
----</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>XS (~15 min to re-run the sweep harness and re-deliver).</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>Low — the harness and the shipped fixes are correct; only the recorded Excel'...</t>
-        </is>
-      </c>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>The full-inventory 4-login access sweep (VeritaAssure_Function_Inventory.xlsx) was first generated with the medical-director test persona mis-seeded as a seatless member, which over-flagged its column. The harness was then corrected to seat the MD as the active writer it actually is (scripts/qa-sweep/inventory-sweep.ts). The delivered Excel still shows the old md results; re-running reclassifies the md-artifact flags down to the real findings, which were already fixed in PR A (#1441). Only worth doing if the sheet gets filed or shared externally.</t>
-        </is>
-      </c>
-      <c r="G13" s="3" t="inlineStr">
-        <is>
-          <t>this session, QA sweep (2026-10-03 to 2026-10-04).</t>
-        </is>
-      </c>
-      <c r="H13" s="3" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:H13"/>
+  <autoFilter ref="A1:H12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1093,7 +1054,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H59"/>
+  <dimension ref="A1:H60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1151,24 +1112,24 @@
     <row r="2" ht="90" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>C58</t>
+          <t>C59</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>VeritaDC per-document attestation tracker + "My Documents" rename (built as #45)</t>
+          <t>Confirm the finding-closure signer policy (was #43)</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr"/>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>was M / Importance: Medium-High</t>
+          <t>was XS / Importance: Medium</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Effort: was M / Importance: Medium-High</t>
+          <t>Effort: was XS / Importance: Medium</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
@@ -1177,24 +1138,24 @@
     <row r="3" ht="90" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>C57</t>
+          <t>C58</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Hide sections a lab does not use from a master list (was #47)</t>
+          <t>VeritaDC per-document attestation tracker + "My Documents" rename (built as #45)</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr"/>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>was S-M / Importance: Medium-High (prospect-requested)</t>
+          <t>was M / Importance: Medium-High</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Effort: was S-M / Importance: Medium-High (prospect-requested)</t>
+          <t>Effort: was M / Importance: Medium-High</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr"/>
@@ -1203,24 +1164,24 @@
     <row r="4" ht="90" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>C56</t>
+          <t>C57</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>VeritaCEU: curated free continuing-education provider list (was #53)</t>
+          <t>Hide sections a lab does not use from a master list (was #47)</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr"/>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>was S / Importance: Low-Medium</t>
+          <t>was S-M / Importance: Medium-High (prospect-requested)</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Effort: was S / Importance: Low-Medium</t>
+          <t>Effort: was S-M / Importance: Medium-High (prospect-requested)</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr"/>
@@ -1229,24 +1190,24 @@
     <row r="5" ht="90" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>C55</t>
+          <t>C56</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>VeritaScan: let sites add their own custom questions (was #55)</t>
+          <t>VeritaCEU: curated free continuing-education provider list (was #53)</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr"/>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>was M / Importance: Medium-High</t>
+          <t>was S / Importance: Low-Medium</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Effort: was M / Importance: Medium-High</t>
+          <t>Effort: was S / Importance: Low-Medium</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr"/>
@@ -1255,24 +1216,24 @@
     <row r="6" ht="90" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>C54</t>
+          <t>C55</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>VeritaQC: at-entry warning when a QC point is outside 2 SD (was #56)</t>
+          <t>VeritaScan: let sites add their own custom questions (was #55)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr"/>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>was S-M (shipped S) / Importance: High</t>
+          <t>was M / Importance: Medium-High</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Effort: was S-M (shipped S) / Importance: High</t>
+          <t>Effort: was M / Importance: Medium-High</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
@@ -1281,24 +1242,24 @@
     <row r="7" ht="90" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>C53</t>
+          <t>C54</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>VeritaTrack: quarterly task loaded as monthly until re-saved (was #54)</t>
+          <t>VeritaQC: at-entry warning when a QC point is outside 2 SD (was #56)</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr"/>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>was S / Importance: Medium</t>
+          <t>was S-M (shipped S) / Importance: High</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Effort: was S / Importance: Medium</t>
+          <t>Effort: was S-M (shipped S) / Importance: High</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr"/>
@@ -1307,24 +1268,24 @@
     <row r="8" ht="90" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>C52</t>
+          <t>C53</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>VeritaResponse internal NCE / non-conforming event (was #36)</t>
+          <t>VeritaTrack: quarterly task loaded as monthly until re-saved (was #54)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr"/>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>was L (shipped as MEDIUM) / Importance: High</t>
+          <t>was S / Importance: Medium</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Effort: was L (shipped as MEDIUM) / Importance: High</t>
+          <t>Effort: was S / Importance: Medium</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
@@ -1333,24 +1294,24 @@
     <row r="9" ht="90" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>C49</t>
+          <t>C52</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Competency "assessed this cycle" cadence-aware window (was #50)</t>
+          <t>VeritaResponse internal NCE / non-conforming event (was #36)</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr"/>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>was S-M / Importance: Medium</t>
+          <t>was L (shipped as MEDIUM) / Importance: High</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Effort: was S-M / Importance: Medium</t>
+          <t>Effort: was L (shipped as MEDIUM) / Importance: High</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr"/>
@@ -1359,12 +1320,12 @@
     <row r="10" ht="90" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>C50</t>
+          <t>C49</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>VeritaTrack task owner + owner-only reminder routing (was #51)</t>
+          <t>Competency "assessed this cycle" cadence-aware window (was #50)</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr"/>
@@ -1385,24 +1346,24 @@
     <row r="11" ht="90" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>C51</t>
+          <t>C50</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Designate Medical Director by picking a lab member (was #52, core)</t>
+          <t>VeritaTrack task owner + owner-only reminder routing (was #51)</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr"/>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>was S-M / Importance: Medium-High</t>
+          <t>was S-M / Importance: Medium</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Effort: was S-M / Importance: Medium-High</t>
+          <t>Effort: was S-M / Importance: Medium</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr"/>
@@ -1411,24 +1372,24 @@
     <row r="12" ht="90" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>C47</t>
+          <t>C51</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Unregulated-analyte / Alternative Assessment (AAA) coverage (was #18)</t>
+          <t>Designate Medical Director by picking a lab member (was #52, core)</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr"/>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>was S (Phase 3) / Importance: Medium</t>
+          <t>was S-M / Importance: Medium-High</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Effort: was S (Phase 3) / Importance: Medium</t>
+          <t>Effort: was S-M / Importance: Medium-High</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr"/>
@@ -1437,24 +1398,24 @@
     <row r="13" ht="90" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>C48</t>
+          <t>C47</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>VeritaResponse post-survey deficiency module (was #17)</t>
+          <t>Unregulated-analyte / Alternative Assessment (AAA) coverage (was #18)</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr"/>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>was XL / Importance: High</t>
+          <t>was S (Phase 3) / Importance: Medium</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Effort: was XL / Importance: High</t>
+          <t>Effort: was S (Phase 3) / Importance: Medium</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr"/>
@@ -1463,39 +1424,38 @@
     <row r="14" ht="90" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>C45</t>
+          <t>C48</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Unify coverage/competency recurrence helper (was #49) - closed as non-issue</t>
+          <t>VeritaResponse post-survey deficiency module (was #17)</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr"/>
-      <c r="D14" s="2" t="inlineStr"/>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>was XL / Importance: High</t>
+        </is>
+      </c>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: Investigated 2026-09-24 before building. The coverage recurrence math (+6-month interval, signed-resets-to-missing, nextDueOn/overdue, isFailVerdict) is ALREADY single-source in server/veritacheckCoverage.ts (computeCoverageFrom). server/coverageReport.ts and the routes.ts coverage export do not recompute it; they consume the computed nextDueOn/overdue/status fields and apply small surface-specific presentation labels (deliberately different vocabularies per surface, so they should not be merged). The only truly identical duplicate is a one-line date formatter. The competency "owed" derivation is NOT the same cadence: competency follows the CLIA milestone schedule (initial / semiannual year 1 / annual, 42 CFR 493.1451(b)(8) and 493.1235), which is a different regulatory interval from the coverage 6-month rule (493.1281 / 493.1255) and must stay separate. No worthwhile extraction; merging the two cadences would be wrong. Closed 2026-09-24. (The year-1 competency-window refinement remains tracked separately as #50.)</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-24 session, "keep working" pass; scoped read-only, found no real duplication.
----</t>
-        </is>
-      </c>
+          <t>Effort: was XL / Importance: High</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr"/>
       <c r="H14" s="2" t="inlineStr"/>
     </row>
     <row r="15" ht="90" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>C46</t>
+          <t>C45</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Verified-users product-update send path (wrong-list incident fix)</t>
+          <t>Unify coverage/competency recurrence helper (was #49) - closed as non-issue</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr"/>
@@ -1503,12 +1463,12 @@
       <c r="E15" s="3" t="inlineStr"/>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: Shipped PR #1324 (merged 4e05506a, deploy ACTIVE). New POST /api/admin/users/send targets registered VeritaAssure account holders (the users table), never the Lab Director's Briefing subscriber list. Separate explicitly-named endpoint (not a flag with a dangerous default), account-holder email framing, excludes suppressed emails and RFC-reserved test domains, CC owner, dryRun + testTo previews. Public unsubscribe now upserts a suppression row so opt-outs are honored across both audiences. Live dryRun: 49 verified-user recipients vs 673 on the Briefing list. Receipts: scripts/verify-product-update-send.mts 24/24, tsc clean, rendered sample inspected. Fixes the fallout from the 2026-09-23/24 wrong-list send (a product update went to the 675-person Briefing list). Nothing sends without Michael's explicit "send it."</t>
+          <t>Closure evidence: Investigated 2026-09-24 before building. The coverage recurrence math (+6-month interval, signed-resets-to-missing, nextDueOn/overdue, isFailVerdict) is ALREADY single-source in server/veritacheckCoverage.ts (computeCoverageFrom). server/coverageReport.ts and the routes.ts coverage export do not recompute it; they consume the computed nextDueOn/overdue/status fields and apply small surface-specific presentation labels (deliberately different vocabularies per surface, so they should not be merged). The only truly identical duplicate is a one-line date formatter. The competency "owed" derivation is NOT the same cadence: competency follows the CLIA milestone schedule (initial / semiannual year 1 / annual, 42 CFR 493.1451(b)(8) and 493.1235), which is a different regulatory interval from the coverage 6-month rule (493.1281 / 493.1255) and must stay separate. No worthwhile extraction; merging the two cadences would be wrong. Closed 2026-09-24. (The year-1 competency-window refinement remains tracked separately as #50.)</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>2026-09-24 session; Michael selected this as the next build after the #41 close.
+          <t>2026-09-24 session, "keep working" pass; scoped read-only, found no real duplication.
 ---</t>
         </is>
       </c>
@@ -1517,12 +1477,12 @@
     <row r="16" ht="90" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>C44</t>
+          <t>C46</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Verify-script convention backfill (was #41) + audit matcher fix</t>
+          <t>Verified-users product-update send path (wrong-list incident fix)</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr"/>
@@ -1530,12 +1490,12 @@
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: #41 was fully backfilled on 2026-06-13 (all 8 high-stakes scripts landed; see C30); it had only been mis-filed in OPEN. A 2026-09-24 re-audit initially reported 4 of 5 recent math/logic commits as missing a verify script, which was a FALSE POSITIVE: scripts/audit_verify_script_coverage.py matched only scripts/verify-*.js / .cjs, so it ignored the .mjs / .mts / .ts verify scripts the repo now ships (e.g. verify-ptcoag-multi.mts, verify-tea-criterion-format.mjs). Fixed the matcher to accept .js/.cjs/.mjs/.ts/.mts; re-run shows 5 of 5 covered, 0 debt. The convention is being followed. Closed 2026-09-24.</t>
+          <t>Closure evidence: Shipped PR #1324 (merged 4e05506a, deploy ACTIVE). New POST /api/admin/users/send targets registered VeritaAssure account holders (the users table), never the Lab Director's Briefing subscriber list. Separate explicitly-named endpoint (not a flag with a dangerous default), account-holder email framing, excludes suppressed emails and RFC-reserved test domains, CC owner, dryRun + testTo previews. Public unsubscribe now upserts a suppression row so opt-outs are honored across both audiences. Live dryRun: 49 verified-user recipients vs 673 on the Briefing list. Receipts: scripts/verify-product-update-send.mts 24/24, tsc clean, rendered sample inspected. Fixes the fallout from the 2026-09-23/24 wrong-list send (a product update went to the 675-person Briefing list). Nothing sends without Michael's explicit "send it."</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 session, "keep working" pass; audit tooling bug found + fixed.
+          <t>2026-09-24 session; Michael selected this as the next build after the #41 close.
 ---</t>
         </is>
       </c>
@@ -1544,12 +1504,12 @@
     <row r="17" ht="90" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>C43</t>
+          <t>C44</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>VeritaStaff instrument-centric (dual) assignment view</t>
+          <t>Verify-script convention backfill (was #41) + audit matcher fix</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr"/>
@@ -1557,12 +1517,12 @@
       <c r="E17" s="3" t="inlineStr"/>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1320. GET/PUT /staff/instruments/:id/employees (transpose of the per-employee endpoints); an "Assign by Instrument" dialog lets a director pick a test system or manual test and check off who runs it. Same staff_employee_instruments join, with the 42 CFR 493.1235(a) duty-change event emitted on newly-added pairs so both orientations trigger the same reassessment. GET verified live on SCAHC lab 2. Closed 2026-09-24.</t>
+          <t>Closure evidence: #41 was fully backfilled on 2026-06-13 (all 8 high-stakes scripts landed; see C30); it had only been mis-filed in OPEN. A 2026-09-24 re-audit initially reported 4 of 5 recent math/logic commits as missing a verify script, which was a FALSE POSITIVE: scripts/audit_verify_script_coverage.py matched only scripts/verify-*.js / .cjs, so it ignored the .mjs / .mts / .ts verify scripts the repo now ships (e.g. verify-ptcoag-multi.mts, verify-tea-criterion-format.mjs). Fixed the matcher to accept .js/.cjs/.mjs/.ts/.mts; re-run shows 5 of 5 covered, 0 debt. The convention is being followed. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>2026-09-24 session, Michael ("in staff we should also give the dual view when assigning coverage to test systems or manual tests").
+          <t>2026-09-24 session, "keep working" pass; audit tooling bug found + fixed.
 ---</t>
         </is>
       </c>
@@ -1571,12 +1531,12 @@
     <row r="18" ht="90" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>C42</t>
+          <t>C43</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>VeritaComp coverage map (required-vs-assessed matrix, dual view)</t>
+          <t>VeritaStaff instrument-centric (dual) assignment view</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr"/>
@@ -1584,12 +1544,12 @@
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1319 (+ status layer PR #1316). /competency/owed returns per-item assessed (locked passing assessment this cycle on a covering method group) + per-employee CLIA status; CompetencyCoverageMap renders a By-employee / By-instrument matrix (Assessed / Owed / Overdue / Gap). Verified live on SCAHC lab 2 (owed 116, assessed 2, gaps 0). Completes #48 as the VeritaCheck-parity coverage map. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1320. GET/PUT /staff/instruments/:id/employees (transpose of the per-employee endpoints); an "Assign by Instrument" dialog lets a director pick a test system or manual test and check off who runs it. Same staff_employee_instruments join, with the 42 CFR 493.1235(a) duty-change event emitted on newly-added pairs so both orientations trigger the same reassessment. GET verified live on SCAHC lab 2. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 session, Michael ("are we building the competencies to have a coverage map, same as veritacheck?" then "build it").
+          <t>2026-09-24 session, Michael ("in staff we should also give the dual view when assigning coverage to test systems or manual tests").
 ---</t>
         </is>
       </c>
@@ -1598,12 +1558,12 @@
     <row r="19" ht="90" customHeight="1">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>C41</t>
+          <t>C42</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>VeritaCheck coverage recurrence (method comparison + cal-ver/linearity + reports)</t>
+          <t>VeritaComp coverage map (required-vs-assessed matrix, dual view)</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr"/>
@@ -1611,12 +1571,12 @@
       <c r="E19" s="3" t="inlineStr"/>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: PRs #1317 (method comparison), #1318 (cal-ver/linearity), #1321 (report Next-due columns). Periodic verification (correlation/method comparison 42 CFR 493.1281; cal-ver/linearity 42 CFR 493.1255; both 6-month) now recurs: a signed study banks the cycle and rolls to next-due = signed + 6 months instead of reading "done" forever. Status Missing/Failed/Completed-unsigned + a "Next due on" column on-screen and in both coverage exports; also credits the previously-ignored "correlation" study type. Root cause: computeCoverageFrom marked requirements done on mere existence, no date logic. Verified live on SCAHC lab 2 (101 correlations + 11 cal-ver rows now carry a next-due). Engine-level, all facilities. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1319 (+ status layer PR #1316). /competency/owed returns per-item assessed (locked passing assessment this cycle on a covering method group) + per-employee CLIA status; CompetencyCoverageMap renders a By-employee / By-instrument matrix (Assessed / Owed / Overdue / Gap). Verified live on SCAHC lab 2 (owed 116, assessed 2, gaps 0). Completes #48 as the VeritaCheck-parity coverage map. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>2026-09-24 session, Michael ("Look at San Carlos... they finished their last set of correlations (all 103) but their menu never reset").
+          <t>2026-09-24 session, Michael ("are we building the competencies to have a coverage map, same as veritacheck?" then "build it").
 ---</t>
         </is>
       </c>
@@ -1625,12 +1585,12 @@
     <row r="20" ht="90" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>C40</t>
+          <t>C41</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>VeritaComp Competencies Owed derived from VeritaStaff, with gap detection (was #48)</t>
+          <t>VeritaCheck coverage recurrence (method comparison + cal-ver/linearity + reports)</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr"/>
@@ -1638,12 +1598,12 @@
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1314 (squash 2bcb0db9). GET /api/labs/:labId/competency/owed derives each VeritaStaff testing employee's owed competencies from their assigned instruments (staff_employee_instruments -&gt; veritamap_instruments + tests), on the CLIA timeline, and flags instruments not covered by any competency program as gaps. CompetenciesOwedSection renders it on the VeritaComp landing page. Reuses the shipped bridge + suggested-method-groups match rules; no new tables. Verified live on prod with real assignment data: 2 instruments assigned to a demo staffer produced owed=2, gaps=2 (HIGH, Technical Supervisor), then reverted cleanly. Closed 2026-09-24.</t>
+          <t>Closure evidence: PRs #1317 (method comparison), #1318 (cal-ver/linearity), #1321 (report Next-due columns). Periodic verification (correlation/method comparison 42 CFR 493.1281; cal-ver/linearity 42 CFR 493.1255; both 6-month) now recurs: a signed study banks the cycle and rolls to next-due = signed + 6 months instead of reading "done" forever. Status Missing/Failed/Completed-unsigned + a "Next due on" column on-screen and in both coverage exports; also credits the previously-ignored "correlation" study type. Root cause: computeCoverageFrom marked requirements done on mere existence, no date logic. Verified live on SCAHC lab 2 (101 correlations + 11 cal-ver rows now carry a next-due). Engine-level, all facilities. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23/24 session, Michael ("veritacomp bases what competencies they owe (currently untrue, but needs to be true)"). Option 1 (unify roster on VeritaStaff, match instruments by id).
+          <t>2026-09-24 session, Michael ("Look at San Carlos... they finished their last set of correlations (all 103) but their menu never reset").
 ---</t>
         </is>
       </c>
@@ -1652,12 +1612,12 @@
     <row r="21" ht="90" customHeight="1">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>C39</t>
+          <t>C40</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>VeritaScan line items can attach or link evidence (was #46)</t>
+          <t>VeritaComp Competencies Owed derived from VeritaStaff, with gap detection (was #48)</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr"/>
@@ -1665,12 +1625,12 @@
       <c r="E21" s="3" t="inlineStr"/>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1312 (squash a1dda93d). VeritaScan scan checklist items now show linked evidence as chips (open link, remove) plus a writer "Link evidence" affordance whose picker links an existing VeritaDC/Library document; a shortcut deep-links to the Library for new (governed) documents. Reuses the already-shipped lab_documents + document_checklist_links + coverage endpoints (URL-pointer only, no file storage, no new tables). Browser-verified live on prod (scan 23): the affordance renders and the picker opens. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1314 (squash 2bcb0db9). GET /api/labs/:labId/competency/owed derives each VeritaStaff testing employee's owed competencies from their assigned instruments (staff_employee_instruments -&gt; veritamap_instruments + tests), on the CLIA timeline, and flags instruments not covered by any competency program as gaps. CompetenciesOwedSection renders it on the VeritaComp landing page. Reuses the shipped bridge + suggested-method-groups match rules; no new tables. Verified live on prod with real assignment data: 2 instruments assigned to a demo staffer produced owed=2, gaps=2 (HIGH, Technical Supervisor), then reverted cleanly. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>2026-09-23 session, Michael. Recurring request. Companion: cross-module evidence display on the VeritaDC policy shipped in PR #1313 (by-target cross-links surfaced in the policy View modal, browser-verified live).
+          <t>2026-09-23/24 session, Michael ("veritacomp bases what competencies they owe (currently untrue, but needs to be true)"). Option 1 (unify roster on VeritaStaff, match instruments by id).
 ---</t>
         </is>
       </c>
@@ -1679,12 +1639,12 @@
     <row r="22" ht="90" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>C38</t>
+          <t>C39</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>VeritaTrack calendar month cells expand to reveal hidden tasks (was #45)</t>
+          <t>VeritaScan line items can attach or link evidence (was #46)</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr"/>
@@ -1692,12 +1652,12 @@
       <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: VeritaTrack CalendarView month cells with more than three tasks now expand in place (chevron, "+N more" toggling to "Show less", due dates), so no task is hidden with no path to it (client/src/pages/VeritaTrackAppPage.tsx CalendarView). Shipped 2026-09-23. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1312 (squash a1dda93d). VeritaScan scan checklist items now show linked evidence as chips (open link, remove) plus a writer "Link evidence" affordance whose picker links an existing VeritaDC/Library document; a shortcut deep-links to the Library for new (governed) documents. Reuses the already-shipped lab_documents + document_checklist_links + coverage endpoints (URL-pointer only, no file storage, no new tables). Browser-verified live on prod (scan 23): the affordance renders and the picker opens. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23 session, Michael screenshot of the VeritaTrack calendar (lab 3, September cell).
+          <t>2026-09-23 session, Michael. Recurring request. Companion: cross-module evidence display on the VeritaDC policy shipped in PR #1313 (by-target cross-links surfaced in the policy View modal, browser-verified live).
 ---</t>
         </is>
       </c>
@@ -1706,12 +1666,12 @@
     <row r="23" ht="90" customHeight="1">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>C37</t>
+          <t>C38</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Long Excel column headers no longer clip CFR citations (was #44)</t>
+          <t>VeritaTrack calendar month cells expand to reveal hidden tasks (was #45)</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr"/>
@@ -1719,12 +1679,12 @@
       <c r="E23" s="3" t="inlineStr"/>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. The VeritaMap export derives the header row height from the longest wrapped header via headerRowHeight(headers, colWidths) (server/routes.ts:15935) instead of a fixed 20, so "Reference Range Attestation (42 CFR 493.1253)" and the other long headers print in full. No new code this session. Closed 2026-09-24.</t>
+          <t>Closure evidence: VeritaTrack CalendarView month cells with more than three tasks now expand in place (chevron, "+N more" toggling to "Show less", due dates), so no task is hidden with no path to it (client/src/pages/VeritaTrackAppPage.tsx CalendarView). Shipped 2026-09-23. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+          <t>2026-09-23 session, Michael screenshot of the VeritaTrack calendar (lab 3, September cell).
 ---</t>
         </is>
       </c>
@@ -1733,12 +1693,12 @@
     <row r="24" ht="90" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>C36</t>
+          <t>C37</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>License stamp no longer clobbers the §6 header/footer or names the wrong lab (was #43)</t>
+          <t>Long Excel column headers no longer clip CFR citations (was #44)</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr"/>
@@ -1746,7 +1706,7 @@
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. setHeaderFooter (shared/licenseExceljs.ts:155-209) now preserves an existing §6 header and appends (not overwrites) the footer left section, and customer-facing exports name the scoped lab: the VeritaScan library export reads req.scope.lab.name / clia_number (server/routes.ts:16572-16573), not the licensee. No new code this session (avoided regressing the existing fix). Closed 2026-09-24.</t>
+          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. The VeritaMap export derives the header row height from the longest wrapped header via headerRowHeight(headers, colWidths) (server/routes.ts:15935) instead of a fixed 20, so "Reference Range Attestation (42 CFR 493.1253)" and the other long headers print in full. No new code this session. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -1760,18 +1720,45 @@
     <row r="25" ht="90" customHeight="1">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>C34</t>
+          <t>C36</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>Wire the two static-audit guards into CI (was #43)</t>
+          <t>License stamp no longer clobbers the §6 header/footer or names the wrong lab (was #43)</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr"/>
       <c r="D25" s="3" t="inlineStr"/>
       <c r="E25" s="3" t="inlineStr"/>
       <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. setHeaderFooter (shared/licenseExceljs.ts:155-209) now preserves an existing §6 header and appends (not overwrites) the footer left section, and customer-facing exports name the scoped lab: the VeritaScan library export reads req.scope.lab.name / clia_number (server/routes.ts:16572-16573), not the licensee. No new code this session (avoided regressing the existing fix). Closed 2026-09-24.</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+---</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26" ht="90" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>C34</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Wire the two static-audit guards into CI (was #43)</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr"/>
+      <c r="D26" s="2" t="inlineStr"/>
+      <c r="E26" s="2" t="inlineStr"/>
+      <c r="F26" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: both guards wired into the Multi-Lab Mutations Audit CI
 workflow (.github/workflows/multilab-mutations-audit.yml) as steps:
@@ -1783,24 +1770,24 @@
 (same caveat as the existing guards already in that workflow).</t>
         </is>
       </c>
-      <c r="G25" s="3" t="inlineStr"/>
-      <c r="H25" s="3" t="inlineStr"/>
-    </row>
-    <row r="26" ht="90" customHeight="1">
-      <c r="A26" s="2" t="inlineStr">
+      <c r="G26" s="2" t="inlineStr"/>
+      <c r="H26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27" ht="90" customHeight="1">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>C35</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="B27" s="3" t="inlineStr">
         <is>
           <t>Legacy /api/studies over-returns studies across labs (was #44)</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr"/>
-      <c r="D26" s="2" t="inlineStr"/>
-      <c r="E26" s="2" t="inlineStr"/>
-      <c r="F26" s="2" t="inlineStr">
+      <c r="C27" s="3" t="inlineStr"/>
+      <c r="D27" s="3" t="inlineStr"/>
+      <c r="E27" s="3" t="inlineStr"/>
+      <c r="F27" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: GET /api/studies now scopes its list to the active lab
 when one is resolved from the Referer (server/routes.ts), so every returned row
@@ -1810,24 +1797,24 @@
 mirroring the /api/labs/:labId/studies handler. Closed 2026-06-14.</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr"/>
-      <c r="H26" s="2" t="inlineStr"/>
-    </row>
-    <row r="27" ht="90" customHeight="1">
-      <c r="A27" s="3" t="inlineStr">
+      <c r="G27" s="3" t="inlineStr"/>
+      <c r="H27" s="3" t="inlineStr"/>
+    </row>
+    <row r="28" ht="90" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>C30</t>
         </is>
       </c>
-      <c r="B27" s="3" t="inlineStr">
+      <c r="B28" s="2" t="inlineStr">
         <is>
           <t>Verify-script convention backfill (was #41)</t>
         </is>
       </c>
-      <c r="C27" s="3" t="inlineStr"/>
-      <c r="D27" s="3" t="inlineStr"/>
-      <c r="E27" s="3" t="inlineStr"/>
-      <c r="F27" s="3" t="inlineStr">
+      <c r="C28" s="2" t="inlineStr"/>
+      <c r="D28" s="2" t="inlineStr"/>
+      <c r="E28" s="2" t="inlineStr"/>
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: all 8 high-stakes math/logic commits now ship a paired
 scripts/verify-*.js (EP17 sensitivity, Deming lot-to-lot, CUMSUM+QC+multi-analyte,
@@ -1835,30 +1822,30 @@
 TEa boundary), per the strike-throughs in #41. Closed 2026-06-13.</t>
         </is>
       </c>
-      <c r="G27" s="3" t="inlineStr">
+      <c r="G28" s="2" t="inlineStr">
         <is>
           <t>scripts/audit_verify_script_coverage.py lookback, 2026-06-02; backfills
 landed 2026-06-03..06.
 ---</t>
         </is>
       </c>
-      <c r="H27" s="3" t="inlineStr"/>
-    </row>
-    <row r="28" ht="90" customHeight="1">
-      <c r="A28" s="2" t="inlineStr">
+      <c r="H28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29" ht="90" customHeight="1">
+      <c r="A29" s="3" t="inlineStr">
         <is>
           <t>C31</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="B29" s="3" t="inlineStr">
         <is>
           <t>VeritaPT AAA create/update/delete silently no-op in the multi-lab UI</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr"/>
-      <c r="D28" s="2" t="inlineStr"/>
-      <c r="E28" s="2" t="inlineStr"/>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="C29" s="3" t="inlineStr"/>
+      <c r="D29" s="3" t="inlineStr"/>
+      <c r="E29" s="3" t="inlineStr"/>
+      <c r="F29" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #754 (commit 92ad499) added lab-scoped POST/PUT/DELETE
 /api/labs/:labId/pt/aa-records. The UI posted to the lab-scoped path but only GET
@@ -1869,30 +1856,30 @@
 route mis-filed records to the user's default lab on multi-lab accounts).</t>
         </is>
       </c>
-      <c r="G28" s="2" t="inlineStr">
+      <c r="G29" s="3" t="inlineStr">
         <is>
           <t>2026-06-13, found during #18 Phase 3 QA;
 scripts/audit-labscoped-write-routes.mjs now guards the class.
 ---</t>
         </is>
       </c>
-      <c r="H28" s="2" t="inlineStr"/>
-    </row>
-    <row r="29" ht="90" customHeight="1">
-      <c r="A29" s="3" t="inlineStr">
+      <c r="H29" s="3" t="inlineStr"/>
+    </row>
+    <row r="30" ht="90" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>C32</t>
         </is>
       </c>
-      <c r="B29" s="3" t="inlineStr">
+      <c r="B30" s="2" t="inlineStr">
         <is>
           <t>VeritaComp "Unlock assessment" false-success no-op</t>
         </is>
       </c>
-      <c r="C29" s="3" t="inlineStr"/>
-      <c r="D29" s="3" t="inlineStr"/>
-      <c r="E29" s="3" t="inlineStr"/>
-      <c r="F29" s="3" t="inlineStr">
+      <c r="C30" s="2" t="inlineStr"/>
+      <c r="D30" s="2" t="inlineStr"/>
+      <c r="E30" s="2" t="inlineStr"/>
+      <c r="F30" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #755 (commit 4234007) moved the unlock route to
 /api/labs/:labId/competency/assessments/:id/unlock (the path the client calls).
@@ -1903,29 +1890,29 @@
 HTML).</t>
         </is>
       </c>
-      <c r="G29" s="3" t="inlineStr">
+      <c r="G30" s="2" t="inlineStr">
         <is>
           <t>2026-06-13, found by scripts/audit-labscoped-write-routes.mjs.
 ---</t>
         </is>
       </c>
-      <c r="H29" s="3" t="inlineStr"/>
-    </row>
-    <row r="30" ht="90" customHeight="1">
-      <c r="A30" s="2" t="inlineStr">
+      <c r="H30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31" ht="90" customHeight="1">
+      <c r="A31" s="3" t="inlineStr">
         <is>
           <t>C33</t>
         </is>
       </c>
-      <c r="B30" s="2" t="inlineStr">
+      <c r="B31" s="3" t="inlineStr">
         <is>
           <t>FK-cascade delete 500s + NavBar laptop-width overflow</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr"/>
-      <c r="D30" s="2" t="inlineStr"/>
-      <c r="E30" s="2" t="inlineStr"/>
-      <c r="F30" s="2" t="inlineStr">
+      <c r="C31" s="3" t="inlineStr"/>
+      <c r="D31" s="3" t="inlineStr"/>
+      <c r="E31" s="3" t="inlineStr"/>
+      <c r="F31" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PRs #749/#750 fixed NavBar horizontal overflow at laptop
 widths (collapse to the hamburger below 1560px); prod-verified at 1280-1920 with the
@@ -1936,37 +1923,9 @@
 500 -&gt; 200. scripts/audit-delete-cascades.mjs guards the class.</t>
         </is>
       </c>
-      <c r="G30" s="2" t="inlineStr">
+      <c r="G31" s="3" t="inlineStr">
         <is>
           <t>2026-06-13 browser QA of the A7-D4 wave + retro-QC of the 72h PR window.
----</t>
-        </is>
-      </c>
-      <c r="H30" s="2" t="inlineStr"/>
-    </row>
-    <row r="31" ht="90" customHeight="1">
-      <c r="A31" s="3" t="inlineStr">
-        <is>
-          <t>C1</t>
-        </is>
-      </c>
-      <c r="B31" s="3" t="inlineStr">
-        <is>
-          <t>FAQ "over 25 years" -&gt; "over 23 years"</t>
-        </is>
-      </c>
-      <c r="C31" s="3" t="inlineStr"/>
-      <c r="D31" s="3" t="inlineStr"/>
-      <c r="E31" s="3" t="inlineStr"/>
-      <c r="F31" s="3" t="inlineStr">
-        <is>
-          <t>Closure evidence: client/src/pages/FAQPage.tsx line 20 reads "over
-23 years" as of 2026-05-01.</t>
-        </is>
-      </c>
-      <c r="G31" s="3" t="inlineStr">
-        <is>
-          <t>session 299e9a73 turn 14, ~2026-04-28.
 ---</t>
         </is>
       </c>
@@ -1975,18 +1934,46 @@
     <row r="32" ht="90" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>C5</t>
+          <t>C1</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>David's VeritaQA grey-button bug (seat permissions mode)</t>
+          <t>FAQ "over 25 years" -&gt; "over 23 years"</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr"/>
       <c r="D32" s="2" t="inlineStr"/>
       <c r="E32" s="2" t="inlineStr"/>
       <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Closure evidence: client/src/pages/FAQPage.tsx line 20 reads "over
+23 years" as of 2026-05-01.</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>session 299e9a73 turn 14, ~2026-04-28.
+---</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33" ht="90" customHeight="1">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>David's VeritaQA grey-button bug (seat permissions mode)</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr"/>
+      <c r="D33" s="3" t="inlineStr"/>
+      <c r="E33" s="3" t="inlineStr"/>
+      <c r="F33" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #10 squash-merged as commit a43fbba on
 2026-05-01 23:19 MST. Railway deploy succeeded; deployed bundle
@@ -1999,7 +1986,7 @@
 against his exact stored shape (14 of 14 expected outcomes matched).</t>
         </is>
       </c>
-      <c r="G32" s="2" t="inlineStr">
+      <c r="G33" s="3" t="inlineStr">
         <is>
           <t>2026-05-01 David's report; veritabench + veritastock
 weren't in MODULE_LIST so seat permissions silently defaulted to
@@ -2007,46 +1994,17 @@
 ---</t>
         </is>
       </c>
-      <c r="H32" s="2" t="inlineStr"/>
-    </row>
-    <row r="33" ht="90" customHeight="1">
-      <c r="A33" s="3" t="inlineStr">
-        <is>
-          <t>C2</t>
-        </is>
-      </c>
-      <c r="B33" s="3" t="inlineStr">
-        <is>
-          <t>TeamPage present-tense "TJC surveyor" check</t>
-        </is>
-      </c>
-      <c r="C33" s="3" t="inlineStr"/>
-      <c r="D33" s="3" t="inlineStr"/>
-      <c r="E33" s="3" t="inlineStr"/>
-      <c r="F33" s="3" t="inlineStr">
-        <is>
-          <t>Closure evidence: site-wide search confirmed all surveyor language
-is past-tense, consistent with user's 2021-2025 service. User closed
-the item in session 299e9a73 turn 4.</t>
-        </is>
-      </c>
-      <c r="G33" s="3" t="inlineStr">
-        <is>
-          <t>session 299e9a73, ~2026-04-28.
----</t>
-        </is>
-      </c>
       <c r="H33" s="3" t="inlineStr"/>
     </row>
     <row r="34" ht="90" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>C3</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>My Studies CSV/XLSX export (John as design partner)</t>
+          <t>TeamPage present-tense "TJC surveyor" check</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr"/>
@@ -2054,14 +2012,14 @@
       <c r="E34" s="2" t="inlineStr"/>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: client/src/pages/DashboardPage.tsx line 46 calls
-/api/my-studies/export. server/routes.ts line 1491 implements the
-endpoint. Pulled forward into pre-COLA per user instruction.</t>
+          <t>Closure evidence: site-wide search confirmed all surveyor language
+is past-tense, consistent with user's 2021-2025 service. User closed
+the item in session 299e9a73 turn 4.</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>session 299e9a73 turn 5, ~2026-04-28.
+          <t>session 299e9a73, ~2026-04-28.
 ---</t>
         </is>
       </c>
@@ -2070,12 +2028,12 @@
     <row r="35" ht="90" customHeight="1">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>C4</t>
+          <t>C3</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>Rotate GitHub PAT (because old PAT was committed in SESSION_HANDOFF files)</t>
+          <t>My Studies CSV/XLSX export (John as design partner)</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr"/>
@@ -2083,13 +2041,14 @@
       <c r="E35" s="3" t="inlineStr"/>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: no ghp_* or github_pat_* patterns in current
-SESSION_HANDOFF.md or SESSION_HANDOFF-2.md as of 2026-05-01.</t>
+          <t>Closure evidence: client/src/pages/DashboardPage.tsx line 46 calls
+/api/my-studies/export. server/routes.ts line 1491 implements the
+endpoint. Pulled forward into pre-COLA per user instruction.</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>session 299e9a73, ~2026-04-28.
+          <t>session 299e9a73 turn 5, ~2026-04-28.
 ---</t>
         </is>
       </c>
@@ -2098,18 +2057,46 @@
     <row r="36" ht="90" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>C6</t>
+          <t>C4</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>VeritaPolicy service-line filtering removed (formerly #4)</t>
+          <t>Rotate GitHub PAT (because old PAT was committed in SESSION_HANDOFF files)</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr"/>
       <c r="D36" s="2" t="inlineStr"/>
       <c r="E36" s="2" t="inlineStr"/>
       <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Closure evidence: no ghp_* or github_pat_* patterns in current
+SESSION_HANDOFF.md or SESSION_HANDOFF-2.md as of 2026-05-01.</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>session 299e9a73, ~2026-04-28.
+---</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr"/>
+    </row>
+    <row r="37" ht="90" customHeight="1">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>C6</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>VeritaPolicy service-line filtering removed (formerly #4)</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr"/>
+      <c r="D37" s="3" t="inlineStr"/>
+      <c r="E37" s="3" t="inlineStr"/>
+      <c r="F37" s="3" t="inlineStr">
         <is>
           <t>Closure rationale (operator decision 2026-05-10): Keep all
 VeritaPolicy rows. CFR-only references with no accreditor reference
@@ -2118,29 +2105,29 @@
 report misread the design intent.</t>
         </is>
       </c>
-      <c r="G36" s="2" t="inlineStr">
+      <c r="G37" s="3" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H36" s="2" t="inlineStr"/>
-    </row>
-    <row r="37" ht="90" customHeight="1">
-      <c r="A37" s="3" t="inlineStr">
+      <c r="H37" s="3" t="inlineStr"/>
+    </row>
+    <row r="38" ht="90" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
         <is>
           <t>C7</t>
         </is>
       </c>
-      <c r="B37" s="3" t="inlineStr">
+      <c r="B38" s="2" t="inlineStr">
         <is>
           <t>CLIA number format validation (formerly #13)</t>
         </is>
       </c>
-      <c r="C37" s="3" t="inlineStr"/>
-      <c r="D37" s="3" t="inlineStr"/>
-      <c r="E37" s="3" t="inlineStr"/>
-      <c r="F37" s="3" t="inlineStr">
+      <c r="C38" s="2" t="inlineStr"/>
+      <c r="D38" s="2" t="inlineStr"/>
+      <c r="E38" s="2" t="inlineStr"/>
+      <c r="F38" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: shared/validateClia.ts defines CLIA_REGEX =
 /^\d{2}D\d{7}$/ (line 24), validateClia() helper with whitespace
@@ -2151,30 +2138,30 @@
 shape exists and behaves as specified.</t>
         </is>
       </c>
-      <c r="G37" s="3" t="inlineStr">
+      <c r="G38" s="2" t="inlineStr">
         <is>
           <t>Agent verification 2026-05-10 via grep + file read.
 Operator confirmed shipped 2026-05-10.
 ---</t>
         </is>
       </c>
-      <c r="H37" s="3" t="inlineStr"/>
-    </row>
-    <row r="38" ht="90" customHeight="1">
-      <c r="A38" s="2" t="inlineStr">
+      <c r="H38" s="2" t="inlineStr"/>
+    </row>
+    <row r="39" ht="90" customHeight="1">
+      <c r="A39" s="3" t="inlineStr">
         <is>
           <t>C8</t>
         </is>
       </c>
-      <c r="B38" s="2" t="inlineStr">
+      <c r="B39" s="3" t="inlineStr">
         <is>
           <t>VeritaMap lab-wide menu toggle (formerly #19)</t>
         </is>
       </c>
-      <c r="C38" s="2" t="inlineStr"/>
-      <c r="D38" s="2" t="inlineStr"/>
-      <c r="E38" s="2" t="inlineStr"/>
-      <c r="F38" s="2" t="inlineStr">
+      <c r="C39" s="3" t="inlineStr"/>
+      <c r="D39" s="3" t="inlineStr"/>
+      <c r="E39" s="3" t="inlineStr"/>
+      <c r="F39" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: client/src/pages/VeritaMapLabwidePage.tsx
 exists and implements the labwide read-only union view. Route is
@@ -2184,59 +2171,59 @@
 parking lot plan (read-only union view, per-session toggle) shipped.</t>
         </is>
       </c>
-      <c r="G38" s="2" t="inlineStr">
+      <c r="G39" s="3" t="inlineStr">
         <is>
           <t>Agent verification 2026-05-10 via grep + file read.
 Operator confirmed shipped 2026-05-10.
 ---</t>
         </is>
       </c>
-      <c r="H38" s="2" t="inlineStr"/>
-    </row>
-    <row r="39" ht="90" customHeight="1">
-      <c r="A39" s="3" t="inlineStr">
-        <is>
-          <t>C9</t>
-        </is>
-      </c>
-      <c r="B39" s="3" t="inlineStr">
-        <is>
-          <t>Tier-1 smoke test checklist (formerly #6)</t>
-        </is>
-      </c>
-      <c r="C39" s="3" t="inlineStr"/>
-      <c r="D39" s="3" t="inlineStr"/>
-      <c r="E39" s="3" t="inlineStr"/>
-      <c r="F39" s="3" t="inlineStr">
-        <is>
-          <t>Closure evidence: docs/smoke-test-tier1.md documents the Tier-1
-smoke-test process and post-deploy verification steps. Shipped via
-PR #81 as part of the 2026-05-10 wave.</t>
-        </is>
-      </c>
-      <c r="G39" s="3" t="inlineStr">
-        <is>
-          <t>Operator instruction 2026-05-10 in this session.
----</t>
-        </is>
-      </c>
       <c r="H39" s="3" t="inlineStr"/>
     </row>
     <row r="40" ht="90" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>C10</t>
+          <t>C9</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Per-module gating (formerly #7)</t>
+          <t>Tier-1 smoke test checklist (formerly #6)</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr"/>
       <c r="D40" s="2" t="inlineStr"/>
       <c r="E40" s="2" t="inlineStr"/>
       <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>Closure evidence: docs/smoke-test-tier1.md documents the Tier-1
+smoke-test process and post-deploy verification steps. Shipped via
+PR #81 as part of the 2026-05-10 wave.</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>Operator instruction 2026-05-10 in this session.
+---</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr"/>
+    </row>
+    <row r="41" ht="90" customHeight="1">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>C10</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>Per-module gating (formerly #7)</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr"/>
+      <c r="D41" s="3" t="inlineStr"/>
+      <c r="E41" s="3" t="inlineStr"/>
+      <c r="F41" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: Client-side useIsReadOnly module keys wired
 on client/src/pages/VeritaPolicyAppPage.tsx and
@@ -2251,29 +2238,29 @@
 PR #76.</t>
         </is>
       </c>
-      <c r="G40" s="2" t="inlineStr">
+      <c r="G41" s="3" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H40" s="2" t="inlineStr"/>
-    </row>
-    <row r="41" ht="90" customHeight="1">
-      <c r="A41" s="3" t="inlineStr">
+      <c r="H41" s="3" t="inlineStr"/>
+    </row>
+    <row r="42" ht="90" customHeight="1">
+      <c r="A42" s="2" t="inlineStr">
         <is>
           <t>C11</t>
         </is>
       </c>
-      <c r="B41" s="3" t="inlineStr">
+      <c r="B42" s="2" t="inlineStr">
         <is>
           <t>VeritaStock shipped copy (formerly #8)</t>
         </is>
       </c>
-      <c r="C41" s="3" t="inlineStr"/>
-      <c r="D41" s="3" t="inlineStr"/>
-      <c r="E41" s="3" t="inlineStr"/>
-      <c r="F41" s="3" t="inlineStr">
+      <c r="C42" s="2" t="inlineStr"/>
+      <c r="D42" s="2" t="inlineStr"/>
+      <c r="E42" s="2" t="inlineStr"/>
+      <c r="F42" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: client/src/pages/ArticleInventoryManagementPage.tsx
 line 305 footer reads "platform that includes VeritaStock™" instead
@@ -2281,29 +2268,29 @@
 on /resources/laboratory-inventory-management. Shipped via PR #75.</t>
         </is>
       </c>
-      <c r="G41" s="3" t="inlineStr">
+      <c r="G42" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H41" s="3" t="inlineStr"/>
-    </row>
-    <row r="42" ht="90" customHeight="1">
-      <c r="A42" s="2" t="inlineStr">
+      <c r="H42" s="2" t="inlineStr"/>
+    </row>
+    <row r="43" ht="90" customHeight="1">
+      <c r="A43" s="3" t="inlineStr">
         <is>
           <t>C12</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
+      <c r="B43" s="3" t="inlineStr">
         <is>
           <t>Admin report one-row-per-lab (formerly #14)</t>
         </is>
       </c>
-      <c r="C42" s="2" t="inlineStr"/>
-      <c r="D42" s="2" t="inlineStr"/>
-      <c r="E42" s="2" t="inlineStr"/>
-      <c r="F42" s="2" t="inlineStr">
+      <c r="C43" s="3" t="inlineStr"/>
+      <c r="D43" s="3" t="inlineStr"/>
+      <c r="E43" s="3" t="inlineStr"/>
+      <c r="F43" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: /api/admin/report rewritten in
 server/routes.ts (~line 595) to LEFT JOIN labs on
@@ -2318,33 +2305,6 @@
 prerequisite, not a code bug). Shipped via PR #85.</t>
         </is>
       </c>
-      <c r="G42" s="2" t="inlineStr">
-        <is>
-          <t>Operator instruction 2026-05-10 in this session.
----</t>
-        </is>
-      </c>
-      <c r="H42" s="2" t="inlineStr"/>
-    </row>
-    <row r="43" ht="90" customHeight="1">
-      <c r="A43" s="3" t="inlineStr">
-        <is>
-          <t>C14</t>
-        </is>
-      </c>
-      <c r="B43" s="3" t="inlineStr">
-        <is>
-          <t>UI relabel "CLIA TEa" -&gt; "Lab-Set Internal Goal" (formerly #1)</t>
-        </is>
-      </c>
-      <c r="C43" s="3" t="inlineStr"/>
-      <c r="D43" s="3" t="inlineStr"/>
-      <c r="E43" s="3" t="inlineStr"/>
-      <c r="F43" s="3" t="inlineStr">
-        <is>
-          <t>Closure evidence: Shipped across four PRs over 2026-05-10.</t>
-        </is>
-      </c>
       <c r="G43" s="3" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
@@ -2356,18 +2316,45 @@
     <row r="44" ht="90" customHeight="1">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>C13</t>
+          <t>C14</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>WSLH PT vendor (formerly #15)</t>
+          <t>UI relabel "CLIA TEa" -&gt; "Lab-Set Internal Goal" (formerly #1)</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr"/>
       <c r="D44" s="2" t="inlineStr"/>
       <c r="E44" s="2" t="inlineStr"/>
       <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>Closure evidence: Shipped across four PRs over 2026-05-10.</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>Operator instruction 2026-05-10 in this session.
+---</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr"/>
+    </row>
+    <row r="45" ht="90" customHeight="1">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>C13</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>WSLH PT vendor (formerly #15)</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr"/>
+      <c r="D45" s="3" t="inlineStr"/>
+      <c r="E45" s="3" t="inlineStr"/>
+      <c r="F45" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: Shipped 2026-05-10 via PR #79 (merge commit
 eeebc6e; merged after rebase to resolve a server/db.ts collision
@@ -2385,38 +2372,9 @@
 'WSLH' is the post-deploy success signal. Shipped via PR #79.</t>
         </is>
       </c>
-      <c r="G44" s="2" t="inlineStr">
+      <c r="G45" s="3" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
----</t>
-        </is>
-      </c>
-      <c r="H44" s="2" t="inlineStr"/>
-    </row>
-    <row r="45" ht="90" customHeight="1">
-      <c r="A45" s="3" t="inlineStr">
-        <is>
-          <t>C15</t>
-        </is>
-      </c>
-      <c r="B45" s="3" t="inlineStr">
-        <is>
-          <t>VeritaStock lot tracking + expiration + reorder alerts (formerly #21)</t>
-        </is>
-      </c>
-      <c r="C45" s="3" t="inlineStr"/>
-      <c r="D45" s="3" t="inlineStr"/>
-      <c r="E45" s="3" t="inlineStr"/>
-      <c r="F45" s="3" t="inlineStr">
-        <is>
-          <t>Closure evidence: VeritaStock™ shipped the bench-level inventory
-features the Perplexity competitor analysis identified as a gap:</t>
-        </is>
-      </c>
-      <c r="G45" s="3" t="inlineStr">
-        <is>
-          <t>Originally Perplexity competitor analysis 2026-05-10.
-Audit 2026-05-21 confirmed the feature set ships today.
 ---</t>
         </is>
       </c>
@@ -2425,12 +2383,12 @@
     <row r="46" ht="90" customHeight="1">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>C16</t>
+          <t>C15</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>PAL studies guided workflow (formerly #23)</t>
+          <t>VeritaStock lot tracking + expiration + reorder alerts (formerly #21)</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr"/>
@@ -2438,15 +2396,14 @@
       <c r="E46" s="2" t="inlineStr"/>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: VeritaCheck™ already ships the Precision /
-Accuracy / Linearity (PAL) study set under EP-protocol naming:</t>
+          <t>Closure evidence: VeritaStock™ shipped the bench-level inventory
+features the Perplexity competitor analysis identified as a gap:</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
           <t>Originally Perplexity competitor analysis 2026-05-10.
-Audit 2026-05-21 confirmed the EP studies cover the PAL framing in
-full.
+Audit 2026-05-21 confirmed the feature set ships today.
 ---</t>
         </is>
       </c>
@@ -2455,12 +2412,12 @@
     <row r="47" ht="90" customHeight="1">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>C17</t>
+          <t>C16</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>Source-grounded 21/29/45 CFR + 42 CFR 482-485 (formerly #26)</t>
+          <t>PAL studies guided workflow (formerly #23)</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr"/>
@@ -2468,35 +2425,65 @@
       <c r="E47" s="3" t="inlineStr"/>
       <c r="F47" s="3" t="inlineStr">
         <is>
+          <t>Closure evidence: VeritaCheck™ already ships the Precision /
+Accuracy / Linearity (PAL) study set under EP-protocol naming:</t>
+        </is>
+      </c>
+      <c r="G47" s="3" t="inlineStr">
+        <is>
+          <t>Originally Perplexity competitor analysis 2026-05-10.
+Audit 2026-05-21 confirmed the EP studies cover the PAL framing in
+full.
+---</t>
+        </is>
+      </c>
+      <c r="H47" s="3" t="inlineStr"/>
+    </row>
+    <row r="48" ht="90" customHeight="1">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>C17</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Source-grounded 21/29/45 CFR + 42 CFR 482-485 (formerly #26)</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr"/>
+      <c r="D48" s="2" t="inlineStr"/>
+      <c r="E48" s="2" t="inlineStr"/>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
           <t>Closure evidence: PR #301 (commit 8c27806, merged 2026-05-21)
 source-grounded the 74 remaining non-493 entries in
 server/cfrRequirements.ts against verbatim eCFR XML. Breakdown
 shipped:</t>
         </is>
       </c>
-      <c r="G47" s="3" t="inlineStr">
+      <c r="G48" s="2" t="inlineStr">
         <is>
           <t>PR #301; tasks #18 in the in-session task tracker.
 ---</t>
         </is>
       </c>
-      <c r="H47" s="3" t="inlineStr"/>
-    </row>
-    <row r="48" ht="90" customHeight="1">
-      <c r="A48" s="2" t="inlineStr">
+      <c r="H48" s="2" t="inlineStr"/>
+    </row>
+    <row r="49" ht="90" customHeight="1">
+      <c r="A49" s="3" t="inlineStr">
         <is>
           <t>C18</t>
         </is>
       </c>
-      <c r="B48" s="2" t="inlineStr">
+      <c r="B49" s="3" t="inlineStr">
         <is>
           <t>VeritaPolicy "Non CLIA" chapter rename (formerly #3)</t>
         </is>
       </c>
-      <c r="C48" s="2" t="inlineStr"/>
-      <c r="D48" s="2" t="inlineStr"/>
-      <c r="E48" s="2" t="inlineStr"/>
-      <c r="F48" s="2" t="inlineStr">
+      <c r="C49" s="3" t="inlineStr"/>
+      <c r="D49" s="3" t="inlineStr"/>
+      <c r="E49" s="3" t="inlineStr"/>
+      <c r="F49" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #300 (commit 34d7707, merged 2026-05-21)
 renamed all 44 user-facing chapter labels in
@@ -2507,7 +2494,7 @@
 page.</t>
         </is>
       </c>
-      <c r="G48" s="2" t="inlineStr">
+      <c r="G49" s="3" t="inlineStr">
         <is>
           <t>CAP customer screenshot of the /veritapolicy chapter
 headers, 2026-05-01 evening. PR #300; tasks #17 in the in-session
@@ -2515,23 +2502,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H48" s="2" t="inlineStr"/>
-    </row>
-    <row r="49" ht="90" customHeight="1">
-      <c r="A49" s="3" t="inlineStr">
+      <c r="H49" s="3" t="inlineStr"/>
+    </row>
+    <row r="50" ht="90" customHeight="1">
+      <c r="A50" s="2" t="inlineStr">
         <is>
           <t>C19</t>
         </is>
       </c>
-      <c r="B49" s="3" t="inlineStr">
+      <c r="B50" s="2" t="inlineStr">
         <is>
           <t>VeritaStock department-scope toggle (formerly #31)</t>
         </is>
       </c>
-      <c r="C49" s="3" t="inlineStr"/>
-      <c r="D49" s="3" t="inlineStr"/>
-      <c r="E49" s="3" t="inlineStr"/>
-      <c r="F49" s="3" t="inlineStr">
+      <c r="C50" s="2" t="inlineStr"/>
+      <c r="D50" s="2" t="inlineStr"/>
+      <c r="E50" s="2" t="inlineStr"/>
+      <c r="F50" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #319 (commit d01f5fe, merged 2026-05-22)
 shipped the persistent dept-scope toggle on VeritaStockPage. A new
@@ -2542,7 +2529,7 @@
 workspace without re-filtering.</t>
         </is>
       </c>
-      <c r="G49" s="3" t="inlineStr">
+      <c r="G50" s="2" t="inlineStr">
         <is>
           <t>John, San Carlos lab, 2026-05-21. Same conversation that
 drove the vendor dropdown (PR #304), FILTERED VIEW banner (PR #305),
@@ -2550,23 +2537,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H49" s="3" t="inlineStr"/>
-    </row>
-    <row r="50" ht="90" customHeight="1">
-      <c r="A50" s="2" t="inlineStr">
+      <c r="H50" s="2" t="inlineStr"/>
+    </row>
+    <row r="51" ht="90" customHeight="1">
+      <c r="A51" s="3" t="inlineStr">
         <is>
           <t>C20</t>
         </is>
       </c>
-      <c r="B50" s="2" t="inlineStr">
+      <c r="B51" s="3" t="inlineStr">
         <is>
           <t>Primary-lab seat counting (formerly #12)</t>
         </is>
       </c>
-      <c r="C50" s="2" t="inlineStr"/>
-      <c r="D50" s="2" t="inlineStr"/>
-      <c r="E50" s="2" t="inlineStr"/>
-      <c r="F50" s="2" t="inlineStr">
+      <c r="C51" s="3" t="inlineStr"/>
+      <c r="D51" s="3" t="inlineStr"/>
+      <c r="E51" s="3" t="inlineStr"/>
+      <c r="F51" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: is_primary_lab INTEGER NOT NULL DEFAULT 0
 column was added to the lab_members table at db.ts:1276, with the
@@ -2577,7 +2564,7 @@
 is_primary_lab=1 ordering).</t>
         </is>
       </c>
-      <c r="G50" s="2" t="inlineStr">
+      <c r="G51" s="3" t="inlineStr">
         <is>
           <t>2026-05-07 multi-lab discussion. Build shipped as part
 of the Multi-Lab Tier 2 architecture work (Phase 3.x series, prior
@@ -2586,23 +2573,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H50" s="2" t="inlineStr"/>
-    </row>
-    <row r="51" ht="90" customHeight="1">
-      <c r="A51" s="3" t="inlineStr">
+      <c r="H51" s="3" t="inlineStr"/>
+    </row>
+    <row r="52" ht="90" customHeight="1">
+      <c r="A52" s="2" t="inlineStr">
         <is>
           <t>C21</t>
         </is>
       </c>
-      <c r="B51" s="3" t="inlineStr">
+      <c r="B52" s="2" t="inlineStr">
         <is>
           <t>Multi-lab pricing model — Option A (formerly #11)</t>
         </is>
       </c>
-      <c r="C51" s="3" t="inlineStr"/>
-      <c r="D51" s="3" t="inlineStr"/>
-      <c r="E51" s="3" t="inlineStr"/>
-      <c r="F51" s="3" t="inlineStr">
+      <c r="C52" s="2" t="inlineStr"/>
+      <c r="D52" s="2" t="inlineStr"/>
+      <c r="E52" s="2" t="inlineStr"/>
+      <c r="F52" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #322 (commit 0ccd925, merged 2026-05-22)
 added the customer-facing line to the pricing page that reflects
@@ -2615,7 +2602,7 @@
 Enterprise+ block, reads:</t>
         </is>
       </c>
-      <c r="G51" s="3" t="inlineStr">
+      <c r="G52" s="2" t="inlineStr">
         <is>
           <t>2026-05-07 multi-lab discussion (Lisa Veri's
 canonical-case session). PR #322 (initial build); softening PR
@@ -2624,30 +2611,30 @@
 ---</t>
         </is>
       </c>
-      <c r="H51" s="3" t="inlineStr"/>
-    </row>
-    <row r="52" ht="90" customHeight="1">
-      <c r="A52" s="2" t="inlineStr">
+      <c r="H52" s="2" t="inlineStr"/>
+    </row>
+    <row r="53" ht="90" customHeight="1">
+      <c r="A53" s="3" t="inlineStr">
         <is>
           <t>C22</t>
         </is>
       </c>
-      <c r="B52" s="2" t="inlineStr">
+      <c r="B53" s="3" t="inlineStr">
         <is>
           <t>VeritaOps cost-per-test module (formerly #10)</t>
         </is>
       </c>
-      <c r="C52" s="2" t="inlineStr"/>
-      <c r="D52" s="2" t="inlineStr"/>
-      <c r="E52" s="2" t="inlineStr"/>
-      <c r="F52" s="2" t="inlineStr">
+      <c r="C53" s="3" t="inlineStr"/>
+      <c r="D53" s="3" t="inlineStr"/>
+      <c r="E53" s="3" t="inlineStr"/>
+      <c r="F53" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: v1 of the VeritaOps Cost-Per-Reportable-Test
 (CPRT) module shipped across PR #325 through PR #330 on 2026-05-22.
 The module is feature-complete for the typical lab director workflow.</t>
         </is>
       </c>
-      <c r="G52" s="2" t="inlineStr">
+      <c r="G53" s="3" t="inlineStr">
         <is>
           <t>This thread, 2026-05-07 12:05 PM CDT, user message:
 "Parking lot: build an operations module for cost per test
@@ -2656,262 +2643,262 @@
 ---</t>
         </is>
       </c>
-      <c r="H52" s="2" t="inlineStr"/>
-    </row>
-    <row r="53" ht="90" customHeight="1">
-      <c r="A53" s="3" t="inlineStr">
+      <c r="H53" s="3" t="inlineStr"/>
+    </row>
+    <row r="54" ht="90" customHeight="1">
+      <c r="A54" s="2" t="inlineStr">
         <is>
           <t>C23</t>
         </is>
       </c>
-      <c r="B53" s="3" t="inlineStr">
+      <c r="B54" s="2" t="inlineStr">
         <is>
           <t>CCL lab name visual disambiguation in lab switcher (formerly #34)</t>
         </is>
       </c>
-      <c r="C53" s="3" t="inlineStr"/>
-      <c r="D53" s="3" t="inlineStr">
+      <c r="C54" s="2" t="inlineStr"/>
+      <c r="D54" s="2" t="inlineStr">
         <is>
           <t>XS (under 1 day, actual)</t>
         </is>
       </c>
-      <c r="E53" s="3" t="inlineStr">
+      <c r="E54" s="2" t="inlineStr">
         <is>
           <t>Low — cosmetic; only mattered when Lisa or Michael picked the wrong lab from...</t>
         </is>
       </c>
-      <c r="F53" s="3" t="inlineStr">
+      <c r="F54" s="2" t="inlineStr">
         <is>
           <t>Effort: XS (under 1 day, actual)
 Importance: Low — cosmetic; only mattered when Lisa or Michael picked the wrong lab from the dropdown.</t>
         </is>
       </c>
-      <c r="G53" s="3" t="inlineStr">
+      <c r="G54" s="2" t="inlineStr">
         <is>
           <t>flagged 2026-05-23 immediately after provisioning Lisa's CCL lab; closed 2026-05-24.
 ---</t>
         </is>
       </c>
-      <c r="H53" s="3" t="inlineStr"/>
-    </row>
-    <row r="54" ht="90" customHeight="1">
-      <c r="A54" s="2" t="inlineStr">
+      <c r="H54" s="2" t="inlineStr"/>
+    </row>
+    <row r="55" ht="90" customHeight="1">
+      <c r="A55" s="3" t="inlineStr">
         <is>
           <t>C24</t>
         </is>
       </c>
-      <c r="B54" s="2" t="inlineStr">
+      <c r="B55" s="3" t="inlineStr">
         <is>
           <t>VC Unlimited Y1/Y2 price disclosure UX (formerly #35)</t>
         </is>
       </c>
-      <c r="C54" s="2" t="inlineStr"/>
-      <c r="D54" s="2" t="inlineStr">
+      <c r="C55" s="3" t="inlineStr"/>
+      <c r="D55" s="3" t="inlineStr">
         <is>
           <t>XS (under 1 day, actual)</t>
         </is>
       </c>
-      <c r="E54" s="2" t="inlineStr">
+      <c r="E55" s="3" t="inlineStr">
         <is>
           <t>Low when shipped (proactive, no customer complaint yet) — but high if a procu...</t>
         </is>
       </c>
-      <c r="F54" s="2" t="inlineStr">
+      <c r="F55" s="3" t="inlineStr">
         <is>
           <t>Effort: XS (under 1 day, actual)
 Importance: Low when shipped (proactive, no customer complaint yet) — but high if a procurement reviewer later disputes the $499 renewal as undisclosed.</t>
         </is>
       </c>
-      <c r="G54" s="2" t="inlineStr">
+      <c r="G55" s="3" t="inlineStr">
         <is>
           <t>Pricing rebuild 2026-05-23; closed 2026-05-24 proactively before any customer dispute.
 ---</t>
         </is>
       </c>
-      <c r="H54" s="2" t="inlineStr"/>
-    </row>
-    <row r="55" ht="90" customHeight="1">
-      <c r="A55" s="3" t="inlineStr">
+      <c r="H55" s="3" t="inlineStr"/>
+    </row>
+    <row r="56" ht="90" customHeight="1">
+      <c r="A56" s="2" t="inlineStr">
         <is>
           <t>C25</t>
         </is>
       </c>
-      <c r="B55" s="3" t="inlineStr">
+      <c r="B56" s="2" t="inlineStr">
         <is>
           <t>VeritaQC Phase 1 (Levey-Jennings + Westgard live engine) (formerly #20)</t>
         </is>
       </c>
-      <c r="C55" s="3" t="inlineStr"/>
-      <c r="D55" s="3" t="inlineStr">
+      <c r="C56" s="2" t="inlineStr"/>
+      <c r="D56" s="2" t="inlineStr">
         <is>
           <t>L (about 5 days end-to-end, actual: Phase 0 schema → Phase 1A evaluator → 1B...</t>
         </is>
       </c>
-      <c r="E55" s="3" t="inlineStr">
+      <c r="E56" s="2" t="inlineStr">
         <is>
           <t>High — largest single gap vs myLabCompliance.io per Perplexity competitor ana...</t>
         </is>
       </c>
-      <c r="F55" s="3" t="inlineStr">
+      <c r="F56" s="2" t="inlineStr">
         <is>
           <t>Effort: L (about 5 days end-to-end, actual: Phase 0 schema → Phase 1A evaluator → 1B entry UI → 1C daily review → 1D monthly PDF + attestation)
 Importance: High — largest single gap vs myLabCompliance.io per Perplexity competitor analysis; promotes VeritaAssure from documentation tool to lab operations platform.</t>
         </is>
       </c>
-      <c r="G55" s="3" t="inlineStr">
+      <c r="G56" s="2" t="inlineStr">
         <is>
           <t>Perplexity competitor analysis 2026-05-10. Scoping confirmed via the build_phase1_mockup.py iterations 2026-05-24. Shipped 2026-05-25.
 ---</t>
         </is>
       </c>
-      <c r="H55" s="3" t="inlineStr"/>
-    </row>
-    <row r="56" ht="90" customHeight="1">
-      <c r="A56" s="2" t="inlineStr">
+      <c r="H56" s="2" t="inlineStr"/>
+    </row>
+    <row r="57" ht="90" customHeight="1">
+      <c r="A57" s="3" t="inlineStr">
         <is>
           <t>C26</t>
         </is>
       </c>
-      <c r="B56" s="2" t="inlineStr">
+      <c r="B57" s="3" t="inlineStr">
         <is>
           <t>VeritaLab CMS-116 application support + state licensing registry (formerly #22)</t>
         </is>
       </c>
-      <c r="C56" s="2" t="inlineStr"/>
-      <c r="D56" s="2" t="inlineStr">
+      <c r="C57" s="3" t="inlineStr"/>
+      <c r="D57" s="3" t="inlineStr">
         <is>
           <t>M (1-2 weeks for v1, actual)</t>
         </is>
       </c>
-      <c r="E56" s="2" t="inlineStr">
+      <c r="E57" s="3" t="inlineStr">
         <is>
           <t>Medium — competitor parity (myLabCompliance.io) plus useful at lab startup an...</t>
         </is>
       </c>
-      <c r="F56" s="2" t="inlineStr">
+      <c r="F57" s="3" t="inlineStr">
         <is>
           <t>Effort: M (1-2 weeks for v1, actual)
 Importance: Medium — competitor parity (myLabCompliance.io) plus useful at lab startup and at certificate-type changes.</t>
         </is>
       </c>
-      <c r="G56" s="2" t="inlineStr">
+      <c r="G57" s="3" t="inlineStr">
         <is>
           <t>Perplexity competitor analysis (myLabCompliance.io), 2026-05-10. Reclassified as a VeritaLab extension 2026-05-25. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H56" s="2" t="inlineStr"/>
-    </row>
-    <row r="57" ht="90" customHeight="1">
-      <c r="A57" s="3" t="inlineStr">
+      <c r="H57" s="3" t="inlineStr"/>
+    </row>
+    <row r="58" ht="90" customHeight="1">
+      <c r="A58" s="2" t="inlineStr">
         <is>
           <t>C27</t>
         </is>
       </c>
-      <c r="B57" s="3" t="inlineStr">
+      <c r="B58" s="2" t="inlineStr">
         <is>
           <t>Active vs view-only seat split (formerly #33)</t>
         </is>
       </c>
-      <c r="C57" s="3" t="inlineStr"/>
-      <c r="D57" s="3" t="inlineStr">
+      <c r="C58" s="2" t="inlineStr"/>
+      <c r="D58" s="2" t="inlineStr">
         <is>
           <t>M (~1 week of engineering, actual: shipped in a single multi-PR session)</t>
         </is>
       </c>
-      <c r="E57" s="3" t="inlineStr">
+      <c r="E58" s="2" t="inlineStr">
         <is>
           <t>Medium — closed the gap between /pricing copy and product behavior; gives sal...</t>
         </is>
       </c>
-      <c r="F57" s="3" t="inlineStr">
+      <c r="F58" s="2" t="inlineStr">
         <is>
           <t>Effort: M (~1 week of engineering, actual: shipped in a single multi-PR session)
 Importance: Medium — closed the gap between /pricing copy and product behavior; gives sales a clean answer for "do you charge for our medical director?"</t>
         </is>
       </c>
-      <c r="G57" s="3" t="inlineStr">
+      <c r="G58" s="2" t="inlineStr">
         <is>
           <t>Pricing analysis doc Decision 3 (2026-05-21); MEDIUM scenario revised 2026-05-29 to retire the "unlimited view-only" claim. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H57" s="3" t="inlineStr"/>
-    </row>
-    <row r="58" ht="90" customHeight="1">
-      <c r="A58" s="2" t="inlineStr">
+      <c r="H58" s="2" t="inlineStr"/>
+    </row>
+    <row r="59" ht="90" customHeight="1">
+      <c r="A59" s="3" t="inlineStr">
         <is>
           <t>C28</t>
         </is>
       </c>
-      <c r="B58" s="2" t="inlineStr">
+      <c r="B59" s="3" t="inlineStr">
         <is>
           <t>"Why VeritaCheck" comparative one-pager (formerly #37)</t>
         </is>
       </c>
-      <c r="C58" s="2" t="inlineStr"/>
-      <c r="D58" s="2" t="inlineStr">
+      <c r="C59" s="3" t="inlineStr"/>
+      <c r="D59" s="3" t="inlineStr">
         <is>
           <t>S (one design pass + four claim paragraphs + PDF + matching marketing-site pa...</t>
         </is>
       </c>
-      <c r="E58" s="2" t="inlineStr">
+      <c r="E59" s="3" t="inlineStr">
         <is>
           <t>Medium — closed a positioning gap surfaced by six COLA conference attendees a...</t>
         </is>
       </c>
-      <c r="F58" s="2" t="inlineStr">
+      <c r="F59" s="3" t="inlineStr">
         <is>
           <t>Effort: S (one design pass + four claim paragraphs + PDF + matching marketing-site page, actual)
 Importance: Medium — closed a positioning gap surfaced by six COLA conference attendees attached to a legacy verification tool; converts product-quality advantage into a leave-behind Lisa can hand out.</t>
         </is>
       </c>
-      <c r="G58" s="2" t="inlineStr">
+      <c r="G59" s="3" t="inlineStr">
         <is>
           <t>2026-05-11 / 2026-05-12 conference notes review with Michael. Conference attendees (Whitehead, Odegard, Othman, Molinelli, Kyle, Allred) expressed interest in equivalent / superior product. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H58" s="2" t="inlineStr"/>
-    </row>
-    <row r="59" ht="90" customHeight="1">
-      <c r="A59" s="3" t="inlineStr">
+      <c r="H59" s="3" t="inlineStr"/>
+    </row>
+    <row r="60" ht="90" customHeight="1">
+      <c r="A60" s="2" t="inlineStr">
         <is>
           <t>C29</t>
         </is>
       </c>
-      <c r="B59" s="3" t="inlineStr">
+      <c r="B60" s="2" t="inlineStr">
         <is>
           <t>VeritaPolicy approval workflow — MediaLab functional mirror</t>
         </is>
       </c>
-      <c r="C59" s="3" t="inlineStr"/>
-      <c r="D59" s="3" t="inlineStr">
+      <c r="C60" s="2" t="inlineStr"/>
+      <c r="D60" s="2" t="inlineStr">
         <is>
           <t>XL (one focused session, 12 PRs landed)</t>
         </is>
       </c>
-      <c r="E59" s="3" t="inlineStr">
+      <c r="E60" s="2" t="inlineStr">
         <is>
           <t>High — replaces MediaLab Document Control ($752/$2,250 starting price, scalin...</t>
         </is>
       </c>
-      <c r="F59" s="3" t="inlineStr">
+      <c r="F60" s="2" t="inlineStr">
         <is>
           <t>Effort: XL (one focused session, 12 PRs landed)
 Importance: High — replaces MediaLab Document Control ($752/$2,250 starting price, scaling to $10K-$20K/yr at enterprise per Capterra public data) with an included VeritaPolicy feature; closes a real positioning gap and gives sales a direct comparator line.</t>
         </is>
       </c>
-      <c r="G59" s="3" t="inlineStr">
+      <c r="G60" s="2" t="inlineStr">
         <is>
           <t>Pricing strategy conversation 2026-05-29 (Michael: "I don't like bolt-ons; we should replicate this") → scoped 8 phases → shipped all 12 PRs in single session. Shipped 2026-05-29.
 ---</t>
         </is>
       </c>
-      <c r="H59" s="3" t="inlineStr"/>
+      <c r="H60" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H59"/>
+  <autoFilter ref="A1:H60"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
TASK: Parking lot - close #43 as C59 (keep finding-closure MD/designee/owner-only); regen xlsx
PLAN:
  1. Record operator decision to keep finding closure MD/designee/owner-only; move #43 to CLOSED as C59.
  2. Regenerate PARKING_LOT.xlsx (OPEN 12 -> 11).

Self-check:
  - No code change (prod already enforces this).
  - md + xlsx committed together per the sync rule.
  - Gate 3 N/A (internal documentation).
</commit_message>
<xml_diff>
--- a/PARKING_LOT.xlsx
+++ b/PARKING_LOT.xlsx
@@ -12,8 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RETIRED" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$59</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$60</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RETIRED'!$A$1:$H$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1006,83 +1006,44 @@
     <row r="12" ht="90" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>44</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Confirm the finding-closure signer policy (non-MD admins now blocked)</t>
+          <t>Regenerate the 119-function access-inventory Excel with the corrected MD persona</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Open, awaiting operator confirmation. Reverting is a one-line change (re-add the owner/admin path in the findings/:id/signoff handler) if admins should retain finding closure.
+          <t>Open, low priority. Offered to Michael; skippable if the sweep was a one-off working artifact.
 ---</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>XS (a yes/no decision; ~15 min to loosen the gate if reversed).</t>
+          <t>XS (~15 min to re-run the sweep harness and re-deliver).</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Medium — changes who can close VeritaResponse findings in production; affects...</t>
+          <t>Low — the harness and the shipped fixes are correct; only the recorded Excel'...</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Item 5 Phase 2 tightened VeritaResponse finding closure from "any owner / admin / edit-seat" to "the designated medical director, a delegated designee holding finding-closure for the lab's complexity, or the account owner as a logged break-glass override." This is live on prod (#1443). It follows the agreed MD-or-designee model (QB=1), and the same gate now guards QC period-review co-sign. It has not been confirmed against real customer workflows: if any lab relies on non-MD admins closing findings, they now need a Letter of Delegation, or the gate must be loosened.</t>
+          <t>The full-inventory 4-login access sweep (VeritaAssure_Function_Inventory.xlsx) was first generated with the medical-director test persona mis-seeded as a seatless member, which over-flagged its column. The harness was then corrected to seat the MD as the active writer it actually is (scripts/qa-sweep/inventory-sweep.ts). The delivered Excel still shows the old md results; re-running reclassifies the md-artifact flags down to the real findings, which were already fixed in PR A (#1441). Only worth doing if the sheet gets filed or shared externally.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>this session, delegation feature build (2026-10-04). Flagged repeatedly in-session; awaiting explicit operator sign-off.</t>
+          <t>this session, QA sweep (2026-10-03 to 2026-10-04).</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr"/>
     </row>
-    <row r="13" ht="90" customHeight="1">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>44</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>Regenerate the 119-function access-inventory Excel with the corrected MD persona</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>Open, low priority. Offered to Michael; skippable if the sweep was a one-off working artifact.
----</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>XS (~15 min to re-run the sweep harness and re-deliver).</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>Low — the harness and the shipped fixes are correct; only the recorded Excel'...</t>
-        </is>
-      </c>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>The full-inventory 4-login access sweep (VeritaAssure_Function_Inventory.xlsx) was first generated with the medical-director test persona mis-seeded as a seatless member, which over-flagged its column. The harness was then corrected to seat the MD as the active writer it actually is (scripts/qa-sweep/inventory-sweep.ts). The delivered Excel still shows the old md results; re-running reclassifies the md-artifact flags down to the real findings, which were already fixed in PR A (#1441). Only worth doing if the sheet gets filed or shared externally.</t>
-        </is>
-      </c>
-      <c r="G13" s="3" t="inlineStr">
-        <is>
-          <t>this session, QA sweep (2026-10-03 to 2026-10-04).</t>
-        </is>
-      </c>
-      <c r="H13" s="3" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:H13"/>
+  <autoFilter ref="A1:H12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1093,7 +1054,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H59"/>
+  <dimension ref="A1:H60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1151,24 +1112,24 @@
     <row r="2" ht="90" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>C58</t>
+          <t>C59</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>VeritaDC per-document attestation tracker + "My Documents" rename (built as #45)</t>
+          <t>Confirm the finding-closure signer policy (was #43)</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr"/>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>was M / Importance: Medium-High</t>
+          <t>was XS / Importance: Medium</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Effort: was M / Importance: Medium-High</t>
+          <t>Effort: was XS / Importance: Medium</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
@@ -1177,24 +1138,24 @@
     <row r="3" ht="90" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>C57</t>
+          <t>C58</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Hide sections a lab does not use from a master list (was #47)</t>
+          <t>VeritaDC per-document attestation tracker + "My Documents" rename (built as #45)</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr"/>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>was S-M / Importance: Medium-High (prospect-requested)</t>
+          <t>was M / Importance: Medium-High</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Effort: was S-M / Importance: Medium-High (prospect-requested)</t>
+          <t>Effort: was M / Importance: Medium-High</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr"/>
@@ -1203,24 +1164,24 @@
     <row r="4" ht="90" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>C56</t>
+          <t>C57</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>VeritaCEU: curated free continuing-education provider list (was #53)</t>
+          <t>Hide sections a lab does not use from a master list (was #47)</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr"/>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>was S / Importance: Low-Medium</t>
+          <t>was S-M / Importance: Medium-High (prospect-requested)</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Effort: was S / Importance: Low-Medium</t>
+          <t>Effort: was S-M / Importance: Medium-High (prospect-requested)</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr"/>
@@ -1229,24 +1190,24 @@
     <row r="5" ht="90" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>C55</t>
+          <t>C56</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>VeritaScan: let sites add their own custom questions (was #55)</t>
+          <t>VeritaCEU: curated free continuing-education provider list (was #53)</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr"/>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>was M / Importance: Medium-High</t>
+          <t>was S / Importance: Low-Medium</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Effort: was M / Importance: Medium-High</t>
+          <t>Effort: was S / Importance: Low-Medium</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr"/>
@@ -1255,24 +1216,24 @@
     <row r="6" ht="90" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>C54</t>
+          <t>C55</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>VeritaQC: at-entry warning when a QC point is outside 2 SD (was #56)</t>
+          <t>VeritaScan: let sites add their own custom questions (was #55)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr"/>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>was S-M (shipped S) / Importance: High</t>
+          <t>was M / Importance: Medium-High</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Effort: was S-M (shipped S) / Importance: High</t>
+          <t>Effort: was M / Importance: Medium-High</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
@@ -1281,24 +1242,24 @@
     <row r="7" ht="90" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>C53</t>
+          <t>C54</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>VeritaTrack: quarterly task loaded as monthly until re-saved (was #54)</t>
+          <t>VeritaQC: at-entry warning when a QC point is outside 2 SD (was #56)</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr"/>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>was S / Importance: Medium</t>
+          <t>was S-M (shipped S) / Importance: High</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Effort: was S / Importance: Medium</t>
+          <t>Effort: was S-M (shipped S) / Importance: High</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr"/>
@@ -1307,24 +1268,24 @@
     <row r="8" ht="90" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>C52</t>
+          <t>C53</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>VeritaResponse internal NCE / non-conforming event (was #36)</t>
+          <t>VeritaTrack: quarterly task loaded as monthly until re-saved (was #54)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr"/>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>was L (shipped as MEDIUM) / Importance: High</t>
+          <t>was S / Importance: Medium</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Effort: was L (shipped as MEDIUM) / Importance: High</t>
+          <t>Effort: was S / Importance: Medium</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
@@ -1333,24 +1294,24 @@
     <row r="9" ht="90" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>C49</t>
+          <t>C52</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Competency "assessed this cycle" cadence-aware window (was #50)</t>
+          <t>VeritaResponse internal NCE / non-conforming event (was #36)</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr"/>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>was S-M / Importance: Medium</t>
+          <t>was L (shipped as MEDIUM) / Importance: High</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Effort: was S-M / Importance: Medium</t>
+          <t>Effort: was L (shipped as MEDIUM) / Importance: High</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr"/>
@@ -1359,12 +1320,12 @@
     <row r="10" ht="90" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>C50</t>
+          <t>C49</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>VeritaTrack task owner + owner-only reminder routing (was #51)</t>
+          <t>Competency "assessed this cycle" cadence-aware window (was #50)</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr"/>
@@ -1385,24 +1346,24 @@
     <row r="11" ht="90" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>C51</t>
+          <t>C50</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Designate Medical Director by picking a lab member (was #52, core)</t>
+          <t>VeritaTrack task owner + owner-only reminder routing (was #51)</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr"/>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>was S-M / Importance: Medium-High</t>
+          <t>was S-M / Importance: Medium</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Effort: was S-M / Importance: Medium-High</t>
+          <t>Effort: was S-M / Importance: Medium</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr"/>
@@ -1411,24 +1372,24 @@
     <row r="12" ht="90" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>C47</t>
+          <t>C51</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Unregulated-analyte / Alternative Assessment (AAA) coverage (was #18)</t>
+          <t>Designate Medical Director by picking a lab member (was #52, core)</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr"/>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>was S (Phase 3) / Importance: Medium</t>
+          <t>was S-M / Importance: Medium-High</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Effort: was S (Phase 3) / Importance: Medium</t>
+          <t>Effort: was S-M / Importance: Medium-High</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr"/>
@@ -1437,24 +1398,24 @@
     <row r="13" ht="90" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>C48</t>
+          <t>C47</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>VeritaResponse post-survey deficiency module (was #17)</t>
+          <t>Unregulated-analyte / Alternative Assessment (AAA) coverage (was #18)</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr"/>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>was XL / Importance: High</t>
+          <t>was S (Phase 3) / Importance: Medium</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Effort: was XL / Importance: High</t>
+          <t>Effort: was S (Phase 3) / Importance: Medium</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr"/>
@@ -1463,39 +1424,38 @@
     <row r="14" ht="90" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>C45</t>
+          <t>C48</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Unify coverage/competency recurrence helper (was #49) - closed as non-issue</t>
+          <t>VeritaResponse post-survey deficiency module (was #17)</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr"/>
-      <c r="D14" s="2" t="inlineStr"/>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>was XL / Importance: High</t>
+        </is>
+      </c>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: Investigated 2026-09-24 before building. The coverage recurrence math (+6-month interval, signed-resets-to-missing, nextDueOn/overdue, isFailVerdict) is ALREADY single-source in server/veritacheckCoverage.ts (computeCoverageFrom). server/coverageReport.ts and the routes.ts coverage export do not recompute it; they consume the computed nextDueOn/overdue/status fields and apply small surface-specific presentation labels (deliberately different vocabularies per surface, so they should not be merged). The only truly identical duplicate is a one-line date formatter. The competency "owed" derivation is NOT the same cadence: competency follows the CLIA milestone schedule (initial / semiannual year 1 / annual, 42 CFR 493.1451(b)(8) and 493.1235), which is a different regulatory interval from the coverage 6-month rule (493.1281 / 493.1255) and must stay separate. No worthwhile extraction; merging the two cadences would be wrong. Closed 2026-09-24. (The year-1 competency-window refinement remains tracked separately as #50.)</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-24 session, "keep working" pass; scoped read-only, found no real duplication.
----</t>
-        </is>
-      </c>
+          <t>Effort: was XL / Importance: High</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr"/>
       <c r="H14" s="2" t="inlineStr"/>
     </row>
     <row r="15" ht="90" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>C46</t>
+          <t>C45</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Verified-users product-update send path (wrong-list incident fix)</t>
+          <t>Unify coverage/competency recurrence helper (was #49) - closed as non-issue</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr"/>
@@ -1503,12 +1463,12 @@
       <c r="E15" s="3" t="inlineStr"/>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: Shipped PR #1324 (merged 4e05506a, deploy ACTIVE). New POST /api/admin/users/send targets registered VeritaAssure account holders (the users table), never the Lab Director's Briefing subscriber list. Separate explicitly-named endpoint (not a flag with a dangerous default), account-holder email framing, excludes suppressed emails and RFC-reserved test domains, CC owner, dryRun + testTo previews. Public unsubscribe now upserts a suppression row so opt-outs are honored across both audiences. Live dryRun: 49 verified-user recipients vs 673 on the Briefing list. Receipts: scripts/verify-product-update-send.mts 24/24, tsc clean, rendered sample inspected. Fixes the fallout from the 2026-09-23/24 wrong-list send (a product update went to the 675-person Briefing list). Nothing sends without Michael's explicit "send it."</t>
+          <t>Closure evidence: Investigated 2026-09-24 before building. The coverage recurrence math (+6-month interval, signed-resets-to-missing, nextDueOn/overdue, isFailVerdict) is ALREADY single-source in server/veritacheckCoverage.ts (computeCoverageFrom). server/coverageReport.ts and the routes.ts coverage export do not recompute it; they consume the computed nextDueOn/overdue/status fields and apply small surface-specific presentation labels (deliberately different vocabularies per surface, so they should not be merged). The only truly identical duplicate is a one-line date formatter. The competency "owed" derivation is NOT the same cadence: competency follows the CLIA milestone schedule (initial / semiannual year 1 / annual, 42 CFR 493.1451(b)(8) and 493.1235), which is a different regulatory interval from the coverage 6-month rule (493.1281 / 493.1255) and must stay separate. No worthwhile extraction; merging the two cadences would be wrong. Closed 2026-09-24. (The year-1 competency-window refinement remains tracked separately as #50.)</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>2026-09-24 session; Michael selected this as the next build after the #41 close.
+          <t>2026-09-24 session, "keep working" pass; scoped read-only, found no real duplication.
 ---</t>
         </is>
       </c>
@@ -1517,12 +1477,12 @@
     <row r="16" ht="90" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>C44</t>
+          <t>C46</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Verify-script convention backfill (was #41) + audit matcher fix</t>
+          <t>Verified-users product-update send path (wrong-list incident fix)</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr"/>
@@ -1530,12 +1490,12 @@
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: #41 was fully backfilled on 2026-06-13 (all 8 high-stakes scripts landed; see C30); it had only been mis-filed in OPEN. A 2026-09-24 re-audit initially reported 4 of 5 recent math/logic commits as missing a verify script, which was a FALSE POSITIVE: scripts/audit_verify_script_coverage.py matched only scripts/verify-*.js / .cjs, so it ignored the .mjs / .mts / .ts verify scripts the repo now ships (e.g. verify-ptcoag-multi.mts, verify-tea-criterion-format.mjs). Fixed the matcher to accept .js/.cjs/.mjs/.ts/.mts; re-run shows 5 of 5 covered, 0 debt. The convention is being followed. Closed 2026-09-24.</t>
+          <t>Closure evidence: Shipped PR #1324 (merged 4e05506a, deploy ACTIVE). New POST /api/admin/users/send targets registered VeritaAssure account holders (the users table), never the Lab Director's Briefing subscriber list. Separate explicitly-named endpoint (not a flag with a dangerous default), account-holder email framing, excludes suppressed emails and RFC-reserved test domains, CC owner, dryRun + testTo previews. Public unsubscribe now upserts a suppression row so opt-outs are honored across both audiences. Live dryRun: 49 verified-user recipients vs 673 on the Briefing list. Receipts: scripts/verify-product-update-send.mts 24/24, tsc clean, rendered sample inspected. Fixes the fallout from the 2026-09-23/24 wrong-list send (a product update went to the 675-person Briefing list). Nothing sends without Michael's explicit "send it."</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 session, "keep working" pass; audit tooling bug found + fixed.
+          <t>2026-09-24 session; Michael selected this as the next build after the #41 close.
 ---</t>
         </is>
       </c>
@@ -1544,12 +1504,12 @@
     <row r="17" ht="90" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>C43</t>
+          <t>C44</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>VeritaStaff instrument-centric (dual) assignment view</t>
+          <t>Verify-script convention backfill (was #41) + audit matcher fix</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr"/>
@@ -1557,12 +1517,12 @@
       <c r="E17" s="3" t="inlineStr"/>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1320. GET/PUT /staff/instruments/:id/employees (transpose of the per-employee endpoints); an "Assign by Instrument" dialog lets a director pick a test system or manual test and check off who runs it. Same staff_employee_instruments join, with the 42 CFR 493.1235(a) duty-change event emitted on newly-added pairs so both orientations trigger the same reassessment. GET verified live on SCAHC lab 2. Closed 2026-09-24.</t>
+          <t>Closure evidence: #41 was fully backfilled on 2026-06-13 (all 8 high-stakes scripts landed; see C30); it had only been mis-filed in OPEN. A 2026-09-24 re-audit initially reported 4 of 5 recent math/logic commits as missing a verify script, which was a FALSE POSITIVE: scripts/audit_verify_script_coverage.py matched only scripts/verify-*.js / .cjs, so it ignored the .mjs / .mts / .ts verify scripts the repo now ships (e.g. verify-ptcoag-multi.mts, verify-tea-criterion-format.mjs). Fixed the matcher to accept .js/.cjs/.mjs/.ts/.mts; re-run shows 5 of 5 covered, 0 debt. The convention is being followed. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>2026-09-24 session, Michael ("in staff we should also give the dual view when assigning coverage to test systems or manual tests").
+          <t>2026-09-24 session, "keep working" pass; audit tooling bug found + fixed.
 ---</t>
         </is>
       </c>
@@ -1571,12 +1531,12 @@
     <row r="18" ht="90" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>C42</t>
+          <t>C43</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>VeritaComp coverage map (required-vs-assessed matrix, dual view)</t>
+          <t>VeritaStaff instrument-centric (dual) assignment view</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr"/>
@@ -1584,12 +1544,12 @@
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1319 (+ status layer PR #1316). /competency/owed returns per-item assessed (locked passing assessment this cycle on a covering method group) + per-employee CLIA status; CompetencyCoverageMap renders a By-employee / By-instrument matrix (Assessed / Owed / Overdue / Gap). Verified live on SCAHC lab 2 (owed 116, assessed 2, gaps 0). Completes #48 as the VeritaCheck-parity coverage map. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1320. GET/PUT /staff/instruments/:id/employees (transpose of the per-employee endpoints); an "Assign by Instrument" dialog lets a director pick a test system or manual test and check off who runs it. Same staff_employee_instruments join, with the 42 CFR 493.1235(a) duty-change event emitted on newly-added pairs so both orientations trigger the same reassessment. GET verified live on SCAHC lab 2. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 session, Michael ("are we building the competencies to have a coverage map, same as veritacheck?" then "build it").
+          <t>2026-09-24 session, Michael ("in staff we should also give the dual view when assigning coverage to test systems or manual tests").
 ---</t>
         </is>
       </c>
@@ -1598,12 +1558,12 @@
     <row r="19" ht="90" customHeight="1">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>C41</t>
+          <t>C42</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>VeritaCheck coverage recurrence (method comparison + cal-ver/linearity + reports)</t>
+          <t>VeritaComp coverage map (required-vs-assessed matrix, dual view)</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr"/>
@@ -1611,12 +1571,12 @@
       <c r="E19" s="3" t="inlineStr"/>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: PRs #1317 (method comparison), #1318 (cal-ver/linearity), #1321 (report Next-due columns). Periodic verification (correlation/method comparison 42 CFR 493.1281; cal-ver/linearity 42 CFR 493.1255; both 6-month) now recurs: a signed study banks the cycle and rolls to next-due = signed + 6 months instead of reading "done" forever. Status Missing/Failed/Completed-unsigned + a "Next due on" column on-screen and in both coverage exports; also credits the previously-ignored "correlation" study type. Root cause: computeCoverageFrom marked requirements done on mere existence, no date logic. Verified live on SCAHC lab 2 (101 correlations + 11 cal-ver rows now carry a next-due). Engine-level, all facilities. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1319 (+ status layer PR #1316). /competency/owed returns per-item assessed (locked passing assessment this cycle on a covering method group) + per-employee CLIA status; CompetencyCoverageMap renders a By-employee / By-instrument matrix (Assessed / Owed / Overdue / Gap). Verified live on SCAHC lab 2 (owed 116, assessed 2, gaps 0). Completes #48 as the VeritaCheck-parity coverage map. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>2026-09-24 session, Michael ("Look at San Carlos... they finished their last set of correlations (all 103) but their menu never reset").
+          <t>2026-09-24 session, Michael ("are we building the competencies to have a coverage map, same as veritacheck?" then "build it").
 ---</t>
         </is>
       </c>
@@ -1625,12 +1585,12 @@
     <row r="20" ht="90" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>C40</t>
+          <t>C41</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>VeritaComp Competencies Owed derived from VeritaStaff, with gap detection (was #48)</t>
+          <t>VeritaCheck coverage recurrence (method comparison + cal-ver/linearity + reports)</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr"/>
@@ -1638,12 +1598,12 @@
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1314 (squash 2bcb0db9). GET /api/labs/:labId/competency/owed derives each VeritaStaff testing employee's owed competencies from their assigned instruments (staff_employee_instruments -&gt; veritamap_instruments + tests), on the CLIA timeline, and flags instruments not covered by any competency program as gaps. CompetenciesOwedSection renders it on the VeritaComp landing page. Reuses the shipped bridge + suggested-method-groups match rules; no new tables. Verified live on prod with real assignment data: 2 instruments assigned to a demo staffer produced owed=2, gaps=2 (HIGH, Technical Supervisor), then reverted cleanly. Closed 2026-09-24.</t>
+          <t>Closure evidence: PRs #1317 (method comparison), #1318 (cal-ver/linearity), #1321 (report Next-due columns). Periodic verification (correlation/method comparison 42 CFR 493.1281; cal-ver/linearity 42 CFR 493.1255; both 6-month) now recurs: a signed study banks the cycle and rolls to next-due = signed + 6 months instead of reading "done" forever. Status Missing/Failed/Completed-unsigned + a "Next due on" column on-screen and in both coverage exports; also credits the previously-ignored "correlation" study type. Root cause: computeCoverageFrom marked requirements done on mere existence, no date logic. Verified live on SCAHC lab 2 (101 correlations + 11 cal-ver rows now carry a next-due). Engine-level, all facilities. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23/24 session, Michael ("veritacomp bases what competencies they owe (currently untrue, but needs to be true)"). Option 1 (unify roster on VeritaStaff, match instruments by id).
+          <t>2026-09-24 session, Michael ("Look at San Carlos... they finished their last set of correlations (all 103) but their menu never reset").
 ---</t>
         </is>
       </c>
@@ -1652,12 +1612,12 @@
     <row r="21" ht="90" customHeight="1">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>C39</t>
+          <t>C40</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>VeritaScan line items can attach or link evidence (was #46)</t>
+          <t>VeritaComp Competencies Owed derived from VeritaStaff, with gap detection (was #48)</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr"/>
@@ -1665,12 +1625,12 @@
       <c r="E21" s="3" t="inlineStr"/>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1312 (squash a1dda93d). VeritaScan scan checklist items now show linked evidence as chips (open link, remove) plus a writer "Link evidence" affordance whose picker links an existing VeritaDC/Library document; a shortcut deep-links to the Library for new (governed) documents. Reuses the already-shipped lab_documents + document_checklist_links + coverage endpoints (URL-pointer only, no file storage, no new tables). Browser-verified live on prod (scan 23): the affordance renders and the picker opens. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1314 (squash 2bcb0db9). GET /api/labs/:labId/competency/owed derives each VeritaStaff testing employee's owed competencies from their assigned instruments (staff_employee_instruments -&gt; veritamap_instruments + tests), on the CLIA timeline, and flags instruments not covered by any competency program as gaps. CompetenciesOwedSection renders it on the VeritaComp landing page. Reuses the shipped bridge + suggested-method-groups match rules; no new tables. Verified live on prod with real assignment data: 2 instruments assigned to a demo staffer produced owed=2, gaps=2 (HIGH, Technical Supervisor), then reverted cleanly. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>2026-09-23 session, Michael. Recurring request. Companion: cross-module evidence display on the VeritaDC policy shipped in PR #1313 (by-target cross-links surfaced in the policy View modal, browser-verified live).
+          <t>2026-09-23/24 session, Michael ("veritacomp bases what competencies they owe (currently untrue, but needs to be true)"). Option 1 (unify roster on VeritaStaff, match instruments by id).
 ---</t>
         </is>
       </c>
@@ -1679,12 +1639,12 @@
     <row r="22" ht="90" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>C38</t>
+          <t>C39</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>VeritaTrack calendar month cells expand to reveal hidden tasks (was #45)</t>
+          <t>VeritaScan line items can attach or link evidence (was #46)</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr"/>
@@ -1692,12 +1652,12 @@
       <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: VeritaTrack CalendarView month cells with more than three tasks now expand in place (chevron, "+N more" toggling to "Show less", due dates), so no task is hidden with no path to it (client/src/pages/VeritaTrackAppPage.tsx CalendarView). Shipped 2026-09-23. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1312 (squash a1dda93d). VeritaScan scan checklist items now show linked evidence as chips (open link, remove) plus a writer "Link evidence" affordance whose picker links an existing VeritaDC/Library document; a shortcut deep-links to the Library for new (governed) documents. Reuses the already-shipped lab_documents + document_checklist_links + coverage endpoints (URL-pointer only, no file storage, no new tables). Browser-verified live on prod (scan 23): the affordance renders and the picker opens. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23 session, Michael screenshot of the VeritaTrack calendar (lab 3, September cell).
+          <t>2026-09-23 session, Michael. Recurring request. Companion: cross-module evidence display on the VeritaDC policy shipped in PR #1313 (by-target cross-links surfaced in the policy View modal, browser-verified live).
 ---</t>
         </is>
       </c>
@@ -1706,12 +1666,12 @@
     <row r="23" ht="90" customHeight="1">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>C37</t>
+          <t>C38</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Long Excel column headers no longer clip CFR citations (was #44)</t>
+          <t>VeritaTrack calendar month cells expand to reveal hidden tasks (was #45)</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr"/>
@@ -1719,12 +1679,12 @@
       <c r="E23" s="3" t="inlineStr"/>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. The VeritaMap export derives the header row height from the longest wrapped header via headerRowHeight(headers, colWidths) (server/routes.ts:15935) instead of a fixed 20, so "Reference Range Attestation (42 CFR 493.1253)" and the other long headers print in full. No new code this session. Closed 2026-09-24.</t>
+          <t>Closure evidence: VeritaTrack CalendarView month cells with more than three tasks now expand in place (chevron, "+N more" toggling to "Show less", due dates), so no task is hidden with no path to it (client/src/pages/VeritaTrackAppPage.tsx CalendarView). Shipped 2026-09-23. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+          <t>2026-09-23 session, Michael screenshot of the VeritaTrack calendar (lab 3, September cell).
 ---</t>
         </is>
       </c>
@@ -1733,12 +1693,12 @@
     <row r="24" ht="90" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>C36</t>
+          <t>C37</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>License stamp no longer clobbers the §6 header/footer or names the wrong lab (was #43)</t>
+          <t>Long Excel column headers no longer clip CFR citations (was #44)</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr"/>
@@ -1746,7 +1706,7 @@
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. setHeaderFooter (shared/licenseExceljs.ts:155-209) now preserves an existing §6 header and appends (not overwrites) the footer left section, and customer-facing exports name the scoped lab: the VeritaScan library export reads req.scope.lab.name / clia_number (server/routes.ts:16572-16573), not the licensee. No new code this session (avoided regressing the existing fix). Closed 2026-09-24.</t>
+          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. The VeritaMap export derives the header row height from the longest wrapped header via headerRowHeight(headers, colWidths) (server/routes.ts:15935) instead of a fixed 20, so "Reference Range Attestation (42 CFR 493.1253)" and the other long headers print in full. No new code this session. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -1760,18 +1720,45 @@
     <row r="25" ht="90" customHeight="1">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>C34</t>
+          <t>C36</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>Wire the two static-audit guards into CI (was #43)</t>
+          <t>License stamp no longer clobbers the §6 header/footer or names the wrong lab (was #43)</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr"/>
       <c r="D25" s="3" t="inlineStr"/>
       <c r="E25" s="3" t="inlineStr"/>
       <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. setHeaderFooter (shared/licenseExceljs.ts:155-209) now preserves an existing §6 header and appends (not overwrites) the footer left section, and customer-facing exports name the scoped lab: the VeritaScan library export reads req.scope.lab.name / clia_number (server/routes.ts:16572-16573), not the licensee. No new code this session (avoided regressing the existing fix). Closed 2026-09-24.</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+---</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26" ht="90" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>C34</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Wire the two static-audit guards into CI (was #43)</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr"/>
+      <c r="D26" s="2" t="inlineStr"/>
+      <c r="E26" s="2" t="inlineStr"/>
+      <c r="F26" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: both guards wired into the Multi-Lab Mutations Audit CI
 workflow (.github/workflows/multilab-mutations-audit.yml) as steps:
@@ -1783,24 +1770,24 @@
 (same caveat as the existing guards already in that workflow).</t>
         </is>
       </c>
-      <c r="G25" s="3" t="inlineStr"/>
-      <c r="H25" s="3" t="inlineStr"/>
-    </row>
-    <row r="26" ht="90" customHeight="1">
-      <c r="A26" s="2" t="inlineStr">
+      <c r="G26" s="2" t="inlineStr"/>
+      <c r="H26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27" ht="90" customHeight="1">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>C35</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="B27" s="3" t="inlineStr">
         <is>
           <t>Legacy /api/studies over-returns studies across labs (was #44)</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr"/>
-      <c r="D26" s="2" t="inlineStr"/>
-      <c r="E26" s="2" t="inlineStr"/>
-      <c r="F26" s="2" t="inlineStr">
+      <c r="C27" s="3" t="inlineStr"/>
+      <c r="D27" s="3" t="inlineStr"/>
+      <c r="E27" s="3" t="inlineStr"/>
+      <c r="F27" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: GET /api/studies now scopes its list to the active lab
 when one is resolved from the Referer (server/routes.ts), so every returned row
@@ -1810,24 +1797,24 @@
 mirroring the /api/labs/:labId/studies handler. Closed 2026-06-14.</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr"/>
-      <c r="H26" s="2" t="inlineStr"/>
-    </row>
-    <row r="27" ht="90" customHeight="1">
-      <c r="A27" s="3" t="inlineStr">
+      <c r="G27" s="3" t="inlineStr"/>
+      <c r="H27" s="3" t="inlineStr"/>
+    </row>
+    <row r="28" ht="90" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>C30</t>
         </is>
       </c>
-      <c r="B27" s="3" t="inlineStr">
+      <c r="B28" s="2" t="inlineStr">
         <is>
           <t>Verify-script convention backfill (was #41)</t>
         </is>
       </c>
-      <c r="C27" s="3" t="inlineStr"/>
-      <c r="D27" s="3" t="inlineStr"/>
-      <c r="E27" s="3" t="inlineStr"/>
-      <c r="F27" s="3" t="inlineStr">
+      <c r="C28" s="2" t="inlineStr"/>
+      <c r="D28" s="2" t="inlineStr"/>
+      <c r="E28" s="2" t="inlineStr"/>
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: all 8 high-stakes math/logic commits now ship a paired
 scripts/verify-*.js (EP17 sensitivity, Deming lot-to-lot, CUMSUM+QC+multi-analyte,
@@ -1835,30 +1822,30 @@
 TEa boundary), per the strike-throughs in #41. Closed 2026-06-13.</t>
         </is>
       </c>
-      <c r="G27" s="3" t="inlineStr">
+      <c r="G28" s="2" t="inlineStr">
         <is>
           <t>scripts/audit_verify_script_coverage.py lookback, 2026-06-02; backfills
 landed 2026-06-03..06.
 ---</t>
         </is>
       </c>
-      <c r="H27" s="3" t="inlineStr"/>
-    </row>
-    <row r="28" ht="90" customHeight="1">
-      <c r="A28" s="2" t="inlineStr">
+      <c r="H28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29" ht="90" customHeight="1">
+      <c r="A29" s="3" t="inlineStr">
         <is>
           <t>C31</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="B29" s="3" t="inlineStr">
         <is>
           <t>VeritaPT AAA create/update/delete silently no-op in the multi-lab UI</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr"/>
-      <c r="D28" s="2" t="inlineStr"/>
-      <c r="E28" s="2" t="inlineStr"/>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="C29" s="3" t="inlineStr"/>
+      <c r="D29" s="3" t="inlineStr"/>
+      <c r="E29" s="3" t="inlineStr"/>
+      <c r="F29" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #754 (commit 92ad499) added lab-scoped POST/PUT/DELETE
 /api/labs/:labId/pt/aa-records. The UI posted to the lab-scoped path but only GET
@@ -1869,30 +1856,30 @@
 route mis-filed records to the user's default lab on multi-lab accounts).</t>
         </is>
       </c>
-      <c r="G28" s="2" t="inlineStr">
+      <c r="G29" s="3" t="inlineStr">
         <is>
           <t>2026-06-13, found during #18 Phase 3 QA;
 scripts/audit-labscoped-write-routes.mjs now guards the class.
 ---</t>
         </is>
       </c>
-      <c r="H28" s="2" t="inlineStr"/>
-    </row>
-    <row r="29" ht="90" customHeight="1">
-      <c r="A29" s="3" t="inlineStr">
+      <c r="H29" s="3" t="inlineStr"/>
+    </row>
+    <row r="30" ht="90" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>C32</t>
         </is>
       </c>
-      <c r="B29" s="3" t="inlineStr">
+      <c r="B30" s="2" t="inlineStr">
         <is>
           <t>VeritaComp "Unlock assessment" false-success no-op</t>
         </is>
       </c>
-      <c r="C29" s="3" t="inlineStr"/>
-      <c r="D29" s="3" t="inlineStr"/>
-      <c r="E29" s="3" t="inlineStr"/>
-      <c r="F29" s="3" t="inlineStr">
+      <c r="C30" s="2" t="inlineStr"/>
+      <c r="D30" s="2" t="inlineStr"/>
+      <c r="E30" s="2" t="inlineStr"/>
+      <c r="F30" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #755 (commit 4234007) moved the unlock route to
 /api/labs/:labId/competency/assessments/:id/unlock (the path the client calls).
@@ -1903,29 +1890,29 @@
 HTML).</t>
         </is>
       </c>
-      <c r="G29" s="3" t="inlineStr">
+      <c r="G30" s="2" t="inlineStr">
         <is>
           <t>2026-06-13, found by scripts/audit-labscoped-write-routes.mjs.
 ---</t>
         </is>
       </c>
-      <c r="H29" s="3" t="inlineStr"/>
-    </row>
-    <row r="30" ht="90" customHeight="1">
-      <c r="A30" s="2" t="inlineStr">
+      <c r="H30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31" ht="90" customHeight="1">
+      <c r="A31" s="3" t="inlineStr">
         <is>
           <t>C33</t>
         </is>
       </c>
-      <c r="B30" s="2" t="inlineStr">
+      <c r="B31" s="3" t="inlineStr">
         <is>
           <t>FK-cascade delete 500s + NavBar laptop-width overflow</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr"/>
-      <c r="D30" s="2" t="inlineStr"/>
-      <c r="E30" s="2" t="inlineStr"/>
-      <c r="F30" s="2" t="inlineStr">
+      <c r="C31" s="3" t="inlineStr"/>
+      <c r="D31" s="3" t="inlineStr"/>
+      <c r="E31" s="3" t="inlineStr"/>
+      <c r="F31" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PRs #749/#750 fixed NavBar horizontal overflow at laptop
 widths (collapse to the hamburger below 1560px); prod-verified at 1280-1920 with the
@@ -1936,37 +1923,9 @@
 500 -&gt; 200. scripts/audit-delete-cascades.mjs guards the class.</t>
         </is>
       </c>
-      <c r="G30" s="2" t="inlineStr">
+      <c r="G31" s="3" t="inlineStr">
         <is>
           <t>2026-06-13 browser QA of the A7-D4 wave + retro-QC of the 72h PR window.
----</t>
-        </is>
-      </c>
-      <c r="H30" s="2" t="inlineStr"/>
-    </row>
-    <row r="31" ht="90" customHeight="1">
-      <c r="A31" s="3" t="inlineStr">
-        <is>
-          <t>C1</t>
-        </is>
-      </c>
-      <c r="B31" s="3" t="inlineStr">
-        <is>
-          <t>FAQ "over 25 years" -&gt; "over 23 years"</t>
-        </is>
-      </c>
-      <c r="C31" s="3" t="inlineStr"/>
-      <c r="D31" s="3" t="inlineStr"/>
-      <c r="E31" s="3" t="inlineStr"/>
-      <c r="F31" s="3" t="inlineStr">
-        <is>
-          <t>Closure evidence: client/src/pages/FAQPage.tsx line 20 reads "over
-23 years" as of 2026-05-01.</t>
-        </is>
-      </c>
-      <c r="G31" s="3" t="inlineStr">
-        <is>
-          <t>session 299e9a73 turn 14, ~2026-04-28.
 ---</t>
         </is>
       </c>
@@ -1975,18 +1934,46 @@
     <row r="32" ht="90" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>C5</t>
+          <t>C1</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>David's VeritaQA grey-button bug (seat permissions mode)</t>
+          <t>FAQ "over 25 years" -&gt; "over 23 years"</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr"/>
       <c r="D32" s="2" t="inlineStr"/>
       <c r="E32" s="2" t="inlineStr"/>
       <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Closure evidence: client/src/pages/FAQPage.tsx line 20 reads "over
+23 years" as of 2026-05-01.</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>session 299e9a73 turn 14, ~2026-04-28.
+---</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33" ht="90" customHeight="1">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>David's VeritaQA grey-button bug (seat permissions mode)</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr"/>
+      <c r="D33" s="3" t="inlineStr"/>
+      <c r="E33" s="3" t="inlineStr"/>
+      <c r="F33" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #10 squash-merged as commit a43fbba on
 2026-05-01 23:19 MST. Railway deploy succeeded; deployed bundle
@@ -1999,7 +1986,7 @@
 against his exact stored shape (14 of 14 expected outcomes matched).</t>
         </is>
       </c>
-      <c r="G32" s="2" t="inlineStr">
+      <c r="G33" s="3" t="inlineStr">
         <is>
           <t>2026-05-01 David's report; veritabench + veritastock
 weren't in MODULE_LIST so seat permissions silently defaulted to
@@ -2007,46 +1994,17 @@
 ---</t>
         </is>
       </c>
-      <c r="H32" s="2" t="inlineStr"/>
-    </row>
-    <row r="33" ht="90" customHeight="1">
-      <c r="A33" s="3" t="inlineStr">
-        <is>
-          <t>C2</t>
-        </is>
-      </c>
-      <c r="B33" s="3" t="inlineStr">
-        <is>
-          <t>TeamPage present-tense "TJC surveyor" check</t>
-        </is>
-      </c>
-      <c r="C33" s="3" t="inlineStr"/>
-      <c r="D33" s="3" t="inlineStr"/>
-      <c r="E33" s="3" t="inlineStr"/>
-      <c r="F33" s="3" t="inlineStr">
-        <is>
-          <t>Closure evidence: site-wide search confirmed all surveyor language
-is past-tense, consistent with user's 2021-2025 service. User closed
-the item in session 299e9a73 turn 4.</t>
-        </is>
-      </c>
-      <c r="G33" s="3" t="inlineStr">
-        <is>
-          <t>session 299e9a73, ~2026-04-28.
----</t>
-        </is>
-      </c>
       <c r="H33" s="3" t="inlineStr"/>
     </row>
     <row r="34" ht="90" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>C3</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>My Studies CSV/XLSX export (John as design partner)</t>
+          <t>TeamPage present-tense "TJC surveyor" check</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr"/>
@@ -2054,14 +2012,14 @@
       <c r="E34" s="2" t="inlineStr"/>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: client/src/pages/DashboardPage.tsx line 46 calls
-/api/my-studies/export. server/routes.ts line 1491 implements the
-endpoint. Pulled forward into pre-COLA per user instruction.</t>
+          <t>Closure evidence: site-wide search confirmed all surveyor language
+is past-tense, consistent with user's 2021-2025 service. User closed
+the item in session 299e9a73 turn 4.</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>session 299e9a73 turn 5, ~2026-04-28.
+          <t>session 299e9a73, ~2026-04-28.
 ---</t>
         </is>
       </c>
@@ -2070,12 +2028,12 @@
     <row r="35" ht="90" customHeight="1">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>C4</t>
+          <t>C3</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>Rotate GitHub PAT (because old PAT was committed in SESSION_HANDOFF files)</t>
+          <t>My Studies CSV/XLSX export (John as design partner)</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr"/>
@@ -2083,13 +2041,14 @@
       <c r="E35" s="3" t="inlineStr"/>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: no ghp_* or github_pat_* patterns in current
-SESSION_HANDOFF.md or SESSION_HANDOFF-2.md as of 2026-05-01.</t>
+          <t>Closure evidence: client/src/pages/DashboardPage.tsx line 46 calls
+/api/my-studies/export. server/routes.ts line 1491 implements the
+endpoint. Pulled forward into pre-COLA per user instruction.</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>session 299e9a73, ~2026-04-28.
+          <t>session 299e9a73 turn 5, ~2026-04-28.
 ---</t>
         </is>
       </c>
@@ -2098,18 +2057,46 @@
     <row r="36" ht="90" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>C6</t>
+          <t>C4</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>VeritaPolicy service-line filtering removed (formerly #4)</t>
+          <t>Rotate GitHub PAT (because old PAT was committed in SESSION_HANDOFF files)</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr"/>
       <c r="D36" s="2" t="inlineStr"/>
       <c r="E36" s="2" t="inlineStr"/>
       <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Closure evidence: no ghp_* or github_pat_* patterns in current
+SESSION_HANDOFF.md or SESSION_HANDOFF-2.md as of 2026-05-01.</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>session 299e9a73, ~2026-04-28.
+---</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr"/>
+    </row>
+    <row r="37" ht="90" customHeight="1">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>C6</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>VeritaPolicy service-line filtering removed (formerly #4)</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr"/>
+      <c r="D37" s="3" t="inlineStr"/>
+      <c r="E37" s="3" t="inlineStr"/>
+      <c r="F37" s="3" t="inlineStr">
         <is>
           <t>Closure rationale (operator decision 2026-05-10): Keep all
 VeritaPolicy rows. CFR-only references with no accreditor reference
@@ -2118,29 +2105,29 @@
 report misread the design intent.</t>
         </is>
       </c>
-      <c r="G36" s="2" t="inlineStr">
+      <c r="G37" s="3" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H36" s="2" t="inlineStr"/>
-    </row>
-    <row r="37" ht="90" customHeight="1">
-      <c r="A37" s="3" t="inlineStr">
+      <c r="H37" s="3" t="inlineStr"/>
+    </row>
+    <row r="38" ht="90" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
         <is>
           <t>C7</t>
         </is>
       </c>
-      <c r="B37" s="3" t="inlineStr">
+      <c r="B38" s="2" t="inlineStr">
         <is>
           <t>CLIA number format validation (formerly #13)</t>
         </is>
       </c>
-      <c r="C37" s="3" t="inlineStr"/>
-      <c r="D37" s="3" t="inlineStr"/>
-      <c r="E37" s="3" t="inlineStr"/>
-      <c r="F37" s="3" t="inlineStr">
+      <c r="C38" s="2" t="inlineStr"/>
+      <c r="D38" s="2" t="inlineStr"/>
+      <c r="E38" s="2" t="inlineStr"/>
+      <c r="F38" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: shared/validateClia.ts defines CLIA_REGEX =
 /^\d{2}D\d{7}$/ (line 24), validateClia() helper with whitespace
@@ -2151,30 +2138,30 @@
 shape exists and behaves as specified.</t>
         </is>
       </c>
-      <c r="G37" s="3" t="inlineStr">
+      <c r="G38" s="2" t="inlineStr">
         <is>
           <t>Agent verification 2026-05-10 via grep + file read.
 Operator confirmed shipped 2026-05-10.
 ---</t>
         </is>
       </c>
-      <c r="H37" s="3" t="inlineStr"/>
-    </row>
-    <row r="38" ht="90" customHeight="1">
-      <c r="A38" s="2" t="inlineStr">
+      <c r="H38" s="2" t="inlineStr"/>
+    </row>
+    <row r="39" ht="90" customHeight="1">
+      <c r="A39" s="3" t="inlineStr">
         <is>
           <t>C8</t>
         </is>
       </c>
-      <c r="B38" s="2" t="inlineStr">
+      <c r="B39" s="3" t="inlineStr">
         <is>
           <t>VeritaMap lab-wide menu toggle (formerly #19)</t>
         </is>
       </c>
-      <c r="C38" s="2" t="inlineStr"/>
-      <c r="D38" s="2" t="inlineStr"/>
-      <c r="E38" s="2" t="inlineStr"/>
-      <c r="F38" s="2" t="inlineStr">
+      <c r="C39" s="3" t="inlineStr"/>
+      <c r="D39" s="3" t="inlineStr"/>
+      <c r="E39" s="3" t="inlineStr"/>
+      <c r="F39" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: client/src/pages/VeritaMapLabwidePage.tsx
 exists and implements the labwide read-only union view. Route is
@@ -2184,59 +2171,59 @@
 parking lot plan (read-only union view, per-session toggle) shipped.</t>
         </is>
       </c>
-      <c r="G38" s="2" t="inlineStr">
+      <c r="G39" s="3" t="inlineStr">
         <is>
           <t>Agent verification 2026-05-10 via grep + file read.
 Operator confirmed shipped 2026-05-10.
 ---</t>
         </is>
       </c>
-      <c r="H38" s="2" t="inlineStr"/>
-    </row>
-    <row r="39" ht="90" customHeight="1">
-      <c r="A39" s="3" t="inlineStr">
-        <is>
-          <t>C9</t>
-        </is>
-      </c>
-      <c r="B39" s="3" t="inlineStr">
-        <is>
-          <t>Tier-1 smoke test checklist (formerly #6)</t>
-        </is>
-      </c>
-      <c r="C39" s="3" t="inlineStr"/>
-      <c r="D39" s="3" t="inlineStr"/>
-      <c r="E39" s="3" t="inlineStr"/>
-      <c r="F39" s="3" t="inlineStr">
-        <is>
-          <t>Closure evidence: docs/smoke-test-tier1.md documents the Tier-1
-smoke-test process and post-deploy verification steps. Shipped via
-PR #81 as part of the 2026-05-10 wave.</t>
-        </is>
-      </c>
-      <c r="G39" s="3" t="inlineStr">
-        <is>
-          <t>Operator instruction 2026-05-10 in this session.
----</t>
-        </is>
-      </c>
       <c r="H39" s="3" t="inlineStr"/>
     </row>
     <row r="40" ht="90" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>C10</t>
+          <t>C9</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Per-module gating (formerly #7)</t>
+          <t>Tier-1 smoke test checklist (formerly #6)</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr"/>
       <c r="D40" s="2" t="inlineStr"/>
       <c r="E40" s="2" t="inlineStr"/>
       <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>Closure evidence: docs/smoke-test-tier1.md documents the Tier-1
+smoke-test process and post-deploy verification steps. Shipped via
+PR #81 as part of the 2026-05-10 wave.</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>Operator instruction 2026-05-10 in this session.
+---</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr"/>
+    </row>
+    <row r="41" ht="90" customHeight="1">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>C10</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>Per-module gating (formerly #7)</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr"/>
+      <c r="D41" s="3" t="inlineStr"/>
+      <c r="E41" s="3" t="inlineStr"/>
+      <c r="F41" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: Client-side useIsReadOnly module keys wired
 on client/src/pages/VeritaPolicyAppPage.tsx and
@@ -2251,29 +2238,29 @@
 PR #76.</t>
         </is>
       </c>
-      <c r="G40" s="2" t="inlineStr">
+      <c r="G41" s="3" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H40" s="2" t="inlineStr"/>
-    </row>
-    <row r="41" ht="90" customHeight="1">
-      <c r="A41" s="3" t="inlineStr">
+      <c r="H41" s="3" t="inlineStr"/>
+    </row>
+    <row r="42" ht="90" customHeight="1">
+      <c r="A42" s="2" t="inlineStr">
         <is>
           <t>C11</t>
         </is>
       </c>
-      <c r="B41" s="3" t="inlineStr">
+      <c r="B42" s="2" t="inlineStr">
         <is>
           <t>VeritaStock shipped copy (formerly #8)</t>
         </is>
       </c>
-      <c r="C41" s="3" t="inlineStr"/>
-      <c r="D41" s="3" t="inlineStr"/>
-      <c r="E41" s="3" t="inlineStr"/>
-      <c r="F41" s="3" t="inlineStr">
+      <c r="C42" s="2" t="inlineStr"/>
+      <c r="D42" s="2" t="inlineStr"/>
+      <c r="E42" s="2" t="inlineStr"/>
+      <c r="F42" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: client/src/pages/ArticleInventoryManagementPage.tsx
 line 305 footer reads "platform that includes VeritaStock™" instead
@@ -2281,29 +2268,29 @@
 on /resources/laboratory-inventory-management. Shipped via PR #75.</t>
         </is>
       </c>
-      <c r="G41" s="3" t="inlineStr">
+      <c r="G42" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H41" s="3" t="inlineStr"/>
-    </row>
-    <row r="42" ht="90" customHeight="1">
-      <c r="A42" s="2" t="inlineStr">
+      <c r="H42" s="2" t="inlineStr"/>
+    </row>
+    <row r="43" ht="90" customHeight="1">
+      <c r="A43" s="3" t="inlineStr">
         <is>
           <t>C12</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
+      <c r="B43" s="3" t="inlineStr">
         <is>
           <t>Admin report one-row-per-lab (formerly #14)</t>
         </is>
       </c>
-      <c r="C42" s="2" t="inlineStr"/>
-      <c r="D42" s="2" t="inlineStr"/>
-      <c r="E42" s="2" t="inlineStr"/>
-      <c r="F42" s="2" t="inlineStr">
+      <c r="C43" s="3" t="inlineStr"/>
+      <c r="D43" s="3" t="inlineStr"/>
+      <c r="E43" s="3" t="inlineStr"/>
+      <c r="F43" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: /api/admin/report rewritten in
 server/routes.ts (~line 595) to LEFT JOIN labs on
@@ -2318,33 +2305,6 @@
 prerequisite, not a code bug). Shipped via PR #85.</t>
         </is>
       </c>
-      <c r="G42" s="2" t="inlineStr">
-        <is>
-          <t>Operator instruction 2026-05-10 in this session.
----</t>
-        </is>
-      </c>
-      <c r="H42" s="2" t="inlineStr"/>
-    </row>
-    <row r="43" ht="90" customHeight="1">
-      <c r="A43" s="3" t="inlineStr">
-        <is>
-          <t>C14</t>
-        </is>
-      </c>
-      <c r="B43" s="3" t="inlineStr">
-        <is>
-          <t>UI relabel "CLIA TEa" -&gt; "Lab-Set Internal Goal" (formerly #1)</t>
-        </is>
-      </c>
-      <c r="C43" s="3" t="inlineStr"/>
-      <c r="D43" s="3" t="inlineStr"/>
-      <c r="E43" s="3" t="inlineStr"/>
-      <c r="F43" s="3" t="inlineStr">
-        <is>
-          <t>Closure evidence: Shipped across four PRs over 2026-05-10.</t>
-        </is>
-      </c>
       <c r="G43" s="3" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
@@ -2356,18 +2316,45 @@
     <row r="44" ht="90" customHeight="1">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>C13</t>
+          <t>C14</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>WSLH PT vendor (formerly #15)</t>
+          <t>UI relabel "CLIA TEa" -&gt; "Lab-Set Internal Goal" (formerly #1)</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr"/>
       <c r="D44" s="2" t="inlineStr"/>
       <c r="E44" s="2" t="inlineStr"/>
       <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>Closure evidence: Shipped across four PRs over 2026-05-10.</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>Operator instruction 2026-05-10 in this session.
+---</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr"/>
+    </row>
+    <row r="45" ht="90" customHeight="1">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>C13</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>WSLH PT vendor (formerly #15)</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr"/>
+      <c r="D45" s="3" t="inlineStr"/>
+      <c r="E45" s="3" t="inlineStr"/>
+      <c r="F45" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: Shipped 2026-05-10 via PR #79 (merge commit
 eeebc6e; merged after rebase to resolve a server/db.ts collision
@@ -2385,38 +2372,9 @@
 'WSLH' is the post-deploy success signal. Shipped via PR #79.</t>
         </is>
       </c>
-      <c r="G44" s="2" t="inlineStr">
+      <c r="G45" s="3" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
----</t>
-        </is>
-      </c>
-      <c r="H44" s="2" t="inlineStr"/>
-    </row>
-    <row r="45" ht="90" customHeight="1">
-      <c r="A45" s="3" t="inlineStr">
-        <is>
-          <t>C15</t>
-        </is>
-      </c>
-      <c r="B45" s="3" t="inlineStr">
-        <is>
-          <t>VeritaStock lot tracking + expiration + reorder alerts (formerly #21)</t>
-        </is>
-      </c>
-      <c r="C45" s="3" t="inlineStr"/>
-      <c r="D45" s="3" t="inlineStr"/>
-      <c r="E45" s="3" t="inlineStr"/>
-      <c r="F45" s="3" t="inlineStr">
-        <is>
-          <t>Closure evidence: VeritaStock™ shipped the bench-level inventory
-features the Perplexity competitor analysis identified as a gap:</t>
-        </is>
-      </c>
-      <c r="G45" s="3" t="inlineStr">
-        <is>
-          <t>Originally Perplexity competitor analysis 2026-05-10.
-Audit 2026-05-21 confirmed the feature set ships today.
 ---</t>
         </is>
       </c>
@@ -2425,12 +2383,12 @@
     <row r="46" ht="90" customHeight="1">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>C16</t>
+          <t>C15</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>PAL studies guided workflow (formerly #23)</t>
+          <t>VeritaStock lot tracking + expiration + reorder alerts (formerly #21)</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr"/>
@@ -2438,15 +2396,14 @@
       <c r="E46" s="2" t="inlineStr"/>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: VeritaCheck™ already ships the Precision /
-Accuracy / Linearity (PAL) study set under EP-protocol naming:</t>
+          <t>Closure evidence: VeritaStock™ shipped the bench-level inventory
+features the Perplexity competitor analysis identified as a gap:</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
           <t>Originally Perplexity competitor analysis 2026-05-10.
-Audit 2026-05-21 confirmed the EP studies cover the PAL framing in
-full.
+Audit 2026-05-21 confirmed the feature set ships today.
 ---</t>
         </is>
       </c>
@@ -2455,12 +2412,12 @@
     <row r="47" ht="90" customHeight="1">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>C17</t>
+          <t>C16</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>Source-grounded 21/29/45 CFR + 42 CFR 482-485 (formerly #26)</t>
+          <t>PAL studies guided workflow (formerly #23)</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr"/>
@@ -2468,35 +2425,65 @@
       <c r="E47" s="3" t="inlineStr"/>
       <c r="F47" s="3" t="inlineStr">
         <is>
+          <t>Closure evidence: VeritaCheck™ already ships the Precision /
+Accuracy / Linearity (PAL) study set under EP-protocol naming:</t>
+        </is>
+      </c>
+      <c r="G47" s="3" t="inlineStr">
+        <is>
+          <t>Originally Perplexity competitor analysis 2026-05-10.
+Audit 2026-05-21 confirmed the EP studies cover the PAL framing in
+full.
+---</t>
+        </is>
+      </c>
+      <c r="H47" s="3" t="inlineStr"/>
+    </row>
+    <row r="48" ht="90" customHeight="1">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>C17</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Source-grounded 21/29/45 CFR + 42 CFR 482-485 (formerly #26)</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr"/>
+      <c r="D48" s="2" t="inlineStr"/>
+      <c r="E48" s="2" t="inlineStr"/>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
           <t>Closure evidence: PR #301 (commit 8c27806, merged 2026-05-21)
 source-grounded the 74 remaining non-493 entries in
 server/cfrRequirements.ts against verbatim eCFR XML. Breakdown
 shipped:</t>
         </is>
       </c>
-      <c r="G47" s="3" t="inlineStr">
+      <c r="G48" s="2" t="inlineStr">
         <is>
           <t>PR #301; tasks #18 in the in-session task tracker.
 ---</t>
         </is>
       </c>
-      <c r="H47" s="3" t="inlineStr"/>
-    </row>
-    <row r="48" ht="90" customHeight="1">
-      <c r="A48" s="2" t="inlineStr">
+      <c r="H48" s="2" t="inlineStr"/>
+    </row>
+    <row r="49" ht="90" customHeight="1">
+      <c r="A49" s="3" t="inlineStr">
         <is>
           <t>C18</t>
         </is>
       </c>
-      <c r="B48" s="2" t="inlineStr">
+      <c r="B49" s="3" t="inlineStr">
         <is>
           <t>VeritaPolicy "Non CLIA" chapter rename (formerly #3)</t>
         </is>
       </c>
-      <c r="C48" s="2" t="inlineStr"/>
-      <c r="D48" s="2" t="inlineStr"/>
-      <c r="E48" s="2" t="inlineStr"/>
-      <c r="F48" s="2" t="inlineStr">
+      <c r="C49" s="3" t="inlineStr"/>
+      <c r="D49" s="3" t="inlineStr"/>
+      <c r="E49" s="3" t="inlineStr"/>
+      <c r="F49" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #300 (commit 34d7707, merged 2026-05-21)
 renamed all 44 user-facing chapter labels in
@@ -2507,7 +2494,7 @@
 page.</t>
         </is>
       </c>
-      <c r="G48" s="2" t="inlineStr">
+      <c r="G49" s="3" t="inlineStr">
         <is>
           <t>CAP customer screenshot of the /veritapolicy chapter
 headers, 2026-05-01 evening. PR #300; tasks #17 in the in-session
@@ -2515,23 +2502,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H48" s="2" t="inlineStr"/>
-    </row>
-    <row r="49" ht="90" customHeight="1">
-      <c r="A49" s="3" t="inlineStr">
+      <c r="H49" s="3" t="inlineStr"/>
+    </row>
+    <row r="50" ht="90" customHeight="1">
+      <c r="A50" s="2" t="inlineStr">
         <is>
           <t>C19</t>
         </is>
       </c>
-      <c r="B49" s="3" t="inlineStr">
+      <c r="B50" s="2" t="inlineStr">
         <is>
           <t>VeritaStock department-scope toggle (formerly #31)</t>
         </is>
       </c>
-      <c r="C49" s="3" t="inlineStr"/>
-      <c r="D49" s="3" t="inlineStr"/>
-      <c r="E49" s="3" t="inlineStr"/>
-      <c r="F49" s="3" t="inlineStr">
+      <c r="C50" s="2" t="inlineStr"/>
+      <c r="D50" s="2" t="inlineStr"/>
+      <c r="E50" s="2" t="inlineStr"/>
+      <c r="F50" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #319 (commit d01f5fe, merged 2026-05-22)
 shipped the persistent dept-scope toggle on VeritaStockPage. A new
@@ -2542,7 +2529,7 @@
 workspace without re-filtering.</t>
         </is>
       </c>
-      <c r="G49" s="3" t="inlineStr">
+      <c r="G50" s="2" t="inlineStr">
         <is>
           <t>John, San Carlos lab, 2026-05-21. Same conversation that
 drove the vendor dropdown (PR #304), FILTERED VIEW banner (PR #305),
@@ -2550,23 +2537,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H49" s="3" t="inlineStr"/>
-    </row>
-    <row r="50" ht="90" customHeight="1">
-      <c r="A50" s="2" t="inlineStr">
+      <c r="H50" s="2" t="inlineStr"/>
+    </row>
+    <row r="51" ht="90" customHeight="1">
+      <c r="A51" s="3" t="inlineStr">
         <is>
           <t>C20</t>
         </is>
       </c>
-      <c r="B50" s="2" t="inlineStr">
+      <c r="B51" s="3" t="inlineStr">
         <is>
           <t>Primary-lab seat counting (formerly #12)</t>
         </is>
       </c>
-      <c r="C50" s="2" t="inlineStr"/>
-      <c r="D50" s="2" t="inlineStr"/>
-      <c r="E50" s="2" t="inlineStr"/>
-      <c r="F50" s="2" t="inlineStr">
+      <c r="C51" s="3" t="inlineStr"/>
+      <c r="D51" s="3" t="inlineStr"/>
+      <c r="E51" s="3" t="inlineStr"/>
+      <c r="F51" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: is_primary_lab INTEGER NOT NULL DEFAULT 0
 column was added to the lab_members table at db.ts:1276, with the
@@ -2577,7 +2564,7 @@
 is_primary_lab=1 ordering).</t>
         </is>
       </c>
-      <c r="G50" s="2" t="inlineStr">
+      <c r="G51" s="3" t="inlineStr">
         <is>
           <t>2026-05-07 multi-lab discussion. Build shipped as part
 of the Multi-Lab Tier 2 architecture work (Phase 3.x series, prior
@@ -2586,23 +2573,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H50" s="2" t="inlineStr"/>
-    </row>
-    <row r="51" ht="90" customHeight="1">
-      <c r="A51" s="3" t="inlineStr">
+      <c r="H51" s="3" t="inlineStr"/>
+    </row>
+    <row r="52" ht="90" customHeight="1">
+      <c r="A52" s="2" t="inlineStr">
         <is>
           <t>C21</t>
         </is>
       </c>
-      <c r="B51" s="3" t="inlineStr">
+      <c r="B52" s="2" t="inlineStr">
         <is>
           <t>Multi-lab pricing model — Option A (formerly #11)</t>
         </is>
       </c>
-      <c r="C51" s="3" t="inlineStr"/>
-      <c r="D51" s="3" t="inlineStr"/>
-      <c r="E51" s="3" t="inlineStr"/>
-      <c r="F51" s="3" t="inlineStr">
+      <c r="C52" s="2" t="inlineStr"/>
+      <c r="D52" s="2" t="inlineStr"/>
+      <c r="E52" s="2" t="inlineStr"/>
+      <c r="F52" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #322 (commit 0ccd925, merged 2026-05-22)
 added the customer-facing line to the pricing page that reflects
@@ -2615,7 +2602,7 @@
 Enterprise+ block, reads:</t>
         </is>
       </c>
-      <c r="G51" s="3" t="inlineStr">
+      <c r="G52" s="2" t="inlineStr">
         <is>
           <t>2026-05-07 multi-lab discussion (Lisa Veri's
 canonical-case session). PR #322 (initial build); softening PR
@@ -2624,30 +2611,30 @@
 ---</t>
         </is>
       </c>
-      <c r="H51" s="3" t="inlineStr"/>
-    </row>
-    <row r="52" ht="90" customHeight="1">
-      <c r="A52" s="2" t="inlineStr">
+      <c r="H52" s="2" t="inlineStr"/>
+    </row>
+    <row r="53" ht="90" customHeight="1">
+      <c r="A53" s="3" t="inlineStr">
         <is>
           <t>C22</t>
         </is>
       </c>
-      <c r="B52" s="2" t="inlineStr">
+      <c r="B53" s="3" t="inlineStr">
         <is>
           <t>VeritaOps cost-per-test module (formerly #10)</t>
         </is>
       </c>
-      <c r="C52" s="2" t="inlineStr"/>
-      <c r="D52" s="2" t="inlineStr"/>
-      <c r="E52" s="2" t="inlineStr"/>
-      <c r="F52" s="2" t="inlineStr">
+      <c r="C53" s="3" t="inlineStr"/>
+      <c r="D53" s="3" t="inlineStr"/>
+      <c r="E53" s="3" t="inlineStr"/>
+      <c r="F53" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: v1 of the VeritaOps Cost-Per-Reportable-Test
 (CPRT) module shipped across PR #325 through PR #330 on 2026-05-22.
 The module is feature-complete for the typical lab director workflow.</t>
         </is>
       </c>
-      <c r="G52" s="2" t="inlineStr">
+      <c r="G53" s="3" t="inlineStr">
         <is>
           <t>This thread, 2026-05-07 12:05 PM CDT, user message:
 "Parking lot: build an operations module for cost per test
@@ -2656,262 +2643,262 @@
 ---</t>
         </is>
       </c>
-      <c r="H52" s="2" t="inlineStr"/>
-    </row>
-    <row r="53" ht="90" customHeight="1">
-      <c r="A53" s="3" t="inlineStr">
+      <c r="H53" s="3" t="inlineStr"/>
+    </row>
+    <row r="54" ht="90" customHeight="1">
+      <c r="A54" s="2" t="inlineStr">
         <is>
           <t>C23</t>
         </is>
       </c>
-      <c r="B53" s="3" t="inlineStr">
+      <c r="B54" s="2" t="inlineStr">
         <is>
           <t>CCL lab name visual disambiguation in lab switcher (formerly #34)</t>
         </is>
       </c>
-      <c r="C53" s="3" t="inlineStr"/>
-      <c r="D53" s="3" t="inlineStr">
+      <c r="C54" s="2" t="inlineStr"/>
+      <c r="D54" s="2" t="inlineStr">
         <is>
           <t>XS (under 1 day, actual)</t>
         </is>
       </c>
-      <c r="E53" s="3" t="inlineStr">
+      <c r="E54" s="2" t="inlineStr">
         <is>
           <t>Low — cosmetic; only mattered when Lisa or Michael picked the wrong lab from...</t>
         </is>
       </c>
-      <c r="F53" s="3" t="inlineStr">
+      <c r="F54" s="2" t="inlineStr">
         <is>
           <t>Effort: XS (under 1 day, actual)
 Importance: Low — cosmetic; only mattered when Lisa or Michael picked the wrong lab from the dropdown.</t>
         </is>
       </c>
-      <c r="G53" s="3" t="inlineStr">
+      <c r="G54" s="2" t="inlineStr">
         <is>
           <t>flagged 2026-05-23 immediately after provisioning Lisa's CCL lab; closed 2026-05-24.
 ---</t>
         </is>
       </c>
-      <c r="H53" s="3" t="inlineStr"/>
-    </row>
-    <row r="54" ht="90" customHeight="1">
-      <c r="A54" s="2" t="inlineStr">
+      <c r="H54" s="2" t="inlineStr"/>
+    </row>
+    <row r="55" ht="90" customHeight="1">
+      <c r="A55" s="3" t="inlineStr">
         <is>
           <t>C24</t>
         </is>
       </c>
-      <c r="B54" s="2" t="inlineStr">
+      <c r="B55" s="3" t="inlineStr">
         <is>
           <t>VC Unlimited Y1/Y2 price disclosure UX (formerly #35)</t>
         </is>
       </c>
-      <c r="C54" s="2" t="inlineStr"/>
-      <c r="D54" s="2" t="inlineStr">
+      <c r="C55" s="3" t="inlineStr"/>
+      <c r="D55" s="3" t="inlineStr">
         <is>
           <t>XS (under 1 day, actual)</t>
         </is>
       </c>
-      <c r="E54" s="2" t="inlineStr">
+      <c r="E55" s="3" t="inlineStr">
         <is>
           <t>Low when shipped (proactive, no customer complaint yet) — but high if a procu...</t>
         </is>
       </c>
-      <c r="F54" s="2" t="inlineStr">
+      <c r="F55" s="3" t="inlineStr">
         <is>
           <t>Effort: XS (under 1 day, actual)
 Importance: Low when shipped (proactive, no customer complaint yet) — but high if a procurement reviewer later disputes the $499 renewal as undisclosed.</t>
         </is>
       </c>
-      <c r="G54" s="2" t="inlineStr">
+      <c r="G55" s="3" t="inlineStr">
         <is>
           <t>Pricing rebuild 2026-05-23; closed 2026-05-24 proactively before any customer dispute.
 ---</t>
         </is>
       </c>
-      <c r="H54" s="2" t="inlineStr"/>
-    </row>
-    <row r="55" ht="90" customHeight="1">
-      <c r="A55" s="3" t="inlineStr">
+      <c r="H55" s="3" t="inlineStr"/>
+    </row>
+    <row r="56" ht="90" customHeight="1">
+      <c r="A56" s="2" t="inlineStr">
         <is>
           <t>C25</t>
         </is>
       </c>
-      <c r="B55" s="3" t="inlineStr">
+      <c r="B56" s="2" t="inlineStr">
         <is>
           <t>VeritaQC Phase 1 (Levey-Jennings + Westgard live engine) (formerly #20)</t>
         </is>
       </c>
-      <c r="C55" s="3" t="inlineStr"/>
-      <c r="D55" s="3" t="inlineStr">
+      <c r="C56" s="2" t="inlineStr"/>
+      <c r="D56" s="2" t="inlineStr">
         <is>
           <t>L (about 5 days end-to-end, actual: Phase 0 schema → Phase 1A evaluator → 1B...</t>
         </is>
       </c>
-      <c r="E55" s="3" t="inlineStr">
+      <c r="E56" s="2" t="inlineStr">
         <is>
           <t>High — largest single gap vs myLabCompliance.io per Perplexity competitor ana...</t>
         </is>
       </c>
-      <c r="F55" s="3" t="inlineStr">
+      <c r="F56" s="2" t="inlineStr">
         <is>
           <t>Effort: L (about 5 days end-to-end, actual: Phase 0 schema → Phase 1A evaluator → 1B entry UI → 1C daily review → 1D monthly PDF + attestation)
 Importance: High — largest single gap vs myLabCompliance.io per Perplexity competitor analysis; promotes VeritaAssure from documentation tool to lab operations platform.</t>
         </is>
       </c>
-      <c r="G55" s="3" t="inlineStr">
+      <c r="G56" s="2" t="inlineStr">
         <is>
           <t>Perplexity competitor analysis 2026-05-10. Scoping confirmed via the build_phase1_mockup.py iterations 2026-05-24. Shipped 2026-05-25.
 ---</t>
         </is>
       </c>
-      <c r="H55" s="3" t="inlineStr"/>
-    </row>
-    <row r="56" ht="90" customHeight="1">
-      <c r="A56" s="2" t="inlineStr">
+      <c r="H56" s="2" t="inlineStr"/>
+    </row>
+    <row r="57" ht="90" customHeight="1">
+      <c r="A57" s="3" t="inlineStr">
         <is>
           <t>C26</t>
         </is>
       </c>
-      <c r="B56" s="2" t="inlineStr">
+      <c r="B57" s="3" t="inlineStr">
         <is>
           <t>VeritaLab CMS-116 application support + state licensing registry (formerly #22)</t>
         </is>
       </c>
-      <c r="C56" s="2" t="inlineStr"/>
-      <c r="D56" s="2" t="inlineStr">
+      <c r="C57" s="3" t="inlineStr"/>
+      <c r="D57" s="3" t="inlineStr">
         <is>
           <t>M (1-2 weeks for v1, actual)</t>
         </is>
       </c>
-      <c r="E56" s="2" t="inlineStr">
+      <c r="E57" s="3" t="inlineStr">
         <is>
           <t>Medium — competitor parity (myLabCompliance.io) plus useful at lab startup an...</t>
         </is>
       </c>
-      <c r="F56" s="2" t="inlineStr">
+      <c r="F57" s="3" t="inlineStr">
         <is>
           <t>Effort: M (1-2 weeks for v1, actual)
 Importance: Medium — competitor parity (myLabCompliance.io) plus useful at lab startup and at certificate-type changes.</t>
         </is>
       </c>
-      <c r="G56" s="2" t="inlineStr">
+      <c r="G57" s="3" t="inlineStr">
         <is>
           <t>Perplexity competitor analysis (myLabCompliance.io), 2026-05-10. Reclassified as a VeritaLab extension 2026-05-25. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H56" s="2" t="inlineStr"/>
-    </row>
-    <row r="57" ht="90" customHeight="1">
-      <c r="A57" s="3" t="inlineStr">
+      <c r="H57" s="3" t="inlineStr"/>
+    </row>
+    <row r="58" ht="90" customHeight="1">
+      <c r="A58" s="2" t="inlineStr">
         <is>
           <t>C27</t>
         </is>
       </c>
-      <c r="B57" s="3" t="inlineStr">
+      <c r="B58" s="2" t="inlineStr">
         <is>
           <t>Active vs view-only seat split (formerly #33)</t>
         </is>
       </c>
-      <c r="C57" s="3" t="inlineStr"/>
-      <c r="D57" s="3" t="inlineStr">
+      <c r="C58" s="2" t="inlineStr"/>
+      <c r="D58" s="2" t="inlineStr">
         <is>
           <t>M (~1 week of engineering, actual: shipped in a single multi-PR session)</t>
         </is>
       </c>
-      <c r="E57" s="3" t="inlineStr">
+      <c r="E58" s="2" t="inlineStr">
         <is>
           <t>Medium — closed the gap between /pricing copy and product behavior; gives sal...</t>
         </is>
       </c>
-      <c r="F57" s="3" t="inlineStr">
+      <c r="F58" s="2" t="inlineStr">
         <is>
           <t>Effort: M (~1 week of engineering, actual: shipped in a single multi-PR session)
 Importance: Medium — closed the gap between /pricing copy and product behavior; gives sales a clean answer for "do you charge for our medical director?"</t>
         </is>
       </c>
-      <c r="G57" s="3" t="inlineStr">
+      <c r="G58" s="2" t="inlineStr">
         <is>
           <t>Pricing analysis doc Decision 3 (2026-05-21); MEDIUM scenario revised 2026-05-29 to retire the "unlimited view-only" claim. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H57" s="3" t="inlineStr"/>
-    </row>
-    <row r="58" ht="90" customHeight="1">
-      <c r="A58" s="2" t="inlineStr">
+      <c r="H58" s="2" t="inlineStr"/>
+    </row>
+    <row r="59" ht="90" customHeight="1">
+      <c r="A59" s="3" t="inlineStr">
         <is>
           <t>C28</t>
         </is>
       </c>
-      <c r="B58" s="2" t="inlineStr">
+      <c r="B59" s="3" t="inlineStr">
         <is>
           <t>"Why VeritaCheck" comparative one-pager (formerly #37)</t>
         </is>
       </c>
-      <c r="C58" s="2" t="inlineStr"/>
-      <c r="D58" s="2" t="inlineStr">
+      <c r="C59" s="3" t="inlineStr"/>
+      <c r="D59" s="3" t="inlineStr">
         <is>
           <t>S (one design pass + four claim paragraphs + PDF + matching marketing-site pa...</t>
         </is>
       </c>
-      <c r="E58" s="2" t="inlineStr">
+      <c r="E59" s="3" t="inlineStr">
         <is>
           <t>Medium — closed a positioning gap surfaced by six COLA conference attendees a...</t>
         </is>
       </c>
-      <c r="F58" s="2" t="inlineStr">
+      <c r="F59" s="3" t="inlineStr">
         <is>
           <t>Effort: S (one design pass + four claim paragraphs + PDF + matching marketing-site page, actual)
 Importance: Medium — closed a positioning gap surfaced by six COLA conference attendees attached to a legacy verification tool; converts product-quality advantage into a leave-behind Lisa can hand out.</t>
         </is>
       </c>
-      <c r="G58" s="2" t="inlineStr">
+      <c r="G59" s="3" t="inlineStr">
         <is>
           <t>2026-05-11 / 2026-05-12 conference notes review with Michael. Conference attendees (Whitehead, Odegard, Othman, Molinelli, Kyle, Allred) expressed interest in equivalent / superior product. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H58" s="2" t="inlineStr"/>
-    </row>
-    <row r="59" ht="90" customHeight="1">
-      <c r="A59" s="3" t="inlineStr">
+      <c r="H59" s="3" t="inlineStr"/>
+    </row>
+    <row r="60" ht="90" customHeight="1">
+      <c r="A60" s="2" t="inlineStr">
         <is>
           <t>C29</t>
         </is>
       </c>
-      <c r="B59" s="3" t="inlineStr">
+      <c r="B60" s="2" t="inlineStr">
         <is>
           <t>VeritaPolicy approval workflow — MediaLab functional mirror</t>
         </is>
       </c>
-      <c r="C59" s="3" t="inlineStr"/>
-      <c r="D59" s="3" t="inlineStr">
+      <c r="C60" s="2" t="inlineStr"/>
+      <c r="D60" s="2" t="inlineStr">
         <is>
           <t>XL (one focused session, 12 PRs landed)</t>
         </is>
       </c>
-      <c r="E59" s="3" t="inlineStr">
+      <c r="E60" s="2" t="inlineStr">
         <is>
           <t>High — replaces MediaLab Document Control ($752/$2,250 starting price, scalin...</t>
         </is>
       </c>
-      <c r="F59" s="3" t="inlineStr">
+      <c r="F60" s="2" t="inlineStr">
         <is>
           <t>Effort: XL (one focused session, 12 PRs landed)
 Importance: High — replaces MediaLab Document Control ($752/$2,250 starting price, scaling to $10K-$20K/yr at enterprise per Capterra public data) with an included VeritaPolicy feature; closes a real positioning gap and gives sales a direct comparator line.</t>
         </is>
       </c>
-      <c r="G59" s="3" t="inlineStr">
+      <c r="G60" s="2" t="inlineStr">
         <is>
           <t>Pricing strategy conversation 2026-05-29 (Michael: "I don't like bolt-ons; we should replicate this") → scoped 8 phases → shipped all 12 PRs in single session. Shipped 2026-05-29.
 ---</t>
         </is>
       </c>
-      <c r="H59" s="3" t="inlineStr"/>
+      <c r="H60" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H59"/>
+  <autoFilter ref="A1:H60"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
TASK: Promote VeritaQC to Live (import click-through verified); close #40 as C60; regen xlsx PLAN:   1. VeritaAssurePage: VeritaQC badge "Phase 1 preview" to "Live" (emerald) - all 18 modules now Live.   2. Update the badge Playwright spec: no module remains "Phase 1 preview".   3. Close parking-lot #40 as C60 (browser click-through verified, 15 replicates imported) and regenerate the xlsx. Self-check:   - #40 verified in the in-app browser end to end (study-type/instrument/control-lot Radix Selects all rendered and selected; Import landed 15 replicates). Operator authorized the promotion.   - Spec updated to match (Phase 1 preview count 0); PARKING_LOT md + xlsx committed together per the sync rule.   - Public marketing page badge only; no module behavior changed. Typecheck clean.
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PARKING_LOT.xlsx
+++ b/PARKING_LOT.xlsx
@@ -12,8 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RETIRED" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$60</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$61</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RETIRED'!$A$1:$H$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -924,55 +924,15 @@
     <row r="10" ht="90" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>42</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>VeritaQC Import Phase A: human-in-the-loop Gate 3 click-through (deferred)</t>
+          <t>Outbound demo-invite messaging campaign to 1st-degree LinkedIn contacts</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Open, awaiting Michael's 5-minute click test. Will move task #77 to completed only after he reports the user-visible result.
----</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>XS (~5 minutes of Michael's time on a live URL).</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>Low. Backend contract is fully verified via 35/35 passing offline contract ch...</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>Effort: XS (~5 minutes of Michael's time on a live URL).
-Importance: Low. Backend contract is fully verified via 35/35 passing offline contract checks (scripts/verify-veritaqc-import.js) plus three live-API smoke checks against prod (candidates, preview, mappings PUT/GET) on Riverside Regional with seed lot SEED-1780436709094 (18 Glucose results). The browser-driven click was not run because Claude-in-Chrome's renderer froze repeatedly on the Radix Select inside VeritaCheckPage, not on Phase A code itself. Risk of a UX bug surviving to a customer is small but not zero.</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>task #77 stalled at Gate 3 step 8 on 2026-06-02. PR #500 squash-merged at commit 17a91ff, prod /api/health confirmed ACTIVE on that commit at 20:43 UTC.</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr"/>
-    </row>
-    <row r="11" ht="90" customHeight="1">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>42</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>Outbound demo-invite messaging campaign to 1st-degree LinkedIn contacts</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>Parked. Plan documented. Implementation deferred until trigger conditions met.
 ---
@@ -981,69 +941,69 @@
 _(item #51 closed 2026-09-2...</t>
         </is>
       </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>L (1 week prep + 4-6 weeks of staged sends)</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>High. Converts existing warm network (~2,500 1st-degree contacts and growing...</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>A staged outbound DM campaign walking Michael's 1st-degree LinkedIn contacts through tier-segmented demo invitations for VeritaAssure. Goal: convert warmest contacts into demo conversations first, then chain into trials and paid subscriptions. Separate pipeline from COLA cohort follow-up and from content-driven inbound; all three feed the same demo funnel but originate from different warmth sources.</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 session, after weekly LinkedIn invite batch completion (80 sent, cap hit at #84 Victoria Allen).</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11" ht="90" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Regenerate the 119-function access-inventory Excel with the corrected MD persona</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Open, low priority. Offered to Michael; skippable if the sweep was a one-off working artifact.
+---</t>
+        </is>
+      </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>L (1 week prep + 4-6 weeks of staged sends)</t>
+          <t>XS (~15 min to re-run the sweep harness and re-deliver).</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>High. Converts existing warm network (~2,500 1st-degree contacts and growing...</t>
+          <t>Low — the harness and the shipped fixes are correct; only the recorded Excel'...</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>A staged outbound DM campaign walking Michael's 1st-degree LinkedIn contacts through tier-segmented demo invitations for VeritaAssure. Goal: convert warmest contacts into demo conversations first, then chain into trials and paid subscriptions. Separate pipeline from COLA cohort follow-up and from content-driven inbound; all three feed the same demo funnel but originate from different warmth sources.</t>
+          <t>The full-inventory 4-login access sweep (VeritaAssure_Function_Inventory.xlsx) was first generated with the medical-director test persona mis-seeded as a seatless member, which over-flagged its column. The harness was then corrected to seat the MD as the active writer it actually is (scripts/qa-sweep/inventory-sweep.ts). The delivered Excel still shows the old md results; re-running reclassifies the md-artifact flags down to the real findings, which were already fixed in PR A (#1441). Only worth doing if the sheet gets filed or shared externally.</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>2026-06-04 session, after weekly LinkedIn invite batch completion (80 sent, cap hit at #84 Victoria Allen).</t>
+          <t>this session, QA sweep (2026-10-03 to 2026-10-04).</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr"/>
     </row>
-    <row r="12" ht="90" customHeight="1">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>44</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Regenerate the 119-function access-inventory Excel with the corrected MD persona</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Open, low priority. Offered to Michael; skippable if the sweep was a one-off working artifact.
----</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>XS (~15 min to re-run the sweep harness and re-deliver).</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>Low — the harness and the shipped fixes are correct; only the recorded Excel'...</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>The full-inventory 4-login access sweep (VeritaAssure_Function_Inventory.xlsx) was first generated with the medical-director test persona mis-seeded as a seatless member, which over-flagged its column. The harness was then corrected to seat the MD as the active writer it actually is (scripts/qa-sweep/inventory-sweep.ts). The delivered Excel still shows the old md results; re-running reclassifies the md-artifact flags down to the real findings, which were already fixed in PR A (#1441). Only worth doing if the sheet gets filed or shared externally.</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>this session, QA sweep (2026-10-03 to 2026-10-04).</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:H12"/>
+  <autoFilter ref="A1:H11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1054,7 +1014,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H60"/>
+  <dimension ref="A1:H61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1112,24 +1072,24 @@
     <row r="2" ht="90" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>C59</t>
+          <t>C60</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Confirm the finding-closure signer policy (was #43)</t>
+          <t>VeritaQC Import Phase A browser click-through (was #40)</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr"/>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>was XS / Importance: Medium</t>
+          <t>was XS / Importance: Low</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Effort: was XS / Importance: Medium</t>
+          <t>Effort: was XS / Importance: Low</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
@@ -1138,24 +1098,24 @@
     <row r="3" ht="90" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>C58</t>
+          <t>C59</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>VeritaDC per-document attestation tracker + "My Documents" rename (built as #45)</t>
+          <t>Confirm the finding-closure signer policy (was #43)</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr"/>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>was M / Importance: Medium-High</t>
+          <t>was XS / Importance: Medium</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Effort: was M / Importance: Medium-High</t>
+          <t>Effort: was XS / Importance: Medium</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr"/>
@@ -1164,24 +1124,24 @@
     <row r="4" ht="90" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>C57</t>
+          <t>C58</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Hide sections a lab does not use from a master list (was #47)</t>
+          <t>VeritaDC per-document attestation tracker + "My Documents" rename (built as #45)</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr"/>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>was S-M / Importance: Medium-High (prospect-requested)</t>
+          <t>was M / Importance: Medium-High</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Effort: was S-M / Importance: Medium-High (prospect-requested)</t>
+          <t>Effort: was M / Importance: Medium-High</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr"/>
@@ -1190,24 +1150,24 @@
     <row r="5" ht="90" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>C56</t>
+          <t>C57</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>VeritaCEU: curated free continuing-education provider list (was #53)</t>
+          <t>Hide sections a lab does not use from a master list (was #47)</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr"/>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>was S / Importance: Low-Medium</t>
+          <t>was S-M / Importance: Medium-High (prospect-requested)</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Effort: was S / Importance: Low-Medium</t>
+          <t>Effort: was S-M / Importance: Medium-High (prospect-requested)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr"/>
@@ -1216,24 +1176,24 @@
     <row r="6" ht="90" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>C55</t>
+          <t>C56</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>VeritaScan: let sites add their own custom questions (was #55)</t>
+          <t>VeritaCEU: curated free continuing-education provider list (was #53)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr"/>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>was M / Importance: Medium-High</t>
+          <t>was S / Importance: Low-Medium</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Effort: was M / Importance: Medium-High</t>
+          <t>Effort: was S / Importance: Low-Medium</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
@@ -1242,24 +1202,24 @@
     <row r="7" ht="90" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>C54</t>
+          <t>C55</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>VeritaQC: at-entry warning when a QC point is outside 2 SD (was #56)</t>
+          <t>VeritaScan: let sites add their own custom questions (was #55)</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr"/>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>was S-M (shipped S) / Importance: High</t>
+          <t>was M / Importance: Medium-High</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Effort: was S-M (shipped S) / Importance: High</t>
+          <t>Effort: was M / Importance: Medium-High</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr"/>
@@ -1268,24 +1228,24 @@
     <row r="8" ht="90" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>C53</t>
+          <t>C54</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>VeritaTrack: quarterly task loaded as monthly until re-saved (was #54)</t>
+          <t>VeritaQC: at-entry warning when a QC point is outside 2 SD (was #56)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr"/>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>was S / Importance: Medium</t>
+          <t>was S-M (shipped S) / Importance: High</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Effort: was S / Importance: Medium</t>
+          <t>Effort: was S-M (shipped S) / Importance: High</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
@@ -1294,24 +1254,24 @@
     <row r="9" ht="90" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>C52</t>
+          <t>C53</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>VeritaResponse internal NCE / non-conforming event (was #36)</t>
+          <t>VeritaTrack: quarterly task loaded as monthly until re-saved (was #54)</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr"/>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>was L (shipped as MEDIUM) / Importance: High</t>
+          <t>was S / Importance: Medium</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Effort: was L (shipped as MEDIUM) / Importance: High</t>
+          <t>Effort: was S / Importance: Medium</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr"/>
@@ -1320,24 +1280,24 @@
     <row r="10" ht="90" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>C49</t>
+          <t>C52</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Competency "assessed this cycle" cadence-aware window (was #50)</t>
+          <t>VeritaResponse internal NCE / non-conforming event (was #36)</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr"/>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>was S-M / Importance: Medium</t>
+          <t>was L (shipped as MEDIUM) / Importance: High</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Effort: was S-M / Importance: Medium</t>
+          <t>Effort: was L (shipped as MEDIUM) / Importance: High</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
@@ -1346,12 +1306,12 @@
     <row r="11" ht="90" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>C50</t>
+          <t>C49</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>VeritaTrack task owner + owner-only reminder routing (was #51)</t>
+          <t>Competency "assessed this cycle" cadence-aware window (was #50)</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr"/>
@@ -1372,24 +1332,24 @@
     <row r="12" ht="90" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>C51</t>
+          <t>C50</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Designate Medical Director by picking a lab member (was #52, core)</t>
+          <t>VeritaTrack task owner + owner-only reminder routing (was #51)</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr"/>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>was S-M / Importance: Medium-High</t>
+          <t>was S-M / Importance: Medium</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Effort: was S-M / Importance: Medium-High</t>
+          <t>Effort: was S-M / Importance: Medium</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr"/>
@@ -1398,24 +1358,24 @@
     <row r="13" ht="90" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>C47</t>
+          <t>C51</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Unregulated-analyte / Alternative Assessment (AAA) coverage (was #18)</t>
+          <t>Designate Medical Director by picking a lab member (was #52, core)</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr"/>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>was S (Phase 3) / Importance: Medium</t>
+          <t>was S-M / Importance: Medium-High</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Effort: was S (Phase 3) / Importance: Medium</t>
+          <t>Effort: was S-M / Importance: Medium-High</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr"/>
@@ -1424,24 +1384,24 @@
     <row r="14" ht="90" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>C48</t>
+          <t>C47</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>VeritaResponse post-survey deficiency module (was #17)</t>
+          <t>Unregulated-analyte / Alternative Assessment (AAA) coverage (was #18)</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr"/>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>was XL / Importance: High</t>
+          <t>was S (Phase 3) / Importance: Medium</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Effort: was XL / Importance: High</t>
+          <t>Effort: was S (Phase 3) / Importance: Medium</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr"/>
@@ -1450,39 +1410,38 @@
     <row r="15" ht="90" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>C45</t>
+          <t>C48</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Unify coverage/competency recurrence helper (was #49) - closed as non-issue</t>
+          <t>VeritaResponse post-survey deficiency module (was #17)</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr"/>
-      <c r="D15" s="3" t="inlineStr"/>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>was XL / Importance: High</t>
+        </is>
+      </c>
       <c r="E15" s="3" t="inlineStr"/>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: Investigated 2026-09-24 before building. The coverage recurrence math (+6-month interval, signed-resets-to-missing, nextDueOn/overdue, isFailVerdict) is ALREADY single-source in server/veritacheckCoverage.ts (computeCoverageFrom). server/coverageReport.ts and the routes.ts coverage export do not recompute it; they consume the computed nextDueOn/overdue/status fields and apply small surface-specific presentation labels (deliberately different vocabularies per surface, so they should not be merged). The only truly identical duplicate is a one-line date formatter. The competency "owed" derivation is NOT the same cadence: competency follows the CLIA milestone schedule (initial / semiannual year 1 / annual, 42 CFR 493.1451(b)(8) and 493.1235), which is a different regulatory interval from the coverage 6-month rule (493.1281 / 493.1255) and must stay separate. No worthwhile extraction; merging the two cadences would be wrong. Closed 2026-09-24. (The year-1 competency-window refinement remains tracked separately as #50.)</t>
-        </is>
-      </c>
-      <c r="G15" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-24 session, "keep working" pass; scoped read-only, found no real duplication.
----</t>
-        </is>
-      </c>
+          <t>Effort: was XL / Importance: High</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr"/>
       <c r="H15" s="3" t="inlineStr"/>
     </row>
     <row r="16" ht="90" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>C46</t>
+          <t>C45</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Verified-users product-update send path (wrong-list incident fix)</t>
+          <t>Unify coverage/competency recurrence helper (was #49) - closed as non-issue</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr"/>
@@ -1490,12 +1449,12 @@
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: Shipped PR #1324 (merged 4e05506a, deploy ACTIVE). New POST /api/admin/users/send targets registered VeritaAssure account holders (the users table), never the Lab Director's Briefing subscriber list. Separate explicitly-named endpoint (not a flag with a dangerous default), account-holder email framing, excludes suppressed emails and RFC-reserved test domains, CC owner, dryRun + testTo previews. Public unsubscribe now upserts a suppression row so opt-outs are honored across both audiences. Live dryRun: 49 verified-user recipients vs 673 on the Briefing list. Receipts: scripts/verify-product-update-send.mts 24/24, tsc clean, rendered sample inspected. Fixes the fallout from the 2026-09-23/24 wrong-list send (a product update went to the 675-person Briefing list). Nothing sends without Michael's explicit "send it."</t>
+          <t>Closure evidence: Investigated 2026-09-24 before building. The coverage recurrence math (+6-month interval, signed-resets-to-missing, nextDueOn/overdue, isFailVerdict) is ALREADY single-source in server/veritacheckCoverage.ts (computeCoverageFrom). server/coverageReport.ts and the routes.ts coverage export do not recompute it; they consume the computed nextDueOn/overdue/status fields and apply small surface-specific presentation labels (deliberately different vocabularies per surface, so they should not be merged). The only truly identical duplicate is a one-line date formatter. The competency "owed" derivation is NOT the same cadence: competency follows the CLIA milestone schedule (initial / semiannual year 1 / annual, 42 CFR 493.1451(b)(8) and 493.1235), which is a different regulatory interval from the coverage 6-month rule (493.1281 / 493.1255) and must stay separate. No worthwhile extraction; merging the two cadences would be wrong. Closed 2026-09-24. (The year-1 competency-window refinement remains tracked separately as #50.)</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 session; Michael selected this as the next build after the #41 close.
+          <t>2026-09-24 session, "keep working" pass; scoped read-only, found no real duplication.
 ---</t>
         </is>
       </c>
@@ -1504,12 +1463,12 @@
     <row r="17" ht="90" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>C44</t>
+          <t>C46</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Verify-script convention backfill (was #41) + audit matcher fix</t>
+          <t>Verified-users product-update send path (wrong-list incident fix)</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr"/>
@@ -1517,12 +1476,12 @@
       <c r="E17" s="3" t="inlineStr"/>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: #41 was fully backfilled on 2026-06-13 (all 8 high-stakes scripts landed; see C30); it had only been mis-filed in OPEN. A 2026-09-24 re-audit initially reported 4 of 5 recent math/logic commits as missing a verify script, which was a FALSE POSITIVE: scripts/audit_verify_script_coverage.py matched only scripts/verify-*.js / .cjs, so it ignored the .mjs / .mts / .ts verify scripts the repo now ships (e.g. verify-ptcoag-multi.mts, verify-tea-criterion-format.mjs). Fixed the matcher to accept .js/.cjs/.mjs/.ts/.mts; re-run shows 5 of 5 covered, 0 debt. The convention is being followed. Closed 2026-09-24.</t>
+          <t>Closure evidence: Shipped PR #1324 (merged 4e05506a, deploy ACTIVE). New POST /api/admin/users/send targets registered VeritaAssure account holders (the users table), never the Lab Director's Briefing subscriber list. Separate explicitly-named endpoint (not a flag with a dangerous default), account-holder email framing, excludes suppressed emails and RFC-reserved test domains, CC owner, dryRun + testTo previews. Public unsubscribe now upserts a suppression row so opt-outs are honored across both audiences. Live dryRun: 49 verified-user recipients vs 673 on the Briefing list. Receipts: scripts/verify-product-update-send.mts 24/24, tsc clean, rendered sample inspected. Fixes the fallout from the 2026-09-23/24 wrong-list send (a product update went to the 675-person Briefing list). Nothing sends without Michael's explicit "send it."</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>2026-09-24 session, "keep working" pass; audit tooling bug found + fixed.
+          <t>2026-09-24 session; Michael selected this as the next build after the #41 close.
 ---</t>
         </is>
       </c>
@@ -1531,12 +1490,12 @@
     <row r="18" ht="90" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>C43</t>
+          <t>C44</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>VeritaStaff instrument-centric (dual) assignment view</t>
+          <t>Verify-script convention backfill (was #41) + audit matcher fix</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr"/>
@@ -1544,12 +1503,12 @@
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1320. GET/PUT /staff/instruments/:id/employees (transpose of the per-employee endpoints); an "Assign by Instrument" dialog lets a director pick a test system or manual test and check off who runs it. Same staff_employee_instruments join, with the 42 CFR 493.1235(a) duty-change event emitted on newly-added pairs so both orientations trigger the same reassessment. GET verified live on SCAHC lab 2. Closed 2026-09-24.</t>
+          <t>Closure evidence: #41 was fully backfilled on 2026-06-13 (all 8 high-stakes scripts landed; see C30); it had only been mis-filed in OPEN. A 2026-09-24 re-audit initially reported 4 of 5 recent math/logic commits as missing a verify script, which was a FALSE POSITIVE: scripts/audit_verify_script_coverage.py matched only scripts/verify-*.js / .cjs, so it ignored the .mjs / .mts / .ts verify scripts the repo now ships (e.g. verify-ptcoag-multi.mts, verify-tea-criterion-format.mjs). Fixed the matcher to accept .js/.cjs/.mjs/.ts/.mts; re-run shows 5 of 5 covered, 0 debt. The convention is being followed. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 session, Michael ("in staff we should also give the dual view when assigning coverage to test systems or manual tests").
+          <t>2026-09-24 session, "keep working" pass; audit tooling bug found + fixed.
 ---</t>
         </is>
       </c>
@@ -1558,12 +1517,12 @@
     <row r="19" ht="90" customHeight="1">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>C42</t>
+          <t>C43</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>VeritaComp coverage map (required-vs-assessed matrix, dual view)</t>
+          <t>VeritaStaff instrument-centric (dual) assignment view</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr"/>
@@ -1571,12 +1530,12 @@
       <c r="E19" s="3" t="inlineStr"/>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1319 (+ status layer PR #1316). /competency/owed returns per-item assessed (locked passing assessment this cycle on a covering method group) + per-employee CLIA status; CompetencyCoverageMap renders a By-employee / By-instrument matrix (Assessed / Owed / Overdue / Gap). Verified live on SCAHC lab 2 (owed 116, assessed 2, gaps 0). Completes #48 as the VeritaCheck-parity coverage map. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1320. GET/PUT /staff/instruments/:id/employees (transpose of the per-employee endpoints); an "Assign by Instrument" dialog lets a director pick a test system or manual test and check off who runs it. Same staff_employee_instruments join, with the 42 CFR 493.1235(a) duty-change event emitted on newly-added pairs so both orientations trigger the same reassessment. GET verified live on SCAHC lab 2. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>2026-09-24 session, Michael ("are we building the competencies to have a coverage map, same as veritacheck?" then "build it").
+          <t>2026-09-24 session, Michael ("in staff we should also give the dual view when assigning coverage to test systems or manual tests").
 ---</t>
         </is>
       </c>
@@ -1585,12 +1544,12 @@
     <row r="20" ht="90" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>C41</t>
+          <t>C42</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>VeritaCheck coverage recurrence (method comparison + cal-ver/linearity + reports)</t>
+          <t>VeritaComp coverage map (required-vs-assessed matrix, dual view)</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr"/>
@@ -1598,12 +1557,12 @@
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: PRs #1317 (method comparison), #1318 (cal-ver/linearity), #1321 (report Next-due columns). Periodic verification (correlation/method comparison 42 CFR 493.1281; cal-ver/linearity 42 CFR 493.1255; both 6-month) now recurs: a signed study banks the cycle and rolls to next-due = signed + 6 months instead of reading "done" forever. Status Missing/Failed/Completed-unsigned + a "Next due on" column on-screen and in both coverage exports; also credits the previously-ignored "correlation" study type. Root cause: computeCoverageFrom marked requirements done on mere existence, no date logic. Verified live on SCAHC lab 2 (101 correlations + 11 cal-ver rows now carry a next-due). Engine-level, all facilities. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1319 (+ status layer PR #1316). /competency/owed returns per-item assessed (locked passing assessment this cycle on a covering method group) + per-employee CLIA status; CompetencyCoverageMap renders a By-employee / By-instrument matrix (Assessed / Owed / Overdue / Gap). Verified live on SCAHC lab 2 (owed 116, assessed 2, gaps 0). Completes #48 as the VeritaCheck-parity coverage map. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 session, Michael ("Look at San Carlos... they finished their last set of correlations (all 103) but their menu never reset").
+          <t>2026-09-24 session, Michael ("are we building the competencies to have a coverage map, same as veritacheck?" then "build it").
 ---</t>
         </is>
       </c>
@@ -1612,12 +1571,12 @@
     <row r="21" ht="90" customHeight="1">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>C40</t>
+          <t>C41</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>VeritaComp Competencies Owed derived from VeritaStaff, with gap detection (was #48)</t>
+          <t>VeritaCheck coverage recurrence (method comparison + cal-ver/linearity + reports)</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr"/>
@@ -1625,12 +1584,12 @@
       <c r="E21" s="3" t="inlineStr"/>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1314 (squash 2bcb0db9). GET /api/labs/:labId/competency/owed derives each VeritaStaff testing employee's owed competencies from their assigned instruments (staff_employee_instruments -&gt; veritamap_instruments + tests), on the CLIA timeline, and flags instruments not covered by any competency program as gaps. CompetenciesOwedSection renders it on the VeritaComp landing page. Reuses the shipped bridge + suggested-method-groups match rules; no new tables. Verified live on prod with real assignment data: 2 instruments assigned to a demo staffer produced owed=2, gaps=2 (HIGH, Technical Supervisor), then reverted cleanly. Closed 2026-09-24.</t>
+          <t>Closure evidence: PRs #1317 (method comparison), #1318 (cal-ver/linearity), #1321 (report Next-due columns). Periodic verification (correlation/method comparison 42 CFR 493.1281; cal-ver/linearity 42 CFR 493.1255; both 6-month) now recurs: a signed study banks the cycle and rolls to next-due = signed + 6 months instead of reading "done" forever. Status Missing/Failed/Completed-unsigned + a "Next due on" column on-screen and in both coverage exports; also credits the previously-ignored "correlation" study type. Root cause: computeCoverageFrom marked requirements done on mere existence, no date logic. Verified live on SCAHC lab 2 (101 correlations + 11 cal-ver rows now carry a next-due). Engine-level, all facilities. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>2026-09-23/24 session, Michael ("veritacomp bases what competencies they owe (currently untrue, but needs to be true)"). Option 1 (unify roster on VeritaStaff, match instruments by id).
+          <t>2026-09-24 session, Michael ("Look at San Carlos... they finished their last set of correlations (all 103) but their menu never reset").
 ---</t>
         </is>
       </c>
@@ -1639,12 +1598,12 @@
     <row r="22" ht="90" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>C39</t>
+          <t>C40</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>VeritaScan line items can attach or link evidence (was #46)</t>
+          <t>VeritaComp Competencies Owed derived from VeritaStaff, with gap detection (was #48)</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr"/>
@@ -1652,12 +1611,12 @@
       <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1312 (squash a1dda93d). VeritaScan scan checklist items now show linked evidence as chips (open link, remove) plus a writer "Link evidence" affordance whose picker links an existing VeritaDC/Library document; a shortcut deep-links to the Library for new (governed) documents. Reuses the already-shipped lab_documents + document_checklist_links + coverage endpoints (URL-pointer only, no file storage, no new tables). Browser-verified live on prod (scan 23): the affordance renders and the picker opens. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1314 (squash 2bcb0db9). GET /api/labs/:labId/competency/owed derives each VeritaStaff testing employee's owed competencies from their assigned instruments (staff_employee_instruments -&gt; veritamap_instruments + tests), on the CLIA timeline, and flags instruments not covered by any competency program as gaps. CompetenciesOwedSection renders it on the VeritaComp landing page. Reuses the shipped bridge + suggested-method-groups match rules; no new tables. Verified live on prod with real assignment data: 2 instruments assigned to a demo staffer produced owed=2, gaps=2 (HIGH, Technical Supervisor), then reverted cleanly. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23 session, Michael. Recurring request. Companion: cross-module evidence display on the VeritaDC policy shipped in PR #1313 (by-target cross-links surfaced in the policy View modal, browser-verified live).
+          <t>2026-09-23/24 session, Michael ("veritacomp bases what competencies they owe (currently untrue, but needs to be true)"). Option 1 (unify roster on VeritaStaff, match instruments by id).
 ---</t>
         </is>
       </c>
@@ -1666,12 +1625,12 @@
     <row r="23" ht="90" customHeight="1">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>C38</t>
+          <t>C39</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>VeritaTrack calendar month cells expand to reveal hidden tasks (was #45)</t>
+          <t>VeritaScan line items can attach or link evidence (was #46)</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr"/>
@@ -1679,12 +1638,12 @@
       <c r="E23" s="3" t="inlineStr"/>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: VeritaTrack CalendarView month cells with more than three tasks now expand in place (chevron, "+N more" toggling to "Show less", due dates), so no task is hidden with no path to it (client/src/pages/VeritaTrackAppPage.tsx CalendarView). Shipped 2026-09-23. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1312 (squash a1dda93d). VeritaScan scan checklist items now show linked evidence as chips (open link, remove) plus a writer "Link evidence" affordance whose picker links an existing VeritaDC/Library document; a shortcut deep-links to the Library for new (governed) documents. Reuses the already-shipped lab_documents + document_checklist_links + coverage endpoints (URL-pointer only, no file storage, no new tables). Browser-verified live on prod (scan 23): the affordance renders and the picker opens. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>2026-09-23 session, Michael screenshot of the VeritaTrack calendar (lab 3, September cell).
+          <t>2026-09-23 session, Michael. Recurring request. Companion: cross-module evidence display on the VeritaDC policy shipped in PR #1313 (by-target cross-links surfaced in the policy View modal, browser-verified live).
 ---</t>
         </is>
       </c>
@@ -1693,12 +1652,12 @@
     <row r="24" ht="90" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>C37</t>
+          <t>C38</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Long Excel column headers no longer clip CFR citations (was #44)</t>
+          <t>VeritaTrack calendar month cells expand to reveal hidden tasks (was #45)</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr"/>
@@ -1706,12 +1665,12 @@
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. The VeritaMap export derives the header row height from the longest wrapped header via headerRowHeight(headers, colWidths) (server/routes.ts:15935) instead of a fixed 20, so "Reference Range Attestation (42 CFR 493.1253)" and the other long headers print in full. No new code this session. Closed 2026-09-24.</t>
+          <t>Closure evidence: VeritaTrack CalendarView month cells with more than three tasks now expand in place (chevron, "+N more" toggling to "Show less", due dates), so no task is hidden with no path to it (client/src/pages/VeritaTrackAppPage.tsx CalendarView). Shipped 2026-09-23. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+          <t>2026-09-23 session, Michael screenshot of the VeritaTrack calendar (lab 3, September cell).
 ---</t>
         </is>
       </c>
@@ -1720,12 +1679,12 @@
     <row r="25" ht="90" customHeight="1">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>C36</t>
+          <t>C37</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>License stamp no longer clobbers the §6 header/footer or names the wrong lab (was #43)</t>
+          <t>Long Excel column headers no longer clip CFR citations (was #44)</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr"/>
@@ -1733,7 +1692,7 @@
       <c r="E25" s="3" t="inlineStr"/>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. setHeaderFooter (shared/licenseExceljs.ts:155-209) now preserves an existing §6 header and appends (not overwrites) the footer left section, and customer-facing exports name the scoped lab: the VeritaScan library export reads req.scope.lab.name / clia_number (server/routes.ts:16572-16573), not the licensee. No new code this session (avoided regressing the existing fix). Closed 2026-09-24.</t>
+          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. The VeritaMap export derives the header row height from the longest wrapped header via headerRowHeight(headers, colWidths) (server/routes.ts:15935) instead of a fixed 20, so "Reference Range Attestation (42 CFR 493.1253)" and the other long headers print in full. No new code this session. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G25" s="3" t="inlineStr">
@@ -1747,18 +1706,45 @@
     <row r="26" ht="90" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>C34</t>
+          <t>C36</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Wire the two static-audit guards into CI (was #43)</t>
+          <t>License stamp no longer clobbers the §6 header/footer or names the wrong lab (was #43)</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr"/>
       <c r="D26" s="2" t="inlineStr"/>
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. setHeaderFooter (shared/licenseExceljs.ts:155-209) now preserves an existing §6 header and appends (not overwrites) the footer left section, and customer-facing exports name the scoped lab: the VeritaScan library export reads req.scope.lab.name / clia_number (server/routes.ts:16572-16573), not the licensee. No new code this session (avoided regressing the existing fix). Closed 2026-09-24.</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+---</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27" ht="90" customHeight="1">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>C34</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Wire the two static-audit guards into CI (was #43)</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr"/>
+      <c r="D27" s="3" t="inlineStr"/>
+      <c r="E27" s="3" t="inlineStr"/>
+      <c r="F27" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: both guards wired into the Multi-Lab Mutations Audit CI
 workflow (.github/workflows/multilab-mutations-audit.yml) as steps:
@@ -1770,24 +1756,24 @@
 (same caveat as the existing guards already in that workflow).</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr"/>
-      <c r="H26" s="2" t="inlineStr"/>
-    </row>
-    <row r="27" ht="90" customHeight="1">
-      <c r="A27" s="3" t="inlineStr">
+      <c r="G27" s="3" t="inlineStr"/>
+      <c r="H27" s="3" t="inlineStr"/>
+    </row>
+    <row r="28" ht="90" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>C35</t>
         </is>
       </c>
-      <c r="B27" s="3" t="inlineStr">
+      <c r="B28" s="2" t="inlineStr">
         <is>
           <t>Legacy /api/studies over-returns studies across labs (was #44)</t>
         </is>
       </c>
-      <c r="C27" s="3" t="inlineStr"/>
-      <c r="D27" s="3" t="inlineStr"/>
-      <c r="E27" s="3" t="inlineStr"/>
-      <c r="F27" s="3" t="inlineStr">
+      <c r="C28" s="2" t="inlineStr"/>
+      <c r="D28" s="2" t="inlineStr"/>
+      <c r="E28" s="2" t="inlineStr"/>
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: GET /api/studies now scopes its list to the active lab
 when one is resolved from the Referer (server/routes.ts), so every returned row
@@ -1797,24 +1783,24 @@
 mirroring the /api/labs/:labId/studies handler. Closed 2026-06-14.</t>
         </is>
       </c>
-      <c r="G27" s="3" t="inlineStr"/>
-      <c r="H27" s="3" t="inlineStr"/>
-    </row>
-    <row r="28" ht="90" customHeight="1">
-      <c r="A28" s="2" t="inlineStr">
+      <c r="G28" s="2" t="inlineStr"/>
+      <c r="H28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29" ht="90" customHeight="1">
+      <c r="A29" s="3" t="inlineStr">
         <is>
           <t>C30</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="B29" s="3" t="inlineStr">
         <is>
           <t>Verify-script convention backfill (was #41)</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr"/>
-      <c r="D28" s="2" t="inlineStr"/>
-      <c r="E28" s="2" t="inlineStr"/>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="C29" s="3" t="inlineStr"/>
+      <c r="D29" s="3" t="inlineStr"/>
+      <c r="E29" s="3" t="inlineStr"/>
+      <c r="F29" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: all 8 high-stakes math/logic commits now ship a paired
 scripts/verify-*.js (EP17 sensitivity, Deming lot-to-lot, CUMSUM+QC+multi-analyte,
@@ -1822,30 +1808,30 @@
 TEa boundary), per the strike-throughs in #41. Closed 2026-06-13.</t>
         </is>
       </c>
-      <c r="G28" s="2" t="inlineStr">
+      <c r="G29" s="3" t="inlineStr">
         <is>
           <t>scripts/audit_verify_script_coverage.py lookback, 2026-06-02; backfills
 landed 2026-06-03..06.
 ---</t>
         </is>
       </c>
-      <c r="H28" s="2" t="inlineStr"/>
-    </row>
-    <row r="29" ht="90" customHeight="1">
-      <c r="A29" s="3" t="inlineStr">
+      <c r="H29" s="3" t="inlineStr"/>
+    </row>
+    <row r="30" ht="90" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>C31</t>
         </is>
       </c>
-      <c r="B29" s="3" t="inlineStr">
+      <c r="B30" s="2" t="inlineStr">
         <is>
           <t>VeritaPT AAA create/update/delete silently no-op in the multi-lab UI</t>
         </is>
       </c>
-      <c r="C29" s="3" t="inlineStr"/>
-      <c r="D29" s="3" t="inlineStr"/>
-      <c r="E29" s="3" t="inlineStr"/>
-      <c r="F29" s="3" t="inlineStr">
+      <c r="C30" s="2" t="inlineStr"/>
+      <c r="D30" s="2" t="inlineStr"/>
+      <c r="E30" s="2" t="inlineStr"/>
+      <c r="F30" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #754 (commit 92ad499) added lab-scoped POST/PUT/DELETE
 /api/labs/:labId/pt/aa-records. The UI posted to the lab-scoped path but only GET
@@ -1856,30 +1842,30 @@
 route mis-filed records to the user's default lab on multi-lab accounts).</t>
         </is>
       </c>
-      <c r="G29" s="3" t="inlineStr">
+      <c r="G30" s="2" t="inlineStr">
         <is>
           <t>2026-06-13, found during #18 Phase 3 QA;
 scripts/audit-labscoped-write-routes.mjs now guards the class.
 ---</t>
         </is>
       </c>
-      <c r="H29" s="3" t="inlineStr"/>
-    </row>
-    <row r="30" ht="90" customHeight="1">
-      <c r="A30" s="2" t="inlineStr">
+      <c r="H30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31" ht="90" customHeight="1">
+      <c r="A31" s="3" t="inlineStr">
         <is>
           <t>C32</t>
         </is>
       </c>
-      <c r="B30" s="2" t="inlineStr">
+      <c r="B31" s="3" t="inlineStr">
         <is>
           <t>VeritaComp "Unlock assessment" false-success no-op</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr"/>
-      <c r="D30" s="2" t="inlineStr"/>
-      <c r="E30" s="2" t="inlineStr"/>
-      <c r="F30" s="2" t="inlineStr">
+      <c r="C31" s="3" t="inlineStr"/>
+      <c r="D31" s="3" t="inlineStr"/>
+      <c r="E31" s="3" t="inlineStr"/>
+      <c r="F31" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #755 (commit 4234007) moved the unlock route to
 /api/labs/:labId/competency/assessments/:id/unlock (the path the client calls).
@@ -1890,29 +1876,29 @@
 HTML).</t>
         </is>
       </c>
-      <c r="G30" s="2" t="inlineStr">
+      <c r="G31" s="3" t="inlineStr">
         <is>
           <t>2026-06-13, found by scripts/audit-labscoped-write-routes.mjs.
 ---</t>
         </is>
       </c>
-      <c r="H30" s="2" t="inlineStr"/>
-    </row>
-    <row r="31" ht="90" customHeight="1">
-      <c r="A31" s="3" t="inlineStr">
+      <c r="H31" s="3" t="inlineStr"/>
+    </row>
+    <row r="32" ht="90" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t>C33</t>
         </is>
       </c>
-      <c r="B31" s="3" t="inlineStr">
+      <c r="B32" s="2" t="inlineStr">
         <is>
           <t>FK-cascade delete 500s + NavBar laptop-width overflow</t>
         </is>
       </c>
-      <c r="C31" s="3" t="inlineStr"/>
-      <c r="D31" s="3" t="inlineStr"/>
-      <c r="E31" s="3" t="inlineStr"/>
-      <c r="F31" s="3" t="inlineStr">
+      <c r="C32" s="2" t="inlineStr"/>
+      <c r="D32" s="2" t="inlineStr"/>
+      <c r="E32" s="2" t="inlineStr"/>
+      <c r="F32" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PRs #749/#750 fixed NavBar horizontal overflow at laptop
 widths (collapse to the hamburger below 1560px); prod-verified at 1280-1920 with the
@@ -1923,37 +1909,9 @@
 500 -&gt; 200. scripts/audit-delete-cascades.mjs guards the class.</t>
         </is>
       </c>
-      <c r="G31" s="3" t="inlineStr">
+      <c r="G32" s="2" t="inlineStr">
         <is>
           <t>2026-06-13 browser QA of the A7-D4 wave + retro-QC of the 72h PR window.
----</t>
-        </is>
-      </c>
-      <c r="H31" s="3" t="inlineStr"/>
-    </row>
-    <row r="32" ht="90" customHeight="1">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>C1</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>FAQ "over 25 years" -&gt; "over 23 years"</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr"/>
-      <c r="D32" s="2" t="inlineStr"/>
-      <c r="E32" s="2" t="inlineStr"/>
-      <c r="F32" s="2" t="inlineStr">
-        <is>
-          <t>Closure evidence: client/src/pages/FAQPage.tsx line 20 reads "over
-23 years" as of 2026-05-01.</t>
-        </is>
-      </c>
-      <c r="G32" s="2" t="inlineStr">
-        <is>
-          <t>session 299e9a73 turn 14, ~2026-04-28.
 ---</t>
         </is>
       </c>
@@ -1962,18 +1920,46 @@
     <row r="33" ht="90" customHeight="1">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>C5</t>
+          <t>C1</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>David's VeritaQA grey-button bug (seat permissions mode)</t>
+          <t>FAQ "over 25 years" -&gt; "over 23 years"</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr"/>
       <c r="D33" s="3" t="inlineStr"/>
       <c r="E33" s="3" t="inlineStr"/>
       <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>Closure evidence: client/src/pages/FAQPage.tsx line 20 reads "over
+23 years" as of 2026-05-01.</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>session 299e9a73 turn 14, ~2026-04-28.
+---</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr"/>
+    </row>
+    <row r="34" ht="90" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>David's VeritaQA grey-button bug (seat permissions mode)</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr"/>
+      <c r="D34" s="2" t="inlineStr"/>
+      <c r="E34" s="2" t="inlineStr"/>
+      <c r="F34" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #10 squash-merged as commit a43fbba on
 2026-05-01 23:19 MST. Railway deploy succeeded; deployed bundle
@@ -1986,7 +1972,7 @@
 against his exact stored shape (14 of 14 expected outcomes matched).</t>
         </is>
       </c>
-      <c r="G33" s="3" t="inlineStr">
+      <c r="G34" s="2" t="inlineStr">
         <is>
           <t>2026-05-01 David's report; veritabench + veritastock
 weren't in MODULE_LIST so seat permissions silently defaulted to
@@ -1994,46 +1980,17 @@
 ---</t>
         </is>
       </c>
-      <c r="H33" s="3" t="inlineStr"/>
-    </row>
-    <row r="34" ht="90" customHeight="1">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>C2</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>TeamPage present-tense "TJC surveyor" check</t>
-        </is>
-      </c>
-      <c r="C34" s="2" t="inlineStr"/>
-      <c r="D34" s="2" t="inlineStr"/>
-      <c r="E34" s="2" t="inlineStr"/>
-      <c r="F34" s="2" t="inlineStr">
-        <is>
-          <t>Closure evidence: site-wide search confirmed all surveyor language
-is past-tense, consistent with user's 2021-2025 service. User closed
-the item in session 299e9a73 turn 4.</t>
-        </is>
-      </c>
-      <c r="G34" s="2" t="inlineStr">
-        <is>
-          <t>session 299e9a73, ~2026-04-28.
----</t>
-        </is>
-      </c>
       <c r="H34" s="2" t="inlineStr"/>
     </row>
     <row r="35" ht="90" customHeight="1">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>C3</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>My Studies CSV/XLSX export (John as design partner)</t>
+          <t>TeamPage present-tense "TJC surveyor" check</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr"/>
@@ -2041,14 +1998,14 @@
       <c r="E35" s="3" t="inlineStr"/>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: client/src/pages/DashboardPage.tsx line 46 calls
-/api/my-studies/export. server/routes.ts line 1491 implements the
-endpoint. Pulled forward into pre-COLA per user instruction.</t>
+          <t>Closure evidence: site-wide search confirmed all surveyor language
+is past-tense, consistent with user's 2021-2025 service. User closed
+the item in session 299e9a73 turn 4.</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>session 299e9a73 turn 5, ~2026-04-28.
+          <t>session 299e9a73, ~2026-04-28.
 ---</t>
         </is>
       </c>
@@ -2057,12 +2014,12 @@
     <row r="36" ht="90" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>C4</t>
+          <t>C3</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Rotate GitHub PAT (because old PAT was committed in SESSION_HANDOFF files)</t>
+          <t>My Studies CSV/XLSX export (John as design partner)</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr"/>
@@ -2070,13 +2027,14 @@
       <c r="E36" s="2" t="inlineStr"/>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: no ghp_* or github_pat_* patterns in current
-SESSION_HANDOFF.md or SESSION_HANDOFF-2.md as of 2026-05-01.</t>
+          <t>Closure evidence: client/src/pages/DashboardPage.tsx line 46 calls
+/api/my-studies/export. server/routes.ts line 1491 implements the
+endpoint. Pulled forward into pre-COLA per user instruction.</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>session 299e9a73, ~2026-04-28.
+          <t>session 299e9a73 turn 5, ~2026-04-28.
 ---</t>
         </is>
       </c>
@@ -2085,18 +2043,46 @@
     <row r="37" ht="90" customHeight="1">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>C6</t>
+          <t>C4</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>VeritaPolicy service-line filtering removed (formerly #4)</t>
+          <t>Rotate GitHub PAT (because old PAT was committed in SESSION_HANDOFF files)</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr"/>
       <c r="D37" s="3" t="inlineStr"/>
       <c r="E37" s="3" t="inlineStr"/>
       <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>Closure evidence: no ghp_* or github_pat_* patterns in current
+SESSION_HANDOFF.md or SESSION_HANDOFF-2.md as of 2026-05-01.</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>session 299e9a73, ~2026-04-28.
+---</t>
+        </is>
+      </c>
+      <c r="H37" s="3" t="inlineStr"/>
+    </row>
+    <row r="38" ht="90" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>C6</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>VeritaPolicy service-line filtering removed (formerly #4)</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr"/>
+      <c r="D38" s="2" t="inlineStr"/>
+      <c r="E38" s="2" t="inlineStr"/>
+      <c r="F38" s="2" t="inlineStr">
         <is>
           <t>Closure rationale (operator decision 2026-05-10): Keep all
 VeritaPolicy rows. CFR-only references with no accreditor reference
@@ -2105,29 +2091,29 @@
 report misread the design intent.</t>
         </is>
       </c>
-      <c r="G37" s="3" t="inlineStr">
+      <c r="G38" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H37" s="3" t="inlineStr"/>
-    </row>
-    <row r="38" ht="90" customHeight="1">
-      <c r="A38" s="2" t="inlineStr">
+      <c r="H38" s="2" t="inlineStr"/>
+    </row>
+    <row r="39" ht="90" customHeight="1">
+      <c r="A39" s="3" t="inlineStr">
         <is>
           <t>C7</t>
         </is>
       </c>
-      <c r="B38" s="2" t="inlineStr">
+      <c r="B39" s="3" t="inlineStr">
         <is>
           <t>CLIA number format validation (formerly #13)</t>
         </is>
       </c>
-      <c r="C38" s="2" t="inlineStr"/>
-      <c r="D38" s="2" t="inlineStr"/>
-      <c r="E38" s="2" t="inlineStr"/>
-      <c r="F38" s="2" t="inlineStr">
+      <c r="C39" s="3" t="inlineStr"/>
+      <c r="D39" s="3" t="inlineStr"/>
+      <c r="E39" s="3" t="inlineStr"/>
+      <c r="F39" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: shared/validateClia.ts defines CLIA_REGEX =
 /^\d{2}D\d{7}$/ (line 24), validateClia() helper with whitespace
@@ -2138,30 +2124,30 @@
 shape exists and behaves as specified.</t>
         </is>
       </c>
-      <c r="G38" s="2" t="inlineStr">
+      <c r="G39" s="3" t="inlineStr">
         <is>
           <t>Agent verification 2026-05-10 via grep + file read.
 Operator confirmed shipped 2026-05-10.
 ---</t>
         </is>
       </c>
-      <c r="H38" s="2" t="inlineStr"/>
-    </row>
-    <row r="39" ht="90" customHeight="1">
-      <c r="A39" s="3" t="inlineStr">
+      <c r="H39" s="3" t="inlineStr"/>
+    </row>
+    <row r="40" ht="90" customHeight="1">
+      <c r="A40" s="2" t="inlineStr">
         <is>
           <t>C8</t>
         </is>
       </c>
-      <c r="B39" s="3" t="inlineStr">
+      <c r="B40" s="2" t="inlineStr">
         <is>
           <t>VeritaMap lab-wide menu toggle (formerly #19)</t>
         </is>
       </c>
-      <c r="C39" s="3" t="inlineStr"/>
-      <c r="D39" s="3" t="inlineStr"/>
-      <c r="E39" s="3" t="inlineStr"/>
-      <c r="F39" s="3" t="inlineStr">
+      <c r="C40" s="2" t="inlineStr"/>
+      <c r="D40" s="2" t="inlineStr"/>
+      <c r="E40" s="2" t="inlineStr"/>
+      <c r="F40" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: client/src/pages/VeritaMapLabwidePage.tsx
 exists and implements the labwide read-only union view. Route is
@@ -2171,59 +2157,59 @@
 parking lot plan (read-only union view, per-session toggle) shipped.</t>
         </is>
       </c>
-      <c r="G39" s="3" t="inlineStr">
+      <c r="G40" s="2" t="inlineStr">
         <is>
           <t>Agent verification 2026-05-10 via grep + file read.
 Operator confirmed shipped 2026-05-10.
 ---</t>
         </is>
       </c>
-      <c r="H39" s="3" t="inlineStr"/>
-    </row>
-    <row r="40" ht="90" customHeight="1">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t>C9</t>
-        </is>
-      </c>
-      <c r="B40" s="2" t="inlineStr">
-        <is>
-          <t>Tier-1 smoke test checklist (formerly #6)</t>
-        </is>
-      </c>
-      <c r="C40" s="2" t="inlineStr"/>
-      <c r="D40" s="2" t="inlineStr"/>
-      <c r="E40" s="2" t="inlineStr"/>
-      <c r="F40" s="2" t="inlineStr">
-        <is>
-          <t>Closure evidence: docs/smoke-test-tier1.md documents the Tier-1
-smoke-test process and post-deploy verification steps. Shipped via
-PR #81 as part of the 2026-05-10 wave.</t>
-        </is>
-      </c>
-      <c r="G40" s="2" t="inlineStr">
-        <is>
-          <t>Operator instruction 2026-05-10 in this session.
----</t>
-        </is>
-      </c>
       <c r="H40" s="2" t="inlineStr"/>
     </row>
     <row r="41" ht="90" customHeight="1">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>C10</t>
+          <t>C9</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>Per-module gating (formerly #7)</t>
+          <t>Tier-1 smoke test checklist (formerly #6)</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr"/>
       <c r="D41" s="3" t="inlineStr"/>
       <c r="E41" s="3" t="inlineStr"/>
       <c r="F41" s="3" t="inlineStr">
+        <is>
+          <t>Closure evidence: docs/smoke-test-tier1.md documents the Tier-1
+smoke-test process and post-deploy verification steps. Shipped via
+PR #81 as part of the 2026-05-10 wave.</t>
+        </is>
+      </c>
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>Operator instruction 2026-05-10 in this session.
+---</t>
+        </is>
+      </c>
+      <c r="H41" s="3" t="inlineStr"/>
+    </row>
+    <row r="42" ht="90" customHeight="1">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>C10</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Per-module gating (formerly #7)</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr"/>
+      <c r="D42" s="2" t="inlineStr"/>
+      <c r="E42" s="2" t="inlineStr"/>
+      <c r="F42" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: Client-side useIsReadOnly module keys wired
 on client/src/pages/VeritaPolicyAppPage.tsx and
@@ -2238,29 +2224,29 @@
 PR #76.</t>
         </is>
       </c>
-      <c r="G41" s="3" t="inlineStr">
+      <c r="G42" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H41" s="3" t="inlineStr"/>
-    </row>
-    <row r="42" ht="90" customHeight="1">
-      <c r="A42" s="2" t="inlineStr">
+      <c r="H42" s="2" t="inlineStr"/>
+    </row>
+    <row r="43" ht="90" customHeight="1">
+      <c r="A43" s="3" t="inlineStr">
         <is>
           <t>C11</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
+      <c r="B43" s="3" t="inlineStr">
         <is>
           <t>VeritaStock shipped copy (formerly #8)</t>
         </is>
       </c>
-      <c r="C42" s="2" t="inlineStr"/>
-      <c r="D42" s="2" t="inlineStr"/>
-      <c r="E42" s="2" t="inlineStr"/>
-      <c r="F42" s="2" t="inlineStr">
+      <c r="C43" s="3" t="inlineStr"/>
+      <c r="D43" s="3" t="inlineStr"/>
+      <c r="E43" s="3" t="inlineStr"/>
+      <c r="F43" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: client/src/pages/ArticleInventoryManagementPage.tsx
 line 305 footer reads "platform that includes VeritaStock™" instead
@@ -2268,29 +2254,29 @@
 on /resources/laboratory-inventory-management. Shipped via PR #75.</t>
         </is>
       </c>
-      <c r="G42" s="2" t="inlineStr">
+      <c r="G43" s="3" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
 ---</t>
         </is>
       </c>
-      <c r="H42" s="2" t="inlineStr"/>
-    </row>
-    <row r="43" ht="90" customHeight="1">
-      <c r="A43" s="3" t="inlineStr">
+      <c r="H43" s="3" t="inlineStr"/>
+    </row>
+    <row r="44" ht="90" customHeight="1">
+      <c r="A44" s="2" t="inlineStr">
         <is>
           <t>C12</t>
         </is>
       </c>
-      <c r="B43" s="3" t="inlineStr">
+      <c r="B44" s="2" t="inlineStr">
         <is>
           <t>Admin report one-row-per-lab (formerly #14)</t>
         </is>
       </c>
-      <c r="C43" s="3" t="inlineStr"/>
-      <c r="D43" s="3" t="inlineStr"/>
-      <c r="E43" s="3" t="inlineStr"/>
-      <c r="F43" s="3" t="inlineStr">
+      <c r="C44" s="2" t="inlineStr"/>
+      <c r="D44" s="2" t="inlineStr"/>
+      <c r="E44" s="2" t="inlineStr"/>
+      <c r="F44" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: /api/admin/report rewritten in
 server/routes.ts (~line 595) to LEFT JOIN labs on
@@ -2305,33 +2291,6 @@
 prerequisite, not a code bug). Shipped via PR #85.</t>
         </is>
       </c>
-      <c r="G43" s="3" t="inlineStr">
-        <is>
-          <t>Operator instruction 2026-05-10 in this session.
----</t>
-        </is>
-      </c>
-      <c r="H43" s="3" t="inlineStr"/>
-    </row>
-    <row r="44" ht="90" customHeight="1">
-      <c r="A44" s="2" t="inlineStr">
-        <is>
-          <t>C14</t>
-        </is>
-      </c>
-      <c r="B44" s="2" t="inlineStr">
-        <is>
-          <t>UI relabel "CLIA TEa" -&gt; "Lab-Set Internal Goal" (formerly #1)</t>
-        </is>
-      </c>
-      <c r="C44" s="2" t="inlineStr"/>
-      <c r="D44" s="2" t="inlineStr"/>
-      <c r="E44" s="2" t="inlineStr"/>
-      <c r="F44" s="2" t="inlineStr">
-        <is>
-          <t>Closure evidence: Shipped across four PRs over 2026-05-10.</t>
-        </is>
-      </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
@@ -2343,18 +2302,45 @@
     <row r="45" ht="90" customHeight="1">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>C13</t>
+          <t>C14</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>WSLH PT vendor (formerly #15)</t>
+          <t>UI relabel "CLIA TEa" -&gt; "Lab-Set Internal Goal" (formerly #1)</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr"/>
       <c r="D45" s="3" t="inlineStr"/>
       <c r="E45" s="3" t="inlineStr"/>
       <c r="F45" s="3" t="inlineStr">
+        <is>
+          <t>Closure evidence: Shipped across four PRs over 2026-05-10.</t>
+        </is>
+      </c>
+      <c r="G45" s="3" t="inlineStr">
+        <is>
+          <t>Operator instruction 2026-05-10 in this session.
+---</t>
+        </is>
+      </c>
+      <c r="H45" s="3" t="inlineStr"/>
+    </row>
+    <row r="46" ht="90" customHeight="1">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>C13</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>WSLH PT vendor (formerly #15)</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr"/>
+      <c r="D46" s="2" t="inlineStr"/>
+      <c r="E46" s="2" t="inlineStr"/>
+      <c r="F46" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: Shipped 2026-05-10 via PR #79 (merge commit
 eeebc6e; merged after rebase to resolve a server/db.ts collision
@@ -2372,38 +2358,9 @@
 'WSLH' is the post-deploy success signal. Shipped via PR #79.</t>
         </is>
       </c>
-      <c r="G45" s="3" t="inlineStr">
+      <c r="G46" s="2" t="inlineStr">
         <is>
           <t>Operator instruction 2026-05-10 in this session.
----</t>
-        </is>
-      </c>
-      <c r="H45" s="3" t="inlineStr"/>
-    </row>
-    <row r="46" ht="90" customHeight="1">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>C15</t>
-        </is>
-      </c>
-      <c r="B46" s="2" t="inlineStr">
-        <is>
-          <t>VeritaStock lot tracking + expiration + reorder alerts (formerly #21)</t>
-        </is>
-      </c>
-      <c r="C46" s="2" t="inlineStr"/>
-      <c r="D46" s="2" t="inlineStr"/>
-      <c r="E46" s="2" t="inlineStr"/>
-      <c r="F46" s="2" t="inlineStr">
-        <is>
-          <t>Closure evidence: VeritaStock™ shipped the bench-level inventory
-features the Perplexity competitor analysis identified as a gap:</t>
-        </is>
-      </c>
-      <c r="G46" s="2" t="inlineStr">
-        <is>
-          <t>Originally Perplexity competitor analysis 2026-05-10.
-Audit 2026-05-21 confirmed the feature set ships today.
 ---</t>
         </is>
       </c>
@@ -2412,12 +2369,12 @@
     <row r="47" ht="90" customHeight="1">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>C16</t>
+          <t>C15</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>PAL studies guided workflow (formerly #23)</t>
+          <t>VeritaStock lot tracking + expiration + reorder alerts (formerly #21)</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr"/>
@@ -2425,15 +2382,14 @@
       <c r="E47" s="3" t="inlineStr"/>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: VeritaCheck™ already ships the Precision /
-Accuracy / Linearity (PAL) study set under EP-protocol naming:</t>
+          <t>Closure evidence: VeritaStock™ shipped the bench-level inventory
+features the Perplexity competitor analysis identified as a gap:</t>
         </is>
       </c>
       <c r="G47" s="3" t="inlineStr">
         <is>
           <t>Originally Perplexity competitor analysis 2026-05-10.
-Audit 2026-05-21 confirmed the EP studies cover the PAL framing in
-full.
+Audit 2026-05-21 confirmed the feature set ships today.
 ---</t>
         </is>
       </c>
@@ -2442,12 +2398,12 @@
     <row r="48" ht="90" customHeight="1">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>C17</t>
+          <t>C16</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Source-grounded 21/29/45 CFR + 42 CFR 482-485 (formerly #26)</t>
+          <t>PAL studies guided workflow (formerly #23)</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr"/>
@@ -2455,35 +2411,65 @@
       <c r="E48" s="2" t="inlineStr"/>
       <c r="F48" s="2" t="inlineStr">
         <is>
+          <t>Closure evidence: VeritaCheck™ already ships the Precision /
+Accuracy / Linearity (PAL) study set under EP-protocol naming:</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>Originally Perplexity competitor analysis 2026-05-10.
+Audit 2026-05-21 confirmed the EP studies cover the PAL framing in
+full.
+---</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr"/>
+    </row>
+    <row r="49" ht="90" customHeight="1">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>C17</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>Source-grounded 21/29/45 CFR + 42 CFR 482-485 (formerly #26)</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr"/>
+      <c r="D49" s="3" t="inlineStr"/>
+      <c r="E49" s="3" t="inlineStr"/>
+      <c r="F49" s="3" t="inlineStr">
+        <is>
           <t>Closure evidence: PR #301 (commit 8c27806, merged 2026-05-21)
 source-grounded the 74 remaining non-493 entries in
 server/cfrRequirements.ts against verbatim eCFR XML. Breakdown
 shipped:</t>
         </is>
       </c>
-      <c r="G48" s="2" t="inlineStr">
+      <c r="G49" s="3" t="inlineStr">
         <is>
           <t>PR #301; tasks #18 in the in-session task tracker.
 ---</t>
         </is>
       </c>
-      <c r="H48" s="2" t="inlineStr"/>
-    </row>
-    <row r="49" ht="90" customHeight="1">
-      <c r="A49" s="3" t="inlineStr">
+      <c r="H49" s="3" t="inlineStr"/>
+    </row>
+    <row r="50" ht="90" customHeight="1">
+      <c r="A50" s="2" t="inlineStr">
         <is>
           <t>C18</t>
         </is>
       </c>
-      <c r="B49" s="3" t="inlineStr">
+      <c r="B50" s="2" t="inlineStr">
         <is>
           <t>VeritaPolicy "Non CLIA" chapter rename (formerly #3)</t>
         </is>
       </c>
-      <c r="C49" s="3" t="inlineStr"/>
-      <c r="D49" s="3" t="inlineStr"/>
-      <c r="E49" s="3" t="inlineStr"/>
-      <c r="F49" s="3" t="inlineStr">
+      <c r="C50" s="2" t="inlineStr"/>
+      <c r="D50" s="2" t="inlineStr"/>
+      <c r="E50" s="2" t="inlineStr"/>
+      <c r="F50" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: PR #300 (commit 34d7707, merged 2026-05-21)
 renamed all 44 user-facing chapter labels in
@@ -2494,7 +2480,7 @@
 page.</t>
         </is>
       </c>
-      <c r="G49" s="3" t="inlineStr">
+      <c r="G50" s="2" t="inlineStr">
         <is>
           <t>CAP customer screenshot of the /veritapolicy chapter
 headers, 2026-05-01 evening. PR #300; tasks #17 in the in-session
@@ -2502,23 +2488,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H49" s="3" t="inlineStr"/>
-    </row>
-    <row r="50" ht="90" customHeight="1">
-      <c r="A50" s="2" t="inlineStr">
+      <c r="H50" s="2" t="inlineStr"/>
+    </row>
+    <row r="51" ht="90" customHeight="1">
+      <c r="A51" s="3" t="inlineStr">
         <is>
           <t>C19</t>
         </is>
       </c>
-      <c r="B50" s="2" t="inlineStr">
+      <c r="B51" s="3" t="inlineStr">
         <is>
           <t>VeritaStock department-scope toggle (formerly #31)</t>
         </is>
       </c>
-      <c r="C50" s="2" t="inlineStr"/>
-      <c r="D50" s="2" t="inlineStr"/>
-      <c r="E50" s="2" t="inlineStr"/>
-      <c r="F50" s="2" t="inlineStr">
+      <c r="C51" s="3" t="inlineStr"/>
+      <c r="D51" s="3" t="inlineStr"/>
+      <c r="E51" s="3" t="inlineStr"/>
+      <c r="F51" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #319 (commit d01f5fe, merged 2026-05-22)
 shipped the persistent dept-scope toggle on VeritaStockPage. A new
@@ -2529,7 +2515,7 @@
 workspace without re-filtering.</t>
         </is>
       </c>
-      <c r="G50" s="2" t="inlineStr">
+      <c r="G51" s="3" t="inlineStr">
         <is>
           <t>John, San Carlos lab, 2026-05-21. Same conversation that
 drove the vendor dropdown (PR #304), FILTERED VIEW banner (PR #305),
@@ -2537,23 +2523,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H50" s="2" t="inlineStr"/>
-    </row>
-    <row r="51" ht="90" customHeight="1">
-      <c r="A51" s="3" t="inlineStr">
+      <c r="H51" s="3" t="inlineStr"/>
+    </row>
+    <row r="52" ht="90" customHeight="1">
+      <c r="A52" s="2" t="inlineStr">
         <is>
           <t>C20</t>
         </is>
       </c>
-      <c r="B51" s="3" t="inlineStr">
+      <c r="B52" s="2" t="inlineStr">
         <is>
           <t>Primary-lab seat counting (formerly #12)</t>
         </is>
       </c>
-      <c r="C51" s="3" t="inlineStr"/>
-      <c r="D51" s="3" t="inlineStr"/>
-      <c r="E51" s="3" t="inlineStr"/>
-      <c r="F51" s="3" t="inlineStr">
+      <c r="C52" s="2" t="inlineStr"/>
+      <c r="D52" s="2" t="inlineStr"/>
+      <c r="E52" s="2" t="inlineStr"/>
+      <c r="F52" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: is_primary_lab INTEGER NOT NULL DEFAULT 0
 column was added to the lab_members table at db.ts:1276, with the
@@ -2564,7 +2550,7 @@
 is_primary_lab=1 ordering).</t>
         </is>
       </c>
-      <c r="G51" s="3" t="inlineStr">
+      <c r="G52" s="2" t="inlineStr">
         <is>
           <t>2026-05-07 multi-lab discussion. Build shipped as part
 of the Multi-Lab Tier 2 architecture work (Phase 3.x series, prior
@@ -2573,23 +2559,23 @@
 ---</t>
         </is>
       </c>
-      <c r="H51" s="3" t="inlineStr"/>
-    </row>
-    <row r="52" ht="90" customHeight="1">
-      <c r="A52" s="2" t="inlineStr">
+      <c r="H52" s="2" t="inlineStr"/>
+    </row>
+    <row r="53" ht="90" customHeight="1">
+      <c r="A53" s="3" t="inlineStr">
         <is>
           <t>C21</t>
         </is>
       </c>
-      <c r="B52" s="2" t="inlineStr">
+      <c r="B53" s="3" t="inlineStr">
         <is>
           <t>Multi-lab pricing model — Option A (formerly #11)</t>
         </is>
       </c>
-      <c r="C52" s="2" t="inlineStr"/>
-      <c r="D52" s="2" t="inlineStr"/>
-      <c r="E52" s="2" t="inlineStr"/>
-      <c r="F52" s="2" t="inlineStr">
+      <c r="C53" s="3" t="inlineStr"/>
+      <c r="D53" s="3" t="inlineStr"/>
+      <c r="E53" s="3" t="inlineStr"/>
+      <c r="F53" s="3" t="inlineStr">
         <is>
           <t>Closure evidence: PR #322 (commit 0ccd925, merged 2026-05-22)
 added the customer-facing line to the pricing page that reflects
@@ -2602,7 +2588,7 @@
 Enterprise+ block, reads:</t>
         </is>
       </c>
-      <c r="G52" s="2" t="inlineStr">
+      <c r="G53" s="3" t="inlineStr">
         <is>
           <t>2026-05-07 multi-lab discussion (Lisa Veri's
 canonical-case session). PR #322 (initial build); softening PR
@@ -2611,30 +2597,30 @@
 ---</t>
         </is>
       </c>
-      <c r="H52" s="2" t="inlineStr"/>
-    </row>
-    <row r="53" ht="90" customHeight="1">
-      <c r="A53" s="3" t="inlineStr">
+      <c r="H53" s="3" t="inlineStr"/>
+    </row>
+    <row r="54" ht="90" customHeight="1">
+      <c r="A54" s="2" t="inlineStr">
         <is>
           <t>C22</t>
         </is>
       </c>
-      <c r="B53" s="3" t="inlineStr">
+      <c r="B54" s="2" t="inlineStr">
         <is>
           <t>VeritaOps cost-per-test module (formerly #10)</t>
         </is>
       </c>
-      <c r="C53" s="3" t="inlineStr"/>
-      <c r="D53" s="3" t="inlineStr"/>
-      <c r="E53" s="3" t="inlineStr"/>
-      <c r="F53" s="3" t="inlineStr">
+      <c r="C54" s="2" t="inlineStr"/>
+      <c r="D54" s="2" t="inlineStr"/>
+      <c r="E54" s="2" t="inlineStr"/>
+      <c r="F54" s="2" t="inlineStr">
         <is>
           <t>Closure evidence: v1 of the VeritaOps Cost-Per-Reportable-Test
 (CPRT) module shipped across PR #325 through PR #330 on 2026-05-22.
 The module is feature-complete for the typical lab director workflow.</t>
         </is>
       </c>
-      <c r="G53" s="3" t="inlineStr">
+      <c r="G54" s="2" t="inlineStr">
         <is>
           <t>This thread, 2026-05-07 12:05 PM CDT, user message:
 "Parking lot: build an operations module for cost per test
@@ -2643,262 +2629,262 @@
 ---</t>
         </is>
       </c>
-      <c r="H53" s="3" t="inlineStr"/>
-    </row>
-    <row r="54" ht="90" customHeight="1">
-      <c r="A54" s="2" t="inlineStr">
+      <c r="H54" s="2" t="inlineStr"/>
+    </row>
+    <row r="55" ht="90" customHeight="1">
+      <c r="A55" s="3" t="inlineStr">
         <is>
           <t>C23</t>
         </is>
       </c>
-      <c r="B54" s="2" t="inlineStr">
+      <c r="B55" s="3" t="inlineStr">
         <is>
           <t>CCL lab name visual disambiguation in lab switcher (formerly #34)</t>
         </is>
       </c>
-      <c r="C54" s="2" t="inlineStr"/>
-      <c r="D54" s="2" t="inlineStr">
+      <c r="C55" s="3" t="inlineStr"/>
+      <c r="D55" s="3" t="inlineStr">
         <is>
           <t>XS (under 1 day, actual)</t>
         </is>
       </c>
-      <c r="E54" s="2" t="inlineStr">
+      <c r="E55" s="3" t="inlineStr">
         <is>
           <t>Low — cosmetic; only mattered when Lisa or Michael picked the wrong lab from...</t>
         </is>
       </c>
-      <c r="F54" s="2" t="inlineStr">
+      <c r="F55" s="3" t="inlineStr">
         <is>
           <t>Effort: XS (under 1 day, actual)
 Importance: Low — cosmetic; only mattered when Lisa or Michael picked the wrong lab from the dropdown.</t>
         </is>
       </c>
-      <c r="G54" s="2" t="inlineStr">
+      <c r="G55" s="3" t="inlineStr">
         <is>
           <t>flagged 2026-05-23 immediately after provisioning Lisa's CCL lab; closed 2026-05-24.
 ---</t>
         </is>
       </c>
-      <c r="H54" s="2" t="inlineStr"/>
-    </row>
-    <row r="55" ht="90" customHeight="1">
-      <c r="A55" s="3" t="inlineStr">
+      <c r="H55" s="3" t="inlineStr"/>
+    </row>
+    <row r="56" ht="90" customHeight="1">
+      <c r="A56" s="2" t="inlineStr">
         <is>
           <t>C24</t>
         </is>
       </c>
-      <c r="B55" s="3" t="inlineStr">
+      <c r="B56" s="2" t="inlineStr">
         <is>
           <t>VC Unlimited Y1/Y2 price disclosure UX (formerly #35)</t>
         </is>
       </c>
-      <c r="C55" s="3" t="inlineStr"/>
-      <c r="D55" s="3" t="inlineStr">
+      <c r="C56" s="2" t="inlineStr"/>
+      <c r="D56" s="2" t="inlineStr">
         <is>
           <t>XS (under 1 day, actual)</t>
         </is>
       </c>
-      <c r="E55" s="3" t="inlineStr">
+      <c r="E56" s="2" t="inlineStr">
         <is>
           <t>Low when shipped (proactive, no customer complaint yet) — but high if a procu...</t>
         </is>
       </c>
-      <c r="F55" s="3" t="inlineStr">
+      <c r="F56" s="2" t="inlineStr">
         <is>
           <t>Effort: XS (under 1 day, actual)
 Importance: Low when shipped (proactive, no customer complaint yet) — but high if a procurement reviewer later disputes the $499 renewal as undisclosed.</t>
         </is>
       </c>
-      <c r="G55" s="3" t="inlineStr">
+      <c r="G56" s="2" t="inlineStr">
         <is>
           <t>Pricing rebuild 2026-05-23; closed 2026-05-24 proactively before any customer dispute.
 ---</t>
         </is>
       </c>
-      <c r="H55" s="3" t="inlineStr"/>
-    </row>
-    <row r="56" ht="90" customHeight="1">
-      <c r="A56" s="2" t="inlineStr">
+      <c r="H56" s="2" t="inlineStr"/>
+    </row>
+    <row r="57" ht="90" customHeight="1">
+      <c r="A57" s="3" t="inlineStr">
         <is>
           <t>C25</t>
         </is>
       </c>
-      <c r="B56" s="2" t="inlineStr">
+      <c r="B57" s="3" t="inlineStr">
         <is>
           <t>VeritaQC Phase 1 (Levey-Jennings + Westgard live engine) (formerly #20)</t>
         </is>
       </c>
-      <c r="C56" s="2" t="inlineStr"/>
-      <c r="D56" s="2" t="inlineStr">
+      <c r="C57" s="3" t="inlineStr"/>
+      <c r="D57" s="3" t="inlineStr">
         <is>
           <t>L (about 5 days end-to-end, actual: Phase 0 schema → Phase 1A evaluator → 1B...</t>
         </is>
       </c>
-      <c r="E56" s="2" t="inlineStr">
+      <c r="E57" s="3" t="inlineStr">
         <is>
           <t>High — largest single gap vs myLabCompliance.io per Perplexity competitor ana...</t>
         </is>
       </c>
-      <c r="F56" s="2" t="inlineStr">
+      <c r="F57" s="3" t="inlineStr">
         <is>
           <t>Effort: L (about 5 days end-to-end, actual: Phase 0 schema → Phase 1A evaluator → 1B entry UI → 1C daily review → 1D monthly PDF + attestation)
 Importance: High — largest single gap vs myLabCompliance.io per Perplexity competitor analysis; promotes VeritaAssure from documentation tool to lab operations platform.</t>
         </is>
       </c>
-      <c r="G56" s="2" t="inlineStr">
+      <c r="G57" s="3" t="inlineStr">
         <is>
           <t>Perplexity competitor analysis 2026-05-10. Scoping confirmed via the build_phase1_mockup.py iterations 2026-05-24. Shipped 2026-05-25.
 ---</t>
         </is>
       </c>
-      <c r="H56" s="2" t="inlineStr"/>
-    </row>
-    <row r="57" ht="90" customHeight="1">
-      <c r="A57" s="3" t="inlineStr">
+      <c r="H57" s="3" t="inlineStr"/>
+    </row>
+    <row r="58" ht="90" customHeight="1">
+      <c r="A58" s="2" t="inlineStr">
         <is>
           <t>C26</t>
         </is>
       </c>
-      <c r="B57" s="3" t="inlineStr">
+      <c r="B58" s="2" t="inlineStr">
         <is>
           <t>VeritaLab CMS-116 application support + state licensing registry (formerly #22)</t>
         </is>
       </c>
-      <c r="C57" s="3" t="inlineStr"/>
-      <c r="D57" s="3" t="inlineStr">
+      <c r="C58" s="2" t="inlineStr"/>
+      <c r="D58" s="2" t="inlineStr">
         <is>
           <t>M (1-2 weeks for v1, actual)</t>
         </is>
       </c>
-      <c r="E57" s="3" t="inlineStr">
+      <c r="E58" s="2" t="inlineStr">
         <is>
           <t>Medium — competitor parity (myLabCompliance.io) plus useful at lab startup an...</t>
         </is>
       </c>
-      <c r="F57" s="3" t="inlineStr">
+      <c r="F58" s="2" t="inlineStr">
         <is>
           <t>Effort: M (1-2 weeks for v1, actual)
 Importance: Medium — competitor parity (myLabCompliance.io) plus useful at lab startup and at certificate-type changes.</t>
         </is>
       </c>
-      <c r="G57" s="3" t="inlineStr">
+      <c r="G58" s="2" t="inlineStr">
         <is>
           <t>Perplexity competitor analysis (myLabCompliance.io), 2026-05-10. Reclassified as a VeritaLab extension 2026-05-25. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H57" s="3" t="inlineStr"/>
-    </row>
-    <row r="58" ht="90" customHeight="1">
-      <c r="A58" s="2" t="inlineStr">
+      <c r="H58" s="2" t="inlineStr"/>
+    </row>
+    <row r="59" ht="90" customHeight="1">
+      <c r="A59" s="3" t="inlineStr">
         <is>
           <t>C27</t>
         </is>
       </c>
-      <c r="B58" s="2" t="inlineStr">
+      <c r="B59" s="3" t="inlineStr">
         <is>
           <t>Active vs view-only seat split (formerly #33)</t>
         </is>
       </c>
-      <c r="C58" s="2" t="inlineStr"/>
-      <c r="D58" s="2" t="inlineStr">
+      <c r="C59" s="3" t="inlineStr"/>
+      <c r="D59" s="3" t="inlineStr">
         <is>
           <t>M (~1 week of engineering, actual: shipped in a single multi-PR session)</t>
         </is>
       </c>
-      <c r="E58" s="2" t="inlineStr">
+      <c r="E59" s="3" t="inlineStr">
         <is>
           <t>Medium — closed the gap between /pricing copy and product behavior; gives sal...</t>
         </is>
       </c>
-      <c r="F58" s="2" t="inlineStr">
+      <c r="F59" s="3" t="inlineStr">
         <is>
           <t>Effort: M (~1 week of engineering, actual: shipped in a single multi-PR session)
 Importance: Medium — closed the gap between /pricing copy and product behavior; gives sales a clean answer for "do you charge for our medical director?"</t>
         </is>
       </c>
-      <c r="G58" s="2" t="inlineStr">
+      <c r="G59" s="3" t="inlineStr">
         <is>
           <t>Pricing analysis doc Decision 3 (2026-05-21); MEDIUM scenario revised 2026-05-29 to retire the "unlimited view-only" claim. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H58" s="2" t="inlineStr"/>
-    </row>
-    <row r="59" ht="90" customHeight="1">
-      <c r="A59" s="3" t="inlineStr">
+      <c r="H59" s="3" t="inlineStr"/>
+    </row>
+    <row r="60" ht="90" customHeight="1">
+      <c r="A60" s="2" t="inlineStr">
         <is>
           <t>C28</t>
         </is>
       </c>
-      <c r="B59" s="3" t="inlineStr">
+      <c r="B60" s="2" t="inlineStr">
         <is>
           <t>"Why VeritaCheck" comparative one-pager (formerly #37)</t>
         </is>
       </c>
-      <c r="C59" s="3" t="inlineStr"/>
-      <c r="D59" s="3" t="inlineStr">
+      <c r="C60" s="2" t="inlineStr"/>
+      <c r="D60" s="2" t="inlineStr">
         <is>
           <t>S (one design pass + four claim paragraphs + PDF + matching marketing-site pa...</t>
         </is>
       </c>
-      <c r="E59" s="3" t="inlineStr">
+      <c r="E60" s="2" t="inlineStr">
         <is>
           <t>Medium — closed a positioning gap surfaced by six COLA conference attendees a...</t>
         </is>
       </c>
-      <c r="F59" s="3" t="inlineStr">
+      <c r="F60" s="2" t="inlineStr">
         <is>
           <t>Effort: S (one design pass + four claim paragraphs + PDF + matching marketing-site page, actual)
 Importance: Medium — closed a positioning gap surfaced by six COLA conference attendees attached to a legacy verification tool; converts product-quality advantage into a leave-behind Lisa can hand out.</t>
         </is>
       </c>
-      <c r="G59" s="3" t="inlineStr">
+      <c r="G60" s="2" t="inlineStr">
         <is>
           <t>2026-05-11 / 2026-05-12 conference notes review with Michael. Conference attendees (Whitehead, Odegard, Othman, Molinelli, Kyle, Allred) expressed interest in equivalent / superior product. Shipped 2026-05-28.
 ---</t>
         </is>
       </c>
-      <c r="H59" s="3" t="inlineStr"/>
-    </row>
-    <row r="60" ht="90" customHeight="1">
-      <c r="A60" s="2" t="inlineStr">
+      <c r="H60" s="2" t="inlineStr"/>
+    </row>
+    <row r="61" ht="90" customHeight="1">
+      <c r="A61" s="3" t="inlineStr">
         <is>
           <t>C29</t>
         </is>
       </c>
-      <c r="B60" s="2" t="inlineStr">
+      <c r="B61" s="3" t="inlineStr">
         <is>
           <t>VeritaPolicy approval workflow — MediaLab functional mirror</t>
         </is>
       </c>
-      <c r="C60" s="2" t="inlineStr"/>
-      <c r="D60" s="2" t="inlineStr">
+      <c r="C61" s="3" t="inlineStr"/>
+      <c r="D61" s="3" t="inlineStr">
         <is>
           <t>XL (one focused session, 12 PRs landed)</t>
         </is>
       </c>
-      <c r="E60" s="2" t="inlineStr">
+      <c r="E61" s="3" t="inlineStr">
         <is>
           <t>High — replaces MediaLab Document Control ($752/$2,250 starting price, scalin...</t>
         </is>
       </c>
-      <c r="F60" s="2" t="inlineStr">
+      <c r="F61" s="3" t="inlineStr">
         <is>
           <t>Effort: XL (one focused session, 12 PRs landed)
 Importance: High — replaces MediaLab Document Control ($752/$2,250 starting price, scaling to $10K-$20K/yr at enterprise per Capterra public data) with an included VeritaPolicy feature; closes a real positioning gap and gives sales a direct comparator line.</t>
         </is>
       </c>
-      <c r="G60" s="2" t="inlineStr">
+      <c r="G61" s="3" t="inlineStr">
         <is>
           <t>Pricing strategy conversation 2026-05-29 (Michael: "I don't like bolt-ons; we should replicate this") → scoped 8 phases → shipped all 12 PRs in single session. Shipped 2026-05-29.
 ---</t>
         </is>
       </c>
-      <c r="H60" s="2" t="inlineStr"/>
+      <c r="H61" s="3" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H60"/>
+  <autoFilter ref="A1:H61"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
TASK: Promote VeritaQC to Live (#40 verified); close #40 as C60; regen xlsx
PLAN:
  1. VeritaQC badge Phase 1 preview -> Live; all 18 modules Live.
  2. Badge spec updated (no Phase 1 preview).
  3. Close #40 as C60; regen xlsx.

Self-check:
  - #40 browser click-through verified (15 replicates imported); operator-authorized.
  - md + xlsx synced; typecheck clean.
</commit_message>
<xml_diff>
--- a/PARKING_LOT.xlsx
+++ b/PARKING_LOT.xlsx
@@ -12,8 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RETIRED" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$60</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$61</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RETIRED'!$A$1:$H$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -924,55 +924,15 @@
     <row r="10" ht="90" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>42</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>VeritaQC Import Phase A: human-in-the-loop Gate 3 click-through (deferred)</t>
+          <t>Outbound demo-invite messaging campaign to 1st-degree LinkedIn contacts</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Open, awaiting Michael's 5-minute click test. Will move task #77 to completed only after he reports the user-visible result.
----</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>XS (~5 minutes of Michael's time on a live URL).</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>Low. Backend contract is fully verified via 35/35 passing offline contract ch...</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>Effort: XS (~5 minutes of Michael's time on a live URL).
-Importance: Low. Backend contract is fully verified via 35/35 passing offline contract checks (scripts/verify-veritaqc-import.js) plus three live-API smoke checks against prod (candidates, preview, mappings PUT/GET) on Riverside Regional with seed lot SEED-1780436709094 (18 Glucose results). The browser-driven click was not run because Claude-in-Chrome's renderer froze repeatedly on the Radix Select inside VeritaCheckPage, not on Phase A code itself. Risk of a UX bug surviving to a customer is small but not zero.</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>task #77 stalled at Gate 3 step 8 on 2026-06-02. PR #500 squash-merged at commit 17a91ff, prod /api/health confirmed ACTIVE on that commit at 20:43 UTC.</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr"/>
-    </row>
-    <row r="11" ht="90" customHeight="1">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>42</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>Outbound demo-invite messaging campaign to 1st-degree LinkedIn contacts</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>Parked. Plan documented. Implementation deferred until trigger conditions met.
 ---
@@ -981,69 +941,69 @@
 _(item #51 closed 2026-09-2...</t>
         </is>
       </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>L (1 week prep + 4-6 weeks of staged sends)</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>High. Converts existing warm network (~2,500 1st-degree contacts and growing...</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>A staged outbound DM campaign walking Michael's 1st-degree LinkedIn contacts through tier-segmented demo invitations for VeritaAssure. Goal: convert warmest contacts into demo conversations first, then chain into trials and paid subscriptions. Separate pipeline from COLA cohort follow-up and from content-driven inbound; all three feed the same demo funnel but originate from different warmth sources.</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 session, after weekly LinkedIn invite batch completion (80 sent, cap hit at #84 Victoria Allen).</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11" ht="90" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Regenerate the 119-function access-inventory Excel with the corrected MD persona</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Open, low priority. Offered to Michael; skippable if the sweep was a one-off working artifact.
+---</t>
+        </is>
+      </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>L (1 week prep + 4-6 weeks of staged sends)</t>
+          <t>XS (~15 min to re-run the sweep harness and re-deliver).</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>High. Converts existing warm network (~2,500 1st-degree contacts and growing...</t>
+          <t>Low — the harness and the shipped fixes are correct; only the recorded Excel'...</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>A staged outbound DM campaign walking Michael's 1st-degree LinkedIn contacts through tier-segmented demo invitations for VeritaAssure. Goal: convert warmest contacts into demo conversations first, then chain into trials and paid subscriptions. Separate pipeline from COLA cohort follow-up and from content-driven inbound; all three feed the same demo funnel but originate from different warmth sources.</t>
+          <t>The full-inventory 4-login access sweep (VeritaAssure_Function_Inventory.xlsx) was first generated with the medical-director test persona mis-seeded as a seatless member, which over-flagged its column. The harness was then corrected to seat the MD as the active writer it actually is (scripts/qa-sweep/inventory-sweep.ts). The delivered Excel still shows the old md results; re-running reclassifies the md-artifact flags down to the real findings, which were already fixed in PR A (#1441). Only worth doing if the sheet gets filed or shared externally.</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>2026-06-04 session, after weekly LinkedIn invite batch completion (80 sent, cap hit at #84 Victoria Allen).</t>
+          <t>this session, QA sweep (2026-10-03 to 2026-10-04).</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr"/>
     </row>
-    <row r="12" ht="90" customHeight="1">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>44</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Regenerate the 119-function access-inventory Excel with the corrected MD persona</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Open, low priority. Offered to Michael; skippable if the sweep was a one-off working artifact.
----</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>XS (~15 min to re-run the sweep harness and re-deliver).</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>Low — the harness and the shipped fixes are correct; only the recorded Excel'...</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>The full-inventory 4-login access sweep (VeritaAssure_Function_Inventory.xlsx) was first generated with the medical-director test persona mis-seeded as a seatless member, which over-flagged its column. The harness was then corrected to seat the MD as the active writer it actually is (scripts/qa-sweep/inventory-sweep.ts). The delivered Excel still shows the old md results; re-running reclassifies the md-artifact flags down to the real findings, which were already fixed in PR A (#1441). Only worth doing if the sheet gets filed or shared externally.</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>this session, QA sweep (2026-10-03 to 2026-10-04).</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:H12"/>
+  <autoFilter ref="A1:H11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1054,7 +1014,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H60"/>
+  <dimension ref="A1:H61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1112,24 +1072,24 @@
     <row r="2" ht="90" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>C59</t>
+          <t>C60</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Confirm the finding-closure signer policy (was #43)</t>
+          <t>VeritaQC Import Phase A browser click-through (was #40)</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr"/>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>was XS / Importance: Medium</t>
+          <t>was XS / Importance: Low</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Effort: was XS / Importance: Medium</t>
+          <t>Effort: was XS / Importance: Low</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
@@ -1138,24 +1098,24 @@
     <row r="3" ht="90" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>C58</t>
+          <t>C59</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>VeritaDC per-document attestation tracker + "My Documents" rename (built as #45)</t>
+          <t>Confirm the finding-closure signer policy (was #43)</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr"/>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>was M / Importance: Medium-High</t>
+          <t>was XS / Importance: Medium</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Effort: was M / Importance: Medium-High</t>
+          <t>Effort: was XS / Importance: Medium</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr"/>
@@ -1164,24 +1124,24 @@
     <row r="4" ht="90" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>C57</t>
+          <t>C58</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Hide sections a lab does not use from a master list (was #47)</t>
+          <t>VeritaDC per-document attestation tracker + "My Documents" rename (built as #45)</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr"/>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>was S-M / Importance: Medium-High (prospect-requested)</t>
+          <t>was M / Importance: Medium-High</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Effort: was S-M / Importance: Medium-High (prospect-requested)</t>
+          <t>Effort: was M / Importance: Medium-High</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr"/>
@@ -1190,24 +1150,24 @@
     <row r="5" ht="90" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>C56</t>
+          <t>C57</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>VeritaCEU: curated free continuing-education provider list (was #53)</t>
+          <t>Hide sections a lab does not use from a master list (was #47)</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr"/>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>was S / Importance: Low-Medium</t>
+          <t>was S-M / Importance: Medium-High (prospect-requested)</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Effort: was S / Importance: Low-Medium</t>
+          <t>Effort: was S-M / Importance: Medium-High (prospect-requested)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr"/>
@@ -1216,24 +1176,24 @@
     <row r="6" ht="90" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>C55</t>
+          <t>C56</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>VeritaScan: let sites add their own custom questions (was #55)</t>
+          <t>VeritaCEU: curated free continuing-education provider list (was #53)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr"/>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>was M / Importance: Medium-High</t>
+          <t>was S / Importance: Low-Medium</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Effort: was M / Importance: Medium-High</t>
+          <t>Effort: was S / Importance: Low-Medium</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
@@ -1242,24 +1202,24 @@
     <row r="7" ht="90" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>C54</t>
+          <t>C55</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>VeritaQC: at-entry warning when a QC point is outside 2 SD (was #56)</t>
+          <t>VeritaScan: let sites add their own custom questions (was #55)</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr"/>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>was S-M (shipped S) / Importance: High</t>
+          <t>was M / Importance: Medium-High</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Effort: was S-M (shipped S) / Importance: High</t>
+          <t>Effort: was M / Importance: Medium-High</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr"/>
@@ -1268,24 +1228,24 @@
     <row r="8" ht="90" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>C53</t>
+          <t>C54</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>VeritaTrack: quarterly task loaded as monthly until re-saved (was #54)</t>
+          <t>VeritaQC: at-entry warning when a QC point is outside 2 SD (was #56)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr"/>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>was S / Importance: Medium</t>
+          <t>was S-M (shipped S) / Importance: High</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Effort: was S / Importance: Medium</t>
+          <t>Effort: was S-M (shipped S) / Importance: High</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
@@ -1294,24 +1254,24 @@
     <row r="9" ht="90" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>C52</t>
+          <t>C53</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>VeritaResponse internal NCE / non-conforming event (was #36)</t>
+          <t>VeritaTrack: quarterly task loaded as monthly until re-saved (was #54)</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr"/>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>was L (shipped as MEDIUM) / Importance: High</t>
+          <t>was S / Importance: Medium</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Effort: was L (shipped as MEDIUM) / Importance: High</t>
+          <t>Effort: was S / Importance: Medium</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr"/>
@@ -1320,24 +1280,24 @@
     <row r="10" ht="90" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>C49</t>
+          <t>C52</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Competency "assessed this cycle" cadence-aware window (was #50)</t>
+          <t>VeritaResponse internal NCE / non-conforming event (was #36)</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr"/>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>was S-M / Importance: Medium</t>
+          <t>was L (shipped as MEDIUM) / Importance: High</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Effort: was S-M / Importance: Medium</t>
+          <t>Effort: was L (shipped as MEDIUM) / Importance: High</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
@@ -1346,12 +1306,12 @@
     <row r="11" ht="90" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>C50</t>
+          <t>C49</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>VeritaTrack task owner + owner-only reminder routing (was #51)</t>
+          <t>Competency "assessed this cycle" cadence-aware window (was #50)</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr"/>
@@ -1372,24 +1332,24 @@
     <row r="12" ht="90" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>C51</t>
+          <t>C50</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Designate Medical Director by picking a lab member (was #52, core)</t>
+          <t>VeritaTrack task owner + owner-only reminder routing (was #51)</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr"/>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>was S-M / Importance: Medium-High</t>
+          <t>was S-M / Importance: Medium</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Effort: was S-M / Importance: Medium-High</t>
+          <t>Effort: was S-M / Importance: Medium</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr"/>
@@ -1398,24 +1358,24 @@
     <row r="13" ht="90" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>C47</t>
+          <t>C51</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Unregulated-analyte / Alternative Assessment (AAA) coverage (was #18)</t>
+          <t>Designate Medical Director by picking a lab member (was #52, core)</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr"/>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>was S (Phase 3) / Importance: Medium</t>
+          <t>was S-M / Importance: Medium-High</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Effort: was S (Phase 3) / Importance: Medium</t>
+          <t>Effort: was S-M / Importance: Medium-High</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr"/>
@@ -1424,24 +1384,24 @@
     <row r="14" ht="90" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>C48</t>
+          <t>C47</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>VeritaResponse post-survey deficiency module (was #17)</t>
+          <t>Unregulated-analyte / Alternative Assessment (AAA) coverage (was #18)</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr"/>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>was XL / Importance: High</t>
+          <t>was S (Phase 3) / Importance: Medium</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Effort: was XL / Importance: High</t>
+          <t>Effort: was S (Phase 3) / Importance: Medium</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr"/>
@@ -1450,39 +1410,38 @@
     <row r="15" ht="90" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>C45</t>
+          <t>C48</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Unify coverage/competency recurrence helper (was #49) - closed as non-issue</t>
+          <t>VeritaResponse post-survey deficiency module (was #17)</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr"/>
-      <c r="D15" s="3" t="inlineStr"/>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>was XL / Importance: High</t>
+        </is>
+      </c>
       <c r="E15" s="3" t="inlineStr"/>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: Investigated 2026-09-24 before building. The coverage recurrence math (+6-month interval, signed-resets-to-missing, nextDueOn/overdue, isFailVerdict) is ALREADY single-source in server/veritacheckCoverage.ts (computeCoverageFrom). server/coverageReport.ts and the routes.ts coverage export do not recompute it; they consume the computed nextDueOn/overdue/status fields and apply small surface-specific presentation labels (deliberately different vocabularies per surface, so they should not be merged). The only truly identical duplicate is a one-line date formatter. The competency "owed" derivation is NOT the same cadence: competency follows the CLIA milestone schedule (initial / semiannual year 1 / annual, 42 CFR 493.1451(b)(8) and 493.1235), which is a different regulatory interval from the coverage 6-month rule (493.1281 / 493.1255) and must stay separate. No worthwhile extraction; merging the two cadences would be wrong. Closed 2026-09-24. (The year-1 competency-window refinement remains tracked separately as #50.)</t>
-        </is>
-      </c>
-      <c r="G15" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-24 session, "keep working" pass; scoped read-only, found no real duplication.
----</t>
-        </is>
-      </c>
+          <t>Effort: was XL / Importance: High</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr"/>
       <c r="H15" s="3" t="inlineStr"/>
     </row>
     <row r="16" ht="90" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>C46</t>
+          <t>C45</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Verified-users product-update send path (wrong-list incident fix)</t>
+          <t>Unify coverage/competency recurrence helper (was #49) - closed as non-issue</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr"/>
@@ -1490,12 +1449,12 @@
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: Shipped PR #1324 (merged 4e05506a, deploy ACTIVE). New POST /api/admin/users/send targets registered VeritaAssure account holders (the users table), never the Lab Director's Briefing subscriber list. Separate explicitly-named endpoint (not a flag with a dangerous default), account-holder email framing, excludes suppressed emails and RFC-reserved test domains, CC owner, dryRun + testTo previews. Public unsubscribe now upserts a suppression row so opt-outs are honored across both audiences. Live dryRun: 49 verified-user recipients vs 673 on the Briefing list. Receipts: scripts/verify-product-update-send.mts 24/24, tsc clean, rendered sample inspected. Fixes the fallout from the 2026-09-23/24 wrong-list send (a product update went to the 675-person Briefing list). Nothing sends without Michael's explicit "send it."</t>
+          <t>Closure evidence: Investigated 2026-09-24 before building. The coverage recurrence math (+6-month interval, signed-resets-to-missing, nextDueOn/overdue, isFailVerdict) is ALREADY single-source in server/veritacheckCoverage.ts (computeCoverageFrom). server/coverageReport.ts and the routes.ts coverage export do not recompute it; they consume the computed nextDueOn/overdue/status fields and apply small surface-specific presentation labels (deliberately different vocabularies per surface, so they should not be merged). The only truly identical duplicate is a one-line date formatter. The competency "owed" derivation is NOT the same cadence: competency follows the CLIA milestone schedule (initial / semiannual year 1 / annual, 42 CFR 493.1451(b)(8) and 493.1235), which is a different regulatory interval from the coverage 6-month rule (493.1281 / 493.1255) and must stay separate. No worthwhile extraction; merging the two cadences would be wrong. Closed 2026-09-24. (The year-1 competency-window refinement remains tracked separately as #50.)</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 session; Michael selected this as the next build after the #41 close.
+          <t>2026-09-24 session, "keep working" pass; scoped read-only, found no real duplication.
 ---</t>
         </is>
       </c>
@@ -1504,12 +1463,12 @@
     <row r="17" ht="90" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>C44</t>
+          <t>C46</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Verify-script convention backfill (was #41) + audit matcher fix</t>
+          <t>Verified-users product-update send path (wrong-list incident fix)</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr"/>
@@ -1517,12 +1476,12 @@
       <c r="E17" s="3" t="inlineStr"/>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: #41 was fully backfilled on 2026-06-13 (all 8 high-stakes scripts landed; see C30); it had only been mis-filed in OPEN. A 2026-09-24 re-audit initially reported 4 of 5 recent math/logic commits as missing a verify script, which was a FALSE POSITIVE: scripts/audit_verify_script_coverage.py matched only scripts/verify-*.js / .cjs, so it ignored the .mjs / .mts / .ts verify scripts the repo now ships (e.g. verify-ptcoag-multi.mts, verify-tea-criterion-format.mjs). Fixed the matcher to accept .js/.cjs/.mjs/.ts/.mts; re-run shows 5 of 5 covered, 0 debt. The convention is being followed. Closed 2026-09-24.</t>
+          <t>Closure evidence: Shipped PR #1324 (merged 4e05506a, deploy ACTIVE). New POST /api/admin/users/send targets registered VeritaAssure account holders (the users table), never the Lab Director's Briefing subscriber list. Separate explicitly-named endpoint (not a flag with a dangerous default), account-holder email framing, excludes suppressed emails and RFC-reserved test domains, CC owner, dryRun + testTo previews. Public unsubscribe now upserts a suppression row so opt-outs are honored across both audiences. Live dryRun: 49 verified-user recipients vs 673 on the Briefing list. Receipts: scripts/verify-product-update-send.mts 24/24, tsc clean, rendered sample inspected. Fixes the fallout from the 2026-09-23/24 wrong-list send (a product update went to the 675-person Briefing list). Nothing sends without Michael's explicit "send it."</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>2026-09-24 session, "keep working" pass; audit tooling bug found + fixed.
+          <t>2026-09-24 session; Michael selected this as the next build after the #41 close.
 ---</t>
         </is>
       </c>
@@ -1531,12 +1490,12 @@
     <row r="18" ht="90" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>C43</t>
+          <t>C44</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>VeritaStaff instrument-centric (dual) assignment view</t>
+          <t>Verify-script convention backfill (was #41) + audit matcher fix</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr"/>
@@ -1544,12 +1503,12 @@
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1320. GET/PUT /staff/instruments/:id/employees (transpose of the per-employee endpoints); an "Assign by Instrument" dialog lets a director pick a test system or manual test and check off who runs it. Same staff_employee_instruments join, with the 42 CFR 493.1235(a) duty-change event emitted on newly-added pairs so both orientations trigger the same reassessment. GET verified live on SCAHC lab 2. Closed 2026-09-24.</t>
+          <t>Closure evidence: #41 was fully backfilled on 2026-06-13 (all 8 high-stakes scripts landed; see C30); it had only been mis-filed in OPEN. A 2026-09-24 re-audit initially reported 4 of 5 recent math/logic commits as missing a verify script, which was a FALSE POSITIVE: scripts/audit_verify_script_coverage.py matched only scripts/verify-*.js / .cjs, so it ignored the .mjs / .mts / .ts verify scripts the repo now ships (e.g. verify-ptcoag-multi.mts, verify-tea-criterion-format.mjs). Fixed the matcher to accept .js/.cjs/.mjs/.ts/.mts; re-run shows 5 of 5 covered, 0 debt. The convention is being followed. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 session, Michael ("in staff we should also give the dual view when assigning coverage to test systems or manual tests").
+          <t>2026-09-24 session, "keep working" pass; audit tooling bug found + fixed.
 ---</t>
         </is>
       </c>
@@ -1558,12 +1517,12 @@
     <row r="19" ht="90" customHeight="1">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>C42</t>
+          <t>C43</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>VeritaComp coverage map (required-vs-assessed matrix, dual view)</t>
+          <t>VeritaStaff instrument-centric (dual) assignment view</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr"/>
@@ -1571,12 +1530,12 @@
       <c r="E19" s="3" t="inlineStr"/>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1319 (+ status layer PR #1316). /competency/owed returns per-item assessed (locked passing assessment this cycle on a covering method group) + per-employee CLIA status; CompetencyCoverageMap renders a By-employee / By-instrument matrix (Assessed / Owed / Overdue / Gap). Verified live on SCAHC lab 2 (owed 116, assessed 2, gaps 0). Completes #48 as the VeritaCheck-parity coverage map. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1320. GET/PUT /staff/instruments/:id/employees (transpose of the per-employee endpoints); an "Assign by Instrument" dialog lets a director pick a test system or manual test and check off who runs it. Same staff_employee_instruments join, with the 42 CFR 493.1235(a) duty-change event emitted on newly-added pairs so both orientations trigger the same reassessment. GET verified live on SCAHC lab 2. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>2026-09-24 session, Michael ("are we building the competencies to have a coverage map, same as veritacheck?" then "build it").
+          <t>2026-09-24 session, Michael ("in staff we should also give the dual view when assigning coverage to test systems or manual tests").
 ---</t>
         </is>
       </c>
@@ -1585,12 +1544,12 @@
     <row r="20" ht="90" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>C41</t>
+          <t>C42</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>VeritaCheck coverage recurrence (method comparison + cal-ver/linearity + reports)</t>
+          <t>VeritaComp coverage map (required-vs-assessed matrix, dual view)</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr"/>
@@ -1598,12 +1557,12 @@
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: PRs #1317 (method comparison), #1318 (cal-ver/linearity), #1321 (report Next-due columns). Periodic verification (correlation/method comparison 42 CFR 493.1281; cal-ver/linearity 42 CFR 493.1255; both 6-month) now recurs: a signed study banks the cycle and rolls to next-due = signed + 6 months instead of reading "done" forever. Status Missing/Failed/Completed-unsigned + a "Next due on" column on-screen and in both coverage exports; also credits the previously-ignored "correlation" study type. Root cause: computeCoverageFrom marked requirements done on mere existence, no date logic. Verified live on SCAHC lab 2 (101 correlations + 11 cal-ver rows now carry a next-due). Engine-level, all facilities. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1319 (+ status layer PR #1316). /competency/owed returns per-item assessed (locked passing assessment this cycle on a covering method group) + per-employee CLIA status; CompetencyCoverageMap renders a By-employee / By-instrument matrix (Assessed / Owed / Overdue / Gap). Verified live on SCAHC lab 2 (owed 116, assessed 2, gaps 0). Completes #48 as the VeritaCheck-parity coverage map. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 session, Michael ("Look at San Carlos... they finished their last set of correlations (all 103) but their menu never reset").
+          <t>2026-09-24 session, Michael ("are we building the competencies to have a coverage map, same as veritacheck?" then "build it").
 ---</t>
         </is>
       </c>
@@ -1612,12 +1571,12 @@
     <row r="21" ht="90" customHeight="1">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>C40</t>
+          <t>C41</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>VeritaComp Competencies Owed derived from VeritaStaff, with gap detection (was #48)</t>
+          <t>VeritaCheck coverage recurrence (method comparison + cal-ver/linearity + reports)</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr"/>
@@ -1625,12 +1584,12 @@
       <c r="E21" s="3" t="inlineStr"/>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1314 (squash 2bcb0db9). GET /api/labs/:labId/competency/owed derives each VeritaStaff testing employee's owed competencies from their assigned instruments (staff_employee_instruments -&gt; veritamap_instruments + tests), on the CLIA timeline, and flags instruments not covered by any competency program as gaps. CompetenciesOwedSection renders it on the VeritaComp landing page. Reuses the shipped bridge + suggested-method-groups match rules; no new tables. Verified live on prod with real assignment data: 2 instruments assigned to a demo staffer produced owed=2, gaps=2 (HIGH, Technical Supervisor), then reverted cleanly. Closed 2026-09-24.</t>
+          <t>Closure evidence: PRs #1317 (method comparison), #1318 (cal-ver/linearity), #1321 (report Next-due columns). Periodic verification (correlation/method comparison 42 CFR 493.1281; cal-ver/linearity 42 CFR 493.1255; both 6-month) now recurs: a signed study banks the cycle and rolls to next-due = signed + 6 months instead of reading "done" forever. Status Missing/Failed/Completed-unsigned + a "Next due on" column on-screen and in both coverage exports; also credits the previously-ignored "correlation" study type. Root cause: computeCoverageFrom marked requirements done on mere existence, no date logic. Verified live on SCAHC lab 2 (101 correlations + 11 cal-ver rows now carry a next-due). Engine-level, all facilities. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>2026-09-23/24 session, Michael ("veritacomp bases what competencies they owe (currently untrue, but needs to be true)"). Option 1 (unify roster on VeritaStaff, match instruments by id).
+          <t>2026-09-24 session, Michael ("Look at San Carlos... they finished their last set of correlations (all 103) but their menu never reset").
 ---</t>
         </is>
       </c>
@@ -1639,12 +1598,12 @@
     <row r="22" ht="90" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>C39</t>
+          <t>C40</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>VeritaScan line items can attach or link evidence (was #46)</t>
+          <t>VeritaComp Competencies Owed derived from VeritaStaff, with gap detection (was #48)</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr"/>
@@ -1652,12 +1611,12 @@
       <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: PR #1312 (squash a1dda93d). VeritaScan scan checklist items now show linked evidence as chips (open link, remove) plus a writer "Link evidence" affordance whose picker links an existing VeritaDC/Library document; a shortcut deep-links to the Library for new (governed) documents. Reuses the already-shipped lab_documents + document_checklist_links + coverage endpoints (URL-pointer only, no file storage, no new tables). Browser-verified live on prod (scan 23): the affordance renders and the picker opens. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1314 (squash 2bcb0db9). GET /api/labs/:labId/competency/owed derives each VeritaStaff testing employee's owed competencies from their assigned instruments (staff_employee_instruments -&gt; veritamap_instruments + tests), on the CLIA timeline, and flags instruments not covered by any competency program as gaps. CompetenciesOwedSection renders it on the VeritaComp landing page. Reuses the shipped bridge + suggested-method-groups match rules; no new tables. Verified live on prod with real assignment data: 2 instruments assigned to a demo staffer produced owed=2, gaps=2 (HIGH, Technical Supervisor), then reverted cleanly. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23 session, Michael. Recurring request. Companion: cross-module evidence display on the VeritaDC policy shipped in PR #1313 (by-target cross-links surfaced in the policy View modal, browser-verified live).
+          <t>2026-09-23/24 session, Michael ("veritacomp bases what competencies they owe (currently untrue, but needs to be true)"). Option 1 (unify roster on VeritaStaff, match instruments by id).
 ---</t>
         </is>
       </c>
@@ -1666,12 +1625,12 @@
     <row r="23" ht="90" customHeight="1">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>C38</t>
+          <t>C39</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>VeritaTrack calendar month cells expand to reveal hidden tasks (was #45)</t>
+          <t>VeritaScan line items can attach or link evidence (was #46)</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr"/>
@@ -1679,12 +1638,12 @@
       <c r="E23" s="3" t="inlineStr"/>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: VeritaTrack CalendarView month cells with more than three tasks now expand in place (chevron, "+N more" toggling to "Show less", due dates), so no task is hidden with no path to it (client/src/pages/VeritaTrackAppPage.tsx CalendarView). Shipped 2026-09-23. Closed 2026-09-24.</t>
+          <t>Closure evidence: PR #1312 (squash a1dda93d). VeritaScan scan checklist items now show linked evidence as chips (open link, remove) plus a writer "Link evidence" affordance whose picker links an existing VeritaDC/Library document; a shortcut deep-links to the Library for new (governed) documents. Reuses the already-shipped lab_documents + document_checklist_links + coverage endpoints (URL-pointer only, no file storage, no new tables). Browser-verified live on prod (scan 23): the affordance renders and the picker opens. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>2026-09-23 session, Michael screenshot of the VeritaTrack calendar (lab 3, September cell).
+          <t>2026-09-23 session, Michael. Recurring request. Companion: cross-module evidence display on the VeritaDC policy shipped in PR #1313 (by-target cross-links surfaced in the policy View modal, browser-verified live).
 ---</t>
         </is>
       </c>
@@ -1693,12 +1652,12 @@
     <row r="24" ht="90" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>C37</t>
+          <t>C38</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Long Excel column headers no longer clip CFR citations (was #44)</t>
+          <t>VeritaTrack calendar month cells expand to reveal hidden tasks (was #45)</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr"/>
@@ -1706,12 +1665,12 @@
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. The VeritaMap export derives the header row height from the longest wrapped header via headerRowHeight(headers, colWidths) (server/routes.ts:15935) instead of a fixed 20, so "Reference Range Attestation (42 CFR 493.1253)" and the other long headers print in full. No new code this session. Closed 2026-09-24.</t>
+          <t>Closure evidence: VeritaTrack CalendarView month cells with more than three tasks now expand in place (chevron, "+N more" toggling to "Show less", due dates), so no task is hidden with no path to it (client/src/pages/VeritaTrackAppPage.tsx CalendarView). Shipped 2026-09-23. Closed 2026-09-24.</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>parked 2026-07-16 (PR 4 Gate 3 render); found already-fixed 2026-09-24.
+          <t>2026-09-23 session, Michael screenshot of the VeritaTrack calendar (lab 3, September cell).
 ---</t>
         </is>
       </c>
@@ -1720,12 +1679,12 @@
     <row r="25" ht="90" customHeight="1">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>C36</t>
+          <t>C37</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>License stamp no longer clobbers the §6 header/footer or names the wrong lab (was #43)</t>
+          <t>Long Excel column headers no longer clip CFR citations (was #44)</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr"/>
@@ -1733,7 +1692,7 @@
       <c r="E25" s="3" t="inlineStr"/>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. setHeaderFooter (shared/licenseExceljs.ts:155-209) now preserves an existing §6 header and appends (not overwrites) the footer left section, and customer-facing exports name the scoped lab: the VeritaScan library export reads req.scope.lab.name / clia_number (server/routes.ts:16572-16573), not the licensee. No new code this session (avoided regressing the existing fix). Closed 2026-09-24.</t>
+          <t>Closure evidence: Verified already fixed on main during the 2026-09-24 session. The VeritaMap export derives the header row height from the longest wrapped header via headerRowHeight(headers, colWidths) (server/routes.ts:15935) instead of a fixed 20, so "Reference Range Attestation (42 CFR 493.1253)" and the other long headers print in full. No new code this session. Close